<commit_message>
Auto: update momentum data - 2026-03-03 05:08 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -503,11 +503,11 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>45.19</v>
+        <v>43.98</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>-5.26</v>
+        <v>-7.8</v>
       </c>
     </row>
     <row r="4">
@@ -529,11 +529,11 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>4.15</v>
+        <v>4.18</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>-11.7</v>
+        <v>-11.06</v>
       </c>
     </row>
     <row r="5">
@@ -555,11 +555,11 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>32.3</v>
+        <v>31.4</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>-7.42</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="6">
@@ -581,11 +581,11 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>10.2</v>
+        <v>10.1</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>-4.67</v>
+        <v>-5.61</v>
       </c>
     </row>
     <row r="7">
@@ -607,11 +607,11 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>-7.48</v>
+        <v>-8.84</v>
       </c>
     </row>
     <row r="8">
@@ -633,11 +633,11 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>63.01</v>
+        <v>62.13</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>-5.94</v>
+        <v>-7.25</v>
       </c>
     </row>
     <row r="9">
@@ -659,24 +659,24 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>321.55</v>
+        <v>312.05</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>-5.43</v>
+        <v>-8.220000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NEUEON</t>
+          <t>SETUINFRA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10.8</v>
+        <v>0.4</v>
       </c>
       <c r="C10" t="n">
-        <v>11.34</v>
+        <v>0.42</v>
       </c>
       <c r="D10" t="n">
         <v>5</v>
@@ -685,7 +685,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>11.34</v>
+        <v>0.42</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
@@ -695,14 +695,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SETUINFRA</t>
+          <t>NEUEON</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.4</v>
+        <v>10.8</v>
       </c>
       <c r="C11" t="n">
-        <v>0.42</v>
+        <v>11.34</v>
       </c>
       <c r="D11" t="n">
         <v>5</v>
@@ -711,7 +711,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.42</v>
+        <v>11.34</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
@@ -737,24 +737,24 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>23.9</v>
+        <v>24.77</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>-7.69</v>
+        <v>-4.33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.41</v>
+        <v>16.92</v>
       </c>
       <c r="C13" t="n">
-        <v>1.48</v>
+        <v>17.76</v>
       </c>
       <c r="D13" t="n">
         <v>4.96</v>
@@ -763,7 +763,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>1.48</v>
+        <v>17.76</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
@@ -773,14 +773,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.92</v>
+        <v>12.91</v>
       </c>
       <c r="C14" t="n">
-        <v>17.76</v>
+        <v>13.55</v>
       </c>
       <c r="D14" t="n">
         <v>4.96</v>
@@ -789,24 +789,24 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>17.76</v>
+        <v>13</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>-4.06</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12.91</v>
+        <v>1.41</v>
       </c>
       <c r="C15" t="n">
-        <v>13.55</v>
+        <v>1.48</v>
       </c>
       <c r="D15" t="n">
         <v>4.96</v>
@@ -815,11 +815,11 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>13.4</v>
+        <v>1.35</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>-1.11</v>
+        <v>-8.779999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -841,11 +841,11 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>70.95999999999999</v>
+        <v>71.16</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>-8.5</v>
+        <v>-8.24</v>
       </c>
     </row>
     <row r="17">
@@ -867,11 +867,11 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>33.52</v>
+        <v>32.34</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>-1.82</v>
+        <v>-5.27</v>
       </c>
     </row>
     <row r="18">
@@ -893,11 +893,11 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>6.42</v>
+        <v>6.39</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>-8.15</v>
+        <v>-8.58</v>
       </c>
     </row>
     <row r="19">
@@ -945,24 +945,24 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>1.58</v>
+        <v>1.57</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>-0.63</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>DHARIWAL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>21.33</v>
+        <v>41.8</v>
       </c>
       <c r="C21" t="n">
-        <v>22.3</v>
+        <v>43.7</v>
       </c>
       <c r="D21" t="n">
         <v>4.55</v>
@@ -971,24 +971,24 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>21.21</v>
+        <v>43.85</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>-4.89</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DHARIWAL</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>41.8</v>
+        <v>21.33</v>
       </c>
       <c r="C22" t="n">
-        <v>43.7</v>
+        <v>22.3</v>
       </c>
       <c r="D22" t="n">
         <v>4.55</v>
@@ -997,11 +997,11 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>43.85</v>
+        <v>20.27</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>0.34</v>
+        <v>-9.1</v>
       </c>
     </row>
     <row r="23">
@@ -1023,11 +1023,11 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>479</v>
+        <v>484.7</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>-4.77</v>
+        <v>-3.64</v>
       </c>
     </row>
     <row r="24">
@@ -1049,11 +1049,11 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>-5.74</v>
+        <v>-4.92</v>
       </c>
     </row>
     <row r="25">
@@ -1075,11 +1075,11 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>19.39</v>
+        <v>19.37</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>-2.56</v>
+        <v>-2.66</v>
       </c>
     </row>
     <row r="26">
@@ -1101,11 +1101,11 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>116.75</v>
+        <v>117.1</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>-5</v>
+        <v>-4.72</v>
       </c>
     </row>
     <row r="27">
@@ -1127,11 +1127,11 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>6.88</v>
+        <v>6.72</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>-4.31</v>
+        <v>-6.54</v>
       </c>
     </row>
     <row r="28">
@@ -1153,11 +1153,11 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>16.08</v>
+        <v>16.05</v>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>-0.06</v>
+        <v>-0.25</v>
       </c>
     </row>
     <row r="29">
@@ -1179,24 +1179,24 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>279.85</v>
+        <v>281.45</v>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>-2.83</v>
+        <v>-2.27</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GJL</t>
+          <t>GPECO</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>163.4</v>
+        <v>355</v>
       </c>
       <c r="C30" t="n">
-        <v>168</v>
+        <v>365</v>
       </c>
       <c r="D30" t="n">
         <v>2.82</v>
@@ -1205,24 +1205,24 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>171.55</v>
+        <v>331</v>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>2.11</v>
+        <v>-9.32</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GPECO</t>
+          <t>GJL</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>355</v>
+        <v>163.4</v>
       </c>
       <c r="C31" t="n">
-        <v>365</v>
+        <v>168</v>
       </c>
       <c r="D31" t="n">
         <v>2.82</v>
@@ -1231,11 +1231,11 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>339</v>
+        <v>171.55</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>-7.12</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="32">
@@ -1257,11 +1257,11 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>58.01</v>
+        <v>55.26</v>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>-3.32</v>
+        <v>-7.9</v>
       </c>
     </row>
     <row r="33">
@@ -1309,11 +1309,11 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>56.8</v>
+        <v>56.02</v>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>-3.71</v>
+        <v>-5.03</v>
       </c>
     </row>
     <row r="35">
@@ -1335,11 +1335,11 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>-2.27</v>
       </c>
     </row>
     <row r="36">
@@ -1361,11 +1361,11 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>16.42</v>
+        <v>15.42</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>-3.13</v>
+        <v>-9.029999999999999</v>
       </c>
     </row>
     <row r="37">
@@ -1387,11 +1387,11 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>167.64</v>
+        <v>166.3</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>-2.53</v>
+        <v>-3.31</v>
       </c>
     </row>
     <row r="38">
@@ -1413,11 +1413,11 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>-1.93</v>
+        <v>-3.94</v>
       </c>
     </row>
     <row r="39">
@@ -1465,11 +1465,11 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>2.21</v>
+        <v>2.24</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>-1.78</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="41">
@@ -1491,11 +1491,11 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>108</v>
+        <v>108.29</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="42">
@@ -1517,11 +1517,11 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>136.77</v>
+        <v>136.79</v>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>2.83</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="43">
@@ -1543,11 +1543,11 @@
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>1.97</v>
+        <v>1.95</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>-1.01</v>
+        <v>-2.01</v>
       </c>
     </row>
     <row r="44">
@@ -1569,11 +1569,11 @@
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>29.2</v>
+        <v>28.5</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>-4.11</v>
+        <v>-6.4</v>
       </c>
     </row>
     <row r="45">
@@ -1621,11 +1621,11 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>184.5</v>
+        <v>183</v>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>-0.22</v>
+        <v>-1.03</v>
       </c>
     </row>
     <row r="47">
@@ -1647,11 +1647,11 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>5.15</v>
+        <v>5.21</v>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>2.18</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="48">
@@ -1673,11 +1673,11 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>18.98</v>
+        <v>19</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>-5.1</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="49">
@@ -1721,11 +1721,11 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>64.5</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>-3.44</v>
+        <v>-4.04</v>
       </c>
     </row>
     <row r="51">
@@ -1747,11 +1747,11 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>89.90000000000001</v>
+        <v>89</v>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>-1.75</v>
+        <v>-2.73</v>
       </c>
     </row>
     <row r="52">
@@ -1773,11 +1773,11 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>4946.5</v>
+        <v>4980.1</v>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>-0.05</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="53">
@@ -1799,11 +1799,11 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>45.3</v>
+        <v>44.8</v>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>-6.98</v>
+        <v>-8.01</v>
       </c>
     </row>
     <row r="54">
@@ -1825,11 +1825,11 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>17.11</v>
+        <v>17.1</v>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>-4.41</v>
+        <v>-4.47</v>
       </c>
     </row>
     <row r="55">
@@ -1851,11 +1851,11 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>25.4</v>
+        <v>24.75</v>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>-2.27</v>
+        <v>-4.77</v>
       </c>
     </row>
     <row r="56">
@@ -1877,11 +1877,11 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>17.4</v>
+        <v>17.68</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>-3.12</v>
+        <v>-1.56</v>
       </c>
     </row>
     <row r="57">
@@ -1903,11 +1903,11 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>112.49</v>
+        <v>112</v>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>-4.66</v>
+        <v>-5.08</v>
       </c>
     </row>
     <row r="58">
@@ -1929,11 +1929,11 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>1.39</v>
+        <v>1.44</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="59">
@@ -1955,11 +1955,11 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>212</v>
+        <v>211.9</v>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>-2.3</v>
+        <v>-2.35</v>
       </c>
     </row>
     <row r="60">
@@ -1981,11 +1981,11 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>16.5</v>
+        <v>16.37</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>-4.62</v>
+        <v>-5.38</v>
       </c>
     </row>
     <row r="61">
@@ -2007,11 +2007,11 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>54.57</v>
+        <v>52.88</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>-2.55</v>
+        <v>-5.57</v>
       </c>
     </row>
     <row r="62">
@@ -2033,11 +2033,11 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>-1.76</v>
+        <v>-4.69</v>
       </c>
     </row>
     <row r="63">
@@ -2059,11 +2059,11 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>87.98</v>
+        <v>88.84999999999999</v>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>0.09</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="64">
@@ -2085,11 +2085,11 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>37.89</v>
+        <v>37.42</v>
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>-1.53</v>
+        <v>-2.75</v>
       </c>
     </row>
     <row r="65">
@@ -2111,11 +2111,11 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>707.85</v>
+        <v>675</v>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>-1.73</v>
+        <v>-6.29</v>
       </c>
     </row>
     <row r="66">
@@ -2137,11 +2137,11 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>618.65</v>
+        <v>617</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>2.09</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="67">
@@ -2163,11 +2163,11 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>60.1</v>
+        <v>59.1</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>-0.83</v>
+        <v>-2.48</v>
       </c>
     </row>
     <row r="68">
@@ -2189,11 +2189,11 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>7.05</v>
+        <v>6.51</v>
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>3.52</v>
+        <v>-4.41</v>
       </c>
     </row>
     <row r="69">
@@ -2215,11 +2215,11 @@
         <v>0</v>
       </c>
       <c r="F69" t="n">
-        <v>166.09</v>
+        <v>166.75</v>
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>-0.37</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="70">
@@ -2241,11 +2241,11 @@
         <v>0</v>
       </c>
       <c r="F70" t="n">
-        <v>407.65</v>
+        <v>411</v>
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>-0.55</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="71">
@@ -2267,11 +2267,11 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>29.31</v>
+        <v>28.35</v>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>-1.97</v>
+        <v>-5.18</v>
       </c>
     </row>
     <row r="72">
@@ -2293,11 +2293,11 @@
         <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>64.78</v>
+        <v>63</v>
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>-1.33</v>
+        <v>-4.04</v>
       </c>
     </row>
     <row r="73">
@@ -2319,11 +2319,11 @@
         <v>0</v>
       </c>
       <c r="F73" t="n">
-        <v>470.6</v>
+        <v>471.4</v>
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>-1.96</v>
+        <v>-1.79</v>
       </c>
     </row>
     <row r="74">
@@ -2345,11 +2345,11 @@
         <v>0</v>
       </c>
       <c r="F74" t="n">
-        <v>523</v>
+        <v>532.2</v>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>1.55</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="75">
@@ -2371,11 +2371,11 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>5711</v>
+        <v>5648.5</v>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>-1.19</v>
+        <v>-2.27</v>
       </c>
     </row>
     <row r="76">
@@ -2397,11 +2397,11 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>64.27</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>-0.97</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="77">
@@ -2423,11 +2423,11 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>3423.8</v>
+        <v>3466</v>
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>2.05</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="78">
@@ -2449,24 +2449,24 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>78.90000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>-2</v>
+        <v>-3.24</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>RADAAN</t>
+          <t>BHADORA</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>3.12</v>
+        <v>64.45</v>
       </c>
       <c r="C79" t="n">
-        <v>3.12</v>
+        <v>64.45</v>
       </c>
       <c r="D79" t="n">
         <v>0</v>
@@ -2475,24 +2475,24 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>2.98</v>
+        <v>61.1</v>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>-4.49</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ALLDIGI</t>
+          <t>VINYLINDIA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>823.55</v>
+        <v>209.89</v>
       </c>
       <c r="C80" t="n">
-        <v>823.55</v>
+        <v>209.89</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
@@ -2501,24 +2501,24 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>824.1</v>
+        <v>205</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>0.07000000000000001</v>
+        <v>-2.33</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TRIGYN</t>
+          <t>HTMEDIA</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>52.11</v>
+        <v>21.82</v>
       </c>
       <c r="C81" t="n">
-        <v>52.11</v>
+        <v>21.82</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
@@ -2527,24 +2527,24 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>51.4</v>
+        <v>20.7</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>-1.36</v>
+        <v>-5.13</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>1.7</v>
+        <v>4.1</v>
       </c>
       <c r="C82" t="n">
-        <v>1.7</v>
+        <v>4.1</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
@@ -2553,24 +2553,24 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>1.67</v>
+        <v>4.05</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>-1.76</v>
+        <v>-1.22</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ARCHIES</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>15.82</v>
+        <v>0.22</v>
       </c>
       <c r="C83" t="n">
-        <v>15.82</v>
+        <v>0.22</v>
       </c>
       <c r="D83" t="n">
         <v>0</v>
@@ -2579,24 +2579,24 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>14.95</v>
+        <v>0.21</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>-5.5</v>
+        <v>-4.55</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PRAKASHSTL</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>4.37</v>
+        <v>12.7</v>
       </c>
       <c r="C84" t="n">
-        <v>4.37</v>
+        <v>12.7</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -2605,24 +2605,24 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>4.39</v>
+        <v>12.7</v>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>0.46</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AILIMITED</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>36.55</v>
+        <v>5.03</v>
       </c>
       <c r="C85" t="n">
-        <v>36.55</v>
+        <v>5.03</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -2631,24 +2631,24 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>38.35</v>
+        <v>4.89</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>4.92</v>
+        <v>-2.78</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PREMIER</t>
+          <t>HALEOSLABS</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2.99</v>
+        <v>1260.3</v>
       </c>
       <c r="C86" t="n">
-        <v>2.99</v>
+        <v>1260.3</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
@@ -2657,24 +2657,24 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>2.85</v>
+        <v>1251</v>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>-4.68</v>
+        <v>-0.74</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>TIL</t>
+          <t>TECHLABS</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>208.98</v>
+        <v>195</v>
       </c>
       <c r="C87" t="n">
-        <v>208.98</v>
+        <v>195</v>
       </c>
       <c r="D87" t="n">
         <v>0</v>
@@ -2683,24 +2683,24 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>213.79</v>
+        <v>199.9</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>2.3</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>RELCHEMQ</t>
+          <t>ONECAP-RE</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>122.33</v>
+        <v>0.2</v>
       </c>
       <c r="C88" t="n">
-        <v>122.33</v>
+        <v>0.2</v>
       </c>
       <c r="D88" t="n">
         <v>0</v>
@@ -2709,24 +2709,24 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>118.61</v>
+        <v>0.18</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>-3.04</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>OBCL</t>
+          <t>MARUSHIKA</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>55.99</v>
+        <v>103.15</v>
       </c>
       <c r="C89" t="n">
-        <v>55.99</v>
+        <v>103.15</v>
       </c>
       <c r="D89" t="n">
         <v>0</v>
@@ -2735,24 +2735,24 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>55.06</v>
+        <v>101.5</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>-1.66</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BANG</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>41.52</v>
+        <v>1.7</v>
       </c>
       <c r="C90" t="n">
-        <v>41.52</v>
+        <v>1.7</v>
       </c>
       <c r="D90" t="n">
         <v>0</v>
@@ -2761,24 +2761,24 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>41.99</v>
+        <v>1.69</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>1.13</v>
+        <v>-0.59</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>HALEOSLABS</t>
+          <t>GOLDTECH</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1260.3</v>
+        <v>39.8</v>
       </c>
       <c r="C91" t="n">
-        <v>1260.3</v>
+        <v>39.8</v>
       </c>
       <c r="D91" t="n">
         <v>0</v>
@@ -2787,24 +2787,24 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>1246</v>
+        <v>39</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>-1.13</v>
+        <v>-2.01</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>AHLEAST</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>160.77</v>
+        <v>0.87</v>
       </c>
       <c r="C92" t="n">
-        <v>160.77</v>
+        <v>0.87</v>
       </c>
       <c r="D92" t="n">
         <v>0</v>
@@ -2813,24 +2813,24 @@
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>158.01</v>
+        <v>0.86</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>-1.72</v>
+        <v>-1.15</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LPDC</t>
+          <t>FMNL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>6.08</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C93" t="n">
-        <v>6.08</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D93" t="n">
         <v>0</v>
@@ -2839,24 +2839,24 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>6.06</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>-0.33</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>UNIDT</t>
+          <t>PRAKASHSTL</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>174.67</v>
+        <v>4.37</v>
       </c>
       <c r="C94" t="n">
-        <v>174.67</v>
+        <v>4.37</v>
       </c>
       <c r="D94" t="n">
         <v>0</v>
@@ -2865,24 +2865,24 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>172.56</v>
+        <v>4.18</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>-1.21</v>
+        <v>-4.35</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SAHANA</t>
+          <t>ARCHIES</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1008.85</v>
+        <v>15.82</v>
       </c>
       <c r="C95" t="n">
-        <v>1008.85</v>
+        <v>15.82</v>
       </c>
       <c r="D95" t="n">
         <v>0</v>
@@ -2891,24 +2891,24 @@
         <v>0</v>
       </c>
       <c r="F95" t="n">
-        <v>992</v>
+        <v>15.03</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>-1.67</v>
+        <v>-4.99</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>UNIDT</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>522.4</v>
+        <v>174.67</v>
       </c>
       <c r="C96" t="n">
-        <v>522.4</v>
+        <v>174.67</v>
       </c>
       <c r="D96" t="n">
         <v>0</v>
@@ -2917,24 +2917,24 @@
         <v>0</v>
       </c>
       <c r="F96" t="n">
-        <v>521.85</v>
+        <v>171.99</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="n">
-        <v>-0.11</v>
+        <v>-1.53</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SAFARI</t>
+          <t>SAHANA</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1797.2</v>
+        <v>1008.85</v>
       </c>
       <c r="C97" t="n">
-        <v>1797.2</v>
+        <v>1008.85</v>
       </c>
       <c r="D97" t="n">
         <v>0</v>
@@ -2943,24 +2943,24 @@
         <v>0</v>
       </c>
       <c r="F97" t="n">
-        <v>1781.5</v>
+        <v>1001</v>
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>-0.87</v>
+        <v>-0.78</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ISHAN</t>
+          <t>MYMUDRA</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.65</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="C98" t="n">
-        <v>0.65</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="D98" t="n">
         <v>0</v>
@@ -2969,24 +2969,24 @@
         <v>0</v>
       </c>
       <c r="F98" t="n">
-        <v>0.6</v>
+        <v>75</v>
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>-7.69</v>
+        <v>-2.72</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>TSFINV</t>
+          <t>GLOBALVECT</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>402.15</v>
+        <v>163.21</v>
       </c>
       <c r="C99" t="n">
-        <v>402.15</v>
+        <v>163.21</v>
       </c>
       <c r="D99" t="n">
         <v>0</v>
@@ -2995,24 +2995,24 @@
         <v>0</v>
       </c>
       <c r="F99" t="n">
-        <v>394.1</v>
+        <v>155.42</v>
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>-2</v>
+        <v>-4.77</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SHRIRAMPPS</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>79.34999999999999</v>
+        <v>1.66</v>
       </c>
       <c r="C100" t="n">
-        <v>79.34999999999999</v>
+        <v>1.66</v>
       </c>
       <c r="D100" t="n">
         <v>0</v>
@@ -3021,24 +3021,24 @@
         <v>0</v>
       </c>
       <c r="F100" t="n">
-        <v>78.2</v>
+        <v>1.72</v>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>-1.45</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>DELTAMAGNT</t>
+          <t>TSFINV</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>61.04</v>
+        <v>402.15</v>
       </c>
       <c r="C101" t="n">
-        <v>61.04</v>
+        <v>402.15</v>
       </c>
       <c r="D101" t="n">
         <v>0</v>
@@ -3047,24 +3047,24 @@
         <v>0</v>
       </c>
       <c r="F101" t="n">
-        <v>58.41</v>
+        <v>380.1</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>-4.31</v>
+        <v>-5.48</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>UNIINFO</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1</v>
+        <v>14.04</v>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>14.04</v>
       </c>
       <c r="D102" t="n">
         <v>0</v>
@@ -3073,24 +3073,24 @@
         <v>0</v>
       </c>
       <c r="F102" t="n">
-        <v>0.92</v>
+        <v>13.94</v>
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>-8</v>
+        <v>-0.71</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MADHUCON</t>
+          <t>RADAAN</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>4.73</v>
+        <v>3.12</v>
       </c>
       <c r="C103" t="n">
-        <v>4.73</v>
+        <v>3.12</v>
       </c>
       <c r="D103" t="n">
         <v>0</v>
@@ -3099,24 +3099,24 @@
         <v>0</v>
       </c>
       <c r="F103" t="n">
-        <v>4.63</v>
+        <v>3.05</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>-2.11</v>
+        <v>-2.24</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>FINBUD</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>28.67</v>
+        <v>105</v>
       </c>
       <c r="C104" t="n">
-        <v>28.67</v>
+        <v>105</v>
       </c>
       <c r="D104" t="n">
         <v>0</v>
@@ -3125,24 +3125,24 @@
         <v>0</v>
       </c>
       <c r="F104" t="n">
-        <v>27.4</v>
+        <v>100.6</v>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>-4.43</v>
+        <v>-4.19</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>5.68</v>
+        <v>7.79</v>
       </c>
       <c r="C105" t="n">
-        <v>5.68</v>
+        <v>7.79</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
@@ -3151,24 +3151,24 @@
         <v>0</v>
       </c>
       <c r="F105" t="n">
-        <v>5.59</v>
+        <v>7.41</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>-1.58</v>
+        <v>-4.88</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>LYPSAGEMS</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>5.74</v>
+        <v>5.22</v>
       </c>
       <c r="C106" t="n">
-        <v>5.74</v>
+        <v>5.22</v>
       </c>
       <c r="D106" t="n">
         <v>0</v>
@@ -3177,24 +3177,24 @@
         <v>0</v>
       </c>
       <c r="F106" t="n">
-        <v>5.57</v>
+        <v>5.1</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>-2.96</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>GOLDTECH</t>
+          <t>TRIGYN</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>39.8</v>
+        <v>52.11</v>
       </c>
       <c r="C107" t="n">
-        <v>39.8</v>
+        <v>52.11</v>
       </c>
       <c r="D107" t="n">
         <v>0</v>
@@ -3203,24 +3203,24 @@
         <v>0</v>
       </c>
       <c r="F107" t="n">
-        <v>39.53</v>
+        <v>51.25</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>-0.68</v>
+        <v>-1.65</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>OILCOUNTUB</t>
+          <t>AILIMITED</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>47.36</v>
+        <v>36.55</v>
       </c>
       <c r="C108" t="n">
-        <v>47.36</v>
+        <v>36.55</v>
       </c>
       <c r="D108" t="n">
         <v>0</v>
@@ -3229,24 +3229,24 @@
         <v>0</v>
       </c>
       <c r="F108" t="n">
-        <v>47.49</v>
+        <v>38.35</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="n">
-        <v>0.27</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>FMNL</t>
+          <t>ENSER</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>8.300000000000001</v>
+        <v>12</v>
       </c>
       <c r="C109" t="n">
-        <v>8.300000000000001</v>
+        <v>12</v>
       </c>
       <c r="D109" t="n">
         <v>0</v>
@@ -3255,24 +3255,24 @@
         <v>0</v>
       </c>
       <c r="F109" t="n">
-        <v>8.220000000000001</v>
+        <v>12</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="n">
-        <v>-0.96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.87</v>
+        <v>25.34</v>
       </c>
       <c r="C110" t="n">
-        <v>0.87</v>
+        <v>25.34</v>
       </c>
       <c r="D110" t="n">
         <v>0</v>
@@ -3281,24 +3281,24 @@
         <v>0</v>
       </c>
       <c r="F110" t="n">
-        <v>0.85</v>
+        <v>25.15</v>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>-2.3</v>
+        <v>-0.75</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>DICIND</t>
+          <t>GICL</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>526</v>
+        <v>48.4</v>
       </c>
       <c r="C111" t="n">
-        <v>526</v>
+        <v>48.4</v>
       </c>
       <c r="D111" t="n">
         <v>0</v>
@@ -3307,24 +3307,24 @@
         <v>0</v>
       </c>
       <c r="F111" t="n">
-        <v>540.05</v>
+        <v>47.8</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>2.67</v>
+        <v>-1.24</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>AFSL</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>201</v>
+        <v>7.57</v>
       </c>
       <c r="C112" t="n">
-        <v>201</v>
+        <v>7.57</v>
       </c>
       <c r="D112" t="n">
         <v>0</v>
@@ -3333,24 +3333,24 @@
         <v>0</v>
       </c>
       <c r="F112" t="n">
-        <v>201.49</v>
+        <v>7.2</v>
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>0.24</v>
+        <v>-4.89</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>LYPSAGEMS</t>
+          <t>SAHAJ</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>5.22</v>
+        <v>4.85</v>
       </c>
       <c r="C113" t="n">
-        <v>5.22</v>
+        <v>4.85</v>
       </c>
       <c r="D113" t="n">
         <v>0</v>
@@ -3359,24 +3359,24 @@
         <v>0</v>
       </c>
       <c r="F113" t="n">
-        <v>5.23</v>
+        <v>4.65</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>0.19</v>
+        <v>-4.12</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>UNIINFO</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>14.04</v>
+        <v>0.17</v>
       </c>
       <c r="C114" t="n">
-        <v>14.04</v>
+        <v>0.17</v>
       </c>
       <c r="D114" t="n">
         <v>0</v>
@@ -3385,24 +3385,24 @@
         <v>0</v>
       </c>
       <c r="F114" t="n">
-        <v>13.93</v>
+        <v>0.18</v>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>-0.78</v>
+        <v>5.88</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>1.66</v>
+        <v>522.4</v>
       </c>
       <c r="C115" t="n">
-        <v>1.66</v>
+        <v>522.4</v>
       </c>
       <c r="D115" t="n">
         <v>0</v>
@@ -3411,24 +3411,24 @@
         <v>0</v>
       </c>
       <c r="F115" t="n">
-        <v>1.63</v>
+        <v>513.25</v>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>-1.81</v>
+        <v>-1.75</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>HTMEDIA</t>
+          <t>SAFARI</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>21.82</v>
+        <v>1797.2</v>
       </c>
       <c r="C116" t="n">
-        <v>21.82</v>
+        <v>1797.2</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
@@ -3437,24 +3437,24 @@
         <v>0</v>
       </c>
       <c r="F116" t="n">
-        <v>21.47</v>
+        <v>1741.8</v>
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>-1.6</v>
+        <v>-3.08</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>GLOBALVECT</t>
+          <t>ISHAN</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>163.21</v>
+        <v>0.65</v>
       </c>
       <c r="C117" t="n">
-        <v>163.21</v>
+        <v>0.65</v>
       </c>
       <c r="D117" t="n">
         <v>0</v>
@@ -3463,24 +3463,24 @@
         <v>0</v>
       </c>
       <c r="F117" t="n">
-        <v>159.49</v>
+        <v>0.6</v>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>-2.28</v>
+        <v>-7.69</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>SHRIRAMPPS</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.22</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="C118" t="n">
-        <v>0.22</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="D118" t="n">
         <v>0</v>
@@ -3489,24 +3489,24 @@
         <v>0</v>
       </c>
       <c r="F118" t="n">
-        <v>0.22</v>
+        <v>78</v>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>0</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>DELTAMAGNT</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>1.01</v>
+        <v>61.04</v>
       </c>
       <c r="C119" t="n">
-        <v>1.01</v>
+        <v>61.04</v>
       </c>
       <c r="D119" t="n">
         <v>0</v>
@@ -3515,24 +3515,24 @@
         <v>0</v>
       </c>
       <c r="F119" t="n">
-        <v>0.99</v>
+        <v>57.98</v>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>-1.98</v>
+        <v>-5.01</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MARUSHIKA</t>
+          <t>PREMIER</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>103.15</v>
+        <v>2.99</v>
       </c>
       <c r="C120" t="n">
-        <v>103.15</v>
+        <v>2.99</v>
       </c>
       <c r="D120" t="n">
         <v>0</v>
@@ -3541,24 +3541,24 @@
         <v>0</v>
       </c>
       <c r="F120" t="n">
-        <v>101</v>
+        <v>2.87</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>-2.08</v>
+        <v>-4.01</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ONECAP-RE</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.2</v>
+        <v>1.01</v>
       </c>
       <c r="C121" t="n">
-        <v>0.2</v>
+        <v>1.01</v>
       </c>
       <c r="D121" t="n">
         <v>0</v>
@@ -3567,24 +3567,24 @@
         <v>0</v>
       </c>
       <c r="F121" t="n">
-        <v>0.18</v>
+        <v>0.99</v>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>-10</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TECHLABS</t>
+          <t>RELCHEMQ</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>195</v>
+        <v>122.33</v>
       </c>
       <c r="C122" t="n">
-        <v>195</v>
+        <v>122.33</v>
       </c>
       <c r="D122" t="n">
         <v>0</v>
@@ -3593,24 +3593,24 @@
         <v>0</v>
       </c>
       <c r="F122" t="n">
-        <v>203</v>
+        <v>118.03</v>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>4.1</v>
+        <v>-3.52</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SAHAJ</t>
+          <t>OBCL</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>4.85</v>
+        <v>55.99</v>
       </c>
       <c r="C123" t="n">
-        <v>4.85</v>
+        <v>55.99</v>
       </c>
       <c r="D123" t="n">
         <v>0</v>
@@ -3619,24 +3619,24 @@
         <v>0</v>
       </c>
       <c r="F123" t="n">
-        <v>4.85</v>
+        <v>55.07</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>0</v>
+        <v>-1.64</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>BANG</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>5.03</v>
+        <v>41.52</v>
       </c>
       <c r="C124" t="n">
-        <v>5.03</v>
+        <v>41.52</v>
       </c>
       <c r="D124" t="n">
         <v>0</v>
@@ -3645,24 +3645,24 @@
         <v>0</v>
       </c>
       <c r="F124" t="n">
-        <v>4.98</v>
+        <v>40.06</v>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>-0.99</v>
+        <v>-3.52</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>12.7</v>
+        <v>5.68</v>
       </c>
       <c r="C125" t="n">
-        <v>12.7</v>
+        <v>5.68</v>
       </c>
       <c r="D125" t="n">
         <v>0</v>
@@ -3671,24 +3671,24 @@
         <v>0</v>
       </c>
       <c r="F125" t="n">
-        <v>12.7</v>
+        <v>5.83</v>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>0</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>VINYLINDIA</t>
+          <t>AHLEAST</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>209.89</v>
+        <v>160.77</v>
       </c>
       <c r="C126" t="n">
-        <v>209.89</v>
+        <v>160.77</v>
       </c>
       <c r="D126" t="n">
         <v>0</v>
@@ -3697,24 +3697,24 @@
         <v>0</v>
       </c>
       <c r="F126" t="n">
-        <v>207.28</v>
+        <v>160.65</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>-1.24</v>
+        <v>-0.07000000000000001</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>BHADORA</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>64.45</v>
+        <v>6.08</v>
       </c>
       <c r="C127" t="n">
-        <v>64.45</v>
+        <v>6.08</v>
       </c>
       <c r="D127" t="n">
         <v>0</v>
@@ -3723,24 +3723,24 @@
         <v>0</v>
       </c>
       <c r="F127" t="n">
-        <v>63</v>
+        <v>5.83</v>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>-2.25</v>
+        <v>-4.11</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>ALLDIGI</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>7.57</v>
+        <v>823.55</v>
       </c>
       <c r="C128" t="n">
-        <v>7.57</v>
+        <v>823.55</v>
       </c>
       <c r="D128" t="n">
         <v>0</v>
@@ -3749,24 +3749,24 @@
         <v>0</v>
       </c>
       <c r="F128" t="n">
-        <v>7.26</v>
+        <v>803.05</v>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>-4.1</v>
+        <v>-2.49</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>GICL</t>
+          <t>AFSL</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>48.4</v>
+        <v>201</v>
       </c>
       <c r="C129" t="n">
-        <v>48.4</v>
+        <v>201</v>
       </c>
       <c r="D129" t="n">
         <v>0</v>
@@ -3775,24 +3775,24 @@
         <v>0</v>
       </c>
       <c r="F129" t="n">
-        <v>48.2</v>
+        <v>201</v>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>-0.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>OILCOUNTUB</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>25.34</v>
+        <v>47.36</v>
       </c>
       <c r="C130" t="n">
-        <v>25.34</v>
+        <v>47.36</v>
       </c>
       <c r="D130" t="n">
         <v>0</v>
@@ -3801,24 +3801,24 @@
         <v>0</v>
       </c>
       <c r="F130" t="n">
-        <v>24.52</v>
+        <v>47.8</v>
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>-3.24</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>0.17</v>
+        <v>5.74</v>
       </c>
       <c r="C131" t="n">
-        <v>0.17</v>
+        <v>5.74</v>
       </c>
       <c r="D131" t="n">
         <v>0</v>
@@ -3827,24 +3827,24 @@
         <v>0</v>
       </c>
       <c r="F131" t="n">
-        <v>0.18</v>
+        <v>5.73</v>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>5.88</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ENSER</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>12</v>
+        <v>4.73</v>
       </c>
       <c r="C132" t="n">
-        <v>12</v>
+        <v>4.73</v>
       </c>
       <c r="D132" t="n">
         <v>0</v>
@@ -3853,24 +3853,24 @@
         <v>0</v>
       </c>
       <c r="F132" t="n">
-        <v>12</v>
+        <v>4.5</v>
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>0</v>
+        <v>-4.86</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>7.79</v>
+        <v>28.67</v>
       </c>
       <c r="C133" t="n">
-        <v>7.79</v>
+        <v>28.67</v>
       </c>
       <c r="D133" t="n">
         <v>0</v>
@@ -3879,24 +3879,24 @@
         <v>0</v>
       </c>
       <c r="F133" t="n">
-        <v>7.56</v>
+        <v>27.77</v>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>-2.95</v>
+        <v>-3.14</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>FINBUD</t>
+          <t>MITTAL</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>105</v>
+        <v>1</v>
       </c>
       <c r="C134" t="n">
-        <v>105</v>
+        <v>1</v>
       </c>
       <c r="D134" t="n">
         <v>0</v>
@@ -3905,24 +3905,24 @@
         <v>0</v>
       </c>
       <c r="F134" t="n">
-        <v>110.9</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>5.62</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>TIL</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>4.1</v>
+        <v>208.98</v>
       </c>
       <c r="C135" t="n">
-        <v>4.1</v>
+        <v>208.98</v>
       </c>
       <c r="D135" t="n">
         <v>0</v>
@@ -3931,24 +3931,24 @@
         <v>0</v>
       </c>
       <c r="F135" t="n">
-        <v>4.02</v>
+        <v>213</v>
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="n">
-        <v>-1.95</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>MYMUDRA</t>
+          <t>DICIND</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>77.09999999999999</v>
+        <v>526</v>
       </c>
       <c r="C136" t="n">
-        <v>77.09999999999999</v>
+        <v>526</v>
       </c>
       <c r="D136" t="n">
         <v>0</v>
@@ -3957,11 +3957,11 @@
         <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>77.09999999999999</v>
+        <v>521.5</v>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>0</v>
+        <v>-0.86</v>
       </c>
     </row>
     <row r="137">
@@ -3983,24 +3983,24 @@
         <v>0</v>
       </c>
       <c r="F137" t="n">
-        <v>73.06999999999999</v>
+        <v>72.20999999999999</v>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="n">
-        <v>-3.15</v>
+        <v>-4.29</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>447.1</v>
+        <v>41.51</v>
       </c>
       <c r="C138" t="n">
-        <v>447</v>
+        <v>41.5</v>
       </c>
       <c r="D138" t="n">
         <v>-0.02</v>
@@ -4009,24 +4009,24 @@
         <v>0</v>
       </c>
       <c r="F138" t="n">
-        <v>435</v>
+        <v>38.32</v>
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="n">
-        <v>-2.68</v>
+        <v>-7.66</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>41.51</v>
+        <v>447.1</v>
       </c>
       <c r="C139" t="n">
-        <v>41.5</v>
+        <v>447</v>
       </c>
       <c r="D139" t="n">
         <v>-0.02</v>
@@ -4035,24 +4035,24 @@
         <v>0</v>
       </c>
       <c r="F139" t="n">
-        <v>40.05</v>
+        <v>428.35</v>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="n">
-        <v>-3.49</v>
+        <v>-4.17</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SMARTWORKS</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>410.05</v>
+        <v>1186.2</v>
       </c>
       <c r="C140" t="n">
-        <v>409.9</v>
+        <v>1185.7</v>
       </c>
       <c r="D140" t="n">
         <v>-0.04</v>
@@ -4061,24 +4061,24 @@
         <v>0</v>
       </c>
       <c r="F140" t="n">
-        <v>396.45</v>
+        <v>1158.9</v>
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="n">
-        <v>-3.28</v>
+        <v>-2.26</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>DPABHUSHAN</t>
+          <t>SMARTWORKS</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>1186.2</v>
+        <v>410.05</v>
       </c>
       <c r="C141" t="n">
-        <v>1185.7</v>
+        <v>409.9</v>
       </c>
       <c r="D141" t="n">
         <v>-0.04</v>
@@ -4087,24 +4087,24 @@
         <v>0</v>
       </c>
       <c r="F141" t="n">
-        <v>1158.6</v>
+        <v>395</v>
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="n">
-        <v>-2.29</v>
+        <v>-3.64</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CAPITALSFB</t>
+          <t>STANLEY</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>262.1</v>
+        <v>162.07</v>
       </c>
       <c r="C142" t="n">
-        <v>262</v>
+        <v>162</v>
       </c>
       <c r="D142" t="n">
         <v>-0.04</v>
@@ -4113,24 +4113,24 @@
         <v>0</v>
       </c>
       <c r="F142" t="n">
-        <v>262.8</v>
+        <v>155.8</v>
       </c>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="n">
-        <v>0.31</v>
+        <v>-3.83</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>STANLEY</t>
+          <t>CAPITALSFB</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>162.07</v>
+        <v>262.1</v>
       </c>
       <c r="C143" t="n">
-        <v>162</v>
+        <v>262</v>
       </c>
       <c r="D143" t="n">
         <v>-0.04</v>
@@ -4139,11 +4139,11 @@
         <v>0</v>
       </c>
       <c r="F143" t="n">
-        <v>158.2</v>
+        <v>258.55</v>
       </c>
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="n">
-        <v>-2.35</v>
+        <v>-1.32</v>
       </c>
     </row>
     <row r="144">
@@ -4165,11 +4165,11 @@
         <v>0</v>
       </c>
       <c r="F144" t="n">
-        <v>18.93</v>
+        <v>17.7</v>
       </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="n">
-        <v>-0.79</v>
+        <v>-7.23</v>
       </c>
     </row>
     <row r="145">
@@ -4191,24 +4191,24 @@
         <v>0</v>
       </c>
       <c r="F145" t="n">
-        <v>477.4</v>
+        <v>518</v>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="n">
-        <v>7.27</v>
+        <v>16.39</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>KRISHIVAL</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>12.58</v>
+        <v>313.25</v>
       </c>
       <c r="C146" t="n">
-        <v>12.57</v>
+        <v>313</v>
       </c>
       <c r="D146" t="n">
         <v>-0.08</v>
@@ -4217,24 +4217,24 @@
         <v>0</v>
       </c>
       <c r="F146" t="n">
-        <v>11.69</v>
+        <v>321.5</v>
       </c>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="n">
-        <v>-7</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>KRISHIVAL</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>313.25</v>
+        <v>12.58</v>
       </c>
       <c r="C147" t="n">
-        <v>313</v>
+        <v>12.57</v>
       </c>
       <c r="D147" t="n">
         <v>-0.08</v>
@@ -4243,11 +4243,11 @@
         <v>0</v>
       </c>
       <c r="F147" t="n">
-        <v>315</v>
+        <v>12</v>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="n">
-        <v>0.64</v>
+        <v>-4.53</v>
       </c>
     </row>
     <row r="148">
@@ -4269,11 +4269,11 @@
         <v>0</v>
       </c>
       <c r="F148" t="n">
-        <v>30</v>
+        <v>29.5</v>
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="n">
-        <v>1.69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149">
@@ -4295,11 +4295,11 @@
         <v>0</v>
       </c>
       <c r="F149" t="n">
-        <v>34.21</v>
+        <v>32.98</v>
       </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="n">
-        <v>-3.63</v>
+        <v>-7.1</v>
       </c>
     </row>
     <row r="150">
@@ -4321,11 +4321,11 @@
         <v>0</v>
       </c>
       <c r="F150" t="n">
-        <v>28</v>
+        <v>26.51</v>
       </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="n">
-        <v>1.27</v>
+        <v>-4.12</v>
       </c>
     </row>
     <row r="151">
@@ -4347,24 +4347,24 @@
         <v>0</v>
       </c>
       <c r="F151" t="n">
-        <v>543.95</v>
+        <v>516.55</v>
       </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="n">
-        <v>1.29</v>
+        <v>-3.81</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SHANTIGEAR</t>
+          <t>ANANTAM</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>450.1</v>
+        <v>102.53</v>
       </c>
       <c r="C152" t="n">
-        <v>449.5</v>
+        <v>102.4</v>
       </c>
       <c r="D152" t="n">
         <v>-0.13</v>
@@ -4373,24 +4373,24 @@
         <v>0</v>
       </c>
       <c r="F152" t="n">
-        <v>451.4</v>
+        <v>102.81</v>
       </c>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ANANTAM</t>
+          <t>BALAJITELE</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>102.53</v>
+        <v>108.14</v>
       </c>
       <c r="C153" t="n">
-        <v>102.4</v>
+        <v>108</v>
       </c>
       <c r="D153" t="n">
         <v>-0.13</v>
@@ -4399,24 +4399,24 @@
         <v>0</v>
       </c>
       <c r="F153" t="n">
-        <v>102.75</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="n">
-        <v>0.34</v>
+        <v>-8.890000000000001</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>BALAJITELE</t>
+          <t>SHANTIGEAR</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>108.14</v>
+        <v>450.1</v>
       </c>
       <c r="C154" t="n">
-        <v>108</v>
+        <v>449.5</v>
       </c>
       <c r="D154" t="n">
         <v>-0.13</v>
@@ -4425,11 +4425,11 @@
         <v>0</v>
       </c>
       <c r="F154" t="n">
-        <v>101.54</v>
+        <v>450.2</v>
       </c>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="n">
-        <v>-5.98</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="155">
@@ -4451,11 +4451,11 @@
         <v>0</v>
       </c>
       <c r="F155" t="n">
-        <v>13.54</v>
+        <v>13.6</v>
       </c>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="n">
-        <v>0.52</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="156">
@@ -4477,11 +4477,11 @@
         <v>0</v>
       </c>
       <c r="F156" t="n">
-        <v>4.75</v>
+        <v>4.54</v>
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="n">
-        <v>-2.06</v>
+        <v>-6.39</v>
       </c>
     </row>
     <row r="157">
@@ -4503,11 +4503,11 @@
         <v>0</v>
       </c>
       <c r="F157" t="n">
-        <v>4.58</v>
+        <v>4.39</v>
       </c>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="n">
-        <v>-0.65</v>
+        <v>-4.77</v>
       </c>
     </row>
     <row r="158">
@@ -4529,11 +4529,11 @@
         <v>0</v>
       </c>
       <c r="F158" t="n">
-        <v>270.6</v>
+        <v>279.55</v>
       </c>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="n">
-        <v>-4.72</v>
+        <v>-1.57</v>
       </c>
     </row>
     <row r="159">
@@ -4581,11 +4581,11 @@
         <v>0</v>
       </c>
       <c r="F160" t="n">
-        <v>716.9</v>
+        <v>657</v>
       </c>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="n">
-        <v>12.72</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="161">
@@ -4607,11 +4607,11 @@
         <v>0</v>
       </c>
       <c r="F161" t="n">
-        <v>536</v>
+        <v>525.1</v>
       </c>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="n">
-        <v>-2.44</v>
+        <v>-4.42</v>
       </c>
     </row>
     <row r="162">
@@ -4633,24 +4633,24 @@
         <v>0</v>
       </c>
       <c r="F162" t="n">
-        <v>159.31</v>
+        <v>160</v>
       </c>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SWARAJ</t>
+          <t>ELLEN</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>303.25</v>
+        <v>229.25</v>
       </c>
       <c r="C163" t="n">
-        <v>302.25</v>
+        <v>228.49</v>
       </c>
       <c r="D163" t="n">
         <v>-0.33</v>
@@ -4659,24 +4659,24 @@
         <v>0</v>
       </c>
       <c r="F163" t="n">
-        <v>301.6</v>
+        <v>225.85</v>
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="n">
-        <v>-0.22</v>
+        <v>-1.16</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>SUVIDHAA</t>
+          <t>SWARAJ</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>3</v>
+        <v>303.25</v>
       </c>
       <c r="C164" t="n">
-        <v>2.99</v>
+        <v>302.25</v>
       </c>
       <c r="D164" t="n">
         <v>-0.33</v>
@@ -4685,24 +4685,24 @@
         <v>0</v>
       </c>
       <c r="F164" t="n">
-        <v>2.97</v>
+        <v>302</v>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="n">
-        <v>-0.67</v>
+        <v>-0.08</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>ELLEN</t>
+          <t>SUVIDHAA</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>229.25</v>
+        <v>3</v>
       </c>
       <c r="C165" t="n">
-        <v>228.49</v>
+        <v>2.99</v>
       </c>
       <c r="D165" t="n">
         <v>-0.33</v>
@@ -4711,11 +4711,11 @@
         <v>0</v>
       </c>
       <c r="F165" t="n">
-        <v>226.62</v>
+        <v>2.93</v>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="n">
-        <v>-0.82</v>
+        <v>-2.01</v>
       </c>
     </row>
     <row r="166">
@@ -4737,11 +4737,11 @@
         <v>0</v>
       </c>
       <c r="F166" t="n">
-        <v>8.5</v>
+        <v>8.44</v>
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="n">
-        <v>-2.3</v>
+        <v>-2.99</v>
       </c>
     </row>
     <row r="167">
@@ -4763,11 +4763,11 @@
         <v>0</v>
       </c>
       <c r="F167" t="n">
-        <v>684.05</v>
+        <v>681.1</v>
       </c>
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="n">
-        <v>-2.43</v>
+        <v>-2.85</v>
       </c>
     </row>
     <row r="168">
@@ -4789,11 +4789,11 @@
         <v>0</v>
       </c>
       <c r="F168" t="n">
-        <v>116.99</v>
+        <v>115.9</v>
       </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="n">
-        <v>-2.51</v>
+        <v>-3.42</v>
       </c>
     </row>
     <row r="169">
@@ -4815,11 +4815,11 @@
         <v>0</v>
       </c>
       <c r="F169" t="n">
-        <v>80.75</v>
+        <v>79.23999999999999</v>
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="n">
-        <v>-1.52</v>
+        <v>-3.37</v>
       </c>
     </row>
     <row r="170">
@@ -4841,11 +4841,11 @@
         <v>0</v>
       </c>
       <c r="F170" t="n">
-        <v>124.75</v>
+        <v>126.98</v>
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="n">
-        <v>0.36</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="171">
@@ -4867,11 +4867,11 @@
         <v>0</v>
       </c>
       <c r="F171" t="n">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="n">
-        <v>-4.8</v>
+        <v>-6.6</v>
       </c>
     </row>
     <row r="172">
@@ -4893,11 +4893,11 @@
         <v>0</v>
       </c>
       <c r="F172" t="n">
-        <v>44.05</v>
+        <v>44</v>
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="n">
-        <v>-2.05</v>
+        <v>-2.16</v>
       </c>
     </row>
     <row r="173">
@@ -4919,11 +4919,11 @@
         <v>0</v>
       </c>
       <c r="F173" t="n">
-        <v>6.87</v>
+        <v>6.7</v>
       </c>
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="n">
-        <v>-1.15</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="174">
@@ -4945,24 +4945,24 @@
         <v>0</v>
       </c>
       <c r="F174" t="n">
-        <v>61.73</v>
+        <v>60.64</v>
       </c>
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-2.32</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>EDELWEISS</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>2037.2</v>
+        <v>114.42</v>
       </c>
       <c r="C175" t="n">
-        <v>2028</v>
+        <v>113.9</v>
       </c>
       <c r="D175" t="n">
         <v>-0.45</v>
@@ -4971,24 +4971,24 @@
         <v>0</v>
       </c>
       <c r="F175" t="n">
-        <v>2002.7</v>
+        <v>112.54</v>
       </c>
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="n">
-        <v>-1.25</v>
+        <v>-1.19</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>EDELWEISS</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>114.42</v>
+        <v>2037.2</v>
       </c>
       <c r="C176" t="n">
-        <v>113.9</v>
+        <v>2028</v>
       </c>
       <c r="D176" t="n">
         <v>-0.45</v>
@@ -4997,11 +4997,11 @@
         <v>0</v>
       </c>
       <c r="F176" t="n">
-        <v>114.35</v>
+        <v>2031.4</v>
       </c>
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="n">
-        <v>0.4</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="177">
@@ -5023,24 +5023,24 @@
         <v>0</v>
       </c>
       <c r="F177" t="n">
-        <v>25.3</v>
+        <v>25</v>
       </c>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="n">
-        <v>-2.69</v>
+        <v>-3.85</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>SELMC</t>
+          <t>MEDIASSIST</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>29.93</v>
+        <v>370.7</v>
       </c>
       <c r="C178" t="n">
-        <v>29.79</v>
+        <v>368.95</v>
       </c>
       <c r="D178" t="n">
         <v>-0.47</v>
@@ -5049,24 +5049,24 @@
         <v>0</v>
       </c>
       <c r="F178" t="n">
-        <v>29.45</v>
+        <v>361.9</v>
       </c>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
-        <v>-1.14</v>
+        <v>-1.91</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MEDIASSIST</t>
+          <t>SELMC</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>370.7</v>
+        <v>29.93</v>
       </c>
       <c r="C179" t="n">
-        <v>368.95</v>
+        <v>29.79</v>
       </c>
       <c r="D179" t="n">
         <v>-0.47</v>
@@ -5075,11 +5075,11 @@
         <v>0</v>
       </c>
       <c r="F179" t="n">
-        <v>358.1</v>
+        <v>28.5</v>
       </c>
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="n">
-        <v>-2.94</v>
+        <v>-4.33</v>
       </c>
     </row>
     <row r="180">
@@ -5101,24 +5101,24 @@
         <v>0</v>
       </c>
       <c r="F180" t="n">
-        <v>1491.9</v>
+        <v>1514</v>
       </c>
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="n">
-        <v>-0.55</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>HINDCOPPER</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>43.15</v>
+        <v>566.3</v>
       </c>
       <c r="C181" t="n">
-        <v>42.94</v>
+        <v>563.5</v>
       </c>
       <c r="D181" t="n">
         <v>-0.49</v>
@@ -5127,24 +5127,24 @@
         <v>0</v>
       </c>
       <c r="F181" t="n">
-        <v>42.21</v>
+        <v>576</v>
       </c>
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="n">
-        <v>-1.7</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>HINDCOPPER</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>566.3</v>
+        <v>43.15</v>
       </c>
       <c r="C182" t="n">
-        <v>563.5</v>
+        <v>42.94</v>
       </c>
       <c r="D182" t="n">
         <v>-0.49</v>
@@ -5153,11 +5153,11 @@
         <v>0</v>
       </c>
       <c r="F182" t="n">
-        <v>579.85</v>
+        <v>42.57</v>
       </c>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="n">
-        <v>2.9</v>
+        <v>-0.86</v>
       </c>
     </row>
     <row r="183">
@@ -5179,11 +5179,11 @@
         <v>0</v>
       </c>
       <c r="F183" t="n">
-        <v>135.5</v>
+        <v>131.08</v>
       </c>
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="n">
-        <v>-2.15</v>
+        <v>-5.34</v>
       </c>
     </row>
     <row r="184">
@@ -5205,11 +5205,11 @@
         <v>0</v>
       </c>
       <c r="F184" t="n">
-        <v>251.15</v>
+        <v>244</v>
       </c>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="n">
-        <v>-1.43</v>
+        <v>-4.24</v>
       </c>
     </row>
     <row r="185">
@@ -5231,11 +5231,11 @@
         <v>0</v>
       </c>
       <c r="F185" t="n">
-        <v>1276.4</v>
+        <v>1274</v>
       </c>
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="n">
-        <v>0.13</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="186">
@@ -5257,24 +5257,24 @@
         <v>0</v>
       </c>
       <c r="F186" t="n">
-        <v>3.76</v>
+        <v>3.61</v>
       </c>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="n">
-        <v>1.08</v>
+        <v>-2.96</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>ICDSLTD</t>
+          <t>UCAL</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>41.1</v>
+        <v>108.59</v>
       </c>
       <c r="C187" t="n">
-        <v>40.88</v>
+        <v>108</v>
       </c>
       <c r="D187" t="n">
         <v>-0.54</v>
@@ -5283,11 +5283,11 @@
         <v>0</v>
       </c>
       <c r="F187" t="n">
-        <v>40.5</v>
+        <v>101.99</v>
       </c>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="n">
-        <v>-0.93</v>
+        <v>-5.56</v>
       </c>
     </row>
     <row r="188">
@@ -5309,24 +5309,24 @@
         <v>0</v>
       </c>
       <c r="F188" t="n">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="n">
-        <v>-2.94</v>
+        <v>-0.14</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>UCAL</t>
+          <t>ICDSLTD</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>108.59</v>
+        <v>41.1</v>
       </c>
       <c r="C189" t="n">
-        <v>108</v>
+        <v>40.88</v>
       </c>
       <c r="D189" t="n">
         <v>-0.54</v>
@@ -5335,24 +5335,24 @@
         <v>0</v>
       </c>
       <c r="F189" t="n">
-        <v>106.73</v>
+        <v>39.05</v>
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="n">
-        <v>-1.18</v>
+        <v>-4.48</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>ICRA</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>5531</v>
+        <v>15.99</v>
       </c>
       <c r="C190" t="n">
-        <v>5500</v>
+        <v>15.9</v>
       </c>
       <c r="D190" t="n">
         <v>-0.5600000000000001</v>
@@ -5361,24 +5361,24 @@
         <v>0</v>
       </c>
       <c r="F190" t="n">
-        <v>5534.5</v>
+        <v>15.4</v>
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="n">
-        <v>0.63</v>
+        <v>-3.14</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>ICRA</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>15.99</v>
+        <v>5531</v>
       </c>
       <c r="C191" t="n">
-        <v>15.9</v>
+        <v>5500</v>
       </c>
       <c r="D191" t="n">
         <v>-0.5600000000000001</v>
@@ -5387,11 +5387,11 @@
         <v>0</v>
       </c>
       <c r="F191" t="n">
-        <v>16.39</v>
+        <v>5712.5</v>
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="n">
-        <v>3.08</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="192">
@@ -5413,24 +5413,24 @@
         <v>0</v>
       </c>
       <c r="F192" t="n">
-        <v>153.95</v>
+        <v>153.5</v>
       </c>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="n">
-        <v>-1.63</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>IRBINVIT</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>61.86</v>
+        <v>444.7</v>
       </c>
       <c r="C193" t="n">
-        <v>61.5</v>
+        <v>442.1</v>
       </c>
       <c r="D193" t="n">
         <v>-0.58</v>
@@ -5439,11 +5439,11 @@
         <v>0</v>
       </c>
       <c r="F193" t="n">
-        <v>61.67</v>
+        <v>454.15</v>
       </c>
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="n">
-        <v>0.28</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="194">
@@ -5465,24 +5465,24 @@
         <v>0</v>
       </c>
       <c r="F194" t="n">
-        <v>1000.9</v>
+        <v>999</v>
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="n">
-        <v>0.85</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>IRBINVIT</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>444.7</v>
+        <v>61.86</v>
       </c>
       <c r="C195" t="n">
-        <v>442.1</v>
+        <v>61.5</v>
       </c>
       <c r="D195" t="n">
         <v>-0.58</v>
@@ -5491,11 +5491,11 @@
         <v>0</v>
       </c>
       <c r="F195" t="n">
-        <v>453.75</v>
+        <v>61.38</v>
       </c>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="n">
-        <v>2.64</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="196">
@@ -5517,24 +5517,24 @@
         <v>0</v>
       </c>
       <c r="F196" t="n">
-        <v>16.1</v>
+        <v>16.3</v>
       </c>
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="n">
-        <v>-3.71</v>
+        <v>-2.51</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>FOODSIN</t>
+          <t>CAPINVIT</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>58.3</v>
+        <v>70</v>
       </c>
       <c r="C197" t="n">
-        <v>57.95</v>
+        <v>69.58</v>
       </c>
       <c r="D197" t="n">
         <v>-0.6</v>
@@ -5543,24 +5543,24 @@
         <v>0</v>
       </c>
       <c r="F197" t="n">
-        <v>57.26</v>
+        <v>69.8</v>
       </c>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="n">
-        <v>-1.19</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>CAPINVIT</t>
+          <t>FOODSIN</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>70</v>
+        <v>58.3</v>
       </c>
       <c r="C198" t="n">
-        <v>69.58</v>
+        <v>57.95</v>
       </c>
       <c r="D198" t="n">
         <v>-0.6</v>
@@ -5569,11 +5569,11 @@
         <v>0</v>
       </c>
       <c r="F198" t="n">
-        <v>69.59999999999999</v>
+        <v>57.23</v>
       </c>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="n">
-        <v>0.03</v>
+        <v>-1.24</v>
       </c>
     </row>
     <row r="199">
@@ -5595,11 +5595,11 @@
         <v>0</v>
       </c>
       <c r="F199" t="n">
-        <v>24.5</v>
+        <v>24.97</v>
       </c>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="n">
-        <v>-2.2</v>
+        <v>-0.32</v>
       </c>
     </row>
     <row r="200">
@@ -5621,24 +5621,24 @@
         <v>0</v>
       </c>
       <c r="F200" t="n">
-        <v>364.2</v>
+        <v>366.6</v>
       </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="n">
-        <v>5.57</v>
+        <v>6.26</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>SUNDROP</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>209.18</v>
+        <v>646.45</v>
       </c>
       <c r="C201" t="n">
-        <v>207.9</v>
+        <v>642.5</v>
       </c>
       <c r="D201" t="n">
         <v>-0.61</v>
@@ -5647,11 +5647,11 @@
         <v>0</v>
       </c>
       <c r="F201" t="n">
-        <v>199.01</v>
+        <v>632.2</v>
       </c>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="n">
-        <v>-4.28</v>
+        <v>-1.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-03-26 05:27 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -477,11 +477,11 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>15.89</v>
+        <v>14.65</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>-5.13</v>
+        <v>-12.54</v>
       </c>
     </row>
     <row r="3">
@@ -503,11 +503,11 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>33.74</v>
+        <v>34.5</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>-8.74</v>
+        <v>-6.68</v>
       </c>
     </row>
     <row r="4">
@@ -529,11 +529,11 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>705.45</v>
+        <v>720.9</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>6.89</v>
+        <v>9.23</v>
       </c>
     </row>
     <row r="5">
@@ -555,11 +555,11 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>4.7</v>
+        <v>4.61</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>-4.86</v>
+        <v>-6.68</v>
       </c>
     </row>
     <row r="6">
@@ -581,11 +581,11 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>11.86</v>
+        <v>11.74</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>-1.17</v>
+        <v>-2.17</v>
       </c>
     </row>
     <row r="7">
@@ -607,11 +607,11 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>22</v>
+        <v>22.9</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>-4.35</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="8">
@@ -633,11 +633,11 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>105.4</v>
+        <v>105.55</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>-6.73</v>
+        <v>-6.59</v>
       </c>
     </row>
     <row r="9">
@@ -659,11 +659,11 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>9.279999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>-0.22</v>
+        <v>-1.83</v>
       </c>
     </row>
     <row r="10">
@@ -685,11 +685,11 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>134.78</v>
+        <v>130.1</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>2.88</v>
+        <v>-0.6899999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -711,11 +711,11 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>2.74</v>
+        <v>2.61</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>1.48</v>
+        <v>-3.33</v>
       </c>
     </row>
     <row r="12">
@@ -737,11 +737,11 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>111.69</v>
+        <v>106.66</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>-2.88</v>
+        <v>-7.25</v>
       </c>
     </row>
     <row r="13">
@@ -763,11 +763,11 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>64.5</v>
+        <v>64.59</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="14">
@@ -789,11 +789,11 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>1.79</v>
+        <v>1.77</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>-2.19</v>
+        <v>-3.28</v>
       </c>
     </row>
     <row r="15">
@@ -815,11 +815,11 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>129.79</v>
+        <v>128.87</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>-2.56</v>
+        <v>-3.25</v>
       </c>
     </row>
     <row r="16">
@@ -841,11 +841,11 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>-5.88</v>
       </c>
     </row>
     <row r="17">
@@ -867,11 +867,11 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>54.95</v>
+        <v>59</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>-1.87</v>
+        <v>5.36</v>
       </c>
     </row>
     <row r="18">
@@ -893,11 +893,11 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>303.5</v>
+        <v>285</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>1.51</v>
+        <v>-4.68</v>
       </c>
     </row>
     <row r="19">
@@ -919,11 +919,11 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>65.94</v>
+        <v>66.3</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>-1.58</v>
+        <v>-1.04</v>
       </c>
     </row>
     <row r="20">
@@ -945,11 +945,11 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>54.01</v>
+        <v>52.1</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>-5.25</v>
+        <v>-8.6</v>
       </c>
     </row>
     <row r="21">
@@ -971,11 +971,11 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>19.14</v>
+        <v>18.39</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>-2.25</v>
+        <v>-6.08</v>
       </c>
     </row>
     <row r="22">
@@ -997,11 +997,11 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>41.27</v>
+        <v>41.02</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>-3.55</v>
+        <v>-4.14</v>
       </c>
     </row>
     <row r="23">
@@ -1023,11 +1023,11 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>34.76</v>
+        <v>34.46</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>-0.66</v>
+        <v>-1.51</v>
       </c>
     </row>
     <row r="24">
@@ -1049,11 +1049,11 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>23.23</v>
+        <v>22.5</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>-2.39</v>
+        <v>-5.46</v>
       </c>
     </row>
     <row r="25">
@@ -1075,11 +1075,11 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>285.55</v>
+        <v>288</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>2.72</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="26">
@@ -1101,11 +1101,11 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>3.69</v>
+        <v>3.48</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>-0.27</v>
+        <v>-5.95</v>
       </c>
     </row>
     <row r="27">
@@ -1127,11 +1127,11 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>4.73</v>
+        <v>4.58</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>-0.84</v>
+        <v>-3.98</v>
       </c>
     </row>
     <row r="28">
@@ -1153,24 +1153,24 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>38.8</v>
+        <v>38.06</v>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>-0.51</v>
+        <v>-2.41</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SETCO</t>
+          <t>SUNDARAM</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>17.2</v>
+        <v>1.2</v>
       </c>
       <c r="C29" t="n">
-        <v>18.06</v>
+        <v>1.26</v>
       </c>
       <c r="D29" t="n">
         <v>5</v>
@@ -1179,24 +1179,24 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>18.06</v>
+        <v>1.24</v>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>SETCO</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.2</v>
+        <v>17.2</v>
       </c>
       <c r="C30" t="n">
-        <v>1.26</v>
+        <v>18.06</v>
       </c>
       <c r="D30" t="n">
         <v>5</v>
@@ -1205,11 +1205,11 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>1.29</v>
+        <v>18.06</v>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>2.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1231,11 +1231,11 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>13.73</v>
+        <v>13.2</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>-1.08</v>
+        <v>-4.9</v>
       </c>
     </row>
     <row r="32">
@@ -1309,11 +1309,11 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>160</v>
+        <v>160.55</v>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>-0.31</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="35">
@@ -1335,11 +1335,11 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>60.35</v>
+        <v>60.38</v>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="36">
@@ -1361,11 +1361,11 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>27.1</v>
+        <v>27.42</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>-2.17</v>
+        <v>-1.01</v>
       </c>
     </row>
     <row r="37">
@@ -1387,11 +1387,11 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>26.79</v>
+        <v>27.69</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>-0.74</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="38">
@@ -1439,11 +1439,11 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>77.95</v>
+        <v>78.25</v>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>-2.44</v>
+        <v>-2.07</v>
       </c>
     </row>
     <row r="40">
@@ -1465,11 +1465,11 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>78.5</v>
+        <v>77.88</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>-2.36</v>
+        <v>-3.13</v>
       </c>
     </row>
     <row r="41">
@@ -1491,11 +1491,11 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>4.35</v>
+        <v>4.17</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>-2.9</v>
+        <v>-6.92</v>
       </c>
     </row>
     <row r="42">
@@ -1517,11 +1517,11 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>-1.84</v>
       </c>
     </row>
     <row r="43">
@@ -1543,11 +1543,11 @@
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>78.70999999999999</v>
+        <v>80.7</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>-1.37</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="44">
@@ -1569,11 +1569,11 @@
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>10.17</v>
+        <v>10.14</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>-1.26</v>
+        <v>-1.55</v>
       </c>
     </row>
     <row r="45">
@@ -1595,11 +1595,11 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>263.35</v>
+        <v>255</v>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>-2.43</v>
+        <v>-5.52</v>
       </c>
     </row>
     <row r="46">
@@ -1621,11 +1621,11 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>5.57</v>
+        <v>5.45</v>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>-3.8</v>
+        <v>-5.87</v>
       </c>
     </row>
     <row r="47">
@@ -1647,11 +1647,11 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>280.5</v>
+        <v>277.95</v>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>2.35</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="48">
@@ -1673,11 +1673,11 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>7.37</v>
+        <v>7.22</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>-1.73</v>
+        <v>-3.73</v>
       </c>
     </row>
     <row r="49">
@@ -1699,11 +1699,11 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>37.7</v>
+        <v>36.76</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>-1.82</v>
+        <v>-4.27</v>
       </c>
     </row>
     <row r="50">
@@ -1751,24 +1751,24 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>400</v>
+        <v>382.05</v>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>-1.48</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>HARRMALAYA</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2.77</v>
+        <v>165.15</v>
       </c>
       <c r="C52" t="n">
-        <v>2.89</v>
+        <v>172.3</v>
       </c>
       <c r="D52" t="n">
         <v>4.33</v>
@@ -1777,24 +1777,24 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>2.87</v>
+        <v>164.25</v>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-4.67</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>HARRMALAYA</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>165.15</v>
+        <v>2.77</v>
       </c>
       <c r="C53" t="n">
-        <v>172.3</v>
+        <v>2.89</v>
       </c>
       <c r="D53" t="n">
         <v>4.33</v>
@@ -1803,11 +1803,11 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>169.59</v>
+        <v>2.78</v>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>-1.57</v>
+        <v>-3.81</v>
       </c>
     </row>
     <row r="54">
@@ -1829,11 +1829,11 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>49.94</v>
+        <v>48.87</v>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>-2.99</v>
+        <v>-5.07</v>
       </c>
     </row>
     <row r="55">
@@ -1855,11 +1855,11 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>15.59</v>
+        <v>17.25</v>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>3.93</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56">
@@ -1881,11 +1881,11 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>39.8</v>
+        <v>40</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>-2.93</v>
+        <v>-2.44</v>
       </c>
     </row>
     <row r="57">
@@ -1907,11 +1907,11 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>11</v>
+        <v>11.25</v>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>-1.79</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="58">
@@ -1933,11 +1933,11 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>193.01</v>
+        <v>190.75</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>-1.48</v>
+        <v>-2.63</v>
       </c>
     </row>
     <row r="59">
@@ -1959,11 +1959,11 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>31.6</v>
+        <v>30.68</v>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>-4.82</v>
+        <v>-7.59</v>
       </c>
     </row>
     <row r="60">
@@ -1985,11 +1985,11 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>-0.62</v>
+        <v>-1.24</v>
       </c>
     </row>
     <row r="61">
@@ -2011,11 +2011,11 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>124.83</v>
+        <v>120.35</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>-2.25</v>
+        <v>-5.76</v>
       </c>
     </row>
     <row r="62">
@@ -2037,11 +2037,11 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>15.4</v>
+        <v>15</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="63">
@@ -2063,11 +2063,11 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>22.5</v>
+        <v>22.55</v>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>2.74</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="64">
@@ -2115,24 +2115,24 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>46.03</v>
+        <v>46.11</v>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>-4.9</v>
+        <v>-4.73</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>COMPINFO</t>
+          <t>SAMMAANCAP</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1.01</v>
+        <v>138.51</v>
       </c>
       <c r="C66" t="n">
-        <v>1.05</v>
+        <v>144</v>
       </c>
       <c r="D66" t="n">
         <v>3.96</v>
@@ -2141,24 +2141,24 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>0.97</v>
+        <v>146.3</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>-7.62</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SAMMAANCAP</t>
+          <t>COMPINFO</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>138.51</v>
+        <v>1.01</v>
       </c>
       <c r="C67" t="n">
-        <v>144</v>
+        <v>1.05</v>
       </c>
       <c r="D67" t="n">
         <v>3.96</v>
@@ -2167,11 +2167,11 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>154.5</v>
+        <v>1.01</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>7.29</v>
+        <v>-3.81</v>
       </c>
     </row>
     <row r="68">
@@ -2193,11 +2193,11 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>167.6</v>
+        <v>166</v>
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>0.48</v>
+        <v>-0.48</v>
       </c>
     </row>
     <row r="69">
@@ -2245,11 +2245,11 @@
         <v>0</v>
       </c>
       <c r="F70" t="n">
-        <v>53.89</v>
+        <v>50.98</v>
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>-3.34</v>
+        <v>-8.56</v>
       </c>
     </row>
     <row r="71">
@@ -2271,11 +2271,11 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>29.35</v>
+        <v>28.5</v>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>0.44</v>
+        <v>-2.46</v>
       </c>
     </row>
     <row r="72">
@@ -2323,24 +2323,24 @@
         <v>0</v>
       </c>
       <c r="F73" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>-2.41</v>
+        <v>-3.61</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SAMBHAAV</t>
+          <t>ASHIMASYN</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>5.47</v>
+        <v>12.83</v>
       </c>
       <c r="C74" t="n">
-        <v>5.67</v>
+        <v>13.3</v>
       </c>
       <c r="D74" t="n">
         <v>3.66</v>
@@ -2349,24 +2349,24 @@
         <v>0</v>
       </c>
       <c r="F74" t="n">
-        <v>5.35</v>
+        <v>12.66</v>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>-5.64</v>
+        <v>-4.81</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ASHIMASYN</t>
+          <t>SAMBHAAV</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>12.83</v>
+        <v>5.47</v>
       </c>
       <c r="C75" t="n">
-        <v>13.3</v>
+        <v>5.67</v>
       </c>
       <c r="D75" t="n">
         <v>3.66</v>
@@ -2375,11 +2375,11 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>13.18</v>
+        <v>5.57</v>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>-0.9</v>
+        <v>-1.76</v>
       </c>
     </row>
     <row r="76">
@@ -2401,24 +2401,24 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>6.08</v>
+        <v>5.93</v>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>1.84</v>
+        <v>-0.67</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>DONEAR</t>
+          <t>SAGILITY</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>83.02</v>
+        <v>37.32</v>
       </c>
       <c r="C77" t="n">
-        <v>86</v>
+        <v>38.66</v>
       </c>
       <c r="D77" t="n">
         <v>3.59</v>
@@ -2427,24 +2427,24 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>84.53</v>
+        <v>39.85</v>
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>-1.71</v>
+        <v>3.08</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SAGILITY</t>
+          <t>DONEAR</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>37.32</v>
+        <v>83.02</v>
       </c>
       <c r="C78" t="n">
-        <v>38.66</v>
+        <v>86</v>
       </c>
       <c r="D78" t="n">
         <v>3.59</v>
@@ -2453,11 +2453,11 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>39.67</v>
+        <v>84</v>
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>2.61</v>
+        <v>-2.33</v>
       </c>
     </row>
     <row r="79">
@@ -2479,11 +2479,11 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>23.72</v>
+        <v>23.5</v>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>-1.78</v>
+        <v>-2.69</v>
       </c>
     </row>
     <row r="80">
@@ -2505,11 +2505,11 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>790.4</v>
+        <v>788</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>4.23</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="81">
@@ -2531,11 +2531,11 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>6.78</v>
+        <v>6.87</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>0.44</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="82">
@@ -2557,11 +2557,11 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>41.43</v>
+        <v>39.92</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>-0.77</v>
+        <v>-4.38</v>
       </c>
     </row>
     <row r="83">
@@ -2583,11 +2583,11 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>91.44</v>
+        <v>88</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>1.05</v>
+        <v>-2.75</v>
       </c>
     </row>
     <row r="84">
@@ -2609,11 +2609,11 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>133.32</v>
+        <v>130</v>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>-3.38</v>
+        <v>-5.79</v>
       </c>
     </row>
     <row r="85">
@@ -2635,11 +2635,11 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>189.08</v>
+        <v>188.3</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>1.11</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="86">
@@ -2661,11 +2661,11 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>17.33</v>
+        <v>16.61</v>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>2.06</v>
+        <v>-2.18</v>
       </c>
     </row>
     <row r="87">
@@ -2687,11 +2687,11 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>4.32</v>
+        <v>4.2</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>3.1</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="88">
@@ -2713,11 +2713,11 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>97</v>
+        <v>91.92</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>-2.41</v>
+        <v>-7.53</v>
       </c>
     </row>
     <row r="89">
@@ -2739,11 +2739,11 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>182.03</v>
+        <v>181.19</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>-1.03</v>
+        <v>-1.48</v>
       </c>
     </row>
     <row r="90">
@@ -2765,11 +2765,11 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>13.22</v>
+        <v>12.35</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>-3.99</v>
+        <v>-10.31</v>
       </c>
     </row>
     <row r="91">
@@ -2791,11 +2791,11 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>72.59999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>-0.47</v>
+        <v>-2.11</v>
       </c>
     </row>
     <row r="92">
@@ -2817,11 +2817,11 @@
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>76.45</v>
+        <v>75</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>4.87</v>
+        <v>2.88</v>
       </c>
     </row>
     <row r="93">
@@ -2843,11 +2843,11 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>118.63</v>
+        <v>116.1</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>0.96</v>
+        <v>-1.19</v>
       </c>
     </row>
     <row r="94">
@@ -2869,11 +2869,11 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>128.54</v>
+        <v>128.2</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>2.83</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="95">
@@ -2895,11 +2895,11 @@
         <v>0</v>
       </c>
       <c r="F95" t="n">
-        <v>3.95</v>
+        <v>4</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>-2.95</v>
+        <v>-1.72</v>
       </c>
     </row>
     <row r="96">
@@ -2921,11 +2921,11 @@
         <v>0</v>
       </c>
       <c r="F96" t="n">
-        <v>396.75</v>
+        <v>389.75</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="n">
-        <v>0.47</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="97">
@@ -2947,11 +2947,11 @@
         <v>0</v>
       </c>
       <c r="F97" t="n">
-        <v>295.05</v>
+        <v>287</v>
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>1.74</v>
+        <v>-1.03</v>
       </c>
     </row>
     <row r="98">
@@ -2973,11 +2973,11 @@
         <v>0</v>
       </c>
       <c r="F98" t="n">
-        <v>44.98</v>
+        <v>44.1</v>
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>0.42</v>
+        <v>-1.54</v>
       </c>
     </row>
     <row r="99">
@@ -2999,11 +2999,11 @@
         <v>0</v>
       </c>
       <c r="F99" t="n">
-        <v>138.1</v>
+        <v>140.2</v>
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>-3.76</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="100">
@@ -3025,24 +3025,24 @@
         <v>0</v>
       </c>
       <c r="F100" t="n">
-        <v>103.3</v>
+        <v>101</v>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>1.98</v>
+        <v>-0.29</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>BVCL</t>
+          <t>HPAL</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>37.74</v>
+        <v>29.94</v>
       </c>
       <c r="C101" t="n">
-        <v>38.95</v>
+        <v>30.9</v>
       </c>
       <c r="D101" t="n">
         <v>3.21</v>
@@ -3051,24 +3051,24 @@
         <v>0</v>
       </c>
       <c r="F101" t="n">
-        <v>39.69</v>
+        <v>31.15</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>1.9</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HPAL</t>
+          <t>BVCL</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>29.94</v>
+        <v>37.74</v>
       </c>
       <c r="C102" t="n">
-        <v>30.9</v>
+        <v>38.95</v>
       </c>
       <c r="D102" t="n">
         <v>3.21</v>
@@ -3077,11 +3077,11 @@
         <v>0</v>
       </c>
       <c r="F102" t="n">
-        <v>31.67</v>
+        <v>39</v>
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>2.49</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="103">
@@ -3103,11 +3103,11 @@
         <v>0</v>
       </c>
       <c r="F103" t="n">
-        <v>443</v>
+        <v>433.5</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>0.68</v>
+        <v>-1.48</v>
       </c>
     </row>
     <row r="104">
@@ -3129,11 +3129,11 @@
         <v>0</v>
       </c>
       <c r="F104" t="n">
-        <v>4.12</v>
+        <v>4.19</v>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>-3.51</v>
+        <v>-1.87</v>
       </c>
     </row>
     <row r="105">
@@ -3165,14 +3165,14 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>FRESHARA</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>172.55</v>
+        <v>0.32</v>
       </c>
       <c r="C106" t="n">
-        <v>177.95</v>
+        <v>0.33</v>
       </c>
       <c r="D106" t="n">
         <v>3.13</v>
@@ -3181,24 +3181,24 @@
         <v>0</v>
       </c>
       <c r="F106" t="n">
-        <v>170.05</v>
+        <v>0.33</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>-4.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>FRESHARA</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.32</v>
+        <v>172.55</v>
       </c>
       <c r="C107" t="n">
-        <v>0.33</v>
+        <v>177.95</v>
       </c>
       <c r="D107" t="n">
         <v>3.13</v>
@@ -3207,24 +3207,24 @@
         <v>0</v>
       </c>
       <c r="F107" t="n">
-        <v>0.32</v>
+        <v>181</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>-3.03</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>NOVAAGRI</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>8.970000000000001</v>
+        <v>21.14</v>
       </c>
       <c r="C108" t="n">
-        <v>9.25</v>
+        <v>21.8</v>
       </c>
       <c r="D108" t="n">
         <v>3.12</v>
@@ -3233,24 +3233,24 @@
         <v>0</v>
       </c>
       <c r="F108" t="n">
-        <v>9.199999999999999</v>
+        <v>21.6</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="n">
-        <v>-0.54</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>NOVAAGRI</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>21.14</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="C109" t="n">
-        <v>21.8</v>
+        <v>9.25</v>
       </c>
       <c r="D109" t="n">
         <v>3.12</v>
@@ -3259,11 +3259,11 @@
         <v>0</v>
       </c>
       <c r="F109" t="n">
-        <v>22.94</v>
+        <v>9.19</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="n">
-        <v>5.23</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="110">
@@ -3285,11 +3285,11 @@
         <v>0</v>
       </c>
       <c r="F110" t="n">
-        <v>27.45</v>
+        <v>26.46</v>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>2.5</v>
+        <v>-1.19</v>
       </c>
     </row>
     <row r="111">
@@ -3311,11 +3311,11 @@
         <v>0</v>
       </c>
       <c r="F111" t="n">
-        <v>10.78</v>
+        <v>10.24</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>0.28</v>
+        <v>-4.74</v>
       </c>
     </row>
     <row r="112">
@@ -3337,11 +3337,11 @@
         <v>0</v>
       </c>
       <c r="F112" t="n">
-        <v>105.49</v>
+        <v>103.08</v>
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>-1.41</v>
+        <v>-3.66</v>
       </c>
     </row>
     <row r="113">
@@ -3363,11 +3363,11 @@
         <v>0</v>
       </c>
       <c r="F113" t="n">
-        <v>55.51</v>
+        <v>53.81</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>-0.52</v>
+        <v>-3.57</v>
       </c>
     </row>
     <row r="114">
@@ -3389,24 +3389,24 @@
         <v>0</v>
       </c>
       <c r="F114" t="n">
-        <v>400.25</v>
+        <v>389</v>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>14.37</v>
+        <v>11.16</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SUNTV</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>616.3</v>
+        <v>4.62</v>
       </c>
       <c r="C115" t="n">
-        <v>634.95</v>
+        <v>4.76</v>
       </c>
       <c r="D115" t="n">
         <v>3.03</v>
@@ -3415,11 +3415,11 @@
         <v>0</v>
       </c>
       <c r="F115" t="n">
-        <v>622.5</v>
+        <v>4.82</v>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>-1.96</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="116">
@@ -3451,14 +3451,14 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>SUNTV</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>4.62</v>
+        <v>616.3</v>
       </c>
       <c r="C117" t="n">
-        <v>4.76</v>
+        <v>634.95</v>
       </c>
       <c r="D117" t="n">
         <v>3.03</v>
@@ -3467,11 +3467,11 @@
         <v>0</v>
       </c>
       <c r="F117" t="n">
-        <v>4.82</v>
+        <v>603.75</v>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>1.26</v>
+        <v>-4.91</v>
       </c>
     </row>
     <row r="118">
@@ -3493,11 +3493,11 @@
         <v>0</v>
       </c>
       <c r="F118" t="n">
-        <v>284.5</v>
+        <v>283</v>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>-1.9</v>
+        <v>-2.41</v>
       </c>
     </row>
     <row r="119">
@@ -3519,11 +3519,11 @@
         <v>0</v>
       </c>
       <c r="F119" t="n">
-        <v>124.77</v>
+        <v>122</v>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>2.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -3545,11 +3545,11 @@
         <v>0</v>
       </c>
       <c r="F120" t="n">
-        <v>51.12</v>
+        <v>50</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>-1.41</v>
+        <v>-3.57</v>
       </c>
     </row>
     <row r="121">
@@ -3571,11 +3571,11 @@
         <v>0</v>
       </c>
       <c r="F121" t="n">
-        <v>3.81</v>
+        <v>3.73</v>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>-0.26</v>
+        <v>-2.36</v>
       </c>
     </row>
     <row r="122">
@@ -3597,11 +3597,11 @@
         <v>0</v>
       </c>
       <c r="F122" t="n">
-        <v>746</v>
+        <v>733.9</v>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>-0.21</v>
+        <v>-1.83</v>
       </c>
     </row>
     <row r="123">
@@ -3623,11 +3623,11 @@
         <v>0</v>
       </c>
       <c r="F123" t="n">
-        <v>142.9</v>
+        <v>140.5</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>-0.63</v>
+        <v>-2.29</v>
       </c>
     </row>
     <row r="124">
@@ -3649,11 +3649,11 @@
         <v>0</v>
       </c>
       <c r="F124" t="n">
-        <v>437.6</v>
+        <v>402</v>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>0.85</v>
+        <v>-7.35</v>
       </c>
     </row>
     <row r="125">
@@ -3675,11 +3675,11 @@
         <v>0</v>
       </c>
       <c r="F125" t="n">
-        <v>135.38</v>
+        <v>135</v>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>2.92</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="126">
@@ -3701,11 +3701,11 @@
         <v>0</v>
       </c>
       <c r="F126" t="n">
-        <v>60.3</v>
+        <v>58.4</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>-1.95</v>
+        <v>-5.04</v>
       </c>
     </row>
     <row r="127">
@@ -3727,11 +3727,11 @@
         <v>0</v>
       </c>
       <c r="F127" t="n">
-        <v>182.5</v>
+        <v>180.9</v>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>0.33</v>
+        <v>-0.55</v>
       </c>
     </row>
     <row r="128">
@@ -3753,24 +3753,24 @@
         <v>0</v>
       </c>
       <c r="F128" t="n">
-        <v>8.9</v>
+        <v>8.81</v>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>-1.11</v>
+        <v>-2.11</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>HARSHA</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>333.15</v>
+        <v>93.83</v>
       </c>
       <c r="C129" t="n">
-        <v>342.65</v>
+        <v>96.5</v>
       </c>
       <c r="D129" t="n">
         <v>2.85</v>
@@ -3779,24 +3779,24 @@
         <v>0</v>
       </c>
       <c r="F129" t="n">
-        <v>342.6</v>
+        <v>95.8</v>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>-0.01</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>HARSHA</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>93.83</v>
+        <v>333.15</v>
       </c>
       <c r="C130" t="n">
-        <v>96.5</v>
+        <v>342.65</v>
       </c>
       <c r="D130" t="n">
         <v>2.85</v>
@@ -3805,11 +3805,11 @@
         <v>0</v>
       </c>
       <c r="F130" t="n">
-        <v>96.15000000000001</v>
+        <v>333.05</v>
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>-0.36</v>
+        <v>-2.8</v>
       </c>
     </row>
     <row r="131">
@@ -3831,11 +3831,11 @@
         <v>0</v>
       </c>
       <c r="F131" t="n">
-        <v>63.83</v>
+        <v>63.18</v>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>-1.5</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="132">
@@ -3857,24 +3857,24 @@
         <v>0</v>
       </c>
       <c r="F132" t="n">
-        <v>513.8</v>
+        <v>518.7</v>
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>0.55</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SOUTHWEST</t>
+          <t>TERASOFT</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>211.84</v>
+        <v>302.2</v>
       </c>
       <c r="C133" t="n">
-        <v>217.8</v>
+        <v>310.7</v>
       </c>
       <c r="D133" t="n">
         <v>2.81</v>
@@ -3883,24 +3883,24 @@
         <v>0</v>
       </c>
       <c r="F133" t="n">
-        <v>217.52</v>
+        <v>313.55</v>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>-0.13</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>TERASOFT</t>
+          <t>SOUTHWEST</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>302.2</v>
+        <v>211.84</v>
       </c>
       <c r="C134" t="n">
-        <v>310.7</v>
+        <v>217.8</v>
       </c>
       <c r="D134" t="n">
         <v>2.81</v>
@@ -3909,11 +3909,11 @@
         <v>0</v>
       </c>
       <c r="F134" t="n">
-        <v>313.2</v>
+        <v>216.41</v>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>0.8</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="135">
@@ -3935,24 +3935,24 @@
         <v>0</v>
       </c>
       <c r="F135" t="n">
-        <v>360</v>
+        <v>352.65</v>
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="n">
-        <v>-2.7</v>
+        <v>-4.69</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>IBULLSLTD</t>
+          <t>CRIZAC</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>9.390000000000001</v>
+        <v>189.6</v>
       </c>
       <c r="C136" t="n">
-        <v>9.65</v>
+        <v>194.85</v>
       </c>
       <c r="D136" t="n">
         <v>2.77</v>
@@ -3961,24 +3961,24 @@
         <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>10.25</v>
+        <v>195.97</v>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>6.22</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>CRIZAC</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>189.6</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="C137" t="n">
-        <v>194.85</v>
+        <v>9.65</v>
       </c>
       <c r="D137" t="n">
         <v>2.77</v>
@@ -3987,24 +3987,24 @@
         <v>0</v>
       </c>
       <c r="F137" t="n">
-        <v>200.9</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="n">
-        <v>3.1</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>APEX</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>14.99</v>
+        <v>384.45</v>
       </c>
       <c r="C138" t="n">
-        <v>15.4</v>
+        <v>395</v>
       </c>
       <c r="D138" t="n">
         <v>2.74</v>
@@ -4013,24 +4013,24 @@
         <v>0</v>
       </c>
       <c r="F138" t="n">
-        <v>15.6</v>
+        <v>396</v>
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="n">
-        <v>1.3</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>APEX</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>384.45</v>
+        <v>14.99</v>
       </c>
       <c r="C139" t="n">
-        <v>395</v>
+        <v>15.4</v>
       </c>
       <c r="D139" t="n">
         <v>2.74</v>
@@ -4039,24 +4039,24 @@
         <v>0</v>
       </c>
       <c r="F139" t="n">
-        <v>393.5</v>
+        <v>15.42</v>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="n">
-        <v>-0.38</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>RPPL</t>
+          <t>MAXVOLT</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>15.09</v>
+        <v>288.55</v>
       </c>
       <c r="C140" t="n">
-        <v>15.5</v>
+        <v>296.4</v>
       </c>
       <c r="D140" t="n">
         <v>2.72</v>
@@ -4065,24 +4065,24 @@
         <v>0</v>
       </c>
       <c r="F140" t="n">
-        <v>15.51</v>
+        <v>302.5</v>
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="n">
-        <v>0.06</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>MAXVOLT</t>
+          <t>RPPL</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>288.55</v>
+        <v>15.09</v>
       </c>
       <c r="C141" t="n">
-        <v>296.4</v>
+        <v>15.5</v>
       </c>
       <c r="D141" t="n">
         <v>2.72</v>
@@ -4091,11 +4091,11 @@
         <v>0</v>
       </c>
       <c r="F141" t="n">
-        <v>302.95</v>
+        <v>15.5</v>
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="n">
-        <v>2.21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -4117,11 +4117,11 @@
         <v>0</v>
       </c>
       <c r="F142" t="n">
-        <v>17.21</v>
+        <v>17.25</v>
       </c>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="n">
-        <v>-1.49</v>
+        <v>-1.26</v>
       </c>
     </row>
     <row r="143">
@@ -4143,11 +4143,11 @@
         <v>0</v>
       </c>
       <c r="F143" t="n">
-        <v>38.1</v>
+        <v>38.8</v>
       </c>
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="n">
-        <v>-0.24</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="144">
@@ -4169,11 +4169,11 @@
         <v>0</v>
       </c>
       <c r="F144" t="n">
-        <v>895</v>
+        <v>861</v>
       </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="n">
-        <v>-3.22</v>
+        <v>-6.9</v>
       </c>
     </row>
     <row r="145">
@@ -4195,11 +4195,11 @@
         <v>0</v>
       </c>
       <c r="F145" t="n">
-        <v>51.11</v>
+        <v>50.47</v>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="n">
-        <v>3.25</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="146">
@@ -4221,11 +4221,11 @@
         <v>0</v>
       </c>
       <c r="F146" t="n">
-        <v>105.19</v>
+        <v>102</v>
       </c>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="n">
-        <v>0.28</v>
+        <v>-2.76</v>
       </c>
     </row>
     <row r="147">
@@ -4247,11 +4247,11 @@
         <v>0</v>
       </c>
       <c r="F147" t="n">
-        <v>525.35</v>
+        <v>516.1</v>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="n">
-        <v>2.01</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="148">
@@ -4273,11 +4273,11 @@
         <v>0</v>
       </c>
       <c r="F148" t="n">
-        <v>1741.15</v>
+        <v>1698.95</v>
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="n">
-        <v>2.42</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="149">
@@ -4299,11 +4299,11 @@
         <v>0</v>
       </c>
       <c r="F149" t="n">
-        <v>15.55</v>
+        <v>15.7</v>
       </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="n">
-        <v>-3.42</v>
+        <v>-2.48</v>
       </c>
     </row>
     <row r="150">
@@ -4325,11 +4325,11 @@
         <v>0</v>
       </c>
       <c r="F150" t="n">
-        <v>416.9</v>
+        <v>412</v>
       </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="n">
-        <v>0.46</v>
+        <v>-0.72</v>
       </c>
     </row>
     <row r="151">
@@ -4351,11 +4351,11 @@
         <v>0</v>
       </c>
       <c r="F151" t="n">
-        <v>13.33</v>
+        <v>13.02</v>
       </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="n">
-        <v>-0.82</v>
+        <v>-3.12</v>
       </c>
     </row>
     <row r="152">
@@ -4377,11 +4377,11 @@
         <v>0</v>
       </c>
       <c r="F152" t="n">
-        <v>1127.2</v>
+        <v>1112.8</v>
       </c>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="n">
-        <v>3.41</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="153">
@@ -4403,11 +4403,11 @@
         <v>0</v>
       </c>
       <c r="F153" t="n">
-        <v>3.9</v>
+        <v>4.05</v>
       </c>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="n">
-        <v>-1.52</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="154">
@@ -4429,11 +4429,11 @@
         <v>0</v>
       </c>
       <c r="F154" t="n">
-        <v>121.6</v>
+        <v>121.25</v>
       </c>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="n">
-        <v>0.62</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="155">
@@ -4455,11 +4455,11 @@
         <v>0</v>
       </c>
       <c r="F155" t="n">
-        <v>4.79</v>
+        <v>4.82</v>
       </c>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="n">
-        <v>0.42</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="156">
@@ -4481,11 +4481,11 @@
         <v>0</v>
       </c>
       <c r="F156" t="n">
-        <v>95.09</v>
+        <v>94.59</v>
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="n">
-        <v>0.16</v>
+        <v>-0.37</v>
       </c>
     </row>
     <row r="157">
@@ -4507,11 +4507,11 @@
         <v>0</v>
       </c>
       <c r="F157" t="n">
-        <v>1.24</v>
+        <v>1.15</v>
       </c>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="n">
-        <v>3.33</v>
+        <v>-4.17</v>
       </c>
     </row>
     <row r="158">
@@ -4533,11 +4533,11 @@
         <v>0</v>
       </c>
       <c r="F158" t="n">
-        <v>272</v>
+        <v>272.05</v>
       </c>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="159">
@@ -4585,24 +4585,24 @@
         <v>0</v>
       </c>
       <c r="F160" t="n">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="n">
-        <v>0</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ESSENTIA</t>
+          <t>ACCENTMIC</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>1.19</v>
+        <v>357.65</v>
       </c>
       <c r="C161" t="n">
-        <v>1.22</v>
+        <v>366.65</v>
       </c>
       <c r="D161" t="n">
         <v>2.52</v>
@@ -4611,24 +4611,24 @@
         <v>0</v>
       </c>
       <c r="F161" t="n">
-        <v>1.21</v>
+        <v>368.5</v>
       </c>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="n">
-        <v>-0.82</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>ACCENTMIC</t>
+          <t>ESSENTIA</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>357.65</v>
+        <v>1.19</v>
       </c>
       <c r="C162" t="n">
-        <v>366.65</v>
+        <v>1.22</v>
       </c>
       <c r="D162" t="n">
         <v>2.52</v>
@@ -4637,11 +4637,11 @@
         <v>0</v>
       </c>
       <c r="F162" t="n">
-        <v>366</v>
+        <v>1.21</v>
       </c>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="n">
-        <v>-0.18</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="163">
@@ -4663,24 +4663,24 @@
         <v>0</v>
       </c>
       <c r="F163" t="n">
-        <v>752</v>
+        <v>753.9</v>
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="n">
-        <v>0.4</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>UJJIVANSFB</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>51.34</v>
+        <v>866.25</v>
       </c>
       <c r="C164" t="n">
-        <v>52.63</v>
+        <v>888</v>
       </c>
       <c r="D164" t="n">
         <v>2.51</v>
@@ -4689,24 +4689,24 @@
         <v>0</v>
       </c>
       <c r="F164" t="n">
-        <v>53.92</v>
+        <v>872.25</v>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="n">
-        <v>2.45</v>
+        <v>-1.77</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>UJJIVANSFB</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>866.25</v>
+        <v>51.34</v>
       </c>
       <c r="C165" t="n">
-        <v>888</v>
+        <v>52.63</v>
       </c>
       <c r="D165" t="n">
         <v>2.51</v>
@@ -4715,11 +4715,11 @@
         <v>0</v>
       </c>
       <c r="F165" t="n">
-        <v>907.8</v>
+        <v>54.31</v>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="n">
-        <v>2.23</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="166">
@@ -4741,11 +4741,11 @@
         <v>0</v>
       </c>
       <c r="F166" t="n">
-        <v>0.41</v>
+        <v>0.39</v>
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="n">
-        <v>0</v>
+        <v>-4.88</v>
       </c>
     </row>
     <row r="167">
@@ -4767,24 +4767,24 @@
         <v>0</v>
       </c>
       <c r="F167" t="n">
-        <v>162.15</v>
+        <v>160</v>
       </c>
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="n">
-        <v>1.41</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>HIRECT</t>
+          <t>MANINDS</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>1512.6</v>
+        <v>336.7</v>
       </c>
       <c r="C168" t="n">
-        <v>1550</v>
+        <v>345</v>
       </c>
       <c r="D168" t="n">
         <v>2.47</v>
@@ -4793,24 +4793,24 @@
         <v>0</v>
       </c>
       <c r="F168" t="n">
-        <v>1591.8</v>
+        <v>346</v>
       </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="n">
-        <v>2.7</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>MANINDS</t>
+          <t>HIRECT</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>336.7</v>
+        <v>1512.6</v>
       </c>
       <c r="C169" t="n">
-        <v>345</v>
+        <v>1550</v>
       </c>
       <c r="D169" t="n">
         <v>2.47</v>
@@ -4819,24 +4819,24 @@
         <v>0</v>
       </c>
       <c r="F169" t="n">
-        <v>344.55</v>
+        <v>1588</v>
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="n">
-        <v>-0.13</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>NILAINFRA</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>6.92</v>
+        <v>4.87</v>
       </c>
       <c r="C170" t="n">
-        <v>7.09</v>
+        <v>4.99</v>
       </c>
       <c r="D170" t="n">
         <v>2.46</v>
@@ -4845,24 +4845,24 @@
         <v>0</v>
       </c>
       <c r="F170" t="n">
-        <v>7.08</v>
+        <v>4.96</v>
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="n">
-        <v>-0.14</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>ARIES</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>351.2</v>
+        <v>1.22</v>
       </c>
       <c r="C171" t="n">
-        <v>359.85</v>
+        <v>1.25</v>
       </c>
       <c r="D171" t="n">
         <v>2.46</v>
@@ -4871,24 +4871,24 @@
         <v>0</v>
       </c>
       <c r="F171" t="n">
-        <v>356.6</v>
+        <v>1.2</v>
       </c>
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="n">
-        <v>-0.9</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>ARIES</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>4.87</v>
+        <v>351.2</v>
       </c>
       <c r="C172" t="n">
-        <v>4.99</v>
+        <v>359.85</v>
       </c>
       <c r="D172" t="n">
         <v>2.46</v>
@@ -4897,11 +4897,11 @@
         <v>0</v>
       </c>
       <c r="F172" t="n">
-        <v>4.91</v>
+        <v>347.65</v>
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="n">
-        <v>-1.6</v>
+        <v>-3.39</v>
       </c>
     </row>
     <row r="173">
@@ -4923,24 +4923,24 @@
         <v>0</v>
       </c>
       <c r="F173" t="n">
-        <v>4.58</v>
+        <v>4.63</v>
       </c>
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="n">
-        <v>-0.22</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>NILAINFRA</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>1.22</v>
+        <v>6.92</v>
       </c>
       <c r="C174" t="n">
-        <v>1.25</v>
+        <v>7.09</v>
       </c>
       <c r="D174" t="n">
         <v>2.46</v>
@@ -4949,24 +4949,24 @@
         <v>0</v>
       </c>
       <c r="F174" t="n">
-        <v>1.24</v>
+        <v>6.9</v>
       </c>
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="n">
-        <v>-0.8</v>
+        <v>-2.68</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>SIL</t>
+          <t>AIRAN</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>13.17</v>
+        <v>14.79</v>
       </c>
       <c r="C175" t="n">
-        <v>13.49</v>
+        <v>15.15</v>
       </c>
       <c r="D175" t="n">
         <v>2.43</v>
@@ -4975,24 +4975,24 @@
         <v>0</v>
       </c>
       <c r="F175" t="n">
-        <v>13.68</v>
+        <v>14.71</v>
       </c>
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="n">
-        <v>1.41</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>BAJAJINDEF</t>
+          <t>HINDPETRO</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>228.34</v>
+        <v>336.8</v>
       </c>
       <c r="C176" t="n">
-        <v>233.89</v>
+        <v>345</v>
       </c>
       <c r="D176" t="n">
         <v>2.43</v>
@@ -5001,24 +5001,24 @@
         <v>0</v>
       </c>
       <c r="F176" t="n">
-        <v>234.24</v>
+        <v>345.3</v>
       </c>
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>AIRAN</t>
+          <t>BAJAJINDEF</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>14.79</v>
+        <v>228.34</v>
       </c>
       <c r="C177" t="n">
-        <v>15.15</v>
+        <v>233.89</v>
       </c>
       <c r="D177" t="n">
         <v>2.43</v>
@@ -5027,24 +5027,24 @@
         <v>0</v>
       </c>
       <c r="F177" t="n">
-        <v>15.1</v>
+        <v>229</v>
       </c>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="n">
-        <v>-0.33</v>
+        <v>-2.09</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>HINDPETRO</t>
+          <t>SIL</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>336.8</v>
+        <v>13.17</v>
       </c>
       <c r="C178" t="n">
-        <v>345</v>
+        <v>13.49</v>
       </c>
       <c r="D178" t="n">
         <v>2.43</v>
@@ -5053,24 +5053,24 @@
         <v>0</v>
       </c>
       <c r="F178" t="n">
-        <v>347</v>
+        <v>13.17</v>
       </c>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
-        <v>0.58</v>
+        <v>-2.37</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>SERVOTECH</t>
+          <t>IVP</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>68.05</v>
+        <v>132.2</v>
       </c>
       <c r="C179" t="n">
-        <v>69.7</v>
+        <v>135.4</v>
       </c>
       <c r="D179" t="n">
         <v>2.42</v>
@@ -5079,24 +5079,24 @@
         <v>0</v>
       </c>
       <c r="F179" t="n">
-        <v>71.31999999999999</v>
+        <v>128.9</v>
       </c>
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="n">
-        <v>2.32</v>
+        <v>-4.8</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>GAUDIUMIVF</t>
+          <t>SERVOTECH</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>78.09999999999999</v>
+        <v>68.05</v>
       </c>
       <c r="C180" t="n">
-        <v>79.98999999999999</v>
+        <v>69.7</v>
       </c>
       <c r="D180" t="n">
         <v>2.42</v>
@@ -5105,24 +5105,24 @@
         <v>0</v>
       </c>
       <c r="F180" t="n">
-        <v>80.86</v>
+        <v>70.7</v>
       </c>
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="n">
-        <v>1.09</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>IVP</t>
+          <t>GAUDIUMIVF</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>132.2</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="C181" t="n">
-        <v>135.4</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="D181" t="n">
         <v>2.42</v>
@@ -5131,24 +5131,24 @@
         <v>0</v>
       </c>
       <c r="F181" t="n">
-        <v>134.9</v>
+        <v>79</v>
       </c>
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="n">
-        <v>-0.37</v>
+        <v>-1.24</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>INFOBEAN</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>136.62</v>
+        <v>366.25</v>
       </c>
       <c r="C182" t="n">
-        <v>139.89</v>
+        <v>375</v>
       </c>
       <c r="D182" t="n">
         <v>2.39</v>
@@ -5157,24 +5157,24 @@
         <v>0</v>
       </c>
       <c r="F182" t="n">
-        <v>140.06</v>
+        <v>407.75</v>
       </c>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="n">
-        <v>0.12</v>
+        <v>8.73</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>INFOBEAN</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>366.25</v>
+        <v>136.62</v>
       </c>
       <c r="C183" t="n">
-        <v>375</v>
+        <v>139.89</v>
       </c>
       <c r="D183" t="n">
         <v>2.39</v>
@@ -5183,11 +5183,11 @@
         <v>0</v>
       </c>
       <c r="F183" t="n">
-        <v>385</v>
+        <v>137.93</v>
       </c>
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="n">
-        <v>2.67</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="184">
@@ -5209,11 +5209,11 @@
         <v>0</v>
       </c>
       <c r="F184" t="n">
-        <v>296.5</v>
+        <v>297</v>
       </c>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="n">
-        <v>1.94</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="185">
@@ -5235,11 +5235,11 @@
         <v>0</v>
       </c>
       <c r="F185" t="n">
-        <v>104.85</v>
+        <v>103.5</v>
       </c>
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="n">
-        <v>2.39</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="186">
@@ -5261,11 +5261,11 @@
         <v>0</v>
       </c>
       <c r="F186" t="n">
-        <v>17.13</v>
+        <v>16.1</v>
       </c>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="n">
-        <v>1.36</v>
+        <v>-4.73</v>
       </c>
     </row>
     <row r="187">
@@ -5287,11 +5287,11 @@
         <v>0</v>
       </c>
       <c r="F187" t="n">
-        <v>5.2</v>
+        <v>5.16</v>
       </c>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="n">
-        <v>-0.38</v>
+        <v>-1.15</v>
       </c>
     </row>
     <row r="188">
@@ -5313,24 +5313,24 @@
         <v>0</v>
       </c>
       <c r="F188" t="n">
-        <v>368.1</v>
+        <v>375.35</v>
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="n">
-        <v>2.53</v>
+        <v>4.55</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>KANANIIND</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>111.3</v>
+        <v>1.28</v>
       </c>
       <c r="C189" t="n">
-        <v>113.9</v>
+        <v>1.31</v>
       </c>
       <c r="D189" t="n">
         <v>2.34</v>
@@ -5339,24 +5339,24 @@
         <v>0</v>
       </c>
       <c r="F189" t="n">
-        <v>116.8</v>
+        <v>1.26</v>
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="n">
-        <v>2.55</v>
+        <v>-3.82</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>PARSVNATH</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>6.4</v>
+        <v>111.3</v>
       </c>
       <c r="C190" t="n">
-        <v>6.55</v>
+        <v>113.9</v>
       </c>
       <c r="D190" t="n">
         <v>2.34</v>
@@ -5365,24 +5365,24 @@
         <v>0</v>
       </c>
       <c r="F190" t="n">
-        <v>6.65</v>
+        <v>115</v>
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="n">
-        <v>1.53</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>KANANIIND</t>
+          <t>PARSVNATH</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>1.28</v>
+        <v>6.4</v>
       </c>
       <c r="C191" t="n">
-        <v>1.31</v>
+        <v>6.55</v>
       </c>
       <c r="D191" t="n">
         <v>2.34</v>
@@ -5391,11 +5391,11 @@
         <v>0</v>
       </c>
       <c r="F191" t="n">
-        <v>1.29</v>
+        <v>6.71</v>
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="n">
-        <v>-1.53</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="192">
@@ -5417,11 +5417,11 @@
         <v>0</v>
       </c>
       <c r="F192" t="n">
-        <v>23.67</v>
+        <v>23.12</v>
       </c>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="n">
-        <v>1.07</v>
+        <v>-1.28</v>
       </c>
     </row>
     <row r="193">
@@ -5443,24 +5443,24 @@
         <v>0</v>
       </c>
       <c r="F193" t="n">
-        <v>16.9</v>
+        <v>16.84</v>
       </c>
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="n">
-        <v>-1.97</v>
+        <v>-2.32</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>SWIGGY</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>885.5</v>
+        <v>275.75</v>
       </c>
       <c r="C194" t="n">
-        <v>905.9</v>
+        <v>282.1</v>
       </c>
       <c r="D194" t="n">
         <v>2.3</v>
@@ -5469,24 +5469,24 @@
         <v>0</v>
       </c>
       <c r="F194" t="n">
-        <v>913</v>
+        <v>276.5</v>
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="n">
-        <v>0.78</v>
+        <v>-1.99</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>MAXESTATES</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>352.45</v>
+        <v>885.5</v>
       </c>
       <c r="C195" t="n">
-        <v>360.55</v>
+        <v>905.9</v>
       </c>
       <c r="D195" t="n">
         <v>2.3</v>
@@ -5495,11 +5495,11 @@
         <v>0</v>
       </c>
       <c r="F195" t="n">
-        <v>356.8</v>
+        <v>890</v>
       </c>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="n">
-        <v>-1.04</v>
+        <v>-1.76</v>
       </c>
     </row>
     <row r="196">
@@ -5521,24 +5521,24 @@
         <v>0</v>
       </c>
       <c r="F196" t="n">
-        <v>1638.8</v>
+        <v>1629</v>
       </c>
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="n">
-        <v>2.62</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>SWIGGY</t>
+          <t>MAXESTATES</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>275.75</v>
+        <v>352.45</v>
       </c>
       <c r="C197" t="n">
-        <v>282.1</v>
+        <v>360.55</v>
       </c>
       <c r="D197" t="n">
         <v>2.3</v>
@@ -5547,24 +5547,24 @@
         <v>0</v>
       </c>
       <c r="F197" t="n">
-        <v>279.7</v>
+        <v>355</v>
       </c>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="n">
-        <v>-0.85</v>
+        <v>-1.54</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>APCL</t>
+          <t>EMAMIPAP</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>108.7</v>
+        <v>64.42</v>
       </c>
       <c r="C198" t="n">
-        <v>111.2</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="D198" t="n">
         <v>2.3</v>
@@ -5573,24 +5573,24 @@
         <v>0</v>
       </c>
       <c r="F198" t="n">
-        <v>112.94</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="n">
-        <v>1.56</v>
+        <v>-1.38</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>EMAMIPAP</t>
+          <t>APCL</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>64.42</v>
+        <v>108.7</v>
       </c>
       <c r="C199" t="n">
-        <v>65.90000000000001</v>
+        <v>111.2</v>
       </c>
       <c r="D199" t="n">
         <v>2.3</v>
@@ -5599,24 +5599,24 @@
         <v>0</v>
       </c>
       <c r="F199" t="n">
-        <v>65.90000000000001</v>
+        <v>108</v>
       </c>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="n">
-        <v>0</v>
+        <v>-2.88</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>TGBHOTELS</t>
+          <t>CONCOR</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>8.31</v>
+        <v>433.1</v>
       </c>
       <c r="C200" t="n">
-        <v>8.5</v>
+        <v>443</v>
       </c>
       <c r="D200" t="n">
         <v>2.29</v>
@@ -5625,24 +5625,24 @@
         <v>0</v>
       </c>
       <c r="F200" t="n">
-        <v>8.25</v>
+        <v>445</v>
       </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="n">
-        <v>-2.94</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>CONCOR</t>
+          <t>INDOWIND</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>433.1</v>
+        <v>8.31</v>
       </c>
       <c r="C201" t="n">
-        <v>443</v>
+        <v>8.5</v>
       </c>
       <c r="D201" t="n">
         <v>2.29</v>
@@ -5651,11 +5651,11 @@
         <v>0</v>
       </c>
       <c r="F201" t="n">
-        <v>448.2</v>
+        <v>8.43</v>
       </c>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="n">
-        <v>1.17</v>
+        <v>-0.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-03-31 05:31 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -477,11 +477,11 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>1.91</v>
+        <v>2</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>-49.6</v>
+        <v>-47.23</v>
       </c>
     </row>
     <row r="3">
@@ -503,11 +503,11 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>3.63</v>
+        <v>3.6</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>-16.17</v>
+        <v>-16.86</v>
       </c>
     </row>
     <row r="4">
@@ -529,11 +529,11 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>17.49</v>
+        <v>16.2</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>-2.83</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="5">
@@ -555,11 +555,11 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>200.48</v>
+        <v>205</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>-8.039999999999999</v>
+        <v>-5.96</v>
       </c>
     </row>
     <row r="6">
@@ -581,11 +581,11 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>-15.52</v>
+        <v>-12.35</v>
       </c>
     </row>
     <row r="7">
@@ -607,11 +607,11 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>32.86</v>
+        <v>29.79</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>-5.28</v>
+        <v>-14.13</v>
       </c>
     </row>
     <row r="8">
@@ -659,11 +659,11 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>75</v>
+        <v>72.59</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>-3.83</v>
+        <v>-6.92</v>
       </c>
     </row>
     <row r="10">
@@ -685,11 +685,11 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>29.32</v>
+        <v>29.5</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>-5.39</v>
+        <v>-4.81</v>
       </c>
     </row>
     <row r="11">
@@ -711,11 +711,11 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>11.88</v>
+        <v>11.5</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>-11.28</v>
+        <v>-14.12</v>
       </c>
     </row>
     <row r="12">
@@ -737,11 +737,11 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>37</v>
+        <v>38.94</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>-7.45</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="13">
@@ -763,11 +763,11 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>24.75</v>
+        <v>22.05</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>2.91</v>
+        <v>-8.32</v>
       </c>
     </row>
     <row r="14">
@@ -789,11 +789,11 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>217.42</v>
+        <v>210</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>-7.48</v>
+        <v>-10.64</v>
       </c>
     </row>
     <row r="15">
@@ -841,11 +841,11 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>102.98</v>
+        <v>104.8</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>-3.17</v>
+        <v>-1.46</v>
       </c>
     </row>
     <row r="17">
@@ -867,11 +867,11 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>3.2</v>
+        <v>3.15</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>-8.31</v>
+        <v>-9.74</v>
       </c>
     </row>
     <row r="18">
@@ -893,11 +893,11 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>5.59</v>
+        <v>5.55</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>-12.66</v>
+        <v>-13.28</v>
       </c>
     </row>
     <row r="19">
@@ -919,11 +919,11 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>24.38</v>
+        <v>24.84</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>10.77</v>
+        <v>12.86</v>
       </c>
     </row>
     <row r="20">
@@ -945,11 +945,11 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>3.03</v>
+        <v>2.96</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>-5.31</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="21">
@@ -971,11 +971,11 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>22.8</v>
+        <v>21.2</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>-2.81</v>
+        <v>-9.630000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -997,11 +997,11 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>10.62</v>
+        <v>10.74</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>-7.65</v>
+        <v>-6.61</v>
       </c>
     </row>
     <row r="23">
@@ -1023,11 +1023,11 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>19.5</v>
+        <v>19.9</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>-2.5</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="24">
@@ -1049,11 +1049,11 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>-3.48</v>
+        <v>-4.55</v>
       </c>
     </row>
     <row r="25">
@@ -1075,11 +1075,11 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>87.06999999999999</v>
+        <v>83.01000000000001</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>-2.28</v>
+        <v>-6.84</v>
       </c>
     </row>
     <row r="26">
@@ -1101,11 +1101,11 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>109.9</v>
+        <v>105.17</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>-8.42</v>
+        <v>-12.36</v>
       </c>
     </row>
     <row r="27">
@@ -1127,11 +1127,11 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>235</v>
+        <v>218</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>-5.62</v>
+        <v>-12.45</v>
       </c>
     </row>
     <row r="28">
@@ -1153,11 +1153,11 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>90</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>-5.06</v>
+        <v>-3.59</v>
       </c>
     </row>
     <row r="29">
@@ -1179,11 +1179,11 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>2.49</v>
+        <v>2.35</v>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>-7.78</v>
+        <v>-12.96</v>
       </c>
     </row>
     <row r="30">
@@ -1205,11 +1205,11 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>20.8</v>
+        <v>20.89</v>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>-9.529999999999999</v>
+        <v>-9.130000000000001</v>
       </c>
     </row>
     <row r="31">
@@ -1231,11 +1231,11 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>19.03</v>
+        <v>19</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>-7.17</v>
+        <v>-7.32</v>
       </c>
     </row>
     <row r="32">
@@ -1257,11 +1257,11 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>-5.42</v>
+        <v>-5.51</v>
       </c>
     </row>
     <row r="33">
@@ -1283,11 +1283,11 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>2.03</v>
+        <v>2.09</v>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>-6.88</v>
+        <v>-4.13</v>
       </c>
     </row>
     <row r="34">
@@ -1309,11 +1309,11 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>-9.300000000000001</v>
+        <v>-9.58</v>
       </c>
     </row>
     <row r="35">
@@ -1335,11 +1335,11 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>5.14</v>
+        <v>5.08</v>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>-4.99</v>
+        <v>-6.1</v>
       </c>
     </row>
     <row r="36">
@@ -1361,11 +1361,11 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>61.58</v>
+        <v>61</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>-3.48</v>
+        <v>-4.39</v>
       </c>
     </row>
     <row r="37">
@@ -1387,11 +1387,11 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0.42</v>
+        <v>0.38</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>-9.52</v>
       </c>
     </row>
     <row r="38">
@@ -1413,11 +1413,11 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>107.25</v>
+        <v>103.5</v>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>-8.25</v>
+        <v>-11.46</v>
       </c>
     </row>
     <row r="39">
@@ -1465,11 +1465,11 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>13.82</v>
+        <v>13.07</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>-5.43</v>
       </c>
     </row>
     <row r="41">
@@ -1491,11 +1491,11 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>13.55</v>
+        <v>14.65</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>-7.7</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="42">
@@ -1517,11 +1517,11 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>2.69</v>
+        <v>2.57</v>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>-4.95</v>
+        <v>-9.19</v>
       </c>
     </row>
     <row r="43">
@@ -1569,11 +1569,11 @@
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>8.69</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>-2.91</v>
+        <v>-9.390000000000001</v>
       </c>
     </row>
     <row r="45">
@@ -1595,11 +1595,11 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>-3.68</v>
+        <v>-8.550000000000001</v>
       </c>
     </row>
     <row r="46">
@@ -1621,11 +1621,11 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>99.39</v>
+        <v>93</v>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>-5.07</v>
+        <v>-11.17</v>
       </c>
     </row>
     <row r="47">
@@ -1647,11 +1647,11 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>3.9</v>
+        <v>3.68</v>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>-3.7</v>
+        <v>-9.140000000000001</v>
       </c>
     </row>
     <row r="48">
@@ -1673,11 +1673,11 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>284.3</v>
+        <v>300</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>-1.95</v>
+        <v>3.47</v>
       </c>
     </row>
     <row r="49">
@@ -1699,11 +1699,11 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>47.05</v>
+        <v>46.62</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>0.15</v>
+        <v>-0.77</v>
       </c>
     </row>
     <row r="50">
@@ -1725,11 +1725,11 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>234.8</v>
+        <v>253.95</v>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>-3.29</v>
+        <v>4.59</v>
       </c>
     </row>
     <row r="51">
@@ -1777,11 +1777,11 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>5.49</v>
+        <v>5.39</v>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>-1.26</v>
+        <v>-3.06</v>
       </c>
     </row>
     <row r="53">
@@ -1803,11 +1803,11 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>477</v>
+        <v>461</v>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>-7.74</v>
+        <v>-10.83</v>
       </c>
     </row>
     <row r="54">
@@ -1829,11 +1829,11 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>30.68</v>
+        <v>27</v>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>-4.13</v>
+        <v>-15.62</v>
       </c>
     </row>
     <row r="55">
@@ -1855,11 +1855,11 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>19.27</v>
+        <v>17.31</v>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>-3.65</v>
+        <v>-13.45</v>
       </c>
     </row>
     <row r="56">
@@ -1881,11 +1881,11 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>35</v>
+        <v>34.38</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>-7.16</v>
+        <v>-8.81</v>
       </c>
     </row>
     <row r="57">
@@ -1907,11 +1907,11 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>50.34</v>
+        <v>47.45</v>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>-0.32</v>
+        <v>-6.04</v>
       </c>
     </row>
     <row r="58">
@@ -1933,11 +1933,11 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>9.49</v>
+        <v>8.98</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>-1.96</v>
+        <v>-7.23</v>
       </c>
     </row>
     <row r="59">
@@ -1959,11 +1959,11 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>15.75</v>
+        <v>15.15</v>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>-5.69</v>
+        <v>-9.279999999999999</v>
       </c>
     </row>
     <row r="60">
@@ -1985,11 +1985,11 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>20.65</v>
+        <v>20.6</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>-8.75</v>
+        <v>-8.970000000000001</v>
       </c>
     </row>
     <row r="61">
@@ -2011,11 +2011,11 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>2.51</v>
+        <v>2.5</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>-7.04</v>
+        <v>-7.41</v>
       </c>
     </row>
     <row r="62">
@@ -2037,11 +2037,11 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>511.35</v>
+        <v>540</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>-6.85</v>
+        <v>-1.63</v>
       </c>
     </row>
     <row r="63">
@@ -2063,11 +2063,11 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>140.68</v>
+        <v>141</v>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>-1.71</v>
+        <v>-1.49</v>
       </c>
     </row>
     <row r="64">
@@ -2089,11 +2089,11 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>1.4</v>
+        <v>1.29</v>
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>-7.86</v>
       </c>
     </row>
     <row r="65">
@@ -2115,11 +2115,11 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>81.39</v>
+        <v>82</v>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>-1.81</v>
+        <v>-1.07</v>
       </c>
     </row>
     <row r="66">
@@ -2141,11 +2141,11 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>347.6</v>
+        <v>359</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>-3.44</v>
+        <v>-0.28</v>
       </c>
     </row>
     <row r="67">
@@ -2167,11 +2167,11 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>1.75</v>
+        <v>1.71</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>-2.29</v>
       </c>
     </row>
     <row r="68">
@@ -2193,11 +2193,11 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>14.19</v>
+        <v>14.4</v>
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>-5.08</v>
+        <v>-3.68</v>
       </c>
     </row>
     <row r="69">
@@ -2219,11 +2219,11 @@
         <v>0</v>
       </c>
       <c r="F69" t="n">
-        <v>24.1</v>
+        <v>22.1</v>
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>-6.95</v>
+        <v>-14.67</v>
       </c>
     </row>
     <row r="70">
@@ -2245,11 +2245,11 @@
         <v>0</v>
       </c>
       <c r="F70" t="n">
-        <v>4.94</v>
+        <v>4.8</v>
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>-0.8</v>
+        <v>-3.61</v>
       </c>
     </row>
     <row r="71">
@@ -2271,11 +2271,11 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>206.35</v>
+        <v>204</v>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>-8.289999999999999</v>
+        <v>-9.33</v>
       </c>
     </row>
     <row r="72">
@@ -2297,11 +2297,11 @@
         <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>91</v>
+        <v>89.09</v>
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>-4.11</v>
+        <v>-6.12</v>
       </c>
     </row>
     <row r="73">
@@ -2323,11 +2323,11 @@
         <v>0</v>
       </c>
       <c r="F73" t="n">
-        <v>57.52</v>
+        <v>52.96</v>
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>-6.77</v>
+        <v>-14.17</v>
       </c>
     </row>
     <row r="74">
@@ -2349,11 +2349,11 @@
         <v>0</v>
       </c>
       <c r="F74" t="n">
-        <v>813.85</v>
+        <v>790</v>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>-1.99</v>
+        <v>-4.86</v>
       </c>
     </row>
     <row r="75">
@@ -2375,11 +2375,11 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>25.26</v>
+        <v>24.99</v>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>-2.47</v>
+        <v>-3.51</v>
       </c>
     </row>
     <row r="76">
@@ -2401,11 +2401,11 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>22.31</v>
+        <v>21.9</v>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>-4.62</v>
+        <v>-6.37</v>
       </c>
     </row>
     <row r="77">
@@ -2427,11 +2427,11 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>8.5</v>
+        <v>8.52</v>
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>-3.63</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="78">
@@ -2453,11 +2453,11 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>64.97</v>
+        <v>64</v>
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>-2.81</v>
+        <v>-4.26</v>
       </c>
     </row>
     <row r="79">
@@ -2479,11 +2479,11 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>30.35</v>
+        <v>30.2</v>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>-5.16</v>
+        <v>-5.63</v>
       </c>
     </row>
     <row r="80">
@@ -2531,11 +2531,11 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>3.69</v>
+        <v>3.75</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>-7.05</v>
+        <v>-5.54</v>
       </c>
     </row>
     <row r="82">
@@ -2557,11 +2557,11 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>824.3</v>
+        <v>838</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>2.39</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="83">
@@ -2583,11 +2583,11 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>13.81</v>
+        <v>13.11</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>-1</v>
+        <v>-6.02</v>
       </c>
     </row>
     <row r="84">
@@ -2609,11 +2609,11 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>39.99</v>
+        <v>39.48</v>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>3.33</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="85">
@@ -2635,11 +2635,11 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>139.7</v>
+        <v>139.8</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>-2.96</v>
+        <v>-2.89</v>
       </c>
     </row>
     <row r="86">
@@ -2661,11 +2661,11 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>115.93</v>
+        <v>110.18</v>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>-7.99</v>
+        <v>-12.56</v>
       </c>
     </row>
     <row r="87">
@@ -2687,11 +2687,11 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>212.58</v>
+        <v>211.5</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>-1.17</v>
+        <v>-1.67</v>
       </c>
     </row>
     <row r="88">
@@ -2713,11 +2713,11 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>17.87</v>
+        <v>18.1</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>-7.46</v>
+        <v>-6.27</v>
       </c>
     </row>
     <row r="89">
@@ -2739,11 +2739,11 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>118.78</v>
+        <v>113</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>5.33</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="90">
@@ -2765,11 +2765,11 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>4.75</v>
+        <v>4.53</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>-6.68</v>
+        <v>-11</v>
       </c>
     </row>
     <row r="91">
@@ -2791,11 +2791,11 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>156.9</v>
+        <v>157.49</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>-1.93</v>
+        <v>-1.56</v>
       </c>
     </row>
     <row r="92">
@@ -2817,11 +2817,11 @@
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>43.2</v>
+        <v>41.95</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>-5.88</v>
+        <v>-8.609999999999999</v>
       </c>
     </row>
     <row r="93">
@@ -2843,11 +2843,11 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>18.43</v>
+        <v>19.25</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>-5.92</v>
+        <v>-1.74</v>
       </c>
     </row>
     <row r="94">
@@ -2869,11 +2869,11 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>-2.56</v>
+        <v>-5.13</v>
       </c>
     </row>
     <row r="95">
@@ -2895,11 +2895,11 @@
         <v>0</v>
       </c>
       <c r="F95" t="n">
-        <v>300.2</v>
+        <v>294</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>-3.32</v>
+        <v>-5.31</v>
       </c>
     </row>
     <row r="96">
@@ -2921,11 +2921,11 @@
         <v>0</v>
       </c>
       <c r="F96" t="n">
-        <v>4.65</v>
+        <v>4.69</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="n">
-        <v>-3.12</v>
+        <v>-2.29</v>
       </c>
     </row>
     <row r="97">
@@ -2947,11 +2947,11 @@
         <v>0</v>
       </c>
       <c r="F97" t="n">
-        <v>172.26</v>
+        <v>182.8</v>
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>-4.29</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="98">
@@ -2999,11 +2999,11 @@
         <v>0</v>
       </c>
       <c r="F99" t="n">
-        <v>41.98</v>
+        <v>40.96</v>
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>2.39</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="100">
@@ -3025,11 +3025,11 @@
         <v>0</v>
       </c>
       <c r="F100" t="n">
-        <v>17.41</v>
+        <v>17.6</v>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>-9.279999999999999</v>
+        <v>-8.289999999999999</v>
       </c>
     </row>
     <row r="101">
@@ -3077,11 +3077,11 @@
         <v>0</v>
       </c>
       <c r="F102" t="n">
-        <v>387.35</v>
+        <v>386.95</v>
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>1.93</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="103">
@@ -3103,11 +3103,11 @@
         <v>0</v>
       </c>
       <c r="F103" t="n">
-        <v>9.35</v>
+        <v>8.4</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>-4.2</v>
+        <v>-13.93</v>
       </c>
     </row>
     <row r="104">
@@ -3129,11 +3129,11 @@
         <v>0</v>
       </c>
       <c r="F104" t="n">
-        <v>113.7</v>
+        <v>108.8</v>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>-1.97</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="105">
@@ -3155,11 +3155,11 @@
         <v>0</v>
       </c>
       <c r="F105" t="n">
-        <v>133.8</v>
+        <v>120.4</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>5.37</v>
+        <v>-5.18</v>
       </c>
     </row>
     <row r="106">
@@ -3181,11 +3181,11 @@
         <v>0</v>
       </c>
       <c r="F106" t="n">
-        <v>1.25</v>
+        <v>1.3</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>-6.02</v>
+        <v>-2.26</v>
       </c>
     </row>
     <row r="107">
@@ -3207,11 +3207,11 @@
         <v>0</v>
       </c>
       <c r="F107" t="n">
-        <v>15.2</v>
+        <v>12.42</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>-2.5</v>
+        <v>-20.33</v>
       </c>
     </row>
     <row r="108">
@@ -3233,11 +3233,11 @@
         <v>0</v>
       </c>
       <c r="F108" t="n">
-        <v>161.47</v>
+        <v>163.25</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="n">
-        <v>-5.02</v>
+        <v>-3.97</v>
       </c>
     </row>
     <row r="109">
@@ -3259,11 +3259,11 @@
         <v>0</v>
       </c>
       <c r="F109" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="n">
-        <v>-4.17</v>
+        <v>-4.73</v>
       </c>
     </row>
     <row r="110">
@@ -3285,11 +3285,11 @@
         <v>0</v>
       </c>
       <c r="F110" t="n">
-        <v>16.19</v>
+        <v>15.85</v>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>-8.529999999999999</v>
+        <v>-10.45</v>
       </c>
     </row>
     <row r="111">
@@ -3311,11 +3311,11 @@
         <v>0</v>
       </c>
       <c r="F111" t="n">
-        <v>46.24</v>
+        <v>45.4</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>7.56</v>
+        <v>5.61</v>
       </c>
     </row>
     <row r="112">
@@ -3337,11 +3337,11 @@
         <v>0</v>
       </c>
       <c r="F112" t="n">
-        <v>243.3</v>
+        <v>234.75</v>
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>-5.33</v>
+        <v>-8.66</v>
       </c>
     </row>
     <row r="113">
@@ -3363,11 +3363,11 @@
         <v>0</v>
       </c>
       <c r="F113" t="n">
-        <v>196.14</v>
+        <v>191.5</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>-5.66</v>
+        <v>-7.89</v>
       </c>
     </row>
     <row r="114">
@@ -3389,11 +3389,11 @@
         <v>0</v>
       </c>
       <c r="F114" t="n">
-        <v>114.58</v>
+        <v>111.5</v>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>-4.19</v>
+        <v>-6.76</v>
       </c>
     </row>
     <row r="115">
@@ -3415,11 +3415,11 @@
         <v>0</v>
       </c>
       <c r="F115" t="n">
-        <v>41.1</v>
+        <v>41.15</v>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>-0.46</v>
+        <v>-0.34</v>
       </c>
     </row>
     <row r="116">
@@ -3441,11 +3441,11 @@
         <v>0</v>
       </c>
       <c r="F116" t="n">
-        <v>57.22</v>
+        <v>55.26</v>
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>-2.85</v>
+        <v>-6.18</v>
       </c>
     </row>
     <row r="117">
@@ -3493,11 +3493,11 @@
         <v>0</v>
       </c>
       <c r="F118" t="n">
-        <v>50.55</v>
+        <v>49.75</v>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>-5.32</v>
+        <v>-6.82</v>
       </c>
     </row>
     <row r="119">
@@ -3519,11 +3519,11 @@
         <v>0</v>
       </c>
       <c r="F119" t="n">
-        <v>24.99</v>
+        <v>24.59</v>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>-7.1</v>
+        <v>-8.59</v>
       </c>
     </row>
     <row r="120">
@@ -3571,11 +3571,11 @@
         <v>0</v>
       </c>
       <c r="F121" t="n">
-        <v>3188.2</v>
+        <v>3250</v>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>-2.17</v>
+        <v>-0.27</v>
       </c>
     </row>
     <row r="122">
@@ -3597,11 +3597,11 @@
         <v>0</v>
       </c>
       <c r="F122" t="n">
-        <v>73.2</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>-4.85</v>
+        <v>-4.33</v>
       </c>
     </row>
     <row r="123">
@@ -3623,11 +3623,11 @@
         <v>0</v>
       </c>
       <c r="F123" t="n">
-        <v>5.59</v>
+        <v>5.6</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>-3.62</v>
+        <v>-3.45</v>
       </c>
     </row>
     <row r="124">
@@ -3649,11 +3649,11 @@
         <v>0</v>
       </c>
       <c r="F124" t="n">
-        <v>86.81</v>
+        <v>84.06999999999999</v>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>-2.24</v>
+        <v>-5.33</v>
       </c>
     </row>
     <row r="125">
@@ -3675,11 +3675,11 @@
         <v>0</v>
       </c>
       <c r="F125" t="n">
-        <v>8.02</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>-7.82</v>
+        <v>-4.6</v>
       </c>
     </row>
     <row r="126">
@@ -3701,11 +3701,11 @@
         <v>0</v>
       </c>
       <c r="F126" t="n">
-        <v>38.57</v>
+        <v>35.9</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>-3.33</v>
+        <v>-10.03</v>
       </c>
     </row>
     <row r="127">
@@ -3727,11 +3727,11 @@
         <v>0</v>
       </c>
       <c r="F127" t="n">
-        <v>195.4</v>
+        <v>189.73</v>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>-3.26</v>
+        <v>-6.07</v>
       </c>
     </row>
     <row r="128">
@@ -3753,11 +3753,11 @@
         <v>0</v>
       </c>
       <c r="F128" t="n">
-        <v>23.71</v>
+        <v>22.7</v>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>0.25</v>
+        <v>-4.02</v>
       </c>
     </row>
     <row r="129">
@@ -3779,11 +3779,11 @@
         <v>0</v>
       </c>
       <c r="F129" t="n">
-        <v>85.95</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>-6.07</v>
+        <v>-7.21</v>
       </c>
     </row>
     <row r="130">
@@ -3805,11 +3805,11 @@
         <v>0</v>
       </c>
       <c r="F130" t="n">
-        <v>15.08</v>
+        <v>14.63</v>
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>-3.58</v>
+        <v>-6.46</v>
       </c>
     </row>
     <row r="131">
@@ -3831,11 +3831,11 @@
         <v>0</v>
       </c>
       <c r="F131" t="n">
-        <v>279.6</v>
+        <v>279.9</v>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>-3.72</v>
+        <v>-3.62</v>
       </c>
     </row>
     <row r="132">
@@ -3857,11 +3857,11 @@
         <v>0</v>
       </c>
       <c r="F132" t="n">
-        <v>2.16</v>
+        <v>2.07</v>
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>-5.68</v>
+        <v>-9.609999999999999</v>
       </c>
     </row>
     <row r="133">
@@ -3883,11 +3883,11 @@
         <v>0</v>
       </c>
       <c r="F133" t="n">
-        <v>146.35</v>
+        <v>146.01</v>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>-1.71</v>
+        <v>-1.94</v>
       </c>
     </row>
     <row r="134">
@@ -3909,11 +3909,11 @@
         <v>0</v>
       </c>
       <c r="F134" t="n">
-        <v>6.64</v>
+        <v>6.44</v>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>-3.63</v>
+        <v>-6.53</v>
       </c>
     </row>
     <row r="135">
@@ -3935,11 +3935,11 @@
         <v>0</v>
       </c>
       <c r="F135" t="n">
-        <v>6.15</v>
+        <v>6.39</v>
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="n">
-        <v>-4.8</v>
+        <v>-1.08</v>
       </c>
     </row>
     <row r="136">
@@ -3961,11 +3961,11 @@
         <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>13.8</v>
+        <v>11.65</v>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>-6.12</v>
+        <v>-20.75</v>
       </c>
     </row>
     <row r="137">
@@ -3987,11 +3987,11 @@
         <v>0</v>
       </c>
       <c r="F137" t="n">
-        <v>171.23</v>
+        <v>172.9</v>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="n">
-        <v>-2.09</v>
+        <v>-1.14</v>
       </c>
     </row>
     <row r="138">
@@ -4013,11 +4013,11 @@
         <v>0</v>
       </c>
       <c r="F138" t="n">
-        <v>19.57</v>
+        <v>18.99</v>
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="n">
-        <v>-13.79</v>
+        <v>-16.34</v>
       </c>
     </row>
     <row r="139">
@@ -4039,11 +4039,11 @@
         <v>0</v>
       </c>
       <c r="F139" t="n">
-        <v>160.1</v>
+        <v>158.85</v>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="n">
-        <v>-5.8</v>
+        <v>-6.53</v>
       </c>
     </row>
     <row r="140">
@@ -4065,11 +4065,11 @@
         <v>0</v>
       </c>
       <c r="F140" t="n">
-        <v>440</v>
+        <v>465</v>
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="n">
-        <v>-7.37</v>
+        <v>-2.11</v>
       </c>
     </row>
     <row r="141">
@@ -4091,11 +4091,11 @@
         <v>0</v>
       </c>
       <c r="F141" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="n">
-        <v>-5.48</v>
+        <v>-6.45</v>
       </c>
     </row>
     <row r="142">
@@ -4117,11 +4117,11 @@
         <v>0</v>
       </c>
       <c r="F142" t="n">
-        <v>28.3</v>
+        <v>26.01</v>
       </c>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="n">
-        <v>-5.67</v>
+        <v>-13.3</v>
       </c>
     </row>
     <row r="143">
@@ -4143,11 +4143,11 @@
         <v>0</v>
       </c>
       <c r="F143" t="n">
-        <v>22.35</v>
+        <v>21.73</v>
       </c>
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="n">
-        <v>-3.83</v>
+        <v>-6.5</v>
       </c>
     </row>
     <row r="144">
@@ -4169,11 +4169,11 @@
         <v>0</v>
       </c>
       <c r="F144" t="n">
-        <v>1.23</v>
+        <v>1.18</v>
       </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="n">
-        <v>-2.38</v>
+        <v>-6.35</v>
       </c>
     </row>
     <row r="145">
@@ -4195,11 +4195,11 @@
         <v>0</v>
       </c>
       <c r="F145" t="n">
-        <v>40.14</v>
+        <v>38.59</v>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="n">
-        <v>-6.41</v>
+        <v>-10.03</v>
       </c>
     </row>
     <row r="146">
@@ -4221,11 +4221,11 @@
         <v>0</v>
       </c>
       <c r="F146" t="n">
-        <v>557.9</v>
+        <v>579.85</v>
       </c>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="n">
-        <v>-6.23</v>
+        <v>-2.54</v>
       </c>
     </row>
     <row r="147">
@@ -4247,11 +4247,11 @@
         <v>0</v>
       </c>
       <c r="F147" t="n">
-        <v>26.75</v>
+        <v>26.06</v>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="n">
-        <v>-2.37</v>
+        <v>-4.89</v>
       </c>
     </row>
     <row r="148">
@@ -4273,11 +4273,11 @@
         <v>0</v>
       </c>
       <c r="F148" t="n">
-        <v>7.97</v>
+        <v>8</v>
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="n">
-        <v>-4.55</v>
+        <v>-4.19</v>
       </c>
     </row>
     <row r="149">
@@ -4325,11 +4325,11 @@
         <v>0</v>
       </c>
       <c r="F150" t="n">
-        <v>7.22</v>
+        <v>7.06</v>
       </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="n">
-        <v>-7.32</v>
+        <v>-9.369999999999999</v>
       </c>
     </row>
     <row r="151">
@@ -4351,11 +4351,11 @@
         <v>0</v>
       </c>
       <c r="F151" t="n">
-        <v>96.39</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="n">
-        <v>-3.61</v>
+        <v>-4.9</v>
       </c>
     </row>
     <row r="152">
@@ -4377,11 +4377,11 @@
         <v>0</v>
       </c>
       <c r="F152" t="n">
-        <v>7.25</v>
+        <v>7.1</v>
       </c>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="n">
-        <v>-0.68</v>
+        <v>-2.74</v>
       </c>
     </row>
     <row r="153">
@@ -4403,11 +4403,11 @@
         <v>0</v>
       </c>
       <c r="F153" t="n">
-        <v>57.5</v>
+        <v>56.25</v>
       </c>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="n">
-        <v>-4.79</v>
+        <v>-6.86</v>
       </c>
     </row>
     <row r="154">
@@ -4429,11 +4429,11 @@
         <v>0</v>
       </c>
       <c r="F154" t="n">
-        <v>105.31</v>
+        <v>102.5</v>
       </c>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="n">
-        <v>-4.35</v>
+        <v>-6.9</v>
       </c>
     </row>
     <row r="155">
@@ -4455,11 +4455,11 @@
         <v>0</v>
       </c>
       <c r="F155" t="n">
-        <v>21.68</v>
+        <v>21.8</v>
       </c>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="n">
-        <v>-6.35</v>
+        <v>-5.83</v>
       </c>
     </row>
     <row r="156">
@@ -4481,11 +4481,11 @@
         <v>0</v>
       </c>
       <c r="F156" t="n">
-        <v>48.07</v>
+        <v>45.21</v>
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="n">
-        <v>-4.64</v>
+        <v>-10.32</v>
       </c>
     </row>
     <row r="157">
@@ -4507,11 +4507,11 @@
         <v>0</v>
       </c>
       <c r="F157" t="n">
-        <v>65.59999999999999</v>
+        <v>62.61</v>
       </c>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="n">
-        <v>6.15</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="158">
@@ -4533,11 +4533,11 @@
         <v>0</v>
       </c>
       <c r="F158" t="n">
-        <v>90.39</v>
+        <v>87.62</v>
       </c>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="n">
-        <v>-5.44</v>
+        <v>-8.34</v>
       </c>
     </row>
     <row r="159">
@@ -4559,11 +4559,11 @@
         <v>0</v>
       </c>
       <c r="F159" t="n">
-        <v>22.2</v>
+        <v>21.93</v>
       </c>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="n">
-        <v>-5.21</v>
+        <v>-6.36</v>
       </c>
     </row>
     <row r="160">
@@ -4585,11 +4585,11 @@
         <v>0</v>
       </c>
       <c r="F160" t="n">
-        <v>66.11</v>
+        <v>61.6</v>
       </c>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="n">
-        <v>-4.19</v>
+        <v>-10.72</v>
       </c>
     </row>
     <row r="161">
@@ -4611,11 +4611,11 @@
         <v>0</v>
       </c>
       <c r="F161" t="n">
-        <v>30.17</v>
+        <v>32</v>
       </c>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="n">
-        <v>-2.36</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="162">
@@ -4637,11 +4637,11 @@
         <v>0</v>
       </c>
       <c r="F162" t="n">
-        <v>19.74</v>
+        <v>18.39</v>
       </c>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="n">
-        <v>-0.15</v>
+        <v>-6.98</v>
       </c>
     </row>
     <row r="163">
@@ -4663,11 +4663,11 @@
         <v>0</v>
       </c>
       <c r="F163" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="n">
-        <v>-0.82</v>
+        <v>-9.92</v>
       </c>
     </row>
     <row r="164">
@@ -4689,11 +4689,11 @@
         <v>0</v>
       </c>
       <c r="F164" t="n">
-        <v>77.40000000000001</v>
+        <v>76.7</v>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="n">
-        <v>-5.33</v>
+        <v>-6.19</v>
       </c>
     </row>
     <row r="165">
@@ -4715,11 +4715,11 @@
         <v>0</v>
       </c>
       <c r="F165" t="n">
-        <v>64.65000000000001</v>
+        <v>64</v>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="n">
-        <v>-1.15</v>
+        <v>-2.14</v>
       </c>
     </row>
     <row r="166">
@@ -4741,11 +4741,11 @@
         <v>0</v>
       </c>
       <c r="F166" t="n">
-        <v>15.85</v>
+        <v>15.8</v>
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="n">
-        <v>-5.09</v>
+        <v>-5.39</v>
       </c>
     </row>
     <row r="167">
@@ -4767,11 +4767,11 @@
         <v>0</v>
       </c>
       <c r="F167" t="n">
-        <v>26.1</v>
+        <v>25.9</v>
       </c>
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="n">
-        <v>-3.69</v>
+        <v>-4.43</v>
       </c>
     </row>
     <row r="168">
@@ -4793,11 +4793,11 @@
         <v>0</v>
       </c>
       <c r="F168" t="n">
-        <v>2071.2</v>
+        <v>2035</v>
       </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="n">
-        <v>-3.62</v>
+        <v>-5.31</v>
       </c>
     </row>
     <row r="169">
@@ -4819,11 +4819,11 @@
         <v>0</v>
       </c>
       <c r="F169" t="n">
-        <v>72.70999999999999</v>
+        <v>72.95</v>
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="n">
-        <v>-3.05</v>
+        <v>-2.73</v>
       </c>
     </row>
     <row r="170">
@@ -4845,11 +4845,11 @@
         <v>0</v>
       </c>
       <c r="F170" t="n">
-        <v>14.84</v>
+        <v>13.57</v>
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="n">
-        <v>-1</v>
+        <v>-9.470000000000001</v>
       </c>
     </row>
     <row r="171">
@@ -4871,11 +4871,11 @@
         <v>0</v>
       </c>
       <c r="F171" t="n">
-        <v>148.22</v>
+        <v>145.3</v>
       </c>
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="n">
-        <v>-4.52</v>
+        <v>-6.4</v>
       </c>
     </row>
     <row r="172">
@@ -4897,11 +4897,11 @@
         <v>0</v>
       </c>
       <c r="F172" t="n">
-        <v>44.75</v>
+        <v>43</v>
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="n">
-        <v>-4.16</v>
+        <v>-7.9</v>
       </c>
     </row>
     <row r="173">
@@ -4949,11 +4949,11 @@
         <v>0</v>
       </c>
       <c r="F174" t="n">
-        <v>34.35</v>
+        <v>33.57</v>
       </c>
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="n">
-        <v>-5.74</v>
+        <v>-7.88</v>
       </c>
     </row>
     <row r="175">
@@ -4975,11 +4975,11 @@
         <v>0</v>
       </c>
       <c r="F175" t="n">
-        <v>131.4</v>
+        <v>120.9</v>
       </c>
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="n">
-        <v>-1.68</v>
+        <v>-9.539999999999999</v>
       </c>
     </row>
     <row r="176">
@@ -5001,11 +5001,11 @@
         <v>0</v>
       </c>
       <c r="F176" t="n">
-        <v>6.85</v>
+        <v>6.65</v>
       </c>
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="n">
-        <v>-3.66</v>
+        <v>-6.47</v>
       </c>
     </row>
     <row r="177">
@@ -5027,11 +5027,11 @@
         <v>0</v>
       </c>
       <c r="F177" t="n">
-        <v>3.97</v>
+        <v>3.89</v>
       </c>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="n">
-        <v>-11.58</v>
+        <v>-13.36</v>
       </c>
     </row>
     <row r="178">
@@ -5053,11 +5053,11 @@
         <v>0</v>
       </c>
       <c r="F178" t="n">
-        <v>891.8</v>
+        <v>888</v>
       </c>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
-        <v>1.8</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="179">
@@ -5079,11 +5079,11 @@
         <v>0</v>
       </c>
       <c r="F179" t="n">
-        <v>105.6</v>
+        <v>105.95</v>
       </c>
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="n">
-        <v>-4</v>
+        <v>-3.68</v>
       </c>
     </row>
     <row r="180">
@@ -5105,11 +5105,11 @@
         <v>0</v>
       </c>
       <c r="F180" t="n">
-        <v>15.66</v>
+        <v>15.1</v>
       </c>
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="n">
-        <v>-1.51</v>
+        <v>-5.03</v>
       </c>
     </row>
     <row r="181">
@@ -5131,11 +5131,11 @@
         <v>0</v>
       </c>
       <c r="F181" t="n">
-        <v>0.99</v>
+        <v>0.97</v>
       </c>
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="182">
@@ -5157,11 +5157,11 @@
         <v>0</v>
       </c>
       <c r="F182" t="n">
-        <v>133.07</v>
+        <v>136.5</v>
       </c>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="n">
-        <v>-1.36</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="183">
@@ -5209,11 +5209,11 @@
         <v>0</v>
       </c>
       <c r="F184" t="n">
-        <v>147</v>
+        <v>142.8</v>
       </c>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="n">
-        <v>-3.86</v>
+        <v>-6.61</v>
       </c>
     </row>
     <row r="185">
@@ -5235,11 +5235,11 @@
         <v>0</v>
       </c>
       <c r="F185" t="n">
-        <v>25.4</v>
+        <v>25.8</v>
       </c>
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="n">
-        <v>-0.78</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="186">
@@ -5261,11 +5261,11 @@
         <v>0</v>
       </c>
       <c r="F186" t="n">
-        <v>987.5</v>
+        <v>950</v>
       </c>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="n">
-        <v>-0.25</v>
+        <v>-4.04</v>
       </c>
     </row>
     <row r="187">
@@ -5287,11 +5287,11 @@
         <v>0</v>
       </c>
       <c r="F187" t="n">
-        <v>141.71</v>
+        <v>157</v>
       </c>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="n">
-        <v>-0.2</v>
+        <v>10.56</v>
       </c>
     </row>
     <row r="188">
@@ -5313,11 +5313,11 @@
         <v>0</v>
       </c>
       <c r="F188" t="n">
-        <v>47</v>
+        <v>44.4</v>
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="n">
-        <v>0.53</v>
+        <v>-5.03</v>
       </c>
     </row>
     <row r="189">
@@ -5339,11 +5339,11 @@
         <v>0</v>
       </c>
       <c r="F189" t="n">
-        <v>359.9</v>
+        <v>394</v>
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="n">
-        <v>1.94</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="190">
@@ -5365,11 +5365,11 @@
         <v>0</v>
       </c>
       <c r="F190" t="n">
-        <v>140.7</v>
+        <v>143.21</v>
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="n">
-        <v>-2.22</v>
+        <v>-0.48</v>
       </c>
     </row>
     <row r="191">
@@ -5391,11 +5391,11 @@
         <v>0</v>
       </c>
       <c r="F191" t="n">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="n">
-        <v>-0.9399999999999999</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="192">
@@ -5417,11 +5417,11 @@
         <v>0</v>
       </c>
       <c r="F192" t="n">
-        <v>122.39</v>
+        <v>124</v>
       </c>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="n">
-        <v>-0.6</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="193">
@@ -5443,11 +5443,11 @@
         <v>0</v>
       </c>
       <c r="F193" t="n">
-        <v>45.3</v>
+        <v>47.5</v>
       </c>
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="n">
-        <v>-5.61</v>
+        <v>-1.02</v>
       </c>
     </row>
     <row r="194">
@@ -5469,11 +5469,11 @@
         <v>0</v>
       </c>
       <c r="F194" t="n">
-        <v>99.92</v>
+        <v>98</v>
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="n">
-        <v>-0.08</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="195">
@@ -5495,11 +5495,11 @@
         <v>0</v>
       </c>
       <c r="F195" t="n">
-        <v>390</v>
+        <v>372.95</v>
       </c>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="n">
-        <v>-0.64</v>
+        <v>-4.98</v>
       </c>
     </row>
     <row r="196">
@@ -5521,11 +5521,11 @@
         <v>0</v>
       </c>
       <c r="F196" t="n">
-        <v>33.53</v>
+        <v>32.3</v>
       </c>
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="n">
-        <v>-4.36</v>
+        <v>-7.87</v>
       </c>
     </row>
     <row r="197">
@@ -5573,11 +5573,11 @@
         <v>0</v>
       </c>
       <c r="F198" t="n">
-        <v>116.16</v>
+        <v>116.1</v>
       </c>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="n">
-        <v>-1.56</v>
+        <v>-1.61</v>
       </c>
     </row>
     <row r="199">
@@ -5599,11 +5599,11 @@
         <v>0</v>
       </c>
       <c r="F199" t="n">
-        <v>51.83</v>
+        <v>51.5</v>
       </c>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="n">
-        <v>-5.25</v>
+        <v>-5.85</v>
       </c>
     </row>
     <row r="200">
@@ -5625,11 +5625,11 @@
         <v>0</v>
       </c>
       <c r="F200" t="n">
-        <v>1.25</v>
+        <v>1.14</v>
       </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="n">
-        <v>-2.34</v>
+        <v>-10.94</v>
       </c>
     </row>
     <row r="201">
@@ -5651,11 +5651,11 @@
         <v>0</v>
       </c>
       <c r="F201" t="n">
-        <v>72.54000000000001</v>
+        <v>69</v>
       </c>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="n">
-        <v>-4.55</v>
+        <v>-9.210000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-04-03 05:28 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -477,11 +477,11 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>122.05</v>
+        <v>123</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>-15.01</v>
+        <v>-14.35</v>
       </c>
     </row>
     <row r="3">
@@ -529,11 +529,11 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>149.05</v>
+        <v>147</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>-14.83</v>
+        <v>-16</v>
       </c>
     </row>
     <row r="5">
@@ -555,11 +555,11 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>82.76000000000001</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>-2.64</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="6">
@@ -581,11 +581,11 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>73.5</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>-11.45</v>
+        <v>-7.65</v>
       </c>
     </row>
     <row r="7">
@@ -607,11 +607,11 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>12.73</v>
+        <v>13.04</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>-9.07</v>
+        <v>-6.86</v>
       </c>
     </row>
     <row r="8">
@@ -633,11 +633,11 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>29.3</v>
+        <v>31.3</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>-7.8</v>
+        <v>-1.51</v>
       </c>
     </row>
     <row r="9">
@@ -659,11 +659,11 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>5.36</v>
+        <v>5.94</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>-0.74</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -711,11 +711,11 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>30.1</v>
+        <v>32.55</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>1.69</v>
+        <v>9.970000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -737,11 +737,11 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>8.6</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>-3.37</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -763,11 +763,11 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>10.78</v>
+        <v>11.18</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>-7.86</v>
+        <v>-4.44</v>
       </c>
     </row>
     <row r="14">
@@ -815,11 +815,11 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>47</v>
+        <v>52.5</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>-5.91</v>
+        <v>5.11</v>
       </c>
     </row>
     <row r="16">
@@ -841,11 +841,11 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>5.79</v>
+        <v>5.8</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>-5.08</v>
+        <v>-4.92</v>
       </c>
     </row>
     <row r="17">
@@ -893,11 +893,11 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>112.17</v>
+        <v>116.9</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>-5.73</v>
+        <v>-1.76</v>
       </c>
     </row>
     <row r="19">
@@ -919,11 +919,11 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>13.8</v>
+        <v>13.75</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="20">
@@ -945,11 +945,11 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>49.5</v>
+        <v>49.3</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>-6.59</v>
+        <v>-6.96</v>
       </c>
     </row>
     <row r="21">
@@ -971,11 +971,11 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>119.19</v>
+        <v>124.8</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>-4.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -997,11 +997,11 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>32.68</v>
+        <v>35.04</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>-3.34</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="23">
@@ -1023,11 +1023,11 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>23</v>
+        <v>22.5</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>-2.34</v>
+        <v>-4.46</v>
       </c>
     </row>
     <row r="24">
@@ -1049,11 +1049,11 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>28.3</v>
+        <v>27.8</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>-3.08</v>
+        <v>-4.79</v>
       </c>
     </row>
     <row r="25">
@@ -1075,11 +1075,11 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>8.76</v>
+        <v>8.99</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>-4.78</v>
+        <v>-2.28</v>
       </c>
     </row>
     <row r="26">
@@ -1101,11 +1101,11 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>35</v>
+        <v>35.85</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>-5.66</v>
+        <v>-3.37</v>
       </c>
     </row>
     <row r="27">
@@ -1127,11 +1127,11 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>30.15</v>
+        <v>34</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>-11.97</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="28">
@@ -1153,11 +1153,11 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>70.95</v>
+        <v>69.05</v>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>-4.06</v>
+        <v>-6.63</v>
       </c>
     </row>
     <row r="29">
@@ -1179,11 +1179,11 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>-3.72</v>
+        <v>-4.67</v>
       </c>
     </row>
     <row r="30">
@@ -1205,11 +1205,11 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>142.9</v>
+        <v>142.8</v>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>-0.07000000000000001</v>
       </c>
     </row>
     <row r="31">
@@ -1231,11 +1231,11 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>24.05</v>
+        <v>24.17</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1257,11 +1257,11 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>-1.9</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="33">
@@ -1283,11 +1283,11 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>111.1</v>
+        <v>113</v>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>-2.84</v>
+        <v>-1.18</v>
       </c>
     </row>
     <row r="34">
@@ -1309,11 +1309,11 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>5.32</v>
+        <v>5.62</v>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>-7.32</v>
+        <v>-2.09</v>
       </c>
     </row>
     <row r="35">
@@ -1361,11 +1361,11 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>343.15</v>
+        <v>342.9</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>-4.92</v>
+        <v>-4.99</v>
       </c>
     </row>
     <row r="37">
@@ -1387,11 +1387,11 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>12.84</v>
+        <v>12.4</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>-1.83</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="38">
@@ -1413,11 +1413,11 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>17.32</v>
+        <v>17.88</v>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>-3.24</v>
+        <v>-0.11</v>
       </c>
     </row>
     <row r="39">
@@ -1439,11 +1439,11 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>27.3</v>
+        <v>24.75</v>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>-9.34</v>
       </c>
     </row>
     <row r="40">
@@ -1465,11 +1465,11 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>46.05</v>
+        <v>47.34</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>-2.54</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="41">
@@ -1491,11 +1491,11 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>179.49</v>
+        <v>186</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>-5.03</v>
+        <v>-1.59</v>
       </c>
     </row>
     <row r="42">
@@ -1543,11 +1543,11 @@
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>27.45</v>
+        <v>28.25</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>-7.58</v>
+        <v>-4.88</v>
       </c>
     </row>
     <row r="44">
@@ -1595,11 +1595,11 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>3.64</v>
+        <v>3.69</v>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>-1.62</v>
+        <v>-0.27</v>
       </c>
     </row>
     <row r="46">
@@ -1621,11 +1621,11 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>1.95</v>
+        <v>1.96</v>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>-6.25</v>
+        <v>-5.77</v>
       </c>
     </row>
     <row r="47">
@@ -1647,11 +1647,11 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>525.15</v>
+        <v>533.3</v>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>3.99</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="48">
@@ -1699,11 +1699,11 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>6.99</v>
+        <v>7.75</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>-7.42</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="50">
@@ -1751,11 +1751,11 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>139.99</v>
+        <v>139</v>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>-3.74</v>
+        <v>-4.42</v>
       </c>
     </row>
     <row r="52">
@@ -1777,11 +1777,11 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>6.98</v>
+        <v>6.97</v>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>0.43</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="53">
@@ -1803,11 +1803,11 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>49.4</v>
+        <v>51.2</v>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>-2.83</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="54">
@@ -1829,11 +1829,11 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>10.92</v>
+        <v>11.32</v>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>-3.45</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="55">
@@ -1907,11 +1907,11 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>544.9</v>
+        <v>550</v>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>-4.79</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="58">
@@ -1933,11 +1933,11 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>24</v>
+        <v>24.9</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>-7.51</v>
+        <v>-4.05</v>
       </c>
     </row>
     <row r="59">
@@ -1959,11 +1959,11 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>135</v>
+        <v>138.7</v>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>8.43</v>
+        <v>11.41</v>
       </c>
     </row>
     <row r="60">
@@ -1985,11 +1985,11 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>139.69</v>
+        <v>141</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>-2.59</v>
+        <v>-1.67</v>
       </c>
     </row>
     <row r="61">
@@ -2037,11 +2037,11 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>20.66</v>
+        <v>21.89</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>-4.35</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="63">
@@ -2089,11 +2089,11 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>38</v>
+        <v>38.5</v>
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>-2.56</v>
+        <v>-1.28</v>
       </c>
     </row>
     <row r="65">
@@ -2115,11 +2115,11 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>35.31</v>
+        <v>36.05</v>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>-6.59</v>
+        <v>-4.63</v>
       </c>
     </row>
     <row r="66">
@@ -2141,11 +2141,11 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>53.35</v>
+        <v>55.52</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>-2.65</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="67">
@@ -2167,11 +2167,11 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>11.03</v>
+        <v>10.8</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>12.55</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="68">
@@ -2193,11 +2193,11 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>7.7</v>
+        <v>8.08</v>
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>-5.87</v>
+        <v>-1.22</v>
       </c>
     </row>
     <row r="69">
@@ -2219,11 +2219,11 @@
         <v>0</v>
       </c>
       <c r="F69" t="n">
-        <v>12.78</v>
+        <v>13.46</v>
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>-1.54</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="70">
@@ -2271,11 +2271,11 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>1.48</v>
+        <v>1.5</v>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>0</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="72">
@@ -2297,11 +2297,11 @@
         <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>111.77</v>
+        <v>114</v>
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>-4.88</v>
+        <v>-2.98</v>
       </c>
     </row>
     <row r="73">
@@ -2323,11 +2323,11 @@
         <v>0</v>
       </c>
       <c r="F73" t="n">
-        <v>442</v>
+        <v>444.9</v>
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>-3.49</v>
+        <v>-2.86</v>
       </c>
     </row>
     <row r="74">
@@ -2349,11 +2349,11 @@
         <v>0</v>
       </c>
       <c r="F74" t="n">
-        <v>62.17</v>
+        <v>62</v>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>-1.32</v>
+        <v>-1.59</v>
       </c>
     </row>
     <row r="75">
@@ -2375,11 +2375,11 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>92.70999999999999</v>
+        <v>98</v>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>6.56</v>
+        <v>12.64</v>
       </c>
     </row>
     <row r="76">
@@ -2401,11 +2401,11 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>-5.43</v>
+        <v>-4.35</v>
       </c>
     </row>
     <row r="77">
@@ -2427,11 +2427,11 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>5.95</v>
+        <v>5.97</v>
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>0.85</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="78">
@@ -2479,11 +2479,11 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>24.7</v>
+        <v>26.65</v>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>-7.84</v>
+        <v>-0.5600000000000001</v>
       </c>
     </row>
     <row r="80">
@@ -2505,11 +2505,11 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>15.8</v>
+        <v>15.85</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>-3.48</v>
+        <v>-3.18</v>
       </c>
     </row>
     <row r="81">
@@ -2531,11 +2531,11 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>4.95</v>
+        <v>5.43</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>-4.62</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="82">
@@ -2557,11 +2557,11 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>848</v>
+        <v>881.5</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>-6.95</v>
+        <v>-3.27</v>
       </c>
     </row>
     <row r="83">
@@ -2583,11 +2583,11 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>4.24</v>
+        <v>4.3</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>-3.85</v>
+        <v>-2.49</v>
       </c>
     </row>
     <row r="84">
@@ -2609,11 +2609,11 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>51.37</v>
+        <v>53.43</v>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>12.01</v>
+        <v>16.51</v>
       </c>
     </row>
     <row r="85">
@@ -2635,11 +2635,11 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>14289</v>
+        <v>13925</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>-3.43</v>
+        <v>-5.89</v>
       </c>
     </row>
     <row r="86">
@@ -2661,11 +2661,11 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>124.77</v>
+        <v>127.15</v>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>-5.44</v>
+        <v>-3.64</v>
       </c>
     </row>
     <row r="87">
@@ -2687,11 +2687,11 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>115.58</v>
+        <v>119.9</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>-3.68</v>
+        <v>-0.08</v>
       </c>
     </row>
     <row r="88">
@@ -2713,11 +2713,11 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>2.13</v>
+        <v>2</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>-2.74</v>
+        <v>-8.68</v>
       </c>
     </row>
     <row r="89">
@@ -2765,11 +2765,11 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>-3.58</v>
+        <v>-8.1</v>
       </c>
     </row>
     <row r="91">
@@ -2791,11 +2791,11 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>138</v>
+        <v>138.11</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>-6.66</v>
+        <v>-6.58</v>
       </c>
     </row>
     <row r="92">
@@ -2817,11 +2817,11 @@
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>8.49</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>-2.97</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="93">
@@ -2843,11 +2843,11 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>48.48</v>
+        <v>48.31</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>-1.96</v>
+        <v>-2.31</v>
       </c>
     </row>
     <row r="94">
@@ -2869,11 +2869,11 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>55.7</v>
+        <v>58.01</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>-3.63</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="95">
@@ -2895,11 +2895,11 @@
         <v>0</v>
       </c>
       <c r="F95" t="n">
-        <v>740.4</v>
+        <v>772.35</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>-1.93</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="96">
@@ -2921,11 +2921,11 @@
         <v>0</v>
       </c>
       <c r="F96" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="n">
-        <v>-2.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -2973,11 +2973,11 @@
         <v>0</v>
       </c>
       <c r="F98" t="n">
-        <v>6.87</v>
+        <v>6.97</v>
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>-3.24</v>
+        <v>-1.83</v>
       </c>
     </row>
     <row r="99">
@@ -2999,11 +2999,11 @@
         <v>0</v>
       </c>
       <c r="F99" t="n">
-        <v>10.38</v>
+        <v>10.6</v>
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>-2.54</v>
+        <v>-0.47</v>
       </c>
     </row>
     <row r="100">
@@ -3025,11 +3025,11 @@
         <v>0</v>
       </c>
       <c r="F100" t="n">
-        <v>8.15</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>-2.98</v>
+        <v>-3.21</v>
       </c>
     </row>
     <row r="101">
@@ -3051,11 +3051,11 @@
         <v>0</v>
       </c>
       <c r="F101" t="n">
-        <v>175</v>
+        <v>175.05</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>2.34</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="102">
@@ -3103,11 +3103,11 @@
         <v>0</v>
       </c>
       <c r="F103" t="n">
-        <v>23.89</v>
+        <v>24.5</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>-2.49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -3129,11 +3129,11 @@
         <v>0</v>
       </c>
       <c r="F104" t="n">
-        <v>0.42</v>
+        <v>0.41</v>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>-2.33</v>
+        <v>-4.65</v>
       </c>
     </row>
     <row r="105">
@@ -3155,11 +3155,11 @@
         <v>0</v>
       </c>
       <c r="F105" t="n">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>-2.33</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="106">
@@ -3181,11 +3181,11 @@
         <v>0</v>
       </c>
       <c r="F106" t="n">
-        <v>155.25</v>
+        <v>159</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>-4.17</v>
+        <v>-1.85</v>
       </c>
     </row>
     <row r="107">
@@ -3207,11 +3207,11 @@
         <v>0</v>
       </c>
       <c r="F107" t="n">
-        <v>10.05</v>
+        <v>10.01</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="108">
@@ -3233,11 +3233,11 @@
         <v>0</v>
       </c>
       <c r="F108" t="n">
-        <v>145.05</v>
+        <v>145.85</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="n">
-        <v>-3.17</v>
+        <v>-2.64</v>
       </c>
     </row>
     <row r="109">
@@ -3259,11 +3259,11 @@
         <v>0</v>
       </c>
       <c r="F109" t="n">
-        <v>4.35</v>
+        <v>4.86</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="n">
-        <v>-2.68</v>
+        <v>8.720000000000001</v>
       </c>
     </row>
     <row r="110">
@@ -3285,11 +3285,11 @@
         <v>0</v>
       </c>
       <c r="F110" t="n">
-        <v>11.64</v>
+        <v>11.65</v>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>-3.72</v>
+        <v>-3.64</v>
       </c>
     </row>
     <row r="111">
@@ -3311,11 +3311,11 @@
         <v>0</v>
       </c>
       <c r="F111" t="n">
-        <v>343.25</v>
+        <v>365</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>-4.39</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="112">
@@ -3337,11 +3337,11 @@
         <v>0</v>
       </c>
       <c r="F112" t="n">
-        <v>14.69</v>
+        <v>14.67</v>
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>-1.28</v>
+        <v>-1.41</v>
       </c>
     </row>
     <row r="113">
@@ -3363,11 +3363,11 @@
         <v>0</v>
       </c>
       <c r="F113" t="n">
-        <v>930.05</v>
+        <v>965</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>-1.97</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="114">
@@ -3389,11 +3389,11 @@
         <v>0</v>
       </c>
       <c r="F114" t="n">
-        <v>4.11</v>
+        <v>4.08</v>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>-0.96</v>
+        <v>-1.69</v>
       </c>
     </row>
     <row r="115">
@@ -3415,11 +3415,11 @@
         <v>0</v>
       </c>
       <c r="F115" t="n">
-        <v>3.13</v>
+        <v>3.32</v>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>-2.8</v>
+        <v>3.11</v>
       </c>
     </row>
     <row r="116">
@@ -3441,11 +3441,11 @@
         <v>0</v>
       </c>
       <c r="F116" t="n">
-        <v>51.98</v>
+        <v>52.36</v>
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>-2.29</v>
+        <v>-1.58</v>
       </c>
     </row>
     <row r="117">
@@ -3467,11 +3467,11 @@
         <v>0</v>
       </c>
       <c r="F117" t="n">
-        <v>77.25</v>
+        <v>80</v>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>0.32</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="118">
@@ -3493,11 +3493,11 @@
         <v>0</v>
       </c>
       <c r="F118" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>0</v>
+        <v>2.13</v>
       </c>
     </row>
     <row r="119">
@@ -3519,11 +3519,11 @@
         <v>0</v>
       </c>
       <c r="F119" t="n">
-        <v>59.8</v>
+        <v>60.75</v>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>-3.55</v>
+        <v>-2.02</v>
       </c>
     </row>
     <row r="120">
@@ -3545,11 +3545,11 @@
         <v>0</v>
       </c>
       <c r="F120" t="n">
-        <v>2.75</v>
+        <v>2.79</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>-3.51</v>
+        <v>-2.11</v>
       </c>
     </row>
     <row r="121">
@@ -3571,11 +3571,11 @@
         <v>0</v>
       </c>
       <c r="F121" t="n">
-        <v>72.61</v>
+        <v>75.5</v>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>-3.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
@@ -3597,11 +3597,11 @@
         <v>0</v>
       </c>
       <c r="F122" t="n">
-        <v>13.65</v>
+        <v>13.81</v>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>-3.05</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="123">
@@ -3623,11 +3623,11 @@
         <v>0</v>
       </c>
       <c r="F123" t="n">
-        <v>20.75</v>
+        <v>21.7</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>-4.99</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="124">
@@ -3649,11 +3649,11 @@
         <v>0</v>
       </c>
       <c r="F124" t="n">
-        <v>577.3</v>
+        <v>584</v>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>-1.31</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="125">
@@ -3675,11 +3675,11 @@
         <v>0</v>
       </c>
       <c r="F125" t="n">
-        <v>20.73</v>
+        <v>20.39</v>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>0</v>
+        <v>-1.64</v>
       </c>
     </row>
     <row r="126">
@@ -3701,11 +3701,11 @@
         <v>0</v>
       </c>
       <c r="F126" t="n">
-        <v>151.2</v>
+        <v>156.5</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>-4.3</v>
+        <v>-0.95</v>
       </c>
     </row>
     <row r="127">
@@ -3753,11 +3753,11 @@
         <v>0</v>
       </c>
       <c r="F128" t="n">
-        <v>34.3</v>
+        <v>35.9</v>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>0</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="129">
@@ -3779,11 +3779,11 @@
         <v>0</v>
       </c>
       <c r="F129" t="n">
-        <v>33.6</v>
+        <v>34.7</v>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>-3.72</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="130">
@@ -3831,11 +3831,11 @@
         <v>0</v>
       </c>
       <c r="F131" t="n">
-        <v>4.76</v>
+        <v>4.81</v>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>-2.26</v>
+        <v>-1.23</v>
       </c>
     </row>
     <row r="132">
@@ -3857,11 +3857,11 @@
         <v>0</v>
       </c>
       <c r="F132" t="n">
-        <v>2.13</v>
+        <v>2.19</v>
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>-2.29</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="133">
@@ -3883,11 +3883,11 @@
         <v>0</v>
       </c>
       <c r="F133" t="n">
-        <v>57.13</v>
+        <v>62</v>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>-3.66</v>
+        <v>4.55</v>
       </c>
     </row>
     <row r="134">
@@ -3909,11 +3909,11 @@
         <v>0</v>
       </c>
       <c r="F134" t="n">
-        <v>74.52</v>
+        <v>78.5</v>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>-3.07</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="135">
@@ -3935,11 +3935,11 @@
         <v>0</v>
       </c>
       <c r="F135" t="n">
-        <v>385</v>
+        <v>409.7</v>
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="n">
-        <v>-3.74</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="136">
@@ -3961,11 +3961,11 @@
         <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>20.18</v>
+        <v>20.3</v>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>-2.18</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="137">
@@ -3987,11 +3987,11 @@
         <v>0</v>
       </c>
       <c r="F137" t="n">
-        <v>19.26</v>
+        <v>21.89</v>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="n">
-        <v>-1.13</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="138">
@@ -4013,11 +4013,11 @@
         <v>0</v>
       </c>
       <c r="F138" t="n">
-        <v>155.68</v>
+        <v>165</v>
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="n">
-        <v>-2.61</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="139">
@@ -4039,11 +4039,11 @@
         <v>0</v>
       </c>
       <c r="F139" t="n">
-        <v>231.06</v>
+        <v>237.89</v>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="n">
-        <v>-2.92</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="140">
@@ -4065,11 +4065,11 @@
         <v>0</v>
       </c>
       <c r="F140" t="n">
-        <v>8.779999999999999</v>
+        <v>9</v>
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="n">
-        <v>-2.34</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="141">
@@ -4091,11 +4091,11 @@
         <v>0</v>
       </c>
       <c r="F141" t="n">
-        <v>20.55</v>
+        <v>21.2</v>
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="n">
-        <v>-2.61</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="142">
@@ -4117,11 +4117,11 @@
         <v>0</v>
       </c>
       <c r="F142" t="n">
-        <v>4.71</v>
+        <v>4.74</v>
       </c>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="n">
-        <v>-3.48</v>
+        <v>-2.87</v>
       </c>
     </row>
     <row r="143">
@@ -4143,11 +4143,11 @@
         <v>0</v>
       </c>
       <c r="F143" t="n">
-        <v>2.39</v>
+        <v>2.45</v>
       </c>
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="n">
-        <v>-2.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -4169,11 +4169,11 @@
         <v>0</v>
       </c>
       <c r="F144" t="n">
-        <v>1.18</v>
+        <v>1.22</v>
       </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="n">
-        <v>-4.84</v>
+        <v>-1.61</v>
       </c>
     </row>
     <row r="145">
@@ -4195,11 +4195,11 @@
         <v>0</v>
       </c>
       <c r="F145" t="n">
-        <v>2.41</v>
+        <v>2.51</v>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="n">
-        <v>-2.82</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="146">
@@ -4221,11 +4221,11 @@
         <v>0</v>
       </c>
       <c r="F146" t="n">
-        <v>99.95</v>
+        <v>103</v>
       </c>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="n">
-        <v>-1.91</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="147">
@@ -4247,11 +4247,11 @@
         <v>0</v>
       </c>
       <c r="F147" t="n">
-        <v>24.55</v>
+        <v>24.7</v>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="n">
-        <v>-1.76</v>
+        <v>-1.16</v>
       </c>
     </row>
     <row r="148">
@@ -4273,11 +4273,11 @@
         <v>0</v>
       </c>
       <c r="F148" t="n">
-        <v>70.03</v>
+        <v>73.48</v>
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="n">
-        <v>-2.72</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="149">
@@ -4299,11 +4299,11 @@
         <v>0</v>
       </c>
       <c r="F149" t="n">
-        <v>27.62</v>
+        <v>27.5</v>
       </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="n">
-        <v>-0.9</v>
+        <v>-1.33</v>
       </c>
     </row>
     <row r="150">
@@ -4325,11 +4325,11 @@
         <v>0</v>
       </c>
       <c r="F150" t="n">
-        <v>22.45</v>
+        <v>23.13</v>
       </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="n">
-        <v>-1.45</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="151">
@@ -4351,11 +4351,11 @@
         <v>0</v>
       </c>
       <c r="F151" t="n">
-        <v>216.12</v>
+        <v>219.25</v>
       </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="n">
-        <v>-2.56</v>
+        <v>-1.15</v>
       </c>
     </row>
     <row r="152">
@@ -4377,11 +4377,11 @@
         <v>0</v>
       </c>
       <c r="F152" t="n">
-        <v>446.5</v>
+        <v>482.35</v>
       </c>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="n">
-        <v>0.34</v>
+        <v>8.390000000000001</v>
       </c>
     </row>
     <row r="153">
@@ -4403,11 +4403,11 @@
         <v>0</v>
       </c>
       <c r="F153" t="n">
-        <v>85.52</v>
+        <v>86.94</v>
       </c>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="n">
-        <v>-2.21</v>
+        <v>-0.58</v>
       </c>
     </row>
     <row r="154">
@@ -4429,11 +4429,11 @@
         <v>0</v>
       </c>
       <c r="F154" t="n">
-        <v>591.2</v>
+        <v>602</v>
       </c>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="n">
-        <v>-1.46</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="155">
@@ -4455,11 +4455,11 @@
         <v>0</v>
       </c>
       <c r="F155" t="n">
-        <v>13.67</v>
+        <v>14</v>
       </c>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="n">
-        <v>-1.94</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="156">
@@ -4481,11 +4481,11 @@
         <v>0</v>
       </c>
       <c r="F156" t="n">
-        <v>157.51</v>
+        <v>156</v>
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="n">
-        <v>-2.17</v>
+        <v>-3.11</v>
       </c>
     </row>
     <row r="157">
@@ -4507,11 +4507,11 @@
         <v>0</v>
       </c>
       <c r="F157" t="n">
-        <v>7.25</v>
+        <v>7.7</v>
       </c>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="n">
-        <v>-0.55</v>
+        <v>5.62</v>
       </c>
     </row>
     <row r="158">
@@ -4533,11 +4533,11 @@
         <v>0</v>
       </c>
       <c r="F158" t="n">
-        <v>20.7</v>
+        <v>22.1</v>
       </c>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="n">
-        <v>-2.13</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="159">
@@ -4559,11 +4559,11 @@
         <v>0</v>
       </c>
       <c r="F159" t="n">
-        <v>12.93</v>
+        <v>13.25</v>
       </c>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="n">
-        <v>-2.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160">
@@ -4585,11 +4585,11 @@
         <v>0</v>
       </c>
       <c r="F160" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="n">
-        <v>-4</v>
+        <v>-2.67</v>
       </c>
     </row>
     <row r="161">
@@ -4611,11 +4611,11 @@
         <v>0</v>
       </c>
       <c r="F161" t="n">
-        <v>64.7</v>
+        <v>64.56</v>
       </c>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="n">
-        <v>-1.58</v>
+        <v>-1.79</v>
       </c>
     </row>
     <row r="162">
@@ -4637,11 +4637,11 @@
         <v>0</v>
       </c>
       <c r="F162" t="n">
-        <v>7.5</v>
+        <v>7.98</v>
       </c>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="n">
-        <v>-2.47</v>
+        <v>3.77</v>
       </c>
     </row>
     <row r="163">
@@ -4663,11 +4663,11 @@
         <v>0</v>
       </c>
       <c r="F163" t="n">
-        <v>45.83</v>
+        <v>46.31</v>
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="n">
-        <v>-2.49</v>
+        <v>-1.47</v>
       </c>
     </row>
     <row r="164">
@@ -4689,11 +4689,11 @@
         <v>0</v>
       </c>
       <c r="F164" t="n">
-        <v>66.91</v>
+        <v>68.75</v>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="n">
-        <v>-3.03</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="165">
@@ -4715,11 +4715,11 @@
         <v>0</v>
       </c>
       <c r="F165" t="n">
-        <v>241</v>
+        <v>247.5</v>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="n">
-        <v>-3.02</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="166">
@@ -4741,11 +4741,11 @@
         <v>0</v>
       </c>
       <c r="F166" t="n">
-        <v>11.53</v>
+        <v>12.19</v>
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="n">
-        <v>-6.03</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="167">
@@ -4767,11 +4767,11 @@
         <v>0</v>
       </c>
       <c r="F167" t="n">
-        <v>318</v>
+        <v>319.4</v>
       </c>
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="n">
-        <v>8.16</v>
+        <v>8.640000000000001</v>
       </c>
     </row>
     <row r="168">
@@ -4793,11 +4793,11 @@
         <v>0</v>
       </c>
       <c r="F168" t="n">
-        <v>218.82</v>
+        <v>231</v>
       </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="n">
-        <v>-0.41</v>
+        <v>5.13</v>
       </c>
     </row>
     <row r="169">
@@ -4819,11 +4819,11 @@
         <v>0</v>
       </c>
       <c r="F169" t="n">
-        <v>26.81</v>
+        <v>27.8</v>
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="n">
-        <v>-4.22</v>
+        <v>-0.68</v>
       </c>
     </row>
     <row r="170">
@@ -4845,11 +4845,11 @@
         <v>0</v>
       </c>
       <c r="F170" t="n">
-        <v>992.4</v>
+        <v>1014.75</v>
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="n">
-        <v>5.56</v>
+        <v>7.93</v>
       </c>
     </row>
     <row r="171">
@@ -4871,11 +4871,11 @@
         <v>0</v>
       </c>
       <c r="F171" t="n">
-        <v>315.3</v>
+        <v>319.8</v>
       </c>
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="n">
-        <v>-1.44</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="172">
@@ -4897,11 +4897,11 @@
         <v>0</v>
       </c>
       <c r="F172" t="n">
-        <v>119.3</v>
+        <v>117.12</v>
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="n">
-        <v>14.18</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="173">
@@ -4923,11 +4923,11 @@
         <v>0</v>
       </c>
       <c r="F173" t="n">
-        <v>20.42</v>
+        <v>21.15</v>
       </c>
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="n">
-        <v>-3.22</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="174">
@@ -4949,11 +4949,11 @@
         <v>0</v>
       </c>
       <c r="F174" t="n">
-        <v>226</v>
+        <v>238.5</v>
       </c>
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="n">
-        <v>-2.16</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="175">
@@ -4975,11 +4975,11 @@
         <v>0</v>
       </c>
       <c r="F175" t="n">
-        <v>0.88</v>
+        <v>0.98</v>
       </c>
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="n">
-        <v>-3.3</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="176">
@@ -5053,11 +5053,11 @@
         <v>0</v>
       </c>
       <c r="F178" t="n">
-        <v>122.47</v>
+        <v>123.95</v>
       </c>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
-        <v>-0.42</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="179">
@@ -5079,11 +5079,11 @@
         <v>0</v>
       </c>
       <c r="F179" t="n">
-        <v>67.03</v>
+        <v>71</v>
       </c>
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="n">
-        <v>-0.62</v>
+        <v>5.26</v>
       </c>
     </row>
     <row r="180">
@@ -5105,11 +5105,11 @@
         <v>0</v>
       </c>
       <c r="F180" t="n">
-        <v>57.1</v>
+        <v>58.98</v>
       </c>
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="n">
-        <v>-0.68</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="181">
@@ -5157,11 +5157,11 @@
         <v>0</v>
       </c>
       <c r="F182" t="n">
-        <v>465.6</v>
+        <v>476.1</v>
       </c>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="n">
-        <v>-2.59</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="183">
@@ -5183,11 +5183,11 @@
         <v>0</v>
       </c>
       <c r="F183" t="n">
-        <v>182.77</v>
+        <v>182.02</v>
       </c>
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="n">
-        <v>-3.3</v>
+        <v>-3.69</v>
       </c>
     </row>
     <row r="184">
@@ -5209,11 +5209,11 @@
         <v>0</v>
       </c>
       <c r="F184" t="n">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="n">
-        <v>-1.26</v>
+        <v>-5.48</v>
       </c>
     </row>
     <row r="185">
@@ -5235,11 +5235,11 @@
         <v>0</v>
       </c>
       <c r="F185" t="n">
-        <v>83.09999999999999</v>
+        <v>80.25</v>
       </c>
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="n">
-        <v>-1.47</v>
+        <v>-4.85</v>
       </c>
     </row>
     <row r="186">
@@ -5261,11 +5261,11 @@
         <v>0</v>
       </c>
       <c r="F186" t="n">
-        <v>254.59</v>
+        <v>267.53</v>
       </c>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="n">
-        <v>-3.2</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="187">
@@ -5287,11 +5287,11 @@
         <v>0</v>
       </c>
       <c r="F187" t="n">
-        <v>354.5</v>
+        <v>366.1</v>
       </c>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="n">
-        <v>-3.12</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="188">
@@ -5313,11 +5313,11 @@
         <v>0</v>
       </c>
       <c r="F188" t="n">
-        <v>15.32</v>
+        <v>15.99</v>
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="n">
-        <v>-3.53</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="189">
@@ -5339,11 +5339,11 @@
         <v>0</v>
       </c>
       <c r="F189" t="n">
-        <v>227.79</v>
+        <v>237.01</v>
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="n">
-        <v>-2.24</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="190">
@@ -5365,11 +5365,11 @@
         <v>0</v>
       </c>
       <c r="F190" t="n">
-        <v>7.55</v>
+        <v>7.81</v>
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="n">
-        <v>0.67</v>
+        <v>4.13</v>
       </c>
     </row>
     <row r="191">
@@ -5391,11 +5391,11 @@
         <v>0</v>
       </c>
       <c r="F191" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="n">
-        <v>-4</v>
+        <v>4</v>
       </c>
     </row>
     <row r="192">
@@ -5417,11 +5417,11 @@
         <v>0</v>
       </c>
       <c r="F192" t="n">
-        <v>478</v>
+        <v>493.75</v>
       </c>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="n">
-        <v>-2.86</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="193">
@@ -5443,11 +5443,11 @@
         <v>0</v>
       </c>
       <c r="F193" t="n">
-        <v>1.3</v>
+        <v>1.35</v>
       </c>
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="n">
-        <v>0</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="194">
@@ -5469,11 +5469,11 @@
         <v>0</v>
       </c>
       <c r="F194" t="n">
-        <v>31.88</v>
+        <v>32.5</v>
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="n">
-        <v>-1.15</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="195">
@@ -5495,11 +5495,11 @@
         <v>0</v>
       </c>
       <c r="F195" t="n">
-        <v>4.04</v>
+        <v>4.05</v>
       </c>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="n">
-        <v>3.86</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="196">
@@ -5521,11 +5521,11 @@
         <v>0</v>
       </c>
       <c r="F196" t="n">
-        <v>2.57</v>
+        <v>2.7</v>
       </c>
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="n">
-        <v>-3.75</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="197">
@@ -5547,11 +5547,11 @@
         <v>0</v>
       </c>
       <c r="F197" t="n">
-        <v>1.33</v>
+        <v>1.36</v>
       </c>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="n">
-        <v>-2.92</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="198">
@@ -5573,11 +5573,11 @@
         <v>0</v>
       </c>
       <c r="F198" t="n">
-        <v>4.15</v>
+        <v>4.11</v>
       </c>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="n">
-        <v>-1.19</v>
+        <v>-2.14</v>
       </c>
     </row>
     <row r="199">
@@ -5599,11 +5599,11 @@
         <v>0</v>
       </c>
       <c r="F199" t="n">
-        <v>54.67</v>
+        <v>57.7</v>
       </c>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="n">
-        <v>-2.55</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="200">
@@ -5625,11 +5625,11 @@
         <v>0</v>
       </c>
       <c r="F200" t="n">
-        <v>15.82</v>
+        <v>16.29</v>
       </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="n">
-        <v>-1.12</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="201">
@@ -5651,11 +5651,11 @@
         <v>0</v>
       </c>
       <c r="F201" t="n">
-        <v>74.44</v>
+        <v>76.05</v>
       </c>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="n">
-        <v>-2.63</v>
+        <v>-0.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-04-14 05:41 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -477,11 +477,11 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>195.2</v>
+        <v>194.81</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>2.74</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="3">
@@ -503,11 +503,11 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>14.7</v>
+        <v>14.65</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>-0.34</v>
       </c>
     </row>
     <row r="4">
@@ -555,11 +555,11 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>75.59999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>0.13</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="6">
@@ -607,11 +607,11 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>71.73</v>
+        <v>72</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>-9.199999999999999</v>
+        <v>-8.859999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -659,11 +659,11 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>20.78</v>
+        <v>20.16</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>-4.2</v>
+        <v>-7.05</v>
       </c>
     </row>
     <row r="10">
@@ -685,11 +685,11 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>7.27</v>
+        <v>6.36</v>
       </c>
     </row>
     <row r="11">
@@ -711,11 +711,11 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>21.11</v>
+        <v>22.18</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>-9.75</v>
+        <v>-5.17</v>
       </c>
     </row>
     <row r="12">
@@ -763,11 +763,11 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>53.4</v>
+        <v>54.4</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>-2.55</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="14">
@@ -789,11 +789,11 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>7.05</v>
+        <v>7.2</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>-5.87</v>
+        <v>-3.87</v>
       </c>
     </row>
     <row r="15">
@@ -815,11 +815,11 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>107.8</v>
+        <v>105.45</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>-2</v>
+        <v>-4.14</v>
       </c>
     </row>
     <row r="16">
@@ -841,11 +841,11 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>47.28</v>
+        <v>45.94</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>-1.27</v>
+        <v>-4.07</v>
       </c>
     </row>
     <row r="17">
@@ -867,11 +867,11 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>20.95</v>
+        <v>21</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>-0.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -893,11 +893,11 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>4.72</v>
+        <v>4.56</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>-6.35</v>
+        <v>-9.52</v>
       </c>
     </row>
     <row r="19">
@@ -1049,11 +1049,11 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>35.75</v>
+        <v>36.84</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>-3.22</v>
+        <v>-0.27</v>
       </c>
     </row>
     <row r="25">
@@ -1075,11 +1075,11 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>3.3</v>
+        <v>3.22</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>-2.65</v>
+        <v>-5.01</v>
       </c>
     </row>
     <row r="26">
@@ -1309,11 +1309,11 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>22.55</v>
+        <v>21.5</v>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>-4.66</v>
       </c>
     </row>
     <row r="35">
@@ -1335,11 +1335,11 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>13.38</v>
+        <v>12.86</v>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>-4.43</v>
+        <v>-8.140000000000001</v>
       </c>
     </row>
     <row r="36">
@@ -1361,11 +1361,11 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>117.99</v>
+        <v>111.11</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>-1.66</v>
+        <v>-7.39</v>
       </c>
     </row>
     <row r="37">
@@ -1491,11 +1491,11 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>14.7</v>
+        <v>15.39</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>-6.37</v>
+        <v>-1.97</v>
       </c>
     </row>
     <row r="42">
@@ -1595,11 +1595,11 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>23.68</v>
+        <v>23.21</v>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>-1.29</v>
+        <v>-3.25</v>
       </c>
     </row>
     <row r="46">
@@ -1621,11 +1621,11 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>32.4</v>
+        <v>31.11</v>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>-4.4</v>
+        <v>-8.199999999999999</v>
       </c>
     </row>
     <row r="47">
@@ -1699,11 +1699,11 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>5.78</v>
+        <v>5.55</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>-4.46</v>
+        <v>-8.26</v>
       </c>
     </row>
     <row r="50">
@@ -1751,11 +1751,11 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>2.41</v>
+        <v>2.3</v>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>-1.63</v>
+        <v>-6.12</v>
       </c>
     </row>
     <row r="52">
@@ -1777,11 +1777,11 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>2.11</v>
+        <v>2.09</v>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>-4.52</v>
+        <v>-5.43</v>
       </c>
     </row>
     <row r="53">
@@ -1803,11 +1803,11 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>1.68</v>
+        <v>1.73</v>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>-2.33</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="54">
@@ -1829,11 +1829,11 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>164.02</v>
+        <v>165.5</v>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>-0.47</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="55">
@@ -1855,11 +1855,11 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>60.5</v>
+        <v>61</v>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>-3.82</v>
+        <v>-3.02</v>
       </c>
     </row>
     <row r="56">
@@ -1881,11 +1881,11 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>21</v>
+        <v>21.45</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>-1.41</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="57">
@@ -1907,11 +1907,11 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>138.8</v>
+        <v>138.1</v>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>-1.53</v>
+        <v>-2.02</v>
       </c>
     </row>
     <row r="58">
@@ -1933,11 +1933,11 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>9.609999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>-1.94</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="59">
@@ -1959,11 +1959,11 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>1.33</v>
+        <v>1.36</v>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>-2.92</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="60">
@@ -1985,11 +1985,11 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>76.65000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>-3.58</v>
+        <v>-3.21</v>
       </c>
     </row>
     <row r="61">
@@ -2011,11 +2011,11 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>198.16</v>
+        <v>192.5</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>4.3</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="62">
@@ -2037,11 +2037,11 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>220.45</v>
+        <v>219.11</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>-5.75</v>
+        <v>-6.32</v>
       </c>
     </row>
     <row r="63">
@@ -2063,11 +2063,11 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>16.18</v>
+        <v>15.64</v>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>-4.71</v>
+        <v>-7.89</v>
       </c>
     </row>
     <row r="64">
@@ -2089,11 +2089,11 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>9.199999999999999</v>
+        <v>9.17</v>
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>10.18</v>
+        <v>9.82</v>
       </c>
     </row>
     <row r="65">
@@ -2141,11 +2141,11 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>515.95</v>
+        <v>481.5</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>14.66</v>
+        <v>7</v>
       </c>
     </row>
     <row r="67">
@@ -2167,11 +2167,11 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>9.18</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>-6.33</v>
+        <v>-7.65</v>
       </c>
     </row>
     <row r="68">
@@ -2193,11 +2193,11 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>105</v>
+        <v>106.35</v>
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>-2.6</v>
+        <v>-1.35</v>
       </c>
     </row>
     <row r="69">
@@ -2219,11 +2219,11 @@
         <v>0</v>
       </c>
       <c r="F69" t="n">
-        <v>7.27</v>
+        <v>7.36</v>
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>-4.34</v>
+        <v>-3.16</v>
       </c>
     </row>
     <row r="70">
@@ -2245,11 +2245,11 @@
         <v>0</v>
       </c>
       <c r="F70" t="n">
-        <v>42.5</v>
+        <v>41.9</v>
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>-3.17</v>
+        <v>-4.53</v>
       </c>
     </row>
     <row r="71">
@@ -2297,11 +2297,11 @@
         <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>60.25</v>
+        <v>59.32</v>
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>1.26</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="73">
@@ -2375,11 +2375,11 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>1839</v>
+        <v>1839.9</v>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>1.04</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="76">
@@ -2401,11 +2401,11 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>0.98</v>
+        <v>1.03</v>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>-6.67</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="77">
@@ -2427,11 +2427,11 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>326.45</v>
+        <v>321</v>
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>-1.97</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="78">
@@ -2453,11 +2453,11 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>65</v>
+        <v>64.5</v>
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>-2.69</v>
+        <v>-3.44</v>
       </c>
     </row>
     <row r="79">
@@ -2505,11 +2505,11 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>2399.4</v>
+        <v>2397.8</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>0.23</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="81">
@@ -2531,11 +2531,11 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>29.53</v>
+        <v>29.26</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>-3.81</v>
+        <v>-4.69</v>
       </c>
     </row>
     <row r="82">
@@ -2557,11 +2557,11 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>28.5</v>
+        <v>29</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>-1.76</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="83">
@@ -2609,11 +2609,11 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>1.59</v>
+        <v>1.57</v>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>-0.63</v>
+        <v>-1.88</v>
       </c>
     </row>
     <row r="85">
@@ -2635,11 +2635,11 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>17.98</v>
+        <v>18.59</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>-0.39</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="86">
@@ -2661,11 +2661,11 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>56.48</v>
+        <v>54.25</v>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>-1.52</v>
+        <v>-5.41</v>
       </c>
     </row>
     <row r="87">
@@ -2687,11 +2687,11 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>40.56</v>
+        <v>40.94</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>-2.85</v>
+        <v>-1.94</v>
       </c>
     </row>
     <row r="88">
@@ -2739,11 +2739,11 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>70.38</v>
+        <v>69</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>-0.37</v>
+        <v>-2.32</v>
       </c>
     </row>
     <row r="90">
@@ -2765,11 +2765,11 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>10.79</v>
+        <v>10.61</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>0.84</v>
+        <v>-0.84</v>
       </c>
     </row>
     <row r="91">
@@ -2791,11 +2791,11 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>82.90000000000001</v>
+        <v>81.66</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>1.22</v>
+        <v>-0.29</v>
       </c>
     </row>
     <row r="92">
@@ -2817,11 +2817,11 @@
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>5.04</v>
+        <v>4.98</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>-0.79</v>
+        <v>-1.97</v>
       </c>
     </row>
     <row r="93">
@@ -2843,11 +2843,11 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>67.12</v>
+        <v>68</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>-3.29</v>
+        <v>-2.02</v>
       </c>
     </row>
     <row r="94">
@@ -2869,11 +2869,11 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>622.3</v>
+        <v>617.3</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>1.19</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="95">
@@ -2895,11 +2895,11 @@
         <v>0</v>
       </c>
       <c r="F95" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>0</v>
+        <v>-2.08</v>
       </c>
     </row>
     <row r="96">
@@ -2947,11 +2947,11 @@
         <v>0</v>
       </c>
       <c r="F97" t="n">
-        <v>8.94</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>-2.72</v>
+        <v>-3.48</v>
       </c>
     </row>
     <row r="98">
@@ -2999,11 +2999,11 @@
         <v>0</v>
       </c>
       <c r="F99" t="n">
-        <v>1.44</v>
+        <v>1.58</v>
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>-6.49</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="100">
@@ -3025,11 +3025,11 @@
         <v>0</v>
       </c>
       <c r="F100" t="n">
-        <v>199.78</v>
+        <v>200.1</v>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>2.56</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="101">
@@ -3051,11 +3051,11 @@
         <v>0</v>
       </c>
       <c r="F101" t="n">
-        <v>76</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>-4.88</v>
+        <v>-4.38</v>
       </c>
     </row>
     <row r="102">
@@ -3077,11 +3077,11 @@
         <v>0</v>
       </c>
       <c r="F102" t="n">
-        <v>50.86</v>
+        <v>50.67</v>
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>-0.76</v>
+        <v>-1.13</v>
       </c>
     </row>
     <row r="103">
@@ -3103,11 +3103,11 @@
         <v>0</v>
       </c>
       <c r="F103" t="n">
-        <v>30.82</v>
+        <v>30.3</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>-3.69</v>
+        <v>-5.31</v>
       </c>
     </row>
     <row r="104">
@@ -3155,11 +3155,11 @@
         <v>0</v>
       </c>
       <c r="F105" t="n">
-        <v>27.65</v>
+        <v>27.95</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>-6.24</v>
+        <v>-5.22</v>
       </c>
     </row>
     <row r="106">
@@ -3181,11 +3181,11 @@
         <v>0</v>
       </c>
       <c r="F106" t="n">
-        <v>3.15</v>
+        <v>3.16</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>-2.78</v>
+        <v>-2.47</v>
       </c>
     </row>
     <row r="107">
@@ -3207,11 +3207,11 @@
         <v>0</v>
       </c>
       <c r="F107" t="n">
-        <v>2.8</v>
+        <v>2.69</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>2.94</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="108">
@@ -3233,11 +3233,11 @@
         <v>0</v>
       </c>
       <c r="F108" t="n">
-        <v>2.77</v>
+        <v>2.88</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="n">
-        <v>-1.07</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="109">
@@ -3259,11 +3259,11 @@
         <v>0</v>
       </c>
       <c r="F109" t="n">
-        <v>27.95</v>
+        <v>27.3</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="n">
-        <v>0.18</v>
+        <v>-2.15</v>
       </c>
     </row>
     <row r="110">
@@ -3285,11 +3285,11 @@
         <v>0</v>
       </c>
       <c r="F110" t="n">
-        <v>7.68</v>
+        <v>7.8</v>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>-3.64</v>
+        <v>-2.13</v>
       </c>
     </row>
     <row r="111">
@@ -3311,11 +3311,11 @@
         <v>0</v>
       </c>
       <c r="F111" t="n">
-        <v>5.47</v>
+        <v>5.44</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>-4.04</v>
+        <v>-4.56</v>
       </c>
     </row>
     <row r="112">
@@ -3363,11 +3363,11 @@
         <v>0</v>
       </c>
       <c r="F113" t="n">
-        <v>26.4</v>
+        <v>26.74</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>-2.94</v>
+        <v>-1.69</v>
       </c>
     </row>
     <row r="114">
@@ -3389,11 +3389,11 @@
         <v>0</v>
       </c>
       <c r="F114" t="n">
-        <v>15.37</v>
+        <v>15.41</v>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>-0.71</v>
+        <v>-0.45</v>
       </c>
     </row>
     <row r="115">
@@ -3467,11 +3467,11 @@
         <v>0</v>
       </c>
       <c r="F117" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>-6.56</v>
+        <v>-4.92</v>
       </c>
     </row>
     <row r="118">
@@ -3493,11 +3493,11 @@
         <v>0</v>
       </c>
       <c r="F118" t="n">
-        <v>30.21</v>
+        <v>30.4</v>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>-2.04</v>
+        <v>-1.43</v>
       </c>
     </row>
     <row r="119">
@@ -3519,11 +3519,11 @@
         <v>0</v>
       </c>
       <c r="F119" t="n">
-        <v>1.82</v>
+        <v>1.83</v>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>-1.62</v>
+        <v>-1.08</v>
       </c>
     </row>
     <row r="120">
@@ -3545,11 +3545,11 @@
         <v>0</v>
       </c>
       <c r="F120" t="n">
-        <v>4.2</v>
+        <v>4.33</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>-5.62</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="121">
@@ -3571,11 +3571,11 @@
         <v>0</v>
       </c>
       <c r="F121" t="n">
-        <v>1.29</v>
+        <v>1.26</v>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
-        <v>0.78</v>
+        <v>-1.56</v>
       </c>
     </row>
     <row r="122">
@@ -3597,11 +3597,11 @@
         <v>0</v>
       </c>
       <c r="F122" t="n">
-        <v>190.78</v>
+        <v>192</v>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>-5.53</v>
+        <v>-4.93</v>
       </c>
     </row>
     <row r="123">
@@ -3623,11 +3623,11 @@
         <v>0</v>
       </c>
       <c r="F123" t="n">
-        <v>110.25</v>
+        <v>110.2</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>3.38</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="124">
@@ -3649,11 +3649,11 @@
         <v>0</v>
       </c>
       <c r="F124" t="n">
-        <v>40.4</v>
+        <v>40</v>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>-3.58</v>
+        <v>-4.53</v>
       </c>
     </row>
     <row r="125">
@@ -3701,11 +3701,11 @@
         <v>0</v>
       </c>
       <c r="F126" t="n">
-        <v>966.7</v>
+        <v>956.8</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>-4.22</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="127">
@@ -3753,11 +3753,11 @@
         <v>0</v>
       </c>
       <c r="F128" t="n">
-        <v>82.5</v>
+        <v>83</v>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>-2.19</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="129">
@@ -3779,11 +3779,11 @@
         <v>0</v>
       </c>
       <c r="F129" t="n">
-        <v>102.42</v>
+        <v>101.51</v>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>2.52</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="130">
@@ -3805,11 +3805,11 @@
         <v>0</v>
       </c>
       <c r="F130" t="n">
-        <v>870</v>
+        <v>868.55</v>
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>-3.22</v>
+        <v>-3.38</v>
       </c>
     </row>
     <row r="131">
@@ -3831,11 +3831,11 @@
         <v>0</v>
       </c>
       <c r="F131" t="n">
-        <v>54.53</v>
+        <v>54.3</v>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>-2.01</v>
+        <v>-2.43</v>
       </c>
     </row>
     <row r="132">
@@ -3883,11 +3883,11 @@
         <v>0</v>
       </c>
       <c r="F133" t="n">
-        <v>46.78</v>
+        <v>49.1</v>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>2.14</v>
+        <v>7.21</v>
       </c>
     </row>
     <row r="134">
@@ -3909,11 +3909,11 @@
         <v>0</v>
       </c>
       <c r="F134" t="n">
-        <v>6.38</v>
+        <v>6.64</v>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>3.07</v>
+        <v>7.27</v>
       </c>
     </row>
     <row r="135">
@@ -3961,11 +3961,11 @@
         <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>7.12</v>
+        <v>6.59</v>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>-3.13</v>
+        <v>-10.34</v>
       </c>
     </row>
     <row r="137">
@@ -3987,11 +3987,11 @@
         <v>0</v>
       </c>
       <c r="F137" t="n">
-        <v>6.66</v>
+        <v>6.56</v>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="n">
-        <v>1.06</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="138">
@@ -4013,11 +4013,11 @@
         <v>0</v>
       </c>
       <c r="F138" t="n">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="n">
-        <v>-3.47</v>
+        <v>-4.36</v>
       </c>
     </row>
     <row r="139">
@@ -4039,11 +4039,11 @@
         <v>0</v>
       </c>
       <c r="F139" t="n">
-        <v>99.34999999999999</v>
+        <v>98.36</v>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="n">
-        <v>-0.65</v>
+        <v>-1.64</v>
       </c>
     </row>
     <row r="140">
@@ -4065,11 +4065,11 @@
         <v>0</v>
       </c>
       <c r="F140" t="n">
-        <v>18.18</v>
+        <v>18.12</v>
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="n">
-        <v>1.45</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="141">
@@ -4091,11 +4091,11 @@
         <v>0</v>
       </c>
       <c r="F141" t="n">
-        <v>1797.1</v>
+        <v>1796.7</v>
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="n">
-        <v>2.69</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="142">
@@ -4117,11 +4117,11 @@
         <v>0</v>
       </c>
       <c r="F142" t="n">
-        <v>62.8</v>
+        <v>65.83</v>
       </c>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="n">
-        <v>13.15</v>
+        <v>18.61</v>
       </c>
     </row>
     <row r="143">
@@ -4169,11 +4169,11 @@
         <v>0</v>
       </c>
       <c r="F144" t="n">
-        <v>26.44</v>
+        <v>26.52</v>
       </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="n">
-        <v>0.53</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="145">
@@ -4195,11 +4195,11 @@
         <v>0</v>
       </c>
       <c r="F145" t="n">
-        <v>140.98</v>
+        <v>140.43</v>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="n">
-        <v>-0.7</v>
+        <v>-1.09</v>
       </c>
     </row>
     <row r="146">
@@ -4221,11 +4221,11 @@
         <v>0</v>
       </c>
       <c r="F146" t="n">
-        <v>50.95</v>
+        <v>53.13</v>
       </c>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="n">
-        <v>-1.92</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="147">
@@ -4247,11 +4247,11 @@
         <v>0</v>
       </c>
       <c r="F147" t="n">
-        <v>264.7</v>
+        <v>264.2</v>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="n">
-        <v>-1.19</v>
+        <v>-1.38</v>
       </c>
     </row>
     <row r="148">
@@ -4273,11 +4273,11 @@
         <v>0</v>
       </c>
       <c r="F148" t="n">
-        <v>469</v>
+        <v>467.5</v>
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="n">
-        <v>0.44</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="149">
@@ -4299,11 +4299,11 @@
         <v>0</v>
       </c>
       <c r="F149" t="n">
-        <v>5.78</v>
+        <v>6.47</v>
       </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="n">
-        <v>-2.86</v>
+        <v>8.74</v>
       </c>
     </row>
     <row r="150">
@@ -4325,11 +4325,11 @@
         <v>0</v>
       </c>
       <c r="F150" t="n">
-        <v>8.75</v>
+        <v>8.74</v>
       </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="n">
-        <v>-2.67</v>
+        <v>-2.78</v>
       </c>
     </row>
     <row r="151">
@@ -4351,11 +4351,11 @@
         <v>0</v>
       </c>
       <c r="F151" t="n">
-        <v>24.78</v>
+        <v>24.77</v>
       </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="n">
-        <v>-0.68</v>
+        <v>-0.72</v>
       </c>
     </row>
     <row r="152">
@@ -4377,11 +4377,11 @@
         <v>0</v>
       </c>
       <c r="F152" t="n">
-        <v>39.18</v>
+        <v>38.71</v>
       </c>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="n">
-        <v>-2.78</v>
+        <v>-3.95</v>
       </c>
     </row>
     <row r="153">
@@ -4403,11 +4403,11 @@
         <v>0</v>
       </c>
       <c r="F153" t="n">
-        <v>17.29</v>
+        <v>17.78</v>
       </c>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="n">
-        <v>-0.86</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="154">
@@ -4429,11 +4429,11 @@
         <v>0</v>
       </c>
       <c r="F154" t="n">
-        <v>60.48</v>
+        <v>60.5</v>
       </c>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="n">
-        <v>-0.85</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="155">
@@ -4455,11 +4455,11 @@
         <v>0</v>
       </c>
       <c r="F155" t="n">
-        <v>536.05</v>
+        <v>526</v>
       </c>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="n">
-        <v>-2.18</v>
+        <v>-4.01</v>
       </c>
     </row>
     <row r="156">
@@ -4481,11 +4481,11 @@
         <v>0</v>
       </c>
       <c r="F156" t="n">
-        <v>91.01000000000001</v>
+        <v>91</v>
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="n">
-        <v>-1.61</v>
+        <v>-1.62</v>
       </c>
     </row>
     <row r="157">
@@ -4533,11 +4533,11 @@
         <v>0</v>
       </c>
       <c r="F158" t="n">
-        <v>282.9</v>
+        <v>283.9</v>
       </c>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="n">
-        <v>4.39</v>
+        <v>4.76</v>
       </c>
     </row>
     <row r="159">
@@ -4559,11 +4559,11 @@
         <v>0</v>
       </c>
       <c r="F159" t="n">
-        <v>477.6</v>
+        <v>472.65</v>
       </c>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="n">
-        <v>1.19</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="160">
@@ -4585,11 +4585,11 @@
         <v>0</v>
       </c>
       <c r="F160" t="n">
-        <v>218.92</v>
+        <v>220.31</v>
       </c>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="n">
-        <v>-0.26</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="161">
@@ -4611,11 +4611,11 @@
         <v>0</v>
       </c>
       <c r="F161" t="n">
-        <v>40.49</v>
+        <v>40.22</v>
       </c>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="n">
-        <v>-3.34</v>
+        <v>-3.99</v>
       </c>
     </row>
     <row r="162">
@@ -4637,11 +4637,11 @@
         <v>0</v>
       </c>
       <c r="F162" t="n">
-        <v>67.54000000000001</v>
+        <v>67.72</v>
       </c>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="n">
-        <v>-0.68</v>
+        <v>-0.41</v>
       </c>
     </row>
     <row r="163">
@@ -4663,11 +4663,11 @@
         <v>0</v>
       </c>
       <c r="F163" t="n">
-        <v>478.05</v>
+        <v>478.9</v>
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="n">
-        <v>0.64</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="164">
@@ -4689,11 +4689,11 @@
         <v>0</v>
       </c>
       <c r="F164" t="n">
-        <v>140.25</v>
+        <v>141.33</v>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="n">
-        <v>-3.1</v>
+        <v>-2.36</v>
       </c>
     </row>
     <row r="165">
@@ -4715,11 +4715,11 @@
         <v>0</v>
       </c>
       <c r="F165" t="n">
-        <v>25.92</v>
+        <v>25.69</v>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="n">
-        <v>-2.56</v>
+        <v>-3.42</v>
       </c>
     </row>
     <row r="166">
@@ -4741,11 +4741,11 @@
         <v>0</v>
       </c>
       <c r="F166" t="n">
-        <v>32.99</v>
+        <v>34.5</v>
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="n">
-        <v>-1.38</v>
+        <v>3.14</v>
       </c>
     </row>
     <row r="167">
@@ -4767,11 +4767,11 @@
         <v>0</v>
       </c>
       <c r="F167" t="n">
-        <v>28.91</v>
+        <v>29.07</v>
       </c>
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="n">
-        <v>-1.33</v>
+        <v>-0.78</v>
       </c>
     </row>
     <row r="168">
@@ -4793,11 +4793,11 @@
         <v>0</v>
       </c>
       <c r="F168" t="n">
-        <v>84.38</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="n">
-        <v>-1.88</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="169">
@@ -4819,11 +4819,11 @@
         <v>0</v>
       </c>
       <c r="F169" t="n">
-        <v>70</v>
+        <v>70.18000000000001</v>
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="n">
-        <v>-0.68</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="170">
@@ -4845,11 +4845,11 @@
         <v>0</v>
       </c>
       <c r="F170" t="n">
-        <v>152.29</v>
+        <v>156.05</v>
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="n">
-        <v>-3.64</v>
+        <v>-1.26</v>
       </c>
     </row>
     <row r="171">
@@ -4871,11 +4871,11 @@
         <v>0</v>
       </c>
       <c r="F171" t="n">
-        <v>346</v>
+        <v>347.6</v>
       </c>
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="n">
-        <v>-0.12</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="172">
@@ -4897,11 +4897,11 @@
         <v>0</v>
       </c>
       <c r="F172" t="n">
-        <v>27.31</v>
+        <v>27.9</v>
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="n">
-        <v>-4.14</v>
+        <v>-2.07</v>
       </c>
     </row>
     <row r="173">
@@ -4923,11 +4923,11 @@
         <v>0</v>
       </c>
       <c r="F173" t="n">
-        <v>626.85</v>
+        <v>623.5</v>
       </c>
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="n">
-        <v>1.43</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="174">
@@ -4949,11 +4949,11 @@
         <v>0</v>
       </c>
       <c r="F174" t="n">
-        <v>195.55</v>
+        <v>194.5</v>
       </c>
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="n">
-        <v>-3.62</v>
+        <v>-4.14</v>
       </c>
     </row>
     <row r="175">
@@ -4975,11 +4975,11 @@
         <v>0</v>
       </c>
       <c r="F175" t="n">
-        <v>68.87</v>
+        <v>69</v>
       </c>
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="n">
-        <v>-1.47</v>
+        <v>-1.29</v>
       </c>
     </row>
     <row r="176">
@@ -5001,11 +5001,11 @@
         <v>0</v>
       </c>
       <c r="F176" t="n">
-        <v>87.15000000000001</v>
+        <v>87.8</v>
       </c>
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="n">
-        <v>1.34</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="177">
@@ -5027,11 +5027,11 @@
         <v>0</v>
       </c>
       <c r="F177" t="n">
-        <v>426.1</v>
+        <v>423.9</v>
       </c>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="n">
-        <v>-0.21</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="178">
@@ -5053,11 +5053,11 @@
         <v>0</v>
       </c>
       <c r="F178" t="n">
-        <v>68.28</v>
+        <v>68.5</v>
       </c>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
-        <v>-0.5</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="179">
@@ -5079,11 +5079,11 @@
         <v>0</v>
       </c>
       <c r="F179" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180">
@@ -5131,11 +5131,11 @@
         <v>0</v>
       </c>
       <c r="F181" t="n">
-        <v>23.41</v>
+        <v>23.69</v>
       </c>
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="n">
-        <v>-2.66</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="182">
@@ -5157,11 +5157,11 @@
         <v>0</v>
       </c>
       <c r="F182" t="n">
-        <v>372.2</v>
+        <v>373.75</v>
       </c>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="n">
-        <v>-2.04</v>
+        <v>-1.63</v>
       </c>
     </row>
     <row r="183">
@@ -5183,11 +5183,11 @@
         <v>0</v>
       </c>
       <c r="F183" t="n">
-        <v>45.99</v>
+        <v>45.94</v>
       </c>
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="n">
-        <v>1.3</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="184">
@@ -5209,11 +5209,11 @@
         <v>0</v>
       </c>
       <c r="F184" t="n">
-        <v>17.48</v>
+        <v>17.38</v>
       </c>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="n">
-        <v>3.43</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="185">
@@ -5235,11 +5235,11 @@
         <v>0</v>
       </c>
       <c r="F185" t="n">
-        <v>110.98</v>
+        <v>110</v>
       </c>
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="n">
-        <v>-1.87</v>
+        <v>-2.74</v>
       </c>
     </row>
     <row r="186">
@@ -5261,11 +5261,11 @@
         <v>0</v>
       </c>
       <c r="F186" t="n">
-        <v>4.1</v>
+        <v>4.21</v>
       </c>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="n">
-        <v>-3.3</v>
+        <v>-0.71</v>
       </c>
     </row>
     <row r="187">
@@ -5287,11 +5287,11 @@
         <v>0</v>
       </c>
       <c r="F187" t="n">
-        <v>145.32</v>
+        <v>143.25</v>
       </c>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="n">
-        <v>1.62</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="188">
@@ -5313,11 +5313,11 @@
         <v>0</v>
       </c>
       <c r="F188" t="n">
-        <v>182.61</v>
+        <v>188.95</v>
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="n">
-        <v>-1.29</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="189">
@@ -5339,11 +5339,11 @@
         <v>0</v>
       </c>
       <c r="F189" t="n">
-        <v>627</v>
+        <v>619.1</v>
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="n">
-        <v>0.75</v>
+        <v>-0.52</v>
       </c>
     </row>
     <row r="190">
@@ -5365,11 +5365,11 @@
         <v>0</v>
       </c>
       <c r="F190" t="n">
-        <v>944.35</v>
+        <v>943.5</v>
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="n">
-        <v>2.65</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="191">
@@ -5391,11 +5391,11 @@
         <v>0</v>
       </c>
       <c r="F191" t="n">
-        <v>4990</v>
+        <v>4966</v>
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="n">
-        <v>0.6</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="192">
@@ -5417,11 +5417,11 @@
         <v>0</v>
       </c>
       <c r="F192" t="n">
-        <v>62.02</v>
+        <v>62.25</v>
       </c>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="n">
-        <v>1.67</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="193">
@@ -5443,11 +5443,11 @@
         <v>0</v>
       </c>
       <c r="F193" t="n">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="n">
-        <v>-0.3</v>
+        <v>-0.63</v>
       </c>
     </row>
     <row r="194">
@@ -5469,11 +5469,11 @@
         <v>0</v>
       </c>
       <c r="F194" t="n">
-        <v>6.96</v>
+        <v>7.1</v>
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="n">
-        <v>-1.69</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="195">
@@ -5495,11 +5495,11 @@
         <v>0</v>
       </c>
       <c r="F195" t="n">
-        <v>12.3</v>
+        <v>12.78</v>
       </c>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="n">
-        <v>3.89</v>
+        <v>7.94</v>
       </c>
     </row>
     <row r="196">
@@ -5547,11 +5547,11 @@
         <v>0</v>
       </c>
       <c r="F197" t="n">
-        <v>284.6</v>
+        <v>287.05</v>
       </c>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="n">
-        <v>-0.91</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="198">
@@ -5573,11 +5573,11 @@
         <v>0</v>
       </c>
       <c r="F198" t="n">
-        <v>992.95</v>
+        <v>984.5</v>
       </c>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="n">
-        <v>-2.17</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="199">
@@ -5599,11 +5599,11 @@
         <v>0</v>
       </c>
       <c r="F199" t="n">
-        <v>20.48</v>
+        <v>20.45</v>
       </c>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="n">
-        <v>-1.3</v>
+        <v>-1.45</v>
       </c>
     </row>
     <row r="200">
@@ -5625,11 +5625,11 @@
         <v>0</v>
       </c>
       <c r="F200" t="n">
-        <v>462.7</v>
+        <v>464.5</v>
       </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="n">
-        <v>0.98</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="201">
@@ -5651,11 +5651,11 @@
         <v>0</v>
       </c>
       <c r="F201" t="n">
-        <v>72.44</v>
+        <v>73</v>
       </c>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="n">
-        <v>3.95</v>
+        <v>4.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-05-01 06:31 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -529,11 +529,11 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>2.17</v>
+        <v>2.08</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>-1.36</v>
+        <v>-5.45</v>
       </c>
     </row>
     <row r="5">
@@ -555,11 +555,11 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>45.88</v>
+        <v>47</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>-8.06</v>
+        <v>-5.81</v>
       </c>
     </row>
     <row r="6">
@@ -581,11 +581,11 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>194.22</v>
+        <v>194.98</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>-2.41</v>
+        <v>-2.03</v>
       </c>
     </row>
     <row r="7">
@@ -659,11 +659,11 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>803.35</v>
+        <v>815.25</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>8.859999999999999</v>
+        <v>10.47</v>
       </c>
     </row>
     <row r="10">
@@ -685,11 +685,11 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>20.84</v>
+        <v>20.99</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>-6.92</v>
+        <v>-6.25</v>
       </c>
     </row>
     <row r="11">
@@ -737,11 +737,11 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>27.34</v>
+        <v>27.12</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>-5.2</v>
+        <v>-5.96</v>
       </c>
     </row>
     <row r="13">
@@ -763,11 +763,11 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>35.05</v>
+        <v>35.95</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>-8.960000000000001</v>
+        <v>-6.62</v>
       </c>
     </row>
     <row r="14">
@@ -789,11 +789,11 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>48.45</v>
+        <v>49</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>-3.87</v>
+        <v>-2.78</v>
       </c>
     </row>
     <row r="15">
@@ -815,11 +815,11 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>22.25</v>
+        <v>23.15</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>-7.1</v>
+        <v>-3.34</v>
       </c>
     </row>
     <row r="16">
@@ -841,11 +841,11 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>179.95</v>
+        <v>192.05</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>-2.68</v>
+        <v>3.87</v>
       </c>
     </row>
     <row r="17">
@@ -867,11 +867,11 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>-2.85</v>
+        <v>-3.69</v>
       </c>
     </row>
     <row r="18">
@@ -893,11 +893,11 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>5.55</v>
+        <v>5.51</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>-2.12</v>
+        <v>-2.82</v>
       </c>
     </row>
     <row r="19">
@@ -919,24 +919,24 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>85.51000000000001</v>
+        <v>84.95</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>8.27</v>
+        <v>7.56</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DPEL</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>473.4</v>
+        <v>273.95</v>
       </c>
       <c r="C20" t="n">
-        <v>497.05</v>
+        <v>287.64</v>
       </c>
       <c r="D20" t="n">
         <v>5</v>
@@ -945,7 +945,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>497.05</v>
+        <v>287.64</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
@@ -955,14 +955,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>DPEL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>273.95</v>
+        <v>473.4</v>
       </c>
       <c r="C21" t="n">
-        <v>287.64</v>
+        <v>497.05</v>
       </c>
       <c r="D21" t="n">
         <v>5</v>
@@ -971,7 +971,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>287.64</v>
+        <v>497.05</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
@@ -1023,11 +1023,11 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>21.85</v>
+        <v>21.88</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>-0.14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1075,11 +1075,11 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>103.05</v>
+        <v>108.65</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>-5.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1101,24 +1101,24 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>2.72</v>
+        <v>2.74</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>-0.73</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SHRIKANHA</t>
+          <t>SHYAMTEL</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>29.2</v>
+        <v>21.55</v>
       </c>
       <c r="C27" t="n">
-        <v>30.65</v>
+        <v>22.62</v>
       </c>
       <c r="D27" t="n">
         <v>4.97</v>
@@ -1127,24 +1127,24 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>30.4</v>
+        <v>22.62</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>-0.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SHYAMTEL</t>
+          <t>SHRIKANHA</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>21.55</v>
+        <v>29.2</v>
       </c>
       <c r="C28" t="n">
-        <v>22.62</v>
+        <v>30.65</v>
       </c>
       <c r="D28" t="n">
         <v>4.97</v>
@@ -1153,11 +1153,11 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>22.62</v>
+        <v>28.6</v>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>-6.69</v>
       </c>
     </row>
     <row r="29">
@@ -1179,11 +1179,11 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>4.21</v>
+        <v>4.39</v>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>-5.18</v>
+        <v>-1.13</v>
       </c>
     </row>
     <row r="30">
@@ -1205,11 +1205,11 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>108</v>
+        <v>109.25</v>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>-1.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="31">
@@ -1231,11 +1231,11 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>31.46</v>
+        <v>31.85</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>-4.09</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="32">
@@ -1257,11 +1257,11 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>1.9</v>
+        <v>1.92</v>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>-1.04</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -1283,11 +1283,11 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>19.34</v>
+        <v>19.73</v>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>2.76</v>
+        <v>4.84</v>
       </c>
     </row>
     <row r="34">
@@ -1319,14 +1319,14 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GURUNANAK</t>
+          <t>DYNPRO</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>36.9</v>
+        <v>226.92</v>
       </c>
       <c r="C35" t="n">
-        <v>38.7</v>
+        <v>238</v>
       </c>
       <c r="D35" t="n">
         <v>4.88</v>
@@ -1335,24 +1335,24 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>38.7</v>
+        <v>223</v>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>-6.3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DYNPRO</t>
+          <t>GURUNANAK</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>226.92</v>
+        <v>36.9</v>
       </c>
       <c r="C36" t="n">
-        <v>238</v>
+        <v>38.7</v>
       </c>
       <c r="D36" t="n">
         <v>4.88</v>
@@ -1361,11 +1361,11 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>222.95</v>
+        <v>38.7</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>-6.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1387,24 +1387,24 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>3.66</v>
+        <v>3.6</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>-5.91</v>
+        <v>-7.46</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SUPREMEENG</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1.03</v>
+        <v>1.65</v>
       </c>
       <c r="C38" t="n">
-        <v>1.08</v>
+        <v>1.73</v>
       </c>
       <c r="D38" t="n">
         <v>4.85</v>
@@ -1413,24 +1413,24 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>1.61</v>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>-7.41</v>
+        <v>-6.94</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>SUPREMEENG</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1.65</v>
+        <v>1.03</v>
       </c>
       <c r="C39" t="n">
-        <v>1.73</v>
+        <v>1.08</v>
       </c>
       <c r="D39" t="n">
         <v>4.85</v>
@@ -1439,11 +1439,11 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>1.68</v>
+        <v>1.06</v>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>-2.89</v>
+        <v>-1.85</v>
       </c>
     </row>
     <row r="40">
@@ -1465,11 +1465,11 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>63.05</v>
+        <v>60.7</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>1.69</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="41">
@@ -1517,11 +1517,11 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>597.85</v>
+        <v>597.15</v>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>-2.79</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="43">
@@ -1543,11 +1543,11 @@
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>-2.03</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="44">
@@ -1569,11 +1569,11 @@
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>2.47</v>
+        <v>2.45</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>-0.8100000000000001</v>
       </c>
     </row>
     <row r="45">
@@ -1595,11 +1595,11 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>1.37</v>
+        <v>1.32</v>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>-0.72</v>
+        <v>-4.35</v>
       </c>
     </row>
     <row r="46">
@@ -1621,11 +1621,11 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>-4.46</v>
+        <v>-1.91</v>
       </c>
     </row>
     <row r="47">
@@ -1673,11 +1673,11 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>31.62</v>
+        <v>31.25</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>-3.89</v>
+        <v>-5.02</v>
       </c>
     </row>
     <row r="49">
@@ -1699,11 +1699,11 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>127.83</v>
+        <v>127.41</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>-5.17</v>
+        <v>-5.48</v>
       </c>
     </row>
     <row r="50">
@@ -1725,11 +1725,11 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>85.73999999999999</v>
+        <v>84.95</v>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>-3.64</v>
+        <v>-4.53</v>
       </c>
     </row>
     <row r="51">
@@ -1751,11 +1751,11 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>0.46</v>
+        <v>0.48</v>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>-4.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -1777,11 +1777,11 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>6739</v>
+        <v>6815</v>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>-4.41</v>
+        <v>-3.33</v>
       </c>
     </row>
     <row r="53">
@@ -1803,11 +1803,11 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>20.89</v>
+        <v>21.24</v>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>-4.13</v>
+        <v>-2.52</v>
       </c>
     </row>
     <row r="54">
@@ -1829,11 +1829,11 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>131.55</v>
+        <v>129.93</v>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>-4.54</v>
+        <v>-5.71</v>
       </c>
     </row>
     <row r="55">
@@ -1881,11 +1881,11 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>27</v>
+        <v>27.2</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>-3.57</v>
+        <v>-2.86</v>
       </c>
     </row>
     <row r="57">
@@ -1907,11 +1907,11 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>60.47</v>
+        <v>61.5</v>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>-4.91</v>
+        <v>-3.29</v>
       </c>
     </row>
     <row r="58">
@@ -1959,11 +1959,11 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>397.7</v>
+        <v>405</v>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>-1.32</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="60">
@@ -1985,11 +1985,11 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>819.95</v>
+        <v>806.5</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>-1.33</v>
+        <v>-2.95</v>
       </c>
     </row>
     <row r="61">
@@ -2011,11 +2011,11 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>357.35</v>
+        <v>358.95</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>-5.94</v>
+        <v>-5.51</v>
       </c>
     </row>
     <row r="62">
@@ -2037,11 +2037,11 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>30.3</v>
+        <v>31.59</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>-4.72</v>
+        <v>-0.66</v>
       </c>
     </row>
     <row r="63">
@@ -2063,11 +2063,11 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>83.79000000000001</v>
+        <v>84.12</v>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>-5.85</v>
+        <v>-5.48</v>
       </c>
     </row>
     <row r="64">
@@ -2089,11 +2089,11 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>2597</v>
+        <v>2702.3</v>
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>-2.73</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="65">
@@ -2115,11 +2115,11 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>27.5</v>
+        <v>27.69</v>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>-1.43</v>
+        <v>-0.75</v>
       </c>
     </row>
     <row r="66">
@@ -2141,11 +2141,11 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>23.95</v>
+        <v>24</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>-3.54</v>
+        <v>-3.34</v>
       </c>
     </row>
     <row r="67">
@@ -2167,11 +2167,11 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>59.5</v>
+        <v>61.9</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>-5.48</v>
+        <v>-1.67</v>
       </c>
     </row>
     <row r="68">
@@ -2193,11 +2193,11 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>56.5</v>
+        <v>57.5</v>
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>-4.24</v>
+        <v>-2.54</v>
       </c>
     </row>
     <row r="69">
@@ -2219,11 +2219,11 @@
         <v>0</v>
       </c>
       <c r="F69" t="n">
-        <v>16.46</v>
+        <v>16.45</v>
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
-        <v>-7.01</v>
+        <v>-7.06</v>
       </c>
     </row>
     <row r="70">
@@ -2245,11 +2245,11 @@
         <v>0</v>
       </c>
       <c r="F70" t="n">
-        <v>185.5</v>
+        <v>189.4</v>
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>-4.38</v>
+        <v>-2.37</v>
       </c>
     </row>
     <row r="71">
@@ -2271,11 +2271,11 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>53.77</v>
+        <v>54.37</v>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>-3.29</v>
+        <v>-2.21</v>
       </c>
     </row>
     <row r="72">
@@ -2297,11 +2297,11 @@
         <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>173.86</v>
+        <v>173.5</v>
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>-1.66</v>
+        <v>-1.87</v>
       </c>
     </row>
     <row r="73">
@@ -2323,11 +2323,11 @@
         <v>0</v>
       </c>
       <c r="F73" t="n">
-        <v>9.880000000000001</v>
+        <v>10</v>
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
-        <v>-4.26</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="74">
@@ -2349,11 +2349,11 @@
         <v>0</v>
       </c>
       <c r="F74" t="n">
-        <v>459.8</v>
+        <v>491.45</v>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>-4.98</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="75">
@@ -2375,11 +2375,11 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>48.49</v>
+        <v>48.05</v>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>-3.41</v>
+        <v>-4.28</v>
       </c>
     </row>
     <row r="76">
@@ -2401,11 +2401,11 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>100</v>
+        <v>98.5</v>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>-4.58</v>
+        <v>-6.01</v>
       </c>
     </row>
     <row r="77">
@@ -2427,11 +2427,11 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>49.5</v>
+        <v>51.3</v>
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>-5.88</v>
+        <v>-2.45</v>
       </c>
     </row>
     <row r="78">
@@ -2453,11 +2453,11 @@
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>6.98</v>
+        <v>7.09</v>
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>-4.38</v>
+        <v>-2.88</v>
       </c>
     </row>
     <row r="79">
@@ -2479,11 +2479,11 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>982</v>
+        <v>992.9</v>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>-4.66</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="80">
@@ -2505,11 +2505,11 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>6.88</v>
+        <v>6.82</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>-3.23</v>
+        <v>-4.08</v>
       </c>
     </row>
     <row r="81">
@@ -2531,11 +2531,11 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>130.1</v>
+        <v>134</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>-4.34</v>
+        <v>-1.47</v>
       </c>
     </row>
     <row r="82">
@@ -2557,11 +2557,11 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>334.1</v>
+        <v>325.2</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>0.74</v>
+        <v>-1.94</v>
       </c>
     </row>
     <row r="83">
@@ -2583,11 +2583,11 @@
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>2.2</v>
+        <v>2.27</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>-4.35</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="84">
@@ -2609,24 +2609,24 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>278.75</v>
+        <v>280</v>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>-0.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>JETFREIGHT</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>44.62</v>
+        <v>20.71</v>
       </c>
       <c r="C85" t="n">
-        <v>46</v>
+        <v>21.35</v>
       </c>
       <c r="D85" t="n">
         <v>3.09</v>
@@ -2635,24 +2635,24 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>45.19</v>
+        <v>20.35</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>-1.76</v>
+        <v>-4.68</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>JETFREIGHT</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>20.71</v>
+        <v>44.62</v>
       </c>
       <c r="C86" t="n">
-        <v>21.35</v>
+        <v>46</v>
       </c>
       <c r="D86" t="n">
         <v>3.09</v>
@@ -2661,11 +2661,11 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>20.58</v>
+        <v>44.95</v>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>-3.61</v>
+        <v>-2.28</v>
       </c>
     </row>
     <row r="87">
@@ -2687,11 +2687,11 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>4.63</v>
+        <v>4.69</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>-3.74</v>
+        <v>-2.49</v>
       </c>
     </row>
     <row r="88">
@@ -2713,11 +2713,11 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>459.8</v>
+        <v>460.8</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>-0.14</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="89">
@@ -2739,11 +2739,11 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>74.23</v>
+        <v>75.2</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>-1.67</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="90">
@@ -2791,11 +2791,11 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>5.76</v>
+        <v>5.84</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>-2.37</v>
+        <v>-1.02</v>
       </c>
     </row>
     <row r="92">
@@ -2817,11 +2817,11 @@
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>16.41</v>
+        <v>16.39</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>-3.41</v>
+        <v>-3.53</v>
       </c>
     </row>
     <row r="93">
@@ -2843,11 +2843,11 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>88.41</v>
+        <v>89.5</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>-1.11</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="94">
@@ -2869,11 +2869,11 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>2311.7</v>
+        <v>2275</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>-0.12</v>
+        <v>-1.71</v>
       </c>
     </row>
     <row r="95">
@@ -2895,11 +2895,11 @@
         <v>0</v>
       </c>
       <c r="F95" t="n">
-        <v>7.09</v>
+        <v>7.12</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>-2.88</v>
+        <v>-2.47</v>
       </c>
     </row>
     <row r="96">
@@ -2921,11 +2921,11 @@
         <v>0</v>
       </c>
       <c r="F96" t="n">
-        <v>37.5</v>
+        <v>38.8</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="n">
-        <v>-3.85</v>
+        <v>-0.51</v>
       </c>
     </row>
     <row r="97">
@@ -2947,11 +2947,11 @@
         <v>0</v>
       </c>
       <c r="F97" t="n">
-        <v>90.90000000000001</v>
+        <v>91.98999999999999</v>
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="n">
-        <v>-3.3</v>
+        <v>-2.14</v>
       </c>
     </row>
     <row r="98">
@@ -2973,24 +2973,24 @@
         <v>0</v>
       </c>
       <c r="F98" t="n">
-        <v>36.2</v>
+        <v>35.29</v>
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>-2.16</v>
+        <v>-4.62</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>BORANA</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>354.1</v>
+        <v>0.36</v>
       </c>
       <c r="C99" t="n">
-        <v>363.95</v>
+        <v>0.37</v>
       </c>
       <c r="D99" t="n">
         <v>2.78</v>
@@ -2999,24 +2999,24 @@
         <v>0</v>
       </c>
       <c r="F99" t="n">
-        <v>344.9</v>
+        <v>0.37</v>
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="n">
-        <v>-5.23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>BORANA</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0.36</v>
+        <v>354.1</v>
       </c>
       <c r="C100" t="n">
-        <v>0.37</v>
+        <v>363.95</v>
       </c>
       <c r="D100" t="n">
         <v>2.78</v>
@@ -3025,11 +3025,11 @@
         <v>0</v>
       </c>
       <c r="F100" t="n">
-        <v>0.35</v>
+        <v>346</v>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>-5.41</v>
+        <v>-4.93</v>
       </c>
     </row>
     <row r="101">
@@ -3051,24 +3051,24 @@
         <v>0</v>
       </c>
       <c r="F101" t="n">
-        <v>529.05</v>
+        <v>524.75</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="n">
-        <v>-4.67</v>
+        <v>-5.44</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>VINEETLAB</t>
+          <t>JINDALPHOT</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>38.55</v>
+        <v>1102.65</v>
       </c>
       <c r="C102" t="n">
-        <v>39.6</v>
+        <v>1132.65</v>
       </c>
       <c r="D102" t="n">
         <v>2.72</v>
@@ -3077,24 +3077,24 @@
         <v>0</v>
       </c>
       <c r="F102" t="n">
-        <v>38</v>
+        <v>1104.1</v>
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>-4.04</v>
+        <v>-2.52</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>JINDALPHOT</t>
+          <t>VINEETLAB</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>1102.65</v>
+        <v>38.55</v>
       </c>
       <c r="C103" t="n">
-        <v>1132.65</v>
+        <v>39.6</v>
       </c>
       <c r="D103" t="n">
         <v>2.72</v>
@@ -3103,11 +3103,11 @@
         <v>0</v>
       </c>
       <c r="F103" t="n">
-        <v>1103.6</v>
+        <v>37.7</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
-        <v>-2.56</v>
+        <v>-4.8</v>
       </c>
     </row>
     <row r="104">
@@ -3129,11 +3129,11 @@
         <v>0</v>
       </c>
       <c r="F104" t="n">
-        <v>72.2</v>
+        <v>73.3</v>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>-7.44</v>
+        <v>-6.03</v>
       </c>
     </row>
     <row r="105">
@@ -3155,24 +3155,24 @@
         <v>0</v>
       </c>
       <c r="F105" t="n">
-        <v>17.85</v>
+        <v>17.88</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>-4.55</v>
+        <v>-4.39</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>FLFL</t>
+          <t>DCM</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>1.5</v>
+        <v>83.47</v>
       </c>
       <c r="C106" t="n">
-        <v>1.54</v>
+        <v>85.7</v>
       </c>
       <c r="D106" t="n">
         <v>2.67</v>
@@ -3181,24 +3181,24 @@
         <v>0</v>
       </c>
       <c r="F106" t="n">
-        <v>1.55</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>0.65</v>
+        <v>-3.62</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>DCM</t>
+          <t>FLFL</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>83.47</v>
+        <v>1.5</v>
       </c>
       <c r="C107" t="n">
-        <v>85.7</v>
+        <v>1.54</v>
       </c>
       <c r="D107" t="n">
         <v>2.67</v>
@@ -3207,17 +3207,17 @@
         <v>0</v>
       </c>
       <c r="F107" t="n">
-        <v>82</v>
+        <v>1.47</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="n">
-        <v>-4.32</v>
+        <v>-4.55</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>PERFECT</t>
+          <t>EMPOWER</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -3243,7 +3243,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>EMPOWER</t>
+          <t>PERFECT</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -3285,11 +3285,11 @@
         <v>0</v>
       </c>
       <c r="F110" t="n">
-        <v>153.2</v>
+        <v>155.64</v>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>-4.84</v>
+        <v>-3.33</v>
       </c>
     </row>
     <row r="111">
@@ -3311,11 +3311,11 @@
         <v>0</v>
       </c>
       <c r="F111" t="n">
-        <v>195.56</v>
+        <v>201.7</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>-3.38</v>
+        <v>-0.35</v>
       </c>
     </row>
     <row r="112">
@@ -3363,24 +3363,24 @@
         <v>0</v>
       </c>
       <c r="F113" t="n">
-        <v>368.08</v>
+        <v>375.8</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="n">
-        <v>-6.46</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>AVG</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.79</v>
+        <v>166.78</v>
       </c>
       <c r="C114" t="n">
-        <v>0.8100000000000001</v>
+        <v>171</v>
       </c>
       <c r="D114" t="n">
         <v>2.53</v>
@@ -3389,24 +3389,24 @@
         <v>0</v>
       </c>
       <c r="F114" t="n">
-        <v>0.79</v>
+        <v>164.14</v>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>-2.47</v>
+        <v>-4.01</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>DRCSYSTEMS</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>14.61</v>
+        <v>0.79</v>
       </c>
       <c r="C115" t="n">
-        <v>14.98</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D115" t="n">
         <v>2.53</v>
@@ -3415,24 +3415,24 @@
         <v>0</v>
       </c>
       <c r="F115" t="n">
-        <v>14.89</v>
+        <v>0.78</v>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>-0.6</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>LOTUSEYE</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>121.52</v>
+        <v>14.61</v>
       </c>
       <c r="C116" t="n">
-        <v>124.6</v>
+        <v>14.98</v>
       </c>
       <c r="D116" t="n">
         <v>2.53</v>
@@ -3441,24 +3441,24 @@
         <v>0</v>
       </c>
       <c r="F116" t="n">
-        <v>121.42</v>
+        <v>15.15</v>
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>-2.55</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>AVG</t>
+          <t>LOTUSEYE</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>166.78</v>
+        <v>121.52</v>
       </c>
       <c r="C117" t="n">
-        <v>171</v>
+        <v>124.6</v>
       </c>
       <c r="D117" t="n">
         <v>2.53</v>
@@ -3467,24 +3467,24 @@
         <v>0</v>
       </c>
       <c r="F117" t="n">
-        <v>167.97</v>
+        <v>118.1</v>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="n">
-        <v>-1.77</v>
+        <v>-5.22</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SHRENIK</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.4</v>
+        <v>49.65</v>
       </c>
       <c r="C118" t="n">
-        <v>0.41</v>
+        <v>50.89</v>
       </c>
       <c r="D118" t="n">
         <v>2.5</v>
@@ -3493,24 +3493,24 @@
         <v>0</v>
       </c>
       <c r="F118" t="n">
-        <v>0.4</v>
+        <v>49.4</v>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>-2.44</v>
+        <v>-2.93</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>SHRENIK</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>49.65</v>
+        <v>0.4</v>
       </c>
       <c r="C119" t="n">
-        <v>50.89</v>
+        <v>0.41</v>
       </c>
       <c r="D119" t="n">
         <v>2.5</v>
@@ -3519,11 +3519,11 @@
         <v>0</v>
       </c>
       <c r="F119" t="n">
-        <v>49.29</v>
+        <v>0.4</v>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="n">
-        <v>-3.14</v>
+        <v>-2.44</v>
       </c>
     </row>
     <row r="120">
@@ -3545,11 +3545,11 @@
         <v>0</v>
       </c>
       <c r="F120" t="n">
-        <v>158.58</v>
+        <v>157.2</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>-1.5</v>
+        <v>-2.36</v>
       </c>
     </row>
     <row r="121">
@@ -3571,7 +3571,7 @@
         <v>0</v>
       </c>
       <c r="F121" t="n">
-        <v>622.55</v>
+        <v>622.6</v>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
@@ -3597,11 +3597,11 @@
         <v>0</v>
       </c>
       <c r="F122" t="n">
-        <v>83.2</v>
+        <v>83.36</v>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>-1.98</v>
+        <v>-1.79</v>
       </c>
     </row>
     <row r="123">
@@ -3623,11 +3623,11 @@
         <v>0</v>
       </c>
       <c r="F123" t="n">
-        <v>2.02</v>
+        <v>2.05</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
-        <v>-2.88</v>
+        <v>-1.44</v>
       </c>
     </row>
     <row r="124">
@@ -3649,11 +3649,11 @@
         <v>0</v>
       </c>
       <c r="F124" t="n">
-        <v>32.9</v>
+        <v>33.16</v>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>-3.86</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="125">
@@ -3675,11 +3675,11 @@
         <v>0</v>
       </c>
       <c r="F125" t="n">
-        <v>15.88</v>
+        <v>16</v>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="n">
-        <v>-2.99</v>
+        <v>-2.26</v>
       </c>
     </row>
     <row r="126">
@@ -3701,11 +3701,11 @@
         <v>0</v>
       </c>
       <c r="F126" t="n">
-        <v>128.05</v>
+        <v>129.3</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>-3.71</v>
+        <v>-2.77</v>
       </c>
     </row>
     <row r="127">
@@ -3727,24 +3727,24 @@
         <v>0</v>
       </c>
       <c r="F127" t="n">
-        <v>687.7</v>
+        <v>686</v>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>-0.19</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>TREL</t>
+          <t>SHIVATEX</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>26.86</v>
+        <v>172.78</v>
       </c>
       <c r="C128" t="n">
-        <v>27.5</v>
+        <v>176.9</v>
       </c>
       <c r="D128" t="n">
         <v>2.38</v>
@@ -3753,24 +3753,24 @@
         <v>0</v>
       </c>
       <c r="F128" t="n">
-        <v>26.41</v>
+        <v>173.51</v>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>-3.96</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SHIVATEX</t>
+          <t>TREL</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>172.78</v>
+        <v>26.86</v>
       </c>
       <c r="C129" t="n">
-        <v>176.9</v>
+        <v>27.5</v>
       </c>
       <c r="D129" t="n">
         <v>2.38</v>
@@ -3779,11 +3779,11 @@
         <v>0</v>
       </c>
       <c r="F129" t="n">
-        <v>171.96</v>
+        <v>26.95</v>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>-2.79</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="130">
@@ -3831,11 +3831,11 @@
         <v>0</v>
       </c>
       <c r="F131" t="n">
-        <v>79.48999999999999</v>
+        <v>79.15000000000001</v>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>-2.44</v>
+        <v>-2.86</v>
       </c>
     </row>
     <row r="132">
@@ -3857,11 +3857,11 @@
         <v>0</v>
       </c>
       <c r="F132" t="n">
-        <v>36.4</v>
+        <v>37.1</v>
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>-4.84</v>
+        <v>-3.01</v>
       </c>
     </row>
     <row r="133">
@@ -3883,11 +3883,11 @@
         <v>0</v>
       </c>
       <c r="F133" t="n">
-        <v>117.2</v>
+        <v>118.1</v>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>-1.1</v>
+        <v>-0.34</v>
       </c>
     </row>
     <row r="134">
@@ -3909,24 +3909,24 @@
         <v>0</v>
       </c>
       <c r="F134" t="n">
-        <v>58.65</v>
+        <v>59</v>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>-3.77</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>TATAINVEST</t>
+          <t>NIPPOBATRY</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>717.55</v>
+        <v>318.65</v>
       </c>
       <c r="C135" t="n">
-        <v>733.4</v>
+        <v>325.7</v>
       </c>
       <c r="D135" t="n">
         <v>2.21</v>
@@ -3935,24 +3935,24 @@
         <v>0</v>
       </c>
       <c r="F135" t="n">
-        <v>724.5</v>
+        <v>334</v>
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="n">
-        <v>-1.21</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>NIPPOBATRY</t>
+          <t>REMSONSIND</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>318.65</v>
+        <v>107.37</v>
       </c>
       <c r="C136" t="n">
-        <v>325.7</v>
+        <v>109.74</v>
       </c>
       <c r="D136" t="n">
         <v>2.21</v>
@@ -3961,24 +3961,24 @@
         <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>321</v>
+        <v>107.4</v>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>-1.44</v>
+        <v>-2.13</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>REMSONSIND</t>
+          <t>TATAINVEST</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>107.37</v>
+        <v>717.55</v>
       </c>
       <c r="C137" t="n">
-        <v>109.74</v>
+        <v>733.4</v>
       </c>
       <c r="D137" t="n">
         <v>2.21</v>
@@ -3987,11 +3987,11 @@
         <v>0</v>
       </c>
       <c r="F137" t="n">
-        <v>105.7</v>
+        <v>719.5</v>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="n">
-        <v>-3.68</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="138">
@@ -4013,24 +4013,24 @@
         <v>0</v>
       </c>
       <c r="F138" t="n">
-        <v>177.2</v>
+        <v>180</v>
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="n">
-        <v>-3.01</v>
+        <v>-1.48</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>AKG</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>11.5</v>
+        <v>0.46</v>
       </c>
       <c r="C139" t="n">
-        <v>11.75</v>
+        <v>0.47</v>
       </c>
       <c r="D139" t="n">
         <v>2.17</v>
@@ -4039,24 +4039,24 @@
         <v>0</v>
       </c>
       <c r="F139" t="n">
-        <v>11.55</v>
+        <v>0.47</v>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="n">
-        <v>-1.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>AKG</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>0.46</v>
+        <v>11.5</v>
       </c>
       <c r="C140" t="n">
-        <v>0.47</v>
+        <v>11.75</v>
       </c>
       <c r="D140" t="n">
         <v>2.17</v>
@@ -4065,11 +4065,11 @@
         <v>0</v>
       </c>
       <c r="F140" t="n">
-        <v>0.47</v>
+        <v>11.3</v>
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="n">
-        <v>0</v>
+        <v>-3.83</v>
       </c>
     </row>
     <row r="141">
@@ -4091,11 +4091,11 @@
         <v>0</v>
       </c>
       <c r="F141" t="n">
-        <v>159.62</v>
+        <v>164.9</v>
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="n">
-        <v>-3.08</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="142">
@@ -4117,24 +4117,24 @@
         <v>0</v>
       </c>
       <c r="F142" t="n">
-        <v>3.71</v>
+        <v>3.79</v>
       </c>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="n">
-        <v>-2.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>BAHETI</t>
+          <t>RBZJEWEL</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>585.55</v>
+        <v>136.79</v>
       </c>
       <c r="C143" t="n">
-        <v>598</v>
+        <v>139.7</v>
       </c>
       <c r="D143" t="n">
         <v>2.13</v>
@@ -4143,24 +4143,24 @@
         <v>0</v>
       </c>
       <c r="F143" t="n">
-        <v>617</v>
+        <v>135.5</v>
       </c>
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="n">
-        <v>3.18</v>
+        <v>-3.01</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>RBZJEWEL</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>136.79</v>
+        <v>0.47</v>
       </c>
       <c r="C144" t="n">
-        <v>139.7</v>
+        <v>0.48</v>
       </c>
       <c r="D144" t="n">
         <v>2.13</v>
@@ -4169,24 +4169,24 @@
         <v>0</v>
       </c>
       <c r="F144" t="n">
-        <v>136.69</v>
+        <v>0.48</v>
       </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="n">
-        <v>-2.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>BAHETI</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>0.47</v>
+        <v>585.55</v>
       </c>
       <c r="C145" t="n">
-        <v>0.48</v>
+        <v>598</v>
       </c>
       <c r="D145" t="n">
         <v>2.13</v>
@@ -4195,11 +4195,11 @@
         <v>0</v>
       </c>
       <c r="F145" t="n">
-        <v>0.48</v>
+        <v>599</v>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="146">
@@ -4221,11 +4221,11 @@
         <v>0</v>
       </c>
       <c r="F146" t="n">
-        <v>13.64</v>
+        <v>13.68</v>
       </c>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="n">
-        <v>-2.5</v>
+        <v>-2.22</v>
       </c>
     </row>
     <row r="147">
@@ -4247,11 +4247,11 @@
         <v>0</v>
       </c>
       <c r="F147" t="n">
-        <v>40.53</v>
+        <v>42</v>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="n">
-        <v>-2.22</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="148">
@@ -4299,11 +4299,11 @@
         <v>0</v>
       </c>
       <c r="F149" t="n">
-        <v>52.9</v>
+        <v>53.36</v>
       </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="n">
-        <v>-3.56</v>
+        <v>-2.72</v>
       </c>
     </row>
     <row r="150">
@@ -4325,24 +4325,24 @@
         <v>0</v>
       </c>
       <c r="F150" t="n">
-        <v>17.1</v>
+        <v>16.85</v>
       </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="n">
-        <v>-1.44</v>
+        <v>-2.88</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>0.49</v>
+        <v>965.3</v>
       </c>
       <c r="C151" t="n">
-        <v>0.5</v>
+        <v>985</v>
       </c>
       <c r="D151" t="n">
         <v>2.04</v>
@@ -4351,24 +4351,24 @@
         <v>0</v>
       </c>
       <c r="F151" t="n">
-        <v>0.5</v>
+        <v>971.1</v>
       </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="n">
-        <v>0</v>
+        <v>-1.41</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>965.3</v>
+        <v>0.49</v>
       </c>
       <c r="C152" t="n">
-        <v>985</v>
+        <v>0.5</v>
       </c>
       <c r="D152" t="n">
         <v>2.04</v>
@@ -4377,11 +4377,11 @@
         <v>0</v>
       </c>
       <c r="F152" t="n">
-        <v>962.5</v>
+        <v>0.5</v>
       </c>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="n">
-        <v>-2.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153">
@@ -4403,24 +4403,24 @@
         <v>0</v>
       </c>
       <c r="F153" t="n">
-        <v>347.5</v>
+        <v>349.9</v>
       </c>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="n">
-        <v>-3.41</v>
+        <v>-2.74</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>KMSUGAR</t>
+          <t>GLOBALVECT</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>29.26</v>
+        <v>180.69</v>
       </c>
       <c r="C154" t="n">
-        <v>29.85</v>
+        <v>184.34</v>
       </c>
       <c r="D154" t="n">
         <v>2.02</v>
@@ -4429,24 +4429,24 @@
         <v>0</v>
       </c>
       <c r="F154" t="n">
-        <v>30.46</v>
+        <v>181</v>
       </c>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="n">
-        <v>2.04</v>
+        <v>-1.81</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>GLOBALVECT</t>
+          <t>KMSUGAR</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>180.69</v>
+        <v>29.26</v>
       </c>
       <c r="C155" t="n">
-        <v>184.34</v>
+        <v>29.85</v>
       </c>
       <c r="D155" t="n">
         <v>2.02</v>
@@ -4455,11 +4455,11 @@
         <v>0</v>
       </c>
       <c r="F155" t="n">
-        <v>182</v>
+        <v>30.94</v>
       </c>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="n">
-        <v>-1.27</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="156">
@@ -4481,24 +4481,24 @@
         <v>0</v>
       </c>
       <c r="F156" t="n">
-        <v>268.85</v>
+        <v>268</v>
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="n">
-        <v>-1.52</v>
+        <v>-1.83</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>RPPINFRA</t>
+          <t>EIFFL</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>78.44</v>
+        <v>245.13</v>
       </c>
       <c r="C157" t="n">
-        <v>80</v>
+        <v>250</v>
       </c>
       <c r="D157" t="n">
         <v>1.99</v>
@@ -4507,24 +4507,24 @@
         <v>0</v>
       </c>
       <c r="F157" t="n">
-        <v>78.44</v>
+        <v>250</v>
       </c>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="n">
-        <v>-1.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>EIFFL</t>
+          <t>RPPINFRA</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>245.13</v>
+        <v>78.44</v>
       </c>
       <c r="C158" t="n">
-        <v>250</v>
+        <v>80</v>
       </c>
       <c r="D158" t="n">
         <v>1.99</v>
@@ -4533,11 +4533,11 @@
         <v>0</v>
       </c>
       <c r="F158" t="n">
-        <v>246.15</v>
+        <v>80.84</v>
       </c>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="n">
-        <v>-1.54</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="159">
@@ -4559,11 +4559,11 @@
         <v>0</v>
       </c>
       <c r="F159" t="n">
-        <v>127.8</v>
+        <v>128.9</v>
       </c>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="n">
-        <v>-1.68</v>
+        <v>-0.83</v>
       </c>
     </row>
     <row r="160">
@@ -4585,11 +4585,11 @@
         <v>0</v>
       </c>
       <c r="F160" t="n">
-        <v>152.6</v>
+        <v>150.86</v>
       </c>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="n">
-        <v>-2.73</v>
+        <v>-3.84</v>
       </c>
     </row>
     <row r="161">
@@ -4611,11 +4611,11 @@
         <v>0</v>
       </c>
       <c r="F161" t="n">
-        <v>432.95</v>
+        <v>427.35</v>
       </c>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="n">
-        <v>-1.49</v>
+        <v>-2.76</v>
       </c>
     </row>
     <row r="162">
@@ -4663,11 +4663,11 @@
         <v>0</v>
       </c>
       <c r="F163" t="n">
-        <v>1099.15</v>
+        <v>1081</v>
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="n">
-        <v>-2.53</v>
+        <v>-4.14</v>
       </c>
     </row>
     <row r="164">
@@ -4689,11 +4689,11 @@
         <v>0</v>
       </c>
       <c r="F164" t="n">
-        <v>23.69</v>
+        <v>23.5</v>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="n">
-        <v>-1.7</v>
+        <v>-2.49</v>
       </c>
     </row>
     <row r="165">
@@ -4715,11 +4715,11 @@
         <v>0</v>
       </c>
       <c r="F165" t="n">
-        <v>53.67</v>
+        <v>52.75</v>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="n">
-        <v>-2.42</v>
+        <v>-4.09</v>
       </c>
     </row>
     <row r="166">
@@ -4741,24 +4741,24 @@
         <v>0</v>
       </c>
       <c r="F166" t="n">
-        <v>203.8</v>
+        <v>206.2</v>
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="n">
-        <v>-0.59</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>RAJRILTD</t>
+          <t>SINTERCOM</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>21.02</v>
+        <v>72.52</v>
       </c>
       <c r="C167" t="n">
-        <v>21.42</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="D167" t="n">
         <v>1.9</v>
@@ -4767,24 +4767,24 @@
         <v>0</v>
       </c>
       <c r="F167" t="n">
-        <v>21.35</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="n">
-        <v>-0.33</v>
+        <v>-2.44</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>SINTERCOM</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>72.52</v>
+        <v>21.02</v>
       </c>
       <c r="C168" t="n">
-        <v>73.90000000000001</v>
+        <v>21.42</v>
       </c>
       <c r="D168" t="n">
         <v>1.9</v>
@@ -4793,11 +4793,11 @@
         <v>0</v>
       </c>
       <c r="F168" t="n">
-        <v>74.28</v>
+        <v>21.11</v>
       </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="n">
-        <v>0.51</v>
+        <v>-1.45</v>
       </c>
     </row>
     <row r="169">
@@ -4819,11 +4819,11 @@
         <v>0</v>
       </c>
       <c r="F169" t="n">
-        <v>3.74</v>
+        <v>3.78</v>
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="n">
-        <v>-1.06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170">
@@ -4845,11 +4845,11 @@
         <v>0</v>
       </c>
       <c r="F170" t="n">
-        <v>65.59</v>
+        <v>66.95</v>
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="n">
-        <v>-3.19</v>
+        <v>-1.18</v>
       </c>
     </row>
     <row r="171">
@@ -4871,11 +4871,11 @@
         <v>0</v>
       </c>
       <c r="F171" t="n">
-        <v>127.45</v>
+        <v>128</v>
       </c>
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="n">
-        <v>-1.73</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="172">
@@ -4897,11 +4897,11 @@
         <v>0</v>
       </c>
       <c r="F172" t="n">
-        <v>489.1</v>
+        <v>490</v>
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="n">
-        <v>-2.58</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="173">
@@ -4949,11 +4949,11 @@
         <v>0</v>
       </c>
       <c r="F174" t="n">
-        <v>339.55</v>
+        <v>340.9</v>
       </c>
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="n">
-        <v>2.27</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="175">
@@ -4975,11 +4975,11 @@
         <v>0</v>
       </c>
       <c r="F175" t="n">
-        <v>250.56</v>
+        <v>247.35</v>
       </c>
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="n">
-        <v>-2.43</v>
+        <v>-3.68</v>
       </c>
     </row>
     <row r="176">
@@ -5001,11 +5001,11 @@
         <v>0</v>
       </c>
       <c r="F176" t="n">
-        <v>191.48</v>
+        <v>191.17</v>
       </c>
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="n">
-        <v>-1.3</v>
+        <v>-1.46</v>
       </c>
     </row>
     <row r="177">
@@ -5053,11 +5053,11 @@
         <v>0</v>
       </c>
       <c r="F178" t="n">
-        <v>29.87</v>
+        <v>30</v>
       </c>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
-        <v>-2.51</v>
+        <v>-2.09</v>
       </c>
     </row>
     <row r="179">
@@ -5079,11 +5079,11 @@
         <v>0</v>
       </c>
       <c r="F179" t="n">
-        <v>3.2</v>
+        <v>3.27</v>
       </c>
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="n">
-        <v>-4.76</v>
+        <v>-2.68</v>
       </c>
     </row>
     <row r="180">
@@ -5105,11 +5105,11 @@
         <v>0</v>
       </c>
       <c r="F180" t="n">
-        <v>60.96</v>
+        <v>61</v>
       </c>
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="n">
-        <v>-2.31</v>
+        <v>-2.24</v>
       </c>
     </row>
     <row r="181">
@@ -5131,11 +5131,11 @@
         <v>0</v>
       </c>
       <c r="F181" t="n">
-        <v>1.62</v>
+        <v>1.71</v>
       </c>
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="n">
-        <v>-5.26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182">
@@ -5157,11 +5157,11 @@
         <v>0</v>
       </c>
       <c r="F182" t="n">
-        <v>8.550000000000001</v>
+        <v>8.57</v>
       </c>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="n">
-        <v>-0.35</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="183">
@@ -5183,11 +5183,11 @@
         <v>0</v>
       </c>
       <c r="F183" t="n">
-        <v>549.5</v>
+        <v>539</v>
       </c>
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="n">
-        <v>-0.58</v>
+        <v>-2.48</v>
       </c>
     </row>
     <row r="184">
@@ -5209,11 +5209,11 @@
         <v>0</v>
       </c>
       <c r="F184" t="n">
-        <v>5.2</v>
+        <v>5.19</v>
       </c>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="n">
-        <v>-0.95</v>
+        <v>-1.14</v>
       </c>
     </row>
     <row r="185">
@@ -5235,11 +5235,11 @@
         <v>0</v>
       </c>
       <c r="F185" t="n">
-        <v>55.53</v>
+        <v>55.51</v>
       </c>
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="n">
-        <v>-2.56</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="186">
@@ -5261,11 +5261,11 @@
         <v>0</v>
       </c>
       <c r="F186" t="n">
-        <v>4.05</v>
+        <v>3.98</v>
       </c>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="n">
-        <v>-1.94</v>
+        <v>-3.63</v>
       </c>
     </row>
     <row r="187">
@@ -5287,24 +5287,24 @@
         <v>0</v>
       </c>
       <c r="F187" t="n">
-        <v>967.7</v>
+        <v>951</v>
       </c>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="n">
-        <v>-0.88</v>
+        <v>-2.59</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>JAIPURKURT</t>
+          <t>VIPULLTD</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>32.34</v>
+        <v>9.98</v>
       </c>
       <c r="C188" t="n">
-        <v>32.89</v>
+        <v>10.15</v>
       </c>
       <c r="D188" t="n">
         <v>1.7</v>
@@ -5313,24 +5313,24 @@
         <v>0</v>
       </c>
       <c r="F188" t="n">
-        <v>32.69</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="n">
-        <v>-0.61</v>
+        <v>-3.55</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>VIPULLTD</t>
+          <t>JAIPURKURT</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>9.98</v>
+        <v>32.34</v>
       </c>
       <c r="C189" t="n">
-        <v>10.15</v>
+        <v>32.89</v>
       </c>
       <c r="D189" t="n">
         <v>1.7</v>
@@ -5339,11 +5339,11 @@
         <v>0</v>
       </c>
       <c r="F189" t="n">
-        <v>9.9</v>
+        <v>32.65</v>
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="n">
-        <v>-2.46</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="190">
@@ -5365,24 +5365,24 @@
         <v>0</v>
       </c>
       <c r="F190" t="n">
-        <v>373.4</v>
+        <v>381</v>
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="n">
-        <v>-0.43</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>MKPL</t>
+          <t>SPECTRUM</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>5.35</v>
+        <v>1148.7</v>
       </c>
       <c r="C191" t="n">
-        <v>5.44</v>
+        <v>1168</v>
       </c>
       <c r="D191" t="n">
         <v>1.68</v>
@@ -5391,24 +5391,24 @@
         <v>0</v>
       </c>
       <c r="F191" t="n">
-        <v>5.38</v>
+        <v>1215</v>
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="n">
-        <v>-1.1</v>
+        <v>4.02</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>SPECTRUM</t>
+          <t>MKPL</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>1148.7</v>
+        <v>5.35</v>
       </c>
       <c r="C192" t="n">
-        <v>1168</v>
+        <v>5.44</v>
       </c>
       <c r="D192" t="n">
         <v>1.68</v>
@@ -5417,24 +5417,24 @@
         <v>0</v>
       </c>
       <c r="F192" t="n">
-        <v>1159.2</v>
+        <v>5.34</v>
       </c>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="n">
-        <v>-0.75</v>
+        <v>-1.84</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>TTKHLTCARE</t>
+          <t>BIGBLOC</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>898.15</v>
+        <v>48.5</v>
       </c>
       <c r="C193" t="n">
-        <v>913</v>
+        <v>49.3</v>
       </c>
       <c r="D193" t="n">
         <v>1.65</v>
@@ -5443,24 +5443,24 @@
         <v>0</v>
       </c>
       <c r="F193" t="n">
-        <v>903.45</v>
+        <v>48.04</v>
       </c>
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="n">
-        <v>-1.05</v>
+        <v>-2.56</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>BIGBLOC</t>
+          <t>TTKHLTCARE</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>48.5</v>
+        <v>898.15</v>
       </c>
       <c r="C194" t="n">
-        <v>49.3</v>
+        <v>913</v>
       </c>
       <c r="D194" t="n">
         <v>1.65</v>
@@ -5469,24 +5469,24 @@
         <v>0</v>
       </c>
       <c r="F194" t="n">
-        <v>48</v>
+        <v>905</v>
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="n">
-        <v>-2.64</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>DJML</t>
+          <t>SONUINFRA</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>91.5</v>
+        <v>61</v>
       </c>
       <c r="C195" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="D195" t="n">
         <v>1.64</v>
@@ -5495,24 +5495,24 @@
         <v>0</v>
       </c>
       <c r="F195" t="n">
-        <v>91.98999999999999</v>
+        <v>60</v>
       </c>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="n">
-        <v>-1.09</v>
+        <v>-3.23</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>SONUINFRA</t>
+          <t>DJML</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>61</v>
+        <v>91.5</v>
       </c>
       <c r="C196" t="n">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="D196" t="n">
         <v>1.64</v>
@@ -5521,11 +5521,11 @@
         <v>0</v>
       </c>
       <c r="F196" t="n">
-        <v>60</v>
+        <v>92.89</v>
       </c>
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="n">
-        <v>-3.23</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="197">
@@ -5547,11 +5547,11 @@
         <v>0</v>
       </c>
       <c r="F197" t="n">
-        <v>19</v>
+        <v>19.55</v>
       </c>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="n">
-        <v>1.39</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="198">
@@ -5573,11 +5573,11 @@
         <v>0</v>
       </c>
       <c r="F198" t="n">
-        <v>98.8</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="n">
-        <v>-1.2</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="199">
@@ -5599,11 +5599,11 @@
         <v>0</v>
       </c>
       <c r="F199" t="n">
-        <v>305.1</v>
+        <v>296.25</v>
       </c>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="n">
-        <v>-4.64</v>
+        <v>-7.41</v>
       </c>
     </row>
     <row r="200">
@@ -5625,11 +5625,11 @@
         <v>0</v>
       </c>
       <c r="F200" t="n">
-        <v>944.6</v>
+        <v>939.7</v>
       </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="n">
-        <v>-0.04</v>
+        <v>-0.5600000000000001</v>
       </c>
     </row>
     <row r="201">
@@ -5651,11 +5651,11 @@
         <v>0</v>
       </c>
       <c r="F201" t="n">
-        <v>112.25</v>
+        <v>108</v>
       </c>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="n">
-        <v>6.4</v>
+        <v>2.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-05-26 07:03 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,14 +461,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>174.4</v>
+        <v>166.8</v>
       </c>
       <c r="C2" t="n">
-        <v>209.28</v>
+        <v>200.16</v>
       </c>
       <c r="D2" t="n">
         <v>20</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GCHOTELS</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>88.7</v>
+        <v>209.28</v>
       </c>
       <c r="C3" t="n">
-        <v>104.9</v>
+        <v>250.01</v>
       </c>
       <c r="D3" t="n">
-        <v>18.26</v>
+        <v>19.46</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GREENLAM</t>
+          <t>AWFIS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>237.23</v>
+        <v>360.6</v>
       </c>
       <c r="C4" t="n">
-        <v>275.6</v>
+        <v>424</v>
       </c>
       <c r="D4" t="n">
-        <v>16.17</v>
+        <v>17.58</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MANAKSIA</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>57.87</v>
+        <v>12.32</v>
       </c>
       <c r="C5" t="n">
-        <v>67</v>
+        <v>14.04</v>
       </c>
       <c r="D5" t="n">
-        <v>15.78</v>
+        <v>13.96</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHAMUNDA</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>43.15</v>
+        <v>838.25</v>
       </c>
       <c r="C6" t="n">
-        <v>49.5</v>
+        <v>950</v>
       </c>
       <c r="D6" t="n">
-        <v>14.72</v>
+        <v>13.33</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HARIOMPIPE</t>
+          <t>KRSNAA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>344.35</v>
+        <v>553.85</v>
       </c>
       <c r="C7" t="n">
-        <v>392</v>
+        <v>622.55</v>
       </c>
       <c r="D7" t="n">
-        <v>13.84</v>
+        <v>12.4</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>VIKRAN</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>64.8</v>
+        <v>444.95</v>
       </c>
       <c r="C8" t="n">
-        <v>73.5</v>
+        <v>498.2</v>
       </c>
       <c r="D8" t="n">
-        <v>13.43</v>
+        <v>11.97</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>UNIPARTS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10.42</v>
+        <v>559.5</v>
       </c>
       <c r="C9" t="n">
+        <v>625</v>
+      </c>
+      <c r="D9" t="n">
         <v>11.71</v>
-      </c>
-      <c r="D9" t="n">
-        <v>12.38</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,14 +637,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TINNARUBR</t>
+          <t>SUNDRMBRAK</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>740.15</v>
+        <v>757</v>
       </c>
       <c r="C10" t="n">
-        <v>820</v>
+        <v>838.7</v>
       </c>
       <c r="D10" t="n">
         <v>10.79</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>VICTORYEV</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>17.85</v>
+        <v>743.2</v>
       </c>
       <c r="C11" t="n">
-        <v>19.75</v>
+        <v>820</v>
       </c>
       <c r="D11" t="n">
-        <v>10.64</v>
+        <v>10.33</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>KSHINTL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.07</v>
+        <v>695</v>
       </c>
       <c r="C12" t="n">
-        <v>1.18</v>
+        <v>760</v>
       </c>
       <c r="D12" t="n">
-        <v>10.28</v>
+        <v>9.35</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SHRIKRISH</t>
+          <t>FLEXITUFF</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>42.03</v>
+        <v>6.94</v>
       </c>
       <c r="C13" t="n">
-        <v>46.3</v>
+        <v>7.55</v>
       </c>
       <c r="D13" t="n">
-        <v>10.16</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GUJRAFFIA</t>
+          <t>GCHOTELS</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>41.25</v>
+        <v>106.4</v>
       </c>
       <c r="C14" t="n">
-        <v>45.37</v>
+        <v>115</v>
       </c>
       <c r="D14" t="n">
-        <v>9.99</v>
+        <v>8.08</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RCDL</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>26.4</v>
+        <v>37.06</v>
       </c>
       <c r="C15" t="n">
-        <v>28.8</v>
+        <v>40</v>
       </c>
       <c r="D15" t="n">
-        <v>9.09</v>
+        <v>7.93</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>UNIVCABLES</t>
+          <t>HALDER</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1012.05</v>
+        <v>217.58</v>
       </c>
       <c r="C16" t="n">
-        <v>1100</v>
+        <v>232.79</v>
       </c>
       <c r="D16" t="n">
-        <v>8.69</v>
+        <v>6.99</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>K2INFRA</t>
+          <t>IFBIND</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>55</v>
+        <v>1052.2</v>
       </c>
       <c r="C17" t="n">
-        <v>59.45</v>
+        <v>1119.9</v>
       </c>
       <c r="D17" t="n">
-        <v>8.09</v>
+        <v>6.43</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PRECWIRE</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>415.15</v>
+        <v>4.93</v>
       </c>
       <c r="C18" t="n">
-        <v>448</v>
+        <v>5.24</v>
       </c>
       <c r="D18" t="n">
-        <v>7.91</v>
+        <v>6.29</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SCHAND</t>
+          <t>VICTORYEV</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>170.97</v>
+        <v>21.4</v>
       </c>
       <c r="C19" t="n">
-        <v>184.2</v>
+        <v>22.7</v>
       </c>
       <c r="D19" t="n">
-        <v>7.74</v>
+        <v>6.07</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SAGARDEEP</t>
+          <t>ROSSELLIND</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>23.67</v>
+        <v>55.54</v>
       </c>
       <c r="C20" t="n">
-        <v>25.5</v>
+        <v>58.7</v>
       </c>
       <c r="D20" t="n">
-        <v>7.73</v>
+        <v>5.69</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TUNWAL</t>
+          <t>SILLYMONKS</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>34</v>
+        <v>17.01</v>
       </c>
       <c r="C21" t="n">
-        <v>36.6</v>
+        <v>17.9</v>
       </c>
       <c r="D21" t="n">
-        <v>7.65</v>
+        <v>5.23</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BLISSGVS</t>
+          <t>MEGASTAR</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>300.35</v>
+        <v>290.25</v>
       </c>
       <c r="C22" t="n">
-        <v>322.35</v>
+        <v>305</v>
       </c>
       <c r="D22" t="n">
-        <v>7.32</v>
+        <v>5.08</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>INDOTECH</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>148.21</v>
+        <v>2438.9</v>
       </c>
       <c r="C23" t="n">
-        <v>158.9</v>
+        <v>2560.8</v>
       </c>
       <c r="D23" t="n">
-        <v>7.21</v>
+        <v>5</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BALAJIPHOS</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>98</v>
+        <v>463.2</v>
       </c>
       <c r="C24" t="n">
-        <v>105</v>
+        <v>486.35</v>
       </c>
       <c r="D24" t="n">
-        <v>7.14</v>
+        <v>5</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DHARARAIL</t>
+          <t>NIRAJISPAT</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>127.95</v>
+        <v>205.2</v>
       </c>
       <c r="C25" t="n">
-        <v>137</v>
+        <v>215.46</v>
       </c>
       <c r="D25" t="n">
-        <v>7.07</v>
+        <v>5</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TIL</t>
+          <t>REGAAL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>191.69</v>
+        <v>90.69</v>
       </c>
       <c r="C26" t="n">
-        <v>205</v>
+        <v>95.22</v>
       </c>
       <c r="D26" t="n">
-        <v>6.94</v>
+        <v>5</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1450.5</v>
+        <v>367</v>
       </c>
       <c r="C27" t="n">
-        <v>1550</v>
+        <v>385.35</v>
       </c>
       <c r="D27" t="n">
-        <v>6.86</v>
+        <v>5</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>COUNCODOS</t>
+          <t>BIRLACABLE</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4.86</v>
+        <v>167.52</v>
       </c>
       <c r="C28" t="n">
-        <v>5.18</v>
+        <v>175.89</v>
       </c>
       <c r="D28" t="n">
-        <v>6.58</v>
+        <v>5</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LAXMIDENTL</t>
+          <t>ANLON</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>249.28</v>
+        <v>614</v>
       </c>
       <c r="C29" t="n">
-        <v>265.2</v>
+        <v>644.7</v>
       </c>
       <c r="D29" t="n">
-        <v>6.39</v>
+        <v>5</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TECHD</t>
+          <t>OMAXAUTO</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>682.3</v>
+        <v>227.79</v>
       </c>
       <c r="C30" t="n">
-        <v>725</v>
+        <v>239.17</v>
       </c>
       <c r="D30" t="n">
-        <v>6.26</v>
+        <v>5</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>HALEOSLABS</t>
+          <t>KANORICHEM</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1658.8</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="C31" t="n">
-        <v>1759.9</v>
+        <v>96</v>
       </c>
       <c r="D31" t="n">
-        <v>6.09</v>
+        <v>5</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>NGLFINE</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2735.8</v>
+        <v>56.41</v>
       </c>
       <c r="C32" t="n">
-        <v>2900</v>
+        <v>59.23</v>
       </c>
       <c r="D32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>NEOCHEM</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>112</v>
+        <v>299.55</v>
       </c>
       <c r="C33" t="n">
-        <v>118.7</v>
+        <v>314.5</v>
       </c>
       <c r="D33" t="n">
-        <v>5.98</v>
+        <v>4.99</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.54</v>
+        <v>190.4</v>
       </c>
       <c r="C34" t="n">
-        <v>0.57</v>
+        <v>199.9</v>
       </c>
       <c r="D34" t="n">
-        <v>5.56</v>
+        <v>4.99</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>KCK</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>13.25</v>
+        <v>14.83</v>
       </c>
       <c r="C35" t="n">
-        <v>13.95</v>
+        <v>15.57</v>
       </c>
       <c r="D35" t="n">
-        <v>5.28</v>
+        <v>4.99</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MERCANTILE</t>
+          <t>APSISAERO</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>26.03</v>
+        <v>327.4</v>
       </c>
       <c r="C36" t="n">
-        <v>27.39</v>
+        <v>343.75</v>
       </c>
       <c r="D36" t="n">
-        <v>5.22</v>
+        <v>4.99</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>NBIFIN</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1900.1</v>
+        <v>17.64</v>
       </c>
       <c r="C37" t="n">
-        <v>1999</v>
+        <v>18.52</v>
       </c>
       <c r="D37" t="n">
-        <v>5.2</v>
+        <v>4.99</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PRECOT</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>732.6</v>
+        <v>26.25</v>
       </c>
       <c r="C38" t="n">
-        <v>770</v>
+        <v>27.56</v>
       </c>
       <c r="D38" t="n">
-        <v>5.11</v>
+        <v>4.99</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OBSCP</t>
+          <t>OSWALAGRO</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>460.75</v>
+        <v>45.89</v>
       </c>
       <c r="C39" t="n">
-        <v>484</v>
+        <v>48.17</v>
       </c>
       <c r="D39" t="n">
-        <v>5.05</v>
+        <v>4.97</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>CKKRETAIL</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>441.15</v>
+        <v>130.8</v>
       </c>
       <c r="C40" t="n">
-        <v>463.2</v>
+        <v>137.3</v>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>4.97</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>RITEZONE</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>159.55</v>
+        <v>21.15</v>
       </c>
       <c r="C41" t="n">
-        <v>167.52</v>
+        <v>22.2</v>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>4.96</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>HVAX</t>
+          <t>SYNOPTICS</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>813.75</v>
+        <v>48.45</v>
       </c>
       <c r="C42" t="n">
-        <v>854.4</v>
+        <v>50.85</v>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OMAXAUTO</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>216.95</v>
+        <v>198.09</v>
       </c>
       <c r="C43" t="n">
-        <v>227.79</v>
+        <v>207.9</v>
       </c>
       <c r="D43" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DHRUV</t>
+          <t>RFBL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>31</v>
+        <v>66.84999999999999</v>
       </c>
       <c r="C44" t="n">
-        <v>32.55</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="D44" t="n">
-        <v>5</v>
+        <v>4.94</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MANAKSTEEL</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>65.64</v>
+        <v>73.7</v>
       </c>
       <c r="C45" t="n">
-        <v>68.92</v>
+        <v>77.34</v>
       </c>
       <c r="D45" t="n">
-        <v>5</v>
+        <v>4.94</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PARTH</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>427</v>
+        <v>1.62</v>
       </c>
       <c r="C46" t="n">
-        <v>448.35</v>
+        <v>1.7</v>
       </c>
       <c r="D46" t="n">
-        <v>5</v>
+        <v>4.94</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>FAZE3Q</t>
+          <t>ABANSENT</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>482.55</v>
+        <v>28.38</v>
       </c>
       <c r="C47" t="n">
-        <v>506.65</v>
+        <v>29.78</v>
       </c>
       <c r="D47" t="n">
-        <v>4.99</v>
+        <v>4.93</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>KESORAMIND</t>
+          <t>NEWJAISA</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>13.03</v>
+        <v>22.6</v>
       </c>
       <c r="C48" t="n">
-        <v>13.68</v>
+        <v>23.7</v>
       </c>
       <c r="D48" t="n">
-        <v>4.99</v>
+        <v>4.87</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DEEDEV</t>
+          <t>MANAKSTEEL</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>523.8</v>
+        <v>68.92</v>
       </c>
       <c r="C49" t="n">
-        <v>549.95</v>
+        <v>72.25</v>
       </c>
       <c r="D49" t="n">
-        <v>4.99</v>
+        <v>4.83</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>GSTL</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>349.55</v>
+        <v>18.8</v>
       </c>
       <c r="C50" t="n">
-        <v>367</v>
+        <v>19.7</v>
       </c>
       <c r="D50" t="n">
-        <v>4.99</v>
+        <v>4.79</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BNAGROCHEM</t>
+          <t>GLOBALE</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>327.66</v>
+        <v>12.4</v>
       </c>
       <c r="C51" t="n">
-        <v>344</v>
+        <v>12.99</v>
       </c>
       <c r="D51" t="n">
-        <v>4.99</v>
+        <v>4.76</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ANIKINDS</t>
+          <t>SURYALA</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>43.53</v>
+        <v>373.9</v>
       </c>
       <c r="C52" t="n">
-        <v>45.7</v>
+        <v>391.1</v>
       </c>
       <c r="D52" t="n">
-        <v>4.99</v>
+        <v>4.6</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PALREDTEC</t>
+          <t>MANAKALUCO</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>44.2</v>
+        <v>35.1</v>
       </c>
       <c r="C53" t="n">
-        <v>46.4</v>
+        <v>36.7</v>
       </c>
       <c r="D53" t="n">
-        <v>4.98</v>
+        <v>4.56</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ABANSENT</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>27.03</v>
+        <v>5.06</v>
       </c>
       <c r="C54" t="n">
-        <v>28.37</v>
+        <v>5.29</v>
       </c>
       <c r="D54" t="n">
-        <v>4.96</v>
+        <v>4.55</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LATTEYS</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>22.77</v>
+        <v>132.95</v>
       </c>
       <c r="C55" t="n">
-        <v>23.9</v>
+        <v>139</v>
       </c>
       <c r="D55" t="n">
-        <v>4.96</v>
+        <v>4.55</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>RFBL</t>
+          <t>EQUIPPP</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>63.7</v>
+        <v>15.22</v>
       </c>
       <c r="C56" t="n">
-        <v>66.84999999999999</v>
+        <v>15.9</v>
       </c>
       <c r="D56" t="n">
-        <v>4.95</v>
+        <v>4.47</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>WOL3D</t>
+          <t>TREJHARA</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>204.85</v>
+        <v>147.32</v>
       </c>
       <c r="C57" t="n">
-        <v>215</v>
+        <v>153.9</v>
       </c>
       <c r="D57" t="n">
-        <v>4.95</v>
+        <v>4.47</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DIVINEHIRA</t>
+          <t>SICAGEN</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>323.9</v>
+        <v>56.43</v>
       </c>
       <c r="C58" t="n">
-        <v>339.9</v>
+        <v>58.95</v>
       </c>
       <c r="D58" t="n">
-        <v>4.94</v>
+        <v>4.47</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>SUDARSCHEM</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>3.85</v>
+        <v>1043.95</v>
       </c>
       <c r="C59" t="n">
-        <v>4.04</v>
+        <v>1090</v>
       </c>
       <c r="D59" t="n">
-        <v>4.94</v>
+        <v>4.41</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>IDEAFORGE</t>
+          <t>BYKE</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>775.95</v>
+        <v>35.82</v>
       </c>
       <c r="C60" t="n">
-        <v>814</v>
+        <v>37.38</v>
       </c>
       <c r="D60" t="n">
-        <v>4.9</v>
+        <v>4.36</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BYKE</t>
+          <t>RUBYMILLS</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>36.1</v>
+        <v>273.1</v>
       </c>
       <c r="C61" t="n">
-        <v>37.87</v>
+        <v>285</v>
       </c>
       <c r="D61" t="n">
-        <v>4.9</v>
+        <v>4.36</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>APSISAERO</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>311.85</v>
+        <v>0.23</v>
       </c>
       <c r="C62" t="n">
-        <v>327.1</v>
+        <v>0.24</v>
       </c>
       <c r="D62" t="n">
-        <v>4.89</v>
+        <v>4.35</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>SUNDARAM</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>3.27</v>
+        <v>1.39</v>
       </c>
       <c r="C63" t="n">
-        <v>3.43</v>
+        <v>1.45</v>
       </c>
       <c r="D63" t="n">
-        <v>4.89</v>
+        <v>4.32</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MONARCH</t>
+          <t>RAJESHEXPO</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>320.35</v>
+        <v>112.81</v>
       </c>
       <c r="C64" t="n">
-        <v>336</v>
+        <v>117.65</v>
       </c>
       <c r="D64" t="n">
-        <v>4.89</v>
+        <v>4.29</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SANCO</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>3.93</v>
+        <v>3.52</v>
       </c>
       <c r="C65" t="n">
-        <v>4.12</v>
+        <v>3.67</v>
       </c>
       <c r="D65" t="n">
-        <v>4.83</v>
+        <v>4.26</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ADISOFT</t>
+          <t>AAKAAR</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>193.1</v>
+        <v>72.95</v>
       </c>
       <c r="C66" t="n">
-        <v>202.35</v>
+        <v>76</v>
       </c>
       <c r="D66" t="n">
-        <v>4.79</v>
+        <v>4.18</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>FAZE3Q</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>390.3</v>
+        <v>506.65</v>
       </c>
       <c r="C67" t="n">
-        <v>409</v>
+        <v>527.75</v>
       </c>
       <c r="D67" t="n">
-        <v>4.79</v>
+        <v>4.16</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>MONOPHARMA</t>
+          <t>GUJRAFFIA</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>11.5</v>
+        <v>45.37</v>
       </c>
       <c r="C68" t="n">
-        <v>12.05</v>
+        <v>47.25</v>
       </c>
       <c r="D68" t="n">
-        <v>4.78</v>
+        <v>4.14</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SHIVAMAUTO</t>
+          <t>NIMBSPROJ</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>17.99</v>
+        <v>219.01</v>
       </c>
       <c r="C69" t="n">
-        <v>18.85</v>
+        <v>227.99</v>
       </c>
       <c r="D69" t="n">
-        <v>4.78</v>
+        <v>4.1</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>3.36</v>
+        <v>5.96</v>
       </c>
       <c r="C70" t="n">
-        <v>3.52</v>
+        <v>6.2</v>
       </c>
       <c r="D70" t="n">
-        <v>4.76</v>
+        <v>4.03</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BESTAGRO</t>
+          <t>CRIZAC</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>17.78</v>
+        <v>223.99</v>
       </c>
       <c r="C71" t="n">
-        <v>18.6</v>
+        <v>233</v>
       </c>
       <c r="D71" t="n">
-        <v>4.61</v>
+        <v>4.02</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BEWLTD</t>
+          <t>SYSTMTXC</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>61.15</v>
+        <v>65.8</v>
       </c>
       <c r="C72" t="n">
-        <v>63.95</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="D72" t="n">
-        <v>4.58</v>
+        <v>3.95</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>ORTEL</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>229.35</v>
+        <v>1.59</v>
       </c>
       <c r="C73" t="n">
-        <v>239.8</v>
+        <v>1.65</v>
       </c>
       <c r="D73" t="n">
-        <v>4.56</v>
+        <v>3.77</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>IDEAFORGE</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1.76</v>
+        <v>814.7</v>
       </c>
       <c r="C74" t="n">
-        <v>1.84</v>
+        <v>845</v>
       </c>
       <c r="D74" t="n">
-        <v>4.55</v>
+        <v>3.72</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SAIPARENT</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>486.7</v>
+        <v>8.65</v>
       </c>
       <c r="C75" t="n">
-        <v>508</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="D75" t="n">
-        <v>4.38</v>
+        <v>3.7</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TVVISION</t>
+          <t>UNIDT</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>5.26</v>
+        <v>230.55</v>
       </c>
       <c r="C76" t="n">
-        <v>5.49</v>
+        <v>238.99</v>
       </c>
       <c r="D76" t="n">
-        <v>4.37</v>
+        <v>3.66</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>RKDL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.23</v>
+        <v>21.13</v>
       </c>
       <c r="C77" t="n">
-        <v>0.24</v>
+        <v>21.9</v>
       </c>
       <c r="D77" t="n">
-        <v>4.35</v>
+        <v>3.64</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>AAKAAR</t>
+          <t>PINELABS</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>69.5</v>
+        <v>146.2</v>
       </c>
       <c r="C78" t="n">
-        <v>72.5</v>
+        <v>151.5</v>
       </c>
       <c r="D78" t="n">
-        <v>4.32</v>
+        <v>3.63</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>DAVANGERE</t>
+          <t>MERCANTILE</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>4.4</v>
+        <v>26.84</v>
       </c>
       <c r="C79" t="n">
-        <v>4.59</v>
+        <v>27.8</v>
       </c>
       <c r="D79" t="n">
-        <v>4.32</v>
+        <v>3.58</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>2.09</v>
+        <v>7.05</v>
       </c>
       <c r="C80" t="n">
-        <v>2.18</v>
+        <v>7.3</v>
       </c>
       <c r="D80" t="n">
-        <v>4.31</v>
+        <v>3.55</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>KREBSBIO</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>3.97</v>
+        <v>61.81</v>
       </c>
       <c r="C81" t="n">
-        <v>4.14</v>
+        <v>64</v>
       </c>
       <c r="D81" t="n">
-        <v>4.28</v>
+        <v>3.54</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>KSR</t>
+          <t>BTTL</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>37.5</v>
+        <v>34.48</v>
       </c>
       <c r="C82" t="n">
-        <v>39.1</v>
+        <v>35.7</v>
       </c>
       <c r="D82" t="n">
-        <v>4.27</v>
+        <v>3.54</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ARTEMISMED</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>273.03</v>
+        <v>0.85</v>
       </c>
       <c r="C83" t="n">
-        <v>284.65</v>
+        <v>0.88</v>
       </c>
       <c r="D83" t="n">
-        <v>4.26</v>
+        <v>3.53</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>KRITINUT</t>
+          <t>CPEDU</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>90.59</v>
+        <v>176.96</v>
       </c>
       <c r="C84" t="n">
-        <v>94.41</v>
+        <v>183.2</v>
       </c>
       <c r="D84" t="n">
-        <v>4.22</v>
+        <v>3.53</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAIFL</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>5.95</v>
+        <v>62.29</v>
       </c>
       <c r="C85" t="n">
-        <v>6.2</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="D85" t="n">
-        <v>4.2</v>
+        <v>3.53</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>RAMCOSYS</t>
+          <t>EXCELSOFT</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>469.9</v>
+        <v>87.62</v>
       </c>
       <c r="C86" t="n">
-        <v>489.35</v>
+        <v>90.69</v>
       </c>
       <c r="D86" t="n">
-        <v>4.14</v>
+        <v>3.5</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>NILE</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>31.57</v>
+        <v>1816.2</v>
       </c>
       <c r="C87" t="n">
-        <v>32.87</v>
+        <v>1879.8</v>
       </c>
       <c r="D87" t="n">
-        <v>4.12</v>
+        <v>3.5</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GGBL</t>
+          <t>GKWLIMITED</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>336.1</v>
+        <v>1704.6</v>
       </c>
       <c r="C88" t="n">
-        <v>349.9</v>
+        <v>1764.3</v>
       </c>
       <c r="D88" t="n">
-        <v>4.11</v>
+        <v>3.5</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ZODIAC</t>
+          <t>RELIABLE</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>305.2</v>
+        <v>133.24</v>
       </c>
       <c r="C89" t="n">
-        <v>317.7</v>
+        <v>137.9</v>
       </c>
       <c r="D89" t="n">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>TVSSCS</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>1082.05</v>
+        <v>120.81</v>
       </c>
       <c r="C90" t="n">
-        <v>1126.45</v>
+        <v>125</v>
       </c>
       <c r="D90" t="n">
-        <v>4.1</v>
+        <v>3.47</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TVSELECT</t>
+          <t>NIRAJ</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>465.95</v>
+        <v>28.89</v>
       </c>
       <c r="C91" t="n">
-        <v>485</v>
+        <v>29.89</v>
       </c>
       <c r="D91" t="n">
-        <v>4.09</v>
+        <v>3.46</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SUPREMEENG</t>
+          <t>SCANSTL</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.98</v>
+        <v>38.42</v>
       </c>
       <c r="C92" t="n">
-        <v>1.02</v>
+        <v>39.75</v>
       </c>
       <c r="D92" t="n">
-        <v>4.08</v>
+        <v>3.46</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>165.33</v>
+        <v>10.42</v>
       </c>
       <c r="C93" t="n">
-        <v>172</v>
+        <v>10.78</v>
       </c>
       <c r="D93" t="n">
-        <v>4.03</v>
+        <v>3.45</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>DPEL</t>
+          <t>TFL</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>507.55</v>
+        <v>12.76</v>
       </c>
       <c r="C94" t="n">
-        <v>528</v>
+        <v>13.2</v>
       </c>
       <c r="D94" t="n">
-        <v>4.03</v>
+        <v>3.45</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SHIVAMILLS</t>
+          <t>ASHOKAMET</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>65.37</v>
+        <v>15.95</v>
       </c>
       <c r="C95" t="n">
-        <v>68</v>
+        <v>16.5</v>
       </c>
       <c r="D95" t="n">
-        <v>4.02</v>
+        <v>3.45</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>MANGALAM</t>
+          <t>PASUPTAC</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>29.41</v>
+        <v>57.52</v>
       </c>
       <c r="C96" t="n">
-        <v>30.59</v>
+        <v>59.5</v>
       </c>
       <c r="D96" t="n">
-        <v>4.01</v>
+        <v>3.44</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>PVSL</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1855.6</v>
+        <v>105.44</v>
       </c>
       <c r="C97" t="n">
-        <v>1930</v>
+        <v>109</v>
       </c>
       <c r="D97" t="n">
-        <v>4.01</v>
+        <v>3.38</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PERFECT</t>
+          <t>FOCUS</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>2.5</v>
+        <v>83.39</v>
       </c>
       <c r="C98" t="n">
-        <v>2.6</v>
+        <v>86.2</v>
       </c>
       <c r="D98" t="n">
-        <v>4</v>
+        <v>3.37</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>15</v>
+        <v>21.95</v>
       </c>
       <c r="C99" t="n">
-        <v>15.6</v>
+        <v>22.69</v>
       </c>
       <c r="D99" t="n">
-        <v>4</v>
+        <v>3.37</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>HECPROJECT</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>124.58</v>
+        <v>7.16</v>
       </c>
       <c r="C100" t="n">
-        <v>129.55</v>
+        <v>7.4</v>
       </c>
       <c r="D100" t="n">
-        <v>3.99</v>
+        <v>3.35</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>EUROBOND</t>
+          <t>CHEMPLASTS</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>182.73</v>
+        <v>243.89</v>
       </c>
       <c r="C101" t="n">
-        <v>190</v>
+        <v>252</v>
       </c>
       <c r="D101" t="n">
-        <v>3.98</v>
+        <v>3.33</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MARSONS</t>
+          <t>ELLEN</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>151.6</v>
+        <v>265.35</v>
       </c>
       <c r="C102" t="n">
-        <v>157.52</v>
+        <v>274.15</v>
       </c>
       <c r="D102" t="n">
-        <v>3.91</v>
+        <v>3.32</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>AARON</t>
+          <t>AURIGROW</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>119.17</v>
+        <v>0.31</v>
       </c>
       <c r="C103" t="n">
-        <v>123.8</v>
+        <v>0.32</v>
       </c>
       <c r="D103" t="n">
-        <v>3.89</v>
+        <v>3.23</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>LASA</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>6.5</v>
+        <v>8.06</v>
       </c>
       <c r="C104" t="n">
-        <v>6.75</v>
+        <v>8.32</v>
       </c>
       <c r="D104" t="n">
-        <v>3.85</v>
+        <v>3.23</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>THEMISMED</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>1.57</v>
+        <v>100.24</v>
       </c>
       <c r="C105" t="n">
-        <v>1.63</v>
+        <v>103.45</v>
       </c>
       <c r="D105" t="n">
-        <v>3.82</v>
+        <v>3.2</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>SUDEEPPHRM</t>
+          <t>UMAEXPORTS</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>673.35</v>
+        <v>25.19</v>
       </c>
       <c r="C106" t="n">
-        <v>699</v>
+        <v>25.99</v>
       </c>
       <c r="D106" t="n">
-        <v>3.81</v>
+        <v>3.18</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>DHARARAIL</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>6981.5</v>
+        <v>135.85</v>
       </c>
       <c r="C107" t="n">
-        <v>7237</v>
+        <v>140</v>
       </c>
       <c r="D107" t="n">
-        <v>3.66</v>
+        <v>3.05</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>KILITCH</t>
+          <t>JETFREIGHT</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>182.27</v>
+        <v>20.32</v>
       </c>
       <c r="C108" t="n">
-        <v>188.9</v>
+        <v>20.94</v>
       </c>
       <c r="D108" t="n">
-        <v>3.64</v>
+        <v>3.05</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SUBEXLTD</t>
+          <t>DPEL</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>11.05</v>
+        <v>508.75</v>
       </c>
       <c r="C109" t="n">
-        <v>11.45</v>
+        <v>524</v>
       </c>
       <c r="D109" t="n">
-        <v>3.62</v>
+        <v>3</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>CHEVIOT</t>
+          <t>NIPPOBATRY</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>1129.2</v>
+        <v>363.35</v>
       </c>
       <c r="C110" t="n">
-        <v>1170</v>
+        <v>374</v>
       </c>
       <c r="D110" t="n">
-        <v>3.61</v>
+        <v>2.93</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MAHAPEXLTD</t>
+          <t>SAKHTISUG</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>47.69</v>
+        <v>17.96</v>
       </c>
       <c r="C111" t="n">
-        <v>49.4</v>
+        <v>18.48</v>
       </c>
       <c r="D111" t="n">
-        <v>3.59</v>
+        <v>2.9</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>KOPRAN</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>11.78</v>
+        <v>188.48</v>
       </c>
       <c r="C112" t="n">
-        <v>12.2</v>
+        <v>193.9</v>
       </c>
       <c r="D112" t="n">
-        <v>3.57</v>
+        <v>2.88</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>7</v>
+        <v>3.82</v>
       </c>
       <c r="C113" t="n">
-        <v>7.25</v>
+        <v>3.93</v>
       </c>
       <c r="D113" t="n">
-        <v>3.57</v>
+        <v>2.88</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>PURPLEUTED</t>
+          <t>SHRIRAMPPS</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>403.3</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="C114" t="n">
-        <v>417.7</v>
+        <v>93.5</v>
       </c>
       <c r="D114" t="n">
-        <v>3.57</v>
+        <v>2.86</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SHARDUL</t>
+          <t>DJML</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>27.71</v>
+        <v>98.58</v>
       </c>
       <c r="C115" t="n">
-        <v>28.7</v>
+        <v>101.4</v>
       </c>
       <c r="D115" t="n">
-        <v>3.57</v>
+        <v>2.86</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MAGADSUGAR</t>
+          <t>TAMBOLIIN</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>473.25</v>
+        <v>179.87</v>
       </c>
       <c r="C116" t="n">
-        <v>490</v>
+        <v>184.99</v>
       </c>
       <c r="D116" t="n">
-        <v>3.54</v>
+        <v>2.85</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>KOTHARIPRO</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>72.64</v>
+        <v>14.08</v>
       </c>
       <c r="C117" t="n">
-        <v>75.2</v>
+        <v>14.48</v>
       </c>
       <c r="D117" t="n">
-        <v>3.52</v>
+        <v>2.84</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>UNITECH</t>
+          <t>VCL</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>5.13</v>
+        <v>1.42</v>
       </c>
       <c r="C118" t="n">
-        <v>5.31</v>
+        <v>1.46</v>
       </c>
       <c r="D118" t="n">
-        <v>3.51</v>
+        <v>2.82</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>BANARBEADS</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>113.6</v>
+        <v>55.25</v>
       </c>
       <c r="C119" t="n">
-        <v>117.59</v>
+        <v>56.8</v>
       </c>
       <c r="D119" t="n">
-        <v>3.51</v>
+        <v>2.81</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>TRAVELFOOD</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>1124.1</v>
+        <v>1152.6</v>
       </c>
       <c r="C120" t="n">
-        <v>1163.4</v>
+        <v>1185</v>
       </c>
       <c r="D120" t="n">
-        <v>3.5</v>
+        <v>2.81</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>FERMENTA</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>301.45</v>
+        <v>768.4</v>
       </c>
       <c r="C121" t="n">
-        <v>312</v>
+        <v>790</v>
       </c>
       <c r="D121" t="n">
-        <v>3.5</v>
+        <v>2.81</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>EIFFL</t>
+          <t>BANG</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>233.44</v>
+        <v>37.17</v>
       </c>
       <c r="C122" t="n">
-        <v>241.6</v>
+        <v>38.2</v>
       </c>
       <c r="D122" t="n">
-        <v>3.5</v>
+        <v>2.77</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BAJAJST</t>
+          <t>BALPHARMA</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>407.85</v>
+        <v>88.56</v>
       </c>
       <c r="C123" t="n">
-        <v>421.95</v>
+        <v>91</v>
       </c>
       <c r="D123" t="n">
-        <v>3.46</v>
+        <v>2.76</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>TAMBOLIIN</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>165.34</v>
+        <v>14.69</v>
       </c>
       <c r="C124" t="n">
-        <v>171.05</v>
+        <v>15.09</v>
       </c>
       <c r="D124" t="n">
-        <v>3.45</v>
+        <v>2.72</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>DONEAR</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>731.85</v>
+        <v>90.44</v>
       </c>
       <c r="C125" t="n">
-        <v>757</v>
+        <v>92.89</v>
       </c>
       <c r="D125" t="n">
-        <v>3.44</v>
+        <v>2.71</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>BASML</t>
+          <t>BVCL</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>24.17</v>
+        <v>42.81</v>
       </c>
       <c r="C126" t="n">
-        <v>25</v>
+        <v>43.96</v>
       </c>
       <c r="D126" t="n">
-        <v>3.43</v>
+        <v>2.69</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>CENTURYPLY</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>766.65</v>
+        <v>24.23</v>
       </c>
       <c r="C127" t="n">
-        <v>792.95</v>
+        <v>24.88</v>
       </c>
       <c r="D127" t="n">
-        <v>3.43</v>
+        <v>2.68</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>HINDPETRO</t>
+          <t>PIGL</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>389.65</v>
+        <v>105.18</v>
       </c>
       <c r="C128" t="n">
-        <v>403</v>
+        <v>107.98</v>
       </c>
       <c r="D128" t="n">
-        <v>3.43</v>
+        <v>2.66</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>INTERARCH</t>
+          <t>MONEYBOXX</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>1750.3</v>
+        <v>72.88</v>
       </c>
       <c r="C129" t="n">
-        <v>1810</v>
+        <v>74.8</v>
       </c>
       <c r="D129" t="n">
-        <v>3.41</v>
+        <v>2.63</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>DAICHI</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>36.07</v>
+        <v>256</v>
       </c>
       <c r="C130" t="n">
-        <v>37.3</v>
+        <v>262.7</v>
       </c>
       <c r="D130" t="n">
-        <v>3.41</v>
+        <v>2.62</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>MANGALAM</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>16.8</v>
+        <v>29.14</v>
       </c>
       <c r="C131" t="n">
-        <v>17.37</v>
+        <v>29.9</v>
       </c>
       <c r="D131" t="n">
-        <v>3.39</v>
+        <v>2.61</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ASHOKAMET</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>15.94</v>
+        <v>92.55</v>
       </c>
       <c r="C132" t="n">
-        <v>16.48</v>
+        <v>94.95</v>
       </c>
       <c r="D132" t="n">
-        <v>3.39</v>
+        <v>2.59</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>PCJEWELLER</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>77.38</v>
+        <v>8.92</v>
       </c>
       <c r="C133" t="n">
-        <v>80</v>
+        <v>9.15</v>
       </c>
       <c r="D133" t="n">
-        <v>3.39</v>
+        <v>2.58</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>MMP</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>287.33</v>
+        <v>1136.15</v>
       </c>
       <c r="C134" t="n">
-        <v>297</v>
+        <v>1165.4</v>
       </c>
       <c r="D134" t="n">
-        <v>3.37</v>
+        <v>2.57</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>SPECTRUM</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>1734.4</v>
+        <v>1394.1</v>
       </c>
       <c r="C135" t="n">
-        <v>1792.8</v>
+        <v>1429.9</v>
       </c>
       <c r="D135" t="n">
-        <v>3.37</v>
+        <v>2.57</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>3578.4</v>
+        <v>3.9</v>
       </c>
       <c r="C136" t="n">
-        <v>3699</v>
+        <v>4</v>
       </c>
       <c r="D136" t="n">
-        <v>3.37</v>
+        <v>2.56</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>KALPATARU</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>333.8</v>
+        <v>42.9</v>
       </c>
       <c r="C137" t="n">
-        <v>345</v>
+        <v>44</v>
       </c>
       <c r="D137" t="n">
-        <v>3.36</v>
+        <v>2.56</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>BANSWRAS</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>127.42</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="C138" t="n">
-        <v>131.7</v>
+        <v>67</v>
       </c>
       <c r="D138" t="n">
-        <v>3.36</v>
+        <v>2.52</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>BIRLAMONEY</t>
+          <t>SELMC</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>138.41</v>
+        <v>29.75</v>
       </c>
       <c r="C139" t="n">
-        <v>143</v>
+        <v>30.49</v>
       </c>
       <c r="D139" t="n">
-        <v>3.32</v>
+        <v>2.49</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>MODIRUBBER</t>
+          <t>GANGAFORGE</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>128.74</v>
+        <v>2.41</v>
       </c>
       <c r="C140" t="n">
-        <v>133</v>
+        <v>2.47</v>
       </c>
       <c r="D140" t="n">
-        <v>3.31</v>
+        <v>2.49</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>STARCEMENT</t>
+          <t>MBLINFRA</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>220.99</v>
+        <v>26.28</v>
       </c>
       <c r="C141" t="n">
-        <v>228.3</v>
+        <v>26.93</v>
       </c>
       <c r="D141" t="n">
-        <v>3.31</v>
+        <v>2.47</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>MADHUCON</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>5.46</v>
+        <v>6.9</v>
       </c>
       <c r="C142" t="n">
-        <v>5.64</v>
+        <v>7.07</v>
       </c>
       <c r="D142" t="n">
-        <v>3.3</v>
+        <v>2.46</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>MANOMAY</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>182.96</v>
+        <v>116.15</v>
       </c>
       <c r="C143" t="n">
-        <v>189</v>
+        <v>119</v>
       </c>
       <c r="D143" t="n">
-        <v>3.3</v>
+        <v>2.45</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>KOTARISUG</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>36.48</v>
+        <v>25.75</v>
       </c>
       <c r="C144" t="n">
-        <v>37.68</v>
+        <v>26.38</v>
       </c>
       <c r="D144" t="n">
-        <v>3.29</v>
+        <v>2.45</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>PRADPME</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>139.47</v>
+        <v>421.7</v>
       </c>
       <c r="C145" t="n">
-        <v>144.06</v>
+        <v>432</v>
       </c>
       <c r="D145" t="n">
-        <v>3.29</v>
+        <v>2.44</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SHRIRAMPPS</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>84.13</v>
+        <v>3.29</v>
       </c>
       <c r="C146" t="n">
-        <v>86.89</v>
+        <v>3.37</v>
       </c>
       <c r="D146" t="n">
-        <v>3.28</v>
+        <v>2.43</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>MAYURUNIQ</t>
+          <t>ENERGYDEV</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>704.9</v>
+        <v>16.97</v>
       </c>
       <c r="C147" t="n">
-        <v>727.85</v>
+        <v>17.38</v>
       </c>
       <c r="D147" t="n">
-        <v>3.26</v>
+        <v>2.42</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>NDLVENTURE</t>
+          <t>SUPREMEPWR</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>129.24</v>
+        <v>253.85</v>
       </c>
       <c r="C148" t="n">
-        <v>133.45</v>
+        <v>260</v>
       </c>
       <c r="D148" t="n">
-        <v>3.26</v>
+        <v>2.42</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>AYE</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>140.43</v>
+        <v>2.1</v>
       </c>
       <c r="C149" t="n">
-        <v>145</v>
+        <v>2.15</v>
       </c>
       <c r="D149" t="n">
-        <v>3.25</v>
+        <v>2.38</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>HYBRIDFIN</t>
+          <t>HARIOMPIPE</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>18.5</v>
+        <v>413.2</v>
       </c>
       <c r="C150" t="n">
-        <v>19.1</v>
+        <v>423</v>
       </c>
       <c r="D150" t="n">
-        <v>3.24</v>
+        <v>2.37</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>SHIVALIK</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>1.55</v>
+        <v>264.55</v>
       </c>
       <c r="C151" t="n">
-        <v>1.6</v>
+        <v>270.8</v>
       </c>
       <c r="D151" t="n">
-        <v>3.23</v>
+        <v>2.36</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ARIHANTCAP</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>67.43000000000001</v>
+        <v>11.01</v>
       </c>
       <c r="C152" t="n">
-        <v>69.59999999999999</v>
+        <v>11.27</v>
       </c>
       <c r="D152" t="n">
-        <v>3.22</v>
+        <v>2.36</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>CAPTRUST</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>295.6</v>
+        <v>14.46</v>
       </c>
       <c r="C153" t="n">
-        <v>305</v>
+        <v>14.8</v>
       </c>
       <c r="D153" t="n">
-        <v>3.18</v>
+        <v>2.35</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>CHEMCON</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>184.15</v>
+        <v>985</v>
       </c>
       <c r="C154" t="n">
-        <v>190</v>
+        <v>1008</v>
       </c>
       <c r="D154" t="n">
-        <v>3.18</v>
+        <v>2.34</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>UNIMECH</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>11.97</v>
+        <v>951.8</v>
       </c>
       <c r="C155" t="n">
-        <v>12.35</v>
+        <v>973.9</v>
       </c>
       <c r="D155" t="n">
-        <v>3.17</v>
+        <v>2.32</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>QPOWER</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>1124.1</v>
+        <v>6.1</v>
       </c>
       <c r="C156" t="n">
-        <v>1159.7</v>
+        <v>6.24</v>
       </c>
       <c r="D156" t="n">
-        <v>3.17</v>
+        <v>2.3</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>VALUE360</t>
+          <t>TNTELE</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>74.65000000000001</v>
+        <v>9.16</v>
       </c>
       <c r="C157" t="n">
-        <v>77</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="D157" t="n">
-        <v>3.15</v>
+        <v>2.29</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>AMDIND</t>
+          <t>DEVIT</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>45.49</v>
+        <v>29.32</v>
       </c>
       <c r="C158" t="n">
-        <v>46.9</v>
+        <v>29.99</v>
       </c>
       <c r="D158" t="n">
-        <v>3.1</v>
+        <v>2.29</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MOHITIND</t>
+          <t>MAZDA</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>23.01</v>
+        <v>211.16</v>
       </c>
       <c r="C159" t="n">
-        <v>23.72</v>
+        <v>215.97</v>
       </c>
       <c r="D159" t="n">
-        <v>3.09</v>
+        <v>2.28</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>RAMASTEEL</t>
+          <t>LGHL</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>5.22</v>
+        <v>231.75</v>
       </c>
       <c r="C160" t="n">
-        <v>5.38</v>
+        <v>237</v>
       </c>
       <c r="D160" t="n">
-        <v>3.07</v>
+        <v>2.27</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>MOTOGENFIN</t>
+          <t>RHFL</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>27.02</v>
+        <v>2.22</v>
       </c>
       <c r="C161" t="n">
-        <v>27.85</v>
+        <v>2.27</v>
       </c>
       <c r="D161" t="n">
-        <v>3.07</v>
+        <v>2.25</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>LYPSAGEMS</t>
+          <t>IRISDOREME</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>4.92</v>
+        <v>35.6</v>
       </c>
       <c r="C162" t="n">
-        <v>5.07</v>
+        <v>36.4</v>
       </c>
       <c r="D162" t="n">
-        <v>3.05</v>
+        <v>2.25</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>0.33</v>
+        <v>11.15</v>
       </c>
       <c r="C163" t="n">
-        <v>0.34</v>
+        <v>11.4</v>
       </c>
       <c r="D163" t="n">
-        <v>3.03</v>
+        <v>2.24</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>GLOSTERLTD</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>635.8</v>
+        <v>0.45</v>
       </c>
       <c r="C164" t="n">
-        <v>655</v>
+        <v>0.46</v>
       </c>
       <c r="D164" t="n">
-        <v>3.02</v>
+        <v>2.22</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>GALLANTT</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>8</v>
+        <v>699.5</v>
       </c>
       <c r="C165" t="n">
-        <v>8.24</v>
+        <v>715</v>
       </c>
       <c r="D165" t="n">
-        <v>3</v>
+        <v>2.22</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>GOYALALUM</t>
+          <t>KOTHARIPET</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>6.71</v>
+        <v>129.14</v>
       </c>
       <c r="C166" t="n">
-        <v>6.91</v>
+        <v>132</v>
       </c>
       <c r="D166" t="n">
-        <v>2.98</v>
+        <v>2.21</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ANANTAM</t>
+          <t>SCHAND</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>105.37</v>
+        <v>172.19</v>
       </c>
       <c r="C167" t="n">
-        <v>108.5</v>
+        <v>175.95</v>
       </c>
       <c r="D167" t="n">
-        <v>2.97</v>
+        <v>2.18</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>RAYMONDREL</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>26.71</v>
+        <v>613.15</v>
       </c>
       <c r="C168" t="n">
-        <v>27.5</v>
+        <v>626.5</v>
       </c>
       <c r="D168" t="n">
-        <v>2.96</v>
+        <v>2.18</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>REGAAL</t>
+          <t>INA</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>87.42</v>
+        <v>146.83</v>
       </c>
       <c r="C169" t="n">
-        <v>90</v>
+        <v>150</v>
       </c>
       <c r="D169" t="n">
-        <v>2.95</v>
+        <v>2.16</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>RADIANTCMS</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>146.68</v>
+        <v>41.41</v>
       </c>
       <c r="C170" t="n">
-        <v>151</v>
+        <v>42.3</v>
       </c>
       <c r="D170" t="n">
-        <v>2.95</v>
+        <v>2.15</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>HARSHA</t>
+          <t>GULFPETRO</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>406.45</v>
+        <v>33.29</v>
       </c>
       <c r="C171" t="n">
-        <v>418.45</v>
+        <v>34</v>
       </c>
       <c r="D171" t="n">
-        <v>2.95</v>
+        <v>2.13</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>NILE</t>
+          <t>TCIEXP</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>1838</v>
+        <v>512.15</v>
       </c>
       <c r="C172" t="n">
-        <v>1892</v>
+        <v>523</v>
       </c>
       <c r="D172" t="n">
-        <v>2.94</v>
+        <v>2.12</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>JNKINDIA</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>387.6</v>
+        <v>2.39</v>
       </c>
       <c r="C173" t="n">
-        <v>399</v>
+        <v>2.44</v>
       </c>
       <c r="D173" t="n">
-        <v>2.94</v>
+        <v>2.09</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>RMDRIP</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>18.83</v>
+        <v>171.31</v>
       </c>
       <c r="C174" t="n">
-        <v>19.38</v>
+        <v>174.89</v>
       </c>
       <c r="D174" t="n">
-        <v>2.92</v>
+        <v>2.09</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>HEALTHX</t>
+          <t>HTMEDIA</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>289.05</v>
+        <v>22.01</v>
       </c>
       <c r="C175" t="n">
-        <v>297.5</v>
+        <v>22.47</v>
       </c>
       <c r="D175" t="n">
-        <v>2.92</v>
+        <v>2.09</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>100.95</v>
+        <v>0.48</v>
       </c>
       <c r="C176" t="n">
-        <v>103.9</v>
+        <v>0.49</v>
       </c>
       <c r="D176" t="n">
-        <v>2.92</v>
+        <v>2.08</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>JLHL</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>1356.6</v>
+        <v>343.8</v>
       </c>
       <c r="C177" t="n">
-        <v>1396</v>
+        <v>350.95</v>
       </c>
       <c r="D177" t="n">
-        <v>2.9</v>
+        <v>2.08</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>DOLLAR</t>
+          <t>UNIENTER</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>277.05</v>
+        <v>107.52</v>
       </c>
       <c r="C178" t="n">
-        <v>285</v>
+        <v>109.75</v>
       </c>
       <c r="D178" t="n">
-        <v>2.87</v>
+        <v>2.07</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>IRIS</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>4.88</v>
+        <v>263.47</v>
       </c>
       <c r="C179" t="n">
-        <v>5.02</v>
+        <v>268.88</v>
       </c>
       <c r="D179" t="n">
-        <v>2.87</v>
+        <v>2.05</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>LINDEINDIA</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>7222</v>
+        <v>4.88</v>
       </c>
       <c r="C180" t="n">
-        <v>7428</v>
+        <v>4.98</v>
       </c>
       <c r="D180" t="n">
-        <v>2.85</v>
+        <v>2.05</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>24.27</v>
+        <v>6.36</v>
       </c>
       <c r="C181" t="n">
-        <v>24.96</v>
+        <v>6.49</v>
       </c>
       <c r="D181" t="n">
-        <v>2.84</v>
+        <v>2.04</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>PAKKA</t>
+          <t>MAJESAUT</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>91.20999999999999</v>
+        <v>338</v>
       </c>
       <c r="C182" t="n">
-        <v>93.8</v>
+        <v>344.9</v>
       </c>
       <c r="D182" t="n">
-        <v>2.84</v>
+        <v>2.04</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>RADAAN</t>
+          <t>AIRAN</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>3.17</v>
+        <v>16.19</v>
       </c>
       <c r="C183" t="n">
-        <v>3.26</v>
+        <v>16.52</v>
       </c>
       <c r="D183" t="n">
-        <v>2.84</v>
+        <v>2.04</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>AARTECH</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>13.37</v>
+        <v>42.86</v>
       </c>
       <c r="C184" t="n">
-        <v>13.75</v>
+        <v>43.73</v>
       </c>
       <c r="D184" t="n">
-        <v>2.84</v>
+        <v>2.03</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>ANDHRAPAP</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>63.2</v>
+        <v>6.44</v>
       </c>
       <c r="C185" t="n">
-        <v>64.98999999999999</v>
+        <v>6.57</v>
       </c>
       <c r="D185" t="n">
-        <v>2.83</v>
+        <v>2.02</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>BALAMINES</t>
+          <t>TVTODAY</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>1822.5</v>
+        <v>109.98</v>
       </c>
       <c r="C186" t="n">
-        <v>1874</v>
+        <v>112.2</v>
       </c>
       <c r="D186" t="n">
-        <v>2.83</v>
+        <v>2.02</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>TVSSCS</t>
+          <t>DISAQ</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>121.57</v>
+        <v>11567</v>
       </c>
       <c r="C187" t="n">
-        <v>125</v>
+        <v>11800</v>
       </c>
       <c r="D187" t="n">
-        <v>2.82</v>
+        <v>2.01</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>AARVI</t>
+          <t>FIBERWEB</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>128.38</v>
+        <v>29.31</v>
       </c>
       <c r="C188" t="n">
-        <v>132</v>
+        <v>29.9</v>
       </c>
       <c r="D188" t="n">
-        <v>2.82</v>
+        <v>2.01</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>FOODSIN</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>55.45</v>
+        <v>0.5</v>
       </c>
       <c r="C189" t="n">
-        <v>57</v>
+        <v>0.51</v>
       </c>
       <c r="D189" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>LAHOTIOV</t>
+          <t>BALUFORGE</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>42.8</v>
+        <v>466.7</v>
       </c>
       <c r="C190" t="n">
-        <v>44</v>
+        <v>476.05</v>
       </c>
       <c r="D190" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>ELCIDIN</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>368.7</v>
+        <v>122490</v>
       </c>
       <c r="C191" t="n">
-        <v>379</v>
+        <v>124940</v>
       </c>
       <c r="D191" t="n">
-        <v>2.79</v>
+        <v>2</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>ABCOTS</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>213.07</v>
+        <v>7.49</v>
       </c>
       <c r="C192" t="n">
-        <v>219</v>
+        <v>7.64</v>
       </c>
       <c r="D192" t="n">
-        <v>2.78</v>
+        <v>2</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>FCL</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>29.2</v>
+        <v>39.03</v>
       </c>
       <c r="C193" t="n">
-        <v>30</v>
+        <v>39.81</v>
       </c>
       <c r="D193" t="n">
-        <v>2.74</v>
+        <v>2</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>KAVDEFENCE</t>
+          <t>IWP</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>62.77</v>
+        <v>35.35</v>
       </c>
       <c r="C194" t="n">
-        <v>64.48999999999999</v>
+        <v>36.05</v>
       </c>
       <c r="D194" t="n">
-        <v>2.74</v>
+        <v>1.98</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ELPROINTL</t>
+          <t>KHAICHEM</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>172.3</v>
+        <v>55.59</v>
       </c>
       <c r="C195" t="n">
-        <v>176.99</v>
+        <v>56.69</v>
       </c>
       <c r="D195" t="n">
-        <v>2.72</v>
+        <v>1.98</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>PGEL</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>467</v>
+        <v>47.37</v>
       </c>
       <c r="C196" t="n">
-        <v>479.6</v>
+        <v>48.3</v>
       </c>
       <c r="D196" t="n">
-        <v>2.7</v>
+        <v>1.96</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>6.29</v>
+        <v>6.63</v>
       </c>
       <c r="C197" t="n">
-        <v>6.46</v>
+        <v>6.76</v>
       </c>
       <c r="D197" t="n">
-        <v>2.7</v>
+        <v>1.96</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>TREJHARA</t>
+          <t>HEADSUP</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>150.8</v>
+        <v>7.19</v>
       </c>
       <c r="C198" t="n">
-        <v>154.85</v>
+        <v>7.33</v>
       </c>
       <c r="D198" t="n">
-        <v>2.69</v>
+        <v>1.95</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>AVANA</t>
+          <t>CENTEXT</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>154.35</v>
+        <v>20.62</v>
       </c>
       <c r="C199" t="n">
-        <v>158.5</v>
+        <v>21.02</v>
       </c>
       <c r="D199" t="n">
-        <v>2.69</v>
+        <v>1.94</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>SIL</t>
+          <t>ARROWGREEN</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>16.01</v>
+        <v>456.15</v>
       </c>
       <c r="C200" t="n">
-        <v>16.44</v>
+        <v>464.95</v>
       </c>
       <c r="D200" t="n">
-        <v>2.69</v>
+        <v>1.93</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>UCAL</t>
+          <t>KNAGRI</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>89.3</v>
+        <v>191.82</v>
       </c>
       <c r="C201" t="n">
-        <v>91.69</v>
+        <v>195.5</v>
       </c>
       <c r="D201" t="n">
-        <v>2.68</v>
+        <v>1.92</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-05-27 07:51 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>ALUWIND</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>166.8</v>
+        <v>49.75</v>
       </c>
       <c r="C2" t="n">
-        <v>200.16</v>
+        <v>56</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>12.56</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>ALKALI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>209.28</v>
+        <v>74.55</v>
       </c>
       <c r="C3" t="n">
-        <v>250.01</v>
+        <v>83</v>
       </c>
       <c r="D3" t="n">
-        <v>19.46</v>
+        <v>11.33</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AWFIS</t>
+          <t>BIRLAPREC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>360.6</v>
+        <v>44.93</v>
       </c>
       <c r="C4" t="n">
-        <v>424</v>
+        <v>49.99</v>
       </c>
       <c r="D4" t="n">
-        <v>17.58</v>
+        <v>11.26</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12.32</v>
+        <v>200.16</v>
       </c>
       <c r="C5" t="n">
-        <v>14.04</v>
+        <v>220.17</v>
       </c>
       <c r="D5" t="n">
-        <v>13.96</v>
+        <v>10</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>FONEBOX</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>838.25</v>
+        <v>99.2</v>
       </c>
       <c r="C6" t="n">
-        <v>950</v>
+        <v>109</v>
       </c>
       <c r="D6" t="n">
-        <v>13.33</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KRSNAA</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>553.85</v>
+        <v>1048.9</v>
       </c>
       <c r="C7" t="n">
-        <v>622.55</v>
+        <v>1150</v>
       </c>
       <c r="D7" t="n">
-        <v>12.4</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>SPECTRUM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>444.95</v>
+        <v>1383.3</v>
       </c>
       <c r="C8" t="n">
-        <v>498.2</v>
+        <v>1500</v>
       </c>
       <c r="D8" t="n">
-        <v>11.97</v>
+        <v>8.44</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UNIPARTS</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>559.5</v>
+        <v>470.6</v>
       </c>
       <c r="C9" t="n">
-        <v>625</v>
+        <v>510</v>
       </c>
       <c r="D9" t="n">
-        <v>11.71</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SUNDRMBRAK</t>
+          <t>INDOAMIN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>757</v>
+        <v>134.57</v>
       </c>
       <c r="C10" t="n">
-        <v>838.7</v>
+        <v>145.01</v>
       </c>
       <c r="D10" t="n">
-        <v>10.79</v>
+        <v>7.76</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>JOCIL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>743.2</v>
+        <v>145.94</v>
       </c>
       <c r="C11" t="n">
-        <v>820</v>
+        <v>157</v>
       </c>
       <c r="D11" t="n">
-        <v>10.33</v>
+        <v>7.58</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>KSHINTL</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>695</v>
+        <v>44.47</v>
       </c>
       <c r="C12" t="n">
-        <v>760</v>
+        <v>47.7</v>
       </c>
       <c r="D12" t="n">
-        <v>9.35</v>
+        <v>7.26</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FLEXITUFF</t>
+          <t>TIMEX</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6.94</v>
+        <v>374.6</v>
       </c>
       <c r="C13" t="n">
-        <v>7.55</v>
+        <v>401.35</v>
       </c>
       <c r="D13" t="n">
-        <v>8.789999999999999</v>
+        <v>7.14</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GCHOTELS</t>
+          <t>LGHL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>106.4</v>
+        <v>235.4</v>
       </c>
       <c r="C14" t="n">
-        <v>115</v>
+        <v>251</v>
       </c>
       <c r="D14" t="n">
-        <v>8.08</v>
+        <v>6.63</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>TAALTECH</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>37.06</v>
+        <v>3190.4</v>
       </c>
       <c r="C15" t="n">
-        <v>40</v>
+        <v>3398</v>
       </c>
       <c r="D15" t="n">
-        <v>7.93</v>
+        <v>6.51</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HALDER</t>
+          <t>FLYSBS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>217.58</v>
+        <v>433.9</v>
       </c>
       <c r="C16" t="n">
-        <v>232.79</v>
+        <v>462</v>
       </c>
       <c r="D16" t="n">
-        <v>6.99</v>
+        <v>6.48</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IFBIND</t>
+          <t>SHARDUL</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1052.2</v>
+        <v>28.12</v>
       </c>
       <c r="C17" t="n">
-        <v>1119.9</v>
+        <v>29.9</v>
       </c>
       <c r="D17" t="n">
-        <v>6.43</v>
+        <v>6.33</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>FINPIPE</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4.93</v>
+        <v>178.14</v>
       </c>
       <c r="C18" t="n">
-        <v>5.24</v>
+        <v>188.6</v>
       </c>
       <c r="D18" t="n">
-        <v>6.29</v>
+        <v>5.87</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>VICTORYEV</t>
+          <t>JKTYRE</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>21.4</v>
+        <v>394.15</v>
       </c>
       <c r="C19" t="n">
-        <v>22.7</v>
+        <v>416</v>
       </c>
       <c r="D19" t="n">
-        <v>6.07</v>
+        <v>5.54</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ROSSELLIND</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>55.54</v>
+        <v>251.13</v>
       </c>
       <c r="C20" t="n">
-        <v>58.7</v>
+        <v>265</v>
       </c>
       <c r="D20" t="n">
-        <v>5.69</v>
+        <v>5.52</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SILLYMONKS</t>
+          <t>PGHL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>17.01</v>
+        <v>5652.5</v>
       </c>
       <c r="C21" t="n">
-        <v>17.9</v>
+        <v>5949</v>
       </c>
       <c r="D21" t="n">
-        <v>5.23</v>
+        <v>5.25</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MEGASTAR</t>
+          <t>SBGLP</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>290.25</v>
+        <v>25.66</v>
       </c>
       <c r="C22" t="n">
-        <v>305</v>
+        <v>27</v>
       </c>
       <c r="D22" t="n">
-        <v>5.08</v>
+        <v>5.22</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>INDOTECH</t>
+          <t>CARRARO</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2438.9</v>
+        <v>608.5</v>
       </c>
       <c r="C23" t="n">
-        <v>2560.8</v>
+        <v>640.1</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>5.19</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -949,10 +949,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>463.2</v>
+        <v>486.35</v>
       </c>
       <c r="C24" t="n">
-        <v>486.35</v>
+        <v>510.65</v>
       </c>
       <c r="D24" t="n">
         <v>5</v>
@@ -967,14 +967,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NIRAJISPAT</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>205.2</v>
+        <v>1161.05</v>
       </c>
       <c r="C25" t="n">
-        <v>215.46</v>
+        <v>1219.1</v>
       </c>
       <c r="D25" t="n">
         <v>5</v>
@@ -989,14 +989,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REGAAL</t>
+          <t>AUSOMENT</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>90.69</v>
+        <v>139.62</v>
       </c>
       <c r="C26" t="n">
-        <v>95.22</v>
+        <v>146.6</v>
       </c>
       <c r="D26" t="n">
         <v>5</v>
@@ -1011,14 +1011,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>KANORICHEM</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>367</v>
+        <v>96</v>
       </c>
       <c r="C27" t="n">
-        <v>385.35</v>
+        <v>100.8</v>
       </c>
       <c r="D27" t="n">
         <v>5</v>
@@ -1037,10 +1037,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>167.52</v>
+        <v>175.89</v>
       </c>
       <c r="C28" t="n">
-        <v>175.89</v>
+        <v>184.68</v>
       </c>
       <c r="D28" t="n">
         <v>5</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANLON</t>
+          <t>CKKRETAIL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>614</v>
+        <v>137.25</v>
       </c>
       <c r="C29" t="n">
-        <v>644.7</v>
+        <v>144.1</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>OMAXAUTO</t>
+          <t>KHAITANLTD</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>227.79</v>
+        <v>133.75</v>
       </c>
       <c r="C30" t="n">
-        <v>239.17</v>
+        <v>140.43</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>KANORICHEM</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>91.43000000000001</v>
+        <v>32.05</v>
       </c>
       <c r="C31" t="n">
-        <v>96</v>
+        <v>33.65</v>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>POSITRON</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>56.41</v>
+        <v>207.25</v>
       </c>
       <c r="C32" t="n">
-        <v>59.23</v>
+        <v>217.6</v>
       </c>
       <c r="D32" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1147,10 +1147,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>299.55</v>
+        <v>314.5</v>
       </c>
       <c r="C33" t="n">
-        <v>314.5</v>
+        <v>330.2</v>
       </c>
       <c r="D33" t="n">
         <v>4.99</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>190.4</v>
+        <v>397.2</v>
       </c>
       <c r="C34" t="n">
-        <v>199.9</v>
+        <v>417</v>
       </c>
       <c r="D34" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>ANIKINDS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>14.83</v>
+        <v>44.2</v>
       </c>
       <c r="C35" t="n">
-        <v>15.57</v>
+        <v>46.4</v>
       </c>
       <c r="D35" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>APSISAERO</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>327.4</v>
+        <v>25.34</v>
       </c>
       <c r="C36" t="n">
-        <v>343.75</v>
+        <v>26.6</v>
       </c>
       <c r="D36" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>DCMFINSERV</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>17.64</v>
+        <v>5.43</v>
       </c>
       <c r="C37" t="n">
-        <v>18.52</v>
+        <v>5.7</v>
       </c>
       <c r="D37" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>TGL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>26.25</v>
+        <v>22.4</v>
       </c>
       <c r="C38" t="n">
-        <v>27.56</v>
+        <v>23.5</v>
       </c>
       <c r="D38" t="n">
-        <v>4.99</v>
+        <v>4.91</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OSWALAGRO</t>
+          <t>LANDMARK</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>45.89</v>
+        <v>381.3</v>
       </c>
       <c r="C39" t="n">
-        <v>48.17</v>
+        <v>400</v>
       </c>
       <c r="D39" t="n">
-        <v>4.97</v>
+        <v>4.9</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CKKRETAIL</t>
+          <t>SONAMAC</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>130.8</v>
+        <v>37.8</v>
       </c>
       <c r="C40" t="n">
-        <v>137.3</v>
+        <v>39.65</v>
       </c>
       <c r="D40" t="n">
-        <v>4.97</v>
+        <v>4.89</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>RITEZONE</t>
+          <t>LAKPRE</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>21.15</v>
+        <v>5.74</v>
       </c>
       <c r="C41" t="n">
-        <v>22.2</v>
+        <v>6.02</v>
       </c>
       <c r="D41" t="n">
-        <v>4.96</v>
+        <v>4.88</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SYNOPTICS</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>48.45</v>
+        <v>4.31</v>
       </c>
       <c r="C42" t="n">
-        <v>50.85</v>
+        <v>4.52</v>
       </c>
       <c r="D42" t="n">
-        <v>4.95</v>
+        <v>4.87</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>198.09</v>
+        <v>9.08</v>
       </c>
       <c r="C43" t="n">
-        <v>207.9</v>
+        <v>9.52</v>
       </c>
       <c r="D43" t="n">
-        <v>4.95</v>
+        <v>4.85</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>RFBL</t>
+          <t>GSTL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>66.84999999999999</v>
+        <v>19.7</v>
       </c>
       <c r="C44" t="n">
-        <v>70.15000000000001</v>
+        <v>20.65</v>
       </c>
       <c r="D44" t="n">
-        <v>4.94</v>
+        <v>4.82</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>73.7</v>
+        <v>27.66</v>
       </c>
       <c r="C45" t="n">
-        <v>77.34</v>
+        <v>28.99</v>
       </c>
       <c r="D45" t="n">
-        <v>4.94</v>
+        <v>4.81</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1.62</v>
+        <v>3.8</v>
       </c>
       <c r="C46" t="n">
-        <v>1.7</v>
+        <v>3.98</v>
       </c>
       <c r="D46" t="n">
-        <v>4.94</v>
+        <v>4.74</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ABANSENT</t>
+          <t>IL&amp;FSENGG</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>28.38</v>
+        <v>30.36</v>
       </c>
       <c r="C47" t="n">
-        <v>29.78</v>
+        <v>31.8</v>
       </c>
       <c r="D47" t="n">
-        <v>4.93</v>
+        <v>4.74</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>NEWJAISA</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>22.6</v>
+        <v>59.23</v>
       </c>
       <c r="C48" t="n">
-        <v>23.7</v>
+        <v>62</v>
       </c>
       <c r="D48" t="n">
-        <v>4.87</v>
+        <v>4.68</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MANAKSTEEL</t>
+          <t>JETFREIGHT</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>68.92</v>
+        <v>20.4</v>
       </c>
       <c r="C49" t="n">
-        <v>72.25</v>
+        <v>21.35</v>
       </c>
       <c r="D49" t="n">
-        <v>4.83</v>
+        <v>4.66</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GSTL</t>
+          <t>JKIPL</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>18.8</v>
+        <v>84.59</v>
       </c>
       <c r="C50" t="n">
-        <v>19.7</v>
+        <v>88.5</v>
       </c>
       <c r="D50" t="n">
-        <v>4.79</v>
+        <v>4.62</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>GLOBALE</t>
+          <t>MAXPOSURE</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>12.4</v>
+        <v>36.3</v>
       </c>
       <c r="C51" t="n">
-        <v>12.99</v>
+        <v>37.95</v>
       </c>
       <c r="D51" t="n">
-        <v>4.76</v>
+        <v>4.55</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SURYALA</t>
+          <t>PANSARI</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>373.9</v>
+        <v>291.7</v>
       </c>
       <c r="C52" t="n">
-        <v>391.1</v>
+        <v>304.9</v>
       </c>
       <c r="D52" t="n">
-        <v>4.6</v>
+        <v>4.53</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MANAKALUCO</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>35.1</v>
+        <v>0.89</v>
       </c>
       <c r="C53" t="n">
-        <v>36.7</v>
+        <v>0.93</v>
       </c>
       <c r="D53" t="n">
-        <v>4.56</v>
+        <v>4.49</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>VIYASH</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>5.06</v>
+        <v>257.36</v>
       </c>
       <c r="C54" t="n">
-        <v>5.29</v>
+        <v>268.89</v>
       </c>
       <c r="D54" t="n">
-        <v>4.55</v>
+        <v>4.48</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OWAIS</t>
+          <t>JINDWORLD</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>132.95</v>
+        <v>30.15</v>
       </c>
       <c r="C55" t="n">
-        <v>139</v>
+        <v>31.5</v>
       </c>
       <c r="D55" t="n">
-        <v>4.55</v>
+        <v>4.48</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,14 +1649,14 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>EQUIPPP</t>
+          <t>ATLANTAELE</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>15.22</v>
+        <v>1788.9</v>
       </c>
       <c r="C56" t="n">
-        <v>15.9</v>
+        <v>1868.9</v>
       </c>
       <c r="D56" t="n">
         <v>4.47</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TREJHARA</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>147.32</v>
+        <v>1.57</v>
       </c>
       <c r="C57" t="n">
-        <v>153.9</v>
+        <v>1.64</v>
       </c>
       <c r="D57" t="n">
-        <v>4.47</v>
+        <v>4.46</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SICAGEN</t>
+          <t>SURANI</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>56.43</v>
+        <v>126.35</v>
       </c>
       <c r="C58" t="n">
-        <v>58.95</v>
+        <v>131.95</v>
       </c>
       <c r="D58" t="n">
-        <v>4.47</v>
+        <v>4.43</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SUDARSCHEM</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1043.95</v>
+        <v>47.69</v>
       </c>
       <c r="C59" t="n">
-        <v>1090</v>
+        <v>49.8</v>
       </c>
       <c r="D59" t="n">
-        <v>4.41</v>
+        <v>4.42</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BYKE</t>
+          <t>REDTAPE</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>35.82</v>
+        <v>148.49</v>
       </c>
       <c r="C60" t="n">
-        <v>37.38</v>
+        <v>155</v>
       </c>
       <c r="D60" t="n">
-        <v>4.36</v>
+        <v>4.38</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>RUBYMILLS</t>
+          <t>PGHH</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>273.1</v>
+        <v>9873</v>
       </c>
       <c r="C61" t="n">
-        <v>285</v>
+        <v>10300</v>
       </c>
       <c r="D61" t="n">
-        <v>4.36</v>
+        <v>4.32</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.23</v>
+        <v>6.25</v>
       </c>
       <c r="C62" t="n">
-        <v>0.24</v>
+        <v>6.52</v>
       </c>
       <c r="D62" t="n">
-        <v>4.35</v>
+        <v>4.32</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>ARMANFIN</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1.39</v>
+        <v>1750.9</v>
       </c>
       <c r="C63" t="n">
-        <v>1.45</v>
+        <v>1823.8</v>
       </c>
       <c r="D63" t="n">
-        <v>4.32</v>
+        <v>4.16</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>RAJESHEXPO</t>
+          <t>SHIVATEX</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>112.81</v>
+        <v>166.19</v>
       </c>
       <c r="C64" t="n">
-        <v>117.65</v>
+        <v>173.1</v>
       </c>
       <c r="D64" t="n">
-        <v>4.29</v>
+        <v>4.16</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>URAVIDEF</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>3.52</v>
+        <v>118.01</v>
       </c>
       <c r="C65" t="n">
-        <v>3.67</v>
+        <v>122.9</v>
       </c>
       <c r="D65" t="n">
-        <v>4.26</v>
+        <v>4.14</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AAKAAR</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>72.95</v>
+        <v>454.25</v>
       </c>
       <c r="C66" t="n">
-        <v>76</v>
+        <v>473</v>
       </c>
       <c r="D66" t="n">
-        <v>4.18</v>
+        <v>4.13</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>FAZE3Q</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>506.65</v>
+        <v>430.35</v>
       </c>
       <c r="C67" t="n">
-        <v>527.75</v>
+        <v>448</v>
       </c>
       <c r="D67" t="n">
-        <v>4.16</v>
+        <v>4.1</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>GUJRAFFIA</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>45.37</v>
+        <v>385.35</v>
       </c>
       <c r="C68" t="n">
-        <v>47.25</v>
+        <v>401</v>
       </c>
       <c r="D68" t="n">
-        <v>4.14</v>
+        <v>4.06</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>NIMBSPROJ</t>
+          <t>GANDHAR</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>219.01</v>
+        <v>162.5</v>
       </c>
       <c r="C69" t="n">
-        <v>227.99</v>
+        <v>169</v>
       </c>
       <c r="D69" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>CLSEL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>5.96</v>
+        <v>292.4</v>
       </c>
       <c r="C70" t="n">
-        <v>6.2</v>
+        <v>304</v>
       </c>
       <c r="D70" t="n">
-        <v>4.03</v>
+        <v>3.97</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CRIZAC</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>223.99</v>
+        <v>54.84</v>
       </c>
       <c r="C71" t="n">
-        <v>233</v>
+        <v>56.99</v>
       </c>
       <c r="D71" t="n">
-        <v>4.02</v>
+        <v>3.92</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SYSTMTXC</t>
+          <t>SUYOG</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>65.8</v>
+        <v>768.25</v>
       </c>
       <c r="C72" t="n">
-        <v>68.40000000000001</v>
+        <v>797</v>
       </c>
       <c r="D72" t="n">
-        <v>3.95</v>
+        <v>3.74</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ORTEL</t>
+          <t>KDDL</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1.59</v>
+        <v>2698.1</v>
       </c>
       <c r="C73" t="n">
-        <v>1.65</v>
+        <v>2798</v>
       </c>
       <c r="D73" t="n">
-        <v>3.77</v>
+        <v>3.7</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>IDEAFORGE</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>814.7</v>
+        <v>24.5</v>
       </c>
       <c r="C74" t="n">
-        <v>845</v>
+        <v>25.4</v>
       </c>
       <c r="D74" t="n">
-        <v>3.72</v>
+        <v>3.67</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>8.65</v>
+        <v>1437.6</v>
       </c>
       <c r="C75" t="n">
-        <v>8.970000000000001</v>
+        <v>1490</v>
       </c>
       <c r="D75" t="n">
-        <v>3.7</v>
+        <v>3.64</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>UNIDT</t>
+          <t>KHANDSE</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>230.55</v>
+        <v>18.23</v>
       </c>
       <c r="C76" t="n">
-        <v>238.99</v>
+        <v>18.89</v>
       </c>
       <c r="D76" t="n">
-        <v>3.66</v>
+        <v>3.62</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>RKDL</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>21.13</v>
+        <v>14.14</v>
       </c>
       <c r="C77" t="n">
-        <v>21.9</v>
+        <v>14.65</v>
       </c>
       <c r="D77" t="n">
-        <v>3.64</v>
+        <v>3.61</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>PINELABS</t>
+          <t>SECMARK</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>146.2</v>
+        <v>121.61</v>
       </c>
       <c r="C78" t="n">
-        <v>151.5</v>
+        <v>126</v>
       </c>
       <c r="D78" t="n">
-        <v>3.63</v>
+        <v>3.61</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>MERCANTILE</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>26.84</v>
+        <v>10.8</v>
       </c>
       <c r="C79" t="n">
-        <v>27.8</v>
+        <v>11.19</v>
       </c>
       <c r="D79" t="n">
-        <v>3.58</v>
+        <v>3.61</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>QUINT</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>7.05</v>
+        <v>40.35</v>
       </c>
       <c r="C80" t="n">
-        <v>7.3</v>
+        <v>41.8</v>
       </c>
       <c r="D80" t="n">
-        <v>3.55</v>
+        <v>3.59</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>KREBSBIO</t>
+          <t>EBGNG</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>61.81</v>
+        <v>443.25</v>
       </c>
       <c r="C81" t="n">
-        <v>64</v>
+        <v>459</v>
       </c>
       <c r="D81" t="n">
-        <v>3.54</v>
+        <v>3.55</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,14 +2221,14 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BTTL</t>
+          <t>AROGRANITE</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>34.48</v>
+        <v>25.98</v>
       </c>
       <c r="C82" t="n">
-        <v>35.7</v>
+        <v>26.9</v>
       </c>
       <c r="D82" t="n">
         <v>3.54</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.85</v>
+        <v>37</v>
       </c>
       <c r="C83" t="n">
-        <v>0.88</v>
+        <v>38.3</v>
       </c>
       <c r="D83" t="n">
-        <v>3.53</v>
+        <v>3.51</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CPEDU</t>
+          <t>INDOTECH</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>176.96</v>
+        <v>2560.8</v>
       </c>
       <c r="C84" t="n">
-        <v>183.2</v>
+        <v>2650</v>
       </c>
       <c r="D84" t="n">
-        <v>3.53</v>
+        <v>3.48</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>62.29</v>
+        <v>984.7</v>
       </c>
       <c r="C85" t="n">
-        <v>64.48999999999999</v>
+        <v>1019</v>
       </c>
       <c r="D85" t="n">
-        <v>3.53</v>
+        <v>3.48</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>EXCELSOFT</t>
+          <t>INDOUS</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>87.62</v>
+        <v>99.92</v>
       </c>
       <c r="C86" t="n">
-        <v>90.69</v>
+        <v>103.4</v>
       </c>
       <c r="D86" t="n">
-        <v>3.5</v>
+        <v>3.48</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>NILE</t>
+          <t>OMNI</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1816.2</v>
+        <v>424.4</v>
       </c>
       <c r="C87" t="n">
-        <v>1879.8</v>
+        <v>439.15</v>
       </c>
       <c r="D87" t="n">
-        <v>3.5</v>
+        <v>3.48</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GKWLIMITED</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>1704.6</v>
+        <v>13.87</v>
       </c>
       <c r="C88" t="n">
-        <v>1764.3</v>
+        <v>14.35</v>
       </c>
       <c r="D88" t="n">
-        <v>3.5</v>
+        <v>3.46</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>RELIABLE</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>133.24</v>
+        <v>13.2</v>
       </c>
       <c r="C89" t="n">
-        <v>137.9</v>
+        <v>13.65</v>
       </c>
       <c r="D89" t="n">
-        <v>3.5</v>
+        <v>3.41</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TVSSCS</t>
+          <t>DNAMEDIA</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>120.81</v>
+        <v>2.94</v>
       </c>
       <c r="C90" t="n">
-        <v>125</v>
+        <v>3.04</v>
       </c>
       <c r="D90" t="n">
-        <v>3.47</v>
+        <v>3.4</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>NIRAJ</t>
+          <t>OSWALSEEDS</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>28.89</v>
+        <v>11.03</v>
       </c>
       <c r="C91" t="n">
-        <v>29.89</v>
+        <v>11.4</v>
       </c>
       <c r="D91" t="n">
-        <v>3.46</v>
+        <v>3.35</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SCANSTL</t>
+          <t>NILE</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>38.42</v>
+        <v>1849.2</v>
       </c>
       <c r="C92" t="n">
-        <v>39.75</v>
+        <v>1911</v>
       </c>
       <c r="D92" t="n">
-        <v>3.46</v>
+        <v>3.34</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>THYROCARE</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>10.42</v>
+        <v>502.25</v>
       </c>
       <c r="C93" t="n">
-        <v>10.78</v>
+        <v>519</v>
       </c>
       <c r="D93" t="n">
-        <v>3.45</v>
+        <v>3.33</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>TFL</t>
+          <t>FIRSTCRY</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>12.76</v>
+        <v>237.11</v>
       </c>
       <c r="C94" t="n">
-        <v>13.2</v>
+        <v>245</v>
       </c>
       <c r="D94" t="n">
-        <v>3.45</v>
+        <v>3.33</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ASHOKAMET</t>
+          <t>RAJESHEXPO</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>15.95</v>
+        <v>118.45</v>
       </c>
       <c r="C95" t="n">
-        <v>16.5</v>
+        <v>122.39</v>
       </c>
       <c r="D95" t="n">
-        <v>3.45</v>
+        <v>3.33</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PASUPTAC</t>
+          <t>ANLON</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>57.52</v>
+        <v>644.7</v>
       </c>
       <c r="C96" t="n">
-        <v>59.5</v>
+        <v>666</v>
       </c>
       <c r="D96" t="n">
-        <v>3.44</v>
+        <v>3.3</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PVSL</t>
+          <t>FMNL</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>105.44</v>
+        <v>10.65</v>
       </c>
       <c r="C97" t="n">
-        <v>109</v>
+        <v>11</v>
       </c>
       <c r="D97" t="n">
-        <v>3.38</v>
+        <v>3.29</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>83.39</v>
+        <v>5.19</v>
       </c>
       <c r="C98" t="n">
-        <v>86.2</v>
+        <v>5.36</v>
       </c>
       <c r="D98" t="n">
-        <v>3.37</v>
+        <v>3.28</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>ELECTHERM</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>21.95</v>
+        <v>789.15</v>
       </c>
       <c r="C99" t="n">
-        <v>22.69</v>
+        <v>815</v>
       </c>
       <c r="D99" t="n">
-        <v>3.37</v>
+        <v>3.28</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>FOODSIN</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>7.16</v>
+        <v>54.81</v>
       </c>
       <c r="C100" t="n">
-        <v>7.4</v>
+        <v>56.6</v>
       </c>
       <c r="D100" t="n">
-        <v>3.35</v>
+        <v>3.27</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CHEMPLASTS</t>
+          <t>KANANIIND</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>243.89</v>
+        <v>1.54</v>
       </c>
       <c r="C101" t="n">
-        <v>252</v>
+        <v>1.59</v>
       </c>
       <c r="D101" t="n">
-        <v>3.33</v>
+        <v>3.25</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ELLEN</t>
+          <t>SUPERSPIN</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>265.35</v>
+        <v>5.04</v>
       </c>
       <c r="C102" t="n">
-        <v>274.15</v>
+        <v>5.2</v>
       </c>
       <c r="D102" t="n">
-        <v>3.32</v>
+        <v>3.17</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>AURIGROW</t>
+          <t>AGRITECH</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.31</v>
+        <v>108.09</v>
       </c>
       <c r="C103" t="n">
-        <v>0.32</v>
+        <v>111.49</v>
       </c>
       <c r="D103" t="n">
-        <v>3.23</v>
+        <v>3.15</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>LASA</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>8.06</v>
+        <v>40.48</v>
       </c>
       <c r="C104" t="n">
-        <v>8.32</v>
+        <v>41.75</v>
       </c>
       <c r="D104" t="n">
-        <v>3.23</v>
+        <v>3.14</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>THEMISMED</t>
+          <t>TERASOFT</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>100.24</v>
+        <v>357.85</v>
       </c>
       <c r="C105" t="n">
-        <v>103.45</v>
+        <v>369</v>
       </c>
       <c r="D105" t="n">
-        <v>3.2</v>
+        <v>3.12</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>UMAEXPORTS</t>
+          <t>AMJLAND</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>25.19</v>
+        <v>37.32</v>
       </c>
       <c r="C106" t="n">
-        <v>25.99</v>
+        <v>38.48</v>
       </c>
       <c r="D106" t="n">
-        <v>3.18</v>
+        <v>3.11</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>DHARARAIL</t>
+          <t>UMAEXPORTS</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>135.85</v>
+        <v>24.92</v>
       </c>
       <c r="C107" t="n">
-        <v>140</v>
+        <v>25.69</v>
       </c>
       <c r="D107" t="n">
-        <v>3.05</v>
+        <v>3.09</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>JETFREIGHT</t>
+          <t>BCPL</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>20.32</v>
+        <v>79.58</v>
       </c>
       <c r="C108" t="n">
-        <v>20.94</v>
+        <v>81.98999999999999</v>
       </c>
       <c r="D108" t="n">
-        <v>3.05</v>
+        <v>3.03</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>DPEL</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>508.75</v>
+        <v>0.33</v>
       </c>
       <c r="C109" t="n">
-        <v>524</v>
+        <v>0.34</v>
       </c>
       <c r="D109" t="n">
-        <v>3</v>
+        <v>3.03</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>NIPPOBATRY</t>
+          <t>FLEXITUFF</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>363.35</v>
+        <v>6.66</v>
       </c>
       <c r="C110" t="n">
-        <v>374</v>
+        <v>6.86</v>
       </c>
       <c r="D110" t="n">
-        <v>2.93</v>
+        <v>3</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SAKHTISUG</t>
+          <t>COFFEEDAY</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>17.96</v>
+        <v>25.54</v>
       </c>
       <c r="C111" t="n">
-        <v>18.48</v>
+        <v>26.3</v>
       </c>
       <c r="D111" t="n">
-        <v>2.9</v>
+        <v>2.98</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>KOPRAN</t>
+          <t>SUNDRMBRAK</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>188.48</v>
+        <v>726.4</v>
       </c>
       <c r="C112" t="n">
-        <v>193.9</v>
+        <v>748</v>
       </c>
       <c r="D112" t="n">
-        <v>2.88</v>
+        <v>2.97</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>DCMSRIND</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>3.82</v>
+        <v>38.56</v>
       </c>
       <c r="C113" t="n">
-        <v>3.93</v>
+        <v>39.7</v>
       </c>
       <c r="D113" t="n">
-        <v>2.88</v>
+        <v>2.96</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SHRIRAMPPS</t>
+          <t>AHLADA</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>90.90000000000001</v>
+        <v>39.67</v>
       </c>
       <c r="C114" t="n">
-        <v>93.5</v>
+        <v>40.84</v>
       </c>
       <c r="D114" t="n">
-        <v>2.86</v>
+        <v>2.95</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>DJML</t>
+          <t>CLEDUCATE</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>98.58</v>
+        <v>46.04</v>
       </c>
       <c r="C115" t="n">
-        <v>101.4</v>
+        <v>47.4</v>
       </c>
       <c r="D115" t="n">
-        <v>2.86</v>
+        <v>2.95</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>TAMBOLIIN</t>
+          <t>EQUIPPP</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>179.87</v>
+        <v>15.98</v>
       </c>
       <c r="C116" t="n">
-        <v>184.99</v>
+        <v>16.45</v>
       </c>
       <c r="D116" t="n">
-        <v>2.85</v>
+        <v>2.94</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>VIDYAWIRES</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>14.08</v>
+        <v>101.61</v>
       </c>
       <c r="C117" t="n">
-        <v>14.48</v>
+        <v>104.6</v>
       </c>
       <c r="D117" t="n">
-        <v>2.84</v>
+        <v>2.94</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>SMARTLINK</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>1.42</v>
+        <v>159.77</v>
       </c>
       <c r="C118" t="n">
-        <v>1.46</v>
+        <v>164.44</v>
       </c>
       <c r="D118" t="n">
-        <v>2.82</v>
+        <v>2.92</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>TREL</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>55.25</v>
+        <v>24.68</v>
       </c>
       <c r="C119" t="n">
-        <v>56.8</v>
+        <v>25.4</v>
       </c>
       <c r="D119" t="n">
-        <v>2.81</v>
+        <v>2.92</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>TRAVELFOOD</t>
+          <t>JMA</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>1152.6</v>
+        <v>89.36</v>
       </c>
       <c r="C120" t="n">
-        <v>1185</v>
+        <v>91.97</v>
       </c>
       <c r="D120" t="n">
-        <v>2.81</v>
+        <v>2.92</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>AYMSYNTEX</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>768.4</v>
+        <v>217.46</v>
       </c>
       <c r="C121" t="n">
-        <v>790</v>
+        <v>223.8</v>
       </c>
       <c r="D121" t="n">
-        <v>2.81</v>
+        <v>2.92</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>BANG</t>
+          <t>INTENTECH</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>37.17</v>
+        <v>98.03</v>
       </c>
       <c r="C122" t="n">
-        <v>38.2</v>
+        <v>100.87</v>
       </c>
       <c r="D122" t="n">
-        <v>2.77</v>
+        <v>2.9</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BALPHARMA</t>
+          <t>VRAJ</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>88.56</v>
+        <v>122.47</v>
       </c>
       <c r="C123" t="n">
-        <v>91</v>
+        <v>126</v>
       </c>
       <c r="D123" t="n">
-        <v>2.76</v>
+        <v>2.88</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>KRIDHANINF</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>14.69</v>
+        <v>3.13</v>
       </c>
       <c r="C124" t="n">
-        <v>15.09</v>
+        <v>3.22</v>
       </c>
       <c r="D124" t="n">
-        <v>2.72</v>
+        <v>2.88</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>DONEAR</t>
+          <t>KARNIKA</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>90.44</v>
+        <v>145.8</v>
       </c>
       <c r="C125" t="n">
-        <v>92.89</v>
+        <v>150</v>
       </c>
       <c r="D125" t="n">
-        <v>2.71</v>
+        <v>2.88</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>BVCL</t>
+          <t>GOLDENTOBC</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>42.81</v>
+        <v>26.15</v>
       </c>
       <c r="C126" t="n">
-        <v>43.96</v>
+        <v>26.9</v>
       </c>
       <c r="D126" t="n">
-        <v>2.69</v>
+        <v>2.87</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>NATCAPSUQ</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>24.23</v>
+        <v>152.42</v>
       </c>
       <c r="C127" t="n">
-        <v>24.88</v>
+        <v>156.8</v>
       </c>
       <c r="D127" t="n">
-        <v>2.68</v>
+        <v>2.87</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>PIGL</t>
+          <t>TCI</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>105.18</v>
+        <v>899.9</v>
       </c>
       <c r="C128" t="n">
-        <v>107.98</v>
+        <v>924.95</v>
       </c>
       <c r="D128" t="n">
-        <v>2.66</v>
+        <v>2.78</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MONEYBOXX</t>
+          <t>LOKESHMACH</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>72.88</v>
+        <v>260.93</v>
       </c>
       <c r="C129" t="n">
-        <v>74.8</v>
+        <v>268</v>
       </c>
       <c r="D129" t="n">
-        <v>2.63</v>
+        <v>2.71</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>DAICHI</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>256</v>
+        <v>1.5</v>
       </c>
       <c r="C130" t="n">
-        <v>262.7</v>
+        <v>1.54</v>
       </c>
       <c r="D130" t="n">
-        <v>2.62</v>
+        <v>2.67</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MANGALAM</t>
+          <t>RUPA</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>29.14</v>
+        <v>151.07</v>
       </c>
       <c r="C131" t="n">
-        <v>29.9</v>
+        <v>155</v>
       </c>
       <c r="D131" t="n">
-        <v>2.61</v>
+        <v>2.6</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,14 +3321,14 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>92.55</v>
+        <v>72.91</v>
       </c>
       <c r="C132" t="n">
-        <v>94.95</v>
+        <v>74.8</v>
       </c>
       <c r="D132" t="n">
         <v>2.59</v>
@@ -3343,14 +3343,14 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>PCJEWELLER</t>
+          <t>AMNPLST</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>8.92</v>
+        <v>193.02</v>
       </c>
       <c r="C133" t="n">
-        <v>9.15</v>
+        <v>198</v>
       </c>
       <c r="D133" t="n">
         <v>2.58</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>1136.15</v>
+        <v>13.26</v>
       </c>
       <c r="C134" t="n">
-        <v>1165.4</v>
+        <v>13.6</v>
       </c>
       <c r="D134" t="n">
-        <v>2.57</v>
+        <v>2.56</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SPECTRUM</t>
+          <t>LFIC</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>1394.1</v>
+        <v>140.37</v>
       </c>
       <c r="C135" t="n">
-        <v>1429.9</v>
+        <v>143.9</v>
       </c>
       <c r="D135" t="n">
-        <v>2.57</v>
+        <v>2.51</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>VINCOFE</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>3.9</v>
+        <v>149.76</v>
       </c>
       <c r="C136" t="n">
-        <v>4</v>
+        <v>153.5</v>
       </c>
       <c r="D136" t="n">
-        <v>2.56</v>
+        <v>2.5</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>BOHRAIND</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>42.9</v>
+        <v>18.15</v>
       </c>
       <c r="C137" t="n">
-        <v>44</v>
+        <v>18.6</v>
       </c>
       <c r="D137" t="n">
-        <v>2.56</v>
+        <v>2.48</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>AXITA</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>65.34999999999999</v>
+        <v>8.19</v>
       </c>
       <c r="C138" t="n">
-        <v>67</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="D138" t="n">
-        <v>2.52</v>
+        <v>2.44</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SELMC</t>
+          <t>MOKSH</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>29.75</v>
+        <v>11.95</v>
       </c>
       <c r="C139" t="n">
-        <v>30.49</v>
+        <v>12.24</v>
       </c>
       <c r="D139" t="n">
-        <v>2.49</v>
+        <v>2.43</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>GANGAFORGE</t>
+          <t>BASML</t>
         </is>
       </c>
       <c r="B140" t="n">
+        <v>25.33</v>
+      </c>
+      <c r="C140" t="n">
+        <v>25.94</v>
+      </c>
+      <c r="D140" t="n">
         <v>2.41</v>
-      </c>
-      <c r="C140" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="D140" t="n">
-        <v>2.49</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>MBLINFRA</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>26.28</v>
+        <v>7.05</v>
       </c>
       <c r="C141" t="n">
-        <v>26.93</v>
+        <v>7.22</v>
       </c>
       <c r="D141" t="n">
-        <v>2.47</v>
+        <v>2.41</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>DECCANCE</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>6.9</v>
+        <v>615.25</v>
       </c>
       <c r="C142" t="n">
-        <v>7.07</v>
+        <v>630</v>
       </c>
       <c r="D142" t="n">
-        <v>2.46</v>
+        <v>2.4</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>AARTECH</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>116.15</v>
+        <v>44.81</v>
       </c>
       <c r="C143" t="n">
-        <v>119</v>
+        <v>45.87</v>
       </c>
       <c r="D143" t="n">
-        <v>2.45</v>
+        <v>2.37</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>KOTARISUG</t>
+          <t>EUROPRATIK</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>25.75</v>
+        <v>250.05</v>
       </c>
       <c r="C144" t="n">
-        <v>26.38</v>
+        <v>255.95</v>
       </c>
       <c r="D144" t="n">
-        <v>2.45</v>
+        <v>2.36</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>PRADPME</t>
+          <t>NAGAFERT</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>421.7</v>
+        <v>3.83</v>
       </c>
       <c r="C145" t="n">
-        <v>432</v>
+        <v>3.92</v>
       </c>
       <c r="D145" t="n">
-        <v>2.44</v>
+        <v>2.35</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>MANAKSIA</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>3.29</v>
+        <v>61.56</v>
       </c>
       <c r="C146" t="n">
-        <v>3.37</v>
+        <v>63</v>
       </c>
       <c r="D146" t="n">
-        <v>2.43</v>
+        <v>2.34</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ENERGYDEV</t>
+          <t>BAYERCROP</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>16.97</v>
+        <v>4500.8</v>
       </c>
       <c r="C147" t="n">
-        <v>17.38</v>
+        <v>4605</v>
       </c>
       <c r="D147" t="n">
-        <v>2.42</v>
+        <v>2.32</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>SUPREMEPWR</t>
+          <t>NIPPOBATRY</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>253.85</v>
+        <v>366.05</v>
       </c>
       <c r="C148" t="n">
-        <v>260</v>
+        <v>374.5</v>
       </c>
       <c r="D148" t="n">
-        <v>2.42</v>
+        <v>2.31</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>TIPSFILMS</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>2.1</v>
+        <v>368.6</v>
       </c>
       <c r="C149" t="n">
-        <v>2.15</v>
+        <v>377</v>
       </c>
       <c r="D149" t="n">
-        <v>2.38</v>
+        <v>2.28</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>HARIOMPIPE</t>
+          <t>CPPLUS</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>413.2</v>
+        <v>2648.7</v>
       </c>
       <c r="C150" t="n">
-        <v>423</v>
+        <v>2709.1</v>
       </c>
       <c r="D150" t="n">
-        <v>2.37</v>
+        <v>2.28</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>SHIVALIK</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>264.55</v>
+        <v>0.44</v>
       </c>
       <c r="C151" t="n">
-        <v>270.8</v>
+        <v>0.45</v>
       </c>
       <c r="D151" t="n">
-        <v>2.36</v>
+        <v>2.27</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>11.01</v>
+        <v>3.52</v>
       </c>
       <c r="C152" t="n">
-        <v>11.27</v>
+        <v>3.6</v>
       </c>
       <c r="D152" t="n">
-        <v>2.36</v>
+        <v>2.27</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CAPTRUST</t>
+          <t>SHRIKRISH</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>14.46</v>
+        <v>42.05</v>
       </c>
       <c r="C153" t="n">
-        <v>14.8</v>
+        <v>43</v>
       </c>
       <c r="D153" t="n">
-        <v>2.35</v>
+        <v>2.26</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>BYKE</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>985</v>
+        <v>36.48</v>
       </c>
       <c r="C154" t="n">
-        <v>1008</v>
+        <v>37.3</v>
       </c>
       <c r="D154" t="n">
-        <v>2.34</v>
+        <v>2.25</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>UNIMECH</t>
+          <t>PAKKA</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>951.8</v>
+        <v>89.88</v>
       </c>
       <c r="C155" t="n">
-        <v>973.9</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="D155" t="n">
-        <v>2.32</v>
+        <v>2.25</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>KRITIKA</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>6.1</v>
+        <v>6.27</v>
       </c>
       <c r="C156" t="n">
-        <v>6.24</v>
+        <v>6.41</v>
       </c>
       <c r="D156" t="n">
-        <v>2.3</v>
+        <v>2.23</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>TNTELE</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>9.16</v>
+        <v>42.47</v>
       </c>
       <c r="C157" t="n">
-        <v>9.369999999999999</v>
+        <v>43.4</v>
       </c>
       <c r="D157" t="n">
-        <v>2.29</v>
+        <v>2.19</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>DEVIT</t>
+          <t>SOLARWORLD</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>29.32</v>
+        <v>216.3</v>
       </c>
       <c r="C158" t="n">
-        <v>29.99</v>
+        <v>221</v>
       </c>
       <c r="D158" t="n">
-        <v>2.29</v>
+        <v>2.17</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MAZDA</t>
+          <t>DECNGOLD</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>211.16</v>
+        <v>176.86</v>
       </c>
       <c r="C159" t="n">
-        <v>215.97</v>
+        <v>180.7</v>
       </c>
       <c r="D159" t="n">
-        <v>2.28</v>
+        <v>2.17</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>GLOBE</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>231.75</v>
+        <v>2.31</v>
       </c>
       <c r="C160" t="n">
-        <v>237</v>
+        <v>2.36</v>
       </c>
       <c r="D160" t="n">
-        <v>2.27</v>
+        <v>2.16</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>RHFL</t>
+          <t>ANTELOPUS</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>2.22</v>
+        <v>766.85</v>
       </c>
       <c r="C161" t="n">
-        <v>2.27</v>
+        <v>783.25</v>
       </c>
       <c r="D161" t="n">
-        <v>2.25</v>
+        <v>2.14</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>IRISDOREME</t>
+          <t>IWARE</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>35.6</v>
+        <v>359.75</v>
       </c>
       <c r="C162" t="n">
-        <v>36.4</v>
+        <v>367.4</v>
       </c>
       <c r="D162" t="n">
-        <v>2.25</v>
+        <v>2.13</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>11.15</v>
+        <v>3.76</v>
       </c>
       <c r="C163" t="n">
-        <v>11.4</v>
+        <v>3.84</v>
       </c>
       <c r="D163" t="n">
-        <v>2.24</v>
+        <v>2.13</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>FINKURVE</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>0.45</v>
+        <v>63.16</v>
       </c>
       <c r="C164" t="n">
-        <v>0.46</v>
+        <v>64.5</v>
       </c>
       <c r="D164" t="n">
-        <v>2.22</v>
+        <v>2.12</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>GALLANTT</t>
+          <t>DCM</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>699.5</v>
+        <v>92.05</v>
       </c>
       <c r="C165" t="n">
-        <v>715</v>
+        <v>93.98</v>
       </c>
       <c r="D165" t="n">
-        <v>2.22</v>
+        <v>2.1</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>KOTHARIPET</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>129.14</v>
+        <v>15.81</v>
       </c>
       <c r="C166" t="n">
-        <v>132</v>
+        <v>16.14</v>
       </c>
       <c r="D166" t="n">
-        <v>2.21</v>
+        <v>2.09</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>SCHAND</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>172.19</v>
+        <v>0.48</v>
       </c>
       <c r="C167" t="n">
-        <v>175.95</v>
+        <v>0.49</v>
       </c>
       <c r="D167" t="n">
-        <v>2.18</v>
+        <v>2.08</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>RAYMONDREL</t>
+          <t>KEC</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>613.15</v>
+        <v>499.1</v>
       </c>
       <c r="C168" t="n">
-        <v>626.5</v>
+        <v>509.5</v>
       </c>
       <c r="D168" t="n">
-        <v>2.18</v>
+        <v>2.08</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>INA</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>146.83</v>
+        <v>4.85</v>
       </c>
       <c r="C169" t="n">
-        <v>150</v>
+        <v>4.95</v>
       </c>
       <c r="D169" t="n">
-        <v>2.16</v>
+        <v>2.06</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>RADIANTCMS</t>
+          <t>SAAKSHI</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>41.41</v>
+        <v>229.3</v>
       </c>
       <c r="C170" t="n">
-        <v>42.3</v>
+        <v>234</v>
       </c>
       <c r="D170" t="n">
-        <v>2.15</v>
+        <v>2.05</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>GULFPETRO</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>33.29</v>
+        <v>5.84</v>
       </c>
       <c r="C171" t="n">
-        <v>34</v>
+        <v>5.96</v>
       </c>
       <c r="D171" t="n">
-        <v>2.13</v>
+        <v>2.05</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>TCIEXP</t>
+          <t>OMFREIGHT</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>512.15</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="C172" t="n">
-        <v>523</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="D172" t="n">
-        <v>2.12</v>
+        <v>2.04</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>VIPULLTD</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>2.39</v>
+        <v>8.81</v>
       </c>
       <c r="C173" t="n">
-        <v>2.44</v>
+        <v>8.99</v>
       </c>
       <c r="D173" t="n">
-        <v>2.09</v>
+        <v>2.04</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>171.31</v>
+        <v>50.96</v>
       </c>
       <c r="C174" t="n">
-        <v>174.89</v>
+        <v>52</v>
       </c>
       <c r="D174" t="n">
-        <v>2.09</v>
+        <v>2.04</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>HTMEDIA</t>
+          <t>BAJAJCON</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>22.01</v>
+        <v>554.8</v>
       </c>
       <c r="C175" t="n">
-        <v>22.47</v>
+        <v>566</v>
       </c>
       <c r="D175" t="n">
-        <v>2.09</v>
+        <v>2.02</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>IRIS</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>0.48</v>
+        <v>253.79</v>
       </c>
       <c r="C176" t="n">
-        <v>0.49</v>
+        <v>258.88</v>
       </c>
       <c r="D176" t="n">
-        <v>2.08</v>
+        <v>2.01</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>KOHINOOR</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>343.8</v>
+        <v>24.84</v>
       </c>
       <c r="C177" t="n">
-        <v>350.95</v>
+        <v>25.34</v>
       </c>
       <c r="D177" t="n">
-        <v>2.08</v>
+        <v>2.01</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>UNIENTER</t>
+          <t>SRM</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>107.52</v>
+        <v>515.65</v>
       </c>
       <c r="C178" t="n">
-        <v>109.75</v>
+        <v>525.95</v>
       </c>
       <c r="D178" t="n">
-        <v>2.07</v>
+        <v>2</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>IRIS</t>
+          <t>KHAICHEM</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>263.47</v>
+        <v>55.04</v>
       </c>
       <c r="C179" t="n">
-        <v>268.88</v>
+        <v>56.14</v>
       </c>
       <c r="D179" t="n">
-        <v>2.05</v>
+        <v>2</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>DREAMFOLKS</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>4.88</v>
+        <v>78.42</v>
       </c>
       <c r="C180" t="n">
-        <v>4.98</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="D180" t="n">
-        <v>2.05</v>
+        <v>2</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>6.36</v>
+        <v>8.48</v>
       </c>
       <c r="C181" t="n">
-        <v>6.49</v>
+        <v>8.65</v>
       </c>
       <c r="D181" t="n">
-        <v>2.04</v>
+        <v>2</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>MAJESAUT</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>338</v>
+        <v>8.51</v>
       </c>
       <c r="C182" t="n">
-        <v>344.9</v>
+        <v>8.68</v>
       </c>
       <c r="D182" t="n">
-        <v>2.04</v>
+        <v>2</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>AIRAN</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>16.19</v>
+        <v>93.54000000000001</v>
       </c>
       <c r="C183" t="n">
-        <v>16.52</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="D183" t="n">
-        <v>2.04</v>
+        <v>1.99</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>AARTECH</t>
+          <t>GUJAPOLLO</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>42.86</v>
+        <v>389.05</v>
       </c>
       <c r="C184" t="n">
-        <v>43.73</v>
+        <v>396.8</v>
       </c>
       <c r="D184" t="n">
-        <v>2.03</v>
+        <v>1.99</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>6.44</v>
+        <v>6.06</v>
       </c>
       <c r="C185" t="n">
-        <v>6.57</v>
+        <v>6.18</v>
       </c>
       <c r="D185" t="n">
-        <v>2.02</v>
+        <v>1.98</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>TVTODAY</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>109.98</v>
+        <v>55.78</v>
       </c>
       <c r="C186" t="n">
-        <v>112.2</v>
+        <v>56.88</v>
       </c>
       <c r="D186" t="n">
-        <v>2.02</v>
+        <v>1.97</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>DISAQ</t>
+          <t>KANPRPLA</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>11567</v>
+        <v>207.92</v>
       </c>
       <c r="C187" t="n">
-        <v>11800</v>
+        <v>212</v>
       </c>
       <c r="D187" t="n">
-        <v>2.01</v>
+        <v>1.96</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>FIBERWEB</t>
+          <t>SSDL</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>29.31</v>
+        <v>61.59</v>
       </c>
       <c r="C188" t="n">
-        <v>29.9</v>
+        <v>62.8</v>
       </c>
       <c r="D188" t="n">
-        <v>2.01</v>
+        <v>1.96</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>PINELABS</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>0.5</v>
+        <v>137.94</v>
       </c>
       <c r="C189" t="n">
-        <v>0.51</v>
+        <v>140.65</v>
       </c>
       <c r="D189" t="n">
-        <v>2</v>
+        <v>1.96</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>BALUFORGE</t>
+          <t>KNAGRI</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>466.7</v>
+        <v>190.69</v>
       </c>
       <c r="C190" t="n">
-        <v>476.05</v>
+        <v>194.4</v>
       </c>
       <c r="D190" t="n">
-        <v>2</v>
+        <v>1.95</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>ELCIDIN</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>122490</v>
+        <v>61.7</v>
       </c>
       <c r="C191" t="n">
-        <v>124940</v>
+        <v>62.9</v>
       </c>
       <c r="D191" t="n">
-        <v>2</v>
+        <v>1.94</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>IFBIND</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>7.49</v>
+        <v>1147.9</v>
       </c>
       <c r="C192" t="n">
-        <v>7.64</v>
+        <v>1170</v>
       </c>
       <c r="D192" t="n">
-        <v>2</v>
+        <v>1.93</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>FCL</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>39.03</v>
+        <v>2.07</v>
       </c>
       <c r="C193" t="n">
-        <v>39.81</v>
+        <v>2.11</v>
       </c>
       <c r="D193" t="n">
-        <v>2</v>
+        <v>1.93</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>IWP</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>35.35</v>
+        <v>0.52</v>
       </c>
       <c r="C194" t="n">
-        <v>36.05</v>
+        <v>0.53</v>
       </c>
       <c r="D194" t="n">
-        <v>1.98</v>
+        <v>1.92</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>KHAICHEM</t>
+          <t>VINNY</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>55.59</v>
+        <v>1.06</v>
       </c>
       <c r="C195" t="n">
-        <v>56.69</v>
+        <v>1.08</v>
       </c>
       <c r="D195" t="n">
-        <v>1.98</v>
+        <v>1.89</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>AKG</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>47.37</v>
+        <v>11.11</v>
       </c>
       <c r="C196" t="n">
-        <v>48.3</v>
+        <v>11.32</v>
       </c>
       <c r="D196" t="n">
-        <v>1.96</v>
+        <v>1.89</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>OILCOUNTUB</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>6.63</v>
+        <v>55.9</v>
       </c>
       <c r="C197" t="n">
-        <v>6.76</v>
+        <v>56.95</v>
       </c>
       <c r="D197" t="n">
-        <v>1.96</v>
+        <v>1.88</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>HEADSUP</t>
+          <t>INDOTHAI</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>7.19</v>
+        <v>245.15</v>
       </c>
       <c r="C198" t="n">
-        <v>7.33</v>
+        <v>249.75</v>
       </c>
       <c r="D198" t="n">
-        <v>1.95</v>
+        <v>1.88</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>CENTEXT</t>
+          <t>KOTHARIPET</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>20.62</v>
+        <v>126.57</v>
       </c>
       <c r="C199" t="n">
-        <v>21.02</v>
+        <v>128.95</v>
       </c>
       <c r="D199" t="n">
-        <v>1.94</v>
+        <v>1.88</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>ARROWGREEN</t>
+          <t>PPAP</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>456.15</v>
+        <v>211</v>
       </c>
       <c r="C200" t="n">
-        <v>464.95</v>
+        <v>214.95</v>
       </c>
       <c r="D200" t="n">
-        <v>1.93</v>
+        <v>1.87</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>KNAGRI</t>
+          <t>PCJEWELLER</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>191.82</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C201" t="n">
-        <v>195.5</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="D201" t="n">
-        <v>1.92</v>
+        <v>1.86</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-05-29 07:41 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ALUWIND</t>
+          <t>MOTOGENFIN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>49.75</v>
+        <v>27.35</v>
       </c>
       <c r="C2" t="n">
-        <v>56</v>
+        <v>32.82</v>
       </c>
       <c r="D2" t="n">
-        <v>12.56</v>
+        <v>20</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ALKALI</t>
+          <t>SAHLIBHFI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>74.55</v>
+        <v>72.06999999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D3" t="n">
-        <v>11.33</v>
+        <v>19.33</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BIRLAPREC</t>
+          <t>VADILALIND</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>44.93</v>
+        <v>4466.9</v>
       </c>
       <c r="C4" t="n">
-        <v>49.99</v>
+        <v>5150</v>
       </c>
       <c r="D4" t="n">
-        <v>11.26</v>
+        <v>15.29</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>SAYAJIHOTL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>200.16</v>
+        <v>282.95</v>
       </c>
       <c r="C5" t="n">
-        <v>220.17</v>
+        <v>323.95</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>14.49</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FONEBOX</t>
+          <t>COFFEEDAY</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>99.2</v>
+        <v>28.99</v>
       </c>
       <c r="C6" t="n">
-        <v>109</v>
+        <v>33</v>
       </c>
       <c r="D6" t="n">
-        <v>9.880000000000001</v>
+        <v>13.83</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>AVTNPL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1048.9</v>
+        <v>68.64</v>
       </c>
       <c r="C7" t="n">
-        <v>1150</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>9.640000000000001</v>
+        <v>12.03</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SPECTRUM</t>
+          <t>MERCANTILE</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1383.3</v>
+        <v>25.64</v>
       </c>
       <c r="C8" t="n">
-        <v>1500</v>
+        <v>28.59</v>
       </c>
       <c r="D8" t="n">
-        <v>8.44</v>
+        <v>11.51</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>470.6</v>
+        <v>137.91</v>
       </c>
       <c r="C9" t="n">
-        <v>510</v>
+        <v>153.39</v>
       </c>
       <c r="D9" t="n">
-        <v>8.369999999999999</v>
+        <v>11.22</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>INDOAMIN</t>
+          <t>ADISOFT</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>134.57</v>
+        <v>194</v>
       </c>
       <c r="C10" t="n">
-        <v>145.01</v>
+        <v>215</v>
       </c>
       <c r="D10" t="n">
-        <v>7.76</v>
+        <v>10.82</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>JOCIL</t>
+          <t>DYNPRO</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>145.94</v>
+        <v>231.12</v>
       </c>
       <c r="C11" t="n">
-        <v>157</v>
+        <v>255</v>
       </c>
       <c r="D11" t="n">
-        <v>7.58</v>
+        <v>10.33</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>44.47</v>
+        <v>220.17</v>
       </c>
       <c r="C12" t="n">
-        <v>47.7</v>
+        <v>242.18</v>
       </c>
       <c r="D12" t="n">
-        <v>7.26</v>
+        <v>10</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TIMEX</t>
+          <t>CPPLUS</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>374.6</v>
+        <v>2639.6</v>
       </c>
       <c r="C13" t="n">
-        <v>401.35</v>
+        <v>2903.5</v>
       </c>
       <c r="D13" t="n">
-        <v>7.14</v>
+        <v>10</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LGHL</t>
+          <t>SUPRIYA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>235.4</v>
+        <v>807.25</v>
       </c>
       <c r="C14" t="n">
-        <v>251</v>
+        <v>887.3</v>
       </c>
       <c r="D14" t="n">
-        <v>6.63</v>
+        <v>9.92</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TAALTECH</t>
+          <t>FALCONTECH</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3190.4</v>
+        <v>13.65</v>
       </c>
       <c r="C15" t="n">
-        <v>3398</v>
+        <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>6.51</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FLYSBS</t>
+          <t>BIKEWO</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>433.9</v>
+        <v>26.85</v>
       </c>
       <c r="C16" t="n">
-        <v>462</v>
+        <v>29.5</v>
       </c>
       <c r="D16" t="n">
-        <v>6.48</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SHARDUL</t>
+          <t>KIRANVYPAR</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>28.12</v>
+        <v>163.91</v>
       </c>
       <c r="C17" t="n">
-        <v>29.9</v>
+        <v>179.99</v>
       </c>
       <c r="D17" t="n">
-        <v>6.33</v>
+        <v>9.81</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FINPIPE</t>
+          <t>VRAJ</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>178.14</v>
+        <v>122.49</v>
       </c>
       <c r="C18" t="n">
-        <v>188.6</v>
+        <v>134.5</v>
       </c>
       <c r="D18" t="n">
-        <v>5.87</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>JKTYRE</t>
+          <t>ALGOQUANT</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>394.15</v>
+        <v>56.99</v>
       </c>
       <c r="C19" t="n">
-        <v>416</v>
+        <v>62.4</v>
       </c>
       <c r="D19" t="n">
-        <v>5.54</v>
+        <v>9.49</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>251.13</v>
+        <v>8.94</v>
       </c>
       <c r="C20" t="n">
-        <v>265</v>
+        <v>9.76</v>
       </c>
       <c r="D20" t="n">
-        <v>5.52</v>
+        <v>9.17</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PGHL</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>5652.5</v>
+        <v>56.9</v>
       </c>
       <c r="C21" t="n">
-        <v>5949</v>
+        <v>62</v>
       </c>
       <c r="D21" t="n">
-        <v>5.25</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SBGLP</t>
+          <t>WOCKPHARMA</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>25.66</v>
+        <v>1771</v>
       </c>
       <c r="C22" t="n">
-        <v>27</v>
+        <v>1925</v>
       </c>
       <c r="D22" t="n">
-        <v>5.22</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CARRARO</t>
+          <t>NMSTEEL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>608.5</v>
+        <v>23.7</v>
       </c>
       <c r="C23" t="n">
-        <v>640.1</v>
+        <v>25.7</v>
       </c>
       <c r="D23" t="n">
-        <v>5.19</v>
+        <v>8.44</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>EIFFL</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>486.35</v>
+        <v>235.3</v>
       </c>
       <c r="C24" t="n">
-        <v>510.65</v>
+        <v>255</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1161.05</v>
+        <v>14.49</v>
       </c>
       <c r="C25" t="n">
-        <v>1219.1</v>
+        <v>15.68</v>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AUSOMENT</t>
+          <t>PALASHSECU</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>139.62</v>
+        <v>98.95</v>
       </c>
       <c r="C26" t="n">
-        <v>146.6</v>
+        <v>106.75</v>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>7.88</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>KANORICHEM</t>
+          <t>JAGRAN</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>96</v>
+        <v>70.05</v>
       </c>
       <c r="C27" t="n">
-        <v>100.8</v>
+        <v>75.25</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>7.42</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>JPPOWER</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>175.89</v>
+        <v>22.87</v>
       </c>
       <c r="C28" t="n">
-        <v>184.68</v>
+        <v>24.5</v>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>7.13</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CKKRETAIL</t>
+          <t>WIPL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>137.25</v>
+        <v>147.75</v>
       </c>
       <c r="C29" t="n">
-        <v>144.1</v>
+        <v>158</v>
       </c>
       <c r="D29" t="n">
-        <v>4.99</v>
+        <v>6.94</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>KHAITANLTD</t>
+          <t>MONOLITH</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>133.75</v>
+        <v>556.7</v>
       </c>
       <c r="C30" t="n">
-        <v>140.43</v>
+        <v>595</v>
       </c>
       <c r="D30" t="n">
-        <v>4.99</v>
+        <v>6.88</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>SKYGOLD</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>32.05</v>
+        <v>486.65</v>
       </c>
       <c r="C31" t="n">
-        <v>33.65</v>
+        <v>520</v>
       </c>
       <c r="D31" t="n">
-        <v>4.99</v>
+        <v>6.85</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>POSITRON</t>
+          <t>AYMSYNTEX</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>207.25</v>
+        <v>219.48</v>
       </c>
       <c r="C32" t="n">
-        <v>217.6</v>
+        <v>234.1</v>
       </c>
       <c r="D32" t="n">
-        <v>4.99</v>
+        <v>6.66</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>314.5</v>
+        <v>24.4</v>
       </c>
       <c r="C33" t="n">
-        <v>330.2</v>
+        <v>26</v>
       </c>
       <c r="D33" t="n">
-        <v>4.99</v>
+        <v>6.56</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>JASH</t>
+          <t>MMP</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>397.2</v>
+        <v>279.27</v>
       </c>
       <c r="C34" t="n">
-        <v>417</v>
+        <v>296.95</v>
       </c>
       <c r="D34" t="n">
-        <v>4.98</v>
+        <v>6.33</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ANIKINDS</t>
+          <t>ANONDITA</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>44.2</v>
+        <v>1013.25</v>
       </c>
       <c r="C35" t="n">
-        <v>46.4</v>
+        <v>1077</v>
       </c>
       <c r="D35" t="n">
-        <v>4.98</v>
+        <v>6.29</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>LORDSCHLO</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>25.34</v>
+        <v>141.48</v>
       </c>
       <c r="C36" t="n">
-        <v>26.6</v>
+        <v>150.3</v>
       </c>
       <c r="D36" t="n">
-        <v>4.97</v>
+        <v>6.23</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DCMFINSERV</t>
+          <t>SJLOGISTIC</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>5.43</v>
+        <v>339.2</v>
       </c>
       <c r="C37" t="n">
-        <v>5.7</v>
+        <v>360</v>
       </c>
       <c r="D37" t="n">
-        <v>4.97</v>
+        <v>6.13</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TGL</t>
+          <t>TAJGVK</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>22.4</v>
+        <v>321.25</v>
       </c>
       <c r="C38" t="n">
-        <v>23.5</v>
+        <v>340.95</v>
       </c>
       <c r="D38" t="n">
-        <v>4.91</v>
+        <v>6.13</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LANDMARK</t>
+          <t>GANGAFORGE</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>381.3</v>
+        <v>2.34</v>
       </c>
       <c r="C39" t="n">
-        <v>400</v>
+        <v>2.48</v>
       </c>
       <c r="D39" t="n">
-        <v>4.9</v>
+        <v>5.98</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SONAMAC</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>37.8</v>
+        <v>10.36</v>
       </c>
       <c r="C40" t="n">
-        <v>39.65</v>
+        <v>10.98</v>
       </c>
       <c r="D40" t="n">
-        <v>4.89</v>
+        <v>5.98</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LAKPRE</t>
+          <t>SHIVALIK</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>5.74</v>
+        <v>259.15</v>
       </c>
       <c r="C41" t="n">
-        <v>6.02</v>
+        <v>274.5</v>
       </c>
       <c r="D41" t="n">
-        <v>4.88</v>
+        <v>5.92</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>BAJEL</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4.31</v>
+        <v>184.34</v>
       </c>
       <c r="C42" t="n">
-        <v>4.52</v>
+        <v>195</v>
       </c>
       <c r="D42" t="n">
-        <v>4.87</v>
+        <v>5.78</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>9.08</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="C43" t="n">
-        <v>9.52</v>
+        <v>72.72</v>
       </c>
       <c r="D43" t="n">
-        <v>4.85</v>
+        <v>5.76</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GSTL</t>
+          <t>BNALTD</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>19.7</v>
+        <v>359.3</v>
       </c>
       <c r="C44" t="n">
-        <v>20.65</v>
+        <v>379.9</v>
       </c>
       <c r="D44" t="n">
-        <v>4.82</v>
+        <v>5.73</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>BIMETAL</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>27.66</v>
+        <v>572.15</v>
       </c>
       <c r="C45" t="n">
-        <v>28.99</v>
+        <v>604.95</v>
       </c>
       <c r="D45" t="n">
-        <v>4.81</v>
+        <v>5.73</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>INNOVANA</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3.8</v>
+        <v>329.95</v>
       </c>
       <c r="C46" t="n">
-        <v>3.98</v>
+        <v>348.8</v>
       </c>
       <c r="D46" t="n">
-        <v>4.74</v>
+        <v>5.71</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IL&amp;FSENGG</t>
+          <t>VETO</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>30.36</v>
+        <v>122.08</v>
       </c>
       <c r="C47" t="n">
-        <v>31.8</v>
+        <v>129</v>
       </c>
       <c r="D47" t="n">
-        <v>4.74</v>
+        <v>5.67</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>SHUBHSHREE</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>59.23</v>
+        <v>301</v>
       </c>
       <c r="C48" t="n">
-        <v>62</v>
+        <v>318</v>
       </c>
       <c r="D48" t="n">
-        <v>4.68</v>
+        <v>5.65</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>JETFREIGHT</t>
+          <t>DAMODARIND</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>20.4</v>
+        <v>31.66</v>
       </c>
       <c r="C49" t="n">
-        <v>21.35</v>
+        <v>33.4</v>
       </c>
       <c r="D49" t="n">
-        <v>4.66</v>
+        <v>5.5</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>JKIPL</t>
+          <t>EMAMIPAP</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>84.59</v>
+        <v>79.81999999999999</v>
       </c>
       <c r="C50" t="n">
-        <v>88.5</v>
+        <v>84.19</v>
       </c>
       <c r="D50" t="n">
-        <v>4.62</v>
+        <v>5.47</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MAXPOSURE</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>36.3</v>
+        <v>204</v>
       </c>
       <c r="C51" t="n">
-        <v>37.95</v>
+        <v>214.7</v>
       </c>
       <c r="D51" t="n">
-        <v>4.55</v>
+        <v>5.25</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PANSARI</t>
+          <t>ALKALI</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>291.7</v>
+        <v>89.45999999999999</v>
       </c>
       <c r="C52" t="n">
-        <v>304.9</v>
+        <v>94</v>
       </c>
       <c r="D52" t="n">
-        <v>4.53</v>
+        <v>5.07</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>BEDMUTHA</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.89</v>
+        <v>108</v>
       </c>
       <c r="C53" t="n">
-        <v>0.93</v>
+        <v>113.4</v>
       </c>
       <c r="D53" t="n">
-        <v>4.49</v>
+        <v>5</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>VIYASH</t>
+          <t>ATLANTAELE</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>257.36</v>
+        <v>1878.3</v>
       </c>
       <c r="C54" t="n">
-        <v>268.89</v>
+        <v>1972.2</v>
       </c>
       <c r="D54" t="n">
-        <v>4.48</v>
+        <v>5</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>JINDWORLD</t>
+          <t>VIPCLOTHNG</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>30.15</v>
+        <v>26.62</v>
       </c>
       <c r="C55" t="n">
-        <v>31.5</v>
+        <v>27.95</v>
       </c>
       <c r="D55" t="n">
-        <v>4.48</v>
+        <v>5</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ATLANTAELE</t>
+          <t>MRIL</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1788.9</v>
+        <v>38</v>
       </c>
       <c r="C56" t="n">
-        <v>1868.9</v>
+        <v>39.9</v>
       </c>
       <c r="D56" t="n">
-        <v>4.47</v>
+        <v>5</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1.57</v>
+        <v>11.81</v>
       </c>
       <c r="C57" t="n">
-        <v>1.64</v>
+        <v>12.4</v>
       </c>
       <c r="D57" t="n">
-        <v>4.46</v>
+        <v>5</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SURANI</t>
+          <t>CKKRETAIL</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>126.35</v>
+        <v>144.1</v>
       </c>
       <c r="C58" t="n">
-        <v>131.95</v>
+        <v>151.3</v>
       </c>
       <c r="D58" t="n">
-        <v>4.43</v>
+        <v>5</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>47.69</v>
+        <v>715.15</v>
       </c>
       <c r="C59" t="n">
-        <v>49.8</v>
+        <v>750.9</v>
       </c>
       <c r="D59" t="n">
-        <v>4.42</v>
+        <v>5</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>REDTAPE</t>
+          <t>WANBURY</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>148.49</v>
+        <v>300.2</v>
       </c>
       <c r="C60" t="n">
-        <v>155</v>
+        <v>315.2</v>
       </c>
       <c r="D60" t="n">
-        <v>4.38</v>
+        <v>5</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PGHH</t>
+          <t>NIRAJISPAT</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>9873</v>
+        <v>223.24</v>
       </c>
       <c r="C61" t="n">
-        <v>10300</v>
+        <v>234.4</v>
       </c>
       <c r="D61" t="n">
-        <v>4.32</v>
+        <v>5</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>MCON</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>6.25</v>
+        <v>39</v>
       </c>
       <c r="C62" t="n">
-        <v>6.52</v>
+        <v>40.95</v>
       </c>
       <c r="D62" t="n">
-        <v>4.32</v>
+        <v>5</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ARMANFIN</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1750.9</v>
+        <v>1219.1</v>
       </c>
       <c r="C63" t="n">
-        <v>1823.8</v>
+        <v>1280.05</v>
       </c>
       <c r="D63" t="n">
-        <v>4.16</v>
+        <v>5</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SHIVATEX</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>166.19</v>
+        <v>510.65</v>
       </c>
       <c r="C64" t="n">
-        <v>173.1</v>
+        <v>536.15</v>
       </c>
       <c r="D64" t="n">
-        <v>4.16</v>
+        <v>4.99</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>URAVIDEF</t>
+          <t>UTLSOLAR</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>118.01</v>
+        <v>312.8</v>
       </c>
       <c r="C65" t="n">
-        <v>122.9</v>
+        <v>328.4</v>
       </c>
       <c r="D65" t="n">
-        <v>4.14</v>
+        <v>4.99</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>454.25</v>
+        <v>404.6</v>
       </c>
       <c r="C66" t="n">
-        <v>473</v>
+        <v>424.8</v>
       </c>
       <c r="D66" t="n">
-        <v>4.13</v>
+        <v>4.99</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>ARVEE</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>430.35</v>
+        <v>160.03</v>
       </c>
       <c r="C67" t="n">
-        <v>448</v>
+        <v>168</v>
       </c>
       <c r="D67" t="n">
-        <v>4.1</v>
+        <v>4.98</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>STLNETWORK</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>385.35</v>
+        <v>28.93</v>
       </c>
       <c r="C68" t="n">
-        <v>401</v>
+        <v>30.37</v>
       </c>
       <c r="D68" t="n">
-        <v>4.06</v>
+        <v>4.98</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GANDHAR</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>162.5</v>
+        <v>22.51</v>
       </c>
       <c r="C69" t="n">
-        <v>169</v>
+        <v>23.63</v>
       </c>
       <c r="D69" t="n">
-        <v>4</v>
+        <v>4.98</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CLSEL</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>292.4</v>
+        <v>62.19</v>
       </c>
       <c r="C70" t="n">
-        <v>304</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="D70" t="n">
-        <v>3.97</v>
+        <v>4.98</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>54.84</v>
+        <v>56.83</v>
       </c>
       <c r="C71" t="n">
-        <v>56.99</v>
+        <v>59.66</v>
       </c>
       <c r="D71" t="n">
-        <v>3.92</v>
+        <v>4.98</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SUYOG</t>
+          <t>SPECTSTM</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>768.25</v>
+        <v>63.6</v>
       </c>
       <c r="C72" t="n">
-        <v>797</v>
+        <v>66.75</v>
       </c>
       <c r="D72" t="n">
-        <v>3.74</v>
+        <v>4.95</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>KDDL</t>
+          <t>ROXHITECH</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>2698.1</v>
+        <v>36.45</v>
       </c>
       <c r="C73" t="n">
-        <v>2798</v>
+        <v>38.25</v>
       </c>
       <c r="D73" t="n">
-        <v>3.7</v>
+        <v>4.94</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>REGENCERAM</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>24.5</v>
+        <v>40.98</v>
       </c>
       <c r="C74" t="n">
-        <v>25.4</v>
+        <v>43</v>
       </c>
       <c r="D74" t="n">
-        <v>3.67</v>
+        <v>4.93</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1437.6</v>
+        <v>437.45</v>
       </c>
       <c r="C75" t="n">
-        <v>1490</v>
+        <v>459</v>
       </c>
       <c r="D75" t="n">
-        <v>3.64</v>
+        <v>4.93</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>SONAMAC</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>18.23</v>
+        <v>39.65</v>
       </c>
       <c r="C76" t="n">
-        <v>18.89</v>
+        <v>41.6</v>
       </c>
       <c r="D76" t="n">
-        <v>3.62</v>
+        <v>4.92</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>DCMFINSERV</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>14.14</v>
+        <v>5.7</v>
       </c>
       <c r="C77" t="n">
-        <v>14.65</v>
+        <v>5.98</v>
       </c>
       <c r="D77" t="n">
-        <v>3.61</v>
+        <v>4.91</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SECMARK</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>121.61</v>
+        <v>54.28</v>
       </c>
       <c r="C78" t="n">
-        <v>126</v>
+        <v>56.94</v>
       </c>
       <c r="D78" t="n">
-        <v>3.61</v>
+        <v>4.9</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>OMAXAUTO</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>10.8</v>
+        <v>251.12</v>
       </c>
       <c r="C79" t="n">
-        <v>11.19</v>
+        <v>263.4</v>
       </c>
       <c r="D79" t="n">
-        <v>3.61</v>
+        <v>4.89</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>QUINT</t>
+          <t>ORTINGLOBE</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>40.35</v>
+        <v>16.31</v>
       </c>
       <c r="C80" t="n">
-        <v>41.8</v>
+        <v>17.1</v>
       </c>
       <c r="D80" t="n">
-        <v>3.59</v>
+        <v>4.84</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>EBGNG</t>
+          <t>FAZE3Q</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>443.25</v>
+        <v>523.6</v>
       </c>
       <c r="C81" t="n">
-        <v>459</v>
+        <v>548.9</v>
       </c>
       <c r="D81" t="n">
-        <v>3.55</v>
+        <v>4.83</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>AROGRANITE</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>25.98</v>
+        <v>71.55</v>
       </c>
       <c r="C82" t="n">
-        <v>26.9</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="D82" t="n">
-        <v>3.54</v>
+        <v>4.81</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>37</v>
+        <v>40.84</v>
       </c>
       <c r="C83" t="n">
-        <v>38.3</v>
+        <v>42.8</v>
       </c>
       <c r="D83" t="n">
-        <v>3.51</v>
+        <v>4.8</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>INDOTECH</t>
+          <t>CURRENT</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>2560.8</v>
+        <v>113.5</v>
       </c>
       <c r="C84" t="n">
-        <v>2650</v>
+        <v>118.95</v>
       </c>
       <c r="D84" t="n">
-        <v>3.48</v>
+        <v>4.8</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>DEVIT</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>984.7</v>
+        <v>29.11</v>
       </c>
       <c r="C85" t="n">
-        <v>1019</v>
+        <v>30.5</v>
       </c>
       <c r="D85" t="n">
-        <v>3.48</v>
+        <v>4.77</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>ARENTERP</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>99.92</v>
+        <v>39.13</v>
       </c>
       <c r="C86" t="n">
-        <v>103.4</v>
+        <v>40.99</v>
       </c>
       <c r="D86" t="n">
-        <v>3.48</v>
+        <v>4.75</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>OMNI</t>
+          <t>PRIZOR</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>424.4</v>
+        <v>627.4</v>
       </c>
       <c r="C87" t="n">
-        <v>439.15</v>
+        <v>657</v>
       </c>
       <c r="D87" t="n">
-        <v>3.48</v>
+        <v>4.72</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>RUDRA</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>13.87</v>
+        <v>18.42</v>
       </c>
       <c r="C88" t="n">
-        <v>14.35</v>
+        <v>19.29</v>
       </c>
       <c r="D88" t="n">
-        <v>3.46</v>
+        <v>4.72</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>SCANSTL</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>13.2</v>
+        <v>37.99</v>
       </c>
       <c r="C89" t="n">
-        <v>13.65</v>
+        <v>39.77</v>
       </c>
       <c r="D89" t="n">
-        <v>3.41</v>
+        <v>4.69</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>DNAMEDIA</t>
+          <t>BATLIBOI</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>2.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="C90" t="n">
-        <v>3.04</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="D90" t="n">
-        <v>3.4</v>
+        <v>4.67</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>FCSSOFT</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>11.03</v>
+        <v>1.5</v>
       </c>
       <c r="C91" t="n">
-        <v>11.4</v>
+        <v>1.57</v>
       </c>
       <c r="D91" t="n">
-        <v>3.35</v>
+        <v>4.67</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>NILE</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>1849.2</v>
+        <v>201.58</v>
       </c>
       <c r="C92" t="n">
-        <v>1911</v>
+        <v>211</v>
       </c>
       <c r="D92" t="n">
-        <v>3.34</v>
+        <v>4.67</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>THYROCARE</t>
+          <t>LASA</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>502.25</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="C93" t="n">
-        <v>519</v>
+        <v>8.77</v>
       </c>
       <c r="D93" t="n">
-        <v>3.33</v>
+        <v>4.65</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>FIRSTCRY</t>
+          <t>BBTCL</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>237.11</v>
+        <v>208.13</v>
       </c>
       <c r="C94" t="n">
-        <v>245</v>
+        <v>217.8</v>
       </c>
       <c r="D94" t="n">
-        <v>3.33</v>
+        <v>4.65</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>RAJESHEXPO</t>
+          <t>DELTAMAGNT</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>118.45</v>
+        <v>62.12</v>
       </c>
       <c r="C95" t="n">
-        <v>122.39</v>
+        <v>65</v>
       </c>
       <c r="D95" t="n">
-        <v>3.33</v>
+        <v>4.64</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ANLON</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>644.7</v>
+        <v>13.37</v>
       </c>
       <c r="C96" t="n">
-        <v>666</v>
+        <v>13.99</v>
       </c>
       <c r="D96" t="n">
-        <v>3.3</v>
+        <v>4.64</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>FMNL</t>
+          <t>IVALUE</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>10.65</v>
+        <v>243.75</v>
       </c>
       <c r="C97" t="n">
-        <v>11</v>
+        <v>255</v>
       </c>
       <c r="D97" t="n">
-        <v>3.29</v>
+        <v>4.62</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>HBLENGINE</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>5.19</v>
+        <v>817.5</v>
       </c>
       <c r="C98" t="n">
-        <v>5.36</v>
+        <v>855</v>
       </c>
       <c r="D98" t="n">
-        <v>3.28</v>
+        <v>4.59</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ELECTHERM</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>789.15</v>
+        <v>816.75</v>
       </c>
       <c r="C99" t="n">
-        <v>815</v>
+        <v>854</v>
       </c>
       <c r="D99" t="n">
-        <v>3.28</v>
+        <v>4.56</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>FOODSIN</t>
+          <t>GUJRAFFIA</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>54.81</v>
+        <v>45.63</v>
       </c>
       <c r="C100" t="n">
-        <v>56.6</v>
+        <v>47.7</v>
       </c>
       <c r="D100" t="n">
-        <v>3.27</v>
+        <v>4.54</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>KANANIIND</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1.54</v>
+        <v>3.97</v>
       </c>
       <c r="C101" t="n">
-        <v>1.59</v>
+        <v>4.15</v>
       </c>
       <c r="D101" t="n">
-        <v>3.25</v>
+        <v>4.53</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SUPERSPIN</t>
+          <t>STEELXIND</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>5.04</v>
+        <v>11.96</v>
       </c>
       <c r="C102" t="n">
-        <v>5.2</v>
+        <v>12.5</v>
       </c>
       <c r="D102" t="n">
-        <v>3.17</v>
+        <v>4.52</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>AGRITECH</t>
+          <t>GOLDSTAR</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>108.09</v>
+        <v>7.75</v>
       </c>
       <c r="C103" t="n">
-        <v>111.49</v>
+        <v>8.1</v>
       </c>
       <c r="D103" t="n">
-        <v>3.15</v>
+        <v>4.52</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>40.48</v>
+        <v>3.99</v>
       </c>
       <c r="C104" t="n">
-        <v>41.75</v>
+        <v>4.17</v>
       </c>
       <c r="D104" t="n">
-        <v>3.14</v>
+        <v>4.51</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>TERASOFT</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>357.85</v>
+        <v>31.58</v>
       </c>
       <c r="C105" t="n">
-        <v>369</v>
+        <v>33</v>
       </c>
       <c r="D105" t="n">
-        <v>3.12</v>
+        <v>4.5</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>AMJLAND</t>
+          <t>SCPL</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>37.32</v>
+        <v>404.9</v>
       </c>
       <c r="C106" t="n">
-        <v>38.48</v>
+        <v>423</v>
       </c>
       <c r="D106" t="n">
-        <v>3.11</v>
+        <v>4.47</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>UMAEXPORTS</t>
+          <t>RADAAN</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>24.92</v>
+        <v>3.16</v>
       </c>
       <c r="C107" t="n">
-        <v>25.69</v>
+        <v>3.3</v>
       </c>
       <c r="D107" t="n">
-        <v>3.09</v>
+        <v>4.43</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>BCPL</t>
+          <t>ASHAPURMIN</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>79.58</v>
+        <v>654.05</v>
       </c>
       <c r="C108" t="n">
-        <v>81.98999999999999</v>
+        <v>683</v>
       </c>
       <c r="D108" t="n">
-        <v>3.03</v>
+        <v>4.43</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>AKG</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.33</v>
+        <v>11.18</v>
       </c>
       <c r="C109" t="n">
-        <v>0.34</v>
+        <v>11.67</v>
       </c>
       <c r="D109" t="n">
-        <v>3.03</v>
+        <v>4.38</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FLEXITUFF</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>6.66</v>
+        <v>0.23</v>
       </c>
       <c r="C110" t="n">
-        <v>6.86</v>
+        <v>0.24</v>
       </c>
       <c r="D110" t="n">
-        <v>3</v>
+        <v>4.35</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>COFFEEDAY</t>
+          <t>LANCORHOL</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>25.54</v>
+        <v>24.39</v>
       </c>
       <c r="C111" t="n">
-        <v>26.3</v>
+        <v>25.45</v>
       </c>
       <c r="D111" t="n">
-        <v>2.98</v>
+        <v>4.35</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SUNDRMBRAK</t>
+          <t>CANARYS</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>726.4</v>
+        <v>19.65</v>
       </c>
       <c r="C112" t="n">
-        <v>748</v>
+        <v>20.5</v>
       </c>
       <c r="D112" t="n">
-        <v>2.97</v>
+        <v>4.33</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>DCMSRIND</t>
+          <t>BSL</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>38.56</v>
+        <v>136.89</v>
       </c>
       <c r="C113" t="n">
-        <v>39.7</v>
+        <v>142.8</v>
       </c>
       <c r="D113" t="n">
-        <v>2.96</v>
+        <v>4.32</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>AHLADA</t>
+          <t>BAFNAPH</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>39.67</v>
+        <v>129.9</v>
       </c>
       <c r="C114" t="n">
-        <v>40.84</v>
+        <v>135.5</v>
       </c>
       <c r="D114" t="n">
-        <v>2.95</v>
+        <v>4.31</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CLEDUCATE</t>
+          <t>SBGLP</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>46.04</v>
+        <v>26.27</v>
       </c>
       <c r="C115" t="n">
-        <v>47.4</v>
+        <v>27.4</v>
       </c>
       <c r="D115" t="n">
-        <v>2.95</v>
+        <v>4.3</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>EQUIPPP</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>15.98</v>
+        <v>0.93</v>
       </c>
       <c r="C116" t="n">
-        <v>16.45</v>
+        <v>0.97</v>
       </c>
       <c r="D116" t="n">
-        <v>2.94</v>
+        <v>4.3</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>VIDYAWIRES</t>
+          <t>BLBLIMITED</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>101.61</v>
+        <v>16.58</v>
       </c>
       <c r="C117" t="n">
-        <v>104.6</v>
+        <v>17.29</v>
       </c>
       <c r="D117" t="n">
-        <v>2.94</v>
+        <v>4.28</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SMARTLINK</t>
+          <t>GMRAIRPORT</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>159.77</v>
+        <v>97.84</v>
       </c>
       <c r="C118" t="n">
-        <v>164.44</v>
+        <v>102</v>
       </c>
       <c r="D118" t="n">
-        <v>2.92</v>
+        <v>4.25</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>TREL</t>
+          <t>KISSHT</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>24.68</v>
+        <v>261.98</v>
       </c>
       <c r="C119" t="n">
-        <v>25.4</v>
+        <v>273</v>
       </c>
       <c r="D119" t="n">
-        <v>2.92</v>
+        <v>4.21</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>JMA</t>
+          <t>BEEKAY</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>89.36</v>
+        <v>416.55</v>
       </c>
       <c r="C120" t="n">
-        <v>91.97</v>
+        <v>434</v>
       </c>
       <c r="D120" t="n">
-        <v>2.92</v>
+        <v>4.19</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>AYMSYNTEX</t>
+          <t>MAGNUM</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>217.46</v>
+        <v>20.12</v>
       </c>
       <c r="C121" t="n">
-        <v>223.8</v>
+        <v>20.96</v>
       </c>
       <c r="D121" t="n">
-        <v>2.92</v>
+        <v>4.17</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>INTENTECH</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>98.03</v>
+        <v>0.24</v>
       </c>
       <c r="C122" t="n">
-        <v>100.87</v>
+        <v>0.25</v>
       </c>
       <c r="D122" t="n">
-        <v>2.9</v>
+        <v>4.17</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>VRAJ</t>
+          <t>IFBAGRO</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>122.47</v>
+        <v>1050.55</v>
       </c>
       <c r="C123" t="n">
-        <v>126</v>
+        <v>1094</v>
       </c>
       <c r="D123" t="n">
-        <v>2.88</v>
+        <v>4.14</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>KRIDHANINF</t>
+          <t>IDEAFORGE</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>3.13</v>
+        <v>845.3</v>
       </c>
       <c r="C124" t="n">
-        <v>3.22</v>
+        <v>880</v>
       </c>
       <c r="D124" t="n">
-        <v>2.88</v>
+        <v>4.11</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>KARNIKA</t>
+          <t>RVTH</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>145.8</v>
+        <v>790.75</v>
       </c>
       <c r="C125" t="n">
-        <v>150</v>
+        <v>823</v>
       </c>
       <c r="D125" t="n">
-        <v>2.88</v>
+        <v>4.08</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>GOLDENTOBC</t>
+          <t>AARON</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>26.15</v>
+        <v>120.9</v>
       </c>
       <c r="C126" t="n">
-        <v>26.9</v>
+        <v>125.8</v>
       </c>
       <c r="D126" t="n">
-        <v>2.87</v>
+        <v>4.05</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>NATCAPSUQ</t>
+          <t>UNIVASTU</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>152.42</v>
+        <v>75.87</v>
       </c>
       <c r="C127" t="n">
-        <v>156.8</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D127" t="n">
-        <v>2.87</v>
+        <v>3.99</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>TCI</t>
+          <t>UMAEXPORTS</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>899.9</v>
+        <v>25.85</v>
       </c>
       <c r="C128" t="n">
-        <v>924.95</v>
+        <v>26.88</v>
       </c>
       <c r="D128" t="n">
-        <v>2.78</v>
+        <v>3.98</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>LOKESHMACH</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>260.93</v>
+        <v>11.06</v>
       </c>
       <c r="C129" t="n">
-        <v>268</v>
+        <v>11.49</v>
       </c>
       <c r="D129" t="n">
-        <v>2.71</v>
+        <v>3.89</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>VINYAS</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>1.5</v>
+        <v>1106.95</v>
       </c>
       <c r="C130" t="n">
-        <v>1.54</v>
+        <v>1149.95</v>
       </c>
       <c r="D130" t="n">
-        <v>2.67</v>
+        <v>3.88</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>RUPA</t>
+          <t>CORDSCABLE</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>151.07</v>
+        <v>243.58</v>
       </c>
       <c r="C131" t="n">
-        <v>155</v>
+        <v>253</v>
       </c>
       <c r="D131" t="n">
-        <v>2.6</v>
+        <v>3.87</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>72.91</v>
+        <v>175.92</v>
       </c>
       <c r="C132" t="n">
-        <v>74.8</v>
+        <v>182.71</v>
       </c>
       <c r="D132" t="n">
-        <v>2.59</v>
+        <v>3.86</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>AMNPLST</t>
+          <t>LINC</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>193.02</v>
+        <v>98.13</v>
       </c>
       <c r="C133" t="n">
-        <v>198</v>
+        <v>101.9</v>
       </c>
       <c r="D133" t="n">
-        <v>2.58</v>
+        <v>3.84</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>TGL</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>13.26</v>
+        <v>23.5</v>
       </c>
       <c r="C134" t="n">
-        <v>13.6</v>
+        <v>24.4</v>
       </c>
       <c r="D134" t="n">
-        <v>2.56</v>
+        <v>3.83</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>LFIC</t>
+          <t>ANMOL</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>140.37</v>
+        <v>11.56</v>
       </c>
       <c r="C135" t="n">
-        <v>143.9</v>
+        <v>12</v>
       </c>
       <c r="D135" t="n">
-        <v>2.51</v>
+        <v>3.81</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>VINCOFE</t>
+          <t>CEREBRAINT</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>149.76</v>
+        <v>3.44</v>
       </c>
       <c r="C136" t="n">
-        <v>153.5</v>
+        <v>3.57</v>
       </c>
       <c r="D136" t="n">
-        <v>2.5</v>
+        <v>3.78</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>BOHRAIND</t>
+          <t>TAMBOLIIN</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>18.15</v>
+        <v>173.47</v>
       </c>
       <c r="C137" t="n">
-        <v>18.6</v>
+        <v>180</v>
       </c>
       <c r="D137" t="n">
-        <v>2.48</v>
+        <v>3.76</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>AXITA</t>
+          <t>APSISAERO</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>8.19</v>
+        <v>318.05</v>
       </c>
       <c r="C138" t="n">
-        <v>8.390000000000001</v>
+        <v>330</v>
       </c>
       <c r="D138" t="n">
-        <v>2.44</v>
+        <v>3.76</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>MOKSH</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>11.95</v>
+        <v>4</v>
       </c>
       <c r="C139" t="n">
-        <v>12.24</v>
+        <v>4.15</v>
       </c>
       <c r="D139" t="n">
-        <v>2.43</v>
+        <v>3.75</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>BASML</t>
+          <t>TROM</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>25.33</v>
+        <v>54</v>
       </c>
       <c r="C140" t="n">
-        <v>25.94</v>
+        <v>56</v>
       </c>
       <c r="D140" t="n">
-        <v>2.41</v>
+        <v>3.7</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>7.05</v>
+        <v>6.78</v>
       </c>
       <c r="C141" t="n">
-        <v>7.22</v>
+        <v>7.03</v>
       </c>
       <c r="D141" t="n">
-        <v>2.41</v>
+        <v>3.69</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>DECCANCE</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>615.25</v>
+        <v>75.04000000000001</v>
       </c>
       <c r="C142" t="n">
-        <v>630</v>
+        <v>77.8</v>
       </c>
       <c r="D142" t="n">
-        <v>2.4</v>
+        <v>3.68</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>AARTECH</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>44.81</v>
+        <v>192.76</v>
       </c>
       <c r="C143" t="n">
-        <v>45.87</v>
+        <v>199.8</v>
       </c>
       <c r="D143" t="n">
-        <v>2.37</v>
+        <v>3.65</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>EUROPRATIK</t>
+          <t>SECURKLOUD</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>250.05</v>
+        <v>20.5</v>
       </c>
       <c r="C144" t="n">
-        <v>255.95</v>
+        <v>21.24</v>
       </c>
       <c r="D144" t="n">
-        <v>2.36</v>
+        <v>3.61</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>NAGAFERT</t>
+          <t>ARHAM</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>3.83</v>
+        <v>144.6</v>
       </c>
       <c r="C145" t="n">
-        <v>3.92</v>
+        <v>149.8</v>
       </c>
       <c r="D145" t="n">
-        <v>2.35</v>
+        <v>3.6</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>MANAKSIA</t>
+          <t>DEVX</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>61.56</v>
+        <v>38.28</v>
       </c>
       <c r="C146" t="n">
-        <v>63</v>
+        <v>39.65</v>
       </c>
       <c r="D146" t="n">
-        <v>2.34</v>
+        <v>3.58</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>BAYERCROP</t>
+          <t>TNTELE</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>4500.8</v>
+        <v>9.24</v>
       </c>
       <c r="C147" t="n">
-        <v>4605</v>
+        <v>9.57</v>
       </c>
       <c r="D147" t="n">
-        <v>2.32</v>
+        <v>3.57</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>NIPPOBATRY</t>
+          <t>3BBLACKBIO</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>366.05</v>
+        <v>1221.7</v>
       </c>
       <c r="C148" t="n">
-        <v>374.5</v>
+        <v>1265</v>
       </c>
       <c r="D148" t="n">
-        <v>2.31</v>
+        <v>3.54</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>TIPSFILMS</t>
+          <t>BIOFILCHEM</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>368.6</v>
+        <v>35.62</v>
       </c>
       <c r="C149" t="n">
-        <v>377</v>
+        <v>36.85</v>
       </c>
       <c r="D149" t="n">
-        <v>2.28</v>
+        <v>3.45</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CPPLUS</t>
+          <t>CONSOFINVT</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>2648.7</v>
+        <v>231.88</v>
       </c>
       <c r="C150" t="n">
-        <v>2709.1</v>
+        <v>239.85</v>
       </c>
       <c r="D150" t="n">
-        <v>2.28</v>
+        <v>3.44</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>PRAENG</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>0.44</v>
+        <v>22.96</v>
       </c>
       <c r="C151" t="n">
-        <v>0.45</v>
+        <v>23.75</v>
       </c>
       <c r="D151" t="n">
-        <v>2.27</v>
+        <v>3.44</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>GALAPREC</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>3.52</v>
+        <v>944.35</v>
       </c>
       <c r="C152" t="n">
-        <v>3.6</v>
+        <v>976.6</v>
       </c>
       <c r="D152" t="n">
-        <v>2.27</v>
+        <v>3.42</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SHRIKRISH</t>
+          <t>TIMEX</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>42.05</v>
+        <v>423.55</v>
       </c>
       <c r="C153" t="n">
-        <v>43</v>
+        <v>438</v>
       </c>
       <c r="D153" t="n">
-        <v>2.26</v>
+        <v>3.41</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>BYKE</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>36.48</v>
+        <v>6.45</v>
       </c>
       <c r="C154" t="n">
-        <v>37.3</v>
+        <v>6.67</v>
       </c>
       <c r="D154" t="n">
-        <v>2.25</v>
+        <v>3.41</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>PAKKA</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>89.88</v>
+        <v>22.69</v>
       </c>
       <c r="C155" t="n">
-        <v>91.90000000000001</v>
+        <v>23.45</v>
       </c>
       <c r="D155" t="n">
-        <v>2.25</v>
+        <v>3.35</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>SUDEEPPHRM</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>6.27</v>
+        <v>674.7</v>
       </c>
       <c r="C156" t="n">
-        <v>6.41</v>
+        <v>697</v>
       </c>
       <c r="D156" t="n">
-        <v>2.23</v>
+        <v>3.31</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>PCJEWELLER</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>42.47</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C157" t="n">
-        <v>43.4</v>
+        <v>9.5</v>
       </c>
       <c r="D157" t="n">
-        <v>2.19</v>
+        <v>3.26</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>SOLARWORLD</t>
+          <t>SANSTAR</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>216.3</v>
+        <v>115.24</v>
       </c>
       <c r="C158" t="n">
-        <v>221</v>
+        <v>119</v>
       </c>
       <c r="D158" t="n">
-        <v>2.17</v>
+        <v>3.26</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>DECNGOLD</t>
+          <t>CGRAPHICS</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>176.86</v>
+        <v>148</v>
       </c>
       <c r="C159" t="n">
-        <v>180.7</v>
+        <v>152.8</v>
       </c>
       <c r="D159" t="n">
-        <v>2.17</v>
+        <v>3.24</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>2.31</v>
+        <v>93.29000000000001</v>
       </c>
       <c r="C160" t="n">
-        <v>2.36</v>
+        <v>96.31</v>
       </c>
       <c r="D160" t="n">
-        <v>2.16</v>
+        <v>3.24</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ANTELOPUS</t>
+          <t>SURYALA</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>766.85</v>
+        <v>466.8</v>
       </c>
       <c r="C161" t="n">
-        <v>783.25</v>
+        <v>481.9</v>
       </c>
       <c r="D161" t="n">
-        <v>2.14</v>
+        <v>3.23</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>IWARE</t>
+          <t>ORIENTCER</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>359.75</v>
+        <v>42.14</v>
       </c>
       <c r="C162" t="n">
-        <v>367.4</v>
+        <v>43.5</v>
       </c>
       <c r="D162" t="n">
-        <v>2.13</v>
+        <v>3.23</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>RPPINFRA</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>3.76</v>
+        <v>75.05</v>
       </c>
       <c r="C163" t="n">
-        <v>3.84</v>
+        <v>77.44</v>
       </c>
       <c r="D163" t="n">
-        <v>2.13</v>
+        <v>3.18</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>FINKURVE</t>
+          <t>SAHYADRI</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>63.16</v>
+        <v>279.6</v>
       </c>
       <c r="C164" t="n">
-        <v>64.5</v>
+        <v>288.45</v>
       </c>
       <c r="D164" t="n">
-        <v>2.12</v>
+        <v>3.17</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>DCM</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>92.05</v>
+        <v>6.97</v>
       </c>
       <c r="C165" t="n">
-        <v>93.98</v>
+        <v>7.19</v>
       </c>
       <c r="D165" t="n">
-        <v>2.1</v>
+        <v>3.16</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>RUSHIL</t>
+          <t>BTTL</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>15.81</v>
+        <v>34.42</v>
       </c>
       <c r="C166" t="n">
-        <v>16.14</v>
+        <v>35.5</v>
       </c>
       <c r="D166" t="n">
-        <v>2.09</v>
+        <v>3.14</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>ECOLINE</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>0.48</v>
+        <v>153.2</v>
       </c>
       <c r="C167" t="n">
-        <v>0.49</v>
+        <v>158</v>
       </c>
       <c r="D167" t="n">
-        <v>2.08</v>
+        <v>3.13</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>KEC</t>
+          <t>AURIGROW</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>499.1</v>
+        <v>0.32</v>
       </c>
       <c r="C168" t="n">
-        <v>509.5</v>
+        <v>0.33</v>
       </c>
       <c r="D168" t="n">
-        <v>2.08</v>
+        <v>3.13</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>COUNCODOS</t>
+          <t>SINCLAIR</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>4.85</v>
+        <v>74.08</v>
       </c>
       <c r="C169" t="n">
-        <v>4.95</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="D169" t="n">
-        <v>2.06</v>
+        <v>3.13</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SAAKSHI</t>
+          <t>RSDFIN</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>229.3</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="C170" t="n">
-        <v>234</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="D170" t="n">
-        <v>2.05</v>
+        <v>3.12</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>GRCL</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>5.84</v>
+        <v>533.05</v>
       </c>
       <c r="C171" t="n">
-        <v>5.96</v>
+        <v>549.7</v>
       </c>
       <c r="D171" t="n">
-        <v>2.05</v>
+        <v>3.12</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>OMFREIGHT</t>
+          <t>COMPINFO</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>87.31999999999999</v>
+        <v>1.3</v>
       </c>
       <c r="C172" t="n">
-        <v>89.09999999999999</v>
+        <v>1.34</v>
       </c>
       <c r="D172" t="n">
-        <v>2.04</v>
+        <v>3.08</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>VIPULLTD</t>
+          <t>RKDL</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>8.81</v>
+        <v>21.47</v>
       </c>
       <c r="C173" t="n">
-        <v>8.99</v>
+        <v>22.13</v>
       </c>
       <c r="D173" t="n">
-        <v>2.04</v>
+        <v>3.07</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>GOLDTECH</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>50.96</v>
+        <v>48.37</v>
       </c>
       <c r="C174" t="n">
-        <v>52</v>
+        <v>49.85</v>
       </c>
       <c r="D174" t="n">
-        <v>2.04</v>
+        <v>3.06</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>BAJAJCON</t>
+          <t>ZODIACLOTH</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>554.8</v>
+        <v>76.8</v>
       </c>
       <c r="C175" t="n">
-        <v>566</v>
+        <v>79.15000000000001</v>
       </c>
       <c r="D175" t="n">
-        <v>2.02</v>
+        <v>3.06</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>IRIS</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>253.79</v>
+        <v>353.1</v>
       </c>
       <c r="C176" t="n">
-        <v>258.88</v>
+        <v>363.9</v>
       </c>
       <c r="D176" t="n">
-        <v>2.01</v>
+        <v>3.06</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>KOHINOOR</t>
+          <t>SASKEN</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>24.84</v>
+        <v>2161.9</v>
       </c>
       <c r="C177" t="n">
-        <v>25.34</v>
+        <v>2227.9</v>
       </c>
       <c r="D177" t="n">
-        <v>2.01</v>
+        <v>3.05</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>SRM</t>
+          <t>KRISHCA</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>515.65</v>
+        <v>181.5</v>
       </c>
       <c r="C178" t="n">
-        <v>525.95</v>
+        <v>187</v>
       </c>
       <c r="D178" t="n">
-        <v>2</v>
+        <v>3.03</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>KHAICHEM</t>
+          <t>ASAHIINDIA</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>55.04</v>
+        <v>918.55</v>
       </c>
       <c r="C179" t="n">
-        <v>56.14</v>
+        <v>946.25</v>
       </c>
       <c r="D179" t="n">
-        <v>2</v>
+        <v>3.02</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>DREAMFOLKS</t>
+          <t>MPHASIS</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>78.42</v>
+        <v>2232.9</v>
       </c>
       <c r="C180" t="n">
-        <v>79.98999999999999</v>
+        <v>2300</v>
       </c>
       <c r="D180" t="n">
-        <v>2</v>
+        <v>3.01</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>PML</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>8.48</v>
+        <v>563.15</v>
       </c>
       <c r="C181" t="n">
-        <v>8.65</v>
+        <v>580</v>
       </c>
       <c r="D181" t="n">
-        <v>2</v>
+        <v>2.99</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>BIRLAPREC</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>8.51</v>
+        <v>45.45</v>
       </c>
       <c r="C182" t="n">
-        <v>8.68</v>
+        <v>46.8</v>
       </c>
       <c r="D182" t="n">
-        <v>2</v>
+        <v>2.97</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>TERASOFT</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>93.54000000000001</v>
+        <v>375.7</v>
       </c>
       <c r="C183" t="n">
-        <v>95.40000000000001</v>
+        <v>386.8</v>
       </c>
       <c r="D183" t="n">
-        <v>1.99</v>
+        <v>2.95</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>GUJAPOLLO</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>389.05</v>
+        <v>0.34</v>
       </c>
       <c r="C184" t="n">
-        <v>396.8</v>
+        <v>0.35</v>
       </c>
       <c r="D184" t="n">
-        <v>1.99</v>
+        <v>2.94</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>6.06</v>
+        <v>466.7</v>
       </c>
       <c r="C185" t="n">
-        <v>6.18</v>
+        <v>480.4</v>
       </c>
       <c r="D185" t="n">
-        <v>1.98</v>
+        <v>2.94</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>BCONCEPTS</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>55.78</v>
+        <v>199.15</v>
       </c>
       <c r="C186" t="n">
-        <v>56.88</v>
+        <v>204.99</v>
       </c>
       <c r="D186" t="n">
-        <v>1.97</v>
+        <v>2.93</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>KANPRPLA</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>207.92</v>
+        <v>10.92</v>
       </c>
       <c r="C187" t="n">
-        <v>212</v>
+        <v>11.24</v>
       </c>
       <c r="D187" t="n">
-        <v>1.96</v>
+        <v>2.93</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SSDL</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>61.59</v>
+        <v>29.93</v>
       </c>
       <c r="C188" t="n">
-        <v>62.8</v>
+        <v>30.8</v>
       </c>
       <c r="D188" t="n">
-        <v>1.96</v>
+        <v>2.91</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>PINELABS</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>137.94</v>
+        <v>330.2</v>
       </c>
       <c r="C189" t="n">
-        <v>140.65</v>
+        <v>339.7</v>
       </c>
       <c r="D189" t="n">
-        <v>1.96</v>
+        <v>2.88</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>KNAGRI</t>
+          <t>JNKINDIA</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>190.69</v>
+        <v>381.9</v>
       </c>
       <c r="C190" t="n">
-        <v>194.4</v>
+        <v>392.9</v>
       </c>
       <c r="D190" t="n">
-        <v>1.95</v>
+        <v>2.88</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>BIRLACABLE</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>61.7</v>
+        <v>184.68</v>
       </c>
       <c r="C191" t="n">
-        <v>62.9</v>
+        <v>190</v>
       </c>
       <c r="D191" t="n">
-        <v>1.94</v>
+        <v>2.88</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>IFBIND</t>
+          <t>MARINE</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>1147.9</v>
+        <v>247.92</v>
       </c>
       <c r="C192" t="n">
-        <v>1170</v>
+        <v>255</v>
       </c>
       <c r="D192" t="n">
-        <v>1.93</v>
+        <v>2.86</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>MANCREDIT</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>2.07</v>
+        <v>191.54</v>
       </c>
       <c r="C193" t="n">
-        <v>2.11</v>
+        <v>197</v>
       </c>
       <c r="D193" t="n">
-        <v>1.93</v>
+        <v>2.85</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>0.52</v>
+        <v>171.09</v>
       </c>
       <c r="C194" t="n">
-        <v>0.53</v>
+        <v>175.86</v>
       </c>
       <c r="D194" t="n">
-        <v>1.92</v>
+        <v>2.79</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>VINNY</t>
+          <t>TRANSPEK</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>1.06</v>
+        <v>1069.6</v>
       </c>
       <c r="C195" t="n">
-        <v>1.08</v>
+        <v>1099</v>
       </c>
       <c r="D195" t="n">
-        <v>1.89</v>
+        <v>2.75</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>AKG</t>
+          <t>GFLLIMITED</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>11.11</v>
+        <v>47.69</v>
       </c>
       <c r="C196" t="n">
-        <v>11.32</v>
+        <v>49</v>
       </c>
       <c r="D196" t="n">
-        <v>1.89</v>
+        <v>2.75</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>OILCOUNTUB</t>
+          <t>NRL</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>55.9</v>
+        <v>63.16</v>
       </c>
       <c r="C197" t="n">
-        <v>56.95</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="D197" t="n">
-        <v>1.88</v>
+        <v>2.75</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>INDOTHAI</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>245.15</v>
+        <v>379.65</v>
       </c>
       <c r="C198" t="n">
-        <v>249.75</v>
+        <v>390</v>
       </c>
       <c r="D198" t="n">
-        <v>1.88</v>
+        <v>2.73</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>KOTHARIPET</t>
+          <t>EMMBI</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>126.57</v>
+        <v>84.20999999999999</v>
       </c>
       <c r="C199" t="n">
-        <v>128.95</v>
+        <v>86.5</v>
       </c>
       <c r="D199" t="n">
-        <v>1.88</v>
+        <v>2.72</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>PPAP</t>
+          <t>KAMATHOTEL</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>211</v>
+        <v>169.4</v>
       </c>
       <c r="C200" t="n">
-        <v>214.95</v>
+        <v>174</v>
       </c>
       <c r="D200" t="n">
-        <v>1.87</v>
+        <v>2.72</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>PCJEWELLER</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>9.119999999999999</v>
+        <v>918.5</v>
       </c>
       <c r="C201" t="n">
-        <v>9.289999999999999</v>
+        <v>943.3</v>
       </c>
       <c r="D201" t="n">
-        <v>1.86</v>
+        <v>2.7</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-01 09:04 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,14 +461,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MOTOGENFIN</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>27.35</v>
+        <v>68.25</v>
       </c>
       <c r="C2" t="n">
-        <v>32.82</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="D2" t="n">
         <v>20</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SAHLIBHFI</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>72.06999999999999</v>
+        <v>16.69</v>
       </c>
       <c r="C3" t="n">
-        <v>86</v>
+        <v>19.99</v>
       </c>
       <c r="D3" t="n">
-        <v>19.33</v>
+        <v>19.77</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VADILALIND</t>
+          <t>WOCKPHARMA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4466.9</v>
+        <v>2031.4</v>
       </c>
       <c r="C4" t="n">
-        <v>5150</v>
+        <v>2377</v>
       </c>
       <c r="D4" t="n">
-        <v>15.29</v>
+        <v>17.01</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAYAJIHOTL</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>282.95</v>
+        <v>6.01</v>
       </c>
       <c r="C5" t="n">
-        <v>323.95</v>
+        <v>6.97</v>
       </c>
       <c r="D5" t="n">
-        <v>14.49</v>
+        <v>15.97</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>COFFEEDAY</t>
+          <t>IPHL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28.99</v>
+        <v>61.25</v>
       </c>
       <c r="C6" t="n">
-        <v>33</v>
+        <v>69.8</v>
       </c>
       <c r="D6" t="n">
-        <v>13.83</v>
+        <v>13.96</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AVTNPL</t>
+          <t>RILINFRA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>68.64</v>
+        <v>35.4</v>
       </c>
       <c r="C7" t="n">
-        <v>76.90000000000001</v>
+        <v>40</v>
       </c>
       <c r="D7" t="n">
-        <v>12.03</v>
+        <v>12.99</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MERCANTILE</t>
+          <t>TOUCHWOOD</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25.64</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>28.59</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>11.51</v>
+        <v>11.03</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>137.91</v>
+        <v>242.18</v>
       </c>
       <c r="C9" t="n">
-        <v>153.39</v>
+        <v>266.39</v>
       </c>
       <c r="D9" t="n">
-        <v>11.22</v>
+        <v>10</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADISOFT</t>
+          <t>COFFEEDAY</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>194</v>
+        <v>34.78</v>
       </c>
       <c r="C10" t="n">
-        <v>215</v>
+        <v>38.25</v>
       </c>
       <c r="D10" t="n">
-        <v>10.82</v>
+        <v>9.98</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DYNPRO</t>
+          <t>SHARDUL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>231.12</v>
+        <v>28.25</v>
       </c>
       <c r="C11" t="n">
-        <v>255</v>
+        <v>31</v>
       </c>
       <c r="D11" t="n">
-        <v>10.33</v>
+        <v>9.73</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>HARDWYN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>220.17</v>
+        <v>25.16</v>
       </c>
       <c r="C12" t="n">
-        <v>242.18</v>
+        <v>27.48</v>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CPPLUS</t>
+          <t>SOMATEX</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2639.6</v>
+        <v>106.84</v>
       </c>
       <c r="C13" t="n">
-        <v>2903.5</v>
+        <v>116.45</v>
       </c>
       <c r="D13" t="n">
-        <v>10</v>
+        <v>8.99</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SUPRIYA</t>
+          <t>TAALTECH</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>807.25</v>
+        <v>3558.9</v>
       </c>
       <c r="C14" t="n">
-        <v>887.3</v>
+        <v>3876.6</v>
       </c>
       <c r="D14" t="n">
-        <v>9.92</v>
+        <v>8.93</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FALCONTECH</t>
+          <t>DGCONTENT</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>13.65</v>
+        <v>26.65</v>
       </c>
       <c r="C15" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D15" t="n">
-        <v>9.890000000000001</v>
+        <v>8.82</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BIKEWO</t>
+          <t>SAHANA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>26.85</v>
+        <v>823.9</v>
       </c>
       <c r="C16" t="n">
-        <v>29.5</v>
+        <v>895</v>
       </c>
       <c r="D16" t="n">
-        <v>9.869999999999999</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KIRANVYPAR</t>
+          <t>DYNAMIC</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>163.91</v>
+        <v>143</v>
       </c>
       <c r="C17" t="n">
-        <v>179.99</v>
+        <v>154.95</v>
       </c>
       <c r="D17" t="n">
-        <v>9.81</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRAJ</t>
+          <t>NSLNISP</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>122.49</v>
+        <v>44.62</v>
       </c>
       <c r="C18" t="n">
-        <v>134.5</v>
+        <v>48.3</v>
       </c>
       <c r="D18" t="n">
-        <v>9.800000000000001</v>
+        <v>8.25</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ALGOQUANT</t>
+          <t>SVLL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>56.99</v>
+        <v>615.3</v>
       </c>
       <c r="C19" t="n">
-        <v>62.4</v>
+        <v>666</v>
       </c>
       <c r="D19" t="n">
-        <v>9.49</v>
+        <v>8.24</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8.94</v>
+        <v>25.02</v>
       </c>
       <c r="C20" t="n">
-        <v>9.76</v>
+        <v>26.99</v>
       </c>
       <c r="D20" t="n">
-        <v>9.17</v>
+        <v>7.87</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>UHTL</t>
+          <t>SAIPARENT</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>56.9</v>
+        <v>485.9</v>
       </c>
       <c r="C21" t="n">
-        <v>62</v>
+        <v>523.95</v>
       </c>
       <c r="D21" t="n">
-        <v>8.960000000000001</v>
+        <v>7.83</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>WOCKPHARMA</t>
+          <t>MFML</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1771</v>
+        <v>25.01</v>
       </c>
       <c r="C22" t="n">
-        <v>1925</v>
+        <v>26.95</v>
       </c>
       <c r="D22" t="n">
-        <v>8.699999999999999</v>
+        <v>7.76</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NMSTEEL</t>
+          <t>RPPL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>23.7</v>
+        <v>16.91</v>
       </c>
       <c r="C23" t="n">
-        <v>25.7</v>
+        <v>18.2</v>
       </c>
       <c r="D23" t="n">
-        <v>8.44</v>
+        <v>7.63</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EIFFL</t>
+          <t>MSTCLTD</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>235.3</v>
+        <v>440.5</v>
       </c>
       <c r="C24" t="n">
-        <v>255</v>
+        <v>474</v>
       </c>
       <c r="D24" t="n">
-        <v>8.369999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>14.49</v>
+        <v>165.49</v>
       </c>
       <c r="C25" t="n">
-        <v>15.68</v>
+        <v>177.99</v>
       </c>
       <c r="D25" t="n">
-        <v>8.210000000000001</v>
+        <v>7.55</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PALASHSECU</t>
+          <t>VIGOR</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>98.95</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="C26" t="n">
-        <v>106.75</v>
+        <v>70.2</v>
       </c>
       <c r="D26" t="n">
-        <v>7.88</v>
+        <v>7.34</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>JAGRAN</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>70.05</v>
+        <v>15.3</v>
       </c>
       <c r="C27" t="n">
-        <v>75.25</v>
+        <v>16.4</v>
       </c>
       <c r="D27" t="n">
-        <v>7.42</v>
+        <v>7.19</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>JPPOWER</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>22.87</v>
+        <v>10.02</v>
       </c>
       <c r="C28" t="n">
-        <v>24.5</v>
+        <v>10.74</v>
       </c>
       <c r="D28" t="n">
-        <v>7.13</v>
+        <v>7.19</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>WIPL</t>
+          <t>ARIHANT</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>147.75</v>
+        <v>893.85</v>
       </c>
       <c r="C29" t="n">
-        <v>158</v>
+        <v>957.95</v>
       </c>
       <c r="D29" t="n">
-        <v>6.94</v>
+        <v>7.17</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MONOLITH</t>
+          <t>SUVEN</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>556.7</v>
+        <v>279.34</v>
       </c>
       <c r="C30" t="n">
-        <v>595</v>
+        <v>297.95</v>
       </c>
       <c r="D30" t="n">
-        <v>6.88</v>
+        <v>6.66</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SKYGOLD</t>
+          <t>UFLEX</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>486.65</v>
+        <v>423.95</v>
       </c>
       <c r="C31" t="n">
-        <v>520</v>
+        <v>452.05</v>
       </c>
       <c r="D31" t="n">
-        <v>6.85</v>
+        <v>6.63</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AYMSYNTEX</t>
+          <t>BSL</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>219.48</v>
+        <v>131.41</v>
       </c>
       <c r="C32" t="n">
-        <v>234.1</v>
+        <v>139.98</v>
       </c>
       <c r="D32" t="n">
-        <v>6.66</v>
+        <v>6.52</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>SURAJLTD</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>24.4</v>
+        <v>224.37</v>
       </c>
       <c r="C33" t="n">
-        <v>26</v>
+        <v>239</v>
       </c>
       <c r="D33" t="n">
-        <v>6.56</v>
+        <v>6.52</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MMP</t>
+          <t>OLECTRA</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>279.27</v>
+        <v>1180</v>
       </c>
       <c r="C34" t="n">
-        <v>296.95</v>
+        <v>1255</v>
       </c>
       <c r="D34" t="n">
-        <v>6.33</v>
+        <v>6.36</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ANONDITA</t>
+          <t>BANARBEADS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1013.25</v>
+        <v>107.39</v>
       </c>
       <c r="C35" t="n">
-        <v>1077</v>
+        <v>113.88</v>
       </c>
       <c r="D35" t="n">
-        <v>6.29</v>
+        <v>6.04</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LORDSCHLO</t>
+          <t>SHREERAMA</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>141.48</v>
+        <v>42.85</v>
       </c>
       <c r="C36" t="n">
-        <v>150.3</v>
+        <v>45.4</v>
       </c>
       <c r="D36" t="n">
-        <v>6.23</v>
+        <v>5.95</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SJLOGISTIC</t>
+          <t>VASWANI</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>339.2</v>
+        <v>56.63</v>
       </c>
       <c r="C37" t="n">
-        <v>360</v>
+        <v>60</v>
       </c>
       <c r="D37" t="n">
-        <v>6.13</v>
+        <v>5.95</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TAJGVK</t>
+          <t>CPPLUS</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>321.25</v>
+        <v>2903.5</v>
       </c>
       <c r="C38" t="n">
-        <v>340.95</v>
+        <v>3074.7</v>
       </c>
       <c r="D38" t="n">
-        <v>6.13</v>
+        <v>5.9</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GANGAFORGE</t>
+          <t>PTCIL</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2.34</v>
+        <v>16191</v>
       </c>
       <c r="C39" t="n">
-        <v>2.48</v>
+        <v>17124</v>
       </c>
       <c r="D39" t="n">
-        <v>5.98</v>
+        <v>5.76</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>10.36</v>
+        <v>1442.9</v>
       </c>
       <c r="C40" t="n">
-        <v>10.98</v>
+        <v>1525</v>
       </c>
       <c r="D40" t="n">
-        <v>5.98</v>
+        <v>5.69</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SHIVALIK</t>
+          <t>JAIPURKURT</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>259.15</v>
+        <v>32.13</v>
       </c>
       <c r="C41" t="n">
-        <v>274.5</v>
+        <v>33.95</v>
       </c>
       <c r="D41" t="n">
-        <v>5.92</v>
+        <v>5.66</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>5PAISA</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>184.34</v>
+        <v>327.7</v>
       </c>
       <c r="C42" t="n">
-        <v>195</v>
+        <v>346</v>
       </c>
       <c r="D42" t="n">
-        <v>5.78</v>
+        <v>5.58</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BLUSPRING</t>
+          <t>OCCLLTD</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>68.76000000000001</v>
+        <v>114.73</v>
       </c>
       <c r="C43" t="n">
-        <v>72.72</v>
+        <v>121</v>
       </c>
       <c r="D43" t="n">
-        <v>5.76</v>
+        <v>5.47</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BNALTD</t>
+          <t>METROGLOBL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>359.3</v>
+        <v>128.1</v>
       </c>
       <c r="C44" t="n">
-        <v>379.9</v>
+        <v>135</v>
       </c>
       <c r="D44" t="n">
-        <v>5.73</v>
+        <v>5.39</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BIMETAL</t>
+          <t>BCONCEPTS</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>572.15</v>
+        <v>196.42</v>
       </c>
       <c r="C45" t="n">
-        <v>604.95</v>
+        <v>207</v>
       </c>
       <c r="D45" t="n">
-        <v>5.73</v>
+        <v>5.39</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>INNOVANA</t>
+          <t>RADAAN</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>329.95</v>
+        <v>3.03</v>
       </c>
       <c r="C46" t="n">
-        <v>348.8</v>
+        <v>3.19</v>
       </c>
       <c r="D46" t="n">
-        <v>5.71</v>
+        <v>5.28</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>VETO</t>
+          <t>EUROBOND</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>122.08</v>
+        <v>184.26</v>
       </c>
       <c r="C47" t="n">
-        <v>129</v>
+        <v>193.75</v>
       </c>
       <c r="D47" t="n">
-        <v>5.67</v>
+        <v>5.15</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SHUBHSHREE</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>301</v>
+        <v>23.02</v>
       </c>
       <c r="C48" t="n">
-        <v>318</v>
+        <v>24.2</v>
       </c>
       <c r="D48" t="n">
-        <v>5.65</v>
+        <v>5.13</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DAMODARIND</t>
+          <t>RAJPALAYAM</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>31.66</v>
+        <v>804.6</v>
       </c>
       <c r="C49" t="n">
-        <v>33.4</v>
+        <v>845</v>
       </c>
       <c r="D49" t="n">
-        <v>5.5</v>
+        <v>5.02</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>EMAMIPAP</t>
+          <t>DECNGOLD</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>79.81999999999999</v>
+        <v>162.28</v>
       </c>
       <c r="C50" t="n">
-        <v>84.19</v>
+        <v>170.42</v>
       </c>
       <c r="D50" t="n">
-        <v>5.47</v>
+        <v>5.02</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>204</v>
+        <v>536.15</v>
       </c>
       <c r="C51" t="n">
-        <v>214.7</v>
+        <v>562.95</v>
       </c>
       <c r="D51" t="n">
-        <v>5.25</v>
+        <v>5</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ALKALI</t>
+          <t>MASKINVEST</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>89.45999999999999</v>
+        <v>152.05</v>
       </c>
       <c r="C52" t="n">
-        <v>94</v>
+        <v>159.65</v>
       </c>
       <c r="D52" t="n">
-        <v>5.07</v>
+        <v>5</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,14 +1583,14 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BEDMUTHA</t>
+          <t>SWANDEF</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>108</v>
+        <v>2060.2</v>
       </c>
       <c r="C53" t="n">
-        <v>113.4</v>
+        <v>2163.2</v>
       </c>
       <c r="D53" t="n">
         <v>5</v>
@@ -1605,14 +1605,14 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ATLANTAELE</t>
+          <t>JKIPL</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1878.3</v>
+        <v>89.64</v>
       </c>
       <c r="C54" t="n">
-        <v>1972.2</v>
+        <v>94.12</v>
       </c>
       <c r="D54" t="n">
         <v>5</v>
@@ -1627,14 +1627,14 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>VIPCLOTHNG</t>
+          <t>BIRLACABLE</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>26.62</v>
+        <v>193.91</v>
       </c>
       <c r="C55" t="n">
-        <v>27.95</v>
+        <v>203.6</v>
       </c>
       <c r="D55" t="n">
         <v>5</v>
@@ -1649,14 +1649,14 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MRIL</t>
+          <t>HRHNEXT</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C56" t="n">
-        <v>39.9</v>
+        <v>28.35</v>
       </c>
       <c r="D56" t="n">
         <v>5</v>
@@ -1671,14 +1671,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>POLYSIL</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>11.81</v>
+        <v>144.05</v>
       </c>
       <c r="C57" t="n">
-        <v>12.4</v>
+        <v>151.25</v>
       </c>
       <c r="D57" t="n">
         <v>5</v>
@@ -1693,14 +1693,14 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CKKRETAIL</t>
+          <t>PLAZACABLE</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>144.1</v>
+        <v>46.81</v>
       </c>
       <c r="C58" t="n">
-        <v>151.3</v>
+        <v>49.15</v>
       </c>
       <c r="D58" t="n">
         <v>5</v>
@@ -1715,14 +1715,14 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>IZMO</t>
+          <t>SOFTTECH</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>715.15</v>
+        <v>459.3</v>
       </c>
       <c r="C59" t="n">
-        <v>750.9</v>
+        <v>482.25</v>
       </c>
       <c r="D59" t="n">
         <v>5</v>
@@ -1737,14 +1737,14 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>WANBURY</t>
+          <t>BEDMUTHA</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>300.2</v>
+        <v>113.4</v>
       </c>
       <c r="C60" t="n">
-        <v>315.2</v>
+        <v>119.07</v>
       </c>
       <c r="D60" t="n">
         <v>5</v>
@@ -1759,14 +1759,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>NIRAJISPAT</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>223.24</v>
+        <v>1280.05</v>
       </c>
       <c r="C61" t="n">
-        <v>234.4</v>
+        <v>1344.1</v>
       </c>
       <c r="D61" t="n">
         <v>5</v>
@@ -1781,14 +1781,14 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MCON</t>
+          <t>SAKUMA</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="C62" t="n">
-        <v>40.95</v>
+        <v>2.1</v>
       </c>
       <c r="D62" t="n">
         <v>5</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>TERASOFT</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1219.1</v>
+        <v>394.45</v>
       </c>
       <c r="C63" t="n">
-        <v>1280.05</v>
+        <v>414.15</v>
       </c>
       <c r="D63" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,14 +1825,14 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>510.65</v>
+        <v>21.03</v>
       </c>
       <c r="C64" t="n">
-        <v>536.15</v>
+        <v>22.08</v>
       </c>
       <c r="D64" t="n">
         <v>4.99</v>
@@ -1847,14 +1847,14 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>UTLSOLAR</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>312.8</v>
+        <v>750.9</v>
       </c>
       <c r="C65" t="n">
-        <v>328.4</v>
+        <v>788.4</v>
       </c>
       <c r="D65" t="n">
         <v>4.99</v>
@@ -1869,14 +1869,14 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>404.6</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="C66" t="n">
-        <v>424.8</v>
+        <v>68.55</v>
       </c>
       <c r="D66" t="n">
         <v>4.99</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ARVEE</t>
+          <t>MSPL</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>160.03</v>
+        <v>42.72</v>
       </c>
       <c r="C67" t="n">
-        <v>168</v>
+        <v>44.85</v>
       </c>
       <c r="D67" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>STLNETWORK</t>
+          <t>PRIZOR</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>28.93</v>
+        <v>658.75</v>
       </c>
       <c r="C68" t="n">
-        <v>30.37</v>
+        <v>691.65</v>
       </c>
       <c r="D68" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,14 +1935,14 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>YAAP</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>22.51</v>
+        <v>199.95</v>
       </c>
       <c r="C69" t="n">
-        <v>23.63</v>
+        <v>209.9</v>
       </c>
       <c r="D69" t="n">
         <v>4.98</v>
@@ -1957,14 +1957,14 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>GENSOL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>62.19</v>
+        <v>18.87</v>
       </c>
       <c r="C70" t="n">
-        <v>65.29000000000001</v>
+        <v>19.81</v>
       </c>
       <c r="D70" t="n">
         <v>4.98</v>
@@ -1979,14 +1979,14 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>SEMAC</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>56.83</v>
+        <v>303.95</v>
       </c>
       <c r="C71" t="n">
-        <v>59.66</v>
+        <v>319.1</v>
       </c>
       <c r="D71" t="n">
         <v>4.98</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SPECTSTM</t>
+          <t>VTL</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>63.6</v>
+        <v>577.15</v>
       </c>
       <c r="C72" t="n">
-        <v>66.75</v>
+        <v>605.9</v>
       </c>
       <c r="D72" t="n">
-        <v>4.95</v>
+        <v>4.98</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ROXHITECH</t>
+          <t>BILVYAPAR</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>36.45</v>
+        <v>4.62</v>
       </c>
       <c r="C73" t="n">
-        <v>38.25</v>
+        <v>4.85</v>
       </c>
       <c r="D73" t="n">
-        <v>4.94</v>
+        <v>4.98</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>REGENCERAM</t>
+          <t>EPWINDIA</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>40.98</v>
+        <v>129.9</v>
       </c>
       <c r="C74" t="n">
-        <v>43</v>
+        <v>136.35</v>
       </c>
       <c r="D74" t="n">
-        <v>4.93</v>
+        <v>4.97</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>SADBHAV</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>437.45</v>
+        <v>9.65</v>
       </c>
       <c r="C75" t="n">
-        <v>459</v>
+        <v>10.13</v>
       </c>
       <c r="D75" t="n">
-        <v>4.93</v>
+        <v>4.97</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SONAMAC</t>
+          <t>TROM</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>39.65</v>
+        <v>56.7</v>
       </c>
       <c r="C76" t="n">
-        <v>41.6</v>
+        <v>59.5</v>
       </c>
       <c r="D76" t="n">
-        <v>4.92</v>
+        <v>4.94</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>DCMFINSERV</t>
+          <t>VIPCLOTHNG</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>5.7</v>
+        <v>26.52</v>
       </c>
       <c r="C77" t="n">
-        <v>5.98</v>
+        <v>27.83</v>
       </c>
       <c r="D77" t="n">
-        <v>4.91</v>
+        <v>4.94</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>FMNL</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>54.28</v>
+        <v>10.73</v>
       </c>
       <c r="C78" t="n">
-        <v>56.94</v>
+        <v>11.26</v>
       </c>
       <c r="D78" t="n">
-        <v>4.9</v>
+        <v>4.94</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>OMAXAUTO</t>
+          <t>BALAXI</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>251.12</v>
+        <v>26.21</v>
       </c>
       <c r="C79" t="n">
-        <v>263.4</v>
+        <v>27.5</v>
       </c>
       <c r="D79" t="n">
-        <v>4.89</v>
+        <v>4.92</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ORTINGLOBE</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>16.31</v>
+        <v>2.24</v>
       </c>
       <c r="C80" t="n">
-        <v>17.1</v>
+        <v>2.35</v>
       </c>
       <c r="D80" t="n">
-        <v>4.84</v>
+        <v>4.91</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>FAZE3Q</t>
+          <t>SHRIKANHA</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>523.6</v>
+        <v>26.45</v>
       </c>
       <c r="C81" t="n">
-        <v>548.9</v>
+        <v>27.75</v>
       </c>
       <c r="D81" t="n">
-        <v>4.83</v>
+        <v>4.91</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>MRIL</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>71.55</v>
+        <v>39.9</v>
       </c>
       <c r="C82" t="n">
-        <v>74.98999999999999</v>
+        <v>41.85</v>
       </c>
       <c r="D82" t="n">
-        <v>4.81</v>
+        <v>4.89</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>VIPULLTD</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>40.84</v>
+        <v>8.81</v>
       </c>
       <c r="C83" t="n">
-        <v>42.8</v>
+        <v>9.24</v>
       </c>
       <c r="D83" t="n">
-        <v>4.8</v>
+        <v>4.88</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>113.5</v>
+        <v>38</v>
       </c>
       <c r="C84" t="n">
-        <v>118.95</v>
+        <v>39.85</v>
       </c>
       <c r="D84" t="n">
-        <v>4.8</v>
+        <v>4.87</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>DEVIT</t>
+          <t>DCMFINSERV</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>29.11</v>
+        <v>5.98</v>
       </c>
       <c r="C85" t="n">
-        <v>30.5</v>
+        <v>6.27</v>
       </c>
       <c r="D85" t="n">
-        <v>4.77</v>
+        <v>4.85</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ARENTERP</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>39.13</v>
+        <v>4.74</v>
       </c>
       <c r="C86" t="n">
-        <v>40.99</v>
+        <v>4.97</v>
       </c>
       <c r="D86" t="n">
-        <v>4.75</v>
+        <v>4.85</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>PRIZOR</t>
+          <t>SURANI</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>627.4</v>
+        <v>120.2</v>
       </c>
       <c r="C87" t="n">
-        <v>657</v>
+        <v>126</v>
       </c>
       <c r="D87" t="n">
-        <v>4.72</v>
+        <v>4.83</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>RUDRA</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>18.42</v>
+        <v>52.85</v>
       </c>
       <c r="C88" t="n">
-        <v>19.29</v>
+        <v>55.4</v>
       </c>
       <c r="D88" t="n">
-        <v>4.72</v>
+        <v>4.82</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SCANSTL</t>
+          <t>BGLOBAL</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>37.99</v>
+        <v>3.12</v>
       </c>
       <c r="C89" t="n">
-        <v>39.77</v>
+        <v>3.27</v>
       </c>
       <c r="D89" t="n">
-        <v>4.69</v>
+        <v>4.81</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BATLIBOI</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>79.68000000000001</v>
+        <v>53.44</v>
       </c>
       <c r="C90" t="n">
-        <v>83.40000000000001</v>
+        <v>56</v>
       </c>
       <c r="D90" t="n">
-        <v>4.67</v>
+        <v>4.79</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>FCSSOFT</t>
+          <t>TARACHAND</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1.5</v>
+        <v>56.04</v>
       </c>
       <c r="C91" t="n">
-        <v>1.57</v>
+        <v>58.7</v>
       </c>
       <c r="D91" t="n">
-        <v>4.67</v>
+        <v>4.75</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>FINKURVE</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>201.58</v>
+        <v>59.77</v>
       </c>
       <c r="C92" t="n">
-        <v>211</v>
+        <v>62.6</v>
       </c>
       <c r="D92" t="n">
-        <v>4.67</v>
+        <v>4.73</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LASA</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>8.380000000000001</v>
+        <v>284.6</v>
       </c>
       <c r="C93" t="n">
-        <v>8.77</v>
+        <v>298</v>
       </c>
       <c r="D93" t="n">
-        <v>4.65</v>
+        <v>4.71</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>BBTCL</t>
+          <t>UTLSOLAR</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>208.13</v>
+        <v>319.95</v>
       </c>
       <c r="C94" t="n">
-        <v>217.8</v>
+        <v>335</v>
       </c>
       <c r="D94" t="n">
-        <v>4.65</v>
+        <v>4.7</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>DELTAMAGNT</t>
+          <t>SIGACHI</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>62.12</v>
+        <v>21.3</v>
       </c>
       <c r="C95" t="n">
-        <v>65</v>
+        <v>22.3</v>
       </c>
       <c r="D95" t="n">
-        <v>4.64</v>
+        <v>4.69</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>SCPL</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>13.37</v>
+        <v>425.05</v>
       </c>
       <c r="C96" t="n">
-        <v>13.99</v>
+        <v>445</v>
       </c>
       <c r="D96" t="n">
-        <v>4.64</v>
+        <v>4.69</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>IVALUE</t>
+          <t>SADBHIN</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>243.75</v>
+        <v>2.78</v>
       </c>
       <c r="C97" t="n">
-        <v>255</v>
+        <v>2.91</v>
       </c>
       <c r="D97" t="n">
-        <v>4.62</v>
+        <v>4.68</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>HBLENGINE</t>
+          <t>SAREGAMA</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>817.5</v>
+        <v>424.15</v>
       </c>
       <c r="C98" t="n">
-        <v>855</v>
+        <v>444</v>
       </c>
       <c r="D98" t="n">
-        <v>4.59</v>
+        <v>4.68</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>816.75</v>
+        <v>192.01</v>
       </c>
       <c r="C99" t="n">
-        <v>854</v>
+        <v>201</v>
       </c>
       <c r="D99" t="n">
-        <v>4.56</v>
+        <v>4.68</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>GUJRAFFIA</t>
+          <t>BAJAJHIND</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>45.63</v>
+        <v>18.38</v>
       </c>
       <c r="C100" t="n">
-        <v>47.7</v>
+        <v>19.23</v>
       </c>
       <c r="D100" t="n">
-        <v>4.54</v>
+        <v>4.62</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SVPGLOB</t>
+          <t>FEDDERSHOL</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>3.97</v>
+        <v>34.4</v>
       </c>
       <c r="C101" t="n">
-        <v>4.15</v>
+        <v>35.99</v>
       </c>
       <c r="D101" t="n">
-        <v>4.53</v>
+        <v>4.62</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>STEELXIND</t>
+          <t>BAFNAPH</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>11.96</v>
+        <v>131.9</v>
       </c>
       <c r="C102" t="n">
-        <v>12.5</v>
+        <v>138</v>
       </c>
       <c r="D102" t="n">
-        <v>4.52</v>
+        <v>4.62</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>GOLDSTAR</t>
+          <t>GLOBALE</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>7.75</v>
+        <v>13.05</v>
       </c>
       <c r="C103" t="n">
-        <v>8.1</v>
+        <v>13.65</v>
       </c>
       <c r="D103" t="n">
-        <v>4.52</v>
+        <v>4.6</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>MBLINFRA</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>3.99</v>
+        <v>26.29</v>
       </c>
       <c r="C104" t="n">
-        <v>4.17</v>
+        <v>27.5</v>
       </c>
       <c r="D104" t="n">
-        <v>4.51</v>
+        <v>4.6</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>GUJRAFFIA</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>31.58</v>
+        <v>43.9</v>
       </c>
       <c r="C105" t="n">
-        <v>33</v>
+        <v>45.9</v>
       </c>
       <c r="D105" t="n">
-        <v>4.5</v>
+        <v>4.56</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>SCPL</t>
+          <t>PDMJEPAPER</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>404.9</v>
+        <v>81.05</v>
       </c>
       <c r="C106" t="n">
-        <v>423</v>
+        <v>84.73999999999999</v>
       </c>
       <c r="D106" t="n">
-        <v>4.47</v>
+        <v>4.55</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>RADAAN</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>3.16</v>
+        <v>14.77</v>
       </c>
       <c r="C107" t="n">
-        <v>3.3</v>
+        <v>15.44</v>
       </c>
       <c r="D107" t="n">
-        <v>4.43</v>
+        <v>4.54</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ASHAPURMIN</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>654.05</v>
+        <v>3922.4</v>
       </c>
       <c r="C108" t="n">
-        <v>683</v>
+        <v>4100</v>
       </c>
       <c r="D108" t="n">
-        <v>4.43</v>
+        <v>4.53</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>AKG</t>
+          <t>CPEDU</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>11.18</v>
+        <v>183.74</v>
       </c>
       <c r="C109" t="n">
-        <v>11.67</v>
+        <v>192</v>
       </c>
       <c r="D109" t="n">
-        <v>4.38</v>
+        <v>4.5</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>KANANIIND</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.23</v>
+        <v>1.56</v>
       </c>
       <c r="C110" t="n">
-        <v>0.24</v>
+        <v>1.63</v>
       </c>
       <c r="D110" t="n">
-        <v>4.35</v>
+        <v>4.49</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>LANCORHOL</t>
+          <t>SHBAJRG</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>24.39</v>
+        <v>158.1</v>
       </c>
       <c r="C111" t="n">
-        <v>25.45</v>
+        <v>165.2</v>
       </c>
       <c r="D111" t="n">
-        <v>4.35</v>
+        <v>4.49</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CANARYS</t>
+          <t>GHCLTEXTIL</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>19.65</v>
+        <v>95.81</v>
       </c>
       <c r="C112" t="n">
-        <v>20.5</v>
+        <v>100.11</v>
       </c>
       <c r="D112" t="n">
-        <v>4.33</v>
+        <v>4.49</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>BSL</t>
+          <t>TREL</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>136.89</v>
+        <v>25.56</v>
       </c>
       <c r="C113" t="n">
-        <v>142.8</v>
+        <v>26.7</v>
       </c>
       <c r="D113" t="n">
-        <v>4.32</v>
+        <v>4.46</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>BAFNAPH</t>
+          <t>FCSSOFT</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>129.9</v>
+        <v>1.57</v>
       </c>
       <c r="C114" t="n">
-        <v>135.5</v>
+        <v>1.64</v>
       </c>
       <c r="D114" t="n">
-        <v>4.31</v>
+        <v>4.46</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SBGLP</t>
+          <t>SIGNPOST</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>26.27</v>
+        <v>296.55</v>
       </c>
       <c r="C115" t="n">
-        <v>27.4</v>
+        <v>309.75</v>
       </c>
       <c r="D115" t="n">
-        <v>4.3</v>
+        <v>4.45</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>THYROCARE</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.93</v>
+        <v>506.3</v>
       </c>
       <c r="C116" t="n">
-        <v>0.97</v>
+        <v>528.75</v>
       </c>
       <c r="D116" t="n">
-        <v>4.3</v>
+        <v>4.43</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>BLBLIMITED</t>
+          <t>ANONDITA</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>16.58</v>
+        <v>1061.95</v>
       </c>
       <c r="C117" t="n">
-        <v>17.29</v>
+        <v>1109</v>
       </c>
       <c r="D117" t="n">
-        <v>4.28</v>
+        <v>4.43</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>GMRAIRPORT</t>
+          <t>TOKYOPLAST</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>97.84</v>
+        <v>88.01000000000001</v>
       </c>
       <c r="C118" t="n">
-        <v>102</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="D118" t="n">
-        <v>4.25</v>
+        <v>4.42</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>KISSHT</t>
+          <t>BAIDFIN</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>261.98</v>
+        <v>10.33</v>
       </c>
       <c r="C119" t="n">
-        <v>273</v>
+        <v>10.78</v>
       </c>
       <c r="D119" t="n">
-        <v>4.21</v>
+        <v>4.36</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>BEEKAY</t>
+          <t>JAYAGROGN</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>416.55</v>
+        <v>224.47</v>
       </c>
       <c r="C120" t="n">
-        <v>434</v>
+        <v>234.25</v>
       </c>
       <c r="D120" t="n">
-        <v>4.19</v>
+        <v>4.36</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>20.12</v>
+        <v>0.23</v>
       </c>
       <c r="C121" t="n">
-        <v>20.96</v>
+        <v>0.24</v>
       </c>
       <c r="D121" t="n">
-        <v>4.17</v>
+        <v>4.35</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3105,13 +3105,13 @@
         </is>
       </c>
       <c r="B122" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="C122" t="n">
         <v>0.24</v>
       </c>
-      <c r="C122" t="n">
-        <v>0.25</v>
-      </c>
       <c r="D122" t="n">
-        <v>4.17</v>
+        <v>4.35</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IFBAGRO</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1050.55</v>
+        <v>13.82</v>
       </c>
       <c r="C123" t="n">
-        <v>1094</v>
+        <v>14.42</v>
       </c>
       <c r="D123" t="n">
-        <v>4.14</v>
+        <v>4.34</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>IDEAFORGE</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>845.3</v>
+        <v>27.95</v>
       </c>
       <c r="C124" t="n">
-        <v>880</v>
+        <v>29.16</v>
       </c>
       <c r="D124" t="n">
-        <v>4.11</v>
+        <v>4.33</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>RVTH</t>
+          <t>GOLDENTOBC</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>790.75</v>
+        <v>25.46</v>
       </c>
       <c r="C125" t="n">
-        <v>823</v>
+        <v>26.56</v>
       </c>
       <c r="D125" t="n">
-        <v>4.08</v>
+        <v>4.32</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>AARON</t>
+          <t>GOCOLORS</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>120.9</v>
+        <v>315.8</v>
       </c>
       <c r="C126" t="n">
-        <v>125.8</v>
+        <v>329.45</v>
       </c>
       <c r="D126" t="n">
-        <v>4.05</v>
+        <v>4.32</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>UNIVASTU</t>
+          <t>BI</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>75.87</v>
+        <v>62.2</v>
       </c>
       <c r="C127" t="n">
-        <v>78.90000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="D127" t="n">
-        <v>3.99</v>
+        <v>4.18</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>UMAEXPORTS</t>
+          <t>DIL</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>25.85</v>
+        <v>0.96</v>
       </c>
       <c r="C128" t="n">
-        <v>26.88</v>
+        <v>1</v>
       </c>
       <c r="D128" t="n">
-        <v>3.98</v>
+        <v>4.17</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>SUDEEPPHRM</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>11.06</v>
+        <v>742.15</v>
       </c>
       <c r="C129" t="n">
-        <v>11.49</v>
+        <v>772.85</v>
       </c>
       <c r="D129" t="n">
-        <v>3.89</v>
+        <v>4.14</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>VINYAS</t>
+          <t>SPECTSTM</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>1106.95</v>
+        <v>66.75</v>
       </c>
       <c r="C130" t="n">
-        <v>1149.95</v>
+        <v>69.5</v>
       </c>
       <c r="D130" t="n">
-        <v>3.88</v>
+        <v>4.12</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>CORDSCABLE</t>
+          <t>RRIL</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>243.58</v>
+        <v>19.96</v>
       </c>
       <c r="C131" t="n">
-        <v>253</v>
+        <v>20.78</v>
       </c>
       <c r="D131" t="n">
-        <v>3.87</v>
+        <v>4.11</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>TIJARIA</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>175.92</v>
+        <v>4.65</v>
       </c>
       <c r="C132" t="n">
-        <v>182.71</v>
+        <v>4.84</v>
       </c>
       <c r="D132" t="n">
-        <v>3.86</v>
+        <v>4.09</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>LINC</t>
+          <t>ANNAPURNA</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>98.13</v>
+        <v>139.2</v>
       </c>
       <c r="C133" t="n">
-        <v>101.9</v>
+        <v>144.85</v>
       </c>
       <c r="D133" t="n">
-        <v>3.84</v>
+        <v>4.06</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>TGL</t>
+          <t>GENCON</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>23.5</v>
+        <v>39.68</v>
       </c>
       <c r="C134" t="n">
-        <v>24.4</v>
+        <v>41.28</v>
       </c>
       <c r="D134" t="n">
-        <v>3.83</v>
+        <v>4.03</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ANMOL</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>11.56</v>
+        <v>6.49</v>
       </c>
       <c r="C135" t="n">
-        <v>12</v>
+        <v>6.75</v>
       </c>
       <c r="D135" t="n">
-        <v>3.81</v>
+        <v>4.01</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>CEREBRAINT</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>3.44</v>
+        <v>64.42</v>
       </c>
       <c r="C136" t="n">
-        <v>3.57</v>
+        <v>66.98</v>
       </c>
       <c r="D136" t="n">
-        <v>3.78</v>
+        <v>3.97</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>TAMBOLIIN</t>
+          <t>TRIDENT</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>173.47</v>
+        <v>24.04</v>
       </c>
       <c r="C137" t="n">
-        <v>180</v>
+        <v>24.98</v>
       </c>
       <c r="D137" t="n">
-        <v>3.76</v>
+        <v>3.91</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>APSISAERO</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>318.05</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="C138" t="n">
-        <v>330</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D138" t="n">
-        <v>3.76</v>
+        <v>3.9</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ASTRON</t>
+          <t>DENORA</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>4</v>
+        <v>710.35</v>
       </c>
       <c r="C139" t="n">
-        <v>4.15</v>
+        <v>738</v>
       </c>
       <c r="D139" t="n">
-        <v>3.75</v>
+        <v>3.89</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>TROM</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>54</v>
+        <v>54.37</v>
       </c>
       <c r="C140" t="n">
-        <v>56</v>
+        <v>56.48</v>
       </c>
       <c r="D140" t="n">
-        <v>3.7</v>
+        <v>3.88</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>6.78</v>
+        <v>1155.3</v>
       </c>
       <c r="C141" t="n">
-        <v>7.03</v>
+        <v>1200</v>
       </c>
       <c r="D141" t="n">
-        <v>3.69</v>
+        <v>3.87</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>RUBICON</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>75.04000000000001</v>
+        <v>1005.6</v>
       </c>
       <c r="C142" t="n">
-        <v>77.8</v>
+        <v>1044.3</v>
       </c>
       <c r="D142" t="n">
-        <v>3.68</v>
+        <v>3.85</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SREEL</t>
+          <t>AARVI</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>192.76</v>
+        <v>129.99</v>
       </c>
       <c r="C143" t="n">
-        <v>199.8</v>
+        <v>135</v>
       </c>
       <c r="D143" t="n">
-        <v>3.65</v>
+        <v>3.85</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SECURKLOUD</t>
+          <t>JETFREIGHT</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>20.5</v>
+        <v>22.91</v>
       </c>
       <c r="C144" t="n">
-        <v>21.24</v>
+        <v>23.79</v>
       </c>
       <c r="D144" t="n">
-        <v>3.61</v>
+        <v>3.84</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ARHAM</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>144.6</v>
+        <v>29.74</v>
       </c>
       <c r="C145" t="n">
-        <v>149.8</v>
+        <v>30.88</v>
       </c>
       <c r="D145" t="n">
-        <v>3.6</v>
+        <v>3.83</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>DEVX</t>
+          <t>ICIL</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>38.28</v>
+        <v>312.1</v>
       </c>
       <c r="C146" t="n">
-        <v>39.65</v>
+        <v>324</v>
       </c>
       <c r="D146" t="n">
-        <v>3.58</v>
+        <v>3.81</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>TNTELE</t>
+          <t>SKIPPER</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>9.24</v>
+        <v>549.35</v>
       </c>
       <c r="C147" t="n">
-        <v>9.57</v>
+        <v>570</v>
       </c>
       <c r="D147" t="n">
-        <v>3.57</v>
+        <v>3.76</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>3BBLACKBIO</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>1221.7</v>
+        <v>172.52</v>
       </c>
       <c r="C148" t="n">
-        <v>1265</v>
+        <v>179</v>
       </c>
       <c r="D148" t="n">
-        <v>3.54</v>
+        <v>3.76</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>BIOFILCHEM</t>
+          <t>LYKALABS</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>35.62</v>
+        <v>58.3</v>
       </c>
       <c r="C149" t="n">
-        <v>36.85</v>
+        <v>60.48</v>
       </c>
       <c r="D149" t="n">
-        <v>3.45</v>
+        <v>3.74</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CONSOFINVT</t>
+          <t>HEMIPROP</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>231.88</v>
+        <v>139.77</v>
       </c>
       <c r="C150" t="n">
-        <v>239.85</v>
+        <v>145</v>
       </c>
       <c r="D150" t="n">
-        <v>3.44</v>
+        <v>3.74</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>PRAENG</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>22.96</v>
+        <v>865.15</v>
       </c>
       <c r="C151" t="n">
-        <v>23.75</v>
+        <v>897.4</v>
       </c>
       <c r="D151" t="n">
-        <v>3.44</v>
+        <v>3.73</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>GALAPREC</t>
+          <t>DIGIDRIVE</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>944.35</v>
+        <v>19.04</v>
       </c>
       <c r="C152" t="n">
-        <v>976.6</v>
+        <v>19.74</v>
       </c>
       <c r="D152" t="n">
-        <v>3.42</v>
+        <v>3.68</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>TIMEX</t>
+          <t>ASHOKAMET</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>423.55</v>
+        <v>15.76</v>
       </c>
       <c r="C153" t="n">
-        <v>438</v>
+        <v>16.34</v>
       </c>
       <c r="D153" t="n">
-        <v>3.41</v>
+        <v>3.68</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>6.45</v>
+        <v>4.91</v>
       </c>
       <c r="C154" t="n">
-        <v>6.67</v>
+        <v>5.09</v>
       </c>
       <c r="D154" t="n">
-        <v>3.41</v>
+        <v>3.67</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>SPORTKING</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>22.69</v>
+        <v>170.43</v>
       </c>
       <c r="C155" t="n">
-        <v>23.45</v>
+        <v>176.65</v>
       </c>
       <c r="D155" t="n">
-        <v>3.35</v>
+        <v>3.65</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SUDEEPPHRM</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>674.7</v>
+        <v>23.63</v>
       </c>
       <c r="C156" t="n">
-        <v>697</v>
+        <v>24.49</v>
       </c>
       <c r="D156" t="n">
-        <v>3.31</v>
+        <v>3.64</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>PCJEWELLER</t>
+          <t>ZIMLAB</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>9.199999999999999</v>
+        <v>102.29</v>
       </c>
       <c r="C157" t="n">
-        <v>9.5</v>
+        <v>106</v>
       </c>
       <c r="D157" t="n">
-        <v>3.26</v>
+        <v>3.63</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>SANSTAR</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>115.24</v>
+        <v>83.38</v>
       </c>
       <c r="C158" t="n">
-        <v>119</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="D158" t="n">
-        <v>3.26</v>
+        <v>3.62</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>CGRAPHICS</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>148</v>
+        <v>197.75</v>
       </c>
       <c r="C159" t="n">
-        <v>152.8</v>
+        <v>204.9</v>
       </c>
       <c r="D159" t="n">
-        <v>3.24</v>
+        <v>3.62</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>VISHNU</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>93.29000000000001</v>
+        <v>579.1</v>
       </c>
       <c r="C160" t="n">
-        <v>96.31</v>
+        <v>600</v>
       </c>
       <c r="D160" t="n">
-        <v>3.24</v>
+        <v>3.61</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>SURYALA</t>
+          <t>EKC</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>466.8</v>
+        <v>117.75</v>
       </c>
       <c r="C161" t="n">
-        <v>481.9</v>
+        <v>122</v>
       </c>
       <c r="D161" t="n">
-        <v>3.23</v>
+        <v>3.61</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>ORIENTCER</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>42.14</v>
+        <v>82.27</v>
       </c>
       <c r="C162" t="n">
-        <v>43.5</v>
+        <v>85.22</v>
       </c>
       <c r="D162" t="n">
-        <v>3.23</v>
+        <v>3.59</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>RPPINFRA</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>75.05</v>
+        <v>25.08</v>
       </c>
       <c r="C163" t="n">
-        <v>77.44</v>
+        <v>25.98</v>
       </c>
       <c r="D163" t="n">
-        <v>3.18</v>
+        <v>3.59</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>SAHYADRI</t>
+          <t>PASUPTAC</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>279.6</v>
+        <v>59.85</v>
       </c>
       <c r="C164" t="n">
-        <v>288.45</v>
+        <v>61.99</v>
       </c>
       <c r="D164" t="n">
-        <v>3.17</v>
+        <v>3.58</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>DBOL</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>6.97</v>
+        <v>107.95</v>
       </c>
       <c r="C165" t="n">
-        <v>7.19</v>
+        <v>111.8</v>
       </c>
       <c r="D165" t="n">
-        <v>3.16</v>
+        <v>3.57</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>BTTL</t>
+          <t>OSWALSEEDS</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>34.42</v>
+        <v>11</v>
       </c>
       <c r="C166" t="n">
-        <v>35.5</v>
+        <v>11.39</v>
       </c>
       <c r="D166" t="n">
-        <v>3.14</v>
+        <v>3.55</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ECOLINE</t>
+          <t>BVCL</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>153.2</v>
+        <v>43.16</v>
       </c>
       <c r="C167" t="n">
-        <v>158</v>
+        <v>44.69</v>
       </c>
       <c r="D167" t="n">
-        <v>3.13</v>
+        <v>3.54</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>AURIGROW</t>
+          <t>NAHARINDUS</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0.32</v>
+        <v>113.48</v>
       </c>
       <c r="C168" t="n">
-        <v>0.33</v>
+        <v>117.5</v>
       </c>
       <c r="D168" t="n">
-        <v>3.13</v>
+        <v>3.54</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>SINCLAIR</t>
+          <t>NRL</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>74.08</v>
+        <v>66.66</v>
       </c>
       <c r="C169" t="n">
-        <v>76.40000000000001</v>
+        <v>69</v>
       </c>
       <c r="D169" t="n">
-        <v>3.13</v>
+        <v>3.51</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>RSDFIN</t>
+          <t>UNIVASTU</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>80.09999999999999</v>
+        <v>77</v>
       </c>
       <c r="C170" t="n">
-        <v>82.59999999999999</v>
+        <v>79.7</v>
       </c>
       <c r="D170" t="n">
-        <v>3.12</v>
+        <v>3.51</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>GRCL</t>
+          <t>FAZE3Q</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>533.05</v>
+        <v>545.8</v>
       </c>
       <c r="C171" t="n">
-        <v>549.7</v>
+        <v>564.9</v>
       </c>
       <c r="D171" t="n">
-        <v>3.12</v>
+        <v>3.5</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>COMPINFO</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>1.3</v>
+        <v>524.85</v>
       </c>
       <c r="C172" t="n">
-        <v>1.34</v>
+        <v>543.2</v>
       </c>
       <c r="D172" t="n">
-        <v>3.08</v>
+        <v>3.5</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>RKDL</t>
+          <t>SANATHAN</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>21.47</v>
+        <v>405.7</v>
       </c>
       <c r="C173" t="n">
-        <v>22.13</v>
+        <v>419.8</v>
       </c>
       <c r="D173" t="n">
-        <v>3.07</v>
+        <v>3.48</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>GOLDTECH</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>48.37</v>
+        <v>10.93</v>
       </c>
       <c r="C174" t="n">
-        <v>49.85</v>
+        <v>11.31</v>
       </c>
       <c r="D174" t="n">
-        <v>3.06</v>
+        <v>3.48</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ZODIACLOTH</t>
+          <t>DPWIRES</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>76.8</v>
+        <v>185.25</v>
       </c>
       <c r="C175" t="n">
-        <v>79.15000000000001</v>
+        <v>191.7</v>
       </c>
       <c r="D175" t="n">
-        <v>3.06</v>
+        <v>3.48</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>FALCONTECH</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>353.1</v>
+        <v>14.5</v>
       </c>
       <c r="C176" t="n">
-        <v>363.9</v>
+        <v>15</v>
       </c>
       <c r="D176" t="n">
-        <v>3.06</v>
+        <v>3.45</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>SASKEN</t>
+          <t>WELSPUNLIV</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>2161.9</v>
+        <v>137.97</v>
       </c>
       <c r="C177" t="n">
-        <v>2227.9</v>
+        <v>142.73</v>
       </c>
       <c r="D177" t="n">
-        <v>3.05</v>
+        <v>3.45</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>KRISHCA</t>
+          <t>DJML</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>181.5</v>
+        <v>105.18</v>
       </c>
       <c r="C178" t="n">
-        <v>187</v>
+        <v>108.8</v>
       </c>
       <c r="D178" t="n">
-        <v>3.03</v>
+        <v>3.44</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>ASAHIINDIA</t>
+          <t>INDOTHAI</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>918.55</v>
+        <v>227.1</v>
       </c>
       <c r="C179" t="n">
-        <v>946.25</v>
+        <v>234.88</v>
       </c>
       <c r="D179" t="n">
-        <v>3.02</v>
+        <v>3.43</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>MPHASIS</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>2232.9</v>
+        <v>367.45</v>
       </c>
       <c r="C180" t="n">
-        <v>2300</v>
+        <v>380</v>
       </c>
       <c r="D180" t="n">
-        <v>3.01</v>
+        <v>3.42</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>PML</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>563.15</v>
+        <v>40.81</v>
       </c>
       <c r="C181" t="n">
-        <v>580</v>
+        <v>42.2</v>
       </c>
       <c r="D181" t="n">
-        <v>2.99</v>
+        <v>3.41</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>BIRLAPREC</t>
+          <t>IRISDOREME</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>45.45</v>
+        <v>35.78</v>
       </c>
       <c r="C182" t="n">
-        <v>46.8</v>
+        <v>37</v>
       </c>
       <c r="D182" t="n">
-        <v>2.97</v>
+        <v>3.41</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>TERASOFT</t>
+          <t>HIMATSEIDE</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>375.7</v>
+        <v>77.38</v>
       </c>
       <c r="C183" t="n">
-        <v>386.8</v>
+        <v>80</v>
       </c>
       <c r="D183" t="n">
-        <v>2.95</v>
+        <v>3.39</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>0.34</v>
+        <v>168.31</v>
       </c>
       <c r="C184" t="n">
-        <v>0.35</v>
+        <v>174</v>
       </c>
       <c r="D184" t="n">
-        <v>2.94</v>
+        <v>3.38</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>466.7</v>
+        <v>6.82</v>
       </c>
       <c r="C185" t="n">
-        <v>480.4</v>
+        <v>7.05</v>
       </c>
       <c r="D185" t="n">
-        <v>2.94</v>
+        <v>3.37</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>BCONCEPTS</t>
+          <t>VISHWARAJ</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>199.15</v>
+        <v>5.68</v>
       </c>
       <c r="C186" t="n">
-        <v>204.99</v>
+        <v>5.87</v>
       </c>
       <c r="D186" t="n">
-        <v>2.93</v>
+        <v>3.35</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>GOKEX</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>10.92</v>
+        <v>691.8</v>
       </c>
       <c r="C187" t="n">
-        <v>11.24</v>
+        <v>715</v>
       </c>
       <c r="D187" t="n">
-        <v>2.93</v>
+        <v>3.35</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>MAFATIND</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>29.93</v>
+        <v>132.63</v>
       </c>
       <c r="C188" t="n">
-        <v>30.8</v>
+        <v>136.99</v>
       </c>
       <c r="D188" t="n">
-        <v>2.91</v>
+        <v>3.29</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>GOYALALUM</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>330.2</v>
+        <v>6.72</v>
       </c>
       <c r="C189" t="n">
-        <v>339.7</v>
+        <v>6.94</v>
       </c>
       <c r="D189" t="n">
-        <v>2.88</v>
+        <v>3.27</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>JNKINDIA</t>
+          <t>TARMAT</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>381.9</v>
+        <v>51.76</v>
       </c>
       <c r="C190" t="n">
-        <v>392.9</v>
+        <v>53.45</v>
       </c>
       <c r="D190" t="n">
-        <v>2.88</v>
+        <v>3.27</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>184.68</v>
+        <v>24.12</v>
       </c>
       <c r="C191" t="n">
-        <v>190</v>
+        <v>24.9</v>
       </c>
       <c r="D191" t="n">
-        <v>2.88</v>
+        <v>3.23</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>MARINE</t>
+          <t>ASIANENE</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>247.92</v>
+        <v>358.1</v>
       </c>
       <c r="C192" t="n">
-        <v>255</v>
+        <v>369.65</v>
       </c>
       <c r="D192" t="n">
-        <v>2.86</v>
+        <v>3.23</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>MANCREDIT</t>
+          <t>GLOSTERLTD</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>191.54</v>
+        <v>665.75</v>
       </c>
       <c r="C193" t="n">
-        <v>197</v>
+        <v>687</v>
       </c>
       <c r="D193" t="n">
-        <v>2.85</v>
+        <v>3.19</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>TARC</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>171.09</v>
+        <v>129.76</v>
       </c>
       <c r="C194" t="n">
-        <v>175.86</v>
+        <v>133.9</v>
       </c>
       <c r="D194" t="n">
-        <v>2.79</v>
+        <v>3.19</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>TRANSPEK</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>1069.6</v>
+        <v>23.13</v>
       </c>
       <c r="C195" t="n">
-        <v>1099</v>
+        <v>23.86</v>
       </c>
       <c r="D195" t="n">
-        <v>2.75</v>
+        <v>3.16</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>GFLLIMITED</t>
+          <t>AMBIKCO</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>47.69</v>
+        <v>1657.6</v>
       </c>
       <c r="C196" t="n">
-        <v>49</v>
+        <v>1710</v>
       </c>
       <c r="D196" t="n">
-        <v>2.75</v>
+        <v>3.16</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>NRL</t>
+          <t>TTKHLTCARE</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>63.16</v>
+        <v>891.85</v>
       </c>
       <c r="C197" t="n">
-        <v>64.90000000000001</v>
+        <v>920</v>
       </c>
       <c r="D197" t="n">
-        <v>2.75</v>
+        <v>3.16</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>FLYSBS</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>379.65</v>
+        <v>421.55</v>
       </c>
       <c r="C198" t="n">
-        <v>390</v>
+        <v>434.8</v>
       </c>
       <c r="D198" t="n">
-        <v>2.73</v>
+        <v>3.14</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>EMMBI</t>
+          <t>PCJEWELLER</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>84.20999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="C199" t="n">
-        <v>86.5</v>
+        <v>9.9</v>
       </c>
       <c r="D199" t="n">
-        <v>2.72</v>
+        <v>3.13</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>KAMATHOTEL</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>169.4</v>
+        <v>170.69</v>
       </c>
       <c r="C200" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D200" t="n">
-        <v>2.72</v>
+        <v>3.11</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>PIONEEREMB</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>918.5</v>
+        <v>26.11</v>
       </c>
       <c r="C201" t="n">
-        <v>943.3</v>
+        <v>26.92</v>
       </c>
       <c r="D201" t="n">
-        <v>2.7</v>
+        <v>3.1</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-02 08:16 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UHTL</t>
+          <t>COFFEEDAY</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68.25</v>
+        <v>38.25</v>
       </c>
       <c r="C2" t="n">
-        <v>81.90000000000001</v>
+        <v>41.7</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>9.02</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>SHIVATEX</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16.69</v>
+        <v>145.55</v>
       </c>
       <c r="C3" t="n">
-        <v>19.99</v>
+        <v>158.5</v>
       </c>
       <c r="D3" t="n">
-        <v>19.77</v>
+        <v>8.9</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>WOCKPHARMA</t>
+          <t>NITIRAJ</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2031.4</v>
+        <v>174.91</v>
       </c>
       <c r="C4" t="n">
-        <v>2377</v>
+        <v>189.97</v>
       </c>
       <c r="D4" t="n">
-        <v>17.01</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>ARIHANT</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.01</v>
+        <v>737.4</v>
       </c>
       <c r="C5" t="n">
-        <v>6.97</v>
+        <v>800</v>
       </c>
       <c r="D5" t="n">
-        <v>15.97</v>
+        <v>8.49</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IPHL</t>
+          <t>BALKRISHNA</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>61.25</v>
+        <v>18.23</v>
       </c>
       <c r="C6" t="n">
-        <v>69.8</v>
+        <v>19.7</v>
       </c>
       <c r="D6" t="n">
-        <v>13.96</v>
+        <v>8.06</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RILINFRA</t>
+          <t>MERCANTILE</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>35.4</v>
+        <v>25.49</v>
       </c>
       <c r="C7" t="n">
-        <v>40</v>
+        <v>27.49</v>
       </c>
       <c r="D7" t="n">
-        <v>12.99</v>
+        <v>7.85</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TOUCHWOOD</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>70.23999999999999</v>
+        <v>0.14</v>
       </c>
       <c r="C8" t="n">
-        <v>77.98999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="D8" t="n">
-        <v>11.03</v>
+        <v>7.14</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>PANSARI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>242.18</v>
+        <v>283.85</v>
       </c>
       <c r="C9" t="n">
-        <v>266.39</v>
+        <v>304</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>7.1</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>COFFEEDAY</t>
+          <t>GOLDTECH</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>34.78</v>
+        <v>43.26</v>
       </c>
       <c r="C10" t="n">
-        <v>38.25</v>
+        <v>45.8</v>
       </c>
       <c r="D10" t="n">
-        <v>9.98</v>
+        <v>5.87</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SHARDUL</t>
+          <t>TFL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>28.25</v>
+        <v>12.3</v>
       </c>
       <c r="C11" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="D11" t="n">
-        <v>9.73</v>
+        <v>5.69</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HARDWYN</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>25.16</v>
+        <v>159.02</v>
       </c>
       <c r="C12" t="n">
-        <v>27.48</v>
+        <v>168</v>
       </c>
       <c r="D12" t="n">
-        <v>9.220000000000001</v>
+        <v>5.65</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SOMATEX</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>106.84</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="C13" t="n">
-        <v>116.45</v>
+        <v>86.45</v>
       </c>
       <c r="D13" t="n">
-        <v>8.99</v>
+        <v>5.56</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TAALTECH</t>
+          <t>ORTEL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3558.9</v>
+        <v>1.6</v>
       </c>
       <c r="C14" t="n">
-        <v>3876.6</v>
+        <v>1.68</v>
       </c>
       <c r="D14" t="n">
-        <v>8.93</v>
+        <v>5</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DGCONTENT</t>
+          <t>PRIZOR</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>26.65</v>
+        <v>691.65</v>
       </c>
       <c r="C15" t="n">
-        <v>29</v>
+        <v>726.2</v>
       </c>
       <c r="D15" t="n">
-        <v>8.82</v>
+        <v>5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SAHANA</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>823.9</v>
+        <v>266.39</v>
       </c>
       <c r="C16" t="n">
-        <v>895</v>
+        <v>279.7</v>
       </c>
       <c r="D16" t="n">
-        <v>8.630000000000001</v>
+        <v>5</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DYNAMIC</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>143</v>
+        <v>30.89</v>
       </c>
       <c r="C17" t="n">
-        <v>154.95</v>
+        <v>32.43</v>
       </c>
       <c r="D17" t="n">
-        <v>8.359999999999999</v>
+        <v>4.99</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NSLNISP</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>44.62</v>
+        <v>562.95</v>
       </c>
       <c r="C18" t="n">
-        <v>48.3</v>
+        <v>591.05</v>
       </c>
       <c r="D18" t="n">
-        <v>8.25</v>
+        <v>4.99</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SVLL</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>615.3</v>
+        <v>22.08</v>
       </c>
       <c r="C19" t="n">
-        <v>666</v>
+        <v>23.18</v>
       </c>
       <c r="D19" t="n">
-        <v>8.24</v>
+        <v>4.98</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>25.02</v>
+        <v>1.01</v>
       </c>
       <c r="C20" t="n">
-        <v>26.99</v>
+        <v>1.06</v>
       </c>
       <c r="D20" t="n">
-        <v>7.87</v>
+        <v>4.95</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SAIPARENT</t>
+          <t>BOHRAIND</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>485.9</v>
+        <v>17</v>
       </c>
       <c r="C21" t="n">
-        <v>523.95</v>
+        <v>17.84</v>
       </c>
       <c r="D21" t="n">
-        <v>7.83</v>
+        <v>4.94</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MFML</t>
+          <t>BIRLACABLE</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>25.01</v>
+        <v>203.6</v>
       </c>
       <c r="C22" t="n">
-        <v>26.95</v>
+        <v>213.6</v>
       </c>
       <c r="D22" t="n">
-        <v>7.76</v>
+        <v>4.91</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RPPL</t>
+          <t>FCSSOFT</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>16.91</v>
+        <v>1.64</v>
       </c>
       <c r="C23" t="n">
-        <v>18.2</v>
+        <v>1.72</v>
       </c>
       <c r="D23" t="n">
-        <v>7.63</v>
+        <v>4.88</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MSTCLTD</t>
+          <t>SUNTECH</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>440.5</v>
+        <v>38.05</v>
       </c>
       <c r="C24" t="n">
-        <v>474</v>
+        <v>39.9</v>
       </c>
       <c r="D24" t="n">
-        <v>7.6</v>
+        <v>4.86</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>165.49</v>
+        <v>1344.1</v>
       </c>
       <c r="C25" t="n">
-        <v>177.99</v>
+        <v>1409</v>
       </c>
       <c r="D25" t="n">
-        <v>7.55</v>
+        <v>4.83</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VIGOR</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>65.40000000000001</v>
+        <v>2.08</v>
       </c>
       <c r="C26" t="n">
-        <v>70.2</v>
+        <v>2.18</v>
       </c>
       <c r="D26" t="n">
-        <v>7.34</v>
+        <v>4.81</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>MRIL</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15.3</v>
+        <v>41.85</v>
       </c>
       <c r="C27" t="n">
-        <v>16.4</v>
+        <v>43.85</v>
       </c>
       <c r="D27" t="n">
-        <v>7.19</v>
+        <v>4.78</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>10.02</v>
+        <v>181.14</v>
       </c>
       <c r="C28" t="n">
-        <v>10.74</v>
+        <v>189.8</v>
       </c>
       <c r="D28" t="n">
-        <v>7.19</v>
+        <v>4.78</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ARIHANT</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>893.85</v>
+        <v>788.4</v>
       </c>
       <c r="C29" t="n">
-        <v>957.95</v>
+        <v>826</v>
       </c>
       <c r="D29" t="n">
-        <v>7.17</v>
+        <v>4.77</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SUVEN</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>279.34</v>
+        <v>39.9</v>
       </c>
       <c r="C30" t="n">
-        <v>297.95</v>
+        <v>41.8</v>
       </c>
       <c r="D30" t="n">
-        <v>6.66</v>
+        <v>4.76</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>UFLEX</t>
+          <t>GUJRAFFIA</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>423.95</v>
+        <v>42.37</v>
       </c>
       <c r="C31" t="n">
-        <v>452.05</v>
+        <v>44.36</v>
       </c>
       <c r="D31" t="n">
-        <v>6.63</v>
+        <v>4.7</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BSL</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>131.41</v>
+        <v>2.35</v>
       </c>
       <c r="C32" t="n">
-        <v>139.98</v>
+        <v>2.46</v>
       </c>
       <c r="D32" t="n">
-        <v>6.52</v>
+        <v>4.68</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SURAJLTD</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>224.37</v>
+        <v>4.96</v>
       </c>
       <c r="C33" t="n">
-        <v>239</v>
+        <v>5.19</v>
       </c>
       <c r="D33" t="n">
-        <v>6.52</v>
+        <v>4.64</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OLECTRA</t>
+          <t>DEEDEV</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1180</v>
+        <v>623.05</v>
       </c>
       <c r="C34" t="n">
-        <v>1255</v>
+        <v>651.8</v>
       </c>
       <c r="D34" t="n">
-        <v>6.36</v>
+        <v>4.61</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BANARBEADS</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>107.39</v>
+        <v>1.98</v>
       </c>
       <c r="C35" t="n">
-        <v>113.88</v>
+        <v>2.07</v>
       </c>
       <c r="D35" t="n">
-        <v>6.04</v>
+        <v>4.55</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SHREERAMA</t>
+          <t>GENSOL</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>42.85</v>
+        <v>19.8</v>
       </c>
       <c r="C36" t="n">
-        <v>45.4</v>
+        <v>20.7</v>
       </c>
       <c r="D36" t="n">
-        <v>5.95</v>
+        <v>4.55</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>VASWANI</t>
+          <t>AMDIND</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>56.63</v>
+        <v>47.25</v>
       </c>
       <c r="C37" t="n">
-        <v>60</v>
+        <v>49.39</v>
       </c>
       <c r="D37" t="n">
-        <v>5.95</v>
+        <v>4.53</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CPPLUS</t>
+          <t>OILCOUNTUB</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2903.5</v>
+        <v>54.34</v>
       </c>
       <c r="C38" t="n">
-        <v>3074.7</v>
+        <v>56.79</v>
       </c>
       <c r="D38" t="n">
-        <v>5.9</v>
+        <v>4.51</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PTCIL</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>16191</v>
+        <v>20.02</v>
       </c>
       <c r="C39" t="n">
-        <v>17124</v>
+        <v>20.9</v>
       </c>
       <c r="D39" t="n">
-        <v>5.76</v>
+        <v>4.4</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1442.9</v>
+        <v>13.22</v>
       </c>
       <c r="C40" t="n">
-        <v>1525</v>
+        <v>13.8</v>
       </c>
       <c r="D40" t="n">
-        <v>5.69</v>
+        <v>4.39</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>JAIPURKURT</t>
+          <t>SUPREMEENG</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>32.13</v>
+        <v>0.92</v>
       </c>
       <c r="C41" t="n">
-        <v>33.95</v>
+        <v>0.96</v>
       </c>
       <c r="D41" t="n">
-        <v>5.66</v>
+        <v>4.35</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5PAISA</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>327.7</v>
+        <v>13.28</v>
       </c>
       <c r="C42" t="n">
-        <v>346</v>
+        <v>13.85</v>
       </c>
       <c r="D42" t="n">
-        <v>5.58</v>
+        <v>4.29</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OCCLLTD</t>
+          <t>BAFNAPH</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>114.73</v>
+        <v>138.49</v>
       </c>
       <c r="C43" t="n">
-        <v>121</v>
+        <v>144.3</v>
       </c>
       <c r="D43" t="n">
-        <v>5.47</v>
+        <v>4.2</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>METROGLOBL</t>
+          <t>BBTCL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>128.1</v>
+        <v>225.85</v>
       </c>
       <c r="C44" t="n">
-        <v>135</v>
+        <v>235.2</v>
       </c>
       <c r="D44" t="n">
-        <v>5.39</v>
+        <v>4.14</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BCONCEPTS</t>
+          <t>THEINVEST</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>196.42</v>
+        <v>98.93000000000001</v>
       </c>
       <c r="C45" t="n">
-        <v>207</v>
+        <v>103</v>
       </c>
       <c r="D45" t="n">
-        <v>5.39</v>
+        <v>4.11</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>RADAAN</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3.03</v>
+        <v>0.49</v>
       </c>
       <c r="C46" t="n">
-        <v>3.19</v>
+        <v>0.51</v>
       </c>
       <c r="D46" t="n">
-        <v>5.28</v>
+        <v>4.08</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>EUROBOND</t>
+          <t>INSPIRISYS</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>184.26</v>
+        <v>125.52</v>
       </c>
       <c r="C47" t="n">
-        <v>193.75</v>
+        <v>130.57</v>
       </c>
       <c r="D47" t="n">
-        <v>5.15</v>
+        <v>4.02</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>CTE</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>23.02</v>
+        <v>31.73</v>
       </c>
       <c r="C48" t="n">
-        <v>24.2</v>
+        <v>32.99</v>
       </c>
       <c r="D48" t="n">
-        <v>5.13</v>
+        <v>3.97</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>RAJPALAYAM</t>
+          <t>ANANTRAJ</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>804.6</v>
+        <v>538.65</v>
       </c>
       <c r="C49" t="n">
-        <v>845</v>
+        <v>560</v>
       </c>
       <c r="D49" t="n">
-        <v>5.02</v>
+        <v>3.96</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DECNGOLD</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>162.28</v>
+        <v>4118.5</v>
       </c>
       <c r="C50" t="n">
-        <v>170.42</v>
+        <v>4280</v>
       </c>
       <c r="D50" t="n">
-        <v>5.02</v>
+        <v>3.92</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>KANANIIND</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>536.15</v>
+        <v>1.54</v>
       </c>
       <c r="C51" t="n">
-        <v>562.95</v>
+        <v>1.6</v>
       </c>
       <c r="D51" t="n">
-        <v>5</v>
+        <v>3.9</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MASKINVEST</t>
+          <t>RUBICON</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>152.05</v>
+        <v>1171.1</v>
       </c>
       <c r="C52" t="n">
-        <v>159.65</v>
+        <v>1215</v>
       </c>
       <c r="D52" t="n">
-        <v>5</v>
+        <v>3.75</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SWANDEF</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2060.2</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C53" t="n">
-        <v>2163.2</v>
+        <v>0.84</v>
       </c>
       <c r="D53" t="n">
-        <v>5</v>
+        <v>3.7</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>JKIPL</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>89.64</v>
+        <v>298.8</v>
       </c>
       <c r="C54" t="n">
-        <v>94.12</v>
+        <v>309.8</v>
       </c>
       <c r="D54" t="n">
-        <v>5</v>
+        <v>3.68</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>DIVINEHIRA</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>193.91</v>
+        <v>324</v>
       </c>
       <c r="C55" t="n">
-        <v>203.6</v>
+        <v>335.9</v>
       </c>
       <c r="D55" t="n">
-        <v>5</v>
+        <v>3.67</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>HRHNEXT</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>27</v>
+        <v>355.2</v>
       </c>
       <c r="C56" t="n">
-        <v>28.35</v>
+        <v>368</v>
       </c>
       <c r="D56" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>POLYSIL</t>
+          <t>EQUIPPP</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>144.05</v>
+        <v>18.31</v>
       </c>
       <c r="C57" t="n">
-        <v>151.25</v>
+        <v>18.97</v>
       </c>
       <c r="D57" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PLAZACABLE</t>
+          <t>CEREBRAINT</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>46.81</v>
+        <v>3.33</v>
       </c>
       <c r="C58" t="n">
-        <v>49.15</v>
+        <v>3.45</v>
       </c>
       <c r="D58" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SOFTTECH</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>459.3</v>
+        <v>13.21</v>
       </c>
       <c r="C59" t="n">
-        <v>482.25</v>
+        <v>13.68</v>
       </c>
       <c r="D59" t="n">
-        <v>5</v>
+        <v>3.56</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BEDMUTHA</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>113.4</v>
+        <v>176.72</v>
       </c>
       <c r="C60" t="n">
-        <v>119.07</v>
+        <v>183</v>
       </c>
       <c r="D60" t="n">
-        <v>5</v>
+        <v>3.55</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1280.05</v>
+        <v>4.84</v>
       </c>
       <c r="C61" t="n">
-        <v>1344.1</v>
+        <v>5</v>
       </c>
       <c r="D61" t="n">
-        <v>5</v>
+        <v>3.31</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SAKUMA</t>
+          <t>RILINFRA</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2</v>
+        <v>38.05</v>
       </c>
       <c r="C62" t="n">
-        <v>2.1</v>
+        <v>39.3</v>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>3.29</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>TERASOFT</t>
+          <t>NDLVENTURE</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>394.45</v>
+        <v>130.72</v>
       </c>
       <c r="C63" t="n">
-        <v>414.15</v>
+        <v>135</v>
       </c>
       <c r="D63" t="n">
-        <v>4.99</v>
+        <v>3.27</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>IBULLSLTD</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>21.03</v>
+        <v>33.91</v>
       </c>
       <c r="C64" t="n">
-        <v>22.08</v>
+        <v>35</v>
       </c>
       <c r="D64" t="n">
-        <v>4.99</v>
+        <v>3.21</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>IZMO</t>
+          <t>KHANDSE</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>750.9</v>
+        <v>19.37</v>
       </c>
       <c r="C65" t="n">
-        <v>788.4</v>
+        <v>19.99</v>
       </c>
       <c r="D65" t="n">
-        <v>4.99</v>
+        <v>3.2</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>65.29000000000001</v>
+        <v>1.57</v>
       </c>
       <c r="C66" t="n">
-        <v>68.55</v>
+        <v>1.62</v>
       </c>
       <c r="D66" t="n">
-        <v>4.99</v>
+        <v>3.18</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>MSPL</t>
+          <t>PML</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>42.72</v>
+        <v>537</v>
       </c>
       <c r="C67" t="n">
-        <v>44.85</v>
+        <v>553.9</v>
       </c>
       <c r="D67" t="n">
-        <v>4.99</v>
+        <v>3.15</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PRIZOR</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>658.75</v>
+        <v>31.03</v>
       </c>
       <c r="C68" t="n">
-        <v>691.65</v>
+        <v>31.99</v>
       </c>
       <c r="D68" t="n">
-        <v>4.99</v>
+        <v>3.09</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>YAAP</t>
+          <t>JSLL</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>199.95</v>
+        <v>492.2</v>
       </c>
       <c r="C69" t="n">
-        <v>209.9</v>
+        <v>507.4</v>
       </c>
       <c r="D69" t="n">
-        <v>4.98</v>
+        <v>3.09</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>GENSOL</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>18.87</v>
+        <v>19.4</v>
       </c>
       <c r="C70" t="n">
-        <v>19.81</v>
+        <v>20</v>
       </c>
       <c r="D70" t="n">
-        <v>4.98</v>
+        <v>3.09</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SEMAC</t>
+          <t>WEWIN</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>303.95</v>
+        <v>56.75</v>
       </c>
       <c r="C71" t="n">
-        <v>319.1</v>
+        <v>58.5</v>
       </c>
       <c r="D71" t="n">
-        <v>4.98</v>
+        <v>3.08</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>VTL</t>
+          <t>SHBAJRG</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>577.15</v>
+        <v>171.21</v>
       </c>
       <c r="C72" t="n">
-        <v>605.9</v>
+        <v>176.45</v>
       </c>
       <c r="D72" t="n">
-        <v>4.98</v>
+        <v>3.06</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BILVYAPAR</t>
+          <t>OSWALSEEDS</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>4.62</v>
+        <v>11.14</v>
       </c>
       <c r="C73" t="n">
-        <v>4.85</v>
+        <v>11.48</v>
       </c>
       <c r="D73" t="n">
-        <v>4.98</v>
+        <v>3.05</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>EPWINDIA</t>
+          <t>HBSL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>129.9</v>
+        <v>54.23</v>
       </c>
       <c r="C74" t="n">
-        <v>136.35</v>
+        <v>55.88</v>
       </c>
       <c r="D74" t="n">
-        <v>4.97</v>
+        <v>3.04</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SADBHAV</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>9.65</v>
+        <v>14.94</v>
       </c>
       <c r="C75" t="n">
-        <v>10.13</v>
+        <v>15.38</v>
       </c>
       <c r="D75" t="n">
-        <v>4.97</v>
+        <v>2.95</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TROM</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>56.7</v>
+        <v>426.4</v>
       </c>
       <c r="C76" t="n">
-        <v>59.5</v>
+        <v>438.95</v>
       </c>
       <c r="D76" t="n">
-        <v>4.94</v>
+        <v>2.94</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>VIPCLOTHNG</t>
+          <t>SARVESHWAR</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>26.52</v>
+        <v>3.75</v>
       </c>
       <c r="C77" t="n">
-        <v>27.83</v>
+        <v>3.86</v>
       </c>
       <c r="D77" t="n">
-        <v>4.94</v>
+        <v>2.93</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FMNL</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>10.73</v>
+        <v>924.1</v>
       </c>
       <c r="C78" t="n">
-        <v>11.26</v>
+        <v>951</v>
       </c>
       <c r="D78" t="n">
-        <v>4.94</v>
+        <v>2.91</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>BALAXI</t>
+          <t>URAVIDEF</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>26.21</v>
+        <v>118.55</v>
       </c>
       <c r="C79" t="n">
-        <v>27.5</v>
+        <v>122</v>
       </c>
       <c r="D79" t="n">
-        <v>4.92</v>
+        <v>2.91</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>AVG</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>2.24</v>
+        <v>148.6</v>
       </c>
       <c r="C80" t="n">
-        <v>2.35</v>
+        <v>152.93</v>
       </c>
       <c r="D80" t="n">
-        <v>4.91</v>
+        <v>2.91</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SHRIKANHA</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>26.45</v>
+        <v>6.6</v>
       </c>
       <c r="C81" t="n">
-        <v>27.75</v>
+        <v>6.79</v>
       </c>
       <c r="D81" t="n">
-        <v>4.91</v>
+        <v>2.88</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MRIL</t>
+          <t>SYSTMTXC</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>39.9</v>
+        <v>64.16</v>
       </c>
       <c r="C82" t="n">
-        <v>41.85</v>
+        <v>66</v>
       </c>
       <c r="D82" t="n">
-        <v>4.89</v>
+        <v>2.87</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>VIPULLTD</t>
+          <t>AROGRANITE</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>8.81</v>
+        <v>25.47</v>
       </c>
       <c r="C83" t="n">
-        <v>9.24</v>
+        <v>26.19</v>
       </c>
       <c r="D83" t="n">
-        <v>4.88</v>
+        <v>2.83</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>JAIPURKURT</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>38</v>
+        <v>33.02</v>
       </c>
       <c r="C84" t="n">
-        <v>39.85</v>
+        <v>33.95</v>
       </c>
       <c r="D84" t="n">
-        <v>4.87</v>
+        <v>2.82</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>DCMFINSERV</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>5.98</v>
+        <v>17.51</v>
       </c>
       <c r="C85" t="n">
-        <v>6.27</v>
+        <v>18</v>
       </c>
       <c r="D85" t="n">
-        <v>4.85</v>
+        <v>2.8</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>TENNIND</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>4.74</v>
+        <v>557.1</v>
       </c>
       <c r="C86" t="n">
-        <v>4.97</v>
+        <v>572.7</v>
       </c>
       <c r="D86" t="n">
-        <v>4.85</v>
+        <v>2.8</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SURANI</t>
+          <t>BELLACASA</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>120.2</v>
+        <v>238.42</v>
       </c>
       <c r="C87" t="n">
-        <v>126</v>
+        <v>245</v>
       </c>
       <c r="D87" t="n">
-        <v>4.83</v>
+        <v>2.76</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>VINNY</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>52.85</v>
+        <v>1.09</v>
       </c>
       <c r="C88" t="n">
-        <v>55.4</v>
+        <v>1.12</v>
       </c>
       <c r="D88" t="n">
-        <v>4.82</v>
+        <v>2.75</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>BGLOBAL</t>
+          <t>DBSTOCKBRO</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>3.12</v>
+        <v>33.44</v>
       </c>
       <c r="C89" t="n">
-        <v>3.27</v>
+        <v>34.35</v>
       </c>
       <c r="D89" t="n">
-        <v>4.81</v>
+        <v>2.72</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>BSOFT</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>53.44</v>
+        <v>327.8</v>
       </c>
       <c r="C90" t="n">
-        <v>56</v>
+        <v>336.45</v>
       </c>
       <c r="D90" t="n">
-        <v>4.79</v>
+        <v>2.64</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TARACHAND</t>
+          <t>SILLYMONKS</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>56.04</v>
+        <v>16.42</v>
       </c>
       <c r="C91" t="n">
-        <v>58.7</v>
+        <v>16.85</v>
       </c>
       <c r="D91" t="n">
-        <v>4.75</v>
+        <v>2.62</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>FINKURVE</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>59.77</v>
+        <v>10.3</v>
       </c>
       <c r="C92" t="n">
-        <v>62.6</v>
+        <v>10.57</v>
       </c>
       <c r="D92" t="n">
-        <v>4.73</v>
+        <v>2.62</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>HDIL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>284.6</v>
+        <v>1.92</v>
       </c>
       <c r="C93" t="n">
-        <v>298</v>
+        <v>1.97</v>
       </c>
       <c r="D93" t="n">
-        <v>4.71</v>
+        <v>2.6</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>UTLSOLAR</t>
+          <t>HALEOSLABS</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>319.95</v>
+        <v>1423.3</v>
       </c>
       <c r="C94" t="n">
-        <v>335</v>
+        <v>1459.9</v>
       </c>
       <c r="D94" t="n">
-        <v>4.7</v>
+        <v>2.57</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SIGACHI</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>21.3</v>
+        <v>1.95</v>
       </c>
       <c r="C95" t="n">
-        <v>22.3</v>
+        <v>2</v>
       </c>
       <c r="D95" t="n">
-        <v>4.69</v>
+        <v>2.56</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SCPL</t>
+          <t>UNITEDTEA</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>425.05</v>
+        <v>510.1</v>
       </c>
       <c r="C96" t="n">
-        <v>445</v>
+        <v>523.1</v>
       </c>
       <c r="D96" t="n">
-        <v>4.69</v>
+        <v>2.55</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SADBHIN</t>
+          <t>ATLANTAELE</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>2.78</v>
+        <v>1983.6</v>
       </c>
       <c r="C97" t="n">
-        <v>2.91</v>
+        <v>2034</v>
       </c>
       <c r="D97" t="n">
-        <v>4.68</v>
+        <v>2.54</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SAREGAMA</t>
+          <t>NILAINFRA</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>424.15</v>
+        <v>7.9</v>
       </c>
       <c r="C98" t="n">
-        <v>444</v>
+        <v>8.1</v>
       </c>
       <c r="D98" t="n">
-        <v>4.68</v>
+        <v>2.53</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SREEL</t>
+          <t>SJLOGISTIC</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>192.01</v>
+        <v>326.7</v>
       </c>
       <c r="C99" t="n">
-        <v>201</v>
+        <v>334.85</v>
       </c>
       <c r="D99" t="n">
-        <v>4.68</v>
+        <v>2.49</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>BAJAJHIND</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>18.38</v>
+        <v>1202.5</v>
       </c>
       <c r="C100" t="n">
-        <v>19.23</v>
+        <v>1232.5</v>
       </c>
       <c r="D100" t="n">
-        <v>4.62</v>
+        <v>2.49</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FEDDERSHOL</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>34.4</v>
+        <v>40.64</v>
       </c>
       <c r="C101" t="n">
-        <v>35.99</v>
+        <v>41.65</v>
       </c>
       <c r="D101" t="n">
-        <v>4.62</v>
+        <v>2.49</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>BAFNAPH</t>
+          <t>BANSALWIRE</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>131.9</v>
+        <v>308.4</v>
       </c>
       <c r="C102" t="n">
-        <v>138</v>
+        <v>316</v>
       </c>
       <c r="D102" t="n">
-        <v>4.62</v>
+        <v>2.46</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>GLOBALE</t>
+          <t>INDOUS</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>13.05</v>
+        <v>99.76000000000001</v>
       </c>
       <c r="C103" t="n">
-        <v>13.65</v>
+        <v>102.2</v>
       </c>
       <c r="D103" t="n">
-        <v>4.6</v>
+        <v>2.45</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>MBLINFRA</t>
+          <t>HEXATRADEX</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>26.29</v>
+        <v>161.88</v>
       </c>
       <c r="C104" t="n">
-        <v>27.5</v>
+        <v>165.85</v>
       </c>
       <c r="D104" t="n">
-        <v>4.6</v>
+        <v>2.45</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>GUJRAFFIA</t>
+          <t>KRITIKA</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>43.9</v>
+        <v>6.11</v>
       </c>
       <c r="C105" t="n">
-        <v>45.9</v>
+        <v>6.26</v>
       </c>
       <c r="D105" t="n">
-        <v>4.56</v>
+        <v>2.45</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PDMJEPAPER</t>
+          <t>BI</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>81.05</v>
+        <v>64.41</v>
       </c>
       <c r="C106" t="n">
-        <v>84.73999999999999</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="D106" t="n">
-        <v>4.55</v>
+        <v>2.45</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>TREJHARA</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>14.77</v>
+        <v>143.7</v>
       </c>
       <c r="C107" t="n">
-        <v>15.44</v>
+        <v>147.2</v>
       </c>
       <c r="D107" t="n">
-        <v>4.54</v>
+        <v>2.44</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>ASPINWALL</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>3922.4</v>
+        <v>239.88</v>
       </c>
       <c r="C108" t="n">
-        <v>4100</v>
+        <v>245.7</v>
       </c>
       <c r="D108" t="n">
-        <v>4.53</v>
+        <v>2.43</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>CPEDU</t>
+          <t>INDIQUBE</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>183.74</v>
+        <v>156.4</v>
       </c>
       <c r="C109" t="n">
-        <v>192</v>
+        <v>160.18</v>
       </c>
       <c r="D109" t="n">
-        <v>4.5</v>
+        <v>2.42</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>KANANIIND</t>
+          <t>A2ZINFRA</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>1.56</v>
+        <v>14.15</v>
       </c>
       <c r="C110" t="n">
-        <v>1.63</v>
+        <v>14.49</v>
       </c>
       <c r="D110" t="n">
-        <v>4.49</v>
+        <v>2.4</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SHBAJRG</t>
+          <t>TTKHLTCARE</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>158.1</v>
+        <v>916.1</v>
       </c>
       <c r="C111" t="n">
-        <v>165.2</v>
+        <v>938</v>
       </c>
       <c r="D111" t="n">
-        <v>4.49</v>
+        <v>2.39</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>GHCLTEXTIL</t>
+          <t>DAVANGERE</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>95.81</v>
+        <v>3.81</v>
       </c>
       <c r="C112" t="n">
-        <v>100.11</v>
+        <v>3.9</v>
       </c>
       <c r="D112" t="n">
-        <v>4.49</v>
+        <v>2.36</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>TREL</t>
+          <t>GENUSPAPER</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>25.56</v>
+        <v>12.36</v>
       </c>
       <c r="C113" t="n">
-        <v>26.7</v>
+        <v>12.65</v>
       </c>
       <c r="D113" t="n">
-        <v>4.46</v>
+        <v>2.35</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>FCSSOFT</t>
+          <t>PIONEEREMB</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>1.57</v>
+        <v>24.36</v>
       </c>
       <c r="C114" t="n">
-        <v>1.64</v>
+        <v>24.93</v>
       </c>
       <c r="D114" t="n">
-        <v>4.46</v>
+        <v>2.34</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SIGNPOST</t>
+          <t>BEARDSELL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>296.55</v>
+        <v>29.27</v>
       </c>
       <c r="C115" t="n">
-        <v>309.75</v>
+        <v>29.95</v>
       </c>
       <c r="D115" t="n">
-        <v>4.45</v>
+        <v>2.32</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>THYROCARE</t>
+          <t>CRIZAC</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>506.3</v>
+        <v>215.98</v>
       </c>
       <c r="C116" t="n">
-        <v>528.75</v>
+        <v>220.99</v>
       </c>
       <c r="D116" t="n">
-        <v>4.43</v>
+        <v>2.32</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ANONDITA</t>
+          <t>HCL-INSYS</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>1061.95</v>
+        <v>12.12</v>
       </c>
       <c r="C117" t="n">
-        <v>1109</v>
+        <v>12.4</v>
       </c>
       <c r="D117" t="n">
-        <v>4.43</v>
+        <v>2.31</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>TOKYOPLAST</t>
+          <t>GOACARBON</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>88.01000000000001</v>
+        <v>390.85</v>
       </c>
       <c r="C118" t="n">
-        <v>91.90000000000001</v>
+        <v>399.8</v>
       </c>
       <c r="D118" t="n">
-        <v>4.42</v>
+        <v>2.29</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>BAIDFIN</t>
+          <t>LINCOLN</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>10.33</v>
+        <v>606.2</v>
       </c>
       <c r="C119" t="n">
-        <v>10.78</v>
+        <v>620</v>
       </c>
       <c r="D119" t="n">
-        <v>4.36</v>
+        <v>2.28</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>JAYAGROGN</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>224.47</v>
+        <v>6.64</v>
       </c>
       <c r="C120" t="n">
-        <v>234.25</v>
+        <v>6.79</v>
       </c>
       <c r="D120" t="n">
-        <v>4.36</v>
+        <v>2.26</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.23</v>
+        <v>44.4</v>
       </c>
       <c r="C121" t="n">
-        <v>0.24</v>
+        <v>45.4</v>
       </c>
       <c r="D121" t="n">
-        <v>4.35</v>
+        <v>2.25</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.23</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="C122" t="n">
-        <v>0.24</v>
+        <v>8.65</v>
       </c>
       <c r="D122" t="n">
-        <v>4.35</v>
+        <v>2.25</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>MANYAVAR</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>13.82</v>
+        <v>399.05</v>
       </c>
       <c r="C123" t="n">
-        <v>14.42</v>
+        <v>408</v>
       </c>
       <c r="D123" t="n">
-        <v>4.34</v>
+        <v>2.24</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>COMPUSOFT</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>27.95</v>
+        <v>13.55</v>
       </c>
       <c r="C124" t="n">
-        <v>29.16</v>
+        <v>13.85</v>
       </c>
       <c r="D124" t="n">
-        <v>4.33</v>
+        <v>2.21</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>GOLDENTOBC</t>
+          <t>LAGNAM</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>25.46</v>
+        <v>84.04000000000001</v>
       </c>
       <c r="C125" t="n">
-        <v>26.56</v>
+        <v>85.89</v>
       </c>
       <c r="D125" t="n">
-        <v>4.32</v>
+        <v>2.2</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>GOCOLORS</t>
+          <t>FLFL</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>315.8</v>
+        <v>1.4</v>
       </c>
       <c r="C126" t="n">
-        <v>329.45</v>
+        <v>1.43</v>
       </c>
       <c r="D126" t="n">
-        <v>4.32</v>
+        <v>2.14</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>BI</t>
+          <t>GLOBE</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>62.2</v>
+        <v>2.34</v>
       </c>
       <c r="C127" t="n">
-        <v>64.8</v>
+        <v>2.39</v>
       </c>
       <c r="D127" t="n">
-        <v>4.18</v>
+        <v>2.14</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>DIL</t>
+          <t>ATLANTAA</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.96</v>
+        <v>41.12</v>
       </c>
       <c r="C128" t="n">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="D128" t="n">
-        <v>4.17</v>
+        <v>2.14</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SUDEEPPHRM</t>
+          <t>SHRADHA</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>742.15</v>
+        <v>34.27</v>
       </c>
       <c r="C129" t="n">
-        <v>772.85</v>
+        <v>35</v>
       </c>
       <c r="D129" t="n">
-        <v>4.14</v>
+        <v>2.13</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>SPECTSTM</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>66.75</v>
+        <v>24.09</v>
       </c>
       <c r="C130" t="n">
-        <v>69.5</v>
+        <v>24.6</v>
       </c>
       <c r="D130" t="n">
-        <v>4.12</v>
+        <v>2.12</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>RRIL</t>
+          <t>TREL</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>19.96</v>
+        <v>25.66</v>
       </c>
       <c r="C131" t="n">
-        <v>20.78</v>
+        <v>26.2</v>
       </c>
       <c r="D131" t="n">
-        <v>4.11</v>
+        <v>2.1</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>TIJARIA</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>4.65</v>
+        <v>4.81</v>
       </c>
       <c r="C132" t="n">
-        <v>4.84</v>
+        <v>4.91</v>
       </c>
       <c r="D132" t="n">
-        <v>4.09</v>
+        <v>2.08</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ANNAPURNA</t>
+          <t>TIJARIA</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>139.2</v>
+        <v>4.35</v>
       </c>
       <c r="C133" t="n">
-        <v>144.85</v>
+        <v>4.44</v>
       </c>
       <c r="D133" t="n">
-        <v>4.06</v>
+        <v>2.07</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>GENCON</t>
+          <t>LOKESHMACH</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>39.68</v>
+        <v>249.8</v>
       </c>
       <c r="C134" t="n">
-        <v>41.28</v>
+        <v>254.95</v>
       </c>
       <c r="D134" t="n">
-        <v>4.03</v>
+        <v>2.06</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>RELIABLE</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>6.49</v>
+        <v>137.13</v>
       </c>
       <c r="C135" t="n">
-        <v>6.75</v>
+        <v>139.9</v>
       </c>
       <c r="D135" t="n">
-        <v>4.01</v>
+        <v>2.02</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>KALPATARU</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>64.42</v>
+        <v>323.4</v>
       </c>
       <c r="C136" t="n">
-        <v>66.98</v>
+        <v>329.9</v>
       </c>
       <c r="D136" t="n">
-        <v>3.97</v>
+        <v>2.01</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>TRIDENT</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>24.04</v>
+        <v>11.51</v>
       </c>
       <c r="C137" t="n">
-        <v>24.98</v>
+        <v>11.74</v>
       </c>
       <c r="D137" t="n">
-        <v>3.91</v>
+        <v>2</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>MITTAL</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>8.470000000000001</v>
+        <v>1</v>
       </c>
       <c r="C138" t="n">
-        <v>8.800000000000001</v>
+        <v>1.02</v>
       </c>
       <c r="D138" t="n">
-        <v>3.9</v>
+        <v>2</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>DENORA</t>
+          <t>DJML</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>710.35</v>
+        <v>104.85</v>
       </c>
       <c r="C139" t="n">
-        <v>738</v>
+        <v>106.95</v>
       </c>
       <c r="D139" t="n">
-        <v>3.89</v>
+        <v>2</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>AAREYDRUGS</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>54.37</v>
+        <v>77.37</v>
       </c>
       <c r="C140" t="n">
-        <v>56.48</v>
+        <v>78.92</v>
       </c>
       <c r="D140" t="n">
-        <v>3.88</v>
+        <v>2</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>1155.3</v>
+        <v>0.5</v>
       </c>
       <c r="C141" t="n">
-        <v>1200</v>
+        <v>0.51</v>
       </c>
       <c r="D141" t="n">
-        <v>3.87</v>
+        <v>2</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>RUBICON</t>
+          <t>NORBTEAEXP</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>1005.6</v>
+        <v>81.44</v>
       </c>
       <c r="C142" t="n">
-        <v>1044.3</v>
+        <v>83.06999999999999</v>
       </c>
       <c r="D142" t="n">
-        <v>3.85</v>
+        <v>2</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>AARVI</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>129.99</v>
+        <v>3.52</v>
       </c>
       <c r="C143" t="n">
-        <v>135</v>
+        <v>3.59</v>
       </c>
       <c r="D143" t="n">
-        <v>3.85</v>
+        <v>1.99</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>JETFREIGHT</t>
+          <t>AIRAN</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>22.91</v>
+        <v>16.64</v>
       </c>
       <c r="C144" t="n">
-        <v>23.79</v>
+        <v>16.97</v>
       </c>
       <c r="D144" t="n">
-        <v>3.84</v>
+        <v>1.98</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>IMPAL</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>29.74</v>
+        <v>1057.1</v>
       </c>
       <c r="C145" t="n">
-        <v>30.88</v>
+        <v>1078</v>
       </c>
       <c r="D145" t="n">
-        <v>3.83</v>
+        <v>1.98</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ICIL</t>
+          <t>RANASUG</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>312.1</v>
+        <v>12.12</v>
       </c>
       <c r="C146" t="n">
-        <v>324</v>
+        <v>12.36</v>
       </c>
       <c r="D146" t="n">
-        <v>3.81</v>
+        <v>1.98</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SKIPPER</t>
+          <t>RRIL</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>549.35</v>
+        <v>20.16</v>
       </c>
       <c r="C147" t="n">
-        <v>570</v>
+        <v>20.56</v>
       </c>
       <c r="D147" t="n">
-        <v>3.76</v>
+        <v>1.98</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>BLBLIMITED</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>172.52</v>
+        <v>17.05</v>
       </c>
       <c r="C148" t="n">
-        <v>179</v>
+        <v>17.38</v>
       </c>
       <c r="D148" t="n">
-        <v>3.76</v>
+        <v>1.94</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>LYKALABS</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>58.3</v>
+        <v>202.97</v>
       </c>
       <c r="C149" t="n">
-        <v>60.48</v>
+        <v>206.9</v>
       </c>
       <c r="D149" t="n">
-        <v>3.74</v>
+        <v>1.94</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>HEMIPROP</t>
+          <t>HLVLTD</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>139.77</v>
+        <v>7.84</v>
       </c>
       <c r="C150" t="n">
-        <v>145</v>
+        <v>7.99</v>
       </c>
       <c r="D150" t="n">
-        <v>3.74</v>
+        <v>1.91</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>MAHEPC</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>865.15</v>
+        <v>114.75</v>
       </c>
       <c r="C151" t="n">
-        <v>897.4</v>
+        <v>116.93</v>
       </c>
       <c r="D151" t="n">
-        <v>3.73</v>
+        <v>1.9</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>DIGIDRIVE</t>
+          <t>SONAMLTD</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>19.04</v>
+        <v>57.71</v>
       </c>
       <c r="C152" t="n">
-        <v>19.74</v>
+        <v>58.8</v>
       </c>
       <c r="D152" t="n">
-        <v>3.68</v>
+        <v>1.89</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ASHOKAMET</t>
+          <t>PNCINFRA</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>15.76</v>
+        <v>207.07</v>
       </c>
       <c r="C153" t="n">
-        <v>16.34</v>
+        <v>210.95</v>
       </c>
       <c r="D153" t="n">
-        <v>3.68</v>
+        <v>1.87</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>COUNCODOS</t>
+          <t>LATENTVIEW</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>4.91</v>
+        <v>316.4</v>
       </c>
       <c r="C154" t="n">
-        <v>5.09</v>
+        <v>322.3</v>
       </c>
       <c r="D154" t="n">
-        <v>3.67</v>
+        <v>1.86</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>SPORTKING</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>170.43</v>
+        <v>3.23</v>
       </c>
       <c r="C155" t="n">
-        <v>176.65</v>
+        <v>3.29</v>
       </c>
       <c r="D155" t="n">
-        <v>3.65</v>
+        <v>1.86</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>SUVIDHAA</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>23.63</v>
+        <v>2.7</v>
       </c>
       <c r="C156" t="n">
-        <v>24.49</v>
+        <v>2.75</v>
       </c>
       <c r="D156" t="n">
-        <v>3.64</v>
+        <v>1.85</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>ZIMLAB</t>
+          <t>UFLEX</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>102.29</v>
+        <v>440.65</v>
       </c>
       <c r="C157" t="n">
-        <v>106</v>
+        <v>448.8</v>
       </c>
       <c r="D157" t="n">
-        <v>3.63</v>
+        <v>1.85</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>RAMANEWS</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>83.38</v>
+        <v>29.21</v>
       </c>
       <c r="C158" t="n">
-        <v>86.40000000000001</v>
+        <v>29.75</v>
       </c>
       <c r="D158" t="n">
-        <v>3.62</v>
+        <v>1.85</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>197.75</v>
+        <v>0.55</v>
       </c>
       <c r="C159" t="n">
-        <v>204.9</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D159" t="n">
-        <v>3.62</v>
+        <v>1.82</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>VISHNU</t>
+          <t>ROSSELLIND</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>579.1</v>
+        <v>55.98</v>
       </c>
       <c r="C160" t="n">
-        <v>600</v>
+        <v>57</v>
       </c>
       <c r="D160" t="n">
-        <v>3.61</v>
+        <v>1.82</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>EKC</t>
+          <t>RVTH</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>117.75</v>
+        <v>740.5</v>
       </c>
       <c r="C161" t="n">
-        <v>122</v>
+        <v>754</v>
       </c>
       <c r="D161" t="n">
-        <v>3.61</v>
+        <v>1.82</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>KNAGRI</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>82.27</v>
+        <v>185.04</v>
       </c>
       <c r="C162" t="n">
-        <v>85.22</v>
+        <v>188.4</v>
       </c>
       <c r="D162" t="n">
-        <v>3.59</v>
+        <v>1.82</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>VASWANI</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>25.08</v>
+        <v>55.89</v>
       </c>
       <c r="C163" t="n">
-        <v>25.98</v>
+        <v>56.9</v>
       </c>
       <c r="D163" t="n">
-        <v>3.59</v>
+        <v>1.81</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>PASUPTAC</t>
+          <t>BAGFILMS</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>59.85</v>
+        <v>4.98</v>
       </c>
       <c r="C164" t="n">
-        <v>61.99</v>
+        <v>5.07</v>
       </c>
       <c r="D164" t="n">
-        <v>3.58</v>
+        <v>1.81</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>DBOL</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>107.95</v>
+        <v>6.09</v>
       </c>
       <c r="C165" t="n">
-        <v>111.8</v>
+        <v>6.2</v>
       </c>
       <c r="D165" t="n">
-        <v>3.57</v>
+        <v>1.81</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>NIITLTD</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>11</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="C166" t="n">
-        <v>11.39</v>
+        <v>83</v>
       </c>
       <c r="D166" t="n">
-        <v>3.55</v>
+        <v>1.79</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>BVCL</t>
+          <t>VIVIDHA</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>43.16</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="C167" t="n">
-        <v>44.69</v>
+        <v>0.57</v>
       </c>
       <c r="D167" t="n">
-        <v>3.54</v>
+        <v>1.79</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>NAHARINDUS</t>
+          <t>VASCONEQ</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>113.48</v>
+        <v>32.66</v>
       </c>
       <c r="C168" t="n">
-        <v>117.5</v>
+        <v>33.24</v>
       </c>
       <c r="D168" t="n">
-        <v>3.54</v>
+        <v>1.78</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>NRL</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>66.66</v>
+        <v>1.14</v>
       </c>
       <c r="C169" t="n">
-        <v>69</v>
+        <v>1.16</v>
       </c>
       <c r="D169" t="n">
-        <v>3.51</v>
+        <v>1.75</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>UNIVASTU</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>77</v>
+        <v>139.27</v>
       </c>
       <c r="C170" t="n">
-        <v>79.7</v>
+        <v>141.7</v>
       </c>
       <c r="D170" t="n">
-        <v>3.51</v>
+        <v>1.74</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>FAZE3Q</t>
+          <t>PIGL</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>545.8</v>
+        <v>90.18000000000001</v>
       </c>
       <c r="C171" t="n">
-        <v>564.9</v>
+        <v>91.75</v>
       </c>
       <c r="D171" t="n">
-        <v>3.5</v>
+        <v>1.74</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>SIKKO</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>524.85</v>
+        <v>4.06</v>
       </c>
       <c r="C172" t="n">
-        <v>543.2</v>
+        <v>4.13</v>
       </c>
       <c r="D172" t="n">
-        <v>3.5</v>
+        <v>1.72</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SANATHAN</t>
+          <t>KCPSUGIND</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>405.7</v>
+        <v>25.06</v>
       </c>
       <c r="C173" t="n">
-        <v>419.8</v>
+        <v>25.49</v>
       </c>
       <c r="D173" t="n">
-        <v>3.48</v>
+        <v>1.72</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>BLUECHIP</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>10.93</v>
+        <v>2.33</v>
       </c>
       <c r="C174" t="n">
-        <v>11.31</v>
+        <v>2.37</v>
       </c>
       <c r="D174" t="n">
-        <v>3.48</v>
+        <v>1.72</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>DPWIRES</t>
+          <t>BLACKROSE</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>185.25</v>
+        <v>94.2</v>
       </c>
       <c r="C175" t="n">
-        <v>191.7</v>
+        <v>95.8</v>
       </c>
       <c r="D175" t="n">
-        <v>3.48</v>
+        <v>1.7</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>FALCONTECH</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>14.5</v>
+        <v>370.45</v>
       </c>
       <c r="C176" t="n">
-        <v>15</v>
+        <v>376.7</v>
       </c>
       <c r="D176" t="n">
-        <v>3.45</v>
+        <v>1.69</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>WELSPUNLIV</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>137.97</v>
+        <v>13.73</v>
       </c>
       <c r="C177" t="n">
-        <v>142.73</v>
+        <v>13.96</v>
       </c>
       <c r="D177" t="n">
-        <v>3.45</v>
+        <v>1.68</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>DJML</t>
+          <t>WANBURY</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>105.18</v>
+        <v>266.55</v>
       </c>
       <c r="C178" t="n">
-        <v>108.8</v>
+        <v>271</v>
       </c>
       <c r="D178" t="n">
-        <v>3.44</v>
+        <v>1.67</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>INDOTHAI</t>
+          <t>MASFIN</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>227.1</v>
+        <v>304.5</v>
       </c>
       <c r="C179" t="n">
-        <v>234.88</v>
+        <v>309.5</v>
       </c>
       <c r="D179" t="n">
-        <v>3.43</v>
+        <v>1.64</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>KHADIM</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>367.45</v>
+        <v>99.86</v>
       </c>
       <c r="C180" t="n">
-        <v>380</v>
+        <v>101.5</v>
       </c>
       <c r="D180" t="n">
-        <v>3.42</v>
+        <v>1.64</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>40.81</v>
+        <v>55</v>
       </c>
       <c r="C181" t="n">
-        <v>42.2</v>
+        <v>55.9</v>
       </c>
       <c r="D181" t="n">
-        <v>3.41</v>
+        <v>1.64</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>IRISDOREME</t>
+          <t>WINSOME</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>35.78</v>
+        <v>2.45</v>
       </c>
       <c r="C182" t="n">
-        <v>37</v>
+        <v>2.49</v>
       </c>
       <c r="D182" t="n">
-        <v>3.41</v>
+        <v>1.63</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>HIMATSEIDE</t>
+          <t>SHIVALIK</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>77.38</v>
+        <v>271.3</v>
       </c>
       <c r="C183" t="n">
-        <v>80</v>
+        <v>275.7</v>
       </c>
       <c r="D183" t="n">
-        <v>3.39</v>
+        <v>1.62</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>168.31</v>
+        <v>82.66</v>
       </c>
       <c r="C184" t="n">
-        <v>174</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="D184" t="n">
-        <v>3.38</v>
+        <v>1.61</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>LPDC</t>
+          <t>SNOWMAN</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>6.82</v>
+        <v>36.81</v>
       </c>
       <c r="C185" t="n">
-        <v>7.05</v>
+        <v>37.4</v>
       </c>
       <c r="D185" t="n">
-        <v>3.37</v>
+        <v>1.6</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>VISHWARAJ</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>5.68</v>
+        <v>835.7</v>
       </c>
       <c r="C186" t="n">
-        <v>5.87</v>
+        <v>848.95</v>
       </c>
       <c r="D186" t="n">
-        <v>3.35</v>
+        <v>1.59</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>GOKEX</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>691.8</v>
+        <v>30.02</v>
       </c>
       <c r="C187" t="n">
-        <v>715</v>
+        <v>30.49</v>
       </c>
       <c r="D187" t="n">
-        <v>3.35</v>
+        <v>1.57</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>MAFATIND</t>
+          <t>SAKHTISUG</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>132.63</v>
+        <v>17.87</v>
       </c>
       <c r="C188" t="n">
-        <v>136.99</v>
+        <v>18.15</v>
       </c>
       <c r="D188" t="n">
-        <v>3.29</v>
+        <v>1.57</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>GOYALALUM</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>6.72</v>
+        <v>41.83</v>
       </c>
       <c r="C189" t="n">
-        <v>6.94</v>
+        <v>42.48</v>
       </c>
       <c r="D189" t="n">
-        <v>3.27</v>
+        <v>1.55</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>TARMAT</t>
+          <t>MHLXMIRU</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>51.76</v>
+        <v>179.25</v>
       </c>
       <c r="C190" t="n">
-        <v>53.45</v>
+        <v>182.01</v>
       </c>
       <c r="D190" t="n">
-        <v>3.27</v>
+        <v>1.54</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>TIRUPATIFL</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>24.12</v>
+        <v>45.11</v>
       </c>
       <c r="C191" t="n">
-        <v>24.9</v>
+        <v>45.8</v>
       </c>
       <c r="D191" t="n">
-        <v>3.23</v>
+        <v>1.53</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>ASIANENE</t>
+          <t>HMT</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>358.1</v>
+        <v>55.15</v>
       </c>
       <c r="C192" t="n">
-        <v>369.65</v>
+        <v>55.99</v>
       </c>
       <c r="D192" t="n">
-        <v>3.23</v>
+        <v>1.52</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>GLOSTERLTD</t>
+          <t>SIGNPOST</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>665.75</v>
+        <v>273</v>
       </c>
       <c r="C193" t="n">
-        <v>687</v>
+        <v>277.1</v>
       </c>
       <c r="D193" t="n">
-        <v>3.19</v>
+        <v>1.5</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>TARC</t>
+          <t>KENNAMET</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>129.76</v>
+        <v>2863.2</v>
       </c>
       <c r="C194" t="n">
-        <v>133.9</v>
+        <v>2906.1</v>
       </c>
       <c r="D194" t="n">
-        <v>3.19</v>
+        <v>1.5</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>23.13</v>
+        <v>59.25</v>
       </c>
       <c r="C195" t="n">
-        <v>23.86</v>
+        <v>60.13</v>
       </c>
       <c r="D195" t="n">
-        <v>3.16</v>
+        <v>1.49</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>AMBIKCO</t>
+          <t>PRITIKA</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>1657.6</v>
+        <v>63.95</v>
       </c>
       <c r="C196" t="n">
-        <v>1710</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="D196" t="n">
-        <v>3.16</v>
+        <v>1.49</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>TTKHLTCARE</t>
+          <t>ADVANCE</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>891.85</v>
+        <v>102.47</v>
       </c>
       <c r="C197" t="n">
-        <v>920</v>
+        <v>104</v>
       </c>
       <c r="D197" t="n">
-        <v>3.16</v>
+        <v>1.49</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>FLYSBS</t>
+          <t>CLEANMAX</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>421.55</v>
+        <v>1090.4</v>
       </c>
       <c r="C198" t="n">
-        <v>434.8</v>
+        <v>1106.6</v>
       </c>
       <c r="D198" t="n">
-        <v>3.14</v>
+        <v>1.49</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>PCJEWELLER</t>
+          <t>MALLCOM</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>9.6</v>
+        <v>959.8</v>
       </c>
       <c r="C199" t="n">
-        <v>9.9</v>
+        <v>974</v>
       </c>
       <c r="D199" t="n">
-        <v>3.13</v>
+        <v>1.48</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>RUCHIRA</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>170.69</v>
+        <v>115.09</v>
       </c>
       <c r="C200" t="n">
-        <v>176</v>
+        <v>116.79</v>
       </c>
       <c r="D200" t="n">
-        <v>3.11</v>
+        <v>1.48</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>PIONEEREMB</t>
+          <t>ESTER</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>26.11</v>
+        <v>92.64</v>
       </c>
       <c r="C201" t="n">
-        <v>26.92</v>
+        <v>94</v>
       </c>
       <c r="D201" t="n">
-        <v>3.1</v>
+        <v>1.47</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-03 08:36 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>COFFEEDAY</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>38.25</v>
+        <v>24.02</v>
       </c>
       <c r="C2" t="n">
-        <v>41.7</v>
+        <v>27.03</v>
       </c>
       <c r="D2" t="n">
-        <v>9.02</v>
+        <v>12.53</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SHIVATEX</t>
+          <t>SHRIKRISH</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>145.55</v>
+        <v>40.55</v>
       </c>
       <c r="C3" t="n">
-        <v>158.5</v>
+        <v>44.5</v>
       </c>
       <c r="D3" t="n">
-        <v>8.9</v>
+        <v>9.74</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NITIRAJ</t>
+          <t>ORIENTLTD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>174.91</v>
+        <v>61.48</v>
       </c>
       <c r="C4" t="n">
-        <v>189.97</v>
+        <v>66.8</v>
       </c>
       <c r="D4" t="n">
-        <v>8.609999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ARIHANT</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>737.4</v>
+        <v>5.37</v>
       </c>
       <c r="C5" t="n">
-        <v>800</v>
+        <v>5.81</v>
       </c>
       <c r="D5" t="n">
-        <v>8.49</v>
+        <v>8.19</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BALKRISHNA</t>
+          <t>COCKERILL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18.23</v>
+        <v>7593.5</v>
       </c>
       <c r="C6" t="n">
-        <v>19.7</v>
+        <v>8200</v>
       </c>
       <c r="D6" t="n">
-        <v>8.06</v>
+        <v>7.99</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MERCANTILE</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>25.49</v>
+        <v>0.15</v>
       </c>
       <c r="C7" t="n">
-        <v>27.49</v>
+        <v>0.16</v>
       </c>
       <c r="D7" t="n">
-        <v>7.85</v>
+        <v>6.67</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>HALDER</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.14</v>
+        <v>228.79</v>
       </c>
       <c r="C8" t="n">
-        <v>0.15</v>
+        <v>244</v>
       </c>
       <c r="D8" t="n">
-        <v>7.14</v>
+        <v>6.65</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PANSARI</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>283.85</v>
+        <v>14.38</v>
       </c>
       <c r="C9" t="n">
-        <v>304</v>
+        <v>15.3</v>
       </c>
       <c r="D9" t="n">
-        <v>7.1</v>
+        <v>6.4</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GOLDTECH</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>43.26</v>
+        <v>34.78</v>
       </c>
       <c r="C10" t="n">
-        <v>45.8</v>
+        <v>37</v>
       </c>
       <c r="D10" t="n">
-        <v>5.87</v>
+        <v>6.38</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TFL</t>
+          <t>TUNWAL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12.3</v>
+        <v>29.55</v>
       </c>
       <c r="C11" t="n">
-        <v>13</v>
+        <v>31.4</v>
       </c>
       <c r="D11" t="n">
-        <v>5.69</v>
+        <v>6.26</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>PIONRINV</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>159.02</v>
+        <v>106.38</v>
       </c>
       <c r="C12" t="n">
-        <v>168</v>
+        <v>112.98</v>
       </c>
       <c r="D12" t="n">
-        <v>5.65</v>
+        <v>6.2</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>UHTL</t>
+          <t>MUKTAARTS</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>81.90000000000001</v>
+        <v>64.06</v>
       </c>
       <c r="C13" t="n">
-        <v>86.45</v>
+        <v>67.8</v>
       </c>
       <c r="D13" t="n">
-        <v>5.56</v>
+        <v>5.84</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ORTEL</t>
+          <t>RULKA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.6</v>
+        <v>91.7</v>
       </c>
       <c r="C14" t="n">
-        <v>1.68</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>5.67</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PRIZOR</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>691.65</v>
+        <v>90.05</v>
       </c>
       <c r="C15" t="n">
-        <v>726.2</v>
+        <v>95</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>CONCORDBIO</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>266.39</v>
+        <v>1166.2</v>
       </c>
       <c r="C16" t="n">
-        <v>279.7</v>
+        <v>1230</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>5.47</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>IWP</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>30.89</v>
+        <v>34.44</v>
       </c>
       <c r="C17" t="n">
-        <v>32.43</v>
+        <v>36.24</v>
       </c>
       <c r="D17" t="n">
-        <v>4.99</v>
+        <v>5.23</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>PRIZOR</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>562.95</v>
+        <v>726.2</v>
       </c>
       <c r="C18" t="n">
-        <v>591.05</v>
+        <v>762.5</v>
       </c>
       <c r="D18" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IBULLSLTD</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>22.08</v>
+        <v>1104.6</v>
       </c>
       <c r="C19" t="n">
-        <v>23.18</v>
+        <v>1159.8</v>
       </c>
       <c r="D19" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.01</v>
+        <v>827.8</v>
       </c>
       <c r="C20" t="n">
-        <v>1.06</v>
+        <v>869.15</v>
       </c>
       <c r="D20" t="n">
-        <v>4.95</v>
+        <v>5</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BOHRAIND</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>17</v>
+        <v>1411.3</v>
       </c>
       <c r="C21" t="n">
-        <v>17.84</v>
+        <v>1481.8</v>
       </c>
       <c r="D21" t="n">
-        <v>4.94</v>
+        <v>5</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>BAFNAPH</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>203.6</v>
+        <v>145.41</v>
       </c>
       <c r="C22" t="n">
-        <v>213.6</v>
+        <v>152.68</v>
       </c>
       <c r="D22" t="n">
-        <v>4.91</v>
+        <v>5</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FCSSOFT</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.64</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>1.72</v>
+        <v>2.1</v>
       </c>
       <c r="D23" t="n">
-        <v>4.88</v>
+        <v>5</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SUNTECH</t>
+          <t>MASKINVEST</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>38.05</v>
+        <v>150.49</v>
       </c>
       <c r="C24" t="n">
-        <v>39.9</v>
+        <v>158.01</v>
       </c>
       <c r="D24" t="n">
-        <v>4.86</v>
+        <v>5</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>RELINFRA</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1344.1</v>
+        <v>70.64</v>
       </c>
       <c r="C25" t="n">
-        <v>1409</v>
+        <v>74.17</v>
       </c>
       <c r="D25" t="n">
-        <v>4.83</v>
+        <v>5</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2.08</v>
+        <v>279.7</v>
       </c>
       <c r="C26" t="n">
-        <v>2.18</v>
+        <v>293.68</v>
       </c>
       <c r="D26" t="n">
-        <v>4.81</v>
+        <v>5</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MRIL</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>41.85</v>
+        <v>313.7</v>
       </c>
       <c r="C27" t="n">
-        <v>43.85</v>
+        <v>329.35</v>
       </c>
       <c r="D27" t="n">
-        <v>4.78</v>
+        <v>4.99</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>AHLWEST</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>181.14</v>
+        <v>579.85</v>
       </c>
       <c r="C28" t="n">
-        <v>189.8</v>
+        <v>608.8</v>
       </c>
       <c r="D28" t="n">
-        <v>4.78</v>
+        <v>4.99</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IZMO</t>
+          <t>UTLSOLAR</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>788.4</v>
+        <v>319.8</v>
       </c>
       <c r="C29" t="n">
-        <v>826</v>
+        <v>335.75</v>
       </c>
       <c r="D29" t="n">
-        <v>4.77</v>
+        <v>4.99</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>SUPREMEPWR</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>39.9</v>
+        <v>246.25</v>
       </c>
       <c r="C30" t="n">
-        <v>41.8</v>
+        <v>258.55</v>
       </c>
       <c r="D30" t="n">
-        <v>4.76</v>
+        <v>4.99</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GUJRAFFIA</t>
+          <t>MCON</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>42.37</v>
+        <v>43.2</v>
       </c>
       <c r="C31" t="n">
-        <v>44.36</v>
+        <v>45.35</v>
       </c>
       <c r="D31" t="n">
-        <v>4.7</v>
+        <v>4.98</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2.35</v>
+        <v>129.8</v>
       </c>
       <c r="C32" t="n">
-        <v>2.46</v>
+        <v>136.25</v>
       </c>
       <c r="D32" t="n">
-        <v>4.68</v>
+        <v>4.97</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>USASEEDS</t>
         </is>
       </c>
       <c r="B33" t="n">
+        <v>99.75</v>
+      </c>
+      <c r="C33" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="D33" t="n">
         <v>4.96</v>
-      </c>
-      <c r="C33" t="n">
-        <v>5.19</v>
-      </c>
-      <c r="D33" t="n">
-        <v>4.64</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DEEDEV</t>
+          <t>GENSOL</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>623.05</v>
+        <v>20.79</v>
       </c>
       <c r="C34" t="n">
-        <v>651.8</v>
+        <v>21.82</v>
       </c>
       <c r="D34" t="n">
-        <v>4.61</v>
+        <v>4.95</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1.98</v>
+        <v>27.53</v>
       </c>
       <c r="C35" t="n">
-        <v>2.07</v>
+        <v>28.89</v>
       </c>
       <c r="D35" t="n">
-        <v>4.55</v>
+        <v>4.94</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GENSOL</t>
+          <t>VLINFRA</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>19.8</v>
+        <v>30.35</v>
       </c>
       <c r="C36" t="n">
-        <v>20.7</v>
+        <v>31.85</v>
       </c>
       <c r="D36" t="n">
-        <v>4.55</v>
+        <v>4.94</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AMDIND</t>
+          <t>SABEVENTS</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>47.25</v>
+        <v>8.74</v>
       </c>
       <c r="C37" t="n">
-        <v>49.39</v>
+        <v>9.17</v>
       </c>
       <c r="D37" t="n">
-        <v>4.53</v>
+        <v>4.92</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OILCOUNTUB</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>54.34</v>
+        <v>41.85</v>
       </c>
       <c r="C38" t="n">
-        <v>56.79</v>
+        <v>43.9</v>
       </c>
       <c r="D38" t="n">
-        <v>4.51</v>
+        <v>4.9</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>UNIVCABLES</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>20.02</v>
+        <v>1239.2</v>
       </c>
       <c r="C39" t="n">
-        <v>20.9</v>
+        <v>1299.9</v>
       </c>
       <c r="D39" t="n">
-        <v>4.4</v>
+        <v>4.9</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>VIJAYPD</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>13.22</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="C40" t="n">
-        <v>13.8</v>
+        <v>94.3</v>
       </c>
       <c r="D40" t="n">
-        <v>4.39</v>
+        <v>4.89</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SUPREMEENG</t>
+          <t>DYNAMIC</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.92</v>
+        <v>154.45</v>
       </c>
       <c r="C41" t="n">
-        <v>0.96</v>
+        <v>161.95</v>
       </c>
       <c r="D41" t="n">
-        <v>4.35</v>
+        <v>4.86</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>ORTINGLOBE</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>13.28</v>
+        <v>15.74</v>
       </c>
       <c r="C42" t="n">
-        <v>13.85</v>
+        <v>16.5</v>
       </c>
       <c r="D42" t="n">
-        <v>4.29</v>
+        <v>4.83</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BAFNAPH</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>138.49</v>
+        <v>3.95</v>
       </c>
       <c r="C43" t="n">
-        <v>144.3</v>
+        <v>4.14</v>
       </c>
       <c r="D43" t="n">
-        <v>4.2</v>
+        <v>4.81</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BBTCL</t>
+          <t>SYSTMTXC</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>225.85</v>
+        <v>64.73999999999999</v>
       </c>
       <c r="C44" t="n">
-        <v>235.2</v>
+        <v>67.8</v>
       </c>
       <c r="D44" t="n">
-        <v>4.14</v>
+        <v>4.73</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>THEINVEST</t>
+          <t>GLOSTERLTD</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>98.93000000000001</v>
+        <v>657.95</v>
       </c>
       <c r="C45" t="n">
-        <v>103</v>
+        <v>689</v>
       </c>
       <c r="D45" t="n">
-        <v>4.11</v>
+        <v>4.72</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.49</v>
+        <v>1.06</v>
       </c>
       <c r="C46" t="n">
-        <v>0.51</v>
+        <v>1.11</v>
       </c>
       <c r="D46" t="n">
-        <v>4.08</v>
+        <v>4.72</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>INSPIRISYS</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>125.52</v>
+        <v>5.56</v>
       </c>
       <c r="C47" t="n">
-        <v>130.57</v>
+        <v>5.82</v>
       </c>
       <c r="D47" t="n">
-        <v>4.02</v>
+        <v>4.68</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CTE</t>
+          <t>URAVIDEF</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>31.73</v>
+        <v>116.61</v>
       </c>
       <c r="C48" t="n">
-        <v>32.99</v>
+        <v>122</v>
       </c>
       <c r="D48" t="n">
-        <v>3.97</v>
+        <v>4.62</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ANANTRAJ</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>538.65</v>
+        <v>5.19</v>
       </c>
       <c r="C49" t="n">
-        <v>560</v>
+        <v>5.43</v>
       </c>
       <c r="D49" t="n">
-        <v>3.96</v>
+        <v>4.62</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4118.5</v>
+        <v>3.51</v>
       </c>
       <c r="C50" t="n">
-        <v>4280</v>
+        <v>3.67</v>
       </c>
       <c r="D50" t="n">
-        <v>3.92</v>
+        <v>4.56</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>KANANIIND</t>
+          <t>ATCENERGY</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1.54</v>
+        <v>24.15</v>
       </c>
       <c r="C51" t="n">
-        <v>1.6</v>
+        <v>25.25</v>
       </c>
       <c r="D51" t="n">
-        <v>3.9</v>
+        <v>4.55</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>RUBICON</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1171.1</v>
+        <v>13.49</v>
       </c>
       <c r="C52" t="n">
-        <v>1215</v>
+        <v>14.1</v>
       </c>
       <c r="D52" t="n">
-        <v>3.75</v>
+        <v>4.52</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>NHPC</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.8100000000000001</v>
+        <v>72.29000000000001</v>
       </c>
       <c r="C53" t="n">
-        <v>0.84</v>
+        <v>75.56</v>
       </c>
       <c r="D53" t="n">
-        <v>3.7</v>
+        <v>4.52</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>SHRIKANHA</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>298.8</v>
+        <v>29.1</v>
       </c>
       <c r="C54" t="n">
-        <v>309.8</v>
+        <v>30.4</v>
       </c>
       <c r="D54" t="n">
-        <v>3.68</v>
+        <v>4.47</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DIVINEHIRA</t>
+          <t>RFBL</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>324</v>
+        <v>63.2</v>
       </c>
       <c r="C55" t="n">
-        <v>335.9</v>
+        <v>66</v>
       </c>
       <c r="D55" t="n">
-        <v>3.67</v>
+        <v>4.43</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>XELPMOC</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>355.2</v>
+        <v>94.79000000000001</v>
       </c>
       <c r="C56" t="n">
-        <v>368</v>
+        <v>98.97</v>
       </c>
       <c r="D56" t="n">
-        <v>3.6</v>
+        <v>4.41</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>EQUIPPP</t>
+          <t>NBIFIN</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>18.31</v>
+        <v>1868.6</v>
       </c>
       <c r="C57" t="n">
-        <v>18.97</v>
+        <v>1950</v>
       </c>
       <c r="D57" t="n">
-        <v>3.6</v>
+        <v>4.36</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CEREBRAINT</t>
+          <t>MBLINFRA</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>3.33</v>
+        <v>28.66</v>
       </c>
       <c r="C58" t="n">
-        <v>3.45</v>
+        <v>29.9</v>
       </c>
       <c r="D58" t="n">
-        <v>3.6</v>
+        <v>4.33</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>THACKER</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>13.21</v>
+        <v>1435.2</v>
       </c>
       <c r="C59" t="n">
-        <v>13.68</v>
+        <v>1497</v>
       </c>
       <c r="D59" t="n">
-        <v>3.56</v>
+        <v>4.31</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>176.72</v>
+        <v>6.98</v>
       </c>
       <c r="C60" t="n">
-        <v>183</v>
+        <v>7.28</v>
       </c>
       <c r="D60" t="n">
-        <v>3.55</v>
+        <v>4.3</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>SONAMLTD</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4.84</v>
+        <v>57.08</v>
       </c>
       <c r="C61" t="n">
-        <v>5</v>
+        <v>59.5</v>
       </c>
       <c r="D61" t="n">
-        <v>3.31</v>
+        <v>4.24</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>RILINFRA</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>38.05</v>
+        <v>0.48</v>
       </c>
       <c r="C62" t="n">
-        <v>39.3</v>
+        <v>0.5</v>
       </c>
       <c r="D62" t="n">
-        <v>3.29</v>
+        <v>4.17</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>NDLVENTURE</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>130.72</v>
+        <v>0.24</v>
       </c>
       <c r="C63" t="n">
-        <v>135</v>
+        <v>0.25</v>
       </c>
       <c r="D63" t="n">
-        <v>3.27</v>
+        <v>4.17</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>FCSSOFT</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>33.91</v>
+        <v>1.72</v>
       </c>
       <c r="C64" t="n">
-        <v>35</v>
+        <v>1.79</v>
       </c>
       <c r="D64" t="n">
-        <v>3.21</v>
+        <v>4.07</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>19.37</v>
+        <v>6.92</v>
       </c>
       <c r="C65" t="n">
-        <v>19.99</v>
+        <v>7.2</v>
       </c>
       <c r="D65" t="n">
-        <v>3.2</v>
+        <v>4.05</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1.57</v>
+        <v>5.01</v>
       </c>
       <c r="C66" t="n">
-        <v>1.62</v>
+        <v>5.21</v>
       </c>
       <c r="D66" t="n">
-        <v>3.18</v>
+        <v>3.99</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>PML</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>537</v>
+        <v>7.31</v>
       </c>
       <c r="C67" t="n">
-        <v>553.9</v>
+        <v>7.6</v>
       </c>
       <c r="D67" t="n">
-        <v>3.15</v>
+        <v>3.97</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>MAGNUM</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>31.03</v>
+        <v>20.15</v>
       </c>
       <c r="C68" t="n">
-        <v>31.99</v>
+        <v>20.95</v>
       </c>
       <c r="D68" t="n">
-        <v>3.09</v>
+        <v>3.97</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>JSLL</t>
+          <t>RELCHEMQ</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>492.2</v>
+        <v>121.11</v>
       </c>
       <c r="C69" t="n">
-        <v>507.4</v>
+        <v>125.9</v>
       </c>
       <c r="D69" t="n">
-        <v>3.09</v>
+        <v>3.96</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>LASA</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>19.4</v>
+        <v>7.68</v>
       </c>
       <c r="C70" t="n">
-        <v>20</v>
+        <v>7.98</v>
       </c>
       <c r="D70" t="n">
-        <v>3.09</v>
+        <v>3.91</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>WEWIN</t>
+          <t>AYMSYNTEX</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>56.75</v>
+        <v>223.99</v>
       </c>
       <c r="C71" t="n">
-        <v>58.5</v>
+        <v>232.7</v>
       </c>
       <c r="D71" t="n">
-        <v>3.08</v>
+        <v>3.89</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SHBAJRG</t>
+          <t>BTTL</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>171.21</v>
+        <v>37.36</v>
       </c>
       <c r="C72" t="n">
-        <v>176.45</v>
+        <v>38.8</v>
       </c>
       <c r="D72" t="n">
-        <v>3.06</v>
+        <v>3.85</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>AAKASH</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>11.14</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="C73" t="n">
-        <v>11.48</v>
+        <v>9.74</v>
       </c>
       <c r="D73" t="n">
-        <v>3.05</v>
+        <v>3.84</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>HBSL</t>
+          <t>UMAEXPORTS</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>54.23</v>
+        <v>25.19</v>
       </c>
       <c r="C74" t="n">
-        <v>55.88</v>
+        <v>26.15</v>
       </c>
       <c r="D74" t="n">
-        <v>3.04</v>
+        <v>3.81</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>DRCSYSTEMS</t>
+          <t>PRIMECAB</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>14.94</v>
+        <v>107.9</v>
       </c>
       <c r="C75" t="n">
-        <v>15.38</v>
+        <v>112</v>
       </c>
       <c r="D75" t="n">
-        <v>2.95</v>
+        <v>3.8</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>EMKAY</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>426.4</v>
+        <v>247.63</v>
       </c>
       <c r="C76" t="n">
-        <v>438.95</v>
+        <v>257</v>
       </c>
       <c r="D76" t="n">
-        <v>2.94</v>
+        <v>3.78</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SARVESHWAR</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>3.75</v>
+        <v>29.05</v>
       </c>
       <c r="C77" t="n">
-        <v>3.86</v>
+        <v>30.1</v>
       </c>
       <c r="D77" t="n">
-        <v>2.93</v>
+        <v>3.61</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>924.1</v>
+        <v>46.24</v>
       </c>
       <c r="C78" t="n">
-        <v>951</v>
+        <v>47.9</v>
       </c>
       <c r="D78" t="n">
-        <v>2.91</v>
+        <v>3.59</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>URAVIDEF</t>
+          <t>SVLL</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>118.55</v>
+        <v>655.6</v>
       </c>
       <c r="C79" t="n">
-        <v>122</v>
+        <v>679</v>
       </c>
       <c r="D79" t="n">
-        <v>2.91</v>
+        <v>3.57</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>AVG</t>
+          <t>SERVOTECH</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>148.6</v>
+        <v>100.91</v>
       </c>
       <c r="C80" t="n">
-        <v>152.93</v>
+        <v>104.5</v>
       </c>
       <c r="D80" t="n">
-        <v>2.91</v>
+        <v>3.56</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2203,13 +2203,13 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>6.6</v>
+        <v>6.51</v>
       </c>
       <c r="C81" t="n">
-        <v>6.79</v>
+        <v>6.74</v>
       </c>
       <c r="D81" t="n">
-        <v>2.88</v>
+        <v>3.53</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SYSTMTXC</t>
+          <t>INTENTECH</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>64.16</v>
+        <v>95.48</v>
       </c>
       <c r="C82" t="n">
-        <v>66</v>
+        <v>98.8</v>
       </c>
       <c r="D82" t="n">
-        <v>2.87</v>
+        <v>3.48</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>AROGRANITE</t>
+          <t>SILLYMONKS</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>25.47</v>
+        <v>17.01</v>
       </c>
       <c r="C83" t="n">
-        <v>26.19</v>
+        <v>17.6</v>
       </c>
       <c r="D83" t="n">
-        <v>2.83</v>
+        <v>3.47</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>JAIPURKURT</t>
+          <t>JISLDVREQS</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>33.02</v>
+        <v>22.6</v>
       </c>
       <c r="C84" t="n">
-        <v>33.95</v>
+        <v>23.38</v>
       </c>
       <c r="D84" t="n">
-        <v>2.82</v>
+        <v>3.45</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>BLBLIMITED</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>17.51</v>
+        <v>17.31</v>
       </c>
       <c r="C85" t="n">
-        <v>18</v>
+        <v>17.9</v>
       </c>
       <c r="D85" t="n">
-        <v>2.8</v>
+        <v>3.41</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TENNIND</t>
+          <t>AHLADA</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>557.1</v>
+        <v>41.2</v>
       </c>
       <c r="C86" t="n">
-        <v>572.7</v>
+        <v>42.6</v>
       </c>
       <c r="D86" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>BELLACASA</t>
+          <t>SUBEXLTD</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>238.42</v>
+        <v>10.69</v>
       </c>
       <c r="C87" t="n">
-        <v>245</v>
+        <v>11.05</v>
       </c>
       <c r="D87" t="n">
-        <v>2.76</v>
+        <v>3.37</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>VINNY</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>1.09</v>
+        <v>4324.4</v>
       </c>
       <c r="C88" t="n">
-        <v>1.12</v>
+        <v>4470</v>
       </c>
       <c r="D88" t="n">
-        <v>2.75</v>
+        <v>3.37</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>DBSTOCKBRO</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>33.44</v>
+        <v>4.81</v>
       </c>
       <c r="C89" t="n">
-        <v>34.35</v>
+        <v>4.97</v>
       </c>
       <c r="D89" t="n">
-        <v>2.72</v>
+        <v>3.33</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BSOFT</t>
+          <t>EPACKPEB</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>327.8</v>
+        <v>187.64</v>
       </c>
       <c r="C90" t="n">
-        <v>336.45</v>
+        <v>193.87</v>
       </c>
       <c r="D90" t="n">
-        <v>2.64</v>
+        <v>3.32</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SILLYMONKS</t>
+          <t>CLEDUCATE</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>16.42</v>
+        <v>46.47</v>
       </c>
       <c r="C91" t="n">
-        <v>16.85</v>
+        <v>47.99</v>
       </c>
       <c r="D91" t="n">
-        <v>2.62</v>
+        <v>3.27</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>10.3</v>
+        <v>6.2</v>
       </c>
       <c r="C92" t="n">
-        <v>10.57</v>
+        <v>6.4</v>
       </c>
       <c r="D92" t="n">
-        <v>2.62</v>
+        <v>3.23</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>HDIL</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>1.92</v>
+        <v>591.05</v>
       </c>
       <c r="C93" t="n">
-        <v>1.97</v>
+        <v>610</v>
       </c>
       <c r="D93" t="n">
-        <v>2.6</v>
+        <v>3.21</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>HALEOSLABS</t>
+          <t>HBESD</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>1423.3</v>
+        <v>72.38</v>
       </c>
       <c r="C94" t="n">
-        <v>1459.9</v>
+        <v>74.7</v>
       </c>
       <c r="D94" t="n">
-        <v>2.57</v>
+        <v>3.21</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1.95</v>
+        <v>61.59</v>
       </c>
       <c r="C95" t="n">
-        <v>2</v>
+        <v>63.56</v>
       </c>
       <c r="D95" t="n">
-        <v>2.56</v>
+        <v>3.2</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>UNITEDTEA</t>
+          <t>NILASPACES</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>510.1</v>
+        <v>12.84</v>
       </c>
       <c r="C96" t="n">
-        <v>523.1</v>
+        <v>13.25</v>
       </c>
       <c r="D96" t="n">
-        <v>2.55</v>
+        <v>3.19</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ATLANTAELE</t>
+          <t>CARTRADE</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1983.6</v>
+        <v>1795</v>
       </c>
       <c r="C97" t="n">
-        <v>2034</v>
+        <v>1852</v>
       </c>
       <c r="D97" t="n">
-        <v>2.54</v>
+        <v>3.18</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>NILAINFRA</t>
+          <t>VIPULLTD</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>7.9</v>
+        <v>8.9</v>
       </c>
       <c r="C98" t="n">
-        <v>8.1</v>
+        <v>9.18</v>
       </c>
       <c r="D98" t="n">
-        <v>2.53</v>
+        <v>3.15</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SJLOGISTIC</t>
+          <t>DCMSRIND</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>326.7</v>
+        <v>36.84</v>
       </c>
       <c r="C99" t="n">
-        <v>334.85</v>
+        <v>38</v>
       </c>
       <c r="D99" t="n">
-        <v>2.49</v>
+        <v>3.15</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>PREMCO</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1202.5</v>
+        <v>370.4</v>
       </c>
       <c r="C100" t="n">
-        <v>1232.5</v>
+        <v>381.95</v>
       </c>
       <c r="D100" t="n">
-        <v>2.49</v>
+        <v>3.12</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>THOMASCOTT</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>40.64</v>
+        <v>278.4</v>
       </c>
       <c r="C101" t="n">
-        <v>41.65</v>
+        <v>287</v>
       </c>
       <c r="D101" t="n">
-        <v>2.49</v>
+        <v>3.09</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>BANSALWIRE</t>
+          <t>SHEMAROO</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>308.4</v>
+        <v>105.45</v>
       </c>
       <c r="C102" t="n">
-        <v>316</v>
+        <v>108.7</v>
       </c>
       <c r="D102" t="n">
-        <v>2.46</v>
+        <v>3.08</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>ADVAIT</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>99.76000000000001</v>
+        <v>1972.4</v>
       </c>
       <c r="C103" t="n">
-        <v>102.2</v>
+        <v>2032.7</v>
       </c>
       <c r="D103" t="n">
-        <v>2.45</v>
+        <v>3.06</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>HEXATRADEX</t>
+          <t>MOLDTECH</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>161.88</v>
+        <v>118.4</v>
       </c>
       <c r="C104" t="n">
-        <v>165.85</v>
+        <v>122</v>
       </c>
       <c r="D104" t="n">
-        <v>2.45</v>
+        <v>3.04</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>INSPIRISYS</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>6.11</v>
+        <v>125.1</v>
       </c>
       <c r="C105" t="n">
-        <v>6.26</v>
+        <v>128.9</v>
       </c>
       <c r="D105" t="n">
-        <v>2.45</v>
+        <v>3.04</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>BI</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>64.41</v>
+        <v>1.98</v>
       </c>
       <c r="C106" t="n">
-        <v>65.98999999999999</v>
+        <v>2.04</v>
       </c>
       <c r="D106" t="n">
-        <v>2.45</v>
+        <v>3.03</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>TREJHARA</t>
+          <t>VALIANTLAB</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>143.7</v>
+        <v>76.76000000000001</v>
       </c>
       <c r="C107" t="n">
-        <v>147.2</v>
+        <v>79</v>
       </c>
       <c r="D107" t="n">
-        <v>2.44</v>
+        <v>2.92</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ASPINWALL</t>
+          <t>KOHINOOR</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>239.88</v>
+        <v>25.07</v>
       </c>
       <c r="C108" t="n">
-        <v>245.7</v>
+        <v>25.8</v>
       </c>
       <c r="D108" t="n">
-        <v>2.43</v>
+        <v>2.91</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>INDIQUBE</t>
+          <t>AMBALALSA</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>156.4</v>
+        <v>37.3</v>
       </c>
       <c r="C109" t="n">
-        <v>160.18</v>
+        <v>38.38</v>
       </c>
       <c r="D109" t="n">
-        <v>2.42</v>
+        <v>2.9</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>A2ZINFRA</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>14.15</v>
+        <v>68.03</v>
       </c>
       <c r="C110" t="n">
-        <v>14.49</v>
+        <v>70</v>
       </c>
       <c r="D110" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TTKHLTCARE</t>
+          <t>ANTELOPUS</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>916.1</v>
+        <v>854.2</v>
       </c>
       <c r="C111" t="n">
-        <v>938</v>
+        <v>879</v>
       </c>
       <c r="D111" t="n">
-        <v>2.39</v>
+        <v>2.9</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>DAVANGERE</t>
+          <t>COMPUSOFT</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>3.81</v>
+        <v>13.55</v>
       </c>
       <c r="C112" t="n">
-        <v>3.9</v>
+        <v>13.94</v>
       </c>
       <c r="D112" t="n">
-        <v>2.36</v>
+        <v>2.88</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GENUSPAPER</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>12.36</v>
+        <v>0.35</v>
       </c>
       <c r="C113" t="n">
-        <v>12.65</v>
+        <v>0.36</v>
       </c>
       <c r="D113" t="n">
-        <v>2.35</v>
+        <v>2.86</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>PIONEEREMB</t>
+          <t>CENTEXT</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>24.36</v>
+        <v>19.34</v>
       </c>
       <c r="C114" t="n">
-        <v>24.93</v>
+        <v>19.89</v>
       </c>
       <c r="D114" t="n">
-        <v>2.34</v>
+        <v>2.84</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>BEARDSELL</t>
+          <t>VALUE360</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>29.27</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="C115" t="n">
-        <v>29.95</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="D115" t="n">
-        <v>2.32</v>
+        <v>2.83</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CRIZAC</t>
+          <t>TAMBOLIIN</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>215.98</v>
+        <v>180</v>
       </c>
       <c r="C116" t="n">
-        <v>220.99</v>
+        <v>185</v>
       </c>
       <c r="D116" t="n">
-        <v>2.32</v>
+        <v>2.78</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>HCL-INSYS</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>12.12</v>
+        <v>42.82</v>
       </c>
       <c r="C117" t="n">
-        <v>12.4</v>
+        <v>44</v>
       </c>
       <c r="D117" t="n">
-        <v>2.31</v>
+        <v>2.76</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>GOACARBON</t>
+          <t>BORORENEW</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>390.85</v>
+        <v>501.35</v>
       </c>
       <c r="C118" t="n">
-        <v>399.8</v>
+        <v>515.15</v>
       </c>
       <c r="D118" t="n">
-        <v>2.29</v>
+        <v>2.75</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>LINCOLN</t>
+          <t>CORDSCABLE</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>606.2</v>
+        <v>223.04</v>
       </c>
       <c r="C119" t="n">
-        <v>620</v>
+        <v>228.99</v>
       </c>
       <c r="D119" t="n">
-        <v>2.28</v>
+        <v>2.67</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>6.64</v>
+        <v>6.04</v>
       </c>
       <c r="C120" t="n">
-        <v>6.79</v>
+        <v>6.2</v>
       </c>
       <c r="D120" t="n">
-        <v>2.26</v>
+        <v>2.65</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>UFBL</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>44.4</v>
+        <v>487.2</v>
       </c>
       <c r="C121" t="n">
-        <v>45.4</v>
+        <v>499.95</v>
       </c>
       <c r="D121" t="n">
-        <v>2.25</v>
+        <v>2.62</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>KELLTONTEC</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>8.460000000000001</v>
+        <v>16.82</v>
       </c>
       <c r="C122" t="n">
-        <v>8.65</v>
+        <v>17.26</v>
       </c>
       <c r="D122" t="n">
-        <v>2.25</v>
+        <v>2.62</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>MANYAVAR</t>
+          <t>NIRAJ</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>399.05</v>
+        <v>28.73</v>
       </c>
       <c r="C123" t="n">
-        <v>408</v>
+        <v>29.47</v>
       </c>
       <c r="D123" t="n">
-        <v>2.24</v>
+        <v>2.58</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>13.55</v>
+        <v>24.47</v>
       </c>
       <c r="C124" t="n">
-        <v>13.85</v>
+        <v>25.1</v>
       </c>
       <c r="D124" t="n">
-        <v>2.21</v>
+        <v>2.57</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LAGNAM</t>
+          <t>MACPOWER</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>84.04000000000001</v>
+        <v>931.25</v>
       </c>
       <c r="C125" t="n">
-        <v>85.89</v>
+        <v>955</v>
       </c>
       <c r="D125" t="n">
-        <v>2.2</v>
+        <v>2.55</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>FLFL</t>
+          <t>DBSTOCKBRO</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>1.4</v>
+        <v>34.09</v>
       </c>
       <c r="C126" t="n">
-        <v>1.43</v>
+        <v>34.95</v>
       </c>
       <c r="D126" t="n">
-        <v>2.14</v>
+        <v>2.52</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>2.34</v>
+        <v>43.8</v>
       </c>
       <c r="C127" t="n">
-        <v>2.39</v>
+        <v>44.89</v>
       </c>
       <c r="D127" t="n">
-        <v>2.14</v>
+        <v>2.49</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ATLANTAA</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>41.12</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C128" t="n">
-        <v>42</v>
+        <v>0.83</v>
       </c>
       <c r="D128" t="n">
-        <v>2.14</v>
+        <v>2.47</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SHRADHA</t>
+          <t>FERMENTA</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>34.27</v>
+        <v>312.35</v>
       </c>
       <c r="C129" t="n">
-        <v>35</v>
+        <v>320</v>
       </c>
       <c r="D129" t="n">
-        <v>2.13</v>
+        <v>2.45</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>24.09</v>
+        <v>2.46</v>
       </c>
       <c r="C130" t="n">
-        <v>24.6</v>
+        <v>2.52</v>
       </c>
       <c r="D130" t="n">
-        <v>2.12</v>
+        <v>2.44</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>TREL</t>
+          <t>JSLL</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>25.66</v>
+        <v>590.6</v>
       </c>
       <c r="C131" t="n">
-        <v>26.2</v>
+        <v>605</v>
       </c>
       <c r="D131" t="n">
-        <v>2.1</v>
+        <v>2.44</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>TRACXN</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>4.81</v>
+        <v>31.72</v>
       </c>
       <c r="C132" t="n">
-        <v>4.91</v>
+        <v>32.49</v>
       </c>
       <c r="D132" t="n">
-        <v>2.08</v>
+        <v>2.43</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>TIJARIA</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>4.35</v>
+        <v>0.42</v>
       </c>
       <c r="C133" t="n">
-        <v>4.44</v>
+        <v>0.43</v>
       </c>
       <c r="D133" t="n">
-        <v>2.07</v>
+        <v>2.38</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>LOKESHMACH</t>
+          <t>ORBTEXP</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>249.8</v>
+        <v>178.74</v>
       </c>
       <c r="C134" t="n">
-        <v>254.95</v>
+        <v>183</v>
       </c>
       <c r="D134" t="n">
-        <v>2.06</v>
+        <v>2.38</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>RELIABLE</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>137.13</v>
+        <v>10.92</v>
       </c>
       <c r="C135" t="n">
-        <v>139.9</v>
+        <v>11.18</v>
       </c>
       <c r="D135" t="n">
-        <v>2.02</v>
+        <v>2.38</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>KALPATARU</t>
+          <t>ZODIAC</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>323.4</v>
+        <v>287.95</v>
       </c>
       <c r="C136" t="n">
-        <v>329.9</v>
+        <v>294.75</v>
       </c>
       <c r="D136" t="n">
-        <v>2.01</v>
+        <v>2.36</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>ELANTAS</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>11.51</v>
+        <v>9479</v>
       </c>
       <c r="C137" t="n">
-        <v>11.74</v>
+        <v>9701</v>
       </c>
       <c r="D137" t="n">
-        <v>2</v>
+        <v>2.34</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>MOKSH</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>1</v>
+        <v>11.7</v>
       </c>
       <c r="C138" t="n">
-        <v>1.02</v>
+        <v>11.97</v>
       </c>
       <c r="D138" t="n">
-        <v>2</v>
+        <v>2.31</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>DJML</t>
+          <t>WORTHPERI</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>104.85</v>
+        <v>128.91</v>
       </c>
       <c r="C139" t="n">
-        <v>106.95</v>
+        <v>131.89</v>
       </c>
       <c r="D139" t="n">
-        <v>2</v>
+        <v>2.31</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>AAREYDRUGS</t>
+          <t>NITIRAJ</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>77.37</v>
+        <v>194.52</v>
       </c>
       <c r="C140" t="n">
-        <v>78.92</v>
+        <v>199</v>
       </c>
       <c r="D140" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>DEEDEV</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>0.5</v>
+        <v>654.2</v>
       </c>
       <c r="C141" t="n">
-        <v>0.51</v>
+        <v>669</v>
       </c>
       <c r="D141" t="n">
-        <v>2</v>
+        <v>2.26</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>NORBTEAEXP</t>
+          <t>TERASOFT</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>81.44</v>
+        <v>430.1</v>
       </c>
       <c r="C142" t="n">
-        <v>83.06999999999999</v>
+        <v>439.7</v>
       </c>
       <c r="D142" t="n">
-        <v>2</v>
+        <v>2.23</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>UNIMECH</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>3.52</v>
+        <v>993.15</v>
       </c>
       <c r="C143" t="n">
-        <v>3.59</v>
+        <v>1014.95</v>
       </c>
       <c r="D143" t="n">
-        <v>1.99</v>
+        <v>2.2</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>AIRAN</t>
+          <t>DEVIT</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>16.64</v>
+        <v>28.87</v>
       </c>
       <c r="C144" t="n">
-        <v>16.97</v>
+        <v>29.5</v>
       </c>
       <c r="D144" t="n">
-        <v>1.98</v>
+        <v>2.18</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>IMPAL</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>1057.1</v>
+        <v>8.24</v>
       </c>
       <c r="C145" t="n">
-        <v>1078</v>
+        <v>8.42</v>
       </c>
       <c r="D145" t="n">
-        <v>1.98</v>
+        <v>2.18</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>RANASUG</t>
+          <t>HEXATRADEX</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>12.12</v>
+        <v>161.13</v>
       </c>
       <c r="C146" t="n">
-        <v>12.36</v>
+        <v>164.64</v>
       </c>
       <c r="D146" t="n">
-        <v>1.98</v>
+        <v>2.18</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>RRIL</t>
+          <t>ALKALI</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>20.16</v>
+        <v>97.86</v>
       </c>
       <c r="C147" t="n">
-        <v>20.56</v>
+        <v>99.98</v>
       </c>
       <c r="D147" t="n">
-        <v>1.98</v>
+        <v>2.17</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>BLBLIMITED</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>17.05</v>
+        <v>2.31</v>
       </c>
       <c r="C148" t="n">
-        <v>17.38</v>
+        <v>2.36</v>
       </c>
       <c r="D148" t="n">
-        <v>1.94</v>
+        <v>2.16</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SREEL</t>
+          <t>CEREBRAINT</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>202.97</v>
+        <v>3.26</v>
       </c>
       <c r="C149" t="n">
-        <v>206.9</v>
+        <v>3.33</v>
       </c>
       <c r="D149" t="n">
-        <v>1.94</v>
+        <v>2.15</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>HLVLTD</t>
+          <t>RUCHIRA</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>7.84</v>
+        <v>115.46</v>
       </c>
       <c r="C150" t="n">
-        <v>7.99</v>
+        <v>117.9</v>
       </c>
       <c r="D150" t="n">
-        <v>1.91</v>
+        <v>2.11</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MAHEPC</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>114.75</v>
+        <v>7.69</v>
       </c>
       <c r="C151" t="n">
-        <v>116.93</v>
+        <v>7.85</v>
       </c>
       <c r="D151" t="n">
-        <v>1.9</v>
+        <v>2.08</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SONAMLTD</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>57.71</v>
+        <v>485.4</v>
       </c>
       <c r="C152" t="n">
-        <v>58.8</v>
+        <v>495.5</v>
       </c>
       <c r="D152" t="n">
-        <v>1.89</v>
+        <v>2.08</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>PNCINFRA</t>
+          <t>PRAKASHSTL</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>207.07</v>
+        <v>4.35</v>
       </c>
       <c r="C153" t="n">
-        <v>210.95</v>
+        <v>4.44</v>
       </c>
       <c r="D153" t="n">
-        <v>1.87</v>
+        <v>2.07</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>LATENTVIEW</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>316.4</v>
+        <v>6.32</v>
       </c>
       <c r="C154" t="n">
-        <v>322.3</v>
+        <v>6.45</v>
       </c>
       <c r="D154" t="n">
-        <v>1.86</v>
+        <v>2.06</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>ALANKIT</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>3.23</v>
+        <v>8.42</v>
       </c>
       <c r="C155" t="n">
-        <v>3.29</v>
+        <v>8.59</v>
       </c>
       <c r="D155" t="n">
-        <v>1.86</v>
+        <v>2.02</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SUVIDHAA</t>
+          <t>FMNL</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>2.7</v>
+        <v>10.9</v>
       </c>
       <c r="C156" t="n">
-        <v>2.75</v>
+        <v>11.12</v>
       </c>
       <c r="D156" t="n">
-        <v>1.85</v>
+        <v>2.02</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>UFLEX</t>
+          <t>MTARTECH</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>440.65</v>
+        <v>7216</v>
       </c>
       <c r="C157" t="n">
-        <v>448.8</v>
+        <v>7360.5</v>
       </c>
       <c r="D157" t="n">
-        <v>1.85</v>
+        <v>2</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>RAMANEWS</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>29.21</v>
+        <v>0.5</v>
       </c>
       <c r="C158" t="n">
-        <v>29.75</v>
+        <v>0.51</v>
       </c>
       <c r="D158" t="n">
-        <v>1.85</v>
+        <v>2</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>NORBTEAEXP</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>0.55</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="C159" t="n">
-        <v>0.5600000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="D159" t="n">
-        <v>1.82</v>
+        <v>1.99</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ROSSELLIND</t>
+          <t>MADHAVBAUG</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>55.98</v>
+        <v>186.8</v>
       </c>
       <c r="C160" t="n">
-        <v>57</v>
+        <v>190.5</v>
       </c>
       <c r="D160" t="n">
-        <v>1.82</v>
+        <v>1.98</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>RVTH</t>
+          <t>JNKINDIA</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>740.5</v>
+        <v>361.4</v>
       </c>
       <c r="C161" t="n">
-        <v>754</v>
+        <v>368.55</v>
       </c>
       <c r="D161" t="n">
-        <v>1.82</v>
+        <v>1.98</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>KNAGRI</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>185.04</v>
+        <v>23.24</v>
       </c>
       <c r="C162" t="n">
-        <v>188.4</v>
+        <v>23.7</v>
       </c>
       <c r="D162" t="n">
-        <v>1.82</v>
+        <v>1.98</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>VASWANI</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>55.89</v>
+        <v>858.95</v>
       </c>
       <c r="C163" t="n">
-        <v>56.9</v>
+        <v>876</v>
       </c>
       <c r="D163" t="n">
-        <v>1.81</v>
+        <v>1.98</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>BAGFILMS</t>
+          <t>GOCOLORS</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>4.98</v>
+        <v>336.05</v>
       </c>
       <c r="C164" t="n">
-        <v>5.07</v>
+        <v>342.7</v>
       </c>
       <c r="D164" t="n">
-        <v>1.81</v>
+        <v>1.98</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>HEADSUP</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>6.09</v>
+        <v>7.12</v>
       </c>
       <c r="C165" t="n">
-        <v>6.2</v>
+        <v>7.26</v>
       </c>
       <c r="D165" t="n">
-        <v>1.81</v>
+        <v>1.97</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>NIITLTD</t>
+          <t>CAPITALSFB</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>81.54000000000001</v>
+        <v>268.7</v>
       </c>
       <c r="C166" t="n">
-        <v>83</v>
+        <v>274</v>
       </c>
       <c r="D166" t="n">
-        <v>1.79</v>
+        <v>1.97</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>0.5600000000000001</v>
+        <v>11.22</v>
       </c>
       <c r="C167" t="n">
-        <v>0.57</v>
+        <v>11.44</v>
       </c>
       <c r="D167" t="n">
-        <v>1.79</v>
+        <v>1.96</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>VASCONEQ</t>
+          <t>OSELDEVICE</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>32.66</v>
+        <v>471.7</v>
       </c>
       <c r="C168" t="n">
-        <v>33.24</v>
+        <v>480.95</v>
       </c>
       <c r="D168" t="n">
-        <v>1.78</v>
+        <v>1.96</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>IFBAGRO</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>1.14</v>
+        <v>978.7</v>
       </c>
       <c r="C169" t="n">
-        <v>1.16</v>
+        <v>997.7</v>
       </c>
       <c r="D169" t="n">
-        <v>1.75</v>
+        <v>1.94</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>KANANIIND</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>139.27</v>
+        <v>1.55</v>
       </c>
       <c r="C170" t="n">
-        <v>141.7</v>
+        <v>1.58</v>
       </c>
       <c r="D170" t="n">
-        <v>1.74</v>
+        <v>1.94</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>PIGL</t>
+          <t>UGARSUGAR</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>90.18000000000001</v>
+        <v>40.18</v>
       </c>
       <c r="C171" t="n">
-        <v>91.75</v>
+        <v>40.96</v>
       </c>
       <c r="D171" t="n">
-        <v>1.74</v>
+        <v>1.94</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>SIKKO</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>4.06</v>
+        <v>20.25</v>
       </c>
       <c r="C172" t="n">
-        <v>4.13</v>
+        <v>20.64</v>
       </c>
       <c r="D172" t="n">
-        <v>1.72</v>
+        <v>1.93</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>KCPSUGIND</t>
+          <t>TARACHAND</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>25.06</v>
+        <v>60.24</v>
       </c>
       <c r="C173" t="n">
-        <v>25.49</v>
+        <v>61.4</v>
       </c>
       <c r="D173" t="n">
-        <v>1.72</v>
+        <v>1.93</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>BLUECHIP</t>
+          <t>WANBURY</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>2.33</v>
+        <v>258</v>
       </c>
       <c r="C174" t="n">
-        <v>2.37</v>
+        <v>262.95</v>
       </c>
       <c r="D174" t="n">
-        <v>1.72</v>
+        <v>1.92</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>BLACKROSE</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>94.2</v>
+        <v>54.34</v>
       </c>
       <c r="C175" t="n">
-        <v>95.8</v>
+        <v>55.38</v>
       </c>
       <c r="D175" t="n">
-        <v>1.7</v>
+        <v>1.91</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>NEWGEN</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>370.45</v>
+        <v>518.1</v>
       </c>
       <c r="C176" t="n">
-        <v>376.7</v>
+        <v>528</v>
       </c>
       <c r="D176" t="n">
-        <v>1.69</v>
+        <v>1.91</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>PENINLAND</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>13.73</v>
+        <v>16.42</v>
       </c>
       <c r="C177" t="n">
-        <v>13.96</v>
+        <v>16.73</v>
       </c>
       <c r="D177" t="n">
-        <v>1.68</v>
+        <v>1.89</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>WANBURY</t>
+          <t>NRL</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>266.55</v>
+        <v>65.56999999999999</v>
       </c>
       <c r="C178" t="n">
-        <v>271</v>
+        <v>66.81</v>
       </c>
       <c r="D178" t="n">
-        <v>1.67</v>
+        <v>1.89</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MASFIN</t>
+          <t>GTL</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>304.5</v>
+        <v>7.39</v>
       </c>
       <c r="C179" t="n">
-        <v>309.5</v>
+        <v>7.53</v>
       </c>
       <c r="D179" t="n">
-        <v>1.64</v>
+        <v>1.89</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>KHADIM</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>99.86</v>
+        <v>170.12</v>
       </c>
       <c r="C180" t="n">
-        <v>101.5</v>
+        <v>173.3</v>
       </c>
       <c r="D180" t="n">
-        <v>1.64</v>
+        <v>1.87</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>HGM</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>55</v>
+        <v>61.65</v>
       </c>
       <c r="C181" t="n">
-        <v>55.9</v>
+        <v>62.8</v>
       </c>
       <c r="D181" t="n">
-        <v>1.64</v>
+        <v>1.87</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>WINSOME</t>
+          <t>DBOL</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>2.45</v>
+        <v>112.72</v>
       </c>
       <c r="C182" t="n">
-        <v>2.49</v>
+        <v>114.8</v>
       </c>
       <c r="D182" t="n">
-        <v>1.63</v>
+        <v>1.85</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>SHIVALIK</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>271.3</v>
+        <v>19.97</v>
       </c>
       <c r="C183" t="n">
-        <v>275.7</v>
+        <v>20.34</v>
       </c>
       <c r="D183" t="n">
-        <v>1.62</v>
+        <v>1.85</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>82.66</v>
+        <v>0.54</v>
       </c>
       <c r="C184" t="n">
-        <v>83.98999999999999</v>
+        <v>0.55</v>
       </c>
       <c r="D184" t="n">
-        <v>1.61</v>
+        <v>1.85</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SNOWMAN</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>36.81</v>
+        <v>3.83</v>
       </c>
       <c r="C185" t="n">
-        <v>37.4</v>
+        <v>3.9</v>
       </c>
       <c r="D185" t="n">
-        <v>1.6</v>
+        <v>1.83</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>INDOTECH</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>835.7</v>
+        <v>2722.8</v>
       </c>
       <c r="C186" t="n">
-        <v>848.95</v>
+        <v>2772</v>
       </c>
       <c r="D186" t="n">
-        <v>1.59</v>
+        <v>1.81</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>PIGL</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>30.02</v>
+        <v>98.23</v>
       </c>
       <c r="C187" t="n">
-        <v>30.49</v>
+        <v>100</v>
       </c>
       <c r="D187" t="n">
-        <v>1.57</v>
+        <v>1.8</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SAKHTISUG</t>
+          <t>MAYURUNIQ</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>17.87</v>
+        <v>745.25</v>
       </c>
       <c r="C188" t="n">
-        <v>18.15</v>
+        <v>758.7</v>
       </c>
       <c r="D188" t="n">
-        <v>1.57</v>
+        <v>1.8</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>NDLVENTURE</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>41.83</v>
+        <v>133.54</v>
       </c>
       <c r="C189" t="n">
-        <v>42.48</v>
+        <v>135.95</v>
       </c>
       <c r="D189" t="n">
-        <v>1.55</v>
+        <v>1.8</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>MHLXMIRU</t>
+          <t>SEYAIND</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>179.25</v>
+        <v>14.99</v>
       </c>
       <c r="C190" t="n">
-        <v>182.01</v>
+        <v>15.26</v>
       </c>
       <c r="D190" t="n">
-        <v>1.54</v>
+        <v>1.8</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>TIRUPATIFL</t>
+          <t>BAGFILMS</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>45.11</v>
+        <v>5</v>
       </c>
       <c r="C191" t="n">
-        <v>45.8</v>
+        <v>5.09</v>
       </c>
       <c r="D191" t="n">
-        <v>1.53</v>
+        <v>1.8</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>HMT</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>55.15</v>
+        <v>323.2</v>
       </c>
       <c r="C192" t="n">
-        <v>55.99</v>
+        <v>329</v>
       </c>
       <c r="D192" t="n">
-        <v>1.52</v>
+        <v>1.79</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>SIGNPOST</t>
+          <t>SEMAC</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>273</v>
+        <v>335.05</v>
       </c>
       <c r="C193" t="n">
-        <v>277.1</v>
+        <v>341</v>
       </c>
       <c r="D193" t="n">
-        <v>1.5</v>
+        <v>1.78</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>KENNAMET</t>
+          <t>ANUHPHR</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>2863.2</v>
+        <v>75.53</v>
       </c>
       <c r="C194" t="n">
-        <v>2906.1</v>
+        <v>76.87</v>
       </c>
       <c r="D194" t="n">
-        <v>1.5</v>
+        <v>1.77</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ONEPOINT</t>
+          <t>MUNISH</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>59.25</v>
+        <v>65.55</v>
       </c>
       <c r="C195" t="n">
-        <v>60.13</v>
+        <v>66.7</v>
       </c>
       <c r="D195" t="n">
-        <v>1.49</v>
+        <v>1.75</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>PRITIKA</t>
+          <t>ESSENTIA</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>63.95</v>
+        <v>1.73</v>
       </c>
       <c r="C196" t="n">
-        <v>64.90000000000001</v>
+        <v>1.76</v>
       </c>
       <c r="D196" t="n">
-        <v>1.49</v>
+        <v>1.73</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>ADVANCE</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>102.47</v>
+        <v>5.21</v>
       </c>
       <c r="C197" t="n">
-        <v>104</v>
+        <v>5.3</v>
       </c>
       <c r="D197" t="n">
-        <v>1.49</v>
+        <v>1.73</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>CLEANMAX</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>1090.4</v>
+        <v>24.27</v>
       </c>
       <c r="C198" t="n">
-        <v>1106.6</v>
+        <v>24.69</v>
       </c>
       <c r="D198" t="n">
-        <v>1.49</v>
+        <v>1.73</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>MALLCOM</t>
+          <t>KANPRPLA</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>959.8</v>
+        <v>186.78</v>
       </c>
       <c r="C199" t="n">
-        <v>974</v>
+        <v>190</v>
       </c>
       <c r="D199" t="n">
-        <v>1.48</v>
+        <v>1.72</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>RUCHIRA</t>
+          <t>BLUECHIP</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>115.09</v>
+        <v>2.37</v>
       </c>
       <c r="C200" t="n">
-        <v>116.79</v>
+        <v>2.41</v>
       </c>
       <c r="D200" t="n">
-        <v>1.48</v>
+        <v>1.69</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>ESTER</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>92.64</v>
+        <v>447.4</v>
       </c>
       <c r="C201" t="n">
-        <v>94</v>
+        <v>454.95</v>
       </c>
       <c r="D201" t="n">
-        <v>1.47</v>
+        <v>1.69</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-04 08:09 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>ESSEN-RE3</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24.02</v>
+        <v>0.04</v>
       </c>
       <c r="C2" t="n">
-        <v>27.03</v>
+        <v>0.05</v>
       </c>
       <c r="D2" t="n">
-        <v>12.53</v>
+        <v>25</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SHRIKRISH</t>
+          <t>RETAIL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>40.55</v>
+        <v>21.21</v>
       </c>
       <c r="C3" t="n">
-        <v>44.5</v>
+        <v>24.38</v>
       </c>
       <c r="D3" t="n">
-        <v>9.74</v>
+        <v>14.95</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ORIENTLTD</t>
+          <t>TNTELE</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>61.48</v>
+        <v>9.26</v>
       </c>
       <c r="C4" t="n">
-        <v>66.8</v>
+        <v>9.99</v>
       </c>
       <c r="D4" t="n">
-        <v>8.65</v>
+        <v>7.88</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>MFML</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.37</v>
+        <v>24.32</v>
       </c>
       <c r="C5" t="n">
-        <v>5.81</v>
+        <v>26.2</v>
       </c>
       <c r="D5" t="n">
-        <v>8.19</v>
+        <v>7.73</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>COCKERILL</t>
+          <t>AGARIND</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7593.5</v>
+        <v>419.4</v>
       </c>
       <c r="C6" t="n">
-        <v>8200</v>
+        <v>450</v>
       </c>
       <c r="D6" t="n">
-        <v>7.99</v>
+        <v>7.3</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>AVG-RE</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.15</v>
+        <v>3.28</v>
       </c>
       <c r="C7" t="n">
-        <v>0.16</v>
+        <v>3.5</v>
       </c>
       <c r="D7" t="n">
-        <v>6.67</v>
+        <v>6.71</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HALDER</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>228.79</v>
+        <v>15.52</v>
       </c>
       <c r="C8" t="n">
-        <v>244</v>
+        <v>16.49</v>
       </c>
       <c r="D8" t="n">
-        <v>6.65</v>
+        <v>6.25</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>14.38</v>
+        <v>0.16</v>
       </c>
       <c r="C9" t="n">
-        <v>15.3</v>
+        <v>0.17</v>
       </c>
       <c r="D9" t="n">
-        <v>6.4</v>
+        <v>6.25</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>KIRANVYPAR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>34.78</v>
+        <v>156.75</v>
       </c>
       <c r="C10" t="n">
-        <v>37</v>
+        <v>165.99</v>
       </c>
       <c r="D10" t="n">
-        <v>6.38</v>
+        <v>5.89</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TUNWAL</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>29.55</v>
+        <v>35.01</v>
       </c>
       <c r="C11" t="n">
-        <v>31.4</v>
+        <v>37</v>
       </c>
       <c r="D11" t="n">
-        <v>6.26</v>
+        <v>5.68</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PIONRINV</t>
+          <t>PKTEA</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>106.38</v>
+        <v>783.75</v>
       </c>
       <c r="C12" t="n">
-        <v>112.98</v>
+        <v>828</v>
       </c>
       <c r="D12" t="n">
-        <v>6.2</v>
+        <v>5.65</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MUKTAARTS</t>
+          <t>STRIDERS</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>64.06</v>
+        <v>61.8</v>
       </c>
       <c r="C13" t="n">
-        <v>67.8</v>
+        <v>65.25</v>
       </c>
       <c r="D13" t="n">
-        <v>5.84</v>
+        <v>5.58</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RULKA</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>91.7</v>
+        <v>10.59</v>
       </c>
       <c r="C14" t="n">
-        <v>96.90000000000001</v>
+        <v>11.14</v>
       </c>
       <c r="D14" t="n">
-        <v>5.67</v>
+        <v>5.19</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>UHTL</t>
+          <t>MERCANTILE</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>90.05</v>
+        <v>27.43</v>
       </c>
       <c r="C15" t="n">
-        <v>95</v>
+        <v>28.85</v>
       </c>
       <c r="D15" t="n">
-        <v>5.5</v>
+        <v>5.18</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CONCORDBIO</t>
+          <t>IDEAFORGE</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1166.2</v>
+        <v>857.15</v>
       </c>
       <c r="C16" t="n">
-        <v>1230</v>
+        <v>900</v>
       </c>
       <c r="D16" t="n">
-        <v>5.47</v>
+        <v>5</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IWP</t>
+          <t>MASKINVEST</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>34.44</v>
+        <v>158</v>
       </c>
       <c r="C17" t="n">
-        <v>36.24</v>
+        <v>165.9</v>
       </c>
       <c r="D17" t="n">
-        <v>5.23</v>
+        <v>5</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,14 +813,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PRIZOR</t>
+          <t>TANKUP</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>726.2</v>
+        <v>865.45</v>
       </c>
       <c r="C18" t="n">
-        <v>762.5</v>
+        <v>908.7</v>
       </c>
       <c r="D18" t="n">
         <v>5</v>
@@ -835,14 +835,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>BAFNAPH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1104.6</v>
+        <v>152.68</v>
       </c>
       <c r="C19" t="n">
-        <v>1159.8</v>
+        <v>160.31</v>
       </c>
       <c r="D19" t="n">
         <v>5</v>
@@ -857,14 +857,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IZMO</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>827.8</v>
+        <v>329</v>
       </c>
       <c r="C20" t="n">
-        <v>869.15</v>
+        <v>345.45</v>
       </c>
       <c r="D20" t="n">
         <v>5</v>
@@ -879,14 +879,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>UNIMECH</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1411.3</v>
+        <v>1042.8</v>
       </c>
       <c r="C21" t="n">
-        <v>1481.8</v>
+        <v>1094.9</v>
       </c>
       <c r="D21" t="n">
         <v>5</v>
@@ -901,14 +901,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BAFNAPH</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>145.41</v>
+        <v>293.68</v>
       </c>
       <c r="C22" t="n">
-        <v>152.68</v>
+        <v>308.36</v>
       </c>
       <c r="D22" t="n">
         <v>5</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>RELINFRA</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>74.17</v>
       </c>
       <c r="C23" t="n">
-        <v>2.1</v>
+        <v>77.87</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MASKINVEST</t>
+          <t>RNPL</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>150.49</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="C24" t="n">
-        <v>158.01</v>
+        <v>83.05</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RELINFRA</t>
+          <t>UTLSOLAR</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>70.64</v>
+        <v>335.75</v>
       </c>
       <c r="C25" t="n">
-        <v>74.17</v>
+        <v>352.5</v>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>279.7</v>
+        <v>1481.8</v>
       </c>
       <c r="C26" t="n">
-        <v>293.68</v>
+        <v>1555.8</v>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,14 +1011,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>313.7</v>
+        <v>136.25</v>
       </c>
       <c r="C27" t="n">
-        <v>329.35</v>
+        <v>143.05</v>
       </c>
       <c r="D27" t="n">
         <v>4.99</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AHLWEST</t>
+          <t>CLEDUCATE</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>579.85</v>
+        <v>48.79</v>
       </c>
       <c r="C28" t="n">
-        <v>608.8</v>
+        <v>51.22</v>
       </c>
       <c r="D28" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>UTLSOLAR</t>
+          <t>ORTINGLOBE</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>319.8</v>
+        <v>15.69</v>
       </c>
       <c r="C29" t="n">
-        <v>335.75</v>
+        <v>16.47</v>
       </c>
       <c r="D29" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SUPREMEPWR</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>246.25</v>
+        <v>30</v>
       </c>
       <c r="C30" t="n">
-        <v>258.55</v>
+        <v>31.48</v>
       </c>
       <c r="D30" t="n">
-        <v>4.99</v>
+        <v>4.93</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MCON</t>
+          <t>ALLETEC</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>43.2</v>
+        <v>137.05</v>
       </c>
       <c r="C31" t="n">
-        <v>45.35</v>
+        <v>143.8</v>
       </c>
       <c r="D31" t="n">
-        <v>4.98</v>
+        <v>4.93</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>129.8</v>
+        <v>43.9</v>
       </c>
       <c r="C32" t="n">
-        <v>136.25</v>
+        <v>46.05</v>
       </c>
       <c r="D32" t="n">
-        <v>4.97</v>
+        <v>4.9</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>USASEEDS</t>
+          <t>SEMAC</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>99.75</v>
+        <v>351.8</v>
       </c>
       <c r="C33" t="n">
-        <v>104.7</v>
+        <v>369</v>
       </c>
       <c r="D33" t="n">
-        <v>4.96</v>
+        <v>4.89</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GENSOL</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>20.79</v>
+        <v>90.95</v>
       </c>
       <c r="C34" t="n">
-        <v>21.82</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="D34" t="n">
-        <v>4.95</v>
+        <v>4.89</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>27.53</v>
+        <v>25.22</v>
       </c>
       <c r="C35" t="n">
-        <v>28.89</v>
+        <v>26.45</v>
       </c>
       <c r="D35" t="n">
-        <v>4.94</v>
+        <v>4.88</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1213,13 +1213,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>30.35</v>
+        <v>31.85</v>
       </c>
       <c r="C36" t="n">
-        <v>31.85</v>
+        <v>33.4</v>
       </c>
       <c r="D36" t="n">
-        <v>4.94</v>
+        <v>4.87</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SABEVENTS</t>
+          <t>UNIINFO</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>8.74</v>
+        <v>11.35</v>
       </c>
       <c r="C37" t="n">
-        <v>9.17</v>
+        <v>11.9</v>
       </c>
       <c r="D37" t="n">
-        <v>4.92</v>
+        <v>4.85</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>41.85</v>
+        <v>869.15</v>
       </c>
       <c r="C38" t="n">
-        <v>43.9</v>
+        <v>910.9</v>
       </c>
       <c r="D38" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>UNIVCABLES</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1239.2</v>
+        <v>5.43</v>
       </c>
       <c r="C39" t="n">
-        <v>1299.9</v>
+        <v>5.69</v>
       </c>
       <c r="D39" t="n">
-        <v>4.9</v>
+        <v>4.79</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>VIJAYPD</t>
+          <t>ATLANTAELE</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>89.90000000000001</v>
+        <v>2050.1</v>
       </c>
       <c r="C40" t="n">
-        <v>94.3</v>
+        <v>2148</v>
       </c>
       <c r="D40" t="n">
-        <v>4.89</v>
+        <v>4.78</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DYNAMIC</t>
+          <t>VITAL</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>154.45</v>
+        <v>52.5</v>
       </c>
       <c r="C41" t="n">
-        <v>161.95</v>
+        <v>54.99</v>
       </c>
       <c r="D41" t="n">
-        <v>4.86</v>
+        <v>4.74</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ORTINGLOBE</t>
+          <t>DELTIC</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>15.74</v>
+        <v>33.05</v>
       </c>
       <c r="C42" t="n">
-        <v>16.5</v>
+        <v>34.6</v>
       </c>
       <c r="D42" t="n">
-        <v>4.83</v>
+        <v>4.69</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ASTRON</t>
+          <t>ABANSENT</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3.95</v>
+        <v>26.74</v>
       </c>
       <c r="C43" t="n">
-        <v>4.14</v>
+        <v>27.99</v>
       </c>
       <c r="D43" t="n">
-        <v>4.81</v>
+        <v>4.67</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SYSTMTXC</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>64.73999999999999</v>
+        <v>2.58</v>
       </c>
       <c r="C44" t="n">
-        <v>67.8</v>
+        <v>2.7</v>
       </c>
       <c r="D44" t="n">
-        <v>4.73</v>
+        <v>4.65</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GLOSTERLTD</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>657.95</v>
+        <v>12.2</v>
       </c>
       <c r="C45" t="n">
-        <v>689</v>
+        <v>12.76</v>
       </c>
       <c r="D45" t="n">
-        <v>4.72</v>
+        <v>4.59</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1.06</v>
+        <v>620.6</v>
       </c>
       <c r="C46" t="n">
-        <v>1.11</v>
+        <v>649</v>
       </c>
       <c r="D46" t="n">
-        <v>4.72</v>
+        <v>4.58</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>PRIZOR</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>5.56</v>
+        <v>762.5</v>
       </c>
       <c r="C47" t="n">
-        <v>5.82</v>
+        <v>797.3</v>
       </c>
       <c r="D47" t="n">
-        <v>4.68</v>
+        <v>4.56</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>URAVIDEF</t>
+          <t>TGL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>116.61</v>
+        <v>23</v>
       </c>
       <c r="C48" t="n">
-        <v>122</v>
+        <v>24</v>
       </c>
       <c r="D48" t="n">
-        <v>4.62</v>
+        <v>4.35</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>5.19</v>
+        <v>8.83</v>
       </c>
       <c r="C49" t="n">
-        <v>5.43</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D49" t="n">
-        <v>4.62</v>
+        <v>4.19</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>3.51</v>
+        <v>5.78</v>
       </c>
       <c r="C50" t="n">
-        <v>3.67</v>
+        <v>6.02</v>
       </c>
       <c r="D50" t="n">
-        <v>4.56</v>
+        <v>4.15</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ATCENERGY</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>24.15</v>
+        <v>7.98</v>
       </c>
       <c r="C51" t="n">
-        <v>25.25</v>
+        <v>8.31</v>
       </c>
       <c r="D51" t="n">
-        <v>4.55</v>
+        <v>4.14</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>SMLT</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>13.49</v>
+        <v>71.77</v>
       </c>
       <c r="C52" t="n">
-        <v>14.1</v>
+        <v>74.7</v>
       </c>
       <c r="D52" t="n">
-        <v>4.52</v>
+        <v>4.08</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NHPC</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>72.29000000000001</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="C53" t="n">
-        <v>75.56</v>
+        <v>10</v>
       </c>
       <c r="D53" t="n">
-        <v>4.52</v>
+        <v>4.06</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SHRIKANHA</t>
+          <t>NAGREEKEXP</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>29.1</v>
+        <v>27.8</v>
       </c>
       <c r="C54" t="n">
-        <v>30.4</v>
+        <v>28.91</v>
       </c>
       <c r="D54" t="n">
-        <v>4.47</v>
+        <v>3.99</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>RFBL</t>
+          <t>TVVISION</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>63.2</v>
+        <v>5.29</v>
       </c>
       <c r="C55" t="n">
-        <v>66</v>
+        <v>5.5</v>
       </c>
       <c r="D55" t="n">
-        <v>4.43</v>
+        <v>3.97</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>XELPMOC</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>94.79000000000001</v>
+        <v>42.81</v>
       </c>
       <c r="C56" t="n">
-        <v>98.97</v>
+        <v>44.5</v>
       </c>
       <c r="D56" t="n">
-        <v>4.41</v>
+        <v>3.95</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>NBIFIN</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1868.6</v>
+        <v>33.71</v>
       </c>
       <c r="C57" t="n">
-        <v>1950</v>
+        <v>35</v>
       </c>
       <c r="D57" t="n">
-        <v>4.36</v>
+        <v>3.83</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>MBLINFRA</t>
+          <t>WIPL</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>28.66</v>
+        <v>152.5</v>
       </c>
       <c r="C58" t="n">
-        <v>29.9</v>
+        <v>158.3</v>
       </c>
       <c r="D58" t="n">
-        <v>4.33</v>
+        <v>3.8</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>THACKER</t>
+          <t>BIRLACABLE</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1435.2</v>
+        <v>224.46</v>
       </c>
       <c r="C59" t="n">
-        <v>1497</v>
+        <v>233</v>
       </c>
       <c r="D59" t="n">
-        <v>4.31</v>
+        <v>3.8</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>6.98</v>
+        <v>43.25</v>
       </c>
       <c r="C60" t="n">
-        <v>7.28</v>
+        <v>44.87</v>
       </c>
       <c r="D60" t="n">
-        <v>4.3</v>
+        <v>3.75</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SONAMLTD</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>57.08</v>
+        <v>8.09</v>
       </c>
       <c r="C61" t="n">
-        <v>59.5</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="D61" t="n">
-        <v>4.24</v>
+        <v>3.71</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>EMMIL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.48</v>
+        <v>124</v>
       </c>
       <c r="C62" t="n">
-        <v>0.5</v>
+        <v>128.55</v>
       </c>
       <c r="D62" t="n">
-        <v>4.17</v>
+        <v>3.67</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>HARRMALAYA</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.24</v>
+        <v>197.79</v>
       </c>
       <c r="C63" t="n">
-        <v>0.25</v>
+        <v>205</v>
       </c>
       <c r="D63" t="n">
-        <v>4.17</v>
+        <v>3.65</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>FCSSOFT</t>
+          <t>EMKAY</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1.72</v>
+        <v>297.15</v>
       </c>
       <c r="C64" t="n">
-        <v>1.79</v>
+        <v>308</v>
       </c>
       <c r="D64" t="n">
-        <v>4.07</v>
+        <v>3.65</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>ODIGMA</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>6.92</v>
+        <v>20.46</v>
       </c>
       <c r="C65" t="n">
-        <v>7.2</v>
+        <v>21.2</v>
       </c>
       <c r="D65" t="n">
-        <v>4.05</v>
+        <v>3.62</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>GENSOL</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>5.01</v>
+        <v>21.82</v>
       </c>
       <c r="C66" t="n">
-        <v>5.21</v>
+        <v>22.6</v>
       </c>
       <c r="D66" t="n">
-        <v>3.99</v>
+        <v>3.57</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>GOLDENTOBC</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>7.31</v>
+        <v>25.5</v>
       </c>
       <c r="C67" t="n">
-        <v>7.6</v>
+        <v>26.4</v>
       </c>
       <c r="D67" t="n">
-        <v>3.97</v>
+        <v>3.53</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>20.15</v>
+        <v>6.09</v>
       </c>
       <c r="C68" t="n">
-        <v>20.95</v>
+        <v>6.3</v>
       </c>
       <c r="D68" t="n">
-        <v>3.97</v>
+        <v>3.45</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>RELCHEMQ</t>
+          <t>GVT&amp;D</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>121.11</v>
+        <v>4964.5</v>
       </c>
       <c r="C69" t="n">
-        <v>125.9</v>
+        <v>5134</v>
       </c>
       <c r="D69" t="n">
-        <v>3.96</v>
+        <v>3.41</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LASA</t>
+          <t>DAMODARIND</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>7.68</v>
+        <v>30.87</v>
       </c>
       <c r="C70" t="n">
-        <v>7.98</v>
+        <v>31.9</v>
       </c>
       <c r="D70" t="n">
-        <v>3.91</v>
+        <v>3.34</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>AYMSYNTEX</t>
+          <t>AKSHARCHEM</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>223.99</v>
+        <v>228.15</v>
       </c>
       <c r="C71" t="n">
-        <v>232.7</v>
+        <v>235.7</v>
       </c>
       <c r="D71" t="n">
-        <v>3.89</v>
+        <v>3.31</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BTTL</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>37.36</v>
+        <v>1102.8</v>
       </c>
       <c r="C72" t="n">
-        <v>38.8</v>
+        <v>1139</v>
       </c>
       <c r="D72" t="n">
-        <v>3.85</v>
+        <v>3.28</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>AAKASH</t>
+          <t>URAVIDEF</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>9.380000000000001</v>
+        <v>115.81</v>
       </c>
       <c r="C73" t="n">
-        <v>9.74</v>
+        <v>119.6</v>
       </c>
       <c r="D73" t="n">
-        <v>3.84</v>
+        <v>3.27</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>UMAEXPORTS</t>
+          <t>BRANDMAN</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>25.19</v>
+        <v>154.9</v>
       </c>
       <c r="C74" t="n">
-        <v>26.15</v>
+        <v>159.9</v>
       </c>
       <c r="D74" t="n">
-        <v>3.81</v>
+        <v>3.23</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>PRIMECAB</t>
+          <t>SUPREMEENG</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>107.9</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="C75" t="n">
-        <v>112</v>
+        <v>0.97</v>
       </c>
       <c r="D75" t="n">
-        <v>3.8</v>
+        <v>3.19</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>EMKAY</t>
+          <t>KSR</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>247.63</v>
+        <v>33.42</v>
       </c>
       <c r="C76" t="n">
-        <v>257</v>
+        <v>34.48</v>
       </c>
       <c r="D76" t="n">
-        <v>3.78</v>
+        <v>3.17</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>COCKERILL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>29.05</v>
+        <v>9112</v>
       </c>
       <c r="C77" t="n">
-        <v>30.1</v>
+        <v>9400</v>
       </c>
       <c r="D77" t="n">
-        <v>3.61</v>
+        <v>3.16</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>46.24</v>
+        <v>24.09</v>
       </c>
       <c r="C78" t="n">
-        <v>47.9</v>
+        <v>24.85</v>
       </c>
       <c r="D78" t="n">
-        <v>3.59</v>
+        <v>3.15</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SVLL</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>655.6</v>
+        <v>6.69</v>
       </c>
       <c r="C79" t="n">
-        <v>679</v>
+        <v>6.9</v>
       </c>
       <c r="D79" t="n">
-        <v>3.57</v>
+        <v>3.14</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SERVOTECH</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>100.91</v>
+        <v>669.25</v>
       </c>
       <c r="C80" t="n">
-        <v>104.5</v>
+        <v>690</v>
       </c>
       <c r="D80" t="n">
-        <v>3.56</v>
+        <v>3.1</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SHANTI</t>
+          <t>AMJLAND</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>6.51</v>
+        <v>36.84</v>
       </c>
       <c r="C81" t="n">
-        <v>6.74</v>
+        <v>37.98</v>
       </c>
       <c r="D81" t="n">
-        <v>3.53</v>
+        <v>3.09</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>INTENTECH</t>
+          <t>FLEXITUFF</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>95.48</v>
+        <v>6.89</v>
       </c>
       <c r="C82" t="n">
-        <v>98.8</v>
+        <v>7.1</v>
       </c>
       <c r="D82" t="n">
-        <v>3.48</v>
+        <v>3.05</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SILLYMONKS</t>
+          <t>LAMOSAIC</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>17.01</v>
+        <v>29.7</v>
       </c>
       <c r="C83" t="n">
-        <v>17.6</v>
+        <v>30.6</v>
       </c>
       <c r="D83" t="n">
-        <v>3.47</v>
+        <v>3.03</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>JISLDVREQS</t>
+          <t>AEPL</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>22.6</v>
+        <v>16.25</v>
       </c>
       <c r="C84" t="n">
-        <v>23.38</v>
+        <v>16.74</v>
       </c>
       <c r="D84" t="n">
-        <v>3.45</v>
+        <v>3.02</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>BLBLIMITED</t>
+          <t>BPL</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>17.31</v>
+        <v>52.37</v>
       </c>
       <c r="C85" t="n">
-        <v>17.9</v>
+        <v>53.9</v>
       </c>
       <c r="D85" t="n">
-        <v>3.41</v>
+        <v>2.92</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>AHLADA</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>41.2</v>
+        <v>107.85</v>
       </c>
       <c r="C86" t="n">
-        <v>42.6</v>
+        <v>110.98</v>
       </c>
       <c r="D86" t="n">
-        <v>3.4</v>
+        <v>2.9</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SUBEXLTD</t>
+          <t>CONSOFINVT</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>10.69</v>
+        <v>242.97</v>
       </c>
       <c r="C87" t="n">
-        <v>11.05</v>
+        <v>249.94</v>
       </c>
       <c r="D87" t="n">
-        <v>3.37</v>
+        <v>2.87</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>BIRLAPREC</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>4324.4</v>
+        <v>38.76</v>
       </c>
       <c r="C88" t="n">
-        <v>4470</v>
+        <v>39.84</v>
       </c>
       <c r="D88" t="n">
-        <v>3.37</v>
+        <v>2.79</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>4.81</v>
+        <v>0.36</v>
       </c>
       <c r="C89" t="n">
-        <v>4.97</v>
+        <v>0.37</v>
       </c>
       <c r="D89" t="n">
-        <v>3.33</v>
+        <v>2.78</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>EPACKPEB</t>
+          <t>KAVDEFENCE</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>187.64</v>
+        <v>60.33</v>
       </c>
       <c r="C90" t="n">
-        <v>193.87</v>
+        <v>62</v>
       </c>
       <c r="D90" t="n">
-        <v>3.32</v>
+        <v>2.77</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CLEDUCATE</t>
+          <t>KEYFINSERV</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>46.47</v>
+        <v>251.8</v>
       </c>
       <c r="C91" t="n">
-        <v>47.99</v>
+        <v>258.75</v>
       </c>
       <c r="D91" t="n">
-        <v>3.27</v>
+        <v>2.76</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>UFBL</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>6.2</v>
+        <v>474.85</v>
       </c>
       <c r="C92" t="n">
-        <v>6.4</v>
+        <v>487.7</v>
       </c>
       <c r="D92" t="n">
-        <v>3.23</v>
+        <v>2.71</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>VISACHROME</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>591.05</v>
+        <v>52.58</v>
       </c>
       <c r="C93" t="n">
-        <v>610</v>
+        <v>53.99</v>
       </c>
       <c r="D93" t="n">
-        <v>3.21</v>
+        <v>2.68</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>HBESD</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>72.38</v>
+        <v>4.87</v>
       </c>
       <c r="C94" t="n">
-        <v>74.7</v>
+        <v>5</v>
       </c>
       <c r="D94" t="n">
-        <v>3.21</v>
+        <v>2.67</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>61.59</v>
+        <v>1806.2</v>
       </c>
       <c r="C95" t="n">
-        <v>63.56</v>
+        <v>1854</v>
       </c>
       <c r="D95" t="n">
-        <v>3.2</v>
+        <v>2.65</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>NILASPACES</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>12.84</v>
+        <v>45.79</v>
       </c>
       <c r="C96" t="n">
-        <v>13.25</v>
+        <v>47</v>
       </c>
       <c r="D96" t="n">
-        <v>3.19</v>
+        <v>2.64</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CARTRADE</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1795</v>
+        <v>1.54</v>
       </c>
       <c r="C97" t="n">
-        <v>1852</v>
+        <v>1.58</v>
       </c>
       <c r="D97" t="n">
-        <v>3.18</v>
+        <v>2.6</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>VIPULLTD</t>
+          <t>IWP</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>8.9</v>
+        <v>34.13</v>
       </c>
       <c r="C98" t="n">
-        <v>9.18</v>
+        <v>35</v>
       </c>
       <c r="D98" t="n">
-        <v>3.15</v>
+        <v>2.55</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>DCMSRIND</t>
+          <t>SBGLP</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>36.84</v>
+        <v>25.99</v>
       </c>
       <c r="C99" t="n">
-        <v>38</v>
+        <v>26.65</v>
       </c>
       <c r="D99" t="n">
-        <v>3.15</v>
+        <v>2.54</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PREMCO</t>
+          <t>GENUSPAPER</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>370.4</v>
+        <v>12.44</v>
       </c>
       <c r="C100" t="n">
-        <v>381.95</v>
+        <v>12.75</v>
       </c>
       <c r="D100" t="n">
-        <v>3.12</v>
+        <v>2.49</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>THOMASCOTT</t>
+          <t>SRTL</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>278.4</v>
+        <v>41.97</v>
       </c>
       <c r="C101" t="n">
-        <v>287</v>
+        <v>43</v>
       </c>
       <c r="D101" t="n">
-        <v>3.09</v>
+        <v>2.45</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SHEMAROO</t>
+          <t>ANTELOPUS</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>105.45</v>
+        <v>871.8</v>
       </c>
       <c r="C102" t="n">
-        <v>108.7</v>
+        <v>892.95</v>
       </c>
       <c r="D102" t="n">
-        <v>3.08</v>
+        <v>2.43</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ADVAIT</t>
+          <t>RELCHEMQ</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>1972.4</v>
+        <v>121.06</v>
       </c>
       <c r="C103" t="n">
-        <v>2032.7</v>
+        <v>124</v>
       </c>
       <c r="D103" t="n">
-        <v>3.06</v>
+        <v>2.43</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>MOLDTECH</t>
+          <t>TECILCHEM</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>118.4</v>
+        <v>11.62</v>
       </c>
       <c r="C104" t="n">
-        <v>122</v>
+        <v>11.9</v>
       </c>
       <c r="D104" t="n">
-        <v>3.04</v>
+        <v>2.41</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>INSPIRISYS</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>125.1</v>
+        <v>514.6</v>
       </c>
       <c r="C105" t="n">
-        <v>128.9</v>
+        <v>527</v>
       </c>
       <c r="D105" t="n">
-        <v>3.04</v>
+        <v>2.41</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>1.98</v>
+        <v>198.59</v>
       </c>
       <c r="C106" t="n">
-        <v>2.04</v>
+        <v>203.33</v>
       </c>
       <c r="D106" t="n">
-        <v>3.03</v>
+        <v>2.39</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>VALIANTLAB</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>76.76000000000001</v>
+        <v>0.42</v>
       </c>
       <c r="C107" t="n">
-        <v>79</v>
+        <v>0.43</v>
       </c>
       <c r="D107" t="n">
-        <v>2.92</v>
+        <v>2.38</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>KOHINOOR</t>
+          <t>CNL</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>25.07</v>
+        <v>629.95</v>
       </c>
       <c r="C108" t="n">
-        <v>25.8</v>
+        <v>644.9</v>
       </c>
       <c r="D108" t="n">
-        <v>2.91</v>
+        <v>2.37</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>AMBALALSA</t>
+          <t>BCG</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>37.3</v>
+        <v>11.04</v>
       </c>
       <c r="C109" t="n">
-        <v>38.38</v>
+        <v>11.3</v>
       </c>
       <c r="D109" t="n">
-        <v>2.9</v>
+        <v>2.36</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>PRECOT</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>68.03</v>
+        <v>733.55</v>
       </c>
       <c r="C110" t="n">
-        <v>70</v>
+        <v>750.55</v>
       </c>
       <c r="D110" t="n">
-        <v>2.9</v>
+        <v>2.32</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ANTELOPUS</t>
+          <t>MANOMAY</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>854.2</v>
+        <v>173.97</v>
       </c>
       <c r="C111" t="n">
-        <v>879</v>
+        <v>178</v>
       </c>
       <c r="D111" t="n">
-        <v>2.9</v>
+        <v>2.32</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>13.55</v>
+        <v>23.24</v>
       </c>
       <c r="C112" t="n">
-        <v>13.94</v>
+        <v>23.78</v>
       </c>
       <c r="D112" t="n">
-        <v>2.88</v>
+        <v>2.32</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>MODIRUBBER</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.35</v>
+        <v>124.91</v>
       </c>
       <c r="C113" t="n">
-        <v>0.36</v>
+        <v>127.8</v>
       </c>
       <c r="D113" t="n">
-        <v>2.86</v>
+        <v>2.31</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CENTEXT</t>
+          <t>BLUESTONE</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>19.34</v>
+        <v>508.25</v>
       </c>
       <c r="C114" t="n">
-        <v>19.89</v>
+        <v>520</v>
       </c>
       <c r="D114" t="n">
-        <v>2.84</v>
+        <v>2.31</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>VALUE360</t>
+          <t>SUVIDHAA</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>70.59999999999999</v>
+        <v>2.62</v>
       </c>
       <c r="C115" t="n">
-        <v>72.59999999999999</v>
+        <v>2.68</v>
       </c>
       <c r="D115" t="n">
-        <v>2.83</v>
+        <v>2.29</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>TAMBOLIIN</t>
+          <t>JMA</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>180</v>
+        <v>87.87</v>
       </c>
       <c r="C116" t="n">
-        <v>185</v>
+        <v>89.88</v>
       </c>
       <c r="D116" t="n">
-        <v>2.78</v>
+        <v>2.29</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>FOCUS</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>42.82</v>
+        <v>92.61</v>
       </c>
       <c r="C117" t="n">
-        <v>44</v>
+        <v>94.7</v>
       </c>
       <c r="D117" t="n">
-        <v>2.76</v>
+        <v>2.26</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>BORORENEW</t>
+          <t>VISHWARAJ</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>501.35</v>
+        <v>5.75</v>
       </c>
       <c r="C118" t="n">
-        <v>515.15</v>
+        <v>5.88</v>
       </c>
       <c r="D118" t="n">
-        <v>2.75</v>
+        <v>2.26</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CORDSCABLE</t>
+          <t>SUNLITE</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>223.04</v>
+        <v>440.05</v>
       </c>
       <c r="C119" t="n">
-        <v>228.99</v>
+        <v>449.85</v>
       </c>
       <c r="D119" t="n">
-        <v>2.67</v>
+        <v>2.23</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>OBCL</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>6.04</v>
+        <v>50.87</v>
       </c>
       <c r="C120" t="n">
-        <v>6.2</v>
+        <v>52</v>
       </c>
       <c r="D120" t="n">
-        <v>2.65</v>
+        <v>2.22</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>UFBL</t>
+          <t>VIPCLOTHNG</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>487.2</v>
+        <v>25.82</v>
       </c>
       <c r="C121" t="n">
-        <v>499.95</v>
+        <v>26.39</v>
       </c>
       <c r="D121" t="n">
-        <v>2.62</v>
+        <v>2.21</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>KELLTONTEC</t>
+          <t>RILINFRA</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>16.82</v>
+        <v>36.6</v>
       </c>
       <c r="C122" t="n">
-        <v>17.26</v>
+        <v>37.4</v>
       </c>
       <c r="D122" t="n">
-        <v>2.62</v>
+        <v>2.19</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>NIRAJ</t>
+          <t>GFLLIMITED</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>28.73</v>
+        <v>46.48</v>
       </c>
       <c r="C123" t="n">
-        <v>29.47</v>
+        <v>47.5</v>
       </c>
       <c r="D123" t="n">
-        <v>2.58</v>
+        <v>2.19</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>STEELCITY</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>24.47</v>
+        <v>76.92</v>
       </c>
       <c r="C124" t="n">
-        <v>25.1</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="D124" t="n">
-        <v>2.57</v>
+        <v>2.18</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>FLFL</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>931.25</v>
+        <v>1.39</v>
       </c>
       <c r="C125" t="n">
-        <v>955</v>
+        <v>1.42</v>
       </c>
       <c r="D125" t="n">
-        <v>2.55</v>
+        <v>2.16</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>DBSTOCKBRO</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>34.09</v>
+        <v>19.47</v>
       </c>
       <c r="C126" t="n">
-        <v>34.95</v>
+        <v>19.89</v>
       </c>
       <c r="D126" t="n">
-        <v>2.52</v>
+        <v>2.16</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>43.8</v>
+        <v>6.94</v>
       </c>
       <c r="C127" t="n">
-        <v>44.89</v>
+        <v>7.09</v>
       </c>
       <c r="D127" t="n">
-        <v>2.49</v>
+        <v>2.16</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>CEREBRAINT</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.8100000000000001</v>
+        <v>3.28</v>
       </c>
       <c r="C128" t="n">
-        <v>0.83</v>
+        <v>3.35</v>
       </c>
       <c r="D128" t="n">
-        <v>2.47</v>
+        <v>2.13</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>FERMENTA</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>312.35</v>
+        <v>185</v>
       </c>
       <c r="C129" t="n">
-        <v>320</v>
+        <v>188.9</v>
       </c>
       <c r="D129" t="n">
-        <v>2.45</v>
+        <v>2.11</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>EFORCE</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>2.46</v>
+        <v>21.6</v>
       </c>
       <c r="C130" t="n">
-        <v>2.52</v>
+        <v>22.05</v>
       </c>
       <c r="D130" t="n">
-        <v>2.44</v>
+        <v>2.08</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>JSLL</t>
+          <t>HDIL</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>590.6</v>
+        <v>1.92</v>
       </c>
       <c r="C131" t="n">
-        <v>605</v>
+        <v>1.96</v>
       </c>
       <c r="D131" t="n">
-        <v>2.44</v>
+        <v>2.08</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>TRACXN</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>31.72</v>
+        <v>6.78</v>
       </c>
       <c r="C132" t="n">
-        <v>32.49</v>
+        <v>6.92</v>
       </c>
       <c r="D132" t="n">
-        <v>2.43</v>
+        <v>2.06</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>0.42</v>
+        <v>1.97</v>
       </c>
       <c r="C133" t="n">
-        <v>0.43</v>
+        <v>2.01</v>
       </c>
       <c r="D133" t="n">
-        <v>2.38</v>
+        <v>2.03</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ORBTEXP</t>
+          <t>ANONDITA</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>178.74</v>
+        <v>1117.35</v>
       </c>
       <c r="C134" t="n">
-        <v>183</v>
+        <v>1139.9</v>
       </c>
       <c r="D134" t="n">
-        <v>2.38</v>
+        <v>2.02</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>10.92</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="C135" t="n">
-        <v>11.18</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="D135" t="n">
-        <v>2.38</v>
+        <v>2.01</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ZODIAC</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>287.95</v>
+        <v>40</v>
       </c>
       <c r="C136" t="n">
-        <v>294.75</v>
+        <v>40.8</v>
       </c>
       <c r="D136" t="n">
-        <v>2.36</v>
+        <v>2</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ELANTAS</t>
+          <t>SETUINFRA</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>9479</v>
+        <v>0.5</v>
       </c>
       <c r="C137" t="n">
-        <v>9701</v>
+        <v>0.51</v>
       </c>
       <c r="D137" t="n">
-        <v>2.34</v>
+        <v>2</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>MOKSH</t>
+          <t>RUDRA</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>11.7</v>
+        <v>18.13</v>
       </c>
       <c r="C138" t="n">
-        <v>11.97</v>
+        <v>18.49</v>
       </c>
       <c r="D138" t="n">
-        <v>2.31</v>
+        <v>1.99</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>WORTHPERI</t>
+          <t>PIONEEREMB</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>128.91</v>
+        <v>24.44</v>
       </c>
       <c r="C139" t="n">
-        <v>131.89</v>
+        <v>24.92</v>
       </c>
       <c r="D139" t="n">
-        <v>2.31</v>
+        <v>1.96</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>NITIRAJ</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>194.52</v>
+        <v>7.17</v>
       </c>
       <c r="C140" t="n">
-        <v>199</v>
+        <v>7.31</v>
       </c>
       <c r="D140" t="n">
-        <v>2.3</v>
+        <v>1.95</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>DEEDEV</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>654.2</v>
+        <v>490.45</v>
       </c>
       <c r="C141" t="n">
-        <v>669</v>
+        <v>500</v>
       </c>
       <c r="D141" t="n">
-        <v>2.26</v>
+        <v>1.95</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>TERASOFT</t>
+          <t>ITDC</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>430.1</v>
+        <v>535.6</v>
       </c>
       <c r="C142" t="n">
-        <v>439.7</v>
+        <v>546</v>
       </c>
       <c r="D142" t="n">
-        <v>2.23</v>
+        <v>1.94</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>UNIMECH</t>
+          <t>SUTLEJTEX</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>993.15</v>
+        <v>35.22</v>
       </c>
       <c r="C143" t="n">
-        <v>1014.95</v>
+        <v>35.9</v>
       </c>
       <c r="D143" t="n">
-        <v>2.2</v>
+        <v>1.93</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>DEVIT</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>28.87</v>
+        <v>17.15</v>
       </c>
       <c r="C144" t="n">
-        <v>29.5</v>
+        <v>17.48</v>
       </c>
       <c r="D144" t="n">
-        <v>2.18</v>
+        <v>1.92</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>UMAEXPORTS</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>8.24</v>
+        <v>25.5</v>
       </c>
       <c r="C145" t="n">
-        <v>8.42</v>
+        <v>25.99</v>
       </c>
       <c r="D145" t="n">
-        <v>2.18</v>
+        <v>1.92</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>HEXATRADEX</t>
+          <t>UNIDT</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>161.13</v>
+        <v>250.22</v>
       </c>
       <c r="C146" t="n">
-        <v>164.64</v>
+        <v>254.97</v>
       </c>
       <c r="D146" t="n">
-        <v>2.18</v>
+        <v>1.9</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ALKALI</t>
+          <t>SOUTHWEST</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>97.86</v>
+        <v>262.5</v>
       </c>
       <c r="C147" t="n">
-        <v>99.98</v>
+        <v>267.5</v>
       </c>
       <c r="D147" t="n">
-        <v>2.17</v>
+        <v>1.9</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>DANISH</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>2.31</v>
+        <v>896.05</v>
       </c>
       <c r="C148" t="n">
-        <v>2.36</v>
+        <v>913</v>
       </c>
       <c r="D148" t="n">
-        <v>2.16</v>
+        <v>1.89</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CEREBRAINT</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>3.26</v>
+        <v>43.78</v>
       </c>
       <c r="C149" t="n">
-        <v>3.33</v>
+        <v>44.6</v>
       </c>
       <c r="D149" t="n">
-        <v>2.15</v>
+        <v>1.87</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>RUCHIRA</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>115.46</v>
+        <v>0.55</v>
       </c>
       <c r="C150" t="n">
-        <v>117.9</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D150" t="n">
-        <v>2.11</v>
+        <v>1.82</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>HYBRIDFIN</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>7.69</v>
+        <v>16.69</v>
       </c>
       <c r="C151" t="n">
-        <v>7.85</v>
+        <v>16.99</v>
       </c>
       <c r="D151" t="n">
-        <v>2.08</v>
+        <v>1.8</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>MADHAV</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>485.4</v>
+        <v>37.77</v>
       </c>
       <c r="C152" t="n">
-        <v>495.5</v>
+        <v>38.44</v>
       </c>
       <c r="D152" t="n">
-        <v>2.08</v>
+        <v>1.77</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>PRAKASHSTL</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>4.35</v>
+        <v>1.13</v>
       </c>
       <c r="C153" t="n">
-        <v>4.44</v>
+        <v>1.15</v>
       </c>
       <c r="D153" t="n">
-        <v>2.07</v>
+        <v>1.77</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>CENTEXT</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>6.32</v>
+        <v>19.56</v>
       </c>
       <c r="C154" t="n">
-        <v>6.45</v>
+        <v>19.9</v>
       </c>
       <c r="D154" t="n">
-        <v>2.06</v>
+        <v>1.74</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>ALANKIT</t>
+          <t>BAJEL</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>8.42</v>
+        <v>199.93</v>
       </c>
       <c r="C155" t="n">
-        <v>8.59</v>
+        <v>203.38</v>
       </c>
       <c r="D155" t="n">
-        <v>2.02</v>
+        <v>1.73</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>FMNL</t>
+          <t>JISLJALEQS</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>10.9</v>
+        <v>29.12</v>
       </c>
       <c r="C156" t="n">
-        <v>11.12</v>
+        <v>29.62</v>
       </c>
       <c r="D156" t="n">
-        <v>2.02</v>
+        <v>1.72</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>MTARTECH</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>7216</v>
+        <v>5.29</v>
       </c>
       <c r="C157" t="n">
-        <v>7360.5</v>
+        <v>5.38</v>
       </c>
       <c r="D157" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>EFFWA</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>0.5</v>
+        <v>300.9</v>
       </c>
       <c r="C158" t="n">
-        <v>0.51</v>
+        <v>306</v>
       </c>
       <c r="D158" t="n">
-        <v>2</v>
+        <v>1.69</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>NORBTEAEXP</t>
+          <t>SHREERAMA</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>82.84999999999999</v>
+        <v>44.25</v>
       </c>
       <c r="C159" t="n">
-        <v>84.5</v>
+        <v>45</v>
       </c>
       <c r="D159" t="n">
-        <v>1.99</v>
+        <v>1.69</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>MADHAVBAUG</t>
+          <t>URJA</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>186.8</v>
+        <v>10.81</v>
       </c>
       <c r="C160" t="n">
-        <v>190.5</v>
+        <v>10.99</v>
       </c>
       <c r="D160" t="n">
-        <v>1.98</v>
+        <v>1.67</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>JNKINDIA</t>
+          <t>MBLINFRA</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>361.4</v>
+        <v>28.18</v>
       </c>
       <c r="C161" t="n">
-        <v>368.55</v>
+        <v>28.65</v>
       </c>
       <c r="D161" t="n">
-        <v>1.98</v>
+        <v>1.67</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>23.24</v>
+        <v>418.1</v>
       </c>
       <c r="C162" t="n">
-        <v>23.7</v>
+        <v>424.95</v>
       </c>
       <c r="D162" t="n">
-        <v>1.98</v>
+        <v>1.64</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>HMVL</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>858.95</v>
+        <v>76.11</v>
       </c>
       <c r="C163" t="n">
-        <v>876</v>
+        <v>77.34999999999999</v>
       </c>
       <c r="D163" t="n">
-        <v>1.98</v>
+        <v>1.63</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>GOCOLORS</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>336.05</v>
+        <v>23.6</v>
       </c>
       <c r="C164" t="n">
-        <v>342.7</v>
+        <v>23.98</v>
       </c>
       <c r="D164" t="n">
-        <v>1.98</v>
+        <v>1.61</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>HEADSUP</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>7.12</v>
+        <v>418.15</v>
       </c>
       <c r="C165" t="n">
-        <v>7.26</v>
+        <v>424.9</v>
       </c>
       <c r="D165" t="n">
-        <v>1.97</v>
+        <v>1.61</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>CAPITALSFB</t>
+          <t>POWERICA</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>268.7</v>
+        <v>542.3</v>
       </c>
       <c r="C166" t="n">
-        <v>274</v>
+        <v>551</v>
       </c>
       <c r="D166" t="n">
-        <v>1.97</v>
+        <v>1.6</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>TVTODAY</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>11.22</v>
+        <v>111.41</v>
       </c>
       <c r="C167" t="n">
-        <v>11.44</v>
+        <v>113.19</v>
       </c>
       <c r="D167" t="n">
-        <v>1.96</v>
+        <v>1.6</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>OSELDEVICE</t>
+          <t>IVC</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>471.7</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="C168" t="n">
-        <v>480.95</v>
+        <v>8.25</v>
       </c>
       <c r="D168" t="n">
-        <v>1.96</v>
+        <v>1.6</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>IFBAGRO</t>
+          <t>HCL-INSYS</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>978.7</v>
+        <v>13.11</v>
       </c>
       <c r="C169" t="n">
-        <v>997.7</v>
+        <v>13.32</v>
       </c>
       <c r="D169" t="n">
-        <v>1.94</v>
+        <v>1.6</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>KANANIIND</t>
+          <t>HEXATRADEX</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>1.55</v>
+        <v>162.1</v>
       </c>
       <c r="C170" t="n">
-        <v>1.58</v>
+        <v>164.7</v>
       </c>
       <c r="D170" t="n">
-        <v>1.94</v>
+        <v>1.6</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>UGARSUGAR</t>
+          <t>INDOWIND</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>40.18</v>
+        <v>9.43</v>
       </c>
       <c r="C171" t="n">
-        <v>40.96</v>
+        <v>9.58</v>
       </c>
       <c r="D171" t="n">
-        <v>1.94</v>
+        <v>1.59</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>RAJRILTD</t>
+          <t>CONFIPET</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>20.25</v>
+        <v>76.79000000000001</v>
       </c>
       <c r="C172" t="n">
-        <v>20.64</v>
+        <v>78</v>
       </c>
       <c r="D172" t="n">
-        <v>1.93</v>
+        <v>1.58</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>TARACHAND</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>60.24</v>
+        <v>139.82</v>
       </c>
       <c r="C173" t="n">
-        <v>61.4</v>
+        <v>142</v>
       </c>
       <c r="D173" t="n">
-        <v>1.93</v>
+        <v>1.56</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>WANBURY</t>
+          <t>MSPL</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>258</v>
+        <v>41.15</v>
       </c>
       <c r="C174" t="n">
-        <v>262.95</v>
+        <v>41.79</v>
       </c>
       <c r="D174" t="n">
-        <v>1.92</v>
+        <v>1.56</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>JARO</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>54.34</v>
+        <v>596.6</v>
       </c>
       <c r="C175" t="n">
-        <v>55.38</v>
+        <v>605.85</v>
       </c>
       <c r="D175" t="n">
-        <v>1.91</v>
+        <v>1.55</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>NEWGEN</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>518.1</v>
+        <v>86.56</v>
       </c>
       <c r="C176" t="n">
-        <v>528</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="D176" t="n">
-        <v>1.91</v>
+        <v>1.55</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>PENINLAND</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>16.42</v>
+        <v>344.6</v>
       </c>
       <c r="C177" t="n">
-        <v>16.73</v>
+        <v>349.8</v>
       </c>
       <c r="D177" t="n">
-        <v>1.89</v>
+        <v>1.51</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>NRL</t>
+          <t>JUNIPER</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>65.56999999999999</v>
+        <v>194.11</v>
       </c>
       <c r="C178" t="n">
-        <v>66.81</v>
+        <v>196.98</v>
       </c>
       <c r="D178" t="n">
-        <v>1.89</v>
+        <v>1.48</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>GTL</t>
+          <t>KRITINUT</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>7.39</v>
+        <v>89.66</v>
       </c>
       <c r="C179" t="n">
-        <v>7.53</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="D179" t="n">
-        <v>1.89</v>
+        <v>1.48</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>UFO</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>170.12</v>
+        <v>73.79000000000001</v>
       </c>
       <c r="C180" t="n">
-        <v>173.3</v>
+        <v>74.88</v>
       </c>
       <c r="D180" t="n">
-        <v>1.87</v>
+        <v>1.48</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>HGM</t>
+          <t>POWERINDIA</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>61.65</v>
+        <v>35190</v>
       </c>
       <c r="C181" t="n">
-        <v>62.8</v>
+        <v>35705</v>
       </c>
       <c r="D181" t="n">
-        <v>1.87</v>
+        <v>1.46</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>DBOL</t>
+          <t>COMPUSOFT</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>112.72</v>
+        <v>13.78</v>
       </c>
       <c r="C182" t="n">
-        <v>114.8</v>
+        <v>13.98</v>
       </c>
       <c r="D182" t="n">
-        <v>1.85</v>
+        <v>1.45</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>RKSWAMY</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>19.97</v>
+        <v>98.09</v>
       </c>
       <c r="C183" t="n">
-        <v>20.34</v>
+        <v>99.5</v>
       </c>
       <c r="D183" t="n">
-        <v>1.85</v>
+        <v>1.44</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>VASWANI</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>0.54</v>
+        <v>58.95</v>
       </c>
       <c r="C184" t="n">
-        <v>0.55</v>
+        <v>59.8</v>
       </c>
       <c r="D184" t="n">
-        <v>1.85</v>
+        <v>1.44</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>SINGERIND</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>3.83</v>
+        <v>69.41</v>
       </c>
       <c r="C185" t="n">
-        <v>3.9</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="D185" t="n">
-        <v>1.83</v>
+        <v>1.43</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>INDOTECH</t>
+          <t>3IINFOLTD</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>2722.8</v>
+        <v>17.16</v>
       </c>
       <c r="C186" t="n">
-        <v>2772</v>
+        <v>17.4</v>
       </c>
       <c r="D186" t="n">
-        <v>1.81</v>
+        <v>1.4</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>PIGL</t>
+          <t>APCOTEXIND</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>98.23</v>
+        <v>498.45</v>
       </c>
       <c r="C187" t="n">
-        <v>100</v>
+        <v>505.4</v>
       </c>
       <c r="D187" t="n">
-        <v>1.8</v>
+        <v>1.39</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>MAYURUNIQ</t>
+          <t>UEL</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>745.25</v>
+        <v>141.92</v>
       </c>
       <c r="C188" t="n">
-        <v>758.7</v>
+        <v>143.89</v>
       </c>
       <c r="D188" t="n">
-        <v>1.8</v>
+        <v>1.39</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>NDLVENTURE</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>133.54</v>
+        <v>6.48</v>
       </c>
       <c r="C189" t="n">
-        <v>135.95</v>
+        <v>6.57</v>
       </c>
       <c r="D189" t="n">
-        <v>1.8</v>
+        <v>1.39</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>SEYAIND</t>
+          <t>GEECEE</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>14.99</v>
+        <v>325.45</v>
       </c>
       <c r="C190" t="n">
-        <v>15.26</v>
+        <v>329.9</v>
       </c>
       <c r="D190" t="n">
-        <v>1.8</v>
+        <v>1.37</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>BAGFILMS</t>
+          <t>GOLDTECH</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>5</v>
+        <v>43.06</v>
       </c>
       <c r="C191" t="n">
-        <v>5.09</v>
+        <v>43.65</v>
       </c>
       <c r="D191" t="n">
-        <v>1.8</v>
+        <v>1.37</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>DAVANGERE</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>323.2</v>
+        <v>3.64</v>
       </c>
       <c r="C192" t="n">
-        <v>329</v>
+        <v>3.69</v>
       </c>
       <c r="D192" t="n">
-        <v>1.79</v>
+        <v>1.37</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>SEMAC</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>335.05</v>
+        <v>14.64</v>
       </c>
       <c r="C193" t="n">
-        <v>341</v>
+        <v>14.84</v>
       </c>
       <c r="D193" t="n">
-        <v>1.78</v>
+        <v>1.37</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>ANUHPHR</t>
+          <t>BODALCHEM</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>75.53</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="C194" t="n">
-        <v>76.87</v>
+        <v>73.8</v>
       </c>
       <c r="D194" t="n">
-        <v>1.77</v>
+        <v>1.35</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>MUNISH</t>
+          <t>DREAMFOLKS</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>65.55</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="C195" t="n">
-        <v>66.7</v>
+        <v>74.98</v>
       </c>
       <c r="D195" t="n">
-        <v>1.75</v>
+        <v>1.34</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ESSENTIA</t>
+          <t>BOHRAIND</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>1.73</v>
+        <v>17.16</v>
       </c>
       <c r="C196" t="n">
-        <v>1.76</v>
+        <v>17.39</v>
       </c>
       <c r="D196" t="n">
-        <v>1.73</v>
+        <v>1.34</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>HTMEDIA</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>5.21</v>
+        <v>22.5</v>
       </c>
       <c r="C197" t="n">
-        <v>5.3</v>
+        <v>22.8</v>
       </c>
       <c r="D197" t="n">
-        <v>1.73</v>
+        <v>1.33</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>24.27</v>
+        <v>28.82</v>
       </c>
       <c r="C198" t="n">
-        <v>24.69</v>
+        <v>29.2</v>
       </c>
       <c r="D198" t="n">
-        <v>1.73</v>
+        <v>1.32</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>KANPRPLA</t>
+          <t>SABEVENTS</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>186.78</v>
+        <v>8.33</v>
       </c>
       <c r="C199" t="n">
-        <v>190</v>
+        <v>8.44</v>
       </c>
       <c r="D199" t="n">
-        <v>1.72</v>
+        <v>1.32</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>BLUECHIP</t>
+          <t>HIRECT</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>2.37</v>
+        <v>1118.3</v>
       </c>
       <c r="C200" t="n">
-        <v>2.41</v>
+        <v>1133</v>
       </c>
       <c r="D200" t="n">
-        <v>1.69</v>
+        <v>1.31</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>TRANSPEK</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>447.4</v>
+        <v>984.2</v>
       </c>
       <c r="C201" t="n">
-        <v>454.95</v>
+        <v>997</v>
       </c>
       <c r="D201" t="n">
-        <v>1.69</v>
+        <v>1.3</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-05 07:55 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ESSEN-RE3</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.04</v>
+        <v>180.52</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05</v>
+        <v>205</v>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>13.56</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RETAIL</t>
+          <t>ORTINGLOBE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>21.21</v>
+        <v>16.47</v>
       </c>
       <c r="C3" t="n">
-        <v>24.38</v>
+        <v>18.11</v>
       </c>
       <c r="D3" t="n">
-        <v>14.95</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TNTELE</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9.26</v>
+        <v>31.7</v>
       </c>
       <c r="C4" t="n">
-        <v>9.99</v>
+        <v>34.6</v>
       </c>
       <c r="D4" t="n">
-        <v>7.88</v>
+        <v>9.15</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MFML</t>
+          <t>BAFNAPH</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24.32</v>
+        <v>160.31</v>
       </c>
       <c r="C5" t="n">
-        <v>26.2</v>
+        <v>172.89</v>
       </c>
       <c r="D5" t="n">
-        <v>7.73</v>
+        <v>7.85</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AGARIND</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>419.4</v>
+        <v>5.07</v>
       </c>
       <c r="C6" t="n">
-        <v>450</v>
+        <v>5.45</v>
       </c>
       <c r="D6" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AVG-RE</t>
+          <t>RELIABLE</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3.28</v>
+        <v>137.78</v>
       </c>
       <c r="C7" t="n">
-        <v>3.5</v>
+        <v>148</v>
       </c>
       <c r="D7" t="n">
-        <v>6.71</v>
+        <v>7.42</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>VINYAS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15.52</v>
+        <v>1132.15</v>
       </c>
       <c r="C8" t="n">
-        <v>16.49</v>
+        <v>1200</v>
       </c>
       <c r="D8" t="n">
-        <v>6.25</v>
+        <v>5.99</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.16</v>
+        <v>16.7</v>
       </c>
       <c r="C9" t="n">
-        <v>0.17</v>
+        <v>17.55</v>
       </c>
       <c r="D9" t="n">
-        <v>6.25</v>
+        <v>5.09</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KIRANVYPAR</t>
+          <t>RELINFRA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>156.75</v>
+        <v>77.87</v>
       </c>
       <c r="C10" t="n">
-        <v>165.99</v>
+        <v>81.76000000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>5.89</v>
+        <v>5</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>IDEAFORGE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>35.01</v>
+        <v>900</v>
       </c>
       <c r="C11" t="n">
-        <v>37</v>
+        <v>945</v>
       </c>
       <c r="D11" t="n">
-        <v>5.68</v>
+        <v>5</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PKTEA</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>783.75</v>
+        <v>308.36</v>
       </c>
       <c r="C12" t="n">
-        <v>828</v>
+        <v>323.77</v>
       </c>
       <c r="D12" t="n">
-        <v>5.65</v>
+        <v>5</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>STRIDERS</t>
+          <t>PRAMARA</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>61.8</v>
+        <v>143.05</v>
       </c>
       <c r="C13" t="n">
-        <v>65.25</v>
+        <v>150.2</v>
       </c>
       <c r="D13" t="n">
-        <v>5.58</v>
+        <v>5</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>IL&amp;FSENGG</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>10.59</v>
+        <v>27.6</v>
       </c>
       <c r="C14" t="n">
-        <v>11.14</v>
+        <v>28.98</v>
       </c>
       <c r="D14" t="n">
-        <v>5.19</v>
+        <v>5</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MERCANTILE</t>
+          <t>PURPLEUTED</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>27.43</v>
+        <v>377</v>
       </c>
       <c r="C15" t="n">
-        <v>28.85</v>
+        <v>395.85</v>
       </c>
       <c r="D15" t="n">
-        <v>5.18</v>
+        <v>5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,14 +769,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IDEAFORGE</t>
+          <t>SICALLOG</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>857.15</v>
+        <v>68.8</v>
       </c>
       <c r="C16" t="n">
-        <v>900</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="D16" t="n">
         <v>5</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MASKINVEST</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>158</v>
+        <v>46.05</v>
       </c>
       <c r="C17" t="n">
-        <v>165.9</v>
+        <v>48.35</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TANKUP</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>865.45</v>
+        <v>1217.7</v>
       </c>
       <c r="C18" t="n">
-        <v>908.7</v>
+        <v>1278</v>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BAFNAPH</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>152.68</v>
+        <v>6.67</v>
       </c>
       <c r="C19" t="n">
-        <v>160.31</v>
+        <v>7</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>CEREBRAINT</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>329</v>
+        <v>3.44</v>
       </c>
       <c r="C20" t="n">
-        <v>345.45</v>
+        <v>3.61</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>4.94</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>UNIMECH</t>
+          <t>MCON</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1042.8</v>
+        <v>47.6</v>
       </c>
       <c r="C21" t="n">
-        <v>1094.9</v>
+        <v>49.95</v>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>4.94</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>293.68</v>
+        <v>2.25</v>
       </c>
       <c r="C22" t="n">
-        <v>308.36</v>
+        <v>2.36</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>4.89</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RELINFRA</t>
+          <t>ALLETEC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>74.17</v>
+        <v>143.9</v>
       </c>
       <c r="C23" t="n">
-        <v>77.87</v>
+        <v>150.9</v>
       </c>
       <c r="D23" t="n">
-        <v>4.99</v>
+        <v>4.86</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RNPL</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>79.09999999999999</v>
+        <v>5.57</v>
       </c>
       <c r="C24" t="n">
-        <v>83.05</v>
+        <v>5.84</v>
       </c>
       <c r="D24" t="n">
-        <v>4.99</v>
+        <v>4.85</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>UTLSOLAR</t>
+          <t>HIRECT</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>335.75</v>
+        <v>1137.8</v>
       </c>
       <c r="C25" t="n">
-        <v>352.5</v>
+        <v>1192.7</v>
       </c>
       <c r="D25" t="n">
-        <v>4.99</v>
+        <v>4.83</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1481.8</v>
+        <v>2.7</v>
       </c>
       <c r="C26" t="n">
-        <v>1555.8</v>
+        <v>2.83</v>
       </c>
       <c r="D26" t="n">
-        <v>4.99</v>
+        <v>4.81</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>136.25</v>
+        <v>5.69</v>
       </c>
       <c r="C27" t="n">
-        <v>143.05</v>
+        <v>5.96</v>
       </c>
       <c r="D27" t="n">
-        <v>4.99</v>
+        <v>4.75</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CLEDUCATE</t>
+          <t>MODISONLTD</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>48.79</v>
+        <v>345.45</v>
       </c>
       <c r="C28" t="n">
-        <v>51.22</v>
+        <v>361.6</v>
       </c>
       <c r="D28" t="n">
-        <v>4.98</v>
+        <v>4.68</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ORTINGLOBE</t>
+          <t>MAWANASUG</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>15.69</v>
+        <v>97.45</v>
       </c>
       <c r="C29" t="n">
-        <v>16.47</v>
+        <v>102</v>
       </c>
       <c r="D29" t="n">
-        <v>4.97</v>
+        <v>4.67</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BLUECOAST</t>
+          <t>QMSMEDI</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>30</v>
+        <v>87.8</v>
       </c>
       <c r="C30" t="n">
-        <v>31.48</v>
+        <v>91.84999999999999</v>
       </c>
       <c r="D30" t="n">
-        <v>4.93</v>
+        <v>4.61</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ALLETEC</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>137.05</v>
+        <v>6.41</v>
       </c>
       <c r="C31" t="n">
-        <v>143.8</v>
+        <v>6.7</v>
       </c>
       <c r="D31" t="n">
-        <v>4.93</v>
+        <v>4.52</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>DHRUV</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>43.9</v>
+        <v>27.56</v>
       </c>
       <c r="C32" t="n">
-        <v>46.05</v>
+        <v>28.8</v>
       </c>
       <c r="D32" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SEMAC</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>351.8</v>
+        <v>879.4</v>
       </c>
       <c r="C33" t="n">
-        <v>369</v>
+        <v>918.9</v>
       </c>
       <c r="D33" t="n">
-        <v>4.89</v>
+        <v>4.49</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>UHTL</t>
+          <t>PRECOT</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>90.95</v>
+        <v>765.65</v>
       </c>
       <c r="C34" t="n">
-        <v>95.40000000000001</v>
+        <v>800</v>
       </c>
       <c r="D34" t="n">
-        <v>4.89</v>
+        <v>4.49</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>SIKKO</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>25.22</v>
+        <v>4.05</v>
       </c>
       <c r="C35" t="n">
-        <v>26.45</v>
+        <v>4.23</v>
       </c>
       <c r="D35" t="n">
-        <v>4.88</v>
+        <v>4.44</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>VLINFRA</t>
+          <t>CAPTRUST</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>31.85</v>
+        <v>13.3</v>
       </c>
       <c r="C36" t="n">
-        <v>33.4</v>
+        <v>13.89</v>
       </c>
       <c r="D36" t="n">
-        <v>4.87</v>
+        <v>4.44</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>UNIINFO</t>
+          <t>BCG</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>11.35</v>
+        <v>11.59</v>
       </c>
       <c r="C37" t="n">
-        <v>11.9</v>
+        <v>12.1</v>
       </c>
       <c r="D37" t="n">
-        <v>4.85</v>
+        <v>4.4</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IZMO</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>869.15</v>
+        <v>40.86</v>
       </c>
       <c r="C38" t="n">
-        <v>910.9</v>
+        <v>42.65</v>
       </c>
       <c r="D38" t="n">
-        <v>4.8</v>
+        <v>4.38</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5.43</v>
+        <v>0.23</v>
       </c>
       <c r="C39" t="n">
-        <v>5.69</v>
+        <v>0.24</v>
       </c>
       <c r="D39" t="n">
-        <v>4.79</v>
+        <v>4.35</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ATLANTAELE</t>
+          <t>ITDC</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2050.1</v>
+        <v>589.15</v>
       </c>
       <c r="C40" t="n">
-        <v>2148</v>
+        <v>614</v>
       </c>
       <c r="D40" t="n">
-        <v>4.78</v>
+        <v>4.22</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>VITAL</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>52.5</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="C41" t="n">
-        <v>54.99</v>
+        <v>78</v>
       </c>
       <c r="D41" t="n">
-        <v>4.74</v>
+        <v>4.21</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DELTIC</t>
+          <t>AEPL</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>33.05</v>
+        <v>16.02</v>
       </c>
       <c r="C42" t="n">
-        <v>34.6</v>
+        <v>16.69</v>
       </c>
       <c r="D42" t="n">
-        <v>4.69</v>
+        <v>4.18</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ABANSENT</t>
+          <t>INNOVISION</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>26.74</v>
+        <v>285.1</v>
       </c>
       <c r="C43" t="n">
-        <v>27.99</v>
+        <v>297</v>
       </c>
       <c r="D43" t="n">
-        <v>4.67</v>
+        <v>4.17</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>AGARIND</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2.58</v>
+        <v>503.25</v>
       </c>
       <c r="C44" t="n">
-        <v>2.7</v>
+        <v>524</v>
       </c>
       <c r="D44" t="n">
-        <v>4.65</v>
+        <v>4.12</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>AUSOMENT</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>12.2</v>
+        <v>120.99</v>
       </c>
       <c r="C45" t="n">
-        <v>12.76</v>
+        <v>125.9</v>
       </c>
       <c r="D45" t="n">
-        <v>4.59</v>
+        <v>4.06</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>STLTECH</t>
+          <t>IRIS</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>620.6</v>
+        <v>243.1</v>
       </c>
       <c r="C46" t="n">
-        <v>649</v>
+        <v>252.8</v>
       </c>
       <c r="D46" t="n">
-        <v>4.58</v>
+        <v>3.99</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PRIZOR</t>
+          <t>MGEL</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>762.5</v>
+        <v>15.2</v>
       </c>
       <c r="C47" t="n">
-        <v>797.3</v>
+        <v>15.79</v>
       </c>
       <c r="D47" t="n">
-        <v>4.56</v>
+        <v>3.88</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TGL</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>23</v>
+        <v>5.49</v>
       </c>
       <c r="C48" t="n">
-        <v>24</v>
+        <v>5.7</v>
       </c>
       <c r="D48" t="n">
-        <v>4.35</v>
+        <v>3.83</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>ODIGMA</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>8.83</v>
+        <v>20.51</v>
       </c>
       <c r="C49" t="n">
-        <v>9.199999999999999</v>
+        <v>21.29</v>
       </c>
       <c r="D49" t="n">
-        <v>4.19</v>
+        <v>3.8</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>5.78</v>
+        <v>32.76</v>
       </c>
       <c r="C50" t="n">
-        <v>6.02</v>
+        <v>34</v>
       </c>
       <c r="D50" t="n">
-        <v>4.15</v>
+        <v>3.79</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>UMAEXPORTS</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>7.98</v>
+        <v>24.95</v>
       </c>
       <c r="C51" t="n">
-        <v>8.31</v>
+        <v>25.89</v>
       </c>
       <c r="D51" t="n">
-        <v>4.14</v>
+        <v>3.77</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SMLT</t>
+          <t>UNIHEALTH</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>71.77</v>
+        <v>438.5</v>
       </c>
       <c r="C52" t="n">
-        <v>74.7</v>
+        <v>455</v>
       </c>
       <c r="D52" t="n">
-        <v>4.08</v>
+        <v>3.76</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>DAMODARIND</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>9.609999999999999</v>
+        <v>30.39</v>
       </c>
       <c r="C53" t="n">
-        <v>10</v>
+        <v>31.49</v>
       </c>
       <c r="D53" t="n">
-        <v>4.06</v>
+        <v>3.62</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>NAGREEKEXP</t>
+          <t>SHALPAINTS</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>27.8</v>
+        <v>50.09</v>
       </c>
       <c r="C54" t="n">
-        <v>28.91</v>
+        <v>51.9</v>
       </c>
       <c r="D54" t="n">
-        <v>3.99</v>
+        <v>3.61</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TVVISION</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>5.29</v>
+        <v>3.92</v>
       </c>
       <c r="C55" t="n">
-        <v>5.5</v>
+        <v>4.06</v>
       </c>
       <c r="D55" t="n">
-        <v>3.97</v>
+        <v>3.57</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>UTLSOLAR</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>42.81</v>
+        <v>352.5</v>
       </c>
       <c r="C56" t="n">
-        <v>44.5</v>
+        <v>365</v>
       </c>
       <c r="D56" t="n">
-        <v>3.95</v>
+        <v>3.55</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>TVSSCS</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>33.71</v>
+        <v>122.65</v>
       </c>
       <c r="C57" t="n">
-        <v>35</v>
+        <v>127</v>
       </c>
       <c r="D57" t="n">
-        <v>3.83</v>
+        <v>3.55</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>WIPL</t>
+          <t>INDTERRAIN</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>152.5</v>
+        <v>32.59</v>
       </c>
       <c r="C58" t="n">
-        <v>158.3</v>
+        <v>33.74</v>
       </c>
       <c r="D58" t="n">
-        <v>3.8</v>
+        <v>3.53</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>SAPPL</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>224.46</v>
+        <v>270</v>
       </c>
       <c r="C59" t="n">
-        <v>233</v>
+        <v>279.5</v>
       </c>
       <c r="D59" t="n">
-        <v>3.8</v>
+        <v>3.52</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>43.25</v>
+        <v>35.26</v>
       </c>
       <c r="C60" t="n">
-        <v>44.87</v>
+        <v>36.5</v>
       </c>
       <c r="D60" t="n">
-        <v>3.75</v>
+        <v>3.52</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>GOKUL</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>8.09</v>
+        <v>40.43</v>
       </c>
       <c r="C61" t="n">
-        <v>8.390000000000001</v>
+        <v>41.85</v>
       </c>
       <c r="D61" t="n">
-        <v>3.71</v>
+        <v>3.51</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>EMMIL</t>
+          <t>PASUPTAC</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>124</v>
+        <v>68.11</v>
       </c>
       <c r="C62" t="n">
-        <v>128.55</v>
+        <v>70.5</v>
       </c>
       <c r="D62" t="n">
-        <v>3.67</v>
+        <v>3.51</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>HARRMALAYA</t>
+          <t>TNTELE</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>197.79</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="C63" t="n">
-        <v>205</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="D63" t="n">
-        <v>3.65</v>
+        <v>3.49</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>EMKAY</t>
+          <t>KDL</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>297.15</v>
+        <v>111.05</v>
       </c>
       <c r="C64" t="n">
-        <v>308</v>
+        <v>114.9</v>
       </c>
       <c r="D64" t="n">
-        <v>3.65</v>
+        <v>3.47</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ODIGMA</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>20.46</v>
+        <v>44.95</v>
       </c>
       <c r="C65" t="n">
-        <v>21.2</v>
+        <v>46.5</v>
       </c>
       <c r="D65" t="n">
-        <v>3.62</v>
+        <v>3.45</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>GENSOL</t>
+          <t>JNKINDIA</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>21.82</v>
+        <v>421.6</v>
       </c>
       <c r="C66" t="n">
-        <v>22.6</v>
+        <v>436</v>
       </c>
       <c r="D66" t="n">
-        <v>3.57</v>
+        <v>3.42</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GOLDENTOBC</t>
+          <t>URAVIDEF</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>25.5</v>
+        <v>115.12</v>
       </c>
       <c r="C67" t="n">
-        <v>26.4</v>
+        <v>119</v>
       </c>
       <c r="D67" t="n">
-        <v>3.53</v>
+        <v>3.37</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>MAYURUNIQ</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>6.09</v>
+        <v>734.4</v>
       </c>
       <c r="C68" t="n">
-        <v>6.3</v>
+        <v>759</v>
       </c>
       <c r="D68" t="n">
-        <v>3.45</v>
+        <v>3.35</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GVT&amp;D</t>
+          <t>BBTCL</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>4964.5</v>
+        <v>209.92</v>
       </c>
       <c r="C69" t="n">
-        <v>5134</v>
+        <v>216.9</v>
       </c>
       <c r="D69" t="n">
-        <v>3.41</v>
+        <v>3.33</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>DAMODARIND</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>30.87</v>
+        <v>44.54</v>
       </c>
       <c r="C70" t="n">
-        <v>31.9</v>
+        <v>46</v>
       </c>
       <c r="D70" t="n">
-        <v>3.34</v>
+        <v>3.28</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>AKSHARCHEM</t>
+          <t>KAVDEFENCE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>228.15</v>
+        <v>63.34</v>
       </c>
       <c r="C71" t="n">
-        <v>235.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="D71" t="n">
-        <v>3.31</v>
+        <v>3.25</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>DEVX</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1102.8</v>
+        <v>37.54</v>
       </c>
       <c r="C72" t="n">
-        <v>1139</v>
+        <v>38.76</v>
       </c>
       <c r="D72" t="n">
-        <v>3.28</v>
+        <v>3.25</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>URAVIDEF</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>115.81</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="C73" t="n">
-        <v>119.6</v>
+        <v>10.2</v>
       </c>
       <c r="D73" t="n">
-        <v>3.27</v>
+        <v>3.24</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BRANDMAN</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>154.9</v>
+        <v>10.13</v>
       </c>
       <c r="C74" t="n">
-        <v>159.9</v>
+        <v>10.45</v>
       </c>
       <c r="D74" t="n">
-        <v>3.23</v>
+        <v>3.16</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SUPREMEENG</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.9399999999999999</v>
+        <v>7.95</v>
       </c>
       <c r="C75" t="n">
-        <v>0.97</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D75" t="n">
-        <v>3.19</v>
+        <v>3.14</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>KSR</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>33.42</v>
+        <v>7.64</v>
       </c>
       <c r="C76" t="n">
-        <v>34.48</v>
+        <v>7.88</v>
       </c>
       <c r="D76" t="n">
-        <v>3.17</v>
+        <v>3.14</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>COCKERILL</t>
+          <t>SUPREMEENG</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>9112</v>
+        <v>0.96</v>
       </c>
       <c r="C77" t="n">
-        <v>9400</v>
+        <v>0.99</v>
       </c>
       <c r="D77" t="n">
-        <v>3.16</v>
+        <v>3.13</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>24.09</v>
+        <v>11.19</v>
       </c>
       <c r="C78" t="n">
-        <v>24.85</v>
+        <v>11.54</v>
       </c>
       <c r="D78" t="n">
-        <v>3.15</v>
+        <v>3.13</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>SCHNEIDER</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>6.69</v>
+        <v>1109.8</v>
       </c>
       <c r="C79" t="n">
-        <v>6.9</v>
+        <v>1144</v>
       </c>
       <c r="D79" t="n">
-        <v>3.14</v>
+        <v>3.08</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>JBMA</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>669.25</v>
+        <v>1.96</v>
       </c>
       <c r="C80" t="n">
-        <v>690</v>
+        <v>2.02</v>
       </c>
       <c r="D80" t="n">
-        <v>3.1</v>
+        <v>3.06</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>AMJLAND</t>
+          <t>ENERGYDEV</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>36.84</v>
+        <v>16.4</v>
       </c>
       <c r="C81" t="n">
-        <v>37.98</v>
+        <v>16.9</v>
       </c>
       <c r="D81" t="n">
-        <v>3.09</v>
+        <v>3.05</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>FLEXITUFF</t>
+          <t>KAYA</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>6.89</v>
+        <v>251.35</v>
       </c>
       <c r="C82" t="n">
-        <v>7.1</v>
+        <v>258.99</v>
       </c>
       <c r="D82" t="n">
-        <v>3.05</v>
+        <v>3.04</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>LAMOSAIC</t>
+          <t>AGROPHOS</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>29.7</v>
+        <v>30.48</v>
       </c>
       <c r="C83" t="n">
-        <v>30.6</v>
+        <v>31.39</v>
       </c>
       <c r="D83" t="n">
-        <v>3.03</v>
+        <v>2.99</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>AEPL</t>
+          <t>RADAAN</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>16.25</v>
+        <v>3.01</v>
       </c>
       <c r="C84" t="n">
-        <v>16.74</v>
+        <v>3.1</v>
       </c>
       <c r="D84" t="n">
-        <v>3.02</v>
+        <v>2.99</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>BPL</t>
+          <t>FLYSBS</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>52.37</v>
+        <v>412.6</v>
       </c>
       <c r="C85" t="n">
-        <v>53.9</v>
+        <v>424.8</v>
       </c>
       <c r="D85" t="n">
-        <v>2.92</v>
+        <v>2.96</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>GEMAROMA</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>107.85</v>
+        <v>148.13</v>
       </c>
       <c r="C86" t="n">
-        <v>110.98</v>
+        <v>152.5</v>
       </c>
       <c r="D86" t="n">
-        <v>2.9</v>
+        <v>2.95</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CONSOFINVT</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>242.97</v>
+        <v>6.12</v>
       </c>
       <c r="C87" t="n">
-        <v>249.94</v>
+        <v>6.3</v>
       </c>
       <c r="D87" t="n">
-        <v>2.87</v>
+        <v>2.94</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>BIRLAPREC</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>38.76</v>
+        <v>23.03</v>
       </c>
       <c r="C88" t="n">
-        <v>39.84</v>
+        <v>23.7</v>
       </c>
       <c r="D88" t="n">
-        <v>2.79</v>
+        <v>2.91</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>NDLVENTURE</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0.36</v>
+        <v>131.2</v>
       </c>
       <c r="C89" t="n">
-        <v>0.37</v>
+        <v>135</v>
       </c>
       <c r="D89" t="n">
-        <v>2.78</v>
+        <v>2.9</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>KAVDEFENCE</t>
+          <t>CLEDUCATE</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>60.33</v>
+        <v>51.22</v>
       </c>
       <c r="C90" t="n">
-        <v>62</v>
+        <v>52.7</v>
       </c>
       <c r="D90" t="n">
-        <v>2.77</v>
+        <v>2.89</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>KEYFINSERV</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>251.8</v>
+        <v>2.09</v>
       </c>
       <c r="C91" t="n">
-        <v>258.75</v>
+        <v>2.15</v>
       </c>
       <c r="D91" t="n">
-        <v>2.76</v>
+        <v>2.87</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>UFBL</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>474.85</v>
+        <v>19.83</v>
       </c>
       <c r="C92" t="n">
-        <v>487.7</v>
+        <v>20.4</v>
       </c>
       <c r="D92" t="n">
-        <v>2.71</v>
+        <v>2.87</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>VISACHROME</t>
+          <t>SIL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>52.58</v>
+        <v>15.71</v>
       </c>
       <c r="C93" t="n">
-        <v>53.99</v>
+        <v>16.16</v>
       </c>
       <c r="D93" t="n">
-        <v>2.68</v>
+        <v>2.86</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>4.87</v>
+        <v>20.9</v>
       </c>
       <c r="C94" t="n">
-        <v>5</v>
+        <v>21.49</v>
       </c>
       <c r="D94" t="n">
-        <v>2.67</v>
+        <v>2.82</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>WSI</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1806.2</v>
+        <v>68.97</v>
       </c>
       <c r="C95" t="n">
-        <v>1854</v>
+        <v>70.87</v>
       </c>
       <c r="D95" t="n">
-        <v>2.65</v>
+        <v>2.75</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>45.79</v>
+        <v>96</v>
       </c>
       <c r="C96" t="n">
-        <v>47</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="D96" t="n">
-        <v>2.64</v>
+        <v>2.71</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1.54</v>
+        <v>0.37</v>
       </c>
       <c r="C97" t="n">
-        <v>1.58</v>
+        <v>0.38</v>
       </c>
       <c r="D97" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>IWP</t>
+          <t>SHRENIK</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>34.13</v>
+        <v>0.37</v>
       </c>
       <c r="C98" t="n">
-        <v>35</v>
+        <v>0.38</v>
       </c>
       <c r="D98" t="n">
-        <v>2.55</v>
+        <v>2.7</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SBGLP</t>
+          <t>ALANKIT</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>25.99</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="C99" t="n">
-        <v>26.65</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="D99" t="n">
-        <v>2.54</v>
+        <v>2.69</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>GENUSPAPER</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>12.44</v>
+        <v>13.93</v>
       </c>
       <c r="C100" t="n">
-        <v>12.75</v>
+        <v>14.3</v>
       </c>
       <c r="D100" t="n">
-        <v>2.49</v>
+        <v>2.66</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SRTL</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>41.97</v>
+        <v>1.16</v>
       </c>
       <c r="C101" t="n">
-        <v>43</v>
+        <v>1.19</v>
       </c>
       <c r="D101" t="n">
-        <v>2.45</v>
+        <v>2.59</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ANTELOPUS</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>871.8</v>
+        <v>10.14</v>
       </c>
       <c r="C102" t="n">
-        <v>892.95</v>
+        <v>10.4</v>
       </c>
       <c r="D102" t="n">
-        <v>2.43</v>
+        <v>2.56</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>RELCHEMQ</t>
+          <t>TECHLABS</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>121.06</v>
+        <v>164.85</v>
       </c>
       <c r="C103" t="n">
-        <v>124</v>
+        <v>169</v>
       </c>
       <c r="D103" t="n">
-        <v>2.43</v>
+        <v>2.52</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>TECILCHEM</t>
+          <t>DCMSIL</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>11.62</v>
+        <v>62.23</v>
       </c>
       <c r="C104" t="n">
-        <v>11.9</v>
+        <v>63.79</v>
       </c>
       <c r="D104" t="n">
-        <v>2.41</v>
+        <v>2.51</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>ANANTAM</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>514.6</v>
+        <v>104.29</v>
       </c>
       <c r="C105" t="n">
-        <v>527</v>
+        <v>106.9</v>
       </c>
       <c r="D105" t="n">
-        <v>2.41</v>
+        <v>2.5</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>ZEEL</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>198.59</v>
+        <v>104.42</v>
       </c>
       <c r="C106" t="n">
-        <v>203.33</v>
+        <v>107</v>
       </c>
       <c r="D106" t="n">
-        <v>2.39</v>
+        <v>2.47</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>JKIPL</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.42</v>
+        <v>94.66</v>
       </c>
       <c r="C107" t="n">
-        <v>0.43</v>
+        <v>97</v>
       </c>
       <c r="D107" t="n">
-        <v>2.38</v>
+        <v>2.47</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>SANATHAN</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>629.95</v>
+        <v>395.7</v>
       </c>
       <c r="C108" t="n">
-        <v>644.9</v>
+        <v>405.4</v>
       </c>
       <c r="D108" t="n">
-        <v>2.37</v>
+        <v>2.45</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BCG</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>11.04</v>
+        <v>7.36</v>
       </c>
       <c r="C109" t="n">
-        <v>11.3</v>
+        <v>7.54</v>
       </c>
       <c r="D109" t="n">
-        <v>2.36</v>
+        <v>2.45</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>PRECOT</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>733.55</v>
+        <v>28.25</v>
       </c>
       <c r="C110" t="n">
-        <v>750.55</v>
+        <v>28.94</v>
       </c>
       <c r="D110" t="n">
-        <v>2.32</v>
+        <v>2.44</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MANOMAY</t>
+          <t>HALDER</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>173.97</v>
+        <v>250.87</v>
       </c>
       <c r="C111" t="n">
-        <v>178</v>
+        <v>257</v>
       </c>
       <c r="D111" t="n">
-        <v>2.32</v>
+        <v>2.44</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>23.24</v>
+        <v>1555.8</v>
       </c>
       <c r="C112" t="n">
-        <v>23.78</v>
+        <v>1593.8</v>
       </c>
       <c r="D112" t="n">
-        <v>2.32</v>
+        <v>2.44</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MODIRUBBER</t>
+          <t>STARPAPER</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>124.91</v>
+        <v>138.05</v>
       </c>
       <c r="C113" t="n">
-        <v>127.8</v>
+        <v>141.4</v>
       </c>
       <c r="D113" t="n">
-        <v>2.31</v>
+        <v>2.43</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>BLUESTONE</t>
+          <t>VSTL</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>508.25</v>
+        <v>115.22</v>
       </c>
       <c r="C114" t="n">
-        <v>520</v>
+        <v>118</v>
       </c>
       <c r="D114" t="n">
-        <v>2.31</v>
+        <v>2.41</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SUVIDHAA</t>
+          <t>KAPSTON</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>2.62</v>
+        <v>336.8</v>
       </c>
       <c r="C115" t="n">
-        <v>2.68</v>
+        <v>344.85</v>
       </c>
       <c r="D115" t="n">
-        <v>2.29</v>
+        <v>2.39</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>JMA</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>87.87</v>
+        <v>0.42</v>
       </c>
       <c r="C116" t="n">
-        <v>89.88</v>
+        <v>0.43</v>
       </c>
       <c r="D116" t="n">
-        <v>2.29</v>
+        <v>2.38</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>JUNIPER</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>92.61</v>
+        <v>201.21</v>
       </c>
       <c r="C117" t="n">
-        <v>94.7</v>
+        <v>206</v>
       </c>
       <c r="D117" t="n">
-        <v>2.26</v>
+        <v>2.38</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>VISHWARAJ</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>5.75</v>
+        <v>87.23</v>
       </c>
       <c r="C118" t="n">
-        <v>5.88</v>
+        <v>89.28</v>
       </c>
       <c r="D118" t="n">
-        <v>2.26</v>
+        <v>2.35</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SUNLITE</t>
+          <t>REGAAL</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>440.05</v>
+        <v>83.73999999999999</v>
       </c>
       <c r="C119" t="n">
-        <v>449.85</v>
+        <v>85.7</v>
       </c>
       <c r="D119" t="n">
-        <v>2.23</v>
+        <v>2.34</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>OBCL</t>
+          <t>TEXINFRA</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>50.87</v>
+        <v>100.55</v>
       </c>
       <c r="C120" t="n">
-        <v>52</v>
+        <v>102.9</v>
       </c>
       <c r="D120" t="n">
-        <v>2.22</v>
+        <v>2.34</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>VIPCLOTHNG</t>
+          <t>AVADHSUGAR</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>25.82</v>
+        <v>476.85</v>
       </c>
       <c r="C121" t="n">
-        <v>26.39</v>
+        <v>488</v>
       </c>
       <c r="D121" t="n">
-        <v>2.21</v>
+        <v>2.34</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>RILINFRA</t>
+          <t>GANDHAR</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>36.6</v>
+        <v>161.85</v>
       </c>
       <c r="C122" t="n">
-        <v>37.4</v>
+        <v>165.64</v>
       </c>
       <c r="D122" t="n">
-        <v>2.19</v>
+        <v>2.34</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>GFLLIMITED</t>
+          <t>ZUARI</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>46.48</v>
+        <v>217.95</v>
       </c>
       <c r="C123" t="n">
-        <v>47.5</v>
+        <v>223.02</v>
       </c>
       <c r="D123" t="n">
-        <v>2.19</v>
+        <v>2.33</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>STEELCITY</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>76.92</v>
+        <v>1171</v>
       </c>
       <c r="C124" t="n">
-        <v>78.59999999999999</v>
+        <v>1198</v>
       </c>
       <c r="D124" t="n">
-        <v>2.18</v>
+        <v>2.31</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>FLFL</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>1.39</v>
+        <v>4.76</v>
       </c>
       <c r="C125" t="n">
-        <v>1.42</v>
+        <v>4.87</v>
       </c>
       <c r="D125" t="n">
-        <v>2.16</v>
+        <v>2.31</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>KRITIKA</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>19.47</v>
+        <v>6.05</v>
       </c>
       <c r="C126" t="n">
-        <v>19.89</v>
+        <v>6.19</v>
       </c>
       <c r="D126" t="n">
-        <v>2.16</v>
+        <v>2.31</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>IGCL</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>6.94</v>
+        <v>57.06</v>
       </c>
       <c r="C127" t="n">
-        <v>7.09</v>
+        <v>58.38</v>
       </c>
       <c r="D127" t="n">
-        <v>2.16</v>
+        <v>2.31</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>CEREBRAINT</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>3.28</v>
+        <v>6.52</v>
       </c>
       <c r="C128" t="n">
-        <v>3.35</v>
+        <v>6.67</v>
       </c>
       <c r="D128" t="n">
-        <v>2.13</v>
+        <v>2.3</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>ELDEHSG</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>185</v>
+        <v>786.7</v>
       </c>
       <c r="C129" t="n">
-        <v>188.9</v>
+        <v>804.8</v>
       </c>
       <c r="D129" t="n">
-        <v>2.11</v>
+        <v>2.3</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>EFORCE</t>
+          <t>CENTEXT</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>21.6</v>
+        <v>19.53</v>
       </c>
       <c r="C130" t="n">
-        <v>22.05</v>
+        <v>19.98</v>
       </c>
       <c r="D130" t="n">
-        <v>2.08</v>
+        <v>2.3</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>HDIL</t>
+          <t>AJOONI</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>1.92</v>
+        <v>3.91</v>
       </c>
       <c r="C131" t="n">
-        <v>1.96</v>
+        <v>4</v>
       </c>
       <c r="D131" t="n">
-        <v>2.08</v>
+        <v>2.3</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>TARMAT</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>6.78</v>
+        <v>52.31</v>
       </c>
       <c r="C132" t="n">
-        <v>6.92</v>
+        <v>53.51</v>
       </c>
       <c r="D132" t="n">
-        <v>2.06</v>
+        <v>2.29</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>CNL</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>1.97</v>
+        <v>633.55</v>
       </c>
       <c r="C133" t="n">
-        <v>2.01</v>
+        <v>648</v>
       </c>
       <c r="D133" t="n">
-        <v>2.03</v>
+        <v>2.28</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ANONDITA</t>
+          <t>PIGL</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>1117.35</v>
+        <v>101.67</v>
       </c>
       <c r="C134" t="n">
-        <v>1139.9</v>
+        <v>103.99</v>
       </c>
       <c r="D134" t="n">
-        <v>2.02</v>
+        <v>2.28</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>MANAKALUCO</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>8.470000000000001</v>
+        <v>35.59</v>
       </c>
       <c r="C135" t="n">
-        <v>8.640000000000001</v>
+        <v>36.4</v>
       </c>
       <c r="D135" t="n">
-        <v>2.01</v>
+        <v>2.28</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>BPL</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>40</v>
+        <v>51.82</v>
       </c>
       <c r="C136" t="n">
-        <v>40.8</v>
+        <v>53</v>
       </c>
       <c r="D136" t="n">
-        <v>2</v>
+        <v>2.28</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SETUINFRA</t>
+          <t>BIRLACABLE</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.5</v>
+        <v>235.68</v>
       </c>
       <c r="C137" t="n">
-        <v>0.51</v>
+        <v>241</v>
       </c>
       <c r="D137" t="n">
-        <v>2</v>
+        <v>2.26</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>RUDRA</t>
+          <t>SUNFLAG</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>18.13</v>
+        <v>406.85</v>
       </c>
       <c r="C138" t="n">
-        <v>18.49</v>
+        <v>416</v>
       </c>
       <c r="D138" t="n">
-        <v>1.99</v>
+        <v>2.25</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>PIONEEREMB</t>
+          <t>HPAL</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>24.44</v>
+        <v>37.17</v>
       </c>
       <c r="C139" t="n">
-        <v>24.92</v>
+        <v>38</v>
       </c>
       <c r="D139" t="n">
-        <v>1.96</v>
+        <v>2.23</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>7.17</v>
+        <v>338.85</v>
       </c>
       <c r="C140" t="n">
-        <v>7.31</v>
+        <v>346.4</v>
       </c>
       <c r="D140" t="n">
-        <v>1.95</v>
+        <v>2.23</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>BYKE</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>490.45</v>
+        <v>35.2</v>
       </c>
       <c r="C141" t="n">
-        <v>500</v>
+        <v>35.98</v>
       </c>
       <c r="D141" t="n">
-        <v>1.95</v>
+        <v>2.22</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ITDC</t>
+          <t>LIKHITHA</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>535.6</v>
+        <v>209.84</v>
       </c>
       <c r="C142" t="n">
-        <v>546</v>
+        <v>214.5</v>
       </c>
       <c r="D142" t="n">
-        <v>1.94</v>
+        <v>2.22</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>VHL</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>35.22</v>
+        <v>3404.2</v>
       </c>
       <c r="C143" t="n">
-        <v>35.9</v>
+        <v>3479.7</v>
       </c>
       <c r="D143" t="n">
-        <v>1.93</v>
+        <v>2.22</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>KOTARISUG</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>17.15</v>
+        <v>24.93</v>
       </c>
       <c r="C144" t="n">
-        <v>17.48</v>
+        <v>25.48</v>
       </c>
       <c r="D144" t="n">
-        <v>1.92</v>
+        <v>2.21</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>UMAEXPORTS</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>25.5</v>
+        <v>4.99</v>
       </c>
       <c r="C145" t="n">
-        <v>25.99</v>
+        <v>5.1</v>
       </c>
       <c r="D145" t="n">
-        <v>1.92</v>
+        <v>2.2</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>UNIDT</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>250.22</v>
+        <v>7.34</v>
       </c>
       <c r="C146" t="n">
-        <v>254.97</v>
+        <v>7.5</v>
       </c>
       <c r="D146" t="n">
-        <v>1.9</v>
+        <v>2.18</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SOUTHWEST</t>
+          <t>SABEVENTS</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>262.5</v>
+        <v>7.92</v>
       </c>
       <c r="C147" t="n">
-        <v>267.5</v>
+        <v>8.09</v>
       </c>
       <c r="D147" t="n">
-        <v>1.9</v>
+        <v>2.15</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>DANISH</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>896.05</v>
+        <v>13.49</v>
       </c>
       <c r="C148" t="n">
-        <v>913</v>
+        <v>13.78</v>
       </c>
       <c r="D148" t="n">
-        <v>1.89</v>
+        <v>2.15</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>FABTECH</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>43.78</v>
+        <v>149.29</v>
       </c>
       <c r="C149" t="n">
-        <v>44.6</v>
+        <v>152.5</v>
       </c>
       <c r="D149" t="n">
-        <v>1.87</v>
+        <v>2.15</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>0.55</v>
+        <v>3124.7</v>
       </c>
       <c r="C150" t="n">
-        <v>0.5600000000000001</v>
+        <v>3191.6</v>
       </c>
       <c r="D150" t="n">
-        <v>1.82</v>
+        <v>2.14</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>HYBRIDFIN</t>
+          <t>AUTOIND</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>16.69</v>
+        <v>77.34</v>
       </c>
       <c r="C151" t="n">
-        <v>16.99</v>
+        <v>78.98999999999999</v>
       </c>
       <c r="D151" t="n">
-        <v>1.8</v>
+        <v>2.13</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MADHAV</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>37.77</v>
+        <v>38.19</v>
       </c>
       <c r="C152" t="n">
-        <v>38.44</v>
+        <v>39</v>
       </c>
       <c r="D152" t="n">
-        <v>1.77</v>
+        <v>2.12</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>GICL</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>1.13</v>
+        <v>26.93</v>
       </c>
       <c r="C153" t="n">
-        <v>1.15</v>
+        <v>27.5</v>
       </c>
       <c r="D153" t="n">
-        <v>1.77</v>
+        <v>2.12</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>CENTEXT</t>
+          <t>COOLCAPS</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>19.56</v>
+        <v>21.3</v>
       </c>
       <c r="C154" t="n">
-        <v>19.9</v>
+        <v>21.75</v>
       </c>
       <c r="D154" t="n">
-        <v>1.74</v>
+        <v>2.11</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>BAJEL</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>199.93</v>
+        <v>7.15</v>
       </c>
       <c r="C155" t="n">
-        <v>203.38</v>
+        <v>7.3</v>
       </c>
       <c r="D155" t="n">
-        <v>1.73</v>
+        <v>2.1</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>JISLJALEQS</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>29.12</v>
+        <v>6.66</v>
       </c>
       <c r="C156" t="n">
-        <v>29.62</v>
+        <v>6.8</v>
       </c>
       <c r="D156" t="n">
-        <v>1.72</v>
+        <v>2.1</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>BOSCH-HCIL</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>5.29</v>
+        <v>1395.8</v>
       </c>
       <c r="C157" t="n">
-        <v>5.38</v>
+        <v>1424.9</v>
       </c>
       <c r="D157" t="n">
-        <v>1.7</v>
+        <v>2.08</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>EFFWA</t>
+          <t>SAKUMA</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>300.9</v>
+        <v>1.93</v>
       </c>
       <c r="C158" t="n">
-        <v>306</v>
+        <v>1.97</v>
       </c>
       <c r="D158" t="n">
-        <v>1.69</v>
+        <v>2.07</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>SHREERAMA</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>44.25</v>
+        <v>907.55</v>
       </c>
       <c r="C159" t="n">
-        <v>45</v>
+        <v>926.3</v>
       </c>
       <c r="D159" t="n">
-        <v>1.69</v>
+        <v>2.07</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>URJA</t>
+          <t>RPPL</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>10.81</v>
+        <v>18.91</v>
       </c>
       <c r="C160" t="n">
-        <v>10.99</v>
+        <v>19.3</v>
       </c>
       <c r="D160" t="n">
-        <v>1.67</v>
+        <v>2.06</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>MBLINFRA</t>
+          <t>GODIGIT</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>28.18</v>
+        <v>302.8</v>
       </c>
       <c r="C161" t="n">
-        <v>28.65</v>
+        <v>309</v>
       </c>
       <c r="D161" t="n">
-        <v>1.67</v>
+        <v>2.05</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>418.1</v>
+        <v>0.49</v>
       </c>
       <c r="C162" t="n">
-        <v>424.95</v>
+        <v>0.5</v>
       </c>
       <c r="D162" t="n">
-        <v>1.64</v>
+        <v>2.04</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>HMVL</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>76.11</v>
+        <v>4596.5</v>
       </c>
       <c r="C163" t="n">
-        <v>77.34999999999999</v>
+        <v>4690</v>
       </c>
       <c r="D163" t="n">
-        <v>1.63</v>
+        <v>2.03</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>LOVABLE</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>23.6</v>
+        <v>72.04000000000001</v>
       </c>
       <c r="C164" t="n">
-        <v>23.98</v>
+        <v>73.5</v>
       </c>
       <c r="D164" t="n">
-        <v>1.61</v>
+        <v>2.03</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>BBOX</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>418.15</v>
+        <v>1078.2</v>
       </c>
       <c r="C165" t="n">
-        <v>424.9</v>
+        <v>1100</v>
       </c>
       <c r="D165" t="n">
-        <v>1.61</v>
+        <v>2.02</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>POWERICA</t>
+          <t>PIONEEREMB</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>542.3</v>
+        <v>23.42</v>
       </c>
       <c r="C166" t="n">
-        <v>551</v>
+        <v>23.89</v>
       </c>
       <c r="D166" t="n">
-        <v>1.6</v>
+        <v>2.01</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>TVTODAY</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>111.41</v>
+        <v>0.5</v>
       </c>
       <c r="C167" t="n">
-        <v>113.19</v>
+        <v>0.51</v>
       </c>
       <c r="D167" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>IVC</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>8.119999999999999</v>
+        <v>44.89</v>
       </c>
       <c r="C168" t="n">
-        <v>8.25</v>
+        <v>45.79</v>
       </c>
       <c r="D168" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>HCL-INSYS</t>
+          <t>VEEDOL</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>13.11</v>
+        <v>1460.6</v>
       </c>
       <c r="C169" t="n">
-        <v>13.32</v>
+        <v>1489.6</v>
       </c>
       <c r="D169" t="n">
-        <v>1.6</v>
+        <v>1.99</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>HEXATRADEX</t>
+          <t>DIGISPICE</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>162.1</v>
+        <v>20.06</v>
       </c>
       <c r="C170" t="n">
-        <v>164.7</v>
+        <v>20.46</v>
       </c>
       <c r="D170" t="n">
-        <v>1.6</v>
+        <v>1.99</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>INDOWIND</t>
+          <t>AAATECH</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>9.43</v>
+        <v>91.19</v>
       </c>
       <c r="C171" t="n">
-        <v>9.58</v>
+        <v>93</v>
       </c>
       <c r="D171" t="n">
-        <v>1.59</v>
+        <v>1.98</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>CONFIPET</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>76.79000000000001</v>
+        <v>7.11</v>
       </c>
       <c r="C172" t="n">
-        <v>78</v>
+        <v>7.25</v>
       </c>
       <c r="D172" t="n">
-        <v>1.58</v>
+        <v>1.97</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>NITIRAJ</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>139.82</v>
+        <v>184.07</v>
       </c>
       <c r="C173" t="n">
-        <v>142</v>
+        <v>187.7</v>
       </c>
       <c r="D173" t="n">
-        <v>1.56</v>
+        <v>1.97</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>MSPL</t>
+          <t>SAGARDEEP</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>41.15</v>
+        <v>25.47</v>
       </c>
       <c r="C174" t="n">
-        <v>41.79</v>
+        <v>25.97</v>
       </c>
       <c r="D174" t="n">
-        <v>1.56</v>
+        <v>1.96</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>JARO</t>
+          <t>PRIMO</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>596.6</v>
+        <v>21.97</v>
       </c>
       <c r="C175" t="n">
-        <v>605.85</v>
+        <v>22.4</v>
       </c>
       <c r="D175" t="n">
-        <v>1.55</v>
+        <v>1.96</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>BODALCHEM</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>86.56</v>
+        <v>71.59</v>
       </c>
       <c r="C176" t="n">
-        <v>87.90000000000001</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="D176" t="n">
-        <v>1.55</v>
+        <v>1.96</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>344.6</v>
+        <v>39.41</v>
       </c>
       <c r="C177" t="n">
-        <v>349.8</v>
+        <v>40.18</v>
       </c>
       <c r="D177" t="n">
-        <v>1.51</v>
+        <v>1.95</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>JUNIPER</t>
+          <t>SAKHTISUG</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>194.11</v>
+        <v>17.4</v>
       </c>
       <c r="C178" t="n">
-        <v>196.98</v>
+        <v>17.74</v>
       </c>
       <c r="D178" t="n">
-        <v>1.48</v>
+        <v>1.95</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>KRITINUT</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>89.66</v>
+        <v>3.62</v>
       </c>
       <c r="C179" t="n">
-        <v>90.98999999999999</v>
+        <v>3.69</v>
       </c>
       <c r="D179" t="n">
-        <v>1.48</v>
+        <v>1.93</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>UFO</t>
+          <t>ADISOFT</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>73.79000000000001</v>
+        <v>209.85</v>
       </c>
       <c r="C180" t="n">
-        <v>74.88</v>
+        <v>213.9</v>
       </c>
       <c r="D180" t="n">
-        <v>1.48</v>
+        <v>1.93</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>POWERINDIA</t>
+          <t>FINEORG</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>35190</v>
+        <v>4689.7</v>
       </c>
       <c r="C181" t="n">
-        <v>35705</v>
+        <v>4779.9</v>
       </c>
       <c r="D181" t="n">
-        <v>1.46</v>
+        <v>1.92</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>OMINFRAL</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>13.78</v>
+        <v>85.26000000000001</v>
       </c>
       <c r="C182" t="n">
-        <v>13.98</v>
+        <v>86.89</v>
       </c>
       <c r="D182" t="n">
-        <v>1.45</v>
+        <v>1.91</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>RKSWAMY</t>
+          <t>GTLINFRA</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>98.09</v>
+        <v>1.57</v>
       </c>
       <c r="C183" t="n">
-        <v>99.5</v>
+        <v>1.6</v>
       </c>
       <c r="D183" t="n">
-        <v>1.44</v>
+        <v>1.91</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>VASWANI</t>
+          <t>JAYBARMARU</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>58.95</v>
+        <v>126.6</v>
       </c>
       <c r="C184" t="n">
-        <v>59.8</v>
+        <v>129</v>
       </c>
       <c r="D184" t="n">
-        <v>1.44</v>
+        <v>1.9</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SINGERIND</t>
+          <t>IRISDOREME</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>69.41</v>
+        <v>36.47</v>
       </c>
       <c r="C185" t="n">
-        <v>70.40000000000001</v>
+        <v>37.15</v>
       </c>
       <c r="D185" t="n">
-        <v>1.43</v>
+        <v>1.86</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>3IINFOLTD</t>
+          <t>PANACEABIO</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>17.16</v>
+        <v>520.3</v>
       </c>
       <c r="C186" t="n">
-        <v>17.4</v>
+        <v>530</v>
       </c>
       <c r="D186" t="n">
-        <v>1.4</v>
+        <v>1.86</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>APCOTEXIND</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>498.45</v>
+        <v>3.24</v>
       </c>
       <c r="C187" t="n">
-        <v>505.4</v>
+        <v>3.3</v>
       </c>
       <c r="D187" t="n">
-        <v>1.39</v>
+        <v>1.85</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>UEL</t>
+          <t>VIGOR</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>141.92</v>
+        <v>70.7</v>
       </c>
       <c r="C188" t="n">
-        <v>143.89</v>
+        <v>72</v>
       </c>
       <c r="D188" t="n">
-        <v>1.39</v>
+        <v>1.84</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>KPL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>6.48</v>
+        <v>2375.2</v>
       </c>
       <c r="C189" t="n">
-        <v>6.57</v>
+        <v>2419</v>
       </c>
       <c r="D189" t="n">
-        <v>1.39</v>
+        <v>1.84</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>GEECEE</t>
+          <t>DBOL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>325.45</v>
+        <v>109.53</v>
       </c>
       <c r="C190" t="n">
-        <v>329.9</v>
+        <v>111.49</v>
       </c>
       <c r="D190" t="n">
-        <v>1.37</v>
+        <v>1.79</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>GOLDTECH</t>
+          <t>AXITA</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>43.06</v>
+        <v>7.8</v>
       </c>
       <c r="C191" t="n">
-        <v>43.65</v>
+        <v>7.94</v>
       </c>
       <c r="D191" t="n">
-        <v>1.37</v>
+        <v>1.79</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>DAVANGERE</t>
+          <t>MUKTAARTS</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>3.64</v>
+        <v>64.23999999999999</v>
       </c>
       <c r="C192" t="n">
-        <v>3.69</v>
+        <v>65.39</v>
       </c>
       <c r="D192" t="n">
-        <v>1.37</v>
+        <v>1.79</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>JSLL</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>14.64</v>
+        <v>651.9</v>
       </c>
       <c r="C193" t="n">
-        <v>14.84</v>
+        <v>663.5</v>
       </c>
       <c r="D193" t="n">
-        <v>1.37</v>
+        <v>1.78</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>BODALCHEM</t>
+          <t>THEJO</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>72.81999999999999</v>
+        <v>1565.6</v>
       </c>
       <c r="C194" t="n">
-        <v>73.8</v>
+        <v>1593.5</v>
       </c>
       <c r="D194" t="n">
-        <v>1.35</v>
+        <v>1.78</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>DREAMFOLKS</t>
+          <t>RUSTOMJEE</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>73.98999999999999</v>
+        <v>392.35</v>
       </c>
       <c r="C195" t="n">
-        <v>74.98</v>
+        <v>399.35</v>
       </c>
       <c r="D195" t="n">
-        <v>1.34</v>
+        <v>1.78</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>BOHRAIND</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>17.16</v>
+        <v>62.88</v>
       </c>
       <c r="C196" t="n">
-        <v>17.39</v>
+        <v>63.99</v>
       </c>
       <c r="D196" t="n">
-        <v>1.34</v>
+        <v>1.77</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>HTMEDIA</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>22.5</v>
+        <v>2.26</v>
       </c>
       <c r="C197" t="n">
-        <v>22.8</v>
+        <v>2.3</v>
       </c>
       <c r="D197" t="n">
-        <v>1.33</v>
+        <v>1.77</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>AARTECH</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>28.82</v>
+        <v>41.96</v>
       </c>
       <c r="C198" t="n">
-        <v>29.2</v>
+        <v>42.7</v>
       </c>
       <c r="D198" t="n">
-        <v>1.32</v>
+        <v>1.76</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>SABEVENTS</t>
+          <t>KSB</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>8.33</v>
+        <v>795.55</v>
       </c>
       <c r="C199" t="n">
-        <v>8.44</v>
+        <v>809.5</v>
       </c>
       <c r="D199" t="n">
-        <v>1.32</v>
+        <v>1.75</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>HIRECT</t>
+          <t>BCLIND</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>1118.3</v>
+        <v>32.24</v>
       </c>
       <c r="C200" t="n">
-        <v>1133</v>
+        <v>32.8</v>
       </c>
       <c r="D200" t="n">
-        <v>1.31</v>
+        <v>1.74</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>TRANSPEK</t>
+          <t>SRM</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>984.2</v>
+        <v>490.15</v>
       </c>
       <c r="C201" t="n">
-        <v>997</v>
+        <v>498.7</v>
       </c>
       <c r="D201" t="n">
-        <v>1.3</v>
+        <v>1.74</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-08 08:31 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BHAGERIA</t>
+          <t>CNL</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>180.52</v>
+        <v>630.65</v>
       </c>
       <c r="C2" t="n">
-        <v>205</v>
+        <v>756.75</v>
       </c>
       <c r="D2" t="n">
-        <v>13.56</v>
+        <v>20</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ORTINGLOBE</t>
+          <t>FLEXITUFF</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16.47</v>
+        <v>6.93</v>
       </c>
       <c r="C3" t="n">
-        <v>18.11</v>
+        <v>7.7</v>
       </c>
       <c r="D3" t="n">
-        <v>9.960000000000001</v>
+        <v>11.11</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>ORTINGLOBE</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>31.7</v>
+        <v>18.11</v>
       </c>
       <c r="C4" t="n">
-        <v>34.6</v>
+        <v>19.92</v>
       </c>
       <c r="D4" t="n">
-        <v>9.15</v>
+        <v>9.99</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BAFNAPH</t>
+          <t>YCCL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>160.31</v>
+        <v>9.65</v>
       </c>
       <c r="C5" t="n">
-        <v>172.89</v>
+        <v>10.5</v>
       </c>
       <c r="D5" t="n">
-        <v>7.85</v>
+        <v>8.81</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MADHUCON</t>
+          <t>SVLL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.07</v>
+        <v>747.9</v>
       </c>
       <c r="C6" t="n">
-        <v>5.45</v>
+        <v>800</v>
       </c>
       <c r="D6" t="n">
-        <v>7.5</v>
+        <v>6.97</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RELIABLE</t>
+          <t>BAFNAPH</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>137.78</v>
+        <v>176.34</v>
       </c>
       <c r="C7" t="n">
-        <v>148</v>
+        <v>187.4</v>
       </c>
       <c r="D7" t="n">
-        <v>7.42</v>
+        <v>6.27</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>VINYAS</t>
+          <t>AGRITECH</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1132.15</v>
+        <v>129.34</v>
       </c>
       <c r="C8" t="n">
-        <v>1200</v>
+        <v>136.99</v>
       </c>
       <c r="D8" t="n">
-        <v>5.99</v>
+        <v>5.91</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>SBGLP</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16.7</v>
+        <v>24.37</v>
       </c>
       <c r="C9" t="n">
-        <v>17.55</v>
+        <v>25.74</v>
       </c>
       <c r="D9" t="n">
-        <v>5.09</v>
+        <v>5.62</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,14 +637,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RELINFRA</t>
+          <t>PFOCUS</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>77.87</v>
+        <v>240.19</v>
       </c>
       <c r="C10" t="n">
-        <v>81.76000000000001</v>
+        <v>252.19</v>
       </c>
       <c r="D10" t="n">
         <v>5</v>
@@ -659,14 +659,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>IDEAFORGE</t>
+          <t>QPOWER</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>900</v>
+        <v>1072</v>
       </c>
       <c r="C11" t="n">
-        <v>945</v>
+        <v>1125.6</v>
       </c>
       <c r="D11" t="n">
         <v>5</v>
@@ -681,14 +681,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>SICALLOG</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>308.36</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>323.77</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="D12" t="n">
         <v>5</v>
@@ -703,14 +703,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PRAMARA</t>
+          <t>SUPREMEENG</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>143.05</v>
+        <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>150.2</v>
+        <v>1.05</v>
       </c>
       <c r="D13" t="n">
         <v>5</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IL&amp;FSENGG</t>
+          <t>GOLDENTOBC</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>27.6</v>
+        <v>25.06</v>
       </c>
       <c r="C14" t="n">
-        <v>28.98</v>
+        <v>26.31</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PURPLEUTED</t>
+          <t>DCMSIL</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>377</v>
+        <v>65.34</v>
       </c>
       <c r="C15" t="n">
-        <v>395.85</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SICALLOG</t>
+          <t>RNPL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>68.8</v>
+        <v>87.2</v>
       </c>
       <c r="C16" t="n">
-        <v>72.23999999999999</v>
+        <v>91.55</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>CLEDUCATE</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>46.05</v>
+        <v>53.78</v>
       </c>
       <c r="C17" t="n">
-        <v>48.35</v>
+        <v>56.46</v>
       </c>
       <c r="D17" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>GENSOL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1217.7</v>
+        <v>23.74</v>
       </c>
       <c r="C18" t="n">
-        <v>1278</v>
+        <v>24.92</v>
       </c>
       <c r="D18" t="n">
-        <v>4.95</v>
+        <v>4.97</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>6.67</v>
+        <v>48.35</v>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>50.75</v>
       </c>
       <c r="D19" t="n">
-        <v>4.95</v>
+        <v>4.96</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CEREBRAINT</t>
+          <t>GANESHIN</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3.44</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="C20" t="n">
-        <v>3.61</v>
+        <v>86.95</v>
       </c>
       <c r="D20" t="n">
-        <v>4.94</v>
+        <v>4.95</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MCON</t>
+          <t>AGSTRA</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>47.6</v>
+        <v>2.83</v>
       </c>
       <c r="C21" t="n">
-        <v>49.95</v>
+        <v>2.97</v>
       </c>
       <c r="D21" t="n">
-        <v>4.94</v>
+        <v>4.95</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>SIMBHALS</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2.25</v>
+        <v>6.7</v>
       </c>
       <c r="C22" t="n">
-        <v>2.36</v>
+        <v>7.03</v>
       </c>
       <c r="D22" t="n">
-        <v>4.89</v>
+        <v>4.93</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ALLETEC</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>143.9</v>
+        <v>14.67</v>
       </c>
       <c r="C23" t="n">
-        <v>150.9</v>
+        <v>15.39</v>
       </c>
       <c r="D23" t="n">
-        <v>4.86</v>
+        <v>4.91</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>SATIPOLY</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5.57</v>
+        <v>36.15</v>
       </c>
       <c r="C24" t="n">
-        <v>5.84</v>
+        <v>37.9</v>
       </c>
       <c r="D24" t="n">
-        <v>4.85</v>
+        <v>4.84</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HIRECT</t>
+          <t>MUNISH</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1137.8</v>
+        <v>60.8</v>
       </c>
       <c r="C25" t="n">
-        <v>1192.7</v>
+        <v>63.7</v>
       </c>
       <c r="D25" t="n">
-        <v>4.83</v>
+        <v>4.77</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2.7</v>
+        <v>2.31</v>
       </c>
       <c r="C26" t="n">
-        <v>2.83</v>
+        <v>2.42</v>
       </c>
       <c r="D26" t="n">
-        <v>4.81</v>
+        <v>4.76</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>UFBL</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>5.69</v>
+        <v>506</v>
       </c>
       <c r="C27" t="n">
-        <v>5.96</v>
+        <v>530</v>
       </c>
       <c r="D27" t="n">
-        <v>4.75</v>
+        <v>4.74</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MODISONLTD</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>345.45</v>
+        <v>5.96</v>
       </c>
       <c r="C28" t="n">
-        <v>361.6</v>
+        <v>6.24</v>
       </c>
       <c r="D28" t="n">
-        <v>4.68</v>
+        <v>4.7</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MAWANASUG</t>
+          <t>GTECJAINX</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>97.45</v>
+        <v>34.87</v>
       </c>
       <c r="C29" t="n">
-        <v>102</v>
+        <v>36.49</v>
       </c>
       <c r="D29" t="n">
-        <v>4.67</v>
+        <v>4.65</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>QMSMEDI</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>87.8</v>
+        <v>15.73</v>
       </c>
       <c r="C30" t="n">
-        <v>91.84999999999999</v>
+        <v>16.45</v>
       </c>
       <c r="D30" t="n">
-        <v>4.61</v>
+        <v>4.58</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SHANTI</t>
+          <t>DHRUV</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>6.41</v>
+        <v>28.68</v>
       </c>
       <c r="C31" t="n">
-        <v>6.7</v>
+        <v>29.99</v>
       </c>
       <c r="D31" t="n">
-        <v>4.52</v>
+        <v>4.57</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DHRUV</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>27.56</v>
+        <v>0.22</v>
       </c>
       <c r="C32" t="n">
-        <v>28.8</v>
+        <v>0.23</v>
       </c>
       <c r="D32" t="n">
-        <v>4.5</v>
+        <v>4.55</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IZMO</t>
+          <t>NORBTEAEXP</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>879.4</v>
+        <v>76.94</v>
       </c>
       <c r="C33" t="n">
-        <v>918.9</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="D33" t="n">
-        <v>4.49</v>
+        <v>4.5</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PRECOT</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>765.65</v>
+        <v>109.14</v>
       </c>
       <c r="C34" t="n">
-        <v>800</v>
+        <v>114</v>
       </c>
       <c r="D34" t="n">
-        <v>4.49</v>
+        <v>4.45</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SIKKO</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4.05</v>
+        <v>11.25</v>
       </c>
       <c r="C35" t="n">
-        <v>4.23</v>
+        <v>11.74</v>
       </c>
       <c r="D35" t="n">
-        <v>4.44</v>
+        <v>4.36</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAPTRUST</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>13.3</v>
+        <v>18.64</v>
       </c>
       <c r="C36" t="n">
-        <v>13.89</v>
+        <v>19.45</v>
       </c>
       <c r="D36" t="n">
-        <v>4.44</v>
+        <v>4.35</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BCG</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>11.59</v>
+        <v>26.59</v>
       </c>
       <c r="C37" t="n">
-        <v>12.1</v>
+        <v>27.69</v>
       </c>
       <c r="D37" t="n">
-        <v>4.4</v>
+        <v>4.14</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>MCON</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>40.86</v>
+        <v>49.95</v>
       </c>
       <c r="C38" t="n">
-        <v>42.65</v>
+        <v>52</v>
       </c>
       <c r="D38" t="n">
-        <v>4.38</v>
+        <v>4.1</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.23</v>
+        <v>34.39</v>
       </c>
       <c r="C39" t="n">
-        <v>0.24</v>
+        <v>35.8</v>
       </c>
       <c r="D39" t="n">
-        <v>4.35</v>
+        <v>4.1</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ITDC</t>
+          <t>SYSTMTXC</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>589.15</v>
+        <v>66.34</v>
       </c>
       <c r="C40" t="n">
-        <v>614</v>
+        <v>69</v>
       </c>
       <c r="D40" t="n">
-        <v>4.22</v>
+        <v>4.01</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>AKCAPIT</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>74.84999999999999</v>
+        <v>1712</v>
       </c>
       <c r="C41" t="n">
-        <v>78</v>
+        <v>1780</v>
       </c>
       <c r="D41" t="n">
-        <v>4.21</v>
+        <v>3.97</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AEPL</t>
+          <t>RELINFRA</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>16.02</v>
+        <v>81.76000000000001</v>
       </c>
       <c r="C42" t="n">
-        <v>16.69</v>
+        <v>84.98999999999999</v>
       </c>
       <c r="D42" t="n">
-        <v>4.18</v>
+        <v>3.95</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>INNOVISION</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>285.1</v>
+        <v>1.78</v>
       </c>
       <c r="C43" t="n">
-        <v>297</v>
+        <v>1.85</v>
       </c>
       <c r="D43" t="n">
-        <v>4.17</v>
+        <v>3.93</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AGARIND</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>503.25</v>
+        <v>3.85</v>
       </c>
       <c r="C44" t="n">
-        <v>524</v>
+        <v>4</v>
       </c>
       <c r="D44" t="n">
-        <v>4.12</v>
+        <v>3.9</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AUSOMENT</t>
+          <t>SILLYMONKS</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>120.99</v>
+        <v>16.8</v>
       </c>
       <c r="C45" t="n">
-        <v>125.9</v>
+        <v>17.45</v>
       </c>
       <c r="D45" t="n">
-        <v>4.06</v>
+        <v>3.87</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IRIS</t>
+          <t>PERFECT</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>243.1</v>
+        <v>2.7</v>
       </c>
       <c r="C46" t="n">
-        <v>252.8</v>
+        <v>2.8</v>
       </c>
       <c r="D46" t="n">
-        <v>3.99</v>
+        <v>3.7</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MGEL</t>
+          <t>VIVIDHA</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>15.2</v>
+        <v>0.54</v>
       </c>
       <c r="C47" t="n">
-        <v>15.79</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D47" t="n">
-        <v>3.88</v>
+        <v>3.7</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>QUINT</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>5.49</v>
+        <v>39.51</v>
       </c>
       <c r="C48" t="n">
-        <v>5.7</v>
+        <v>40.9</v>
       </c>
       <c r="D48" t="n">
-        <v>3.83</v>
+        <v>3.52</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ODIGMA</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>20.51</v>
+        <v>35.26</v>
       </c>
       <c r="C49" t="n">
-        <v>21.29</v>
+        <v>36.5</v>
       </c>
       <c r="D49" t="n">
-        <v>3.8</v>
+        <v>3.52</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>DELTAMAGNT</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>32.76</v>
+        <v>60.08</v>
       </c>
       <c r="C50" t="n">
-        <v>34</v>
+        <v>62.19</v>
       </c>
       <c r="D50" t="n">
-        <v>3.79</v>
+        <v>3.51</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>UMAEXPORTS</t>
+          <t>UNIINFO</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>24.95</v>
+        <v>11.69</v>
       </c>
       <c r="C51" t="n">
-        <v>25.89</v>
+        <v>12.1</v>
       </c>
       <c r="D51" t="n">
-        <v>3.77</v>
+        <v>3.51</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>UNIHEALTH</t>
+          <t>PML</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>438.5</v>
+        <v>500.95</v>
       </c>
       <c r="C52" t="n">
-        <v>455</v>
+        <v>518.5</v>
       </c>
       <c r="D52" t="n">
-        <v>3.76</v>
+        <v>3.5</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DAMODARIND</t>
+          <t>UNIENTER</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>30.39</v>
+        <v>105.24</v>
       </c>
       <c r="C53" t="n">
-        <v>31.49</v>
+        <v>108.9</v>
       </c>
       <c r="D53" t="n">
-        <v>3.62</v>
+        <v>3.48</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SHALPAINTS</t>
+          <t>AKG</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>50.09</v>
+        <v>11.21</v>
       </c>
       <c r="C54" t="n">
-        <v>51.9</v>
+        <v>11.6</v>
       </c>
       <c r="D54" t="n">
-        <v>3.61</v>
+        <v>3.48</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>SWARAJ</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>3.92</v>
+        <v>240.6</v>
       </c>
       <c r="C55" t="n">
-        <v>4.06</v>
+        <v>248.95</v>
       </c>
       <c r="D55" t="n">
-        <v>3.57</v>
+        <v>3.47</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>UTLSOLAR</t>
+          <t>SINTERCOM</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>352.5</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="C56" t="n">
-        <v>365</v>
+        <v>75</v>
       </c>
       <c r="D56" t="n">
-        <v>3.55</v>
+        <v>3.46</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TVSSCS</t>
+          <t>KHAITANLTD</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>122.65</v>
+        <v>131.51</v>
       </c>
       <c r="C57" t="n">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="D57" t="n">
-        <v>3.55</v>
+        <v>3.41</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>INDTERRAIN</t>
+          <t>DAMODARIND</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>32.59</v>
+        <v>31.33</v>
       </c>
       <c r="C58" t="n">
-        <v>33.74</v>
+        <v>32.39</v>
       </c>
       <c r="D58" t="n">
-        <v>3.53</v>
+        <v>3.38</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SAPPL</t>
+          <t>MERCANTILE</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>270</v>
+        <v>25.16</v>
       </c>
       <c r="C59" t="n">
-        <v>279.5</v>
+        <v>26</v>
       </c>
       <c r="D59" t="n">
-        <v>3.52</v>
+        <v>3.34</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>35.26</v>
+        <v>1.52</v>
       </c>
       <c r="C60" t="n">
-        <v>36.5</v>
+        <v>1.57</v>
       </c>
       <c r="D60" t="n">
-        <v>3.52</v>
+        <v>3.29</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GOKUL</t>
+          <t>DBSTOCKBRO</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>40.43</v>
+        <v>31.95</v>
       </c>
       <c r="C61" t="n">
-        <v>41.85</v>
+        <v>32.99</v>
       </c>
       <c r="D61" t="n">
-        <v>3.51</v>
+        <v>3.26</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PASUPTAC</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>68.11</v>
+        <v>14.53</v>
       </c>
       <c r="C62" t="n">
-        <v>70.5</v>
+        <v>15</v>
       </c>
       <c r="D62" t="n">
-        <v>3.51</v>
+        <v>3.23</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>TNTELE</t>
+          <t>AERONEU</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>9.460000000000001</v>
+        <v>87.58</v>
       </c>
       <c r="C63" t="n">
-        <v>9.789999999999999</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="D63" t="n">
-        <v>3.49</v>
+        <v>3.22</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>KDL</t>
+          <t>KHANDSE</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>111.05</v>
+        <v>18.5</v>
       </c>
       <c r="C64" t="n">
-        <v>114.9</v>
+        <v>19.09</v>
       </c>
       <c r="D64" t="n">
-        <v>3.47</v>
+        <v>3.19</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>44.95</v>
+        <v>6.28</v>
       </c>
       <c r="C65" t="n">
-        <v>46.5</v>
+        <v>6.48</v>
       </c>
       <c r="D65" t="n">
-        <v>3.45</v>
+        <v>3.18</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>JNKINDIA</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>421.6</v>
+        <v>50.11</v>
       </c>
       <c r="C66" t="n">
-        <v>436</v>
+        <v>51.7</v>
       </c>
       <c r="D66" t="n">
-        <v>3.42</v>
+        <v>3.17</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>URAVIDEF</t>
+          <t>SHRIKRISH</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>115.12</v>
+        <v>42.7</v>
       </c>
       <c r="C67" t="n">
-        <v>119</v>
+        <v>44</v>
       </c>
       <c r="D67" t="n">
-        <v>3.37</v>
+        <v>3.04</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>MAYURUNIQ</t>
+          <t>AURIGROW</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>734.4</v>
+        <v>0.33</v>
       </c>
       <c r="C68" t="n">
-        <v>759</v>
+        <v>0.34</v>
       </c>
       <c r="D68" t="n">
-        <v>3.35</v>
+        <v>3.03</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BBTCL</t>
+          <t>GFLLIMITED</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>209.92</v>
+        <v>46.98</v>
       </c>
       <c r="C69" t="n">
-        <v>216.9</v>
+        <v>48.4</v>
       </c>
       <c r="D69" t="n">
-        <v>3.33</v>
+        <v>3.02</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>AIROLAM</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>44.54</v>
+        <v>79.65000000000001</v>
       </c>
       <c r="C70" t="n">
-        <v>46</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="D70" t="n">
-        <v>3.28</v>
+        <v>3</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>KAVDEFENCE</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>63.34</v>
+        <v>19.8</v>
       </c>
       <c r="C71" t="n">
-        <v>65.40000000000001</v>
+        <v>20.39</v>
       </c>
       <c r="D71" t="n">
-        <v>3.25</v>
+        <v>2.98</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>DEVX</t>
+          <t>TARMAT</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>37.54</v>
+        <v>51.77</v>
       </c>
       <c r="C72" t="n">
-        <v>38.76</v>
+        <v>53.29</v>
       </c>
       <c r="D72" t="n">
-        <v>3.25</v>
+        <v>2.94</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>9.880000000000001</v>
+        <v>5.54</v>
       </c>
       <c r="C73" t="n">
-        <v>10.2</v>
+        <v>5.7</v>
       </c>
       <c r="D73" t="n">
-        <v>3.24</v>
+        <v>2.89</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>BMLL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>10.13</v>
+        <v>122.5</v>
       </c>
       <c r="C74" t="n">
-        <v>10.45</v>
+        <v>126</v>
       </c>
       <c r="D74" t="n">
-        <v>3.16</v>
+        <v>2.86</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>BILVYAPAR</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>7.95</v>
+        <v>4.28</v>
       </c>
       <c r="C75" t="n">
-        <v>8.199999999999999</v>
+        <v>4.4</v>
       </c>
       <c r="D75" t="n">
-        <v>3.14</v>
+        <v>2.8</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>7.64</v>
+        <v>112.82</v>
       </c>
       <c r="C76" t="n">
-        <v>7.88</v>
+        <v>115.98</v>
       </c>
       <c r="D76" t="n">
-        <v>3.14</v>
+        <v>2.8</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SUPREMEENG</t>
+          <t>SABEVENTS</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.96</v>
+        <v>7.53</v>
       </c>
       <c r="C77" t="n">
-        <v>0.99</v>
+        <v>7.74</v>
       </c>
       <c r="D77" t="n">
-        <v>3.13</v>
+        <v>2.79</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>KDL</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>11.19</v>
+        <v>114.8</v>
       </c>
       <c r="C78" t="n">
-        <v>11.54</v>
+        <v>118</v>
       </c>
       <c r="D78" t="n">
-        <v>3.13</v>
+        <v>2.79</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SCHNEIDER</t>
+          <t>EMSLIMITED</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>1109.8</v>
+        <v>290.85</v>
       </c>
       <c r="C79" t="n">
-        <v>1144</v>
+        <v>298.95</v>
       </c>
       <c r="D79" t="n">
-        <v>3.08</v>
+        <v>2.78</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>SSDL</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>1.96</v>
+        <v>57.41</v>
       </c>
       <c r="C80" t="n">
-        <v>2.02</v>
+        <v>59</v>
       </c>
       <c r="D80" t="n">
-        <v>3.06</v>
+        <v>2.77</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ENERGYDEV</t>
+          <t>DYNPRO</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>16.4</v>
+        <v>248.05</v>
       </c>
       <c r="C81" t="n">
-        <v>16.9</v>
+        <v>254.9</v>
       </c>
       <c r="D81" t="n">
-        <v>3.05</v>
+        <v>2.76</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>KAYA</t>
+          <t>HEADSUP</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>251.35</v>
+        <v>7.24</v>
       </c>
       <c r="C82" t="n">
-        <v>258.99</v>
+        <v>7.44</v>
       </c>
       <c r="D82" t="n">
-        <v>3.04</v>
+        <v>2.76</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>AGROPHOS</t>
+          <t>NILE</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>30.48</v>
+        <v>1727.6</v>
       </c>
       <c r="C83" t="n">
-        <v>31.39</v>
+        <v>1774.9</v>
       </c>
       <c r="D83" t="n">
-        <v>2.99</v>
+        <v>2.74</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>RADAAN</t>
+          <t>MANAKSIA</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>3.01</v>
+        <v>58.3</v>
       </c>
       <c r="C84" t="n">
-        <v>3.1</v>
+        <v>59.9</v>
       </c>
       <c r="D84" t="n">
-        <v>2.99</v>
+        <v>2.74</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>FLYSBS</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>412.6</v>
+        <v>0.37</v>
       </c>
       <c r="C85" t="n">
-        <v>424.8</v>
+        <v>0.38</v>
       </c>
       <c r="D85" t="n">
-        <v>2.96</v>
+        <v>2.7</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>GEMAROMA</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>148.13</v>
+        <v>24.84</v>
       </c>
       <c r="C86" t="n">
-        <v>152.5</v>
+        <v>25.5</v>
       </c>
       <c r="D86" t="n">
-        <v>2.95</v>
+        <v>2.66</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>AARNAV</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>6.12</v>
+        <v>24.99</v>
       </c>
       <c r="C87" t="n">
-        <v>6.3</v>
+        <v>25.65</v>
       </c>
       <c r="D87" t="n">
-        <v>2.94</v>
+        <v>2.64</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>HITECHGEAR</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>23.03</v>
+        <v>562.2</v>
       </c>
       <c r="C88" t="n">
-        <v>23.7</v>
+        <v>577</v>
       </c>
       <c r="D88" t="n">
-        <v>2.91</v>
+        <v>2.63</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>NDLVENTURE</t>
+          <t>OSWALSEEDS</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>131.2</v>
+        <v>11.06</v>
       </c>
       <c r="C89" t="n">
-        <v>135</v>
+        <v>11.35</v>
       </c>
       <c r="D89" t="n">
-        <v>2.9</v>
+        <v>2.62</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CLEDUCATE</t>
+          <t>SHIVATEX</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>51.22</v>
+        <v>146.59</v>
       </c>
       <c r="C90" t="n">
-        <v>52.7</v>
+        <v>150.4</v>
       </c>
       <c r="D90" t="n">
-        <v>2.89</v>
+        <v>2.6</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>DEEDEV</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>2.09</v>
+        <v>671.15</v>
       </c>
       <c r="C91" t="n">
-        <v>2.15</v>
+        <v>688</v>
       </c>
       <c r="D91" t="n">
-        <v>2.87</v>
+        <v>2.51</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>19.83</v>
+        <v>1.99</v>
       </c>
       <c r="C92" t="n">
-        <v>20.4</v>
+        <v>2.04</v>
       </c>
       <c r="D92" t="n">
-        <v>2.87</v>
+        <v>2.51</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>SIL</t>
+          <t>JALAN</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>15.71</v>
+        <v>2</v>
       </c>
       <c r="C93" t="n">
-        <v>16.16</v>
+        <v>2.05</v>
       </c>
       <c r="D93" t="n">
-        <v>2.86</v>
+        <v>2.5</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>ASHOKAMET</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>20.9</v>
+        <v>15.2</v>
       </c>
       <c r="C94" t="n">
-        <v>21.49</v>
+        <v>15.58</v>
       </c>
       <c r="D94" t="n">
-        <v>2.82</v>
+        <v>2.5</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>WSI</t>
+          <t>SMARTLINK</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>68.97</v>
+        <v>159.05</v>
       </c>
       <c r="C95" t="n">
-        <v>70.87</v>
+        <v>163</v>
       </c>
       <c r="D95" t="n">
-        <v>2.75</v>
+        <v>2.48</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>96</v>
+        <v>16.57</v>
       </c>
       <c r="C96" t="n">
-        <v>98.59999999999999</v>
+        <v>16.98</v>
       </c>
       <c r="D96" t="n">
-        <v>2.71</v>
+        <v>2.47</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>NIPPOBATRY</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.37</v>
+        <v>359.95</v>
       </c>
       <c r="C97" t="n">
-        <v>0.38</v>
+        <v>368.8</v>
       </c>
       <c r="D97" t="n">
-        <v>2.7</v>
+        <v>2.46</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SHRENIK</t>
+          <t>FEDDERSHOL</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.37</v>
+        <v>35.08</v>
       </c>
       <c r="C98" t="n">
-        <v>0.38</v>
+        <v>35.94</v>
       </c>
       <c r="D98" t="n">
-        <v>2.7</v>
+        <v>2.45</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ALANKIT</t>
+          <t>CYBERMEDIA</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>8.550000000000001</v>
+        <v>16.9</v>
       </c>
       <c r="C99" t="n">
-        <v>8.779999999999999</v>
+        <v>17.31</v>
       </c>
       <c r="D99" t="n">
-        <v>2.69</v>
+        <v>2.43</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>MOS</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>13.93</v>
+        <v>16.6</v>
       </c>
       <c r="C100" t="n">
-        <v>14.3</v>
+        <v>17</v>
       </c>
       <c r="D100" t="n">
-        <v>2.66</v>
+        <v>2.41</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>DNAMEDIA</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1.16</v>
+        <v>2.93</v>
       </c>
       <c r="C101" t="n">
-        <v>1.19</v>
+        <v>3</v>
       </c>
       <c r="D101" t="n">
-        <v>2.59</v>
+        <v>2.39</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>AEPL</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>10.14</v>
+        <v>16.3</v>
       </c>
       <c r="C102" t="n">
-        <v>10.4</v>
+        <v>16.68</v>
       </c>
       <c r="D102" t="n">
-        <v>2.56</v>
+        <v>2.33</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>TECHLABS</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>164.85</v>
+        <v>42.78</v>
       </c>
       <c r="C103" t="n">
-        <v>169</v>
+        <v>43.77</v>
       </c>
       <c r="D103" t="n">
-        <v>2.52</v>
+        <v>2.31</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>DCMSIL</t>
+          <t>MAGNUM</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>62.23</v>
+        <v>19.53</v>
       </c>
       <c r="C104" t="n">
-        <v>63.79</v>
+        <v>19.98</v>
       </c>
       <c r="D104" t="n">
-        <v>2.51</v>
+        <v>2.3</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ANANTAM</t>
+          <t>VIPULLTD</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>104.29</v>
+        <v>9.58</v>
       </c>
       <c r="C105" t="n">
-        <v>106.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D105" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ZEEL</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>104.42</v>
+        <v>10.44</v>
       </c>
       <c r="C106" t="n">
-        <v>107</v>
+        <v>10.68</v>
       </c>
       <c r="D106" t="n">
-        <v>2.47</v>
+        <v>2.3</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>JKIPL</t>
+          <t>MIRZAINT</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>94.66</v>
+        <v>30.06</v>
       </c>
       <c r="C107" t="n">
-        <v>97</v>
+        <v>30.75</v>
       </c>
       <c r="D107" t="n">
-        <v>2.47</v>
+        <v>2.3</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SANATHAN</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>395.7</v>
+        <v>7.52</v>
       </c>
       <c r="C108" t="n">
-        <v>405.4</v>
+        <v>7.69</v>
       </c>
       <c r="D108" t="n">
-        <v>2.45</v>
+        <v>2.26</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>ODIGMA</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>7.36</v>
+        <v>21</v>
       </c>
       <c r="C109" t="n">
-        <v>7.54</v>
+        <v>21.47</v>
       </c>
       <c r="D109" t="n">
-        <v>2.45</v>
+        <v>2.24</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>GUJAPOLLO</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>28.25</v>
+        <v>386.25</v>
       </c>
       <c r="C110" t="n">
-        <v>28.94</v>
+        <v>394.9</v>
       </c>
       <c r="D110" t="n">
-        <v>2.44</v>
+        <v>2.24</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>HALDER</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>250.87</v>
+        <v>0.45</v>
       </c>
       <c r="C111" t="n">
-        <v>257</v>
+        <v>0.46</v>
       </c>
       <c r="D111" t="n">
-        <v>2.44</v>
+        <v>2.22</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>XTGLOBAL</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>1555.8</v>
+        <v>29.73</v>
       </c>
       <c r="C112" t="n">
-        <v>1593.8</v>
+        <v>30.39</v>
       </c>
       <c r="D112" t="n">
-        <v>2.44</v>
+        <v>2.22</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>STARPAPER</t>
+          <t>BASML</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>138.05</v>
+        <v>24.46</v>
       </c>
       <c r="C113" t="n">
-        <v>141.4</v>
+        <v>25</v>
       </c>
       <c r="D113" t="n">
-        <v>2.43</v>
+        <v>2.21</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>VSTL</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>115.22</v>
+        <v>13.69</v>
       </c>
       <c r="C114" t="n">
-        <v>118</v>
+        <v>13.99</v>
       </c>
       <c r="D114" t="n">
-        <v>2.41</v>
+        <v>2.19</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>KAPSTON</t>
+          <t>NEXTMEDIA</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>336.8</v>
+        <v>3.8</v>
       </c>
       <c r="C115" t="n">
-        <v>344.85</v>
+        <v>3.88</v>
       </c>
       <c r="D115" t="n">
-        <v>2.39</v>
+        <v>2.11</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>KSR</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.42</v>
+        <v>33</v>
       </c>
       <c r="C116" t="n">
-        <v>0.43</v>
+        <v>33.69</v>
       </c>
       <c r="D116" t="n">
-        <v>2.38</v>
+        <v>2.09</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>JUNIPER</t>
+          <t>VCL</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>201.21</v>
+        <v>1.44</v>
       </c>
       <c r="C117" t="n">
-        <v>206</v>
+        <v>1.47</v>
       </c>
       <c r="D117" t="n">
-        <v>2.38</v>
+        <v>2.08</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CUBEXTUB</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>87.23</v>
+        <v>4.83</v>
       </c>
       <c r="C118" t="n">
-        <v>89.28</v>
+        <v>4.93</v>
       </c>
       <c r="D118" t="n">
-        <v>2.35</v>
+        <v>2.07</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>REGAAL</t>
+          <t>HGINFRA</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>83.73999999999999</v>
+        <v>548.65</v>
       </c>
       <c r="C119" t="n">
-        <v>85.7</v>
+        <v>560</v>
       </c>
       <c r="D119" t="n">
-        <v>2.34</v>
+        <v>2.07</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>TEXINFRA</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>100.55</v>
+        <v>314.34</v>
       </c>
       <c r="C120" t="n">
-        <v>102.9</v>
+        <v>320.8</v>
       </c>
       <c r="D120" t="n">
-        <v>2.34</v>
+        <v>2.06</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>AVADHSUGAR</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>476.85</v>
+        <v>6.78</v>
       </c>
       <c r="C121" t="n">
-        <v>488</v>
+        <v>6.92</v>
       </c>
       <c r="D121" t="n">
-        <v>2.34</v>
+        <v>2.06</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>GANDHAR</t>
+          <t>GOLDTECH</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>161.85</v>
+        <v>44.88</v>
       </c>
       <c r="C122" t="n">
-        <v>165.64</v>
+        <v>45.79</v>
       </c>
       <c r="D122" t="n">
-        <v>2.34</v>
+        <v>2.03</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ZUARI</t>
+          <t>IRISDOREME</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>217.95</v>
+        <v>36.76</v>
       </c>
       <c r="C123" t="n">
-        <v>223.02</v>
+        <v>37.5</v>
       </c>
       <c r="D123" t="n">
-        <v>2.33</v>
+        <v>2.01</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>1171</v>
+        <v>13.55</v>
       </c>
       <c r="C124" t="n">
-        <v>1198</v>
+        <v>13.82</v>
       </c>
       <c r="D124" t="n">
-        <v>2.31</v>
+        <v>1.99</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>DCM</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>4.76</v>
+        <v>98.03</v>
       </c>
       <c r="C125" t="n">
-        <v>4.87</v>
+        <v>99.98</v>
       </c>
       <c r="D125" t="n">
-        <v>2.31</v>
+        <v>1.99</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>6.05</v>
+        <v>8.09</v>
       </c>
       <c r="C126" t="n">
-        <v>6.19</v>
+        <v>8.25</v>
       </c>
       <c r="D126" t="n">
-        <v>2.31</v>
+        <v>1.98</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>IGCL</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>57.06</v>
+        <v>19.39</v>
       </c>
       <c r="C127" t="n">
-        <v>58.38</v>
+        <v>19.77</v>
       </c>
       <c r="D127" t="n">
-        <v>2.31</v>
+        <v>1.96</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>6.52</v>
+        <v>2.05</v>
       </c>
       <c r="C128" t="n">
-        <v>6.67</v>
+        <v>2.09</v>
       </c>
       <c r="D128" t="n">
-        <v>2.3</v>
+        <v>1.95</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ELDEHSG</t>
+          <t>HILINFRA</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>786.7</v>
+        <v>47.28</v>
       </c>
       <c r="C129" t="n">
-        <v>804.8</v>
+        <v>48.2</v>
       </c>
       <c r="D129" t="n">
-        <v>2.3</v>
+        <v>1.95</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CENTEXT</t>
+          <t>HTMEDIA</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>19.53</v>
+        <v>23.06</v>
       </c>
       <c r="C130" t="n">
-        <v>19.98</v>
+        <v>23.5</v>
       </c>
       <c r="D130" t="n">
-        <v>2.3</v>
+        <v>1.91</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>AJOONI</t>
+          <t>GUJRAFFIA</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>3.91</v>
+        <v>42.5</v>
       </c>
       <c r="C131" t="n">
-        <v>4</v>
+        <v>43.3</v>
       </c>
       <c r="D131" t="n">
-        <v>2.3</v>
+        <v>1.88</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>TARMAT</t>
+          <t>AKASH</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>52.31</v>
+        <v>27.73</v>
       </c>
       <c r="C132" t="n">
-        <v>53.51</v>
+        <v>28.25</v>
       </c>
       <c r="D132" t="n">
-        <v>2.29</v>
+        <v>1.88</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>SHANTIGOLD</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>633.55</v>
+        <v>221.13</v>
       </c>
       <c r="C133" t="n">
-        <v>648</v>
+        <v>225.1</v>
       </c>
       <c r="D133" t="n">
-        <v>2.28</v>
+        <v>1.8</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>PIGL</t>
+          <t>DENORA</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>101.67</v>
+        <v>765.5</v>
       </c>
       <c r="C134" t="n">
-        <v>103.99</v>
+        <v>779</v>
       </c>
       <c r="D134" t="n">
-        <v>2.28</v>
+        <v>1.76</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MANAKALUCO</t>
+          <t>ZIMLAB</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>35.59</v>
+        <v>105.12</v>
       </c>
       <c r="C135" t="n">
-        <v>36.4</v>
+        <v>106.94</v>
       </c>
       <c r="D135" t="n">
-        <v>2.28</v>
+        <v>1.73</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>BPL</t>
+          <t>VIVIMEDLAB</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>51.82</v>
+        <v>6.39</v>
       </c>
       <c r="C136" t="n">
-        <v>53</v>
+        <v>6.5</v>
       </c>
       <c r="D136" t="n">
-        <v>2.28</v>
+        <v>1.72</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>235.68</v>
+        <v>318.55</v>
       </c>
       <c r="C137" t="n">
-        <v>241</v>
+        <v>324</v>
       </c>
       <c r="D137" t="n">
-        <v>2.26</v>
+        <v>1.71</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SUNFLAG</t>
+          <t>PRIMESECU</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>406.85</v>
+        <v>300.9</v>
       </c>
       <c r="C138" t="n">
-        <v>416</v>
+        <v>306</v>
       </c>
       <c r="D138" t="n">
-        <v>2.25</v>
+        <v>1.69</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>HPAL</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>37.17</v>
+        <v>40.71</v>
       </c>
       <c r="C139" t="n">
-        <v>38</v>
+        <v>41.4</v>
       </c>
       <c r="D139" t="n">
-        <v>2.23</v>
+        <v>1.69</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>338.85</v>
+        <v>1.18</v>
       </c>
       <c r="C140" t="n">
-        <v>346.4</v>
+        <v>1.2</v>
       </c>
       <c r="D140" t="n">
-        <v>2.23</v>
+        <v>1.69</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>BYKE</t>
+          <t>INSPIRISYS</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>35.2</v>
+        <v>114.74</v>
       </c>
       <c r="C141" t="n">
-        <v>35.98</v>
+        <v>116.59</v>
       </c>
       <c r="D141" t="n">
-        <v>2.22</v>
+        <v>1.61</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>LIKHITHA</t>
+          <t>BLUECHIP</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>209.84</v>
+        <v>2.49</v>
       </c>
       <c r="C142" t="n">
-        <v>214.5</v>
+        <v>2.53</v>
       </c>
       <c r="D142" t="n">
-        <v>2.22</v>
+        <v>1.61</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>VHL</t>
+          <t>VIRINCHI</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>3404.2</v>
+        <v>15.23</v>
       </c>
       <c r="C143" t="n">
-        <v>3479.7</v>
+        <v>15.47</v>
       </c>
       <c r="D143" t="n">
-        <v>2.22</v>
+        <v>1.58</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>KOTARISUG</t>
+          <t>HEXATRADEX</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>24.93</v>
+        <v>165.43</v>
       </c>
       <c r="C144" t="n">
-        <v>25.48</v>
+        <v>168</v>
       </c>
       <c r="D144" t="n">
-        <v>2.21</v>
+        <v>1.55</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>KOPRAN</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>4.99</v>
+        <v>189.08</v>
       </c>
       <c r="C145" t="n">
-        <v>5.1</v>
+        <v>192</v>
       </c>
       <c r="D145" t="n">
-        <v>2.2</v>
+        <v>1.54</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>7.34</v>
+        <v>20.39</v>
       </c>
       <c r="C146" t="n">
-        <v>7.5</v>
+        <v>20.7</v>
       </c>
       <c r="D146" t="n">
-        <v>2.18</v>
+        <v>1.52</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SABEVENTS</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>7.92</v>
+        <v>174.66</v>
       </c>
       <c r="C147" t="n">
-        <v>8.09</v>
+        <v>177.28</v>
       </c>
       <c r="D147" t="n">
-        <v>2.15</v>
+        <v>1.5</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>GSS</t>
+          <t>RFBL</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>13.49</v>
+        <v>70.25</v>
       </c>
       <c r="C148" t="n">
-        <v>13.78</v>
+        <v>71.3</v>
       </c>
       <c r="D148" t="n">
-        <v>2.15</v>
+        <v>1.49</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>FABTECH</t>
+          <t>METROGLOBL</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>149.29</v>
+        <v>128.99</v>
       </c>
       <c r="C149" t="n">
-        <v>152.5</v>
+        <v>130.9</v>
       </c>
       <c r="D149" t="n">
-        <v>2.15</v>
+        <v>1.48</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>JISLDVREQS</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>3124.7</v>
+        <v>23.16</v>
       </c>
       <c r="C150" t="n">
-        <v>3191.6</v>
+        <v>23.5</v>
       </c>
       <c r="D150" t="n">
-        <v>2.14</v>
+        <v>1.47</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>AUTOIND</t>
+          <t>MAHEPC</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>77.34</v>
+        <v>112.8</v>
       </c>
       <c r="C151" t="n">
-        <v>78.98999999999999</v>
+        <v>114.45</v>
       </c>
       <c r="D151" t="n">
-        <v>2.13</v>
+        <v>1.46</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>MURUDCERA</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>38.19</v>
+        <v>31.49</v>
       </c>
       <c r="C152" t="n">
-        <v>39</v>
+        <v>31.95</v>
       </c>
       <c r="D152" t="n">
-        <v>2.12</v>
+        <v>1.46</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>GICL</t>
+          <t>SOLARWORLD</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>26.93</v>
+        <v>191.75</v>
       </c>
       <c r="C153" t="n">
-        <v>27.5</v>
+        <v>194.49</v>
       </c>
       <c r="D153" t="n">
-        <v>2.12</v>
+        <v>1.43</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>COOLCAPS</t>
+          <t>MAGADSUGAR</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>21.3</v>
+        <v>453.25</v>
       </c>
       <c r="C154" t="n">
-        <v>21.75</v>
+        <v>459.7</v>
       </c>
       <c r="D154" t="n">
-        <v>2.11</v>
+        <v>1.42</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>7.15</v>
+        <v>3.56</v>
       </c>
       <c r="C155" t="n">
-        <v>7.3</v>
+        <v>3.61</v>
       </c>
       <c r="D155" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>RBZJEWEL</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>6.66</v>
+        <v>132.7</v>
       </c>
       <c r="C156" t="n">
-        <v>6.8</v>
+        <v>134.54</v>
       </c>
       <c r="D156" t="n">
-        <v>2.1</v>
+        <v>1.39</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>BOSCH-HCIL</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>1395.8</v>
+        <v>209.09</v>
       </c>
       <c r="C157" t="n">
-        <v>1424.9</v>
+        <v>211.98</v>
       </c>
       <c r="D157" t="n">
-        <v>2.08</v>
+        <v>1.38</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>SAKUMA</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>1.93</v>
+        <v>1203.4</v>
       </c>
       <c r="C158" t="n">
-        <v>1.97</v>
+        <v>1220</v>
       </c>
       <c r="D158" t="n">
-        <v>2.07</v>
+        <v>1.38</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>HECPROJECT</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>907.55</v>
+        <v>121.93</v>
       </c>
       <c r="C159" t="n">
-        <v>926.3</v>
+        <v>123.55</v>
       </c>
       <c r="D159" t="n">
-        <v>2.07</v>
+        <v>1.33</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>RPPL</t>
+          <t>CAPITALSFB</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>18.91</v>
+        <v>269.4</v>
       </c>
       <c r="C160" t="n">
-        <v>19.3</v>
+        <v>272.95</v>
       </c>
       <c r="D160" t="n">
-        <v>2.06</v>
+        <v>1.32</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>GODIGIT</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>302.8</v>
+        <v>39.8</v>
       </c>
       <c r="C161" t="n">
-        <v>309</v>
+        <v>40.3</v>
       </c>
       <c r="D161" t="n">
-        <v>2.05</v>
+        <v>1.26</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>TIL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>0.49</v>
+        <v>176.33</v>
       </c>
       <c r="C162" t="n">
-        <v>0.5</v>
+        <v>178.48</v>
       </c>
       <c r="D162" t="n">
-        <v>2.04</v>
+        <v>1.22</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>REGAAL</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>4596.5</v>
+        <v>84.48</v>
       </c>
       <c r="C163" t="n">
-        <v>4690</v>
+        <v>85.5</v>
       </c>
       <c r="D163" t="n">
-        <v>2.03</v>
+        <v>1.21</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>LOVABLE</t>
+          <t>OILCOUNTUB</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>72.04000000000001</v>
+        <v>61.26</v>
       </c>
       <c r="C164" t="n">
-        <v>73.5</v>
+        <v>62</v>
       </c>
       <c r="D164" t="n">
-        <v>2.03</v>
+        <v>1.21</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>BBOX</t>
+          <t>CHEMFAB</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>1078.2</v>
+        <v>420</v>
       </c>
       <c r="C165" t="n">
-        <v>1100</v>
+        <v>425</v>
       </c>
       <c r="D165" t="n">
-        <v>2.02</v>
+        <v>1.19</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>PIONEEREMB</t>
+          <t>PONNIERODE</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>23.42</v>
+        <v>339.6</v>
       </c>
       <c r="C166" t="n">
-        <v>23.89</v>
+        <v>343.65</v>
       </c>
       <c r="D166" t="n">
-        <v>2.01</v>
+        <v>1.19</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>DPEL</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>0.5</v>
+        <v>493.2</v>
       </c>
       <c r="C167" t="n">
-        <v>0.51</v>
+        <v>499</v>
       </c>
       <c r="D167" t="n">
-        <v>2</v>
+        <v>1.18</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>SURAJEST</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>44.89</v>
+        <v>186.69</v>
       </c>
       <c r="C168" t="n">
-        <v>45.79</v>
+        <v>188.9</v>
       </c>
       <c r="D168" t="n">
-        <v>2</v>
+        <v>1.18</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>VEEDOL</t>
+          <t>TAKE</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>1460.6</v>
+        <v>29.57</v>
       </c>
       <c r="C169" t="n">
-        <v>1489.6</v>
+        <v>29.92</v>
       </c>
       <c r="D169" t="n">
-        <v>1.99</v>
+        <v>1.18</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>DIGISPICE</t>
+          <t>VHL</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>20.06</v>
+        <v>3386.5</v>
       </c>
       <c r="C170" t="n">
-        <v>20.46</v>
+        <v>3425</v>
       </c>
       <c r="D170" t="n">
-        <v>1.99</v>
+        <v>1.14</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>AAATECH</t>
+          <t>ORIENTCER</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>91.19</v>
+        <v>38.37</v>
       </c>
       <c r="C171" t="n">
-        <v>93</v>
+        <v>38.8</v>
       </c>
       <c r="D171" t="n">
-        <v>1.98</v>
+        <v>1.12</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>LOKESHMACH</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>7.11</v>
+        <v>250.2</v>
       </c>
       <c r="C172" t="n">
-        <v>7.25</v>
+        <v>253</v>
       </c>
       <c r="D172" t="n">
-        <v>1.97</v>
+        <v>1.12</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>NITIRAJ</t>
+          <t>ANTELOPUS</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>184.07</v>
+        <v>899.35</v>
       </c>
       <c r="C173" t="n">
-        <v>187.7</v>
+        <v>909.4</v>
       </c>
       <c r="D173" t="n">
-        <v>1.97</v>
+        <v>1.12</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SAGARDEEP</t>
+          <t>OSWALAGRO</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>25.47</v>
+        <v>42.52</v>
       </c>
       <c r="C174" t="n">
-        <v>25.97</v>
+        <v>42.98</v>
       </c>
       <c r="D174" t="n">
-        <v>1.96</v>
+        <v>1.08</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>PRIMO</t>
+          <t>GENUSPAPER</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>21.97</v>
+        <v>12.32</v>
       </c>
       <c r="C175" t="n">
-        <v>22.4</v>
+        <v>12.45</v>
       </c>
       <c r="D175" t="n">
-        <v>1.96</v>
+        <v>1.06</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>BODALCHEM</t>
+          <t>3IINFOLTD</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>71.59</v>
+        <v>17.07</v>
       </c>
       <c r="C176" t="n">
-        <v>72.98999999999999</v>
+        <v>17.25</v>
       </c>
       <c r="D176" t="n">
-        <v>1.96</v>
+        <v>1.05</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>DHAMPURSUG</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>39.41</v>
+        <v>142.51</v>
       </c>
       <c r="C177" t="n">
-        <v>40.18</v>
+        <v>143.99</v>
       </c>
       <c r="D177" t="n">
-        <v>1.95</v>
+        <v>1.04</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>SAKHTISUG</t>
+          <t>RCOM</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>17.4</v>
+        <v>0.97</v>
       </c>
       <c r="C178" t="n">
-        <v>17.74</v>
+        <v>0.98</v>
       </c>
       <c r="D178" t="n">
-        <v>1.95</v>
+        <v>1.03</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>QLINE</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>3.62</v>
+        <v>494.85</v>
       </c>
       <c r="C179" t="n">
-        <v>3.69</v>
+        <v>499.9</v>
       </c>
       <c r="D179" t="n">
-        <v>1.93</v>
+        <v>1.02</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ADISOFT</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>209.85</v>
+        <v>4.93</v>
       </c>
       <c r="C180" t="n">
-        <v>213.9</v>
+        <v>4.98</v>
       </c>
       <c r="D180" t="n">
-        <v>1.93</v>
+        <v>1.01</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>FINEORG</t>
+          <t>SUTLEJTEX</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>4689.7</v>
+        <v>38.91</v>
       </c>
       <c r="C181" t="n">
-        <v>4779.9</v>
+        <v>39.3</v>
       </c>
       <c r="D181" t="n">
-        <v>1.92</v>
+        <v>1</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>OMINFRAL</t>
+          <t>NECLIFE</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>85.26000000000001</v>
+        <v>11.98</v>
       </c>
       <c r="C182" t="n">
-        <v>86.89</v>
+        <v>12.1</v>
       </c>
       <c r="D182" t="n">
-        <v>1.91</v>
+        <v>1</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>GTLINFRA</t>
+          <t>IFGLEXPOR</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>1.57</v>
+        <v>194.77</v>
       </c>
       <c r="C183" t="n">
-        <v>1.6</v>
+        <v>196.7</v>
       </c>
       <c r="D183" t="n">
-        <v>1.91</v>
+        <v>0.99</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>JAYBARMARU</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>126.6</v>
+        <v>5.08</v>
       </c>
       <c r="C184" t="n">
-        <v>129</v>
+        <v>5.13</v>
       </c>
       <c r="D184" t="n">
-        <v>1.9</v>
+        <v>0.98</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>IRISDOREME</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>36.47</v>
+        <v>182.55</v>
       </c>
       <c r="C185" t="n">
-        <v>37.15</v>
+        <v>184.34</v>
       </c>
       <c r="D185" t="n">
-        <v>1.86</v>
+        <v>0.98</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>PANACEABIO</t>
+          <t>AFSL</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>520.3</v>
+        <v>201.03</v>
       </c>
       <c r="C186" t="n">
-        <v>530</v>
+        <v>202.96</v>
       </c>
       <c r="D186" t="n">
-        <v>1.86</v>
+        <v>0.96</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>ELECTHERM</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>3.24</v>
+        <v>970.6</v>
       </c>
       <c r="C187" t="n">
-        <v>3.3</v>
+        <v>979.3</v>
       </c>
       <c r="D187" t="n">
-        <v>1.85</v>
+        <v>0.9</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>VIGOR</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>70.7</v>
+        <v>13.97</v>
       </c>
       <c r="C188" t="n">
-        <v>72</v>
+        <v>14.09</v>
       </c>
       <c r="D188" t="n">
-        <v>1.84</v>
+        <v>0.86</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>KPL</t>
+          <t>ANANTAM</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>2375.2</v>
+        <v>104.5</v>
       </c>
       <c r="C189" t="n">
-        <v>2419</v>
+        <v>105.4</v>
       </c>
       <c r="D189" t="n">
-        <v>1.84</v>
+        <v>0.86</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>DBOL</t>
+          <t>DWARKESH</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>109.53</v>
+        <v>44.8</v>
       </c>
       <c r="C190" t="n">
-        <v>111.49</v>
+        <v>45.18</v>
       </c>
       <c r="D190" t="n">
-        <v>1.79</v>
+        <v>0.85</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>AXITA</t>
+          <t>HINDCOMPOS</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>7.8</v>
+        <v>414.5</v>
       </c>
       <c r="C191" t="n">
-        <v>7.94</v>
+        <v>418</v>
       </c>
       <c r="D191" t="n">
-        <v>1.79</v>
+        <v>0.84</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>MUKTAARTS</t>
+          <t>WANBURY</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>64.23999999999999</v>
+        <v>262.3</v>
       </c>
       <c r="C192" t="n">
-        <v>65.39</v>
+        <v>264.5</v>
       </c>
       <c r="D192" t="n">
-        <v>1.79</v>
+        <v>0.84</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>JSLL</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>651.9</v>
+        <v>356.95</v>
       </c>
       <c r="C193" t="n">
-        <v>663.5</v>
+        <v>359.9</v>
       </c>
       <c r="D193" t="n">
-        <v>1.78</v>
+        <v>0.83</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>THEJO</t>
+          <t>YUKEN</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>1565.6</v>
+        <v>684.4</v>
       </c>
       <c r="C194" t="n">
-        <v>1593.5</v>
+        <v>690</v>
       </c>
       <c r="D194" t="n">
-        <v>1.78</v>
+        <v>0.82</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>RUSTOMJEE</t>
+          <t>PURPLEUTED</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>392.35</v>
+        <v>395.85</v>
       </c>
       <c r="C195" t="n">
-        <v>399.35</v>
+        <v>399</v>
       </c>
       <c r="D195" t="n">
-        <v>1.78</v>
+        <v>0.8</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>MENONBE</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>62.88</v>
+        <v>138.71</v>
       </c>
       <c r="C196" t="n">
-        <v>63.99</v>
+        <v>139.75</v>
       </c>
       <c r="D196" t="n">
-        <v>1.77</v>
+        <v>0.75</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>SUNDARAM</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>2.26</v>
+        <v>1.35</v>
       </c>
       <c r="C197" t="n">
-        <v>2.3</v>
+        <v>1.36</v>
       </c>
       <c r="D197" t="n">
-        <v>1.77</v>
+        <v>0.74</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>AARTECH</t>
+          <t>SADBHAV</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>41.96</v>
+        <v>9.57</v>
       </c>
       <c r="C198" t="n">
-        <v>42.7</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="D198" t="n">
-        <v>1.76</v>
+        <v>0.73</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>KSB</t>
+          <t>PENINLAND</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>795.55</v>
+        <v>15.48</v>
       </c>
       <c r="C199" t="n">
-        <v>809.5</v>
+        <v>15.59</v>
       </c>
       <c r="D199" t="n">
-        <v>1.75</v>
+        <v>0.71</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>BCLIND</t>
+          <t>MUKANDLTD</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>32.24</v>
+        <v>138.96</v>
       </c>
       <c r="C200" t="n">
-        <v>32.8</v>
+        <v>139.95</v>
       </c>
       <c r="D200" t="n">
-        <v>1.74</v>
+        <v>0.71</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>SRM</t>
+          <t>BALAXI</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>490.15</v>
+        <v>24.28</v>
       </c>
       <c r="C201" t="n">
-        <v>498.7</v>
+        <v>24.45</v>
       </c>
       <c r="D201" t="n">
-        <v>1.74</v>
+        <v>0.7</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-09 07:05 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>630.65</v>
+        <v>15.52</v>
       </c>
       <c r="C2" t="n">
-        <v>756.75</v>
+        <v>18.6</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>19.85</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FLEXITUFF</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.93</v>
+        <v>48.59</v>
       </c>
       <c r="C3" t="n">
-        <v>7.7</v>
+        <v>52.59</v>
       </c>
       <c r="D3" t="n">
-        <v>11.11</v>
+        <v>8.23</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ORTINGLOBE</t>
+          <t>BAFNAPH</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18.11</v>
+        <v>193.97</v>
       </c>
       <c r="C4" t="n">
-        <v>19.92</v>
+        <v>209.7</v>
       </c>
       <c r="D4" t="n">
-        <v>9.99</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>YCCL</t>
+          <t>JNKINDIA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9.65</v>
+        <v>418.35</v>
       </c>
       <c r="C5" t="n">
-        <v>10.5</v>
+        <v>450.15</v>
       </c>
       <c r="D5" t="n">
-        <v>8.81</v>
+        <v>7.6</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SVLL</t>
+          <t>GRAVISSHO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>747.9</v>
+        <v>28.5</v>
       </c>
       <c r="C6" t="n">
-        <v>800</v>
+        <v>30.65</v>
       </c>
       <c r="D6" t="n">
-        <v>6.97</v>
+        <v>7.54</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BAFNAPH</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>176.34</v>
+        <v>4.77</v>
       </c>
       <c r="C7" t="n">
-        <v>187.4</v>
+        <v>5.1</v>
       </c>
       <c r="D7" t="n">
-        <v>6.27</v>
+        <v>6.92</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AGRITECH</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>129.34</v>
+        <v>1.9</v>
       </c>
       <c r="C8" t="n">
-        <v>136.99</v>
+        <v>2.02</v>
       </c>
       <c r="D8" t="n">
-        <v>5.91</v>
+        <v>6.32</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SBGLP</t>
+          <t>MAGNUM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24.37</v>
+        <v>19.66</v>
       </c>
       <c r="C9" t="n">
-        <v>25.74</v>
+        <v>20.88</v>
       </c>
       <c r="D9" t="n">
-        <v>5.62</v>
+        <v>6.21</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PFOCUS</t>
+          <t>VIPULLTD</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>240.19</v>
+        <v>10.1</v>
       </c>
       <c r="C10" t="n">
-        <v>252.19</v>
+        <v>10.7</v>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>5.94</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>QPOWER</t>
+          <t>KANANIIND</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1072</v>
+        <v>1.56</v>
       </c>
       <c r="C11" t="n">
-        <v>1125.6</v>
+        <v>1.65</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>5.77</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SICALLOG</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>72.23999999999999</v>
+        <v>11.97</v>
       </c>
       <c r="C12" t="n">
-        <v>75.84999999999999</v>
+        <v>12.64</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>5.6</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SUPREMEENG</t>
+          <t>STARTECK</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>269.8</v>
       </c>
       <c r="C13" t="n">
-        <v>1.05</v>
+        <v>283.95</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>5.24</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GOLDENTOBC</t>
+          <t>SILKFLEX</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>25.06</v>
+        <v>190</v>
       </c>
       <c r="C14" t="n">
-        <v>26.31</v>
+        <v>199.5</v>
       </c>
       <c r="D14" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DCMSIL</t>
+          <t>SICALLOG</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>65.34</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="C15" t="n">
-        <v>68.59999999999999</v>
+        <v>79.64</v>
       </c>
       <c r="D15" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RNPL</t>
+          <t>TANKUP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>87.2</v>
+        <v>1001.8</v>
       </c>
       <c r="C16" t="n">
-        <v>91.55</v>
+        <v>1051.85</v>
       </c>
       <c r="D16" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CLEDUCATE</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>53.78</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>56.46</v>
+        <v>2.1</v>
       </c>
       <c r="D17" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GENSOL</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>23.74</v>
+        <v>963.25</v>
       </c>
       <c r="C18" t="n">
-        <v>24.92</v>
+        <v>1011.4</v>
       </c>
       <c r="D18" t="n">
-        <v>4.97</v>
+        <v>5</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>48.35</v>
+        <v>14.24</v>
       </c>
       <c r="C19" t="n">
-        <v>50.75</v>
+        <v>14.95</v>
       </c>
       <c r="D19" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GANESHIN</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>82.84999999999999</v>
+        <v>17.43</v>
       </c>
       <c r="C20" t="n">
-        <v>86.95</v>
+        <v>18.3</v>
       </c>
       <c r="D20" t="n">
-        <v>4.95</v>
+        <v>4.99</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AGSTRA</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2.83</v>
+        <v>36.1</v>
       </c>
       <c r="C21" t="n">
-        <v>2.97</v>
+        <v>37.9</v>
       </c>
       <c r="D21" t="n">
-        <v>4.95</v>
+        <v>4.99</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SIMBHALS</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6.7</v>
+        <v>6.24</v>
       </c>
       <c r="C22" t="n">
-        <v>7.03</v>
+        <v>6.55</v>
       </c>
       <c r="D22" t="n">
-        <v>4.93</v>
+        <v>4.97</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>MCON</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>14.67</v>
+        <v>52.4</v>
       </c>
       <c r="C23" t="n">
-        <v>15.39</v>
+        <v>55</v>
       </c>
       <c r="D23" t="n">
-        <v>4.91</v>
+        <v>4.96</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SATIPOLY</t>
+          <t>SHIVAMILLS</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>36.15</v>
+        <v>63.95</v>
       </c>
       <c r="C24" t="n">
-        <v>37.9</v>
+        <v>67.12</v>
       </c>
       <c r="D24" t="n">
-        <v>4.84</v>
+        <v>4.96</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MUNISH</t>
+          <t>IMPEXFERRO</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>60.8</v>
+        <v>2.42</v>
       </c>
       <c r="C25" t="n">
-        <v>63.7</v>
+        <v>2.54</v>
       </c>
       <c r="D25" t="n">
-        <v>4.77</v>
+        <v>4.96</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>KSR</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2.31</v>
+        <v>32.17</v>
       </c>
       <c r="C26" t="n">
-        <v>2.42</v>
+        <v>33.76</v>
       </c>
       <c r="D26" t="n">
-        <v>4.76</v>
+        <v>4.94</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>UFBL</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>506</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C27" t="n">
-        <v>530</v>
+        <v>0.85</v>
       </c>
       <c r="D27" t="n">
-        <v>4.74</v>
+        <v>4.94</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5.96</v>
+        <v>4.28</v>
       </c>
       <c r="C28" t="n">
-        <v>6.24</v>
+        <v>4.49</v>
       </c>
       <c r="D28" t="n">
-        <v>4.7</v>
+        <v>4.91</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GTECJAINX</t>
+          <t>CHETANA</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>34.87</v>
+        <v>46.85</v>
       </c>
       <c r="C29" t="n">
-        <v>36.49</v>
+        <v>49.15</v>
       </c>
       <c r="D29" t="n">
-        <v>4.65</v>
+        <v>4.91</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>BETA</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>15.73</v>
+        <v>1430.1</v>
       </c>
       <c r="C30" t="n">
-        <v>16.45</v>
+        <v>1500</v>
       </c>
       <c r="D30" t="n">
-        <v>4.58</v>
+        <v>4.89</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DHRUV</t>
+          <t>DIVYADHAN</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>28.68</v>
+        <v>33.75</v>
       </c>
       <c r="C31" t="n">
-        <v>29.99</v>
+        <v>35.4</v>
       </c>
       <c r="D31" t="n">
-        <v>4.57</v>
+        <v>4.89</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>SYNOPTICS</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.22</v>
+        <v>58.35</v>
       </c>
       <c r="C32" t="n">
-        <v>0.23</v>
+        <v>61.2</v>
       </c>
       <c r="D32" t="n">
-        <v>4.55</v>
+        <v>4.88</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>NORBTEAEXP</t>
+          <t>SYSTMTXC</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>76.94</v>
+        <v>65.52</v>
       </c>
       <c r="C33" t="n">
-        <v>80.40000000000001</v>
+        <v>68.7</v>
       </c>
       <c r="D33" t="n">
-        <v>4.5</v>
+        <v>4.85</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RACE</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>109.14</v>
+        <v>40.65</v>
       </c>
       <c r="C34" t="n">
-        <v>114</v>
+        <v>42.6</v>
       </c>
       <c r="D34" t="n">
-        <v>4.45</v>
+        <v>4.8</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>SUPREMEENG</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>11.25</v>
+        <v>1.05</v>
       </c>
       <c r="C35" t="n">
-        <v>11.74</v>
+        <v>1.1</v>
       </c>
       <c r="D35" t="n">
-        <v>4.36</v>
+        <v>4.76</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>LIKHITHA</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>18.64</v>
+        <v>227.2</v>
       </c>
       <c r="C36" t="n">
-        <v>19.45</v>
+        <v>238</v>
       </c>
       <c r="D36" t="n">
-        <v>4.35</v>
+        <v>4.75</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>PANAMAPET</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>26.59</v>
+        <v>334.75</v>
       </c>
       <c r="C37" t="n">
-        <v>27.69</v>
+        <v>350.55</v>
       </c>
       <c r="D37" t="n">
-        <v>4.14</v>
+        <v>4.72</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MCON</t>
+          <t>TREJHARA</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>49.95</v>
+        <v>137.42</v>
       </c>
       <c r="C38" t="n">
-        <v>52</v>
+        <v>143.9</v>
       </c>
       <c r="D38" t="n">
-        <v>4.1</v>
+        <v>4.72</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>A2ZINFRA</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>34.39</v>
+        <v>14.21</v>
       </c>
       <c r="C39" t="n">
-        <v>35.8</v>
+        <v>14.88</v>
       </c>
       <c r="D39" t="n">
-        <v>4.1</v>
+        <v>4.71</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SYSTMTXC</t>
+          <t>SVLL</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>66.34</v>
+        <v>849.15</v>
       </c>
       <c r="C40" t="n">
-        <v>69</v>
+        <v>888.9</v>
       </c>
       <c r="D40" t="n">
-        <v>4.01</v>
+        <v>4.68</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AKCAPIT</t>
+          <t>AURIONPRO</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1712</v>
+        <v>743.1</v>
       </c>
       <c r="C41" t="n">
-        <v>1780</v>
+        <v>777</v>
       </c>
       <c r="D41" t="n">
-        <v>3.97</v>
+        <v>4.56</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>RELINFRA</t>
+          <t>UMESLTD</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>81.76000000000001</v>
+        <v>5.53</v>
       </c>
       <c r="C42" t="n">
-        <v>84.98999999999999</v>
+        <v>5.78</v>
       </c>
       <c r="D42" t="n">
-        <v>3.95</v>
+        <v>4.52</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>FMNL</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1.78</v>
+        <v>10.22</v>
       </c>
       <c r="C43" t="n">
-        <v>1.85</v>
+        <v>10.68</v>
       </c>
       <c r="D43" t="n">
-        <v>3.93</v>
+        <v>4.5</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ASTRON</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3.85</v>
+        <v>40.92</v>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>42.76</v>
       </c>
       <c r="D44" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SILLYMONKS</t>
+          <t>CAPTRUST</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>16.8</v>
+        <v>13.37</v>
       </c>
       <c r="C45" t="n">
-        <v>17.45</v>
+        <v>13.97</v>
       </c>
       <c r="D45" t="n">
-        <v>3.87</v>
+        <v>4.49</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PERFECT</t>
+          <t>MASTERTR</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2.7</v>
+        <v>92.02</v>
       </c>
       <c r="C46" t="n">
-        <v>2.8</v>
+        <v>96.14</v>
       </c>
       <c r="D46" t="n">
-        <v>3.7</v>
+        <v>4.48</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.54</v>
+        <v>16.3</v>
       </c>
       <c r="C47" t="n">
-        <v>0.5600000000000001</v>
+        <v>17</v>
       </c>
       <c r="D47" t="n">
-        <v>3.7</v>
+        <v>4.29</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>QUINT</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>39.51</v>
+        <v>86.25</v>
       </c>
       <c r="C48" t="n">
-        <v>40.9</v>
+        <v>89.95</v>
       </c>
       <c r="D48" t="n">
-        <v>3.52</v>
+        <v>4.29</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>35.26</v>
+        <v>14.27</v>
       </c>
       <c r="C49" t="n">
-        <v>36.5</v>
+        <v>14.88</v>
       </c>
       <c r="D49" t="n">
-        <v>3.52</v>
+        <v>4.27</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DELTAMAGNT</t>
+          <t>PASUPTAC</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>60.08</v>
+        <v>74.34</v>
       </c>
       <c r="C50" t="n">
-        <v>62.19</v>
+        <v>77.5</v>
       </c>
       <c r="D50" t="n">
-        <v>3.51</v>
+        <v>4.25</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>UNIINFO</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>11.69</v>
+        <v>4.8</v>
       </c>
       <c r="C51" t="n">
-        <v>12.1</v>
+        <v>5</v>
       </c>
       <c r="D51" t="n">
-        <v>3.51</v>
+        <v>4.17</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PML</t>
+          <t>PANACEABIO</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>500.95</v>
+        <v>552.9</v>
       </c>
       <c r="C52" t="n">
-        <v>518.5</v>
+        <v>575.85</v>
       </c>
       <c r="D52" t="n">
-        <v>3.5</v>
+        <v>4.15</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>UNIENTER</t>
+          <t>HPAL</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>105.24</v>
+        <v>35.53</v>
       </c>
       <c r="C53" t="n">
-        <v>108.9</v>
+        <v>36.98</v>
       </c>
       <c r="D53" t="n">
-        <v>3.48</v>
+        <v>4.08</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>AKG</t>
+          <t>SUPREME</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>11.21</v>
+        <v>44.98</v>
       </c>
       <c r="C54" t="n">
-        <v>11.6</v>
+        <v>46.79</v>
       </c>
       <c r="D54" t="n">
-        <v>3.48</v>
+        <v>4.02</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SWARAJ</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>240.6</v>
+        <v>89.22</v>
       </c>
       <c r="C55" t="n">
-        <v>248.95</v>
+        <v>92.8</v>
       </c>
       <c r="D55" t="n">
-        <v>3.47</v>
+        <v>4.01</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SINTERCOM</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>72.48999999999999</v>
+        <v>31.47</v>
       </c>
       <c r="C56" t="n">
-        <v>75</v>
+        <v>32.7</v>
       </c>
       <c r="D56" t="n">
-        <v>3.46</v>
+        <v>3.91</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>KHAITANLTD</t>
+          <t>NEXTMEDIA</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>131.51</v>
+        <v>3.84</v>
       </c>
       <c r="C57" t="n">
-        <v>136</v>
+        <v>3.99</v>
       </c>
       <c r="D57" t="n">
-        <v>3.41</v>
+        <v>3.91</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DAMODARIND</t>
+          <t>INSPIRISYS</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>31.33</v>
+        <v>118.44</v>
       </c>
       <c r="C58" t="n">
-        <v>32.39</v>
+        <v>123</v>
       </c>
       <c r="D58" t="n">
-        <v>3.38</v>
+        <v>3.85</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MERCANTILE</t>
+          <t>TRF</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>25.16</v>
+        <v>218.8</v>
       </c>
       <c r="C59" t="n">
-        <v>26</v>
+        <v>226.9</v>
       </c>
       <c r="D59" t="n">
-        <v>3.34</v>
+        <v>3.7</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>TVTODAY</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1.52</v>
+        <v>110.1</v>
       </c>
       <c r="C60" t="n">
-        <v>1.57</v>
+        <v>114.08</v>
       </c>
       <c r="D60" t="n">
-        <v>3.29</v>
+        <v>3.61</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>DBSTOCKBRO</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>31.95</v>
+        <v>37.87</v>
       </c>
       <c r="C61" t="n">
-        <v>32.99</v>
+        <v>39.2</v>
       </c>
       <c r="D61" t="n">
-        <v>3.26</v>
+        <v>3.51</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>DHUNINV</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>14.53</v>
+        <v>771.05</v>
       </c>
       <c r="C62" t="n">
-        <v>15</v>
+        <v>798</v>
       </c>
       <c r="D62" t="n">
-        <v>3.23</v>
+        <v>3.5</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>AERONEU</t>
+          <t>BIL</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>87.58</v>
+        <v>698.05</v>
       </c>
       <c r="C63" t="n">
-        <v>90.40000000000001</v>
+        <v>722.5</v>
       </c>
       <c r="D63" t="n">
-        <v>3.22</v>
+        <v>3.5</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>HECPROJECT</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>18.5</v>
+        <v>121.55</v>
       </c>
       <c r="C64" t="n">
-        <v>19.09</v>
+        <v>125.79</v>
       </c>
       <c r="D64" t="n">
-        <v>3.19</v>
+        <v>3.49</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>6.28</v>
+        <v>41.46</v>
       </c>
       <c r="C65" t="n">
-        <v>6.48</v>
+        <v>42.9</v>
       </c>
       <c r="D65" t="n">
-        <v>3.18</v>
+        <v>3.47</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>50.11</v>
+        <v>2.32</v>
       </c>
       <c r="C66" t="n">
-        <v>51.7</v>
+        <v>2.4</v>
       </c>
       <c r="D66" t="n">
-        <v>3.17</v>
+        <v>3.45</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SHRIKRISH</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>42.7</v>
+        <v>1.16</v>
       </c>
       <c r="C67" t="n">
-        <v>44</v>
+        <v>1.2</v>
       </c>
       <c r="D67" t="n">
-        <v>3.04</v>
+        <v>3.45</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>AURIGROW</t>
+          <t>MERCANTILE</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.33</v>
+        <v>26.39</v>
       </c>
       <c r="C68" t="n">
-        <v>0.34</v>
+        <v>27.3</v>
       </c>
       <c r="D68" t="n">
-        <v>3.03</v>
+        <v>3.45</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GFLLIMITED</t>
+          <t>SMARTLINK</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>46.98</v>
+        <v>164.35</v>
       </c>
       <c r="C69" t="n">
-        <v>48.4</v>
+        <v>170</v>
       </c>
       <c r="D69" t="n">
-        <v>3.02</v>
+        <v>3.44</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>AIROLAM</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>79.65000000000001</v>
+        <v>24.07</v>
       </c>
       <c r="C70" t="n">
-        <v>82.04000000000001</v>
+        <v>24.89</v>
       </c>
       <c r="D70" t="n">
-        <v>3</v>
+        <v>3.41</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>VILAS</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>19.8</v>
+        <v>355.8</v>
       </c>
       <c r="C71" t="n">
-        <v>20.39</v>
+        <v>367.95</v>
       </c>
       <c r="D71" t="n">
-        <v>2.98</v>
+        <v>3.41</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>TARMAT</t>
+          <t>IL&amp;FSENGG</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>51.77</v>
+        <v>29.01</v>
       </c>
       <c r="C72" t="n">
-        <v>53.29</v>
+        <v>30</v>
       </c>
       <c r="D72" t="n">
-        <v>2.94</v>
+        <v>3.41</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>HEADSUP</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>5.54</v>
+        <v>7.06</v>
       </c>
       <c r="C73" t="n">
-        <v>5.7</v>
+        <v>7.3</v>
       </c>
       <c r="D73" t="n">
-        <v>2.89</v>
+        <v>3.4</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BMLL</t>
+          <t>BANSWRAS</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>122.5</v>
+        <v>117.98</v>
       </c>
       <c r="C74" t="n">
-        <v>126</v>
+        <v>121.99</v>
       </c>
       <c r="D74" t="n">
-        <v>2.86</v>
+        <v>3.4</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BILVYAPAR</t>
+          <t>COOLCAPS</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>4.28</v>
+        <v>23.6</v>
       </c>
       <c r="C75" t="n">
-        <v>4.4</v>
+        <v>24.4</v>
       </c>
       <c r="D75" t="n">
-        <v>2.8</v>
+        <v>3.39</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>NIBL</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>112.82</v>
+        <v>30.47</v>
       </c>
       <c r="C76" t="n">
-        <v>115.98</v>
+        <v>31.5</v>
       </c>
       <c r="D76" t="n">
-        <v>2.8</v>
+        <v>3.38</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SABEVENTS</t>
+          <t>ENERGYDEV</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>7.53</v>
+        <v>16.64</v>
       </c>
       <c r="C77" t="n">
-        <v>7.74</v>
+        <v>17.2</v>
       </c>
       <c r="D77" t="n">
-        <v>2.79</v>
+        <v>3.37</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>KDL</t>
+          <t>NIPPOBATRY</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>114.8</v>
+        <v>354.1</v>
       </c>
       <c r="C78" t="n">
-        <v>118</v>
+        <v>366</v>
       </c>
       <c r="D78" t="n">
-        <v>2.79</v>
+        <v>3.36</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>EMSLIMITED</t>
+          <t>ANLON</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>290.85</v>
+        <v>696.85</v>
       </c>
       <c r="C79" t="n">
-        <v>298.95</v>
+        <v>720</v>
       </c>
       <c r="D79" t="n">
-        <v>2.78</v>
+        <v>3.32</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SSDL</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>57.41</v>
+        <v>45.49</v>
       </c>
       <c r="C80" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="D80" t="n">
-        <v>2.77</v>
+        <v>3.32</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>DYNPRO</t>
+          <t>SONAMLTD</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>248.05</v>
+        <v>54.69</v>
       </c>
       <c r="C81" t="n">
-        <v>254.9</v>
+        <v>56.5</v>
       </c>
       <c r="D81" t="n">
-        <v>2.76</v>
+        <v>3.31</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>HEADSUP</t>
+          <t>BRNL</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>7.24</v>
+        <v>18.78</v>
       </c>
       <c r="C82" t="n">
-        <v>7.44</v>
+        <v>19.4</v>
       </c>
       <c r="D82" t="n">
-        <v>2.76</v>
+        <v>3.3</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>NILE</t>
+          <t>KHADIM</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1727.6</v>
+        <v>100.11</v>
       </c>
       <c r="C83" t="n">
-        <v>1774.9</v>
+        <v>103.4</v>
       </c>
       <c r="D83" t="n">
-        <v>2.74</v>
+        <v>3.29</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MANAKSIA</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>58.3</v>
+        <v>7.64</v>
       </c>
       <c r="C84" t="n">
-        <v>59.9</v>
+        <v>7.89</v>
       </c>
       <c r="D84" t="n">
-        <v>2.74</v>
+        <v>3.27</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>LASA</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.37</v>
+        <v>7.66</v>
       </c>
       <c r="C85" t="n">
-        <v>0.38</v>
+        <v>7.91</v>
       </c>
       <c r="D85" t="n">
-        <v>2.7</v>
+        <v>3.26</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>HMVL</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>24.84</v>
+        <v>84.65000000000001</v>
       </c>
       <c r="C86" t="n">
-        <v>25.5</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="D86" t="n">
-        <v>2.66</v>
+        <v>3.25</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>AARNAV</t>
+          <t>RELIABLE</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>24.99</v>
+        <v>145.23</v>
       </c>
       <c r="C87" t="n">
-        <v>25.65</v>
+        <v>149.95</v>
       </c>
       <c r="D87" t="n">
-        <v>2.64</v>
+        <v>3.25</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>HITECHGEAR</t>
+          <t>ALANKIT</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>562.2</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="C88" t="n">
-        <v>577</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="D88" t="n">
-        <v>2.63</v>
+        <v>3.17</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>OSWALSEEDS</t>
+          <t>BORORENEW</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>11.06</v>
+        <v>513.75</v>
       </c>
       <c r="C89" t="n">
-        <v>11.35</v>
+        <v>530</v>
       </c>
       <c r="D89" t="n">
-        <v>2.62</v>
+        <v>3.16</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SHIVATEX</t>
+          <t>SHEMAROO</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>146.59</v>
+        <v>109.35</v>
       </c>
       <c r="C90" t="n">
-        <v>150.4</v>
+        <v>112.79</v>
       </c>
       <c r="D90" t="n">
-        <v>2.6</v>
+        <v>3.15</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DEEDEV</t>
+          <t>OLAELEC</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>671.15</v>
+        <v>44.43</v>
       </c>
       <c r="C91" t="n">
-        <v>688</v>
+        <v>45.83</v>
       </c>
       <c r="D91" t="n">
-        <v>2.51</v>
+        <v>3.15</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>MFML</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>1.99</v>
+        <v>23.84</v>
       </c>
       <c r="C92" t="n">
-        <v>2.04</v>
+        <v>24.59</v>
       </c>
       <c r="D92" t="n">
-        <v>2.51</v>
+        <v>3.15</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>JALAN</t>
+          <t>IGCL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>2</v>
+        <v>55.04</v>
       </c>
       <c r="C93" t="n">
-        <v>2.05</v>
+        <v>56.77</v>
       </c>
       <c r="D93" t="n">
-        <v>2.5</v>
+        <v>3.14</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ASHOKAMET</t>
+          <t>TREL</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>15.2</v>
+        <v>25.41</v>
       </c>
       <c r="C94" t="n">
-        <v>15.58</v>
+        <v>26.2</v>
       </c>
       <c r="D94" t="n">
-        <v>2.5</v>
+        <v>3.11</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SMARTLINK</t>
+          <t>ARIES</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>159.05</v>
+        <v>322.65</v>
       </c>
       <c r="C95" t="n">
-        <v>163</v>
+        <v>332.65</v>
       </c>
       <c r="D95" t="n">
-        <v>2.48</v>
+        <v>3.1</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>HALDYNGL</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>16.57</v>
+        <v>114.46</v>
       </c>
       <c r="C96" t="n">
-        <v>16.98</v>
+        <v>118</v>
       </c>
       <c r="D96" t="n">
-        <v>2.47</v>
+        <v>3.09</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>NIPPOBATRY</t>
+          <t>SANATHAN</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>359.95</v>
+        <v>414.55</v>
       </c>
       <c r="C97" t="n">
-        <v>368.8</v>
+        <v>427.3</v>
       </c>
       <c r="D97" t="n">
-        <v>2.46</v>
+        <v>3.08</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>FEDDERSHOL</t>
+          <t>AYMSYNTEX</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>35.08</v>
+        <v>218.05</v>
       </c>
       <c r="C98" t="n">
-        <v>35.94</v>
+        <v>224.7</v>
       </c>
       <c r="D98" t="n">
-        <v>2.45</v>
+        <v>3.05</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CYBERMEDIA</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>16.9</v>
+        <v>5.57</v>
       </c>
       <c r="C99" t="n">
-        <v>17.31</v>
+        <v>5.74</v>
       </c>
       <c r="D99" t="n">
-        <v>2.43</v>
+        <v>3.05</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MOS</t>
+          <t>NACLIND</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>16.6</v>
+        <v>169.36</v>
       </c>
       <c r="C100" t="n">
-        <v>17</v>
+        <v>174.49</v>
       </c>
       <c r="D100" t="n">
-        <v>2.41</v>
+        <v>3.03</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>DNAMEDIA</t>
+          <t>PREMCO</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>2.93</v>
+        <v>364.8</v>
       </c>
       <c r="C101" t="n">
-        <v>3</v>
+        <v>375.8</v>
       </c>
       <c r="D101" t="n">
-        <v>2.39</v>
+        <v>3.02</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>AEPL</t>
+          <t>DRONE</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>16.3</v>
+        <v>39.8</v>
       </c>
       <c r="C102" t="n">
-        <v>16.68</v>
+        <v>41</v>
       </c>
       <c r="D102" t="n">
-        <v>2.33</v>
+        <v>3.02</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>HBESD</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>42.78</v>
+        <v>75.7</v>
       </c>
       <c r="C103" t="n">
-        <v>43.77</v>
+        <v>77.98</v>
       </c>
       <c r="D103" t="n">
-        <v>2.31</v>
+        <v>3.01</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>19.53</v>
+        <v>20.03</v>
       </c>
       <c r="C104" t="n">
-        <v>19.98</v>
+        <v>20.63</v>
       </c>
       <c r="D104" t="n">
-        <v>2.3</v>
+        <v>3</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>VIPULLTD</t>
+          <t>ORTINGLOBE</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>9.58</v>
+        <v>19.92</v>
       </c>
       <c r="C105" t="n">
-        <v>9.800000000000001</v>
+        <v>20.51</v>
       </c>
       <c r="D105" t="n">
-        <v>2.3</v>
+        <v>2.96</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>AURIGROW</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>10.44</v>
+        <v>0.35</v>
       </c>
       <c r="C106" t="n">
-        <v>10.68</v>
+        <v>0.36</v>
       </c>
       <c r="D106" t="n">
-        <v>2.3</v>
+        <v>2.86</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MIRZAINT</t>
+          <t>AXITA</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>30.06</v>
+        <v>7.77</v>
       </c>
       <c r="C107" t="n">
-        <v>30.75</v>
+        <v>7.99</v>
       </c>
       <c r="D107" t="n">
-        <v>2.3</v>
+        <v>2.83</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>MANAKSIA</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>7.52</v>
+        <v>58.06</v>
       </c>
       <c r="C108" t="n">
-        <v>7.69</v>
+        <v>59.7</v>
       </c>
       <c r="D108" t="n">
-        <v>2.26</v>
+        <v>2.82</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ODIGMA</t>
+          <t>BESTAGRO</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>21</v>
+        <v>15.95</v>
       </c>
       <c r="C109" t="n">
-        <v>21.47</v>
+        <v>16.4</v>
       </c>
       <c r="D109" t="n">
-        <v>2.24</v>
+        <v>2.82</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>GUJAPOLLO</t>
+          <t>DAMODARIND</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>386.25</v>
+        <v>30.16</v>
       </c>
       <c r="C110" t="n">
-        <v>394.9</v>
+        <v>31</v>
       </c>
       <c r="D110" t="n">
-        <v>2.24</v>
+        <v>2.79</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>CHEMFAB</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>0.45</v>
+        <v>407.35</v>
       </c>
       <c r="C111" t="n">
-        <v>0.46</v>
+        <v>418.7</v>
       </c>
       <c r="D111" t="n">
-        <v>2.22</v>
+        <v>2.79</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>IDEA</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>29.73</v>
+        <v>14.4</v>
       </c>
       <c r="C112" t="n">
-        <v>30.39</v>
+        <v>14.8</v>
       </c>
       <c r="D112" t="n">
-        <v>2.22</v>
+        <v>2.78</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>BASML</t>
+          <t>BBTCL</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>24.46</v>
+        <v>221.83</v>
       </c>
       <c r="C113" t="n">
-        <v>25</v>
+        <v>228</v>
       </c>
       <c r="D113" t="n">
-        <v>2.21</v>
+        <v>2.78</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>IFGLEXPOR</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>13.69</v>
+        <v>190.6</v>
       </c>
       <c r="C114" t="n">
-        <v>13.99</v>
+        <v>195.87</v>
       </c>
       <c r="D114" t="n">
-        <v>2.19</v>
+        <v>2.76</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>NEXTMEDIA</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>3.8</v>
+        <v>24.03</v>
       </c>
       <c r="C115" t="n">
-        <v>3.88</v>
+        <v>24.69</v>
       </c>
       <c r="D115" t="n">
-        <v>2.11</v>
+        <v>2.75</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>KSR</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>33</v>
+        <v>34.55</v>
       </c>
       <c r="C116" t="n">
-        <v>33.69</v>
+        <v>35.49</v>
       </c>
       <c r="D116" t="n">
-        <v>2.09</v>
+        <v>2.72</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>INDBANK</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>1.44</v>
+        <v>33.1</v>
       </c>
       <c r="C117" t="n">
-        <v>1.47</v>
+        <v>34</v>
       </c>
       <c r="D117" t="n">
-        <v>2.08</v>
+        <v>2.72</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>COUNCODOS</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>4.83</v>
+        <v>40.79</v>
       </c>
       <c r="C118" t="n">
-        <v>4.93</v>
+        <v>41.9</v>
       </c>
       <c r="D118" t="n">
-        <v>2.07</v>
+        <v>2.72</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>HGINFRA</t>
+          <t>CSLFINANCE</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>548.65</v>
+        <v>220.03</v>
       </c>
       <c r="C119" t="n">
-        <v>560</v>
+        <v>226</v>
       </c>
       <c r="D119" t="n">
-        <v>2.07</v>
+        <v>2.71</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>314.34</v>
+        <v>0.37</v>
       </c>
       <c r="C120" t="n">
-        <v>320.8</v>
+        <v>0.38</v>
       </c>
       <c r="D120" t="n">
-        <v>2.06</v>
+        <v>2.7</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>KABRAEXTRU</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>6.78</v>
+        <v>237.65</v>
       </c>
       <c r="C121" t="n">
-        <v>6.92</v>
+        <v>244</v>
       </c>
       <c r="D121" t="n">
-        <v>2.06</v>
+        <v>2.67</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>GOLDTECH</t>
+          <t>KAPSTON</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>44.88</v>
+        <v>329.7</v>
       </c>
       <c r="C122" t="n">
-        <v>45.79</v>
+        <v>338.5</v>
       </c>
       <c r="D122" t="n">
-        <v>2.03</v>
+        <v>2.67</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IRISDOREME</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>36.76</v>
+        <v>27.18</v>
       </c>
       <c r="C123" t="n">
-        <v>37.5</v>
+        <v>27.9</v>
       </c>
       <c r="D123" t="n">
-        <v>2.01</v>
+        <v>2.65</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>WABAG</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>13.55</v>
+        <v>1544.3</v>
       </c>
       <c r="C124" t="n">
-        <v>13.82</v>
+        <v>1585</v>
       </c>
       <c r="D124" t="n">
-        <v>1.99</v>
+        <v>2.64</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>DCM</t>
+          <t>VINYAS</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>98.03</v>
+        <v>1332.95</v>
       </c>
       <c r="C125" t="n">
-        <v>99.98</v>
+        <v>1368</v>
       </c>
       <c r="D125" t="n">
-        <v>1.99</v>
+        <v>2.63</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>UNIHEALTH</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>8.09</v>
+        <v>462.1</v>
       </c>
       <c r="C126" t="n">
-        <v>8.25</v>
+        <v>474</v>
       </c>
       <c r="D126" t="n">
-        <v>1.98</v>
+        <v>2.58</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>BELRISE</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>19.39</v>
+        <v>215.72</v>
       </c>
       <c r="C127" t="n">
-        <v>19.77</v>
+        <v>221.28</v>
       </c>
       <c r="D127" t="n">
-        <v>1.96</v>
+        <v>2.58</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>INDIANCARD</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>2.05</v>
+        <v>223.36</v>
       </c>
       <c r="C128" t="n">
-        <v>2.09</v>
+        <v>229</v>
       </c>
       <c r="D128" t="n">
-        <v>1.95</v>
+        <v>2.53</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>HILINFRA</t>
+          <t>SUPERSPIN</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>47.28</v>
+        <v>4.78</v>
       </c>
       <c r="C129" t="n">
-        <v>48.2</v>
+        <v>4.9</v>
       </c>
       <c r="D129" t="n">
-        <v>1.95</v>
+        <v>2.51</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>HTMEDIA</t>
+          <t>AMBALALSA</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>23.06</v>
+        <v>34.62</v>
       </c>
       <c r="C130" t="n">
-        <v>23.5</v>
+        <v>35.49</v>
       </c>
       <c r="D130" t="n">
-        <v>1.91</v>
+        <v>2.51</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>GUJRAFFIA</t>
+          <t>JAIPURKURT</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>42.5</v>
+        <v>28.83</v>
       </c>
       <c r="C131" t="n">
-        <v>43.3</v>
+        <v>29.55</v>
       </c>
       <c r="D131" t="n">
-        <v>1.88</v>
+        <v>2.5</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>AKASH</t>
+          <t>SAGARDEEP</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>27.73</v>
+        <v>24.98</v>
       </c>
       <c r="C132" t="n">
-        <v>28.25</v>
+        <v>25.6</v>
       </c>
       <c r="D132" t="n">
-        <v>1.88</v>
+        <v>2.48</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SHANTIGOLD</t>
+          <t>SECURKLOUD</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>221.13</v>
+        <v>20.19</v>
       </c>
       <c r="C133" t="n">
-        <v>225.1</v>
+        <v>20.69</v>
       </c>
       <c r="D133" t="n">
-        <v>1.8</v>
+        <v>2.48</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>DENORA</t>
+          <t>KOKUYOCMLN</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>765.5</v>
+        <v>82.8</v>
       </c>
       <c r="C134" t="n">
-        <v>779</v>
+        <v>84.84999999999999</v>
       </c>
       <c r="D134" t="n">
-        <v>1.76</v>
+        <v>2.48</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ZIMLAB</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>105.12</v>
+        <v>6.48</v>
       </c>
       <c r="C135" t="n">
-        <v>106.94</v>
+        <v>6.64</v>
       </c>
       <c r="D135" t="n">
-        <v>1.73</v>
+        <v>2.47</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>SARVESHWAR</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>6.39</v>
+        <v>3.66</v>
       </c>
       <c r="C136" t="n">
-        <v>6.5</v>
+        <v>3.75</v>
       </c>
       <c r="D136" t="n">
-        <v>1.72</v>
+        <v>2.46</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>318.55</v>
+        <v>80.03</v>
       </c>
       <c r="C137" t="n">
-        <v>324</v>
+        <v>82</v>
       </c>
       <c r="D137" t="n">
-        <v>1.71</v>
+        <v>2.46</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>PRIMESECU</t>
+          <t>GABRIEL</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>300.9</v>
+        <v>981</v>
       </c>
       <c r="C138" t="n">
-        <v>306</v>
+        <v>1005</v>
       </c>
       <c r="D138" t="n">
-        <v>1.69</v>
+        <v>2.45</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>PRITI</t>
+          <t>STEELCITY</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>40.71</v>
+        <v>76.83</v>
       </c>
       <c r="C139" t="n">
-        <v>41.4</v>
+        <v>78.7</v>
       </c>
       <c r="D139" t="n">
-        <v>1.69</v>
+        <v>2.43</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>IRB</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1.18</v>
+        <v>20.65</v>
       </c>
       <c r="C140" t="n">
-        <v>1.2</v>
+        <v>21.15</v>
       </c>
       <c r="D140" t="n">
-        <v>1.69</v>
+        <v>2.42</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>INSPIRISYS</t>
+          <t>BAIDFIN</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>114.74</v>
+        <v>9.98</v>
       </c>
       <c r="C141" t="n">
-        <v>116.59</v>
+        <v>10.22</v>
       </c>
       <c r="D141" t="n">
-        <v>1.61</v>
+        <v>2.4</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>BLUECHIP</t>
+          <t>NDL</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>2.49</v>
+        <v>2.51</v>
       </c>
       <c r="C142" t="n">
-        <v>2.53</v>
+        <v>2.57</v>
       </c>
       <c r="D142" t="n">
-        <v>1.61</v>
+        <v>2.39</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>VIRINCHI</t>
+          <t>TARC</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>15.23</v>
+        <v>123.07</v>
       </c>
       <c r="C143" t="n">
-        <v>15.47</v>
+        <v>126</v>
       </c>
       <c r="D143" t="n">
-        <v>1.58</v>
+        <v>2.38</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>HEXATRADEX</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>165.43</v>
+        <v>346.7</v>
       </c>
       <c r="C144" t="n">
-        <v>168</v>
+        <v>354.9</v>
       </c>
       <c r="D144" t="n">
-        <v>1.55</v>
+        <v>2.37</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>KOPRAN</t>
+          <t>VIKASECO</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>189.08</v>
+        <v>1.27</v>
       </c>
       <c r="C145" t="n">
-        <v>192</v>
+        <v>1.3</v>
       </c>
       <c r="D145" t="n">
-        <v>1.54</v>
+        <v>2.36</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>RAJRILTD</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>20.39</v>
+        <v>137.22</v>
       </c>
       <c r="C146" t="n">
-        <v>20.7</v>
+        <v>140.44</v>
       </c>
       <c r="D146" t="n">
-        <v>1.52</v>
+        <v>2.35</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>174.66</v>
+        <v>389.8</v>
       </c>
       <c r="C147" t="n">
-        <v>177.28</v>
+        <v>398.95</v>
       </c>
       <c r="D147" t="n">
-        <v>1.5</v>
+        <v>2.35</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>RFBL</t>
+          <t>LANDSMILL</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>70.25</v>
+        <v>0.87</v>
       </c>
       <c r="C148" t="n">
-        <v>71.3</v>
+        <v>0.89</v>
       </c>
       <c r="D148" t="n">
-        <v>1.49</v>
+        <v>2.3</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>METROGLOBL</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>128.99</v>
+        <v>96.8</v>
       </c>
       <c r="C149" t="n">
-        <v>130.9</v>
+        <v>99</v>
       </c>
       <c r="D149" t="n">
-        <v>1.48</v>
+        <v>2.27</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>JISLDVREQS</t>
+          <t>TCIEXP</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>23.16</v>
+        <v>513.05</v>
       </c>
       <c r="C150" t="n">
-        <v>23.5</v>
+        <v>524.6</v>
       </c>
       <c r="D150" t="n">
-        <v>1.47</v>
+        <v>2.25</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MAHEPC</t>
+          <t>FCL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>112.8</v>
+        <v>38.14</v>
       </c>
       <c r="C151" t="n">
-        <v>114.45</v>
+        <v>39</v>
       </c>
       <c r="D151" t="n">
-        <v>1.46</v>
+        <v>2.25</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MURUDCERA</t>
+          <t>BMWVENTLTD</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>31.49</v>
+        <v>60.12</v>
       </c>
       <c r="C152" t="n">
-        <v>31.95</v>
+        <v>61.47</v>
       </c>
       <c r="D152" t="n">
-        <v>1.46</v>
+        <v>2.25</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SOLARWORLD</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>191.75</v>
+        <v>44.88</v>
       </c>
       <c r="C153" t="n">
-        <v>194.49</v>
+        <v>45.88</v>
       </c>
       <c r="D153" t="n">
-        <v>1.43</v>
+        <v>2.23</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>MAGADSUGAR</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>453.25</v>
+        <v>54.68</v>
       </c>
       <c r="C154" t="n">
-        <v>459.7</v>
+        <v>55.9</v>
       </c>
       <c r="D154" t="n">
-        <v>1.42</v>
+        <v>2.23</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>GLOBE</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>3.56</v>
+        <v>2.25</v>
       </c>
       <c r="C155" t="n">
-        <v>3.61</v>
+        <v>2.3</v>
       </c>
       <c r="D155" t="n">
-        <v>1.4</v>
+        <v>2.22</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>RBZJEWEL</t>
+          <t>RBMINFRA</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>132.7</v>
+        <v>322.8</v>
       </c>
       <c r="C156" t="n">
-        <v>134.54</v>
+        <v>329.95</v>
       </c>
       <c r="D156" t="n">
-        <v>1.39</v>
+        <v>2.21</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>BHAGERIA</t>
+          <t>AIRAN</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>209.09</v>
+        <v>16.38</v>
       </c>
       <c r="C157" t="n">
-        <v>211.98</v>
+        <v>16.74</v>
       </c>
       <c r="D157" t="n">
-        <v>1.38</v>
+        <v>2.2</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>MMWL</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>1203.4</v>
+        <v>13.17</v>
       </c>
       <c r="C158" t="n">
-        <v>1220</v>
+        <v>13.46</v>
       </c>
       <c r="D158" t="n">
-        <v>1.38</v>
+        <v>2.2</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>HECPROJECT</t>
+          <t>KRONOX</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>121.93</v>
+        <v>132.29</v>
       </c>
       <c r="C159" t="n">
-        <v>123.55</v>
+        <v>135.2</v>
       </c>
       <c r="D159" t="n">
-        <v>1.33</v>
+        <v>2.2</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CAPITALSFB</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>269.4</v>
+        <v>5.49</v>
       </c>
       <c r="C160" t="n">
-        <v>272.95</v>
+        <v>5.61</v>
       </c>
       <c r="D160" t="n">
-        <v>1.32</v>
+        <v>2.19</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>SUNDARAM</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>39.8</v>
+        <v>1.37</v>
       </c>
       <c r="C161" t="n">
-        <v>40.3</v>
+        <v>1.4</v>
       </c>
       <c r="D161" t="n">
-        <v>1.26</v>
+        <v>2.19</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>TIL</t>
+          <t>OBCL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>176.33</v>
+        <v>53.73</v>
       </c>
       <c r="C162" t="n">
-        <v>178.48</v>
+        <v>54.9</v>
       </c>
       <c r="D162" t="n">
-        <v>1.22</v>
+        <v>2.18</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>REGAAL</t>
+          <t>KHANDSE</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>84.48</v>
+        <v>18.5</v>
       </c>
       <c r="C163" t="n">
-        <v>85.5</v>
+        <v>18.9</v>
       </c>
       <c r="D163" t="n">
-        <v>1.21</v>
+        <v>2.16</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>OILCOUNTUB</t>
+          <t>ROML</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>61.26</v>
+        <v>46</v>
       </c>
       <c r="C164" t="n">
-        <v>62</v>
+        <v>46.99</v>
       </c>
       <c r="D164" t="n">
-        <v>1.21</v>
+        <v>2.15</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>CHEMFAB</t>
+          <t>INTENTECH</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>420</v>
+        <v>90.66</v>
       </c>
       <c r="C165" t="n">
-        <v>425</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="D165" t="n">
-        <v>1.19</v>
+        <v>2.14</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>PONNIERODE</t>
+          <t>MAHEPC</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>339.6</v>
+        <v>106.22</v>
       </c>
       <c r="C166" t="n">
-        <v>343.65</v>
+        <v>108.48</v>
       </c>
       <c r="D166" t="n">
-        <v>1.19</v>
+        <v>2.13</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>DPEL</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>493.2</v>
+        <v>767.6</v>
       </c>
       <c r="C167" t="n">
-        <v>499</v>
+        <v>783.95</v>
       </c>
       <c r="D167" t="n">
-        <v>1.18</v>
+        <v>2.13</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>SURAJEST</t>
+          <t>FAZE3Q</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>186.69</v>
+        <v>545.3</v>
       </c>
       <c r="C168" t="n">
-        <v>188.9</v>
+        <v>556.9</v>
       </c>
       <c r="D168" t="n">
-        <v>1.18</v>
+        <v>2.13</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>FINOPB</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>29.57</v>
+        <v>127.73</v>
       </c>
       <c r="C169" t="n">
-        <v>29.92</v>
+        <v>130.44</v>
       </c>
       <c r="D169" t="n">
-        <v>1.18</v>
+        <v>2.12</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>VHL</t>
+          <t>DENTA</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>3386.5</v>
+        <v>243.75</v>
       </c>
       <c r="C170" t="n">
-        <v>3425</v>
+        <v>248.9</v>
       </c>
       <c r="D170" t="n">
-        <v>1.14</v>
+        <v>2.11</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>ORIENTCER</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>38.37</v>
+        <v>32.31</v>
       </c>
       <c r="C171" t="n">
-        <v>38.8</v>
+        <v>32.99</v>
       </c>
       <c r="D171" t="n">
-        <v>1.12</v>
+        <v>2.1</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>LOKESHMACH</t>
+          <t>FOCUS</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>250.2</v>
+        <v>92.52</v>
       </c>
       <c r="C172" t="n">
-        <v>253</v>
+        <v>94.45</v>
       </c>
       <c r="D172" t="n">
-        <v>1.12</v>
+        <v>2.09</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>ANTELOPUS</t>
+          <t>SAHYADRI</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>899.35</v>
+        <v>269.3</v>
       </c>
       <c r="C173" t="n">
-        <v>909.4</v>
+        <v>274.9</v>
       </c>
       <c r="D173" t="n">
-        <v>1.12</v>
+        <v>2.08</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>OSWALAGRO</t>
+          <t>HDIL</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>42.52</v>
+        <v>1.92</v>
       </c>
       <c r="C174" t="n">
-        <v>42.98</v>
+        <v>1.96</v>
       </c>
       <c r="D174" t="n">
-        <v>1.08</v>
+        <v>2.08</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>GENUSPAPER</t>
+          <t>CEINSYS</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>12.32</v>
+        <v>922.8</v>
       </c>
       <c r="C175" t="n">
-        <v>12.45</v>
+        <v>942</v>
       </c>
       <c r="D175" t="n">
-        <v>1.06</v>
+        <v>2.08</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>3IINFOLTD</t>
+          <t>ASMS</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>17.07</v>
+        <v>7.24</v>
       </c>
       <c r="C176" t="n">
-        <v>17.25</v>
+        <v>7.39</v>
       </c>
       <c r="D176" t="n">
-        <v>1.05</v>
+        <v>2.07</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>DHAMPURSUG</t>
+          <t>KOVAI</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>142.51</v>
+        <v>5517.5</v>
       </c>
       <c r="C177" t="n">
-        <v>143.99</v>
+        <v>5631</v>
       </c>
       <c r="D177" t="n">
-        <v>1.04</v>
+        <v>2.06</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>RCOM</t>
+          <t>VADILALIND</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>0.97</v>
+        <v>5632.9</v>
       </c>
       <c r="C178" t="n">
-        <v>0.98</v>
+        <v>5749</v>
       </c>
       <c r="D178" t="n">
-        <v>1.03</v>
+        <v>2.06</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>QLINE</t>
+          <t>SUYOG</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>494.85</v>
+        <v>695.65</v>
       </c>
       <c r="C179" t="n">
-        <v>499.9</v>
+        <v>709.95</v>
       </c>
       <c r="D179" t="n">
-        <v>1.02</v>
+        <v>2.06</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>4.93</v>
+        <v>22.92</v>
       </c>
       <c r="C180" t="n">
-        <v>4.98</v>
+        <v>23.39</v>
       </c>
       <c r="D180" t="n">
-        <v>1.01</v>
+        <v>2.05</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>RCOM</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>38.91</v>
+        <v>0.98</v>
       </c>
       <c r="C181" t="n">
-        <v>39.3</v>
+        <v>1</v>
       </c>
       <c r="D181" t="n">
-        <v>1</v>
+        <v>2.04</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>NECLIFE</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>11.98</v>
+        <v>1.96</v>
       </c>
       <c r="C182" t="n">
-        <v>12.1</v>
+        <v>2</v>
       </c>
       <c r="D182" t="n">
-        <v>1</v>
+        <v>2.04</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>IFGLEXPOR</t>
+          <t>MITTAL</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>194.77</v>
+        <v>0.98</v>
       </c>
       <c r="C183" t="n">
-        <v>196.7</v>
+        <v>1</v>
       </c>
       <c r="D183" t="n">
-        <v>0.99</v>
+        <v>2.04</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>KSHINTL</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>5.08</v>
+        <v>749.8</v>
       </c>
       <c r="C184" t="n">
-        <v>5.13</v>
+        <v>765</v>
       </c>
       <c r="D184" t="n">
-        <v>0.98</v>
+        <v>2.03</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>OAL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>182.55</v>
+        <v>314.65</v>
       </c>
       <c r="C185" t="n">
-        <v>184.34</v>
+        <v>321</v>
       </c>
       <c r="D185" t="n">
-        <v>0.98</v>
+        <v>2.02</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>AFSL</t>
+          <t>BPL</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>201.03</v>
+        <v>51.47</v>
       </c>
       <c r="C186" t="n">
-        <v>202.96</v>
+        <v>52.5</v>
       </c>
       <c r="D186" t="n">
-        <v>0.96</v>
+        <v>2</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>ELECTHERM</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>970.6</v>
+        <v>416.65</v>
       </c>
       <c r="C187" t="n">
-        <v>979.3</v>
+        <v>425</v>
       </c>
       <c r="D187" t="n">
-        <v>0.9</v>
+        <v>2</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>CEMPRO</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>13.97</v>
+        <v>1094.4</v>
       </c>
       <c r="C188" t="n">
-        <v>14.09</v>
+        <v>1116.3</v>
       </c>
       <c r="D188" t="n">
-        <v>0.86</v>
+        <v>2</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ANANTAM</t>
+          <t>BCLIND</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>104.5</v>
+        <v>37.02</v>
       </c>
       <c r="C189" t="n">
-        <v>105.4</v>
+        <v>37.76</v>
       </c>
       <c r="D189" t="n">
-        <v>0.86</v>
+        <v>2</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>DWARKESH</t>
+          <t>ENIL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>44.8</v>
+        <v>115.68</v>
       </c>
       <c r="C190" t="n">
-        <v>45.18</v>
+        <v>117.99</v>
       </c>
       <c r="D190" t="n">
-        <v>0.85</v>
+        <v>2</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>HINDCOMPOS</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>414.5</v>
+        <v>6.07</v>
       </c>
       <c r="C191" t="n">
-        <v>418</v>
+        <v>6.19</v>
       </c>
       <c r="D191" t="n">
-        <v>0.84</v>
+        <v>1.98</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>WANBURY</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>262.3</v>
+        <v>5.05</v>
       </c>
       <c r="C192" t="n">
-        <v>264.5</v>
+        <v>5.15</v>
       </c>
       <c r="D192" t="n">
-        <v>0.84</v>
+        <v>1.98</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>LYKALABS</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>356.95</v>
+        <v>63.69</v>
       </c>
       <c r="C193" t="n">
-        <v>359.9</v>
+        <v>64.95</v>
       </c>
       <c r="D193" t="n">
-        <v>0.83</v>
+        <v>1.98</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>YUKEN</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>684.4</v>
+        <v>3.53</v>
       </c>
       <c r="C194" t="n">
-        <v>690</v>
+        <v>3.6</v>
       </c>
       <c r="D194" t="n">
-        <v>0.82</v>
+        <v>1.98</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>PURPLEUTED</t>
+          <t>AJANTPHARM</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>395.85</v>
+        <v>2968.8</v>
       </c>
       <c r="C195" t="n">
-        <v>399</v>
+        <v>3027.3</v>
       </c>
       <c r="D195" t="n">
-        <v>0.8</v>
+        <v>1.97</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>MENONBE</t>
+          <t>MSTCLTD</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>138.71</v>
+        <v>490.15</v>
       </c>
       <c r="C196" t="n">
-        <v>139.75</v>
+        <v>499.8</v>
       </c>
       <c r="D196" t="n">
-        <v>0.75</v>
+        <v>1.97</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>RPPINFRA</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>1.35</v>
+        <v>59.33</v>
       </c>
       <c r="C197" t="n">
-        <v>1.36</v>
+        <v>60.5</v>
       </c>
       <c r="D197" t="n">
-        <v>0.74</v>
+        <v>1.97</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>SADBHAV</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>9.57</v>
+        <v>1469.2</v>
       </c>
       <c r="C198" t="n">
-        <v>9.640000000000001</v>
+        <v>1497.9</v>
       </c>
       <c r="D198" t="n">
-        <v>0.73</v>
+        <v>1.95</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>PENINLAND</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>15.48</v>
+        <v>139.01</v>
       </c>
       <c r="C199" t="n">
-        <v>15.59</v>
+        <v>141.7</v>
       </c>
       <c r="D199" t="n">
-        <v>0.71</v>
+        <v>1.94</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MUKANDLTD</t>
+          <t>NECCLTD</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>138.96</v>
+        <v>14.96</v>
       </c>
       <c r="C200" t="n">
-        <v>139.95</v>
+        <v>15.25</v>
       </c>
       <c r="D200" t="n">
-        <v>0.71</v>
+        <v>1.94</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>BALAXI</t>
+          <t>TIPSMUSIC</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>24.28</v>
+        <v>656.3</v>
       </c>
       <c r="C201" t="n">
-        <v>24.45</v>
+        <v>669</v>
       </c>
       <c r="D201" t="n">
-        <v>0.7</v>
+        <v>1.94</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-10 07:55 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15.52</v>
+        <v>18.62</v>
       </c>
       <c r="C2" t="n">
-        <v>18.6</v>
+        <v>21.9</v>
       </c>
       <c r="D2" t="n">
-        <v>19.85</v>
+        <v>17.62</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>PIONRINV</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48.59</v>
+        <v>99.14</v>
       </c>
       <c r="C3" t="n">
-        <v>52.59</v>
+        <v>114.98</v>
       </c>
       <c r="D3" t="n">
-        <v>8.23</v>
+        <v>15.98</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BAFNAPH</t>
+          <t>RSDFIN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>193.97</v>
+        <v>78</v>
       </c>
       <c r="C4" t="n">
-        <v>209.7</v>
+        <v>85.98999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>8.109999999999999</v>
+        <v>10.24</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JNKINDIA</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>418.35</v>
+        <v>20.91</v>
       </c>
       <c r="C5" t="n">
-        <v>450.15</v>
+        <v>23</v>
       </c>
       <c r="D5" t="n">
-        <v>7.6</v>
+        <v>10</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GRAVISSHO</t>
+          <t>CLEANMAX</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28.5</v>
+        <v>1232.4</v>
       </c>
       <c r="C6" t="n">
-        <v>30.65</v>
+        <v>1350</v>
       </c>
       <c r="D6" t="n">
-        <v>7.54</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>SUPREMEINF</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4.77</v>
+        <v>76.87</v>
       </c>
       <c r="C7" t="n">
-        <v>5.1</v>
+        <v>83.29000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>6.92</v>
+        <v>8.35</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.9</v>
+        <v>4.9</v>
       </c>
       <c r="C8" t="n">
-        <v>2.02</v>
+        <v>5.28</v>
       </c>
       <c r="D8" t="n">
-        <v>6.32</v>
+        <v>7.76</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>19.66</v>
+        <v>31.61</v>
       </c>
       <c r="C9" t="n">
-        <v>20.88</v>
+        <v>33.99</v>
       </c>
       <c r="D9" t="n">
-        <v>6.21</v>
+        <v>7.53</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VIPULLTD</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10.1</v>
+        <v>0.14</v>
       </c>
       <c r="C10" t="n">
-        <v>10.7</v>
+        <v>0.15</v>
       </c>
       <c r="D10" t="n">
-        <v>5.94</v>
+        <v>7.14</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>KANANIIND</t>
+          <t>COOLCAPS</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.56</v>
+        <v>25.2</v>
       </c>
       <c r="C11" t="n">
-        <v>1.65</v>
+        <v>26.9</v>
       </c>
       <c r="D11" t="n">
-        <v>5.77</v>
+        <v>6.75</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>INNOVANA</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11.97</v>
+        <v>300.55</v>
       </c>
       <c r="C12" t="n">
-        <v>12.64</v>
+        <v>319.9</v>
       </c>
       <c r="D12" t="n">
-        <v>5.6</v>
+        <v>6.44</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>STARTECK</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>269.8</v>
+        <v>23.36</v>
       </c>
       <c r="C13" t="n">
-        <v>283.95</v>
+        <v>24.85</v>
       </c>
       <c r="D13" t="n">
-        <v>5.24</v>
+        <v>6.38</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SILKFLEX</t>
+          <t>AFCONS</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>190</v>
+        <v>315.5</v>
       </c>
       <c r="C14" t="n">
-        <v>199.5</v>
+        <v>335</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>6.18</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SICALLOG</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>75.84999999999999</v>
+        <v>4.72</v>
       </c>
       <c r="C15" t="n">
-        <v>79.64</v>
+        <v>4.98</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>5.51</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TANKUP</t>
+          <t>LYKALABS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1001.8</v>
+        <v>70.05</v>
       </c>
       <c r="C16" t="n">
-        <v>1051.85</v>
+        <v>73.8</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>5.35</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>24.35</v>
       </c>
       <c r="C17" t="n">
-        <v>2.1</v>
+        <v>25.6</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>5.13</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,14 +813,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IZMO</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>963.25</v>
+        <v>0.2</v>
       </c>
       <c r="C18" t="n">
-        <v>1011.4</v>
+        <v>0.21</v>
       </c>
       <c r="D18" t="n">
         <v>5</v>
@@ -835,14 +835,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>SILKFLEX</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>14.24</v>
+        <v>199.5</v>
       </c>
       <c r="C19" t="n">
-        <v>14.95</v>
+        <v>209.45</v>
       </c>
       <c r="D19" t="n">
         <v>4.99</v>
@@ -857,14 +857,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>BOHRAIND</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>17.43</v>
+        <v>17.82</v>
       </c>
       <c r="C20" t="n">
-        <v>18.3</v>
+        <v>18.71</v>
       </c>
       <c r="D20" t="n">
         <v>4.99</v>
@@ -883,10 +883,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>36.1</v>
+        <v>37.9</v>
       </c>
       <c r="C21" t="n">
-        <v>37.9</v>
+        <v>39.79</v>
       </c>
       <c r="D21" t="n">
         <v>4.99</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6.24</v>
+        <v>437.45</v>
       </c>
       <c r="C22" t="n">
-        <v>6.55</v>
+        <v>459.3</v>
       </c>
       <c r="D22" t="n">
-        <v>4.97</v>
+        <v>4.99</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MCON</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>52.4</v>
+        <v>5.52</v>
       </c>
       <c r="C23" t="n">
-        <v>55</v>
+        <v>5.79</v>
       </c>
       <c r="D23" t="n">
-        <v>4.96</v>
+        <v>4.89</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SHIVAMILLS</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>63.95</v>
+        <v>3.49</v>
       </c>
       <c r="C24" t="n">
-        <v>67.12</v>
+        <v>3.66</v>
       </c>
       <c r="D24" t="n">
-        <v>4.96</v>
+        <v>4.87</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IMPEXFERRO</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2.42</v>
+        <v>14.5</v>
       </c>
       <c r="C25" t="n">
-        <v>2.54</v>
+        <v>15.2</v>
       </c>
       <c r="D25" t="n">
-        <v>4.96</v>
+        <v>4.83</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>KSR</t>
+          <t>VIVIDEL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>32.17</v>
+        <v>1000.1</v>
       </c>
       <c r="C26" t="n">
-        <v>33.76</v>
+        <v>1048</v>
       </c>
       <c r="D26" t="n">
-        <v>4.94</v>
+        <v>4.79</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>SSFL</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.8100000000000001</v>
+        <v>212.6</v>
       </c>
       <c r="C27" t="n">
-        <v>0.85</v>
+        <v>222.7</v>
       </c>
       <c r="D27" t="n">
-        <v>4.94</v>
+        <v>4.75</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4.28</v>
+        <v>6.54</v>
       </c>
       <c r="C28" t="n">
-        <v>4.49</v>
+        <v>6.85</v>
       </c>
       <c r="D28" t="n">
-        <v>4.91</v>
+        <v>4.74</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CHETANA</t>
+          <t>CYBERMEDIA</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>46.85</v>
+        <v>16.42</v>
       </c>
       <c r="C29" t="n">
-        <v>49.15</v>
+        <v>17.19</v>
       </c>
       <c r="D29" t="n">
-        <v>4.91</v>
+        <v>4.69</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BETA</t>
+          <t>CONSOFINVT</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1430.1</v>
+        <v>226.44</v>
       </c>
       <c r="C30" t="n">
-        <v>1500</v>
+        <v>237</v>
       </c>
       <c r="D30" t="n">
-        <v>4.89</v>
+        <v>4.66</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DIVYADHAN</t>
+          <t>FELDVR</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>33.75</v>
+        <v>2.58</v>
       </c>
       <c r="C31" t="n">
-        <v>35.4</v>
+        <v>2.7</v>
       </c>
       <c r="D31" t="n">
-        <v>4.89</v>
+        <v>4.65</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SYNOPTICS</t>
+          <t>SUPREMEENG</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>58.35</v>
+        <v>1.08</v>
       </c>
       <c r="C32" t="n">
-        <v>61.2</v>
+        <v>1.13</v>
       </c>
       <c r="D32" t="n">
-        <v>4.88</v>
+        <v>4.63</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SYSTMTXC</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>65.52</v>
+        <v>28.44</v>
       </c>
       <c r="C33" t="n">
-        <v>68.7</v>
+        <v>29.75</v>
       </c>
       <c r="D33" t="n">
-        <v>4.85</v>
+        <v>4.61</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>SIMBHALS</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>40.65</v>
+        <v>7.03</v>
       </c>
       <c r="C34" t="n">
-        <v>42.6</v>
+        <v>7.35</v>
       </c>
       <c r="D34" t="n">
-        <v>4.8</v>
+        <v>4.55</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SUPREMEENG</t>
+          <t>QPOWER</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1.05</v>
+        <v>1133.7</v>
       </c>
       <c r="C35" t="n">
-        <v>1.1</v>
+        <v>1185</v>
       </c>
       <c r="D35" t="n">
-        <v>4.76</v>
+        <v>4.53</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LIKHITHA</t>
+          <t>GTPL</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>227.2</v>
+        <v>63.44</v>
       </c>
       <c r="C36" t="n">
-        <v>238</v>
+        <v>66.3</v>
       </c>
       <c r="D36" t="n">
-        <v>4.75</v>
+        <v>4.51</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PANAMAPET</t>
+          <t>RSWM</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>334.75</v>
+        <v>213.4</v>
       </c>
       <c r="C37" t="n">
-        <v>350.55</v>
+        <v>222.99</v>
       </c>
       <c r="D37" t="n">
-        <v>4.72</v>
+        <v>4.49</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TREJHARA</t>
+          <t>MANAKSTEEL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>137.42</v>
+        <v>66.81</v>
       </c>
       <c r="C38" t="n">
-        <v>143.9</v>
+        <v>69.8</v>
       </c>
       <c r="D38" t="n">
-        <v>4.72</v>
+        <v>4.48</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>A2ZINFRA</t>
+          <t>CEREBRAINT</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>14.21</v>
+        <v>3.59</v>
       </c>
       <c r="C39" t="n">
-        <v>14.88</v>
+        <v>3.75</v>
       </c>
       <c r="D39" t="n">
-        <v>4.71</v>
+        <v>4.46</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SVLL</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>849.15</v>
+        <v>4.49</v>
       </c>
       <c r="C40" t="n">
-        <v>888.9</v>
+        <v>4.69</v>
       </c>
       <c r="D40" t="n">
-        <v>4.68</v>
+        <v>4.45</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AURIONPRO</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>743.1</v>
+        <v>91.44</v>
       </c>
       <c r="C41" t="n">
-        <v>777</v>
+        <v>95.48999999999999</v>
       </c>
       <c r="D41" t="n">
-        <v>4.56</v>
+        <v>4.43</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>UMESLTD</t>
+          <t>SYSTMTXC</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>5.53</v>
+        <v>65.11</v>
       </c>
       <c r="C42" t="n">
-        <v>5.78</v>
+        <v>67.95</v>
       </c>
       <c r="D42" t="n">
-        <v>4.52</v>
+        <v>4.36</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FMNL</t>
+          <t>BONLON</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>10.22</v>
+        <v>42.16</v>
       </c>
       <c r="C43" t="n">
-        <v>10.68</v>
+        <v>43.99</v>
       </c>
       <c r="D43" t="n">
-        <v>4.5</v>
+        <v>4.34</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>SICALLOG</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>40.92</v>
+        <v>79.56999999999999</v>
       </c>
       <c r="C44" t="n">
-        <v>42.76</v>
+        <v>82.98</v>
       </c>
       <c r="D44" t="n">
-        <v>4.5</v>
+        <v>4.29</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAPTRUST</t>
+          <t>MAXVOLT</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>13.37</v>
+        <v>383.6</v>
       </c>
       <c r="C45" t="n">
-        <v>13.97</v>
+        <v>400</v>
       </c>
       <c r="D45" t="n">
-        <v>4.49</v>
+        <v>4.28</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MASTERTR</t>
+          <t>MITCON</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>92.02</v>
+        <v>82.38</v>
       </c>
       <c r="C46" t="n">
-        <v>96.14</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="D46" t="n">
-        <v>4.48</v>
+        <v>4.21</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>16.3</v>
+        <v>68.23</v>
       </c>
       <c r="C47" t="n">
-        <v>17</v>
+        <v>71</v>
       </c>
       <c r="D47" t="n">
-        <v>4.29</v>
+        <v>4.06</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>UHTL</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>86.25</v>
+        <v>1.54</v>
       </c>
       <c r="C48" t="n">
-        <v>89.95</v>
+        <v>1.6</v>
       </c>
       <c r="D48" t="n">
-        <v>4.29</v>
+        <v>3.9</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DRCSYSTEMS</t>
+          <t>TEAMTECH</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>14.27</v>
+        <v>78.95</v>
       </c>
       <c r="C49" t="n">
-        <v>14.88</v>
+        <v>81.95</v>
       </c>
       <c r="D49" t="n">
-        <v>4.27</v>
+        <v>3.8</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PASUPTAC</t>
+          <t>MEESHO</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>74.34</v>
+        <v>166.73</v>
       </c>
       <c r="C50" t="n">
-        <v>77.5</v>
+        <v>173</v>
       </c>
       <c r="D50" t="n">
-        <v>4.25</v>
+        <v>3.76</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>COUNCODOS</t>
+          <t>ARCIIL</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>4.8</v>
+        <v>42.9</v>
       </c>
       <c r="C51" t="n">
-        <v>5</v>
+        <v>44.5</v>
       </c>
       <c r="D51" t="n">
-        <v>4.17</v>
+        <v>3.73</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PANACEABIO</t>
+          <t>HGS</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>552.9</v>
+        <v>400.25</v>
       </c>
       <c r="C52" t="n">
-        <v>575.85</v>
+        <v>415</v>
       </c>
       <c r="D52" t="n">
-        <v>4.15</v>
+        <v>3.69</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>HPAL</t>
+          <t>ENERGYDEV</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>35.53</v>
+        <v>16.69</v>
       </c>
       <c r="C53" t="n">
-        <v>36.98</v>
+        <v>17.3</v>
       </c>
       <c r="D53" t="n">
-        <v>4.08</v>
+        <v>3.65</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SUPREME</t>
+          <t>TECILCHEM</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>44.98</v>
+        <v>11</v>
       </c>
       <c r="C54" t="n">
-        <v>46.79</v>
+        <v>11.4</v>
       </c>
       <c r="D54" t="n">
-        <v>4.02</v>
+        <v>3.64</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PASHUPATI</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>89.22</v>
+        <v>1.93</v>
       </c>
       <c r="C55" t="n">
-        <v>92.8</v>
+        <v>2</v>
       </c>
       <c r="D55" t="n">
-        <v>4.01</v>
+        <v>3.63</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>RSSOFTWARE</t>
+          <t>KHANDSE</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>31.47</v>
+        <v>18.23</v>
       </c>
       <c r="C56" t="n">
-        <v>32.7</v>
+        <v>18.89</v>
       </c>
       <c r="D56" t="n">
-        <v>3.91</v>
+        <v>3.62</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>NEXTMEDIA</t>
+          <t>MERCANTILE</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>3.84</v>
+        <v>25.11</v>
       </c>
       <c r="C57" t="n">
-        <v>3.99</v>
+        <v>26</v>
       </c>
       <c r="D57" t="n">
-        <v>3.91</v>
+        <v>3.54</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>INSPIRISYS</t>
+          <t>WINDMACHIN</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>118.44</v>
+        <v>313.7</v>
       </c>
       <c r="C58" t="n">
-        <v>123</v>
+        <v>324.75</v>
       </c>
       <c r="D58" t="n">
-        <v>3.85</v>
+        <v>3.52</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>TRF</t>
+          <t>DSSL</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>218.8</v>
+        <v>1309.3</v>
       </c>
       <c r="C59" t="n">
-        <v>226.9</v>
+        <v>1355.2</v>
       </c>
       <c r="D59" t="n">
-        <v>3.7</v>
+        <v>3.51</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TVTODAY</t>
+          <t>EUROBOND</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>110.1</v>
+        <v>176.46</v>
       </c>
       <c r="C60" t="n">
-        <v>114.08</v>
+        <v>182.6</v>
       </c>
       <c r="D60" t="n">
-        <v>3.61</v>
+        <v>3.48</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>37.87</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="C61" t="n">
-        <v>39.2</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D61" t="n">
-        <v>3.51</v>
+        <v>3.45</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DHUNINV</t>
+          <t>BANARBEADS</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>771.05</v>
+        <v>99.7</v>
       </c>
       <c r="C62" t="n">
-        <v>798</v>
+        <v>103.1</v>
       </c>
       <c r="D62" t="n">
-        <v>3.5</v>
+        <v>3.41</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BIL</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>698.05</v>
+        <v>34.25</v>
       </c>
       <c r="C63" t="n">
-        <v>722.5</v>
+        <v>35.4</v>
       </c>
       <c r="D63" t="n">
-        <v>3.5</v>
+        <v>3.36</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>HECPROJECT</t>
+          <t>DAMODARIND</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>121.55</v>
+        <v>30.15</v>
       </c>
       <c r="C64" t="n">
-        <v>125.79</v>
+        <v>31.15</v>
       </c>
       <c r="D64" t="n">
-        <v>3.49</v>
+        <v>3.32</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>GRCL</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>41.46</v>
+        <v>540</v>
       </c>
       <c r="C65" t="n">
-        <v>42.9</v>
+        <v>557.9</v>
       </c>
       <c r="D65" t="n">
-        <v>3.47</v>
+        <v>3.31</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>NARMADA</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2.32</v>
+        <v>37.77</v>
       </c>
       <c r="C66" t="n">
-        <v>2.4</v>
+        <v>39</v>
       </c>
       <c r="D66" t="n">
-        <v>3.45</v>
+        <v>3.26</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>KARMAENG</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1.16</v>
+        <v>41.98</v>
       </c>
       <c r="C67" t="n">
-        <v>1.2</v>
+        <v>43.35</v>
       </c>
       <c r="D67" t="n">
-        <v>3.45</v>
+        <v>3.26</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>MERCANTILE</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>26.39</v>
+        <v>96.3</v>
       </c>
       <c r="C68" t="n">
-        <v>27.3</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="D68" t="n">
-        <v>3.45</v>
+        <v>3.22</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SMARTLINK</t>
+          <t>SUPREME</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>164.35</v>
+        <v>44.46</v>
       </c>
       <c r="C69" t="n">
-        <v>170</v>
+        <v>45.88</v>
       </c>
       <c r="D69" t="n">
-        <v>3.44</v>
+        <v>3.19</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>KEYFINSERV</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>24.07</v>
+        <v>255.85</v>
       </c>
       <c r="C70" t="n">
-        <v>24.89</v>
+        <v>263.95</v>
       </c>
       <c r="D70" t="n">
-        <v>3.41</v>
+        <v>3.17</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>VILAS</t>
+          <t>RILINFRA</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>355.8</v>
+        <v>34.9</v>
       </c>
       <c r="C71" t="n">
-        <v>367.95</v>
+        <v>36</v>
       </c>
       <c r="D71" t="n">
-        <v>3.41</v>
+        <v>3.15</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>IL&amp;FSENGG</t>
+          <t>NDL</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>29.01</v>
+        <v>2.56</v>
       </c>
       <c r="C72" t="n">
-        <v>30</v>
+        <v>2.64</v>
       </c>
       <c r="D72" t="n">
-        <v>3.41</v>
+        <v>3.13</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>HEADSUP</t>
+          <t>HITECHCORP</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>7.06</v>
+        <v>309.32</v>
       </c>
       <c r="C73" t="n">
-        <v>7.3</v>
+        <v>319</v>
       </c>
       <c r="D73" t="n">
-        <v>3.4</v>
+        <v>3.13</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BANSWRAS</t>
+          <t>RAJOOENG</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>117.98</v>
+        <v>53.21</v>
       </c>
       <c r="C74" t="n">
-        <v>121.99</v>
+        <v>54.87</v>
       </c>
       <c r="D74" t="n">
-        <v>3.4</v>
+        <v>3.12</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>COOLCAPS</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>23.6</v>
+        <v>13.17</v>
       </c>
       <c r="C75" t="n">
-        <v>24.4</v>
+        <v>13.58</v>
       </c>
       <c r="D75" t="n">
-        <v>3.39</v>
+        <v>3.11</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>NIBL</t>
+          <t>KAPSTON</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>30.47</v>
+        <v>337.5</v>
       </c>
       <c r="C76" t="n">
-        <v>31.5</v>
+        <v>347.9</v>
       </c>
       <c r="D76" t="n">
-        <v>3.38</v>
+        <v>3.08</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ENERGYDEV</t>
+          <t>ATALREAL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>16.64</v>
+        <v>24.72</v>
       </c>
       <c r="C77" t="n">
-        <v>17.2</v>
+        <v>25.47</v>
       </c>
       <c r="D77" t="n">
-        <v>3.37</v>
+        <v>3.03</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>NIPPOBATRY</t>
+          <t>CEMPRO</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>354.1</v>
+        <v>1203.8</v>
       </c>
       <c r="C78" t="n">
-        <v>366</v>
+        <v>1240</v>
       </c>
       <c r="D78" t="n">
-        <v>3.36</v>
+        <v>3.01</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ANLON</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>696.85</v>
+        <v>22.76</v>
       </c>
       <c r="C79" t="n">
-        <v>720</v>
+        <v>23.44</v>
       </c>
       <c r="D79" t="n">
-        <v>3.32</v>
+        <v>2.99</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>AROGRANITE</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>45.49</v>
+        <v>24.76</v>
       </c>
       <c r="C80" t="n">
-        <v>47</v>
+        <v>25.5</v>
       </c>
       <c r="D80" t="n">
-        <v>3.32</v>
+        <v>2.99</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SONAMLTD</t>
+          <t>MITTAL</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>54.69</v>
+        <v>1.01</v>
       </c>
       <c r="C81" t="n">
-        <v>56.5</v>
+        <v>1.04</v>
       </c>
       <c r="D81" t="n">
-        <v>3.31</v>
+        <v>2.97</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BRNL</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>18.78</v>
+        <v>88.67</v>
       </c>
       <c r="C82" t="n">
-        <v>19.4</v>
+        <v>91.3</v>
       </c>
       <c r="D82" t="n">
-        <v>3.3</v>
+        <v>2.97</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>KHADIM</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>100.11</v>
+        <v>48.08</v>
       </c>
       <c r="C83" t="n">
-        <v>103.4</v>
+        <v>49.5</v>
       </c>
       <c r="D83" t="n">
-        <v>3.29</v>
+        <v>2.95</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>LIKHITHA</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>7.64</v>
+        <v>227.11</v>
       </c>
       <c r="C84" t="n">
-        <v>7.89</v>
+        <v>233.8</v>
       </c>
       <c r="D84" t="n">
-        <v>3.27</v>
+        <v>2.95</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>LASA</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>7.66</v>
+        <v>7.46</v>
       </c>
       <c r="C85" t="n">
-        <v>7.91</v>
+        <v>7.68</v>
       </c>
       <c r="D85" t="n">
-        <v>3.26</v>
+        <v>2.95</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>HMVL</t>
+          <t>REDTAPE</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>84.65000000000001</v>
+        <v>133.81</v>
       </c>
       <c r="C86" t="n">
-        <v>87.40000000000001</v>
+        <v>137.7</v>
       </c>
       <c r="D86" t="n">
-        <v>3.25</v>
+        <v>2.91</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>RELIABLE</t>
+          <t>MENNPIS</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>145.23</v>
+        <v>54.25</v>
       </c>
       <c r="C87" t="n">
-        <v>149.95</v>
+        <v>55.83</v>
       </c>
       <c r="D87" t="n">
-        <v>3.25</v>
+        <v>2.91</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ALANKIT</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>8.210000000000001</v>
+        <v>364.45</v>
       </c>
       <c r="C88" t="n">
-        <v>8.470000000000001</v>
+        <v>374.95</v>
       </c>
       <c r="D88" t="n">
-        <v>3.17</v>
+        <v>2.88</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>BORORENEW</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>513.75</v>
+        <v>2.43</v>
       </c>
       <c r="C89" t="n">
-        <v>530</v>
+        <v>2.5</v>
       </c>
       <c r="D89" t="n">
-        <v>3.16</v>
+        <v>2.88</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SHEMAROO</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>109.35</v>
+        <v>6.37</v>
       </c>
       <c r="C90" t="n">
-        <v>112.79</v>
+        <v>6.55</v>
       </c>
       <c r="D90" t="n">
-        <v>3.15</v>
+        <v>2.83</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>OLAELEC</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>44.43</v>
+        <v>31.21</v>
       </c>
       <c r="C91" t="n">
-        <v>45.83</v>
+        <v>32.09</v>
       </c>
       <c r="D91" t="n">
-        <v>3.15</v>
+        <v>2.82</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MFML</t>
+          <t>BELLACASA</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>23.84</v>
+        <v>232.97</v>
       </c>
       <c r="C92" t="n">
-        <v>24.59</v>
+        <v>239.5</v>
       </c>
       <c r="D92" t="n">
-        <v>3.15</v>
+        <v>2.8</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>IGCL</t>
+          <t>KHADIM</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>55.04</v>
+        <v>100</v>
       </c>
       <c r="C93" t="n">
-        <v>56.77</v>
+        <v>102.8</v>
       </c>
       <c r="D93" t="n">
-        <v>3.14</v>
+        <v>2.8</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>TREL</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>25.41</v>
+        <v>0.36</v>
       </c>
       <c r="C94" t="n">
-        <v>26.2</v>
+        <v>0.37</v>
       </c>
       <c r="D94" t="n">
-        <v>3.11</v>
+        <v>2.78</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ARIES</t>
+          <t>AYMSYNTEX</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>322.65</v>
+        <v>218.49</v>
       </c>
       <c r="C95" t="n">
-        <v>332.65</v>
+        <v>224.5</v>
       </c>
       <c r="D95" t="n">
-        <v>3.1</v>
+        <v>2.75</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>HALDYNGL</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>114.46</v>
+        <v>5.84</v>
       </c>
       <c r="C96" t="n">
-        <v>118</v>
+        <v>6</v>
       </c>
       <c r="D96" t="n">
-        <v>3.09</v>
+        <v>2.74</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SANATHAN</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>414.55</v>
+        <v>4.03</v>
       </c>
       <c r="C97" t="n">
-        <v>427.3</v>
+        <v>4.14</v>
       </c>
       <c r="D97" t="n">
-        <v>3.08</v>
+        <v>2.73</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>AYMSYNTEX</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>218.05</v>
+        <v>384.3</v>
       </c>
       <c r="C98" t="n">
-        <v>224.7</v>
+        <v>394.7</v>
       </c>
       <c r="D98" t="n">
-        <v>3.05</v>
+        <v>2.71</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>IWARE</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>5.57</v>
+        <v>330</v>
       </c>
       <c r="C99" t="n">
-        <v>5.74</v>
+        <v>338.95</v>
       </c>
       <c r="D99" t="n">
-        <v>3.05</v>
+        <v>2.71</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>NACLIND</t>
+          <t>ORIENTLTD</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>169.36</v>
+        <v>58.81</v>
       </c>
       <c r="C100" t="n">
-        <v>174.49</v>
+        <v>60.4</v>
       </c>
       <c r="D100" t="n">
-        <v>3.03</v>
+        <v>2.7</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PREMCO</t>
+          <t>MVGJL</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>364.8</v>
+        <v>150</v>
       </c>
       <c r="C101" t="n">
-        <v>375.8</v>
+        <v>154</v>
       </c>
       <c r="D101" t="n">
-        <v>3.02</v>
+        <v>2.67</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>DRONE</t>
+          <t>PAUSHAKLTD</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>39.8</v>
+        <v>466.7</v>
       </c>
       <c r="C102" t="n">
-        <v>41</v>
+        <v>479</v>
       </c>
       <c r="D102" t="n">
-        <v>3.02</v>
+        <v>2.64</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>HBESD</t>
+          <t>AURIGROW</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>75.7</v>
+        <v>0.38</v>
       </c>
       <c r="C103" t="n">
-        <v>77.98</v>
+        <v>0.39</v>
       </c>
       <c r="D103" t="n">
-        <v>3.01</v>
+        <v>2.63</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>KANANIIND</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>20.03</v>
+        <v>1.55</v>
       </c>
       <c r="C104" t="n">
-        <v>20.63</v>
+        <v>1.59</v>
       </c>
       <c r="D104" t="n">
-        <v>3</v>
+        <v>2.58</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ORTINGLOBE</t>
+          <t>AGROPHOS</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>19.92</v>
+        <v>30.23</v>
       </c>
       <c r="C105" t="n">
-        <v>20.51</v>
+        <v>31</v>
       </c>
       <c r="D105" t="n">
-        <v>2.96</v>
+        <v>2.55</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>AURIGROW</t>
+          <t>AMNPLST</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>0.35</v>
+        <v>197.68</v>
       </c>
       <c r="C106" t="n">
-        <v>0.36</v>
+        <v>202.7</v>
       </c>
       <c r="D106" t="n">
-        <v>2.86</v>
+        <v>2.54</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>AXITA</t>
+          <t>UFLEX</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>7.77</v>
+        <v>417.1</v>
       </c>
       <c r="C107" t="n">
-        <v>7.99</v>
+        <v>427.7</v>
       </c>
       <c r="D107" t="n">
-        <v>2.83</v>
+        <v>2.54</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MANAKSIA</t>
+          <t>WEALTH</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>58.06</v>
+        <v>940.2</v>
       </c>
       <c r="C108" t="n">
-        <v>59.7</v>
+        <v>964</v>
       </c>
       <c r="D108" t="n">
-        <v>2.82</v>
+        <v>2.53</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BESTAGRO</t>
+          <t>WAKEFIT</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>15.95</v>
+        <v>118.02</v>
       </c>
       <c r="C109" t="n">
-        <v>16.4</v>
+        <v>120.99</v>
       </c>
       <c r="D109" t="n">
-        <v>2.82</v>
+        <v>2.52</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>DAMODARIND</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>30.16</v>
+        <v>18.63</v>
       </c>
       <c r="C110" t="n">
-        <v>31</v>
+        <v>19.1</v>
       </c>
       <c r="D110" t="n">
-        <v>2.79</v>
+        <v>2.52</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CHEMFAB</t>
+          <t>PRAKASHSTL</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>407.35</v>
+        <v>4.39</v>
       </c>
       <c r="C111" t="n">
-        <v>418.7</v>
+        <v>4.5</v>
       </c>
       <c r="D111" t="n">
-        <v>2.79</v>
+        <v>2.51</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IDEA</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>14.4</v>
+        <v>170.7</v>
       </c>
       <c r="C112" t="n">
-        <v>14.8</v>
+        <v>174.99</v>
       </c>
       <c r="D112" t="n">
-        <v>2.78</v>
+        <v>2.51</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>BBTCL</t>
+          <t>AEGISVOPAK</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>221.83</v>
+        <v>191.67</v>
       </c>
       <c r="C113" t="n">
-        <v>228</v>
+        <v>196.48</v>
       </c>
       <c r="D113" t="n">
-        <v>2.78</v>
+        <v>2.51</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>IFGLEXPOR</t>
+          <t>DCMSRIND</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>190.6</v>
+        <v>40.45</v>
       </c>
       <c r="C114" t="n">
-        <v>195.87</v>
+        <v>41.44</v>
       </c>
       <c r="D114" t="n">
-        <v>2.76</v>
+        <v>2.45</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>FIBERWEB</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>24.03</v>
+        <v>28</v>
       </c>
       <c r="C115" t="n">
-        <v>24.69</v>
+        <v>28.68</v>
       </c>
       <c r="D115" t="n">
-        <v>2.75</v>
+        <v>2.43</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>CENTRUM</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>34.55</v>
+        <v>21.77</v>
       </c>
       <c r="C116" t="n">
-        <v>35.49</v>
+        <v>22.3</v>
       </c>
       <c r="D116" t="n">
-        <v>2.72</v>
+        <v>2.43</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>INDBANK</t>
+          <t>KAVDEFENCE</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>33.1</v>
+        <v>60.44</v>
       </c>
       <c r="C117" t="n">
-        <v>34</v>
+        <v>61.9</v>
       </c>
       <c r="D117" t="n">
-        <v>2.72</v>
+        <v>2.42</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>KOTIC</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>40.79</v>
+        <v>161.84</v>
       </c>
       <c r="C118" t="n">
-        <v>41.9</v>
+        <v>165.75</v>
       </c>
       <c r="D118" t="n">
-        <v>2.72</v>
+        <v>2.42</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CSLFINANCE</t>
+          <t>INVPRECQ</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>220.03</v>
+        <v>613.3</v>
       </c>
       <c r="C119" t="n">
-        <v>226</v>
+        <v>627.9</v>
       </c>
       <c r="D119" t="n">
-        <v>2.71</v>
+        <v>2.38</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>A2ZINFRA</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>0.37</v>
+        <v>14.56</v>
       </c>
       <c r="C120" t="n">
-        <v>0.38</v>
+        <v>14.9</v>
       </c>
       <c r="D120" t="n">
-        <v>2.7</v>
+        <v>2.34</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>KABRAEXTRU</t>
+          <t>SATIA</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>237.65</v>
+        <v>54.71</v>
       </c>
       <c r="C121" t="n">
-        <v>244</v>
+        <v>55.99</v>
       </c>
       <c r="D121" t="n">
-        <v>2.67</v>
+        <v>2.34</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>KAPSTON</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>329.7</v>
+        <v>178.82</v>
       </c>
       <c r="C122" t="n">
-        <v>338.5</v>
+        <v>183</v>
       </c>
       <c r="D122" t="n">
-        <v>2.67</v>
+        <v>2.34</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>27.18</v>
+        <v>0.43</v>
       </c>
       <c r="C123" t="n">
-        <v>27.9</v>
+        <v>0.44</v>
       </c>
       <c r="D123" t="n">
-        <v>2.65</v>
+        <v>2.33</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>WABAG</t>
+          <t>RMDRIP</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>1544.3</v>
+        <v>16.05</v>
       </c>
       <c r="C124" t="n">
-        <v>1585</v>
+        <v>16.42</v>
       </c>
       <c r="D124" t="n">
-        <v>2.64</v>
+        <v>2.31</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>VINYAS</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>1332.95</v>
+        <v>8.27</v>
       </c>
       <c r="C125" t="n">
-        <v>1368</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="D125" t="n">
-        <v>2.63</v>
+        <v>2.3</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>UNIHEALTH</t>
+          <t>NDLVENTURE</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>462.1</v>
+        <v>130.03</v>
       </c>
       <c r="C126" t="n">
-        <v>474</v>
+        <v>133</v>
       </c>
       <c r="D126" t="n">
-        <v>2.58</v>
+        <v>2.28</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>BELRISE</t>
+          <t>BIMETAL</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>215.72</v>
+        <v>641.25</v>
       </c>
       <c r="C127" t="n">
-        <v>221.28</v>
+        <v>655.9</v>
       </c>
       <c r="D127" t="n">
-        <v>2.58</v>
+        <v>2.28</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>INDIANCARD</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>223.36</v>
+        <v>7.53</v>
       </c>
       <c r="C128" t="n">
-        <v>229</v>
+        <v>7.7</v>
       </c>
       <c r="D128" t="n">
-        <v>2.53</v>
+        <v>2.26</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SUPERSPIN</t>
+          <t>3BBLACKBIO</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>4.78</v>
+        <v>1201.5</v>
       </c>
       <c r="C129" t="n">
-        <v>4.9</v>
+        <v>1228</v>
       </c>
       <c r="D129" t="n">
-        <v>2.51</v>
+        <v>2.21</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>AMBALALSA</t>
+          <t>ASMS</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>34.62</v>
+        <v>7.27</v>
       </c>
       <c r="C130" t="n">
-        <v>35.49</v>
+        <v>7.43</v>
       </c>
       <c r="D130" t="n">
-        <v>2.51</v>
+        <v>2.2</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>JAIPURKURT</t>
+          <t>AIROLAM</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>28.83</v>
+        <v>85.13</v>
       </c>
       <c r="C131" t="n">
-        <v>29.55</v>
+        <v>87</v>
       </c>
       <c r="D131" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SAGARDEEP</t>
+          <t>DIFFNKG</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>24.98</v>
+        <v>330.8</v>
       </c>
       <c r="C132" t="n">
-        <v>25.6</v>
+        <v>338</v>
       </c>
       <c r="D132" t="n">
-        <v>2.48</v>
+        <v>2.18</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SECURKLOUD</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>20.19</v>
+        <v>24.47</v>
       </c>
       <c r="C133" t="n">
-        <v>20.69</v>
+        <v>25</v>
       </c>
       <c r="D133" t="n">
-        <v>2.48</v>
+        <v>2.17</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>KOKUYOCMLN</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>82.8</v>
+        <v>11.6</v>
       </c>
       <c r="C134" t="n">
-        <v>84.84999999999999</v>
+        <v>11.85</v>
       </c>
       <c r="D134" t="n">
-        <v>2.48</v>
+        <v>2.16</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>6.48</v>
+        <v>2.34</v>
       </c>
       <c r="C135" t="n">
-        <v>6.64</v>
+        <v>2.39</v>
       </c>
       <c r="D135" t="n">
-        <v>2.47</v>
+        <v>2.14</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SARVESHWAR</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>3.66</v>
+        <v>0.47</v>
       </c>
       <c r="C136" t="n">
-        <v>3.75</v>
+        <v>0.48</v>
       </c>
       <c r="D136" t="n">
-        <v>2.46</v>
+        <v>2.13</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>80.03</v>
+        <v>1.88</v>
       </c>
       <c r="C137" t="n">
-        <v>82</v>
+        <v>1.92</v>
       </c>
       <c r="D137" t="n">
-        <v>2.46</v>
+        <v>2.13</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>GABRIEL</t>
+          <t>DOLPHIN</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>981</v>
+        <v>391.55</v>
       </c>
       <c r="C138" t="n">
-        <v>1005</v>
+        <v>399.9</v>
       </c>
       <c r="D138" t="n">
-        <v>2.45</v>
+        <v>2.13</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>STEELCITY</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>76.83</v>
+        <v>8.02</v>
       </c>
       <c r="C139" t="n">
-        <v>78.7</v>
+        <v>8.19</v>
       </c>
       <c r="D139" t="n">
-        <v>2.43</v>
+        <v>2.12</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>IRB</t>
+          <t>NIRMAN</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>20.65</v>
+        <v>45.25</v>
       </c>
       <c r="C140" t="n">
-        <v>21.15</v>
+        <v>46.2</v>
       </c>
       <c r="D140" t="n">
-        <v>2.42</v>
+        <v>2.1</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>BAIDFIN</t>
+          <t>UNIMECH</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>9.98</v>
+        <v>1149.75</v>
       </c>
       <c r="C141" t="n">
-        <v>10.22</v>
+        <v>1173.95</v>
       </c>
       <c r="D141" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>NDL</t>
+          <t>KALYANIFRG</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>2.51</v>
+        <v>595.5</v>
       </c>
       <c r="C142" t="n">
-        <v>2.57</v>
+        <v>607.95</v>
       </c>
       <c r="D142" t="n">
-        <v>2.39</v>
+        <v>2.09</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>TARC</t>
+          <t>MAHAPEXLTD</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>123.07</v>
+        <v>47.02</v>
       </c>
       <c r="C143" t="n">
-        <v>126</v>
+        <v>48</v>
       </c>
       <c r="D143" t="n">
-        <v>2.38</v>
+        <v>2.08</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>C2C</t>
+          <t>KRIDHANINF</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>346.7</v>
+        <v>2.93</v>
       </c>
       <c r="C144" t="n">
-        <v>354.9</v>
+        <v>2.99</v>
       </c>
       <c r="D144" t="n">
-        <v>2.37</v>
+        <v>2.05</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>VIKASECO</t>
+          <t>BCG</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>1.27</v>
+        <v>10.73</v>
       </c>
       <c r="C145" t="n">
-        <v>1.3</v>
+        <v>10.95</v>
       </c>
       <c r="D145" t="n">
-        <v>2.36</v>
+        <v>2.05</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>HINDCOMPOS</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>137.22</v>
+        <v>419.4</v>
       </c>
       <c r="C146" t="n">
-        <v>140.44</v>
+        <v>427.95</v>
       </c>
       <c r="D146" t="n">
-        <v>2.35</v>
+        <v>2.04</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>389.8</v>
+        <v>1.47</v>
       </c>
       <c r="C147" t="n">
-        <v>398.95</v>
+        <v>1.5</v>
       </c>
       <c r="D147" t="n">
-        <v>2.35</v>
+        <v>2.04</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>LANDSMILL</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.87</v>
+        <v>0.49</v>
       </c>
       <c r="C148" t="n">
-        <v>0.89</v>
+        <v>0.5</v>
       </c>
       <c r="D148" t="n">
-        <v>2.3</v>
+        <v>2.04</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>OWAIS</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>96.8</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="C149" t="n">
-        <v>99</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="D149" t="n">
-        <v>2.27</v>
+        <v>2.04</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>TCIEXP</t>
+          <t>GLOBALVECT</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>513.05</v>
+        <v>161.42</v>
       </c>
       <c r="C150" t="n">
-        <v>524.6</v>
+        <v>164.7</v>
       </c>
       <c r="D150" t="n">
-        <v>2.25</v>
+        <v>2.03</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>FCL</t>
+          <t>IDBI</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>38.14</v>
+        <v>75.37</v>
       </c>
       <c r="C151" t="n">
-        <v>39</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="D151" t="n">
-        <v>2.25</v>
+        <v>2.03</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>BMWVENTLTD</t>
+          <t>DBOL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>60.12</v>
+        <v>109.72</v>
       </c>
       <c r="C152" t="n">
-        <v>61.47</v>
+        <v>111.95</v>
       </c>
       <c r="D152" t="n">
-        <v>2.25</v>
+        <v>2.03</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>MANCREDIT</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>44.88</v>
+        <v>209.07</v>
       </c>
       <c r="C153" t="n">
-        <v>45.88</v>
+        <v>213.29</v>
       </c>
       <c r="D153" t="n">
-        <v>2.23</v>
+        <v>2.02</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>54.68</v>
+        <v>307.8</v>
       </c>
       <c r="C154" t="n">
-        <v>55.9</v>
+        <v>314</v>
       </c>
       <c r="D154" t="n">
-        <v>2.23</v>
+        <v>2.01</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>2.25</v>
+        <v>93.06</v>
       </c>
       <c r="C155" t="n">
-        <v>2.3</v>
+        <v>94.92</v>
       </c>
       <c r="D155" t="n">
-        <v>2.22</v>
+        <v>2</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>RBMINFRA</t>
+          <t>AMDIND</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>322.8</v>
+        <v>47.2</v>
       </c>
       <c r="C156" t="n">
-        <v>329.95</v>
+        <v>48.14</v>
       </c>
       <c r="D156" t="n">
-        <v>2.21</v>
+        <v>1.99</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>AIRAN</t>
+          <t>IRMENERGY</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>16.38</v>
+        <v>256.85</v>
       </c>
       <c r="C157" t="n">
-        <v>16.74</v>
+        <v>261.95</v>
       </c>
       <c r="D157" t="n">
-        <v>2.2</v>
+        <v>1.99</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>MMWL</t>
+          <t>REPRO</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>13.17</v>
+        <v>359.85</v>
       </c>
       <c r="C158" t="n">
-        <v>13.46</v>
+        <v>367</v>
       </c>
       <c r="D158" t="n">
-        <v>2.2</v>
+        <v>1.99</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>KRONOX</t>
+          <t>EQUIPPP</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>132.29</v>
+        <v>17.15</v>
       </c>
       <c r="C159" t="n">
-        <v>135.2</v>
+        <v>17.49</v>
       </c>
       <c r="D159" t="n">
-        <v>2.2</v>
+        <v>1.98</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>ZENITHDRUG</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>5.49</v>
+        <v>42.95</v>
       </c>
       <c r="C160" t="n">
-        <v>5.61</v>
+        <v>43.8</v>
       </c>
       <c r="D160" t="n">
-        <v>2.19</v>
+        <v>1.98</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>SUNDARAM</t>
+          <t>UEL</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>1.37</v>
+        <v>132.39</v>
       </c>
       <c r="C161" t="n">
-        <v>1.4</v>
+        <v>135</v>
       </c>
       <c r="D161" t="n">
-        <v>2.19</v>
+        <v>1.97</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>OBCL</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>53.73</v>
+        <v>27.01</v>
       </c>
       <c r="C162" t="n">
-        <v>54.9</v>
+        <v>27.54</v>
       </c>
       <c r="D162" t="n">
-        <v>2.18</v>
+        <v>1.96</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>NECCLTD</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>18.5</v>
+        <v>15.01</v>
       </c>
       <c r="C163" t="n">
-        <v>18.9</v>
+        <v>15.3</v>
       </c>
       <c r="D163" t="n">
-        <v>2.16</v>
+        <v>1.93</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ROML</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>46</v>
+        <v>29.99</v>
       </c>
       <c r="C164" t="n">
-        <v>46.99</v>
+        <v>30.57</v>
       </c>
       <c r="D164" t="n">
-        <v>2.15</v>
+        <v>1.93</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>INTENTECH</t>
+          <t>TARMAT</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>90.66</v>
+        <v>51.94</v>
       </c>
       <c r="C165" t="n">
-        <v>92.59999999999999</v>
+        <v>52.94</v>
       </c>
       <c r="D165" t="n">
-        <v>2.14</v>
+        <v>1.93</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>MAHEPC</t>
+          <t>TTKHLTCARE</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>106.22</v>
+        <v>899.35</v>
       </c>
       <c r="C166" t="n">
-        <v>108.48</v>
+        <v>916.7</v>
       </c>
       <c r="D166" t="n">
-        <v>2.13</v>
+        <v>1.93</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>767.6</v>
+        <v>7.31</v>
       </c>
       <c r="C167" t="n">
-        <v>783.95</v>
+        <v>7.45</v>
       </c>
       <c r="D167" t="n">
-        <v>2.13</v>
+        <v>1.92</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>FAZE3Q</t>
+          <t>THEMISMED</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>545.3</v>
+        <v>105.93</v>
       </c>
       <c r="C168" t="n">
-        <v>556.9</v>
+        <v>107.95</v>
       </c>
       <c r="D168" t="n">
-        <v>2.13</v>
+        <v>1.91</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>FINOPB</t>
+          <t>NILASPACES</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>127.73</v>
+        <v>12.06</v>
       </c>
       <c r="C169" t="n">
-        <v>130.44</v>
+        <v>12.29</v>
       </c>
       <c r="D169" t="n">
-        <v>2.12</v>
+        <v>1.91</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>DENTA</t>
+          <t>ESSARSHPNG</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>243.75</v>
+        <v>23.05</v>
       </c>
       <c r="C170" t="n">
-        <v>248.9</v>
+        <v>23.49</v>
       </c>
       <c r="D170" t="n">
-        <v>2.11</v>
+        <v>1.91</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>32.31</v>
+        <v>13.15</v>
       </c>
       <c r="C171" t="n">
-        <v>32.99</v>
+        <v>13.4</v>
       </c>
       <c r="D171" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>FOCUS</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>92.52</v>
+        <v>1471</v>
       </c>
       <c r="C172" t="n">
-        <v>94.45</v>
+        <v>1498.8</v>
       </c>
       <c r="D172" t="n">
-        <v>2.09</v>
+        <v>1.89</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SAHYADRI</t>
+          <t>KOKUYOCMLN</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>269.3</v>
+        <v>83.03</v>
       </c>
       <c r="C173" t="n">
-        <v>274.9</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="D173" t="n">
-        <v>2.08</v>
+        <v>1.89</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>HDIL</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>1.92</v>
+        <v>45.12</v>
       </c>
       <c r="C174" t="n">
-        <v>1.96</v>
+        <v>45.97</v>
       </c>
       <c r="D174" t="n">
-        <v>2.08</v>
+        <v>1.88</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>CEINSYS</t>
+          <t>AMBALALSA</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>922.8</v>
+        <v>34.06</v>
       </c>
       <c r="C175" t="n">
-        <v>942</v>
+        <v>34.7</v>
       </c>
       <c r="D175" t="n">
-        <v>2.08</v>
+        <v>1.88</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>ASMS</t>
+          <t>PREMCO</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>7.24</v>
+        <v>369.95</v>
       </c>
       <c r="C176" t="n">
-        <v>7.39</v>
+        <v>376.9</v>
       </c>
       <c r="D176" t="n">
-        <v>2.07</v>
+        <v>1.88</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>KOVAI</t>
+          <t>RANASUG</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>5517.5</v>
+        <v>12.84</v>
       </c>
       <c r="C177" t="n">
-        <v>5631</v>
+        <v>13.08</v>
       </c>
       <c r="D177" t="n">
-        <v>2.06</v>
+        <v>1.87</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>VADILALIND</t>
+          <t>KAMDHENU</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>5632.9</v>
+        <v>27.28</v>
       </c>
       <c r="C178" t="n">
-        <v>5749</v>
+        <v>27.79</v>
       </c>
       <c r="D178" t="n">
-        <v>2.06</v>
+        <v>1.87</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>SUYOG</t>
+          <t>NOVAAGRI</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>695.65</v>
+        <v>27.78</v>
       </c>
       <c r="C179" t="n">
-        <v>709.95</v>
+        <v>28.3</v>
       </c>
       <c r="D179" t="n">
-        <v>2.06</v>
+        <v>1.87</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>SUMIT</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>22.92</v>
+        <v>41.9</v>
       </c>
       <c r="C180" t="n">
-        <v>23.39</v>
+        <v>42.68</v>
       </c>
       <c r="D180" t="n">
-        <v>2.05</v>
+        <v>1.86</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>RCOM</t>
+          <t>SPENCERS</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>0.98</v>
+        <v>35.57</v>
       </c>
       <c r="C181" t="n">
-        <v>1</v>
+        <v>36.23</v>
       </c>
       <c r="D181" t="n">
-        <v>2.04</v>
+        <v>1.86</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>COMSYN</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>1.96</v>
+        <v>161.89</v>
       </c>
       <c r="C182" t="n">
-        <v>2</v>
+        <v>164.9</v>
       </c>
       <c r="D182" t="n">
-        <v>2.04</v>
+        <v>1.86</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>MOTISONS</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>0.98</v>
+        <v>12.03</v>
       </c>
       <c r="C183" t="n">
-        <v>1</v>
+        <v>12.25</v>
       </c>
       <c r="D183" t="n">
-        <v>2.04</v>
+        <v>1.83</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>KSHINTL</t>
+          <t>AIRAN</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>749.8</v>
+        <v>16.47</v>
       </c>
       <c r="C184" t="n">
-        <v>765</v>
+        <v>16.77</v>
       </c>
       <c r="D184" t="n">
-        <v>2.03</v>
+        <v>1.82</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>OAL</t>
+          <t>SHANTIGOLD</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>314.65</v>
+        <v>218.36</v>
       </c>
       <c r="C185" t="n">
-        <v>321</v>
+        <v>222.25</v>
       </c>
       <c r="D185" t="n">
-        <v>2.02</v>
+        <v>1.78</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>BPL</t>
+          <t>JAYBARMARU</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>51.47</v>
+        <v>138.82</v>
       </c>
       <c r="C186" t="n">
-        <v>52.5</v>
+        <v>141.28</v>
       </c>
       <c r="D186" t="n">
-        <v>2</v>
+        <v>1.77</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>INFLUX</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>416.65</v>
+        <v>232.9</v>
       </c>
       <c r="C187" t="n">
-        <v>425</v>
+        <v>237</v>
       </c>
       <c r="D187" t="n">
-        <v>2</v>
+        <v>1.76</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>CEMPRO</t>
+          <t>ADVANCE</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>1094.4</v>
+        <v>100.49</v>
       </c>
       <c r="C188" t="n">
-        <v>1116.3</v>
+        <v>102.25</v>
       </c>
       <c r="D188" t="n">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>BCLIND</t>
+          <t>PRAENG</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>37.02</v>
+        <v>20.63</v>
       </c>
       <c r="C189" t="n">
-        <v>37.76</v>
+        <v>20.99</v>
       </c>
       <c r="D189" t="n">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>ENIL</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>115.68</v>
+        <v>110.07</v>
       </c>
       <c r="C190" t="n">
-        <v>117.99</v>
+        <v>112</v>
       </c>
       <c r="D190" t="n">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>RAJSREESUG</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>6.07</v>
+        <v>33.4</v>
       </c>
       <c r="C191" t="n">
-        <v>6.19</v>
+        <v>33.97</v>
       </c>
       <c r="D191" t="n">
-        <v>1.98</v>
+        <v>1.71</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>MAGADSUGAR</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>5.05</v>
+        <v>452.25</v>
       </c>
       <c r="C192" t="n">
-        <v>5.15</v>
+        <v>460</v>
       </c>
       <c r="D192" t="n">
-        <v>1.98</v>
+        <v>1.71</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>LYKALABS</t>
+          <t>MENONBE</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>63.69</v>
+        <v>169.81</v>
       </c>
       <c r="C193" t="n">
-        <v>64.95</v>
+        <v>172.69</v>
       </c>
       <c r="D193" t="n">
-        <v>1.98</v>
+        <v>1.7</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>GRMOVER</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>3.53</v>
+        <v>98.33</v>
       </c>
       <c r="C194" t="n">
-        <v>3.6</v>
+        <v>100</v>
       </c>
       <c r="D194" t="n">
-        <v>1.98</v>
+        <v>1.7</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>AJANTPHARM</t>
+          <t>DCAL</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>2968.8</v>
+        <v>187.92</v>
       </c>
       <c r="C195" t="n">
-        <v>3027.3</v>
+        <v>191.1</v>
       </c>
       <c r="D195" t="n">
-        <v>1.97</v>
+        <v>1.69</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>MSTCLTD</t>
+          <t>LASA</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>490.15</v>
+        <v>7.67</v>
       </c>
       <c r="C196" t="n">
-        <v>499.8</v>
+        <v>7.8</v>
       </c>
       <c r="D196" t="n">
-        <v>1.97</v>
+        <v>1.69</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>RPPINFRA</t>
+          <t>KRITIKA</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>59.33</v>
+        <v>5.98</v>
       </c>
       <c r="C197" t="n">
-        <v>60.5</v>
+        <v>6.08</v>
       </c>
       <c r="D197" t="n">
-        <v>1.97</v>
+        <v>1.67</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>SMARTLINK</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>1469.2</v>
+        <v>162.3</v>
       </c>
       <c r="C198" t="n">
-        <v>1497.9</v>
+        <v>165</v>
       </c>
       <c r="D198" t="n">
-        <v>1.95</v>
+        <v>1.66</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>DREAMFOLKS</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>139.01</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="C199" t="n">
-        <v>141.7</v>
+        <v>70.8</v>
       </c>
       <c r="D199" t="n">
-        <v>1.94</v>
+        <v>1.65</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>NECCLTD</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>14.96</v>
+        <v>4.88</v>
       </c>
       <c r="C200" t="n">
-        <v>15.25</v>
+        <v>4.96</v>
       </c>
       <c r="D200" t="n">
-        <v>1.94</v>
+        <v>1.64</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>TIPSMUSIC</t>
+          <t>DONEAR</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>656.3</v>
+        <v>89.44</v>
       </c>
       <c r="C201" t="n">
-        <v>669</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="D201" t="n">
-        <v>1.94</v>
+        <v>1.63</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-11 08:24 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>SHAH-RE1</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>18.62</v>
+        <v>0.01</v>
       </c>
       <c r="C2" t="n">
-        <v>21.9</v>
+        <v>0.02</v>
       </c>
       <c r="D2" t="n">
-        <v>17.62</v>
+        <v>100</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PIONRINV</t>
+          <t>SILLYMONKS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.14</v>
+        <v>18.38</v>
       </c>
       <c r="C3" t="n">
-        <v>114.98</v>
+        <v>19.85</v>
       </c>
       <c r="D3" t="n">
-        <v>15.98</v>
+        <v>8</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RSDFIN</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>78</v>
+        <v>2.13</v>
       </c>
       <c r="C4" t="n">
-        <v>85.98999999999999</v>
+        <v>2.29</v>
       </c>
       <c r="D4" t="n">
-        <v>10.24</v>
+        <v>7.51</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20.91</v>
+        <v>4.81</v>
       </c>
       <c r="C5" t="n">
-        <v>23</v>
+        <v>5.17</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>7.48</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CLEANMAX</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1232.4</v>
+        <v>1.89</v>
       </c>
       <c r="C6" t="n">
-        <v>1350</v>
+        <v>2.03</v>
       </c>
       <c r="D6" t="n">
-        <v>9.539999999999999</v>
+        <v>7.41</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SUPREMEINF</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>76.87</v>
+        <v>0.14</v>
       </c>
       <c r="C7" t="n">
-        <v>83.29000000000001</v>
+        <v>0.15</v>
       </c>
       <c r="D7" t="n">
-        <v>8.35</v>
+        <v>7.14</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.9</v>
+        <v>22.34</v>
       </c>
       <c r="C8" t="n">
-        <v>5.28</v>
+        <v>23.8</v>
       </c>
       <c r="D8" t="n">
-        <v>7.76</v>
+        <v>6.54</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>31.61</v>
+        <v>48.64</v>
       </c>
       <c r="C9" t="n">
-        <v>33.99</v>
+        <v>51.79</v>
       </c>
       <c r="D9" t="n">
-        <v>7.53</v>
+        <v>6.48</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>SECMARK</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.14</v>
+        <v>127.71</v>
       </c>
       <c r="C10" t="n">
-        <v>0.15</v>
+        <v>135.45</v>
       </c>
       <c r="D10" t="n">
-        <v>7.14</v>
+        <v>6.06</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>COOLCAPS</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>25.2</v>
+        <v>23</v>
       </c>
       <c r="C11" t="n">
-        <v>26.9</v>
+        <v>24.33</v>
       </c>
       <c r="D11" t="n">
-        <v>6.75</v>
+        <v>5.78</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INNOVANA</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>300.55</v>
+        <v>0.19</v>
       </c>
       <c r="C12" t="n">
-        <v>319.9</v>
+        <v>0.2</v>
       </c>
       <c r="D12" t="n">
-        <v>6.44</v>
+        <v>5.26</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>23.36</v>
+        <v>8.19</v>
       </c>
       <c r="C13" t="n">
-        <v>24.85</v>
+        <v>8.6</v>
       </c>
       <c r="D13" t="n">
-        <v>6.38</v>
+        <v>5.01</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AFCONS</t>
+          <t>LASA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>315.5</v>
+        <v>7.6</v>
       </c>
       <c r="C14" t="n">
-        <v>335</v>
+        <v>7.98</v>
       </c>
       <c r="D14" t="n">
-        <v>6.18</v>
+        <v>5</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>GJL</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4.72</v>
+        <v>138.1</v>
       </c>
       <c r="C15" t="n">
-        <v>4.98</v>
+        <v>145</v>
       </c>
       <c r="D15" t="n">
-        <v>5.51</v>
+        <v>5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LYKALABS</t>
+          <t>KDL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>70.05</v>
+        <v>114.2</v>
       </c>
       <c r="C16" t="n">
-        <v>73.8</v>
+        <v>119.9</v>
       </c>
       <c r="D16" t="n">
-        <v>5.35</v>
+        <v>4.99</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>24.35</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="C17" t="n">
-        <v>25.6</v>
+        <v>98.8</v>
       </c>
       <c r="D17" t="n">
-        <v>5.13</v>
+        <v>4.99</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>VASCONEQ</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.2</v>
+        <v>33.08</v>
       </c>
       <c r="C18" t="n">
-        <v>0.21</v>
+        <v>34.73</v>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SILKFLEX</t>
+          <t>TIJARIA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>199.5</v>
+        <v>4.43</v>
       </c>
       <c r="C19" t="n">
-        <v>209.45</v>
+        <v>4.65</v>
       </c>
       <c r="D19" t="n">
-        <v>4.99</v>
+        <v>4.97</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BOHRAIND</t>
+          <t>SHEEL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>17.82</v>
+        <v>54.45</v>
       </c>
       <c r="C20" t="n">
-        <v>18.71</v>
+        <v>57.15</v>
       </c>
       <c r="D20" t="n">
-        <v>4.99</v>
+        <v>4.96</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>37.9</v>
+        <v>6.86</v>
       </c>
       <c r="C21" t="n">
-        <v>39.79</v>
+        <v>7.2</v>
       </c>
       <c r="D21" t="n">
-        <v>4.99</v>
+        <v>4.96</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>437.45</v>
+        <v>9.75</v>
       </c>
       <c r="C22" t="n">
-        <v>459.3</v>
+        <v>10.23</v>
       </c>
       <c r="D22" t="n">
-        <v>4.99</v>
+        <v>4.92</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>PPAP</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5.52</v>
+        <v>205.76</v>
       </c>
       <c r="C23" t="n">
-        <v>5.79</v>
+        <v>215.85</v>
       </c>
       <c r="D23" t="n">
-        <v>4.89</v>
+        <v>4.9</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>CEREBRAINT</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.49</v>
+        <v>3.67</v>
       </c>
       <c r="C24" t="n">
-        <v>3.66</v>
+        <v>3.85</v>
       </c>
       <c r="D24" t="n">
-        <v>4.87</v>
+        <v>4.9</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>QVCEL</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>14.5</v>
+        <v>23.5</v>
       </c>
       <c r="C25" t="n">
-        <v>15.2</v>
+        <v>24.65</v>
       </c>
       <c r="D25" t="n">
-        <v>4.83</v>
+        <v>4.89</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VIVIDEL</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1000.1</v>
+        <v>110</v>
       </c>
       <c r="C26" t="n">
-        <v>1048</v>
+        <v>115.2</v>
       </c>
       <c r="D26" t="n">
-        <v>4.79</v>
+        <v>4.73</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SSFL</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>212.6</v>
+        <v>2.55</v>
       </c>
       <c r="C27" t="n">
-        <v>222.7</v>
+        <v>2.67</v>
       </c>
       <c r="D27" t="n">
-        <v>4.75</v>
+        <v>4.71</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>FMNL</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6.54</v>
+        <v>10.01</v>
       </c>
       <c r="C28" t="n">
-        <v>6.85</v>
+        <v>10.48</v>
       </c>
       <c r="D28" t="n">
-        <v>4.74</v>
+        <v>4.7</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CYBERMEDIA</t>
+          <t>WIPL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>16.42</v>
+        <v>148</v>
       </c>
       <c r="C29" t="n">
-        <v>17.19</v>
+        <v>154.9</v>
       </c>
       <c r="D29" t="n">
-        <v>4.69</v>
+        <v>4.66</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CONSOFINVT</t>
+          <t>NOIDATOLL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>226.44</v>
+        <v>4.75</v>
       </c>
       <c r="C30" t="n">
-        <v>237</v>
+        <v>4.97</v>
       </c>
       <c r="D30" t="n">
-        <v>4.66</v>
+        <v>4.63</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FELDVR</t>
+          <t>NECCLTD</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2.58</v>
+        <v>18.01</v>
       </c>
       <c r="C31" t="n">
-        <v>2.7</v>
+        <v>18.84</v>
       </c>
       <c r="D31" t="n">
-        <v>4.65</v>
+        <v>4.61</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SUPREMEENG</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1.08</v>
+        <v>0.22</v>
       </c>
       <c r="C32" t="n">
-        <v>1.13</v>
+        <v>0.23</v>
       </c>
       <c r="D32" t="n">
-        <v>4.63</v>
+        <v>4.55</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>CUDML</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>28.44</v>
+        <v>182.7</v>
       </c>
       <c r="C33" t="n">
-        <v>29.75</v>
+        <v>191</v>
       </c>
       <c r="D33" t="n">
-        <v>4.61</v>
+        <v>4.54</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SIMBHALS</t>
+          <t>SUPREMEENG</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>7.03</v>
+        <v>1.13</v>
       </c>
       <c r="C34" t="n">
-        <v>7.35</v>
+        <v>1.18</v>
       </c>
       <c r="D34" t="n">
-        <v>4.55</v>
+        <v>4.42</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>QPOWER</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1133.7</v>
+        <v>315.2</v>
       </c>
       <c r="C35" t="n">
-        <v>1185</v>
+        <v>329</v>
       </c>
       <c r="D35" t="n">
-        <v>4.53</v>
+        <v>4.38</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GTPL</t>
+          <t>PRIZOR</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>63.44</v>
+        <v>826.75</v>
       </c>
       <c r="C36" t="n">
-        <v>66.3</v>
+        <v>862.5</v>
       </c>
       <c r="D36" t="n">
-        <v>4.51</v>
+        <v>4.32</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>RSWM</t>
+          <t>UNICHEMLAB</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>213.4</v>
+        <v>437.4</v>
       </c>
       <c r="C37" t="n">
-        <v>222.99</v>
+        <v>456</v>
       </c>
       <c r="D37" t="n">
-        <v>4.49</v>
+        <v>4.25</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MANAKSTEEL</t>
+          <t>HDIL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>66.81</v>
+        <v>1.89</v>
       </c>
       <c r="C38" t="n">
-        <v>69.8</v>
+        <v>1.97</v>
       </c>
       <c r="D38" t="n">
-        <v>4.48</v>
+        <v>4.23</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CEREBRAINT</t>
+          <t>RADAAN</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3.59</v>
+        <v>3.07</v>
       </c>
       <c r="C39" t="n">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="D39" t="n">
-        <v>4.46</v>
+        <v>4.23</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>SADBHAV</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>4.49</v>
+        <v>9.4</v>
       </c>
       <c r="C40" t="n">
-        <v>4.69</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="D40" t="n">
-        <v>4.45</v>
+        <v>4.15</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CPCAP</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>91.44</v>
+        <v>4.71</v>
       </c>
       <c r="C41" t="n">
-        <v>95.48999999999999</v>
+        <v>4.9</v>
       </c>
       <c r="D41" t="n">
-        <v>4.43</v>
+        <v>4.03</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SYSTMTXC</t>
+          <t>INTENTECH</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>65.11</v>
+        <v>102.63</v>
       </c>
       <c r="C42" t="n">
-        <v>67.95</v>
+        <v>106.76</v>
       </c>
       <c r="D42" t="n">
-        <v>4.36</v>
+        <v>4.02</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BONLON</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>42.16</v>
+        <v>414.6</v>
       </c>
       <c r="C43" t="n">
-        <v>43.99</v>
+        <v>431.25</v>
       </c>
       <c r="D43" t="n">
-        <v>4.34</v>
+        <v>4.02</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SICALLOG</t>
+          <t>HOLMARC</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>79.56999999999999</v>
+        <v>106.7</v>
       </c>
       <c r="C44" t="n">
-        <v>82.98</v>
+        <v>110.9</v>
       </c>
       <c r="D44" t="n">
-        <v>4.29</v>
+        <v>3.94</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MAXVOLT</t>
+          <t>SUDARSCHEM</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>383.6</v>
+        <v>854.05</v>
       </c>
       <c r="C45" t="n">
-        <v>400</v>
+        <v>887.7</v>
       </c>
       <c r="D45" t="n">
-        <v>4.28</v>
+        <v>3.94</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MITCON</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>82.38</v>
+        <v>21.15</v>
       </c>
       <c r="C46" t="n">
-        <v>85.84999999999999</v>
+        <v>21.98</v>
       </c>
       <c r="D46" t="n">
-        <v>4.21</v>
+        <v>3.92</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>68.23</v>
+        <v>2.3</v>
       </c>
       <c r="C47" t="n">
-        <v>71</v>
+        <v>2.39</v>
       </c>
       <c r="D47" t="n">
-        <v>4.06</v>
+        <v>3.91</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1.54</v>
+        <v>7</v>
       </c>
       <c r="C48" t="n">
-        <v>1.6</v>
+        <v>7.25</v>
       </c>
       <c r="D48" t="n">
-        <v>3.9</v>
+        <v>3.57</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TEAMTECH</t>
+          <t>SILKFLEX</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>78.95</v>
+        <v>209.45</v>
       </c>
       <c r="C49" t="n">
-        <v>81.95</v>
+        <v>216.9</v>
       </c>
       <c r="D49" t="n">
-        <v>3.8</v>
+        <v>3.56</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MEESHO</t>
+          <t>MODIRUBBER</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>166.73</v>
+        <v>126.63</v>
       </c>
       <c r="C50" t="n">
-        <v>173</v>
+        <v>131.1</v>
       </c>
       <c r="D50" t="n">
-        <v>3.76</v>
+        <v>3.53</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ARCIIL</t>
+          <t>FINKURVE</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>42.9</v>
+        <v>64.36</v>
       </c>
       <c r="C51" t="n">
-        <v>44.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="D51" t="n">
-        <v>3.73</v>
+        <v>3.48</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>HGS</t>
+          <t>3IINFOLTD</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>400.25</v>
+        <v>16.43</v>
       </c>
       <c r="C52" t="n">
-        <v>415</v>
+        <v>17</v>
       </c>
       <c r="D52" t="n">
-        <v>3.69</v>
+        <v>3.47</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ENERGYDEV</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>16.69</v>
+        <v>44.17</v>
       </c>
       <c r="C53" t="n">
-        <v>17.3</v>
+        <v>45.7</v>
       </c>
       <c r="D53" t="n">
-        <v>3.65</v>
+        <v>3.46</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TECILCHEM</t>
+          <t>MAHAPEXLTD</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>11</v>
+        <v>48.8</v>
       </c>
       <c r="C54" t="n">
-        <v>11.4</v>
+        <v>50.48</v>
       </c>
       <c r="D54" t="n">
-        <v>3.64</v>
+        <v>3.44</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>ANTELOPUS</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1.93</v>
+        <v>818.8</v>
       </c>
       <c r="C55" t="n">
-        <v>2</v>
+        <v>846.95</v>
       </c>
       <c r="D55" t="n">
-        <v>3.63</v>
+        <v>3.44</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>DBSTOCKBRO</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>18.23</v>
+        <v>31.42</v>
       </c>
       <c r="C56" t="n">
-        <v>18.89</v>
+        <v>32.49</v>
       </c>
       <c r="D56" t="n">
-        <v>3.62</v>
+        <v>3.41</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MERCANTILE</t>
+          <t>MFML</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>25.11</v>
+        <v>23.8</v>
       </c>
       <c r="C57" t="n">
-        <v>26</v>
+        <v>24.59</v>
       </c>
       <c r="D57" t="n">
-        <v>3.54</v>
+        <v>3.32</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>WINDMACHIN</t>
+          <t>HEADSUP</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>313.7</v>
+        <v>7.01</v>
       </c>
       <c r="C58" t="n">
-        <v>324.75</v>
+        <v>7.24</v>
       </c>
       <c r="D58" t="n">
-        <v>3.52</v>
+        <v>3.28</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>ANIKINDS</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1309.3</v>
+        <v>42.56</v>
       </c>
       <c r="C59" t="n">
-        <v>1355.2</v>
+        <v>43.95</v>
       </c>
       <c r="D59" t="n">
-        <v>3.51</v>
+        <v>3.27</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>EUROBOND</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>176.46</v>
+        <v>28.32</v>
       </c>
       <c r="C60" t="n">
-        <v>182.6</v>
+        <v>29.24</v>
       </c>
       <c r="D60" t="n">
-        <v>3.48</v>
+        <v>3.25</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ADL</t>
+          <t>MANAKALUCO</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>72.40000000000001</v>
+        <v>41.21</v>
       </c>
       <c r="C61" t="n">
-        <v>74.90000000000001</v>
+        <v>42.54</v>
       </c>
       <c r="D61" t="n">
-        <v>3.45</v>
+        <v>3.23</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BANARBEADS</t>
+          <t>SURYALAXMI</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>99.7</v>
+        <v>56.01</v>
       </c>
       <c r="C62" t="n">
-        <v>103.1</v>
+        <v>57.8</v>
       </c>
       <c r="D62" t="n">
-        <v>3.41</v>
+        <v>3.2</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>NILASPACES</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>34.25</v>
+        <v>11.9</v>
       </c>
       <c r="C63" t="n">
-        <v>35.4</v>
+        <v>12.28</v>
       </c>
       <c r="D63" t="n">
-        <v>3.36</v>
+        <v>3.19</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DAMODARIND</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>30.15</v>
+        <v>11.99</v>
       </c>
       <c r="C64" t="n">
-        <v>31.15</v>
+        <v>12.36</v>
       </c>
       <c r="D64" t="n">
-        <v>3.32</v>
+        <v>3.09</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>GRCL</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>540</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="C65" t="n">
-        <v>557.9</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="D65" t="n">
-        <v>3.31</v>
+        <v>3.07</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1873,13 +1873,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>37.77</v>
+        <v>43.56</v>
       </c>
       <c r="C66" t="n">
-        <v>39</v>
+        <v>44.89</v>
       </c>
       <c r="D66" t="n">
-        <v>3.26</v>
+        <v>3.05</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>KARMAENG</t>
+          <t>CNL</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>41.98</v>
+        <v>693.95</v>
       </c>
       <c r="C67" t="n">
-        <v>43.35</v>
+        <v>715</v>
       </c>
       <c r="D67" t="n">
-        <v>3.26</v>
+        <v>3.03</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>OWAIS</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>96.3</v>
+        <v>13.58</v>
       </c>
       <c r="C68" t="n">
-        <v>99.40000000000001</v>
+        <v>13.99</v>
       </c>
       <c r="D68" t="n">
-        <v>3.22</v>
+        <v>3.02</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SUPREME</t>
+          <t>GOLDTECH</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>44.46</v>
+        <v>41.72</v>
       </c>
       <c r="C69" t="n">
-        <v>45.88</v>
+        <v>42.98</v>
       </c>
       <c r="D69" t="n">
-        <v>3.19</v>
+        <v>3.02</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>KEYFINSERV</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>255.85</v>
+        <v>21.75</v>
       </c>
       <c r="C70" t="n">
-        <v>263.95</v>
+        <v>22.39</v>
       </c>
       <c r="D70" t="n">
-        <v>3.17</v>
+        <v>2.94</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>RILINFRA</t>
+          <t>NITIRAJ</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>34.9</v>
+        <v>184.63</v>
       </c>
       <c r="C71" t="n">
-        <v>36</v>
+        <v>190</v>
       </c>
       <c r="D71" t="n">
-        <v>3.15</v>
+        <v>2.91</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>NDL</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>2.56</v>
+        <v>37.91</v>
       </c>
       <c r="C72" t="n">
-        <v>2.64</v>
+        <v>39</v>
       </c>
       <c r="D72" t="n">
-        <v>3.13</v>
+        <v>2.88</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>HITECHCORP</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>309.32</v>
+        <v>48.12</v>
       </c>
       <c r="C73" t="n">
-        <v>319</v>
+        <v>49.5</v>
       </c>
       <c r="D73" t="n">
-        <v>3.13</v>
+        <v>2.87</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>RAJOOENG</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>53.21</v>
+        <v>0.36</v>
       </c>
       <c r="C74" t="n">
-        <v>54.87</v>
+        <v>0.37</v>
       </c>
       <c r="D74" t="n">
-        <v>3.12</v>
+        <v>2.78</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>TNTELE</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>13.17</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="C75" t="n">
-        <v>13.58</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D75" t="n">
-        <v>3.11</v>
+        <v>2.76</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>KAPSTON</t>
+          <t>BANARBEADS</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>337.5</v>
+        <v>98.3</v>
       </c>
       <c r="C76" t="n">
-        <v>347.9</v>
+        <v>101</v>
       </c>
       <c r="D76" t="n">
-        <v>3.08</v>
+        <v>2.75</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ATALREAL</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>24.72</v>
+        <v>8.75</v>
       </c>
       <c r="C77" t="n">
-        <v>25.47</v>
+        <v>8.99</v>
       </c>
       <c r="D77" t="n">
-        <v>3.03</v>
+        <v>2.74</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CEMPRO</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1203.8</v>
+        <v>174.72</v>
       </c>
       <c r="C78" t="n">
-        <v>1240</v>
+        <v>179.49</v>
       </c>
       <c r="D78" t="n">
-        <v>3.01</v>
+        <v>2.73</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>22.76</v>
+        <v>13.61</v>
       </c>
       <c r="C79" t="n">
-        <v>23.44</v>
+        <v>13.98</v>
       </c>
       <c r="D79" t="n">
-        <v>2.99</v>
+        <v>2.72</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>AROGRANITE</t>
+          <t>SHRENIK</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>24.76</v>
+        <v>0.37</v>
       </c>
       <c r="C80" t="n">
-        <v>25.5</v>
+        <v>0.38</v>
       </c>
       <c r="D80" t="n">
-        <v>2.99</v>
+        <v>2.7</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>1.01</v>
+        <v>3.86</v>
       </c>
       <c r="C81" t="n">
-        <v>1.04</v>
+        <v>3.96</v>
       </c>
       <c r="D81" t="n">
-        <v>2.97</v>
+        <v>2.59</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>PASHUPATI</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>88.67</v>
+        <v>378.15</v>
       </c>
       <c r="C82" t="n">
-        <v>91.3</v>
+        <v>387.95</v>
       </c>
       <c r="D82" t="n">
-        <v>2.97</v>
+        <v>2.59</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>MENNPIS</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>48.08</v>
+        <v>55.34</v>
       </c>
       <c r="C83" t="n">
-        <v>49.5</v>
+        <v>56.75</v>
       </c>
       <c r="D83" t="n">
-        <v>2.95</v>
+        <v>2.55</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>LIKHITHA</t>
+          <t>MAGADSUGAR</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>227.11</v>
+        <v>448.1</v>
       </c>
       <c r="C84" t="n">
-        <v>233.8</v>
+        <v>459.5</v>
       </c>
       <c r="D84" t="n">
-        <v>2.95</v>
+        <v>2.54</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>NORBTEAEXP</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>7.46</v>
+        <v>76.7</v>
       </c>
       <c r="C85" t="n">
-        <v>7.68</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="D85" t="n">
-        <v>2.95</v>
+        <v>2.48</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>REDTAPE</t>
+          <t>DJML</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>133.81</v>
+        <v>109.32</v>
       </c>
       <c r="C86" t="n">
-        <v>137.7</v>
+        <v>112</v>
       </c>
       <c r="D86" t="n">
-        <v>2.91</v>
+        <v>2.45</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>MENNPIS</t>
+          <t>GROBTEA</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>54.25</v>
+        <v>926.4</v>
       </c>
       <c r="C87" t="n">
-        <v>55.83</v>
+        <v>949</v>
       </c>
       <c r="D87" t="n">
-        <v>2.91</v>
+        <v>2.44</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>364.45</v>
+        <v>79.43000000000001</v>
       </c>
       <c r="C88" t="n">
-        <v>374.95</v>
+        <v>81.37</v>
       </c>
       <c r="D88" t="n">
-        <v>2.88</v>
+        <v>2.44</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>2.43</v>
+        <v>27.44</v>
       </c>
       <c r="C89" t="n">
-        <v>2.5</v>
+        <v>28.1</v>
       </c>
       <c r="D89" t="n">
-        <v>2.88</v>
+        <v>2.41</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>EQUIPPP</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>6.37</v>
+        <v>17.19</v>
       </c>
       <c r="C90" t="n">
-        <v>6.55</v>
+        <v>17.6</v>
       </c>
       <c r="D90" t="n">
-        <v>2.83</v>
+        <v>2.39</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>31.21</v>
+        <v>0.42</v>
       </c>
       <c r="C91" t="n">
-        <v>32.09</v>
+        <v>0.43</v>
       </c>
       <c r="D91" t="n">
-        <v>2.82</v>
+        <v>2.38</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>BELLACASA</t>
+          <t>EMAMIPAP</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>232.97</v>
+        <v>85.01000000000001</v>
       </c>
       <c r="C92" t="n">
-        <v>239.5</v>
+        <v>87</v>
       </c>
       <c r="D92" t="n">
-        <v>2.8</v>
+        <v>2.34</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>KHADIM</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>100</v>
+        <v>39.54</v>
       </c>
       <c r="C93" t="n">
-        <v>102.8</v>
+        <v>40.45</v>
       </c>
       <c r="D93" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0.36</v>
+        <v>7.92</v>
       </c>
       <c r="C94" t="n">
-        <v>0.37</v>
+        <v>8.1</v>
       </c>
       <c r="D94" t="n">
-        <v>2.78</v>
+        <v>2.27</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>AYMSYNTEX</t>
+          <t>KCPSUGIND</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>218.49</v>
+        <v>22.88</v>
       </c>
       <c r="C95" t="n">
-        <v>224.5</v>
+        <v>23.39</v>
       </c>
       <c r="D95" t="n">
-        <v>2.75</v>
+        <v>2.23</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>5.84</v>
+        <v>0.45</v>
       </c>
       <c r="C96" t="n">
-        <v>6</v>
+        <v>0.46</v>
       </c>
       <c r="D96" t="n">
-        <v>2.74</v>
+        <v>2.22</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>LAHOTIOV</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>4.03</v>
+        <v>44.91</v>
       </c>
       <c r="C97" t="n">
-        <v>4.14</v>
+        <v>45.9</v>
       </c>
       <c r="D97" t="n">
-        <v>2.73</v>
+        <v>2.2</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>FIBERWEB</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>384.3</v>
+        <v>27.99</v>
       </c>
       <c r="C98" t="n">
-        <v>394.7</v>
+        <v>28.6</v>
       </c>
       <c r="D98" t="n">
-        <v>2.71</v>
+        <v>2.18</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>IWARE</t>
+          <t>GLOBE</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>330</v>
+        <v>2.29</v>
       </c>
       <c r="C99" t="n">
-        <v>338.95</v>
+        <v>2.34</v>
       </c>
       <c r="D99" t="n">
-        <v>2.71</v>
+        <v>2.18</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ORIENTLTD</t>
+          <t>SELMC</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>58.81</v>
+        <v>29.85</v>
       </c>
       <c r="C100" t="n">
-        <v>60.4</v>
+        <v>30.5</v>
       </c>
       <c r="D100" t="n">
-        <v>2.7</v>
+        <v>2.18</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MVGJL</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>150</v>
+        <v>39.06</v>
       </c>
       <c r="C101" t="n">
-        <v>154</v>
+        <v>39.9</v>
       </c>
       <c r="D101" t="n">
-        <v>2.67</v>
+        <v>2.15</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PAUSHAKLTD</t>
+          <t>SAWALIYA</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>466.7</v>
+        <v>282.75</v>
       </c>
       <c r="C102" t="n">
-        <v>479</v>
+        <v>288.8</v>
       </c>
       <c r="D102" t="n">
-        <v>2.64</v>
+        <v>2.14</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>AURIGROW</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.38</v>
+        <v>7.06</v>
       </c>
       <c r="C103" t="n">
-        <v>0.39</v>
+        <v>7.21</v>
       </c>
       <c r="D103" t="n">
-        <v>2.63</v>
+        <v>2.12</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>KANANIIND</t>
+          <t>TECHERA</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>1.55</v>
+        <v>136.7</v>
       </c>
       <c r="C104" t="n">
-        <v>1.59</v>
+        <v>139.6</v>
       </c>
       <c r="D104" t="n">
-        <v>2.58</v>
+        <v>2.12</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>AGROPHOS</t>
+          <t>VELJAN</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>30.23</v>
+        <v>1282.8</v>
       </c>
       <c r="C105" t="n">
-        <v>31</v>
+        <v>1310</v>
       </c>
       <c r="D105" t="n">
-        <v>2.55</v>
+        <v>2.12</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>AMNPLST</t>
+          <t>SAKUMA</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>197.68</v>
+        <v>1.91</v>
       </c>
       <c r="C106" t="n">
-        <v>202.7</v>
+        <v>1.95</v>
       </c>
       <c r="D106" t="n">
-        <v>2.54</v>
+        <v>2.09</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>UFLEX</t>
+          <t>SCANSTL</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>417.1</v>
+        <v>34.97</v>
       </c>
       <c r="C107" t="n">
-        <v>427.7</v>
+        <v>35.7</v>
       </c>
       <c r="D107" t="n">
-        <v>2.54</v>
+        <v>2.09</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>WEALTH</t>
+          <t>CORALFINAC</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>940.2</v>
+        <v>31.5</v>
       </c>
       <c r="C108" t="n">
-        <v>964</v>
+        <v>32.15</v>
       </c>
       <c r="D108" t="n">
-        <v>2.53</v>
+        <v>2.06</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>WAKEFIT</t>
+          <t>MANOMAY</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>118.02</v>
+        <v>195.73</v>
       </c>
       <c r="C109" t="n">
-        <v>120.99</v>
+        <v>199.7</v>
       </c>
       <c r="D109" t="n">
-        <v>2.52</v>
+        <v>2.03</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>SRTL</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>18.63</v>
+        <v>41.35</v>
       </c>
       <c r="C110" t="n">
-        <v>19.1</v>
+        <v>42.19</v>
       </c>
       <c r="D110" t="n">
-        <v>2.52</v>
+        <v>2.03</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>PRAKASHSTL</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>4.39</v>
+        <v>13.43</v>
       </c>
       <c r="C111" t="n">
-        <v>4.5</v>
+        <v>13.7</v>
       </c>
       <c r="D111" t="n">
-        <v>2.51</v>
+        <v>2.01</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>170.7</v>
+        <v>0.5</v>
       </c>
       <c r="C112" t="n">
-        <v>174.99</v>
+        <v>0.51</v>
       </c>
       <c r="D112" t="n">
-        <v>2.51</v>
+        <v>2</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AEGISVOPAK</t>
+          <t>MAWANASUG</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>191.67</v>
+        <v>101.97</v>
       </c>
       <c r="C113" t="n">
-        <v>196.48</v>
+        <v>104</v>
       </c>
       <c r="D113" t="n">
-        <v>2.51</v>
+        <v>1.99</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>DCMSRIND</t>
+          <t>VASWANI</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>40.45</v>
+        <v>59.52</v>
       </c>
       <c r="C114" t="n">
-        <v>41.44</v>
+        <v>60.7</v>
       </c>
       <c r="D114" t="n">
-        <v>2.45</v>
+        <v>1.98</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>FIBERWEB</t>
+          <t>MITTAL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>28</v>
+        <v>1.02</v>
       </c>
       <c r="C115" t="n">
-        <v>28.68</v>
+        <v>1.04</v>
       </c>
       <c r="D115" t="n">
-        <v>2.43</v>
+        <v>1.96</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CENTRUM</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>21.77</v>
+        <v>31.84</v>
       </c>
       <c r="C116" t="n">
-        <v>22.3</v>
+        <v>32.45</v>
       </c>
       <c r="D116" t="n">
-        <v>2.43</v>
+        <v>1.92</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>KAVDEFENCE</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>60.44</v>
+        <v>197.16</v>
       </c>
       <c r="C117" t="n">
-        <v>61.9</v>
+        <v>200.9</v>
       </c>
       <c r="D117" t="n">
-        <v>2.42</v>
+        <v>1.9</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>KOTIC</t>
+          <t>ADVANCE</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>161.84</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="C118" t="n">
-        <v>165.75</v>
+        <v>100.98</v>
       </c>
       <c r="D118" t="n">
-        <v>2.42</v>
+        <v>1.9</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>INVPRECQ</t>
+          <t>ODIGMA</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>613.3</v>
+        <v>20.5</v>
       </c>
       <c r="C119" t="n">
-        <v>627.9</v>
+        <v>20.89</v>
       </c>
       <c r="D119" t="n">
-        <v>2.38</v>
+        <v>1.9</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>A2ZINFRA</t>
+          <t>EBGNG</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>14.56</v>
+        <v>392.6</v>
       </c>
       <c r="C120" t="n">
-        <v>14.9</v>
+        <v>400</v>
       </c>
       <c r="D120" t="n">
-        <v>2.34</v>
+        <v>1.88</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SATIA</t>
+          <t>VLSFINANCE</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>54.71</v>
+        <v>228</v>
       </c>
       <c r="C121" t="n">
-        <v>55.99</v>
+        <v>232.24</v>
       </c>
       <c r="D121" t="n">
-        <v>2.34</v>
+        <v>1.86</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>SHIVATEX</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>178.82</v>
+        <v>151.5</v>
       </c>
       <c r="C122" t="n">
-        <v>183</v>
+        <v>154.3</v>
       </c>
       <c r="D122" t="n">
-        <v>2.34</v>
+        <v>1.85</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>UEL</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>0.43</v>
+        <v>143.21</v>
       </c>
       <c r="C123" t="n">
-        <v>0.44</v>
+        <v>145.79</v>
       </c>
       <c r="D123" t="n">
-        <v>2.33</v>
+        <v>1.8</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>RMDRIP</t>
+          <t>NAHARPOLY</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>16.05</v>
+        <v>239.7</v>
       </c>
       <c r="C124" t="n">
-        <v>16.42</v>
+        <v>244</v>
       </c>
       <c r="D124" t="n">
-        <v>2.31</v>
+        <v>1.79</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>RMDRIP</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>8.27</v>
+        <v>16.85</v>
       </c>
       <c r="C125" t="n">
-        <v>8.460000000000001</v>
+        <v>17.15</v>
       </c>
       <c r="D125" t="n">
-        <v>2.3</v>
+        <v>1.78</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>NDLVENTURE</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>130.03</v>
+        <v>5.09</v>
       </c>
       <c r="C126" t="n">
-        <v>133</v>
+        <v>5.18</v>
       </c>
       <c r="D126" t="n">
-        <v>2.28</v>
+        <v>1.77</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>BIMETAL</t>
+          <t>SURYODAY</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>641.25</v>
+        <v>170</v>
       </c>
       <c r="C127" t="n">
-        <v>655.9</v>
+        <v>173</v>
       </c>
       <c r="D127" t="n">
-        <v>2.28</v>
+        <v>1.76</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>IFBAGRO</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>7.53</v>
+        <v>929.5</v>
       </c>
       <c r="C128" t="n">
-        <v>7.7</v>
+        <v>945.9</v>
       </c>
       <c r="D128" t="n">
-        <v>2.26</v>
+        <v>1.76</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>3BBLACKBIO</t>
+          <t>MGEL</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>1201.5</v>
+        <v>16.51</v>
       </c>
       <c r="C129" t="n">
-        <v>1228</v>
+        <v>16.8</v>
       </c>
       <c r="D129" t="n">
-        <v>2.21</v>
+        <v>1.76</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ASMS</t>
+          <t>TRIGYN</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>7.27</v>
+        <v>54.93</v>
       </c>
       <c r="C130" t="n">
-        <v>7.43</v>
+        <v>55.88</v>
       </c>
       <c r="D130" t="n">
-        <v>2.2</v>
+        <v>1.73</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>AIROLAM</t>
+          <t>MANGALAM</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>85.13</v>
+        <v>28.3</v>
       </c>
       <c r="C131" t="n">
-        <v>87</v>
+        <v>28.79</v>
       </c>
       <c r="D131" t="n">
-        <v>2.2</v>
+        <v>1.73</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>DIFFNKG</t>
+          <t>ANMOL</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>330.8</v>
+        <v>11.05</v>
       </c>
       <c r="C132" t="n">
-        <v>338</v>
+        <v>11.24</v>
       </c>
       <c r="D132" t="n">
-        <v>2.18</v>
+        <v>1.72</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>IBULLSLTD</t>
+          <t>DIGISPICE</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>24.47</v>
+        <v>20.34</v>
       </c>
       <c r="C133" t="n">
-        <v>25</v>
+        <v>20.69</v>
       </c>
       <c r="D133" t="n">
-        <v>2.17</v>
+        <v>1.72</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>STYL</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>11.6</v>
+        <v>262.45</v>
       </c>
       <c r="C134" t="n">
-        <v>11.85</v>
+        <v>266.9</v>
       </c>
       <c r="D134" t="n">
-        <v>2.16</v>
+        <v>1.7</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>VISAKAIND</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>2.34</v>
+        <v>77.92</v>
       </c>
       <c r="C135" t="n">
-        <v>2.39</v>
+        <v>79.2</v>
       </c>
       <c r="D135" t="n">
-        <v>2.14</v>
+        <v>1.64</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>0.47</v>
+        <v>32.19</v>
       </c>
       <c r="C136" t="n">
-        <v>0.48</v>
+        <v>32.7</v>
       </c>
       <c r="D136" t="n">
-        <v>2.13</v>
+        <v>1.58</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>1.88</v>
+        <v>14.11</v>
       </c>
       <c r="C137" t="n">
-        <v>1.92</v>
+        <v>14.33</v>
       </c>
       <c r="D137" t="n">
-        <v>2.13</v>
+        <v>1.56</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>DOLPHIN</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>391.55</v>
+        <v>3.23</v>
       </c>
       <c r="C138" t="n">
-        <v>399.9</v>
+        <v>3.28</v>
       </c>
       <c r="D138" t="n">
-        <v>2.13</v>
+        <v>1.55</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>KRYSTAL</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>8.02</v>
+        <v>575.1</v>
       </c>
       <c r="C139" t="n">
-        <v>8.19</v>
+        <v>583.9</v>
       </c>
       <c r="D139" t="n">
-        <v>2.12</v>
+        <v>1.53</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>NIRMAN</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>45.25</v>
+        <v>1.97</v>
       </c>
       <c r="C140" t="n">
-        <v>46.2</v>
+        <v>2</v>
       </c>
       <c r="D140" t="n">
-        <v>2.1</v>
+        <v>1.52</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>UNIMECH</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>1149.75</v>
+        <v>24.29</v>
       </c>
       <c r="C141" t="n">
-        <v>1173.95</v>
+        <v>24.66</v>
       </c>
       <c r="D141" t="n">
-        <v>2.1</v>
+        <v>1.52</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>KALYANIFRG</t>
+          <t>ORBTEXP</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>595.5</v>
+        <v>194.96</v>
       </c>
       <c r="C142" t="n">
-        <v>607.95</v>
+        <v>197.9</v>
       </c>
       <c r="D142" t="n">
-        <v>2.09</v>
+        <v>1.51</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>MAHAPEXLTD</t>
+          <t>INDOWIND</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>47.02</v>
+        <v>9.25</v>
       </c>
       <c r="C143" t="n">
-        <v>48</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="D143" t="n">
-        <v>2.08</v>
+        <v>1.51</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>KRIDHANINF</t>
+          <t>ABMINTLLTD</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>2.93</v>
+        <v>42.31</v>
       </c>
       <c r="C144" t="n">
-        <v>2.99</v>
+        <v>42.94</v>
       </c>
       <c r="D144" t="n">
-        <v>2.05</v>
+        <v>1.49</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>BCG</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>10.73</v>
+        <v>3.36</v>
       </c>
       <c r="C145" t="n">
-        <v>10.95</v>
+        <v>3.41</v>
       </c>
       <c r="D145" t="n">
-        <v>2.05</v>
+        <v>1.49</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>HINDCOMPOS</t>
+          <t>SAIPARENT</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>419.4</v>
+        <v>550.65</v>
       </c>
       <c r="C146" t="n">
-        <v>427.95</v>
+        <v>558.85</v>
       </c>
       <c r="D146" t="n">
-        <v>2.04</v>
+        <v>1.49</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>KPL</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>1.47</v>
+        <v>2506.6</v>
       </c>
       <c r="C147" t="n">
-        <v>1.5</v>
+        <v>2544</v>
       </c>
       <c r="D147" t="n">
-        <v>2.04</v>
+        <v>1.49</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>QUICKHEAL</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.49</v>
+        <v>173.04</v>
       </c>
       <c r="C148" t="n">
-        <v>0.5</v>
+        <v>175.6</v>
       </c>
       <c r="D148" t="n">
-        <v>2.04</v>
+        <v>1.48</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>85.65000000000001</v>
+        <v>136.94</v>
       </c>
       <c r="C149" t="n">
-        <v>87.40000000000001</v>
+        <v>138.95</v>
       </c>
       <c r="D149" t="n">
-        <v>2.04</v>
+        <v>1.47</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>GLOBALVECT</t>
+          <t>SIMBHALS</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>161.42</v>
+        <v>6.89</v>
       </c>
       <c r="C150" t="n">
-        <v>164.7</v>
+        <v>6.99</v>
       </c>
       <c r="D150" t="n">
-        <v>2.03</v>
+        <v>1.45</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>IDBI</t>
+          <t>MUKTAARTS</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>75.37</v>
+        <v>60.14</v>
       </c>
       <c r="C151" t="n">
-        <v>76.90000000000001</v>
+        <v>61</v>
       </c>
       <c r="D151" t="n">
-        <v>2.03</v>
+        <v>1.43</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>DBOL</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>109.72</v>
+        <v>178.44</v>
       </c>
       <c r="C152" t="n">
-        <v>111.95</v>
+        <v>181</v>
       </c>
       <c r="D152" t="n">
-        <v>2.03</v>
+        <v>1.43</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>MANCREDIT</t>
+          <t>RENUKA</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>209.07</v>
+        <v>21.84</v>
       </c>
       <c r="C153" t="n">
-        <v>213.29</v>
+        <v>22.15</v>
       </c>
       <c r="D153" t="n">
-        <v>2.02</v>
+        <v>1.42</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>UFO</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>307.8</v>
+        <v>71.98</v>
       </c>
       <c r="C154" t="n">
-        <v>314</v>
+        <v>73</v>
       </c>
       <c r="D154" t="n">
-        <v>2.01</v>
+        <v>1.42</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>93.06</v>
+        <v>137.01</v>
       </c>
       <c r="C155" t="n">
-        <v>94.92</v>
+        <v>138.95</v>
       </c>
       <c r="D155" t="n">
-        <v>2</v>
+        <v>1.42</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>AMDIND</t>
+          <t>BAGFILMS</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>47.2</v>
+        <v>4.97</v>
       </c>
       <c r="C156" t="n">
-        <v>48.14</v>
+        <v>5.04</v>
       </c>
       <c r="D156" t="n">
-        <v>1.99</v>
+        <v>1.41</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>IRMENERGY</t>
+          <t>BAIDFIN</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>256.85</v>
+        <v>10.06</v>
       </c>
       <c r="C157" t="n">
-        <v>261.95</v>
+        <v>10.2</v>
       </c>
       <c r="D157" t="n">
-        <v>1.99</v>
+        <v>1.39</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>REPRO</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>359.85</v>
+        <v>1.45</v>
       </c>
       <c r="C158" t="n">
-        <v>367</v>
+        <v>1.47</v>
       </c>
       <c r="D158" t="n">
-        <v>1.99</v>
+        <v>1.38</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>EQUIPPP</t>
+          <t>RHFL</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>17.15</v>
+        <v>2.18</v>
       </c>
       <c r="C159" t="n">
-        <v>17.49</v>
+        <v>2.21</v>
       </c>
       <c r="D159" t="n">
-        <v>1.98</v>
+        <v>1.38</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ZENITHDRUG</t>
+          <t>MAGNUM</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>42.95</v>
+        <v>19.72</v>
       </c>
       <c r="C160" t="n">
-        <v>43.8</v>
+        <v>19.99</v>
       </c>
       <c r="D160" t="n">
-        <v>1.98</v>
+        <v>1.37</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>UEL</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>132.39</v>
+        <v>3.65</v>
       </c>
       <c r="C161" t="n">
-        <v>135</v>
+        <v>3.7</v>
       </c>
       <c r="D161" t="n">
-        <v>1.97</v>
+        <v>1.37</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>SALSTEEL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>27.01</v>
+        <v>59.21</v>
       </c>
       <c r="C162" t="n">
-        <v>27.54</v>
+        <v>60</v>
       </c>
       <c r="D162" t="n">
-        <v>1.96</v>
+        <v>1.33</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>NECCLTD</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>15.01</v>
+        <v>370.1</v>
       </c>
       <c r="C163" t="n">
-        <v>15.3</v>
+        <v>374.95</v>
       </c>
       <c r="D163" t="n">
-        <v>1.93</v>
+        <v>1.31</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>UNIVASTU</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>29.99</v>
+        <v>78.31</v>
       </c>
       <c r="C164" t="n">
-        <v>30.57</v>
+        <v>79.33</v>
       </c>
       <c r="D164" t="n">
-        <v>1.93</v>
+        <v>1.3</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>TARMAT</t>
+          <t>GOKUL</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>51.94</v>
+        <v>40.94</v>
       </c>
       <c r="C165" t="n">
-        <v>52.94</v>
+        <v>41.47</v>
       </c>
       <c r="D165" t="n">
-        <v>1.93</v>
+        <v>1.29</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>TTKHLTCARE</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>899.35</v>
+        <v>14.86</v>
       </c>
       <c r="C166" t="n">
-        <v>916.7</v>
+        <v>15.05</v>
       </c>
       <c r="D166" t="n">
-        <v>1.93</v>
+        <v>1.28</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>VIRINCHI</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>7.31</v>
+        <v>14.85</v>
       </c>
       <c r="C167" t="n">
-        <v>7.45</v>
+        <v>15.04</v>
       </c>
       <c r="D167" t="n">
-        <v>1.92</v>
+        <v>1.28</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>THEMISMED</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>105.93</v>
+        <v>55.24</v>
       </c>
       <c r="C168" t="n">
-        <v>107.95</v>
+        <v>55.94</v>
       </c>
       <c r="D168" t="n">
-        <v>1.91</v>
+        <v>1.27</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>NILASPACES</t>
+          <t>JAIBALAJI</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>12.06</v>
+        <v>66.05</v>
       </c>
       <c r="C169" t="n">
-        <v>12.29</v>
+        <v>66.89</v>
       </c>
       <c r="D169" t="n">
-        <v>1.91</v>
+        <v>1.27</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>ESSARSHPNG</t>
+          <t>SENORES</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>23.05</v>
+        <v>1112.6</v>
       </c>
       <c r="C170" t="n">
-        <v>23.49</v>
+        <v>1126.2</v>
       </c>
       <c r="D170" t="n">
-        <v>1.91</v>
+        <v>1.22</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>IITL</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>13.15</v>
+        <v>141.34</v>
       </c>
       <c r="C171" t="n">
-        <v>13.4</v>
+        <v>143.05</v>
       </c>
       <c r="D171" t="n">
-        <v>1.9</v>
+        <v>1.21</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>TREL</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>1471</v>
+        <v>25.84</v>
       </c>
       <c r="C172" t="n">
-        <v>1498.8</v>
+        <v>26.15</v>
       </c>
       <c r="D172" t="n">
-        <v>1.89</v>
+        <v>1.2</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>KOKUYOCMLN</t>
+          <t>SANOFICONR</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>83.03</v>
+        <v>4675</v>
       </c>
       <c r="C173" t="n">
-        <v>84.59999999999999</v>
+        <v>4730</v>
       </c>
       <c r="D173" t="n">
-        <v>1.89</v>
+        <v>1.18</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>VALIANTLAB</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>45.12</v>
+        <v>69.18000000000001</v>
       </c>
       <c r="C174" t="n">
-        <v>45.97</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="D174" t="n">
-        <v>1.88</v>
+        <v>1.17</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>AMBALALSA</t>
+          <t>ATALREAL</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>34.06</v>
+        <v>29.65</v>
       </c>
       <c r="C175" t="n">
-        <v>34.7</v>
+        <v>29.99</v>
       </c>
       <c r="D175" t="n">
-        <v>1.88</v>
+        <v>1.15</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>PREMCO</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>369.95</v>
+        <v>178.45</v>
       </c>
       <c r="C176" t="n">
-        <v>376.9</v>
+        <v>180.49</v>
       </c>
       <c r="D176" t="n">
-        <v>1.88</v>
+        <v>1.14</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>RANASUG</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>12.84</v>
+        <v>909.6</v>
       </c>
       <c r="C177" t="n">
-        <v>13.08</v>
+        <v>920</v>
       </c>
       <c r="D177" t="n">
-        <v>1.87</v>
+        <v>1.14</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>KAMDHENU</t>
+          <t>LANDSMILL</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>27.28</v>
+        <v>0.88</v>
       </c>
       <c r="C178" t="n">
-        <v>27.79</v>
+        <v>0.89</v>
       </c>
       <c r="D178" t="n">
-        <v>1.87</v>
+        <v>1.14</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>NOVAAGRI</t>
+          <t>BEEKAY</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>27.78</v>
+        <v>415.3</v>
       </c>
       <c r="C179" t="n">
-        <v>28.3</v>
+        <v>420</v>
       </c>
       <c r="D179" t="n">
-        <v>1.87</v>
+        <v>1.13</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>SUMIT</t>
+          <t>HECPROJECT</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>41.9</v>
+        <v>120.15</v>
       </c>
       <c r="C180" t="n">
-        <v>42.68</v>
+        <v>121.5</v>
       </c>
       <c r="D180" t="n">
-        <v>1.86</v>
+        <v>1.12</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>SPENCERS</t>
+          <t>GFLLIMITED</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>35.57</v>
+        <v>46.38</v>
       </c>
       <c r="C181" t="n">
-        <v>36.23</v>
+        <v>46.9</v>
       </c>
       <c r="D181" t="n">
-        <v>1.86</v>
+        <v>1.12</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>COMSYN</t>
+          <t>DAVANGERE</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>161.89</v>
+        <v>3.56</v>
       </c>
       <c r="C182" t="n">
-        <v>164.9</v>
+        <v>3.6</v>
       </c>
       <c r="D182" t="n">
-        <v>1.86</v>
+        <v>1.12</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>MOTISONS</t>
+          <t>NEPHROPLUS</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>12.03</v>
+        <v>723.15</v>
       </c>
       <c r="C183" t="n">
-        <v>12.25</v>
+        <v>731.25</v>
       </c>
       <c r="D183" t="n">
-        <v>1.83</v>
+        <v>1.12</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>AIRAN</t>
+          <t>OSWALGREEN</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>16.47</v>
+        <v>22.75</v>
       </c>
       <c r="C184" t="n">
-        <v>16.77</v>
+        <v>23</v>
       </c>
       <c r="D184" t="n">
-        <v>1.82</v>
+        <v>1.1</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SHANTIGOLD</t>
+          <t>CARYSIL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>218.36</v>
+        <v>1191.9</v>
       </c>
       <c r="C185" t="n">
-        <v>222.25</v>
+        <v>1205</v>
       </c>
       <c r="D185" t="n">
-        <v>1.78</v>
+        <v>1.1</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>JAYBARMARU</t>
+          <t>MASTERTR</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>138.82</v>
+        <v>75.17</v>
       </c>
       <c r="C186" t="n">
-        <v>141.28</v>
+        <v>75.98999999999999</v>
       </c>
       <c r="D186" t="n">
-        <v>1.77</v>
+        <v>1.09</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>INFLUX</t>
+          <t>CLEANMAX</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>232.9</v>
+        <v>1335.5</v>
       </c>
       <c r="C187" t="n">
-        <v>237</v>
+        <v>1350</v>
       </c>
       <c r="D187" t="n">
-        <v>1.76</v>
+        <v>1.09</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ADVANCE</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>100.49</v>
+        <v>175.09</v>
       </c>
       <c r="C188" t="n">
-        <v>102.25</v>
+        <v>177</v>
       </c>
       <c r="D188" t="n">
-        <v>1.75</v>
+        <v>1.09</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>PRAENG</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>20.63</v>
+        <v>4.65</v>
       </c>
       <c r="C189" t="n">
-        <v>20.99</v>
+        <v>4.7</v>
       </c>
       <c r="D189" t="n">
-        <v>1.75</v>
+        <v>1.08</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>PYRAMID</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>110.07</v>
+        <v>163.27</v>
       </c>
       <c r="C190" t="n">
-        <v>112</v>
+        <v>165</v>
       </c>
       <c r="D190" t="n">
-        <v>1.75</v>
+        <v>1.06</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>RAJSREESUG</t>
+          <t>EXCELINDUS</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>33.4</v>
+        <v>909.1</v>
       </c>
       <c r="C191" t="n">
-        <v>33.97</v>
+        <v>918.5</v>
       </c>
       <c r="D191" t="n">
-        <v>1.71</v>
+        <v>1.03</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>MAGADSUGAR</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>452.25</v>
+        <v>14.73</v>
       </c>
       <c r="C192" t="n">
-        <v>460</v>
+        <v>14.88</v>
       </c>
       <c r="D192" t="n">
-        <v>1.71</v>
+        <v>1.02</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>MENONBE</t>
+          <t>NILAINFRA</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>169.81</v>
+        <v>7.81</v>
       </c>
       <c r="C193" t="n">
-        <v>172.69</v>
+        <v>7.89</v>
       </c>
       <c r="D193" t="n">
-        <v>1.7</v>
+        <v>1.02</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>GRMOVER</t>
+          <t>BALRAMCHIN</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>98.33</v>
+        <v>536.55</v>
       </c>
       <c r="C194" t="n">
-        <v>100</v>
+        <v>542</v>
       </c>
       <c r="D194" t="n">
-        <v>1.7</v>
+        <v>1.02</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>DCAL</t>
+          <t>ARIES</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>187.92</v>
+        <v>326.65</v>
       </c>
       <c r="C195" t="n">
-        <v>191.1</v>
+        <v>329.95</v>
       </c>
       <c r="D195" t="n">
-        <v>1.69</v>
+        <v>1.01</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>LASA</t>
+          <t>VENUSREM</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>7.67</v>
+        <v>1633.5</v>
       </c>
       <c r="C196" t="n">
-        <v>7.8</v>
+        <v>1650</v>
       </c>
       <c r="D196" t="n">
-        <v>1.69</v>
+        <v>1.01</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>KRITIKA</t>
+          <t>RPPINFRA</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>5.98</v>
+        <v>60.15</v>
       </c>
       <c r="C197" t="n">
-        <v>6.08</v>
+        <v>60.75</v>
       </c>
       <c r="D197" t="n">
-        <v>1.67</v>
+        <v>1</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>SMARTLINK</t>
+          <t>INA</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>162.3</v>
+        <v>115.42</v>
       </c>
       <c r="C198" t="n">
-        <v>165</v>
+        <v>116.57</v>
       </c>
       <c r="D198" t="n">
-        <v>1.66</v>
+        <v>1</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>DREAMFOLKS</t>
+          <t>ARIHANT</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>69.65000000000001</v>
+        <v>882.95</v>
       </c>
       <c r="C199" t="n">
-        <v>70.8</v>
+        <v>891.8</v>
       </c>
       <c r="D199" t="n">
-        <v>1.65</v>
+        <v>1</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>4.88</v>
+        <v>71.88</v>
       </c>
       <c r="C200" t="n">
-        <v>4.96</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="D200" t="n">
-        <v>1.64</v>
+        <v>1</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>DONEAR</t>
+          <t>GSPCROP</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>89.44</v>
+        <v>428.95</v>
       </c>
       <c r="C201" t="n">
-        <v>90.90000000000001</v>
+        <v>433.25</v>
       </c>
       <c r="D201" t="n">
-        <v>1.63</v>
+        <v>1</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-12 08:11 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SILLYMONKS</t>
+          <t>WINSOL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18.38</v>
+        <v>125.95</v>
       </c>
       <c r="C3" t="n">
-        <v>19.85</v>
+        <v>138.7</v>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>10.12</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>CURAA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.13</v>
+        <v>77.58</v>
       </c>
       <c r="C4" t="n">
-        <v>2.29</v>
+        <v>85.3</v>
       </c>
       <c r="D4" t="n">
-        <v>7.51</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.81</v>
+        <v>6.94</v>
       </c>
       <c r="C5" t="n">
-        <v>5.17</v>
+        <v>7.58</v>
       </c>
       <c r="D5" t="n">
-        <v>7.48</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>PPAP</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.89</v>
+        <v>244.82</v>
       </c>
       <c r="C6" t="n">
-        <v>2.03</v>
+        <v>263.79</v>
       </c>
       <c r="D6" t="n">
-        <v>7.41</v>
+        <v>7.75</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>MAGNUM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.14</v>
+        <v>19.55</v>
       </c>
       <c r="C7" t="n">
-        <v>0.15</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
-        <v>7.14</v>
+        <v>7.42</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>22.34</v>
+        <v>1531</v>
       </c>
       <c r="C8" t="n">
-        <v>23.8</v>
+        <v>1644</v>
       </c>
       <c r="D8" t="n">
-        <v>6.54</v>
+        <v>7.38</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>K2INFRA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>48.64</v>
+        <v>48.95</v>
       </c>
       <c r="C9" t="n">
-        <v>51.79</v>
+        <v>52.5</v>
       </c>
       <c r="D9" t="n">
-        <v>6.48</v>
+        <v>7.25</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SECMARK</t>
+          <t>KOTYARK</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>127.71</v>
+        <v>402.6</v>
       </c>
       <c r="C10" t="n">
-        <v>135.45</v>
+        <v>430</v>
       </c>
       <c r="D10" t="n">
-        <v>6.06</v>
+        <v>6.81</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>23</v>
+        <v>14.61</v>
       </c>
       <c r="C11" t="n">
-        <v>24.33</v>
+        <v>15.6</v>
       </c>
       <c r="D11" t="n">
-        <v>5.78</v>
+        <v>6.78</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>HALDER</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.19</v>
+        <v>240.68</v>
       </c>
       <c r="C12" t="n">
-        <v>0.2</v>
+        <v>257</v>
       </c>
       <c r="D12" t="n">
-        <v>5.26</v>
+        <v>6.78</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8.19</v>
+        <v>0.15</v>
       </c>
       <c r="C13" t="n">
-        <v>8.6</v>
+        <v>0.16</v>
       </c>
       <c r="D13" t="n">
-        <v>5.01</v>
+        <v>6.67</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LASA</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7.6</v>
+        <v>4.97</v>
       </c>
       <c r="C14" t="n">
-        <v>7.98</v>
+        <v>5.3</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>6.64</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GJL</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>138.1</v>
+        <v>69.53</v>
       </c>
       <c r="C15" t="n">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>6.43</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>KDL</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>114.2</v>
+        <v>0.79</v>
       </c>
       <c r="C16" t="n">
-        <v>119.9</v>
+        <v>0.84</v>
       </c>
       <c r="D16" t="n">
-        <v>4.99</v>
+        <v>6.33</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>UHTL</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>94.09999999999999</v>
+        <v>243</v>
       </c>
       <c r="C17" t="n">
-        <v>98.8</v>
+        <v>258</v>
       </c>
       <c r="D17" t="n">
-        <v>4.99</v>
+        <v>6.17</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VASCONEQ</t>
+          <t>MTARTECH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>33.08</v>
+        <v>6306</v>
       </c>
       <c r="C18" t="n">
-        <v>34.73</v>
+        <v>6666.5</v>
       </c>
       <c r="D18" t="n">
-        <v>4.99</v>
+        <v>5.72</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TIJARIA</t>
+          <t>VISHWARAJ</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4.43</v>
+        <v>5.46</v>
       </c>
       <c r="C19" t="n">
-        <v>4.65</v>
+        <v>5.76</v>
       </c>
       <c r="D19" t="n">
-        <v>4.97</v>
+        <v>5.49</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SHEEL</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>54.45</v>
+        <v>27.1</v>
       </c>
       <c r="C20" t="n">
-        <v>57.15</v>
+        <v>28.58</v>
       </c>
       <c r="D20" t="n">
-        <v>4.96</v>
+        <v>5.46</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>PARASPETRO</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6.86</v>
+        <v>1.88</v>
       </c>
       <c r="C21" t="n">
-        <v>7.2</v>
+        <v>1.98</v>
       </c>
       <c r="D21" t="n">
-        <v>4.96</v>
+        <v>5.32</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>9.75</v>
+        <v>6.4</v>
       </c>
       <c r="C22" t="n">
-        <v>10.23</v>
+        <v>6.74</v>
       </c>
       <c r="D22" t="n">
-        <v>4.92</v>
+        <v>5.31</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PPAP</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>205.76</v>
+        <v>0.19</v>
       </c>
       <c r="C23" t="n">
-        <v>215.85</v>
+        <v>0.2</v>
       </c>
       <c r="D23" t="n">
-        <v>4.9</v>
+        <v>5.26</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CEREBRAINT</t>
+          <t>GICL</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.67</v>
+        <v>22.06</v>
       </c>
       <c r="C24" t="n">
-        <v>3.85</v>
+        <v>23.2</v>
       </c>
       <c r="D24" t="n">
-        <v>4.9</v>
+        <v>5.17</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>QVCEL</t>
+          <t>SHRIKRISH</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>23.5</v>
+        <v>42.82</v>
       </c>
       <c r="C25" t="n">
-        <v>24.65</v>
+        <v>45</v>
       </c>
       <c r="D25" t="n">
-        <v>4.89</v>
+        <v>5.09</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RACE</t>
+          <t>LASA</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>110</v>
+        <v>7.18</v>
       </c>
       <c r="C26" t="n">
-        <v>115.2</v>
+        <v>7.54</v>
       </c>
       <c r="D26" t="n">
-        <v>4.73</v>
+        <v>5.01</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2.55</v>
+        <v>39.8</v>
       </c>
       <c r="C27" t="n">
-        <v>2.67</v>
+        <v>41.79</v>
       </c>
       <c r="D27" t="n">
-        <v>4.71</v>
+        <v>5</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FMNL</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>10.01</v>
+        <v>10.23</v>
       </c>
       <c r="C28" t="n">
-        <v>10.48</v>
+        <v>10.74</v>
       </c>
       <c r="D28" t="n">
-        <v>4.7</v>
+        <v>4.99</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>WIPL</t>
+          <t>SHEEL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>148</v>
+        <v>57.15</v>
       </c>
       <c r="C29" t="n">
-        <v>154.9</v>
+        <v>60</v>
       </c>
       <c r="D29" t="n">
-        <v>4.66</v>
+        <v>4.99</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NOIDATOLL</t>
+          <t>INNOMET</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4.75</v>
+        <v>100.5</v>
       </c>
       <c r="C30" t="n">
-        <v>4.97</v>
+        <v>105.5</v>
       </c>
       <c r="D30" t="n">
-        <v>4.63</v>
+        <v>4.98</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NECCLTD</t>
+          <t>TCIFINANCE</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>18.01</v>
+        <v>25.3</v>
       </c>
       <c r="C31" t="n">
-        <v>18.84</v>
+        <v>26.56</v>
       </c>
       <c r="D31" t="n">
-        <v>4.61</v>
+        <v>4.98</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.22</v>
+        <v>98.8</v>
       </c>
       <c r="C32" t="n">
-        <v>0.23</v>
+        <v>103.7</v>
       </c>
       <c r="D32" t="n">
-        <v>4.55</v>
+        <v>4.96</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CUDML</t>
+          <t>KDL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>182.7</v>
+        <v>119.9</v>
       </c>
       <c r="C33" t="n">
-        <v>191</v>
+        <v>125.85</v>
       </c>
       <c r="D33" t="n">
-        <v>4.54</v>
+        <v>4.96</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SUPREMEENG</t>
+          <t>SSFL</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.13</v>
+        <v>218</v>
       </c>
       <c r="C34" t="n">
-        <v>1.18</v>
+        <v>228.8</v>
       </c>
       <c r="D34" t="n">
-        <v>4.42</v>
+        <v>4.95</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>GLFL</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>315.2</v>
+        <v>6.32</v>
       </c>
       <c r="C35" t="n">
-        <v>329</v>
+        <v>6.63</v>
       </c>
       <c r="D35" t="n">
-        <v>4.38</v>
+        <v>4.91</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PRIZOR</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>826.75</v>
+        <v>14.52</v>
       </c>
       <c r="C36" t="n">
-        <v>862.5</v>
+        <v>15.22</v>
       </c>
       <c r="D36" t="n">
-        <v>4.32</v>
+        <v>4.82</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>UNICHEMLAB</t>
+          <t>INDOUS</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>437.4</v>
+        <v>90.56999999999999</v>
       </c>
       <c r="C37" t="n">
-        <v>456</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="D37" t="n">
-        <v>4.25</v>
+        <v>4.78</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HDIL</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1.89</v>
+        <v>3.59</v>
       </c>
       <c r="C38" t="n">
-        <v>1.97</v>
+        <v>3.76</v>
       </c>
       <c r="D38" t="n">
-        <v>4.23</v>
+        <v>4.74</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>RADAAN</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3.07</v>
+        <v>43.37</v>
       </c>
       <c r="C39" t="n">
-        <v>3.2</v>
+        <v>45.4</v>
       </c>
       <c r="D39" t="n">
-        <v>4.23</v>
+        <v>4.68</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SADBHAV</t>
+          <t>TGL</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>9.4</v>
+        <v>20.4</v>
       </c>
       <c r="C40" t="n">
-        <v>9.789999999999999</v>
+        <v>21.35</v>
       </c>
       <c r="D40" t="n">
-        <v>4.15</v>
+        <v>4.66</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>TRIDHYA</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4.71</v>
+        <v>9.65</v>
       </c>
       <c r="C41" t="n">
-        <v>4.9</v>
+        <v>10.1</v>
       </c>
       <c r="D41" t="n">
-        <v>4.03</v>
+        <v>4.66</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>INTENTECH</t>
+          <t>NORBTEAEXP</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>102.63</v>
+        <v>74.06</v>
       </c>
       <c r="C42" t="n">
-        <v>106.76</v>
+        <v>77.5</v>
       </c>
       <c r="D42" t="n">
-        <v>4.02</v>
+        <v>4.64</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>BILVYAPAR</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>414.6</v>
+        <v>3.92</v>
       </c>
       <c r="C43" t="n">
-        <v>431.25</v>
+        <v>4.1</v>
       </c>
       <c r="D43" t="n">
-        <v>4.02</v>
+        <v>4.59</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>HOLMARC</t>
+          <t>RPPL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>106.7</v>
+        <v>17.79</v>
       </c>
       <c r="C44" t="n">
-        <v>110.9</v>
+        <v>18.6</v>
       </c>
       <c r="D44" t="n">
-        <v>3.94</v>
+        <v>4.55</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SUDARSCHEM</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>854.05</v>
+        <v>0.22</v>
       </c>
       <c r="C45" t="n">
-        <v>887.7</v>
+        <v>0.23</v>
       </c>
       <c r="D45" t="n">
-        <v>3.94</v>
+        <v>4.55</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>PILITA</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>21.15</v>
+        <v>7.98</v>
       </c>
       <c r="C46" t="n">
-        <v>21.98</v>
+        <v>8.34</v>
       </c>
       <c r="D46" t="n">
-        <v>3.92</v>
+        <v>4.51</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>HINDWAREAP</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2.3</v>
+        <v>213.01</v>
       </c>
       <c r="C47" t="n">
-        <v>2.39</v>
+        <v>222.59</v>
       </c>
       <c r="D47" t="n">
-        <v>3.91</v>
+        <v>4.5</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>SHUBHLAXMI</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>7</v>
+        <v>25.8</v>
       </c>
       <c r="C48" t="n">
-        <v>7.25</v>
+        <v>26.95</v>
       </c>
       <c r="D48" t="n">
-        <v>3.57</v>
+        <v>4.46</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SILKFLEX</t>
+          <t>SAHANA</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>209.45</v>
+        <v>713.85</v>
       </c>
       <c r="C49" t="n">
-        <v>216.9</v>
+        <v>745</v>
       </c>
       <c r="D49" t="n">
-        <v>3.56</v>
+        <v>4.36</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MODIRUBBER</t>
+          <t>CREATIVEYE</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>126.63</v>
+        <v>6.43</v>
       </c>
       <c r="C50" t="n">
-        <v>131.1</v>
+        <v>6.7</v>
       </c>
       <c r="D50" t="n">
-        <v>3.53</v>
+        <v>4.2</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>FINKURVE</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>64.36</v>
+        <v>10.08</v>
       </c>
       <c r="C51" t="n">
-        <v>66.59999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="D51" t="n">
-        <v>3.48</v>
+        <v>4.17</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>3IINFOLTD</t>
+          <t>SAMBHAAV</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>16.43</v>
+        <v>6.24</v>
       </c>
       <c r="C52" t="n">
-        <v>17</v>
+        <v>6.5</v>
       </c>
       <c r="D52" t="n">
-        <v>3.47</v>
+        <v>4.17</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>GANESHIN</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>44.17</v>
+        <v>89.3</v>
       </c>
       <c r="C53" t="n">
-        <v>45.7</v>
+        <v>93</v>
       </c>
       <c r="D53" t="n">
-        <v>3.46</v>
+        <v>4.14</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MAHAPEXLTD</t>
+          <t>PASHUPATI</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>48.8</v>
+        <v>87.88</v>
       </c>
       <c r="C54" t="n">
-        <v>50.48</v>
+        <v>91.5</v>
       </c>
       <c r="D54" t="n">
-        <v>3.44</v>
+        <v>4.12</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ANTELOPUS</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>818.8</v>
+        <v>4.71</v>
       </c>
       <c r="C55" t="n">
-        <v>846.95</v>
+        <v>4.9</v>
       </c>
       <c r="D55" t="n">
-        <v>3.44</v>
+        <v>4.03</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DBSTOCKBRO</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>31.42</v>
+        <v>20</v>
       </c>
       <c r="C56" t="n">
-        <v>32.49</v>
+        <v>20.8</v>
       </c>
       <c r="D56" t="n">
-        <v>3.41</v>
+        <v>4</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MFML</t>
+          <t>HCL-INSYS</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>23.8</v>
+        <v>11.75</v>
       </c>
       <c r="C57" t="n">
-        <v>24.59</v>
+        <v>12.22</v>
       </c>
       <c r="D57" t="n">
-        <v>3.32</v>
+        <v>4</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>HEADSUP</t>
+          <t>EPACKPEB</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>7.01</v>
+        <v>227.27</v>
       </c>
       <c r="C58" t="n">
-        <v>7.24</v>
+        <v>236.28</v>
       </c>
       <c r="D58" t="n">
-        <v>3.28</v>
+        <v>3.96</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ANIKINDS</t>
+          <t>OSWALAGRO</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>42.56</v>
+        <v>42.53</v>
       </c>
       <c r="C59" t="n">
-        <v>43.95</v>
+        <v>44.18</v>
       </c>
       <c r="D59" t="n">
-        <v>3.27</v>
+        <v>3.88</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>28.32</v>
+        <v>7.21</v>
       </c>
       <c r="C60" t="n">
-        <v>29.24</v>
+        <v>7.49</v>
       </c>
       <c r="D60" t="n">
-        <v>3.25</v>
+        <v>3.88</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MANAKALUCO</t>
+          <t>CKKRETAIL</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>41.21</v>
+        <v>140</v>
       </c>
       <c r="C61" t="n">
-        <v>42.54</v>
+        <v>145.4</v>
       </c>
       <c r="D61" t="n">
-        <v>3.23</v>
+        <v>3.86</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SURYALAXMI</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>56.01</v>
+        <v>163.68</v>
       </c>
       <c r="C62" t="n">
-        <v>57.8</v>
+        <v>170</v>
       </c>
       <c r="D62" t="n">
-        <v>3.2</v>
+        <v>3.86</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>NILASPACES</t>
+          <t>DREDGECORP</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>11.9</v>
+        <v>1040.3</v>
       </c>
       <c r="C63" t="n">
-        <v>12.28</v>
+        <v>1080</v>
       </c>
       <c r="D63" t="n">
-        <v>3.19</v>
+        <v>3.82</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>PLAZACABLE</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>11.99</v>
+        <v>46.22</v>
       </c>
       <c r="C64" t="n">
-        <v>12.36</v>
+        <v>47.98</v>
       </c>
       <c r="D64" t="n">
-        <v>3.09</v>
+        <v>3.81</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PASHUPATI</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>87.90000000000001</v>
+        <v>5.89</v>
       </c>
       <c r="C65" t="n">
-        <v>90.59999999999999</v>
+        <v>6.11</v>
       </c>
       <c r="D65" t="n">
-        <v>3.07</v>
+        <v>3.74</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>NARMADA</t>
+          <t>INDOTHAI</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>43.56</v>
+        <v>235.7</v>
       </c>
       <c r="C66" t="n">
-        <v>44.89</v>
+        <v>244.5</v>
       </c>
       <c r="D66" t="n">
-        <v>3.05</v>
+        <v>3.73</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CNL</t>
+          <t>OMNI</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>693.95</v>
+        <v>453</v>
       </c>
       <c r="C67" t="n">
-        <v>715</v>
+        <v>469.8</v>
       </c>
       <c r="D67" t="n">
-        <v>3.03</v>
+        <v>3.71</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>DCMSRIND</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>13.58</v>
+        <v>37.61</v>
       </c>
       <c r="C68" t="n">
-        <v>13.99</v>
+        <v>39</v>
       </c>
       <c r="D68" t="n">
-        <v>3.02</v>
+        <v>3.7</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GOLDTECH</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>41.72</v>
+        <v>21.22</v>
       </c>
       <c r="C69" t="n">
-        <v>42.98</v>
+        <v>22</v>
       </c>
       <c r="D69" t="n">
-        <v>3.02</v>
+        <v>3.68</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>UNITEDTEA</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>21.75</v>
+        <v>510.2</v>
       </c>
       <c r="C70" t="n">
-        <v>22.39</v>
+        <v>529</v>
       </c>
       <c r="D70" t="n">
-        <v>2.94</v>
+        <v>3.68</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>NITIRAJ</t>
+          <t>HAPPSTMNDS</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>184.63</v>
+        <v>345</v>
       </c>
       <c r="C71" t="n">
-        <v>190</v>
+        <v>357.55</v>
       </c>
       <c r="D71" t="n">
-        <v>2.91</v>
+        <v>3.64</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>UNITEDPOLY</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>37.91</v>
+        <v>33.29</v>
       </c>
       <c r="C72" t="n">
-        <v>39</v>
+        <v>34.5</v>
       </c>
       <c r="D72" t="n">
-        <v>2.88</v>
+        <v>3.63</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>48.12</v>
+        <v>74.3</v>
       </c>
       <c r="C73" t="n">
-        <v>49.5</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="D73" t="n">
-        <v>2.87</v>
+        <v>3.62</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>NOIDATOLL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.36</v>
+        <v>4.98</v>
       </c>
       <c r="C74" t="n">
-        <v>0.37</v>
+        <v>5.16</v>
       </c>
       <c r="D74" t="n">
-        <v>2.78</v>
+        <v>3.61</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>TNTELE</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>9.050000000000001</v>
+        <v>13.51</v>
       </c>
       <c r="C75" t="n">
-        <v>9.300000000000001</v>
+        <v>13.99</v>
       </c>
       <c r="D75" t="n">
-        <v>2.76</v>
+        <v>3.55</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>BANARBEADS</t>
+          <t>TARAPUR</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>98.3</v>
+        <v>18.34</v>
       </c>
       <c r="C76" t="n">
-        <v>101</v>
+        <v>18.99</v>
       </c>
       <c r="D76" t="n">
-        <v>2.75</v>
+        <v>3.54</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>HEXT</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>8.75</v>
+        <v>502.25</v>
       </c>
       <c r="C77" t="n">
-        <v>8.99</v>
+        <v>520</v>
       </c>
       <c r="D77" t="n">
-        <v>2.74</v>
+        <v>3.53</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>EXIMROUTES</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>174.72</v>
+        <v>100.45</v>
       </c>
       <c r="C78" t="n">
-        <v>179.49</v>
+        <v>104</v>
       </c>
       <c r="D78" t="n">
-        <v>2.73</v>
+        <v>3.53</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>OMINFRAL</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>13.61</v>
+        <v>80.44</v>
       </c>
       <c r="C79" t="n">
-        <v>13.98</v>
+        <v>83.28</v>
       </c>
       <c r="D79" t="n">
-        <v>2.72</v>
+        <v>3.53</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SHRENIK</t>
+          <t>CENTENKA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.37</v>
+        <v>489.85</v>
       </c>
       <c r="C80" t="n">
-        <v>0.38</v>
+        <v>507.15</v>
       </c>
       <c r="D80" t="n">
-        <v>2.7</v>
+        <v>3.53</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ASTRON</t>
+          <t>BCG</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>3.86</v>
+        <v>10.23</v>
       </c>
       <c r="C81" t="n">
-        <v>3.96</v>
+        <v>10.59</v>
       </c>
       <c r="D81" t="n">
-        <v>2.59</v>
+        <v>3.52</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>378.15</v>
+        <v>23.57</v>
       </c>
       <c r="C82" t="n">
-        <v>387.95</v>
+        <v>24.4</v>
       </c>
       <c r="D82" t="n">
-        <v>2.59</v>
+        <v>3.52</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>MENNPIS</t>
+          <t>BATLIBOI</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>55.34</v>
+        <v>74.48</v>
       </c>
       <c r="C83" t="n">
-        <v>56.75</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="D83" t="n">
-        <v>2.55</v>
+        <v>3.52</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MAGADSUGAR</t>
+          <t>FIBERWEB</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>448.1</v>
+        <v>27.53</v>
       </c>
       <c r="C84" t="n">
-        <v>459.5</v>
+        <v>28.5</v>
       </c>
       <c r="D84" t="n">
-        <v>2.54</v>
+        <v>3.52</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>NORBTEAEXP</t>
+          <t>KRIDHANINF</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>76.7</v>
+        <v>2.85</v>
       </c>
       <c r="C85" t="n">
-        <v>78.59999999999999</v>
+        <v>2.95</v>
       </c>
       <c r="D85" t="n">
-        <v>2.48</v>
+        <v>3.51</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>DJML</t>
+          <t>IRIS</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>109.32</v>
+        <v>223.65</v>
       </c>
       <c r="C86" t="n">
-        <v>112</v>
+        <v>231.5</v>
       </c>
       <c r="D86" t="n">
-        <v>2.45</v>
+        <v>3.51</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>GROBTEA</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>926.4</v>
+        <v>1323.8</v>
       </c>
       <c r="C87" t="n">
-        <v>949</v>
+        <v>1370.1</v>
       </c>
       <c r="D87" t="n">
-        <v>2.44</v>
+        <v>3.5</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>AVROIND</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>79.43000000000001</v>
+        <v>10.58</v>
       </c>
       <c r="C88" t="n">
-        <v>81.37</v>
+        <v>10.95</v>
       </c>
       <c r="D88" t="n">
-        <v>2.44</v>
+        <v>3.5</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>SILLYMONKS</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>27.44</v>
+        <v>18.34</v>
       </c>
       <c r="C89" t="n">
-        <v>28.1</v>
+        <v>18.98</v>
       </c>
       <c r="D89" t="n">
-        <v>2.41</v>
+        <v>3.49</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>EQUIPPP</t>
+          <t>SUDARCOLOR</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>17.19</v>
+        <v>356.95</v>
       </c>
       <c r="C90" t="n">
-        <v>17.6</v>
+        <v>369.4</v>
       </c>
       <c r="D90" t="n">
-        <v>2.39</v>
+        <v>3.49</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.42</v>
+        <v>71.12</v>
       </c>
       <c r="C91" t="n">
-        <v>0.43</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="D91" t="n">
-        <v>2.38</v>
+        <v>3.49</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>EMAMIPAP</t>
+          <t>SOUTHWEST</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>85.01000000000001</v>
+        <v>240.15</v>
       </c>
       <c r="C92" t="n">
-        <v>87</v>
+        <v>248.5</v>
       </c>
       <c r="D92" t="n">
-        <v>2.34</v>
+        <v>3.48</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>IGCL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>39.54</v>
+        <v>55.85</v>
       </c>
       <c r="C93" t="n">
-        <v>40.45</v>
+        <v>57.79</v>
       </c>
       <c r="D93" t="n">
-        <v>2.3</v>
+        <v>3.47</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>MVGJL</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>7.92</v>
+        <v>143.91</v>
       </c>
       <c r="C94" t="n">
-        <v>8.1</v>
+        <v>148.9</v>
       </c>
       <c r="D94" t="n">
-        <v>2.27</v>
+        <v>3.47</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>KCPSUGIND</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>22.88</v>
+        <v>357.65</v>
       </c>
       <c r="C95" t="n">
-        <v>23.39</v>
+        <v>369.95</v>
       </c>
       <c r="D95" t="n">
-        <v>2.23</v>
+        <v>3.44</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>DIGIDRIVE</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0.45</v>
+        <v>17.89</v>
       </c>
       <c r="C96" t="n">
-        <v>0.46</v>
+        <v>18.5</v>
       </c>
       <c r="D96" t="n">
-        <v>2.22</v>
+        <v>3.41</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LAHOTIOV</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>44.91</v>
+        <v>34.33</v>
       </c>
       <c r="C97" t="n">
-        <v>45.9</v>
+        <v>35.5</v>
       </c>
       <c r="D97" t="n">
-        <v>2.2</v>
+        <v>3.41</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>FIBERWEB</t>
+          <t>SHIVATEX</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>27.99</v>
+        <v>147.86</v>
       </c>
       <c r="C98" t="n">
-        <v>28.6</v>
+        <v>152.9</v>
       </c>
       <c r="D98" t="n">
-        <v>2.18</v>
+        <v>3.41</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>IVC</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>2.29</v>
+        <v>8.27</v>
       </c>
       <c r="C99" t="n">
-        <v>2.34</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="D99" t="n">
-        <v>2.18</v>
+        <v>3.39</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SELMC</t>
+          <t>CROWN</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>29.85</v>
+        <v>108.3</v>
       </c>
       <c r="C100" t="n">
-        <v>30.5</v>
+        <v>111.96</v>
       </c>
       <c r="D100" t="n">
-        <v>2.18</v>
+        <v>3.38</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PRITI</t>
+          <t>FOODSIN</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>39.06</v>
+        <v>53.93</v>
       </c>
       <c r="C101" t="n">
-        <v>39.9</v>
+        <v>55.75</v>
       </c>
       <c r="D101" t="n">
-        <v>2.15</v>
+        <v>3.37</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SAWALIYA</t>
+          <t>LOTUSDEV</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>282.75</v>
+        <v>129.27</v>
       </c>
       <c r="C102" t="n">
-        <v>288.8</v>
+        <v>133.62</v>
       </c>
       <c r="D102" t="n">
-        <v>2.14</v>
+        <v>3.37</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>KOTHARIPRO</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>7.06</v>
+        <v>68.5</v>
       </c>
       <c r="C103" t="n">
-        <v>7.21</v>
+        <v>70.8</v>
       </c>
       <c r="D103" t="n">
-        <v>2.12</v>
+        <v>3.36</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>TECHERA</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>136.7</v>
+        <v>47.02</v>
       </c>
       <c r="C104" t="n">
-        <v>139.6</v>
+        <v>48.6</v>
       </c>
       <c r="D104" t="n">
-        <v>2.12</v>
+        <v>3.36</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>VELJAN</t>
+          <t>HINDCOMPOS</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>1282.8</v>
+        <v>402.5</v>
       </c>
       <c r="C105" t="n">
-        <v>1310</v>
+        <v>416</v>
       </c>
       <c r="D105" t="n">
-        <v>2.12</v>
+        <v>3.35</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>SAKUMA</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>1.91</v>
+        <v>6.87</v>
       </c>
       <c r="C106" t="n">
-        <v>1.95</v>
+        <v>7.1</v>
       </c>
       <c r="D106" t="n">
-        <v>2.09</v>
+        <v>3.35</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SCANSTL</t>
+          <t>ASHOKLEY</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>34.97</v>
+        <v>138.58</v>
       </c>
       <c r="C107" t="n">
-        <v>35.7</v>
+        <v>143.22</v>
       </c>
       <c r="D107" t="n">
-        <v>2.09</v>
+        <v>3.35</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CORALFINAC</t>
+          <t>HISARMETAL</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>31.5</v>
+        <v>152.91</v>
       </c>
       <c r="C108" t="n">
-        <v>32.15</v>
+        <v>158</v>
       </c>
       <c r="D108" t="n">
-        <v>2.06</v>
+        <v>3.33</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MANOMAY</t>
+          <t>HCC</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>195.73</v>
+        <v>21.68</v>
       </c>
       <c r="C109" t="n">
-        <v>199.7</v>
+        <v>22.4</v>
       </c>
       <c r="D109" t="n">
-        <v>2.03</v>
+        <v>3.32</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SRTL</t>
+          <t>BETA</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>41.35</v>
+        <v>1476</v>
       </c>
       <c r="C110" t="n">
-        <v>42.19</v>
+        <v>1525</v>
       </c>
       <c r="D110" t="n">
-        <v>2.03</v>
+        <v>3.32</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>KODYTECH</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>13.43</v>
+        <v>904.2</v>
       </c>
       <c r="C111" t="n">
-        <v>13.7</v>
+        <v>934</v>
       </c>
       <c r="D111" t="n">
-        <v>2.01</v>
+        <v>3.3</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>BAFNAPH</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>0.5</v>
+        <v>174.15</v>
       </c>
       <c r="C112" t="n">
-        <v>0.51</v>
+        <v>179.9</v>
       </c>
       <c r="D112" t="n">
-        <v>2</v>
+        <v>3.3</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MAWANASUG</t>
+          <t>AEGISLOG</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>101.97</v>
+        <v>925.9</v>
       </c>
       <c r="C113" t="n">
-        <v>104</v>
+        <v>956.35</v>
       </c>
       <c r="D113" t="n">
-        <v>1.99</v>
+        <v>3.29</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>VASWANI</t>
+          <t>LEMERITE</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>59.52</v>
+        <v>24.92</v>
       </c>
       <c r="C114" t="n">
-        <v>60.7</v>
+        <v>25.74</v>
       </c>
       <c r="D114" t="n">
-        <v>1.98</v>
+        <v>3.29</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>KHANDSE</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>1.02</v>
+        <v>18.01</v>
       </c>
       <c r="C115" t="n">
-        <v>1.04</v>
+        <v>18.6</v>
       </c>
       <c r="D115" t="n">
-        <v>1.96</v>
+        <v>3.28</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>RSSOFTWARE</t>
+          <t>HINDPETRO</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>31.84</v>
+        <v>365.7</v>
       </c>
       <c r="C116" t="n">
-        <v>32.45</v>
+        <v>377.7</v>
       </c>
       <c r="D116" t="n">
-        <v>1.92</v>
+        <v>3.28</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SREEL</t>
+          <t>PRAENG</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>197.16</v>
+        <v>20.24</v>
       </c>
       <c r="C117" t="n">
-        <v>200.9</v>
+        <v>20.9</v>
       </c>
       <c r="D117" t="n">
-        <v>1.9</v>
+        <v>3.26</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ADVANCE</t>
+          <t>ANURAS</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>99.09999999999999</v>
+        <v>1258</v>
       </c>
       <c r="C118" t="n">
-        <v>100.98</v>
+        <v>1299</v>
       </c>
       <c r="D118" t="n">
-        <v>1.9</v>
+        <v>3.26</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ODIGMA</t>
+          <t>CENTRUM</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>20.5</v>
+        <v>21.5</v>
       </c>
       <c r="C119" t="n">
-        <v>20.89</v>
+        <v>22.2</v>
       </c>
       <c r="D119" t="n">
-        <v>1.9</v>
+        <v>3.26</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>EBGNG</t>
+          <t>MOTISONS</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>392.6</v>
+        <v>13.22</v>
       </c>
       <c r="C120" t="n">
-        <v>400</v>
+        <v>13.65</v>
       </c>
       <c r="D120" t="n">
-        <v>1.88</v>
+        <v>3.25</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>VLSFINANCE</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>228</v>
+        <v>251.65</v>
       </c>
       <c r="C121" t="n">
-        <v>232.24</v>
+        <v>259.8</v>
       </c>
       <c r="D121" t="n">
-        <v>1.86</v>
+        <v>3.24</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SHIVATEX</t>
+          <t>MMP</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>151.5</v>
+        <v>251.75</v>
       </c>
       <c r="C122" t="n">
-        <v>154.3</v>
+        <v>259.9</v>
       </c>
       <c r="D122" t="n">
-        <v>1.85</v>
+        <v>3.24</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>UEL</t>
+          <t>MAJESAUT</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>143.21</v>
+        <v>334</v>
       </c>
       <c r="C123" t="n">
-        <v>145.79</v>
+        <v>344.8</v>
       </c>
       <c r="D123" t="n">
-        <v>1.8</v>
+        <v>3.23</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>NAHARPOLY</t>
+          <t>EBGNG</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>239.7</v>
+        <v>418.55</v>
       </c>
       <c r="C124" t="n">
-        <v>244</v>
+        <v>432</v>
       </c>
       <c r="D124" t="n">
-        <v>1.79</v>
+        <v>3.21</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>RMDRIP</t>
+          <t>EVERESTIND</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>16.85</v>
+        <v>331.4</v>
       </c>
       <c r="C125" t="n">
-        <v>17.15</v>
+        <v>342</v>
       </c>
       <c r="D125" t="n">
-        <v>1.78</v>
+        <v>3.2</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>KAMOPAINTS</t>
+          <t>CYIENT</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>5.09</v>
+        <v>846.65</v>
       </c>
       <c r="C126" t="n">
-        <v>5.18</v>
+        <v>873.7</v>
       </c>
       <c r="D126" t="n">
-        <v>1.77</v>
+        <v>3.19</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SURYODAY</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>170</v>
+        <v>23.65</v>
       </c>
       <c r="C127" t="n">
-        <v>173</v>
+        <v>24.4</v>
       </c>
       <c r="D127" t="n">
-        <v>1.76</v>
+        <v>3.17</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IFBAGRO</t>
+          <t>AARVI</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>929.5</v>
+        <v>142.31</v>
       </c>
       <c r="C128" t="n">
-        <v>945.9</v>
+        <v>146.8</v>
       </c>
       <c r="D128" t="n">
-        <v>1.76</v>
+        <v>3.16</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MGEL</t>
+          <t>MANGALAM</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>16.51</v>
+        <v>27.91</v>
       </c>
       <c r="C129" t="n">
-        <v>16.8</v>
+        <v>28.79</v>
       </c>
       <c r="D129" t="n">
-        <v>1.76</v>
+        <v>3.15</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>TRIGYN</t>
+          <t>PRAVEG</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>54.93</v>
+        <v>212.35</v>
       </c>
       <c r="C130" t="n">
-        <v>55.88</v>
+        <v>219</v>
       </c>
       <c r="D130" t="n">
-        <v>1.73</v>
+        <v>3.13</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MANGALAM</t>
+          <t>BESTAGRO</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>28.3</v>
+        <v>15.33</v>
       </c>
       <c r="C131" t="n">
-        <v>28.79</v>
+        <v>15.81</v>
       </c>
       <c r="D131" t="n">
-        <v>1.73</v>
+        <v>3.13</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ANMOL</t>
+          <t>PARACABLES</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>11.05</v>
+        <v>60.85</v>
       </c>
       <c r="C132" t="n">
-        <v>11.24</v>
+        <v>62.75</v>
       </c>
       <c r="D132" t="n">
-        <v>1.72</v>
+        <v>3.12</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>DIGISPICE</t>
+          <t>TARMAT</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>20.34</v>
+        <v>51.84</v>
       </c>
       <c r="C133" t="n">
-        <v>20.69</v>
+        <v>53.45</v>
       </c>
       <c r="D133" t="n">
-        <v>1.72</v>
+        <v>3.11</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>STYL</t>
+          <t>FCL</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>262.45</v>
+        <v>37.03</v>
       </c>
       <c r="C134" t="n">
-        <v>266.9</v>
+        <v>38.18</v>
       </c>
       <c r="D134" t="n">
-        <v>1.7</v>
+        <v>3.11</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>VISAKAIND</t>
+          <t>TIJARIA</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>77.92</v>
+        <v>4.52</v>
       </c>
       <c r="C135" t="n">
-        <v>79.2</v>
+        <v>4.66</v>
       </c>
       <c r="D135" t="n">
-        <v>1.64</v>
+        <v>3.1</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>32.19</v>
+        <v>0.97</v>
       </c>
       <c r="C136" t="n">
-        <v>32.7</v>
+        <v>1</v>
       </c>
       <c r="D136" t="n">
-        <v>1.58</v>
+        <v>3.09</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>GABRIEL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>14.11</v>
+        <v>1008.8</v>
       </c>
       <c r="C137" t="n">
-        <v>14.33</v>
+        <v>1040</v>
       </c>
       <c r="D137" t="n">
-        <v>1.56</v>
+        <v>3.09</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>COCKERILL</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>3.23</v>
+        <v>9605</v>
       </c>
       <c r="C138" t="n">
-        <v>3.28</v>
+        <v>9900</v>
       </c>
       <c r="D138" t="n">
-        <v>1.55</v>
+        <v>3.07</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>KRYSTAL</t>
+          <t>NETWEB</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>575.1</v>
+        <v>4191.4</v>
       </c>
       <c r="C139" t="n">
-        <v>583.9</v>
+        <v>4320</v>
       </c>
       <c r="D139" t="n">
-        <v>1.53</v>
+        <v>3.07</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1.97</v>
+        <v>7.18</v>
       </c>
       <c r="C140" t="n">
-        <v>2</v>
+        <v>7.4</v>
       </c>
       <c r="D140" t="n">
-        <v>1.52</v>
+        <v>3.06</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>24.29</v>
+        <v>482.25</v>
       </c>
       <c r="C141" t="n">
-        <v>24.66</v>
+        <v>497</v>
       </c>
       <c r="D141" t="n">
-        <v>1.52</v>
+        <v>3.06</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ORBTEXP</t>
+          <t>IRISDOREME</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>194.96</v>
+        <v>35.89</v>
       </c>
       <c r="C142" t="n">
-        <v>197.9</v>
+        <v>36.99</v>
       </c>
       <c r="D142" t="n">
-        <v>1.51</v>
+        <v>3.06</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>INDOWIND</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>9.25</v>
+        <v>936.45</v>
       </c>
       <c r="C143" t="n">
-        <v>9.390000000000001</v>
+        <v>965</v>
       </c>
       <c r="D143" t="n">
-        <v>1.51</v>
+        <v>3.05</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ABMINTLLTD</t>
+          <t>APTECHT</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>42.31</v>
+        <v>106.74</v>
       </c>
       <c r="C144" t="n">
-        <v>42.94</v>
+        <v>110</v>
       </c>
       <c r="D144" t="n">
-        <v>1.49</v>
+        <v>3.05</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>MINDTECK</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>3.36</v>
+        <v>200.83</v>
       </c>
       <c r="C145" t="n">
-        <v>3.41</v>
+        <v>206.93</v>
       </c>
       <c r="D145" t="n">
-        <v>1.49</v>
+        <v>3.04</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SAIPARENT</t>
+          <t>TCIEXP</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>550.65</v>
+        <v>504.15</v>
       </c>
       <c r="C146" t="n">
-        <v>558.85</v>
+        <v>519.3</v>
       </c>
       <c r="D146" t="n">
-        <v>1.49</v>
+        <v>3.01</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>KPL</t>
+          <t>DAICHI</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>2506.6</v>
+        <v>233</v>
       </c>
       <c r="C147" t="n">
-        <v>2544</v>
+        <v>240</v>
       </c>
       <c r="D147" t="n">
-        <v>1.49</v>
+        <v>3</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>QUICKHEAL</t>
+          <t>SHBAJRG</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>173.04</v>
+        <v>200.97</v>
       </c>
       <c r="C148" t="n">
-        <v>175.6</v>
+        <v>207</v>
       </c>
       <c r="D148" t="n">
-        <v>1.48</v>
+        <v>3</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>136.94</v>
+        <v>304.9</v>
       </c>
       <c r="C149" t="n">
-        <v>138.95</v>
+        <v>314</v>
       </c>
       <c r="D149" t="n">
-        <v>1.47</v>
+        <v>2.98</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>SIMBHALS</t>
+          <t>MITTAL</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>6.89</v>
+        <v>1.01</v>
       </c>
       <c r="C150" t="n">
-        <v>6.99</v>
+        <v>1.04</v>
       </c>
       <c r="D150" t="n">
-        <v>1.45</v>
+        <v>2.97</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MUKTAARTS</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>60.14</v>
+        <v>1351.1</v>
       </c>
       <c r="C151" t="n">
-        <v>61</v>
+        <v>1391</v>
       </c>
       <c r="D151" t="n">
-        <v>1.43</v>
+        <v>2.95</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>AEGISVOPAK</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>178.44</v>
+        <v>199.14</v>
       </c>
       <c r="C152" t="n">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="D152" t="n">
-        <v>1.43</v>
+        <v>2.94</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>RENUKA</t>
+          <t>DOLPHIN</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>21.84</v>
+        <v>387.55</v>
       </c>
       <c r="C153" t="n">
-        <v>22.15</v>
+        <v>398.9</v>
       </c>
       <c r="D153" t="n">
-        <v>1.42</v>
+        <v>2.93</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>UFO</t>
+          <t>STEELCITY</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>71.98</v>
+        <v>75.09</v>
       </c>
       <c r="C154" t="n">
-        <v>73</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="D154" t="n">
-        <v>1.42</v>
+        <v>2.93</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>HINDZINC</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>137.01</v>
+        <v>545</v>
       </c>
       <c r="C155" t="n">
-        <v>138.95</v>
+        <v>560.95</v>
       </c>
       <c r="D155" t="n">
-        <v>1.42</v>
+        <v>2.93</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>BAGFILMS</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>4.97</v>
+        <v>5.82</v>
       </c>
       <c r="C156" t="n">
-        <v>5.04</v>
+        <v>5.99</v>
       </c>
       <c r="D156" t="n">
-        <v>1.41</v>
+        <v>2.92</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>BAIDFIN</t>
+          <t>AEPL</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>10.06</v>
+        <v>15.88</v>
       </c>
       <c r="C157" t="n">
-        <v>10.2</v>
+        <v>16.34</v>
       </c>
       <c r="D157" t="n">
-        <v>1.39</v>
+        <v>2.9</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>1.45</v>
+        <v>169.85</v>
       </c>
       <c r="C158" t="n">
-        <v>1.47</v>
+        <v>174.78</v>
       </c>
       <c r="D158" t="n">
-        <v>1.38</v>
+        <v>2.9</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>RHFL</t>
+          <t>VASWANI</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>2.18</v>
+        <v>58.02</v>
       </c>
       <c r="C159" t="n">
-        <v>2.21</v>
+        <v>59.7</v>
       </c>
       <c r="D159" t="n">
-        <v>1.38</v>
+        <v>2.9</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>HARIOMPIPE</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>19.72</v>
+        <v>379.9</v>
       </c>
       <c r="C160" t="n">
-        <v>19.99</v>
+        <v>390.85</v>
       </c>
       <c r="D160" t="n">
-        <v>1.37</v>
+        <v>2.88</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>DHANBANK</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>3.65</v>
+        <v>31.24</v>
       </c>
       <c r="C161" t="n">
-        <v>3.7</v>
+        <v>32.14</v>
       </c>
       <c r="D161" t="n">
-        <v>1.37</v>
+        <v>2.88</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SALSTEEL</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>59.21</v>
+        <v>0.35</v>
       </c>
       <c r="C162" t="n">
-        <v>60</v>
+        <v>0.36</v>
       </c>
       <c r="D162" t="n">
-        <v>1.33</v>
+        <v>2.86</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>MONOLITH</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>370.1</v>
+        <v>683.15</v>
       </c>
       <c r="C163" t="n">
-        <v>374.95</v>
+        <v>702.7</v>
       </c>
       <c r="D163" t="n">
-        <v>1.31</v>
+        <v>2.86</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>UNIVASTU</t>
+          <t>JAYNECOIND</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>78.31</v>
+        <v>87.31</v>
       </c>
       <c r="C164" t="n">
-        <v>79.33</v>
+        <v>89.8</v>
       </c>
       <c r="D164" t="n">
-        <v>1.3</v>
+        <v>2.85</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>GOKUL</t>
+          <t>YESBANK</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>40.94</v>
+        <v>22.22</v>
       </c>
       <c r="C165" t="n">
-        <v>41.47</v>
+        <v>22.85</v>
       </c>
       <c r="D165" t="n">
-        <v>1.29</v>
+        <v>2.84</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>RVNL</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>14.86</v>
+        <v>222.19</v>
       </c>
       <c r="C166" t="n">
-        <v>15.05</v>
+        <v>228.5</v>
       </c>
       <c r="D166" t="n">
-        <v>1.28</v>
+        <v>2.84</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>VIRINCHI</t>
+          <t>TDPOWERSYS</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>14.85</v>
+        <v>1126</v>
       </c>
       <c r="C167" t="n">
-        <v>15.04</v>
+        <v>1158</v>
       </c>
       <c r="D167" t="n">
-        <v>1.28</v>
+        <v>2.84</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>PREMIERPOL</t>
+          <t>PNBGILTS</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>55.24</v>
+        <v>85.47</v>
       </c>
       <c r="C168" t="n">
-        <v>55.94</v>
+        <v>87.88</v>
       </c>
       <c r="D168" t="n">
-        <v>1.27</v>
+        <v>2.82</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>JAIBALAJI</t>
+          <t>VINDHYATEL</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>66.05</v>
+        <v>1979.6</v>
       </c>
       <c r="C169" t="n">
-        <v>66.89</v>
+        <v>2035.5</v>
       </c>
       <c r="D169" t="n">
-        <v>1.27</v>
+        <v>2.82</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SENORES</t>
+          <t>PARKHOSPS</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>1112.6</v>
+        <v>273.25</v>
       </c>
       <c r="C170" t="n">
-        <v>1126.2</v>
+        <v>280.95</v>
       </c>
       <c r="D170" t="n">
-        <v>1.22</v>
+        <v>2.82</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>IITL</t>
+          <t>REMSONSIND</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>141.34</v>
+        <v>84.47</v>
       </c>
       <c r="C171" t="n">
-        <v>143.05</v>
+        <v>86.84</v>
       </c>
       <c r="D171" t="n">
-        <v>1.21</v>
+        <v>2.81</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>TREL</t>
+          <t>SENCO</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>25.84</v>
+        <v>328.05</v>
       </c>
       <c r="C172" t="n">
-        <v>26.15</v>
+        <v>337.25</v>
       </c>
       <c r="D172" t="n">
-        <v>1.2</v>
+        <v>2.8</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SANOFICONR</t>
+          <t>DYCL</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>4675</v>
+        <v>303.3</v>
       </c>
       <c r="C173" t="n">
-        <v>4730</v>
+        <v>311.8</v>
       </c>
       <c r="D173" t="n">
-        <v>1.18</v>
+        <v>2.8</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>VALIANTLAB</t>
+          <t>UNIPARTS</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>69.18000000000001</v>
+        <v>637.15</v>
       </c>
       <c r="C174" t="n">
-        <v>69.98999999999999</v>
+        <v>655</v>
       </c>
       <c r="D174" t="n">
-        <v>1.17</v>
+        <v>2.8</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ATALREAL</t>
+          <t>SALASAR</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>29.65</v>
+        <v>6.42</v>
       </c>
       <c r="C175" t="n">
-        <v>29.99</v>
+        <v>6.6</v>
       </c>
       <c r="D175" t="n">
-        <v>1.15</v>
+        <v>2.8</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>UFLEX</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>178.45</v>
+        <v>406.15</v>
       </c>
       <c r="C176" t="n">
-        <v>180.49</v>
+        <v>417.5</v>
       </c>
       <c r="D176" t="n">
-        <v>1.14</v>
+        <v>2.79</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>MURUDCERA</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>909.6</v>
+        <v>30.45</v>
       </c>
       <c r="C177" t="n">
-        <v>920</v>
+        <v>31.3</v>
       </c>
       <c r="D177" t="n">
-        <v>1.14</v>
+        <v>2.79</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>LANDSMILL</t>
+          <t>ARTEMISMED</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>0.88</v>
+        <v>254.75</v>
       </c>
       <c r="C178" t="n">
-        <v>0.89</v>
+        <v>261.85</v>
       </c>
       <c r="D178" t="n">
-        <v>1.14</v>
+        <v>2.79</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>BEEKAY</t>
+          <t>SENORES</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>415.3</v>
+        <v>1160.7</v>
       </c>
       <c r="C179" t="n">
-        <v>420</v>
+        <v>1193</v>
       </c>
       <c r="D179" t="n">
-        <v>1.13</v>
+        <v>2.78</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>HECPROJECT</t>
+          <t>MOTILALOFS</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>120.15</v>
+        <v>831.6</v>
       </c>
       <c r="C180" t="n">
-        <v>121.5</v>
+        <v>854.7</v>
       </c>
       <c r="D180" t="n">
-        <v>1.12</v>
+        <v>2.78</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>GFLLIMITED</t>
+          <t>CPPLUS</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>46.38</v>
+        <v>3343.5</v>
       </c>
       <c r="C181" t="n">
-        <v>46.9</v>
+        <v>3436.4</v>
       </c>
       <c r="D181" t="n">
-        <v>1.12</v>
+        <v>2.78</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>DAVANGERE</t>
+          <t>NITIRAJ</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>3.56</v>
+        <v>196.55</v>
       </c>
       <c r="C182" t="n">
-        <v>3.6</v>
+        <v>202</v>
       </c>
       <c r="D182" t="n">
-        <v>1.12</v>
+        <v>2.77</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>NEPHROPLUS</t>
+          <t>JKTYRE</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>723.15</v>
+        <v>352.45</v>
       </c>
       <c r="C183" t="n">
-        <v>731.25</v>
+        <v>362.2</v>
       </c>
       <c r="D183" t="n">
-        <v>1.12</v>
+        <v>2.77</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>OSWALGREEN</t>
+          <t>MAWANASUG</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>22.75</v>
+        <v>101.1</v>
       </c>
       <c r="C184" t="n">
-        <v>23</v>
+        <v>103.9</v>
       </c>
       <c r="D184" t="n">
-        <v>1.1</v>
+        <v>2.77</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>CARYSIL</t>
+          <t>A2ZINFRA</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>1191.9</v>
+        <v>14.11</v>
       </c>
       <c r="C185" t="n">
-        <v>1205</v>
+        <v>14.5</v>
       </c>
       <c r="D185" t="n">
-        <v>1.1</v>
+        <v>2.76</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>MASTERTR</t>
+          <t>AVADHSUGAR</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>75.17</v>
+        <v>454.55</v>
       </c>
       <c r="C186" t="n">
-        <v>75.98999999999999</v>
+        <v>467.1</v>
       </c>
       <c r="D186" t="n">
-        <v>1.09</v>
+        <v>2.76</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>CLEANMAX</t>
+          <t>HINDCOPPER</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>1335.5</v>
+        <v>499.25</v>
       </c>
       <c r="C187" t="n">
-        <v>1350</v>
+        <v>512.95</v>
       </c>
       <c r="D187" t="n">
-        <v>1.09</v>
+        <v>2.74</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>GRMOVER</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>175.09</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="C188" t="n">
-        <v>177</v>
+        <v>90</v>
       </c>
       <c r="D188" t="n">
-        <v>1.09</v>
+        <v>2.74</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>DECNGOLD</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>4.65</v>
+        <v>153.09</v>
       </c>
       <c r="C189" t="n">
-        <v>4.7</v>
+        <v>157.29</v>
       </c>
       <c r="D189" t="n">
-        <v>1.08</v>
+        <v>2.74</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>PYRAMID</t>
+          <t>SKIPPER</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>163.27</v>
+        <v>520.8</v>
       </c>
       <c r="C190" t="n">
-        <v>165</v>
+        <v>535</v>
       </c>
       <c r="D190" t="n">
-        <v>1.06</v>
+        <v>2.73</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>EXCELINDUS</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>909.1</v>
+        <v>1201.2</v>
       </c>
       <c r="C191" t="n">
-        <v>918.5</v>
+        <v>1234</v>
       </c>
       <c r="D191" t="n">
-        <v>1.03</v>
+        <v>2.73</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>RUSHIL</t>
+          <t>COMPUSOFT</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>14.73</v>
+        <v>13.58</v>
       </c>
       <c r="C192" t="n">
-        <v>14.88</v>
+        <v>13.95</v>
       </c>
       <c r="D192" t="n">
-        <v>1.02</v>
+        <v>2.72</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>NILAINFRA</t>
+          <t>ABCOTS</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>7.81</v>
+        <v>198.38</v>
       </c>
       <c r="C193" t="n">
-        <v>7.89</v>
+        <v>203.78</v>
       </c>
       <c r="D193" t="n">
-        <v>1.02</v>
+        <v>2.72</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>BALRAMCHIN</t>
+          <t>EMBDL</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>536.55</v>
+        <v>56.38</v>
       </c>
       <c r="C194" t="n">
-        <v>542</v>
+        <v>57.9</v>
       </c>
       <c r="D194" t="n">
-        <v>1.02</v>
+        <v>2.7</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ARIES</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>326.65</v>
+        <v>373.95</v>
       </c>
       <c r="C195" t="n">
-        <v>329.95</v>
+        <v>384</v>
       </c>
       <c r="D195" t="n">
-        <v>1.01</v>
+        <v>2.69</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>VENUSREM</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>1633.5</v>
+        <v>2.6</v>
       </c>
       <c r="C196" t="n">
-        <v>1650</v>
+        <v>2.67</v>
       </c>
       <c r="D196" t="n">
-        <v>1.01</v>
+        <v>2.69</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>RPPINFRA</t>
+          <t>CARYSIL</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>60.15</v>
+        <v>1163.8</v>
       </c>
       <c r="C197" t="n">
-        <v>60.75</v>
+        <v>1195</v>
       </c>
       <c r="D197" t="n">
-        <v>1</v>
+        <v>2.68</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>INA</t>
+          <t>JYOTISTRUC</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>115.42</v>
+        <v>11.63</v>
       </c>
       <c r="C198" t="n">
-        <v>116.57</v>
+        <v>11.94</v>
       </c>
       <c r="D198" t="n">
-        <v>1</v>
+        <v>2.67</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ARIHANT</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>882.95</v>
+        <v>50.27</v>
       </c>
       <c r="C199" t="n">
-        <v>891.8</v>
+        <v>51.6</v>
       </c>
       <c r="D199" t="n">
-        <v>1</v>
+        <v>2.65</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>71.88</v>
+        <v>175.31</v>
       </c>
       <c r="C200" t="n">
-        <v>72.59999999999999</v>
+        <v>179.94</v>
       </c>
       <c r="D200" t="n">
-        <v>1</v>
+        <v>2.64</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>GSPCROP</t>
+          <t>TRUALT</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>428.95</v>
+        <v>498.65</v>
       </c>
       <c r="C201" t="n">
-        <v>433.25</v>
+        <v>511.8</v>
       </c>
       <c r="D201" t="n">
-        <v>1</v>
+        <v>2.64</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-15 09:47 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="C2" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
+        <v>33.33</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WINSOL</t>
+          <t>SCANSTL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>125.95</v>
+        <v>37.51</v>
       </c>
       <c r="C3" t="n">
-        <v>138.7</v>
+        <v>43.5</v>
       </c>
       <c r="D3" t="n">
-        <v>10.12</v>
+        <v>15.97</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CURAA</t>
+          <t>K2INFRA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>77.58</v>
+        <v>50.25</v>
       </c>
       <c r="C4" t="n">
-        <v>85.3</v>
+        <v>57</v>
       </c>
       <c r="D4" t="n">
-        <v>9.949999999999999</v>
+        <v>13.43</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>SEPC</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.94</v>
+        <v>6.91</v>
       </c>
       <c r="C5" t="n">
-        <v>7.58</v>
+        <v>7.64</v>
       </c>
       <c r="D5" t="n">
-        <v>9.220000000000001</v>
+        <v>10.56</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PPAP</t>
+          <t>SELMC</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>244.82</v>
+        <v>30</v>
       </c>
       <c r="C6" t="n">
-        <v>263.79</v>
+        <v>32.98</v>
       </c>
       <c r="D6" t="n">
-        <v>7.75</v>
+        <v>9.93</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19.55</v>
+        <v>3.25</v>
       </c>
       <c r="C7" t="n">
-        <v>21</v>
+        <v>3.57</v>
       </c>
       <c r="D7" t="n">
-        <v>7.42</v>
+        <v>9.85</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>NFPSAMPOOR</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1531</v>
+        <v>27.5</v>
       </c>
       <c r="C8" t="n">
-        <v>1644</v>
+        <v>30.1</v>
       </c>
       <c r="D8" t="n">
-        <v>7.38</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>K2INFRA</t>
+          <t>PIONRINV</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>48.95</v>
+        <v>98.7</v>
       </c>
       <c r="C9" t="n">
-        <v>52.5</v>
+        <v>107.99</v>
       </c>
       <c r="D9" t="n">
-        <v>7.25</v>
+        <v>9.41</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KOTYARK</t>
+          <t>VDEAL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>402.6</v>
+        <v>161</v>
       </c>
       <c r="C10" t="n">
-        <v>430</v>
+        <v>175.95</v>
       </c>
       <c r="D10" t="n">
-        <v>6.81</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>14.61</v>
+        <v>86.68000000000001</v>
       </c>
       <c r="C11" t="n">
-        <v>15.6</v>
+        <v>94</v>
       </c>
       <c r="D11" t="n">
-        <v>6.78</v>
+        <v>8.44</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HALDER</t>
+          <t>BETA</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>240.68</v>
+        <v>1771.2</v>
       </c>
       <c r="C12" t="n">
-        <v>257</v>
+        <v>1920</v>
       </c>
       <c r="D12" t="n">
-        <v>6.78</v>
+        <v>8.4</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>BHADORA</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.15</v>
+        <v>59.65</v>
       </c>
       <c r="C13" t="n">
-        <v>0.16</v>
+        <v>64.5</v>
       </c>
       <c r="D13" t="n">
-        <v>6.67</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>COUNCODOS</t>
+          <t>STEELXIND</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4.97</v>
+        <v>11.49</v>
       </c>
       <c r="C14" t="n">
-        <v>5.3</v>
+        <v>12.4</v>
       </c>
       <c r="D14" t="n">
-        <v>6.64</v>
+        <v>7.92</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>URAVIDEF</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>69.53</v>
+        <v>113.74</v>
       </c>
       <c r="C15" t="n">
-        <v>74</v>
+        <v>122.7</v>
       </c>
       <c r="D15" t="n">
-        <v>6.43</v>
+        <v>7.88</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.79</v>
+        <v>32.93</v>
       </c>
       <c r="C16" t="n">
-        <v>0.84</v>
+        <v>35.5</v>
       </c>
       <c r="D16" t="n">
-        <v>6.33</v>
+        <v>7.8</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>NIDAN</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>243</v>
+        <v>13.9</v>
       </c>
       <c r="C17" t="n">
-        <v>258</v>
+        <v>14.95</v>
       </c>
       <c r="D17" t="n">
-        <v>6.17</v>
+        <v>7.55</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MTARTECH</t>
+          <t>RSDFIN</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6306</v>
+        <v>80</v>
       </c>
       <c r="C18" t="n">
-        <v>6666.5</v>
+        <v>85.98999999999999</v>
       </c>
       <c r="D18" t="n">
-        <v>5.72</v>
+        <v>7.49</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>VISHWARAJ</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5.46</v>
+        <v>1.84</v>
       </c>
       <c r="C19" t="n">
-        <v>5.76</v>
+        <v>1.97</v>
       </c>
       <c r="D19" t="n">
-        <v>5.49</v>
+        <v>7.07</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>MUKKA</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>27.1</v>
+        <v>22.81</v>
       </c>
       <c r="C20" t="n">
-        <v>28.58</v>
+        <v>24.4</v>
       </c>
       <c r="D20" t="n">
-        <v>5.46</v>
+        <v>6.97</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PARASPETRO</t>
+          <t>BANSALWIRE</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.88</v>
+        <v>303.85</v>
       </c>
       <c r="C21" t="n">
-        <v>1.98</v>
+        <v>325</v>
       </c>
       <c r="D21" t="n">
-        <v>5.32</v>
+        <v>6.96</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>TREJHARA</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6.4</v>
+        <v>140.55</v>
       </c>
       <c r="C22" t="n">
-        <v>6.74</v>
+        <v>149.99</v>
       </c>
       <c r="D22" t="n">
-        <v>5.31</v>
+        <v>6.72</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="C23" t="n">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="D23" t="n">
-        <v>5.26</v>
+        <v>6.67</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>GICL</t>
+          <t>HALEOSLABS</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>22.06</v>
+        <v>1406.2</v>
       </c>
       <c r="C24" t="n">
-        <v>23.2</v>
+        <v>1499.9</v>
       </c>
       <c r="D24" t="n">
-        <v>5.17</v>
+        <v>6.66</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SHRIKRISH</t>
+          <t>AKASH</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>42.82</v>
+        <v>26.02</v>
       </c>
       <c r="C25" t="n">
-        <v>45</v>
+        <v>27.74</v>
       </c>
       <c r="D25" t="n">
-        <v>5.09</v>
+        <v>6.61</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LASA</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>7.18</v>
+        <v>0.46</v>
       </c>
       <c r="C26" t="n">
-        <v>7.54</v>
+        <v>0.49</v>
       </c>
       <c r="D26" t="n">
-        <v>5.01</v>
+        <v>6.52</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>EMKAYTOOLS</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>39.8</v>
+        <v>96</v>
       </c>
       <c r="C27" t="n">
-        <v>41.79</v>
+        <v>102</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>6.25</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>GICL</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>10.23</v>
+        <v>22.22</v>
       </c>
       <c r="C28" t="n">
-        <v>10.74</v>
+        <v>23.6</v>
       </c>
       <c r="D28" t="n">
-        <v>4.99</v>
+        <v>6.21</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SHEEL</t>
+          <t>MASON</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>57.15</v>
+        <v>138.1</v>
       </c>
       <c r="C29" t="n">
-        <v>60</v>
+        <v>146.6</v>
       </c>
       <c r="D29" t="n">
-        <v>4.99</v>
+        <v>6.15</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>INNOMET</t>
+          <t>BIGBLOC</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>100.5</v>
+        <v>49.22</v>
       </c>
       <c r="C30" t="n">
-        <v>105.5</v>
+        <v>52.22</v>
       </c>
       <c r="D30" t="n">
-        <v>4.98</v>
+        <v>6.1</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TCIFINANCE</t>
+          <t>DGCONTENT</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>25.3</v>
+        <v>25.78</v>
       </c>
       <c r="C31" t="n">
-        <v>26.56</v>
+        <v>27.3</v>
       </c>
       <c r="D31" t="n">
-        <v>4.98</v>
+        <v>5.9</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>UHTL</t>
+          <t>CEINSYS</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>98.8</v>
+        <v>920.6</v>
       </c>
       <c r="C32" t="n">
-        <v>103.7</v>
+        <v>974</v>
       </c>
       <c r="D32" t="n">
-        <v>4.96</v>
+        <v>5.8</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>KDL</t>
+          <t>THEINVEST</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>119.9</v>
+        <v>98.14</v>
       </c>
       <c r="C33" t="n">
-        <v>125.85</v>
+        <v>103.8</v>
       </c>
       <c r="D33" t="n">
-        <v>4.96</v>
+        <v>5.77</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SSFL</t>
+          <t>NURECA</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>218</v>
+        <v>232.1</v>
       </c>
       <c r="C34" t="n">
-        <v>228.8</v>
+        <v>245.45</v>
       </c>
       <c r="D34" t="n">
-        <v>4.95</v>
+        <v>5.75</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GLFL</t>
+          <t>AIROLAM</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6.32</v>
+        <v>85.97</v>
       </c>
       <c r="C35" t="n">
-        <v>6.63</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="D35" t="n">
-        <v>4.91</v>
+        <v>5.73</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SHEKHAWATI</t>
+          <t>MCLOUD</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>14.52</v>
+        <v>22.22</v>
       </c>
       <c r="C36" t="n">
-        <v>15.22</v>
+        <v>23.49</v>
       </c>
       <c r="D36" t="n">
-        <v>4.82</v>
+        <v>5.72</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>ORIENTALTL</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>90.56999999999999</v>
+        <v>6.29</v>
       </c>
       <c r="C37" t="n">
-        <v>94.90000000000001</v>
+        <v>6.65</v>
       </c>
       <c r="D37" t="n">
-        <v>4.78</v>
+        <v>5.72</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>MUKTAARTS</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3.59</v>
+        <v>60.55</v>
       </c>
       <c r="C38" t="n">
-        <v>3.76</v>
+        <v>64</v>
       </c>
       <c r="D38" t="n">
-        <v>4.74</v>
+        <v>5.7</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>FINBUD</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>43.37</v>
+        <v>124</v>
       </c>
       <c r="C39" t="n">
-        <v>45.4</v>
+        <v>131</v>
       </c>
       <c r="D39" t="n">
-        <v>4.68</v>
+        <v>5.65</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TGL</t>
+          <t>GODAVARIB</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>20.4</v>
+        <v>278.05</v>
       </c>
       <c r="C40" t="n">
-        <v>21.35</v>
+        <v>293.7</v>
       </c>
       <c r="D40" t="n">
-        <v>4.66</v>
+        <v>5.63</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TRIDHYA</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>9.65</v>
+        <v>6.8</v>
       </c>
       <c r="C41" t="n">
-        <v>10.1</v>
+        <v>7.18</v>
       </c>
       <c r="D41" t="n">
-        <v>4.66</v>
+        <v>5.59</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>NORBTEAEXP</t>
+          <t>SPUNWEB</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>74.06</v>
+        <v>109.9</v>
       </c>
       <c r="C42" t="n">
-        <v>77.5</v>
+        <v>116</v>
       </c>
       <c r="D42" t="n">
-        <v>4.64</v>
+        <v>5.55</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BILVYAPAR</t>
+          <t>CHAMUNDA</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3.92</v>
+        <v>39.7</v>
       </c>
       <c r="C43" t="n">
-        <v>4.1</v>
+        <v>41.9</v>
       </c>
       <c r="D43" t="n">
-        <v>4.59</v>
+        <v>5.54</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>RPPL</t>
+          <t>CURAA</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>17.79</v>
+        <v>85.33</v>
       </c>
       <c r="C44" t="n">
-        <v>18.6</v>
+        <v>90.02</v>
       </c>
       <c r="D44" t="n">
-        <v>4.55</v>
+        <v>5.5</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>AGARIND</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.22</v>
+        <v>483.55</v>
       </c>
       <c r="C45" t="n">
-        <v>0.23</v>
+        <v>510</v>
       </c>
       <c r="D45" t="n">
-        <v>4.55</v>
+        <v>5.47</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PILITA</t>
+          <t>FINCABLES</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>7.98</v>
+        <v>1035.8</v>
       </c>
       <c r="C46" t="n">
-        <v>8.34</v>
+        <v>1092</v>
       </c>
       <c r="D46" t="n">
-        <v>4.51</v>
+        <v>5.43</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>HINDWAREAP</t>
+          <t>AMANTA</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>213.01</v>
+        <v>151.82</v>
       </c>
       <c r="C47" t="n">
-        <v>222.59</v>
+        <v>160</v>
       </c>
       <c r="D47" t="n">
-        <v>4.5</v>
+        <v>5.39</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SHUBHLAXMI</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>25.8</v>
+        <v>14.8</v>
       </c>
       <c r="C48" t="n">
-        <v>26.95</v>
+        <v>15.59</v>
       </c>
       <c r="D48" t="n">
-        <v>4.46</v>
+        <v>5.34</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SAHANA</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>713.85</v>
+        <v>23.97</v>
       </c>
       <c r="C49" t="n">
-        <v>745</v>
+        <v>25.25</v>
       </c>
       <c r="D49" t="n">
-        <v>4.36</v>
+        <v>5.34</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CREATIVEYE</t>
+          <t>SOMATEX</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>6.43</v>
+        <v>94.95999999999999</v>
       </c>
       <c r="C50" t="n">
-        <v>6.7</v>
+        <v>100</v>
       </c>
       <c r="D50" t="n">
-        <v>4.2</v>
+        <v>5.31</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>TMCV</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>10.08</v>
+        <v>390.3</v>
       </c>
       <c r="C51" t="n">
-        <v>10.5</v>
+        <v>411</v>
       </c>
       <c r="D51" t="n">
-        <v>4.17</v>
+        <v>5.3</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SAMBHAAV</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>6.24</v>
+        <v>0.19</v>
       </c>
       <c r="C52" t="n">
-        <v>6.5</v>
+        <v>0.2</v>
       </c>
       <c r="D52" t="n">
-        <v>4.17</v>
+        <v>5.26</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GANESHIN</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>89.3</v>
+        <v>954.95</v>
       </c>
       <c r="C53" t="n">
-        <v>93</v>
+        <v>1005</v>
       </c>
       <c r="D53" t="n">
-        <v>4.14</v>
+        <v>5.24</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PASHUPATI</t>
+          <t>GGBL</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>87.88</v>
+        <v>308.35</v>
       </c>
       <c r="C54" t="n">
-        <v>91.5</v>
+        <v>324</v>
       </c>
       <c r="D54" t="n">
-        <v>4.12</v>
+        <v>5.08</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>4.71</v>
+        <v>13.11</v>
       </c>
       <c r="C55" t="n">
-        <v>4.9</v>
+        <v>13.77</v>
       </c>
       <c r="D55" t="n">
-        <v>4.03</v>
+        <v>5.03</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>SPCL</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>20</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="C56" t="n">
-        <v>20.8</v>
+        <v>74.45</v>
       </c>
       <c r="D56" t="n">
-        <v>4</v>
+        <v>5.01</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>HCL-INSYS</t>
+          <t>VISHWARAJ</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>11.75</v>
+        <v>5.8</v>
       </c>
       <c r="C57" t="n">
-        <v>12.22</v>
+        <v>6.09</v>
       </c>
       <c r="D57" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>EPACKPEB</t>
+          <t>BIRLACABLE</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>227.27</v>
+        <v>194.13</v>
       </c>
       <c r="C58" t="n">
-        <v>236.28</v>
+        <v>203.83</v>
       </c>
       <c r="D58" t="n">
-        <v>3.96</v>
+        <v>5</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>OSWALAGRO</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>42.53</v>
+        <v>171.86</v>
       </c>
       <c r="C59" t="n">
-        <v>44.18</v>
+        <v>180.45</v>
       </c>
       <c r="D59" t="n">
-        <v>3.88</v>
+        <v>5</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>VIDYAWIRES</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>7.21</v>
+        <v>89.08</v>
       </c>
       <c r="C60" t="n">
-        <v>7.49</v>
+        <v>93.53</v>
       </c>
       <c r="D60" t="n">
-        <v>3.88</v>
+        <v>5</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CKKRETAIL</t>
+          <t>OCCLLTD</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="C61" t="n">
-        <v>145.4</v>
+        <v>135.45</v>
       </c>
       <c r="D61" t="n">
-        <v>3.86</v>
+        <v>5</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>LEMERITE</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>163.68</v>
+        <v>26.07</v>
       </c>
       <c r="C62" t="n">
-        <v>170</v>
+        <v>27.37</v>
       </c>
       <c r="D62" t="n">
-        <v>3.86</v>
+        <v>4.99</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DREDGECORP</t>
+          <t>VEEKAYEM</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1040.3</v>
+        <v>134.2</v>
       </c>
       <c r="C63" t="n">
-        <v>1080</v>
+        <v>140.9</v>
       </c>
       <c r="D63" t="n">
-        <v>3.82</v>
+        <v>4.99</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PLAZACABLE</t>
+          <t>SIDDHIKA</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>46.22</v>
+        <v>205.5</v>
       </c>
       <c r="C64" t="n">
-        <v>47.98</v>
+        <v>215.75</v>
       </c>
       <c r="D64" t="n">
-        <v>3.81</v>
+        <v>4.99</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>NIRAJ</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>5.89</v>
+        <v>28.88</v>
       </c>
       <c r="C65" t="n">
-        <v>6.11</v>
+        <v>30.32</v>
       </c>
       <c r="D65" t="n">
-        <v>3.74</v>
+        <v>4.99</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>INDOTHAI</t>
+          <t>AHLWEST</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>235.7</v>
+        <v>560.7</v>
       </c>
       <c r="C66" t="n">
-        <v>244.5</v>
+        <v>588.7</v>
       </c>
       <c r="D66" t="n">
-        <v>3.73</v>
+        <v>4.99</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>OMNI</t>
+          <t>DEEDEV</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>453</v>
+        <v>656.7</v>
       </c>
       <c r="C67" t="n">
-        <v>469.8</v>
+        <v>689.5</v>
       </c>
       <c r="D67" t="n">
-        <v>3.71</v>
+        <v>4.99</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>DCMSRIND</t>
+          <t>HEXAGON</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>37.61</v>
+        <v>50.66</v>
       </c>
       <c r="C68" t="n">
-        <v>39</v>
+        <v>53.19</v>
       </c>
       <c r="D68" t="n">
-        <v>3.7</v>
+        <v>4.99</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>SICALLOG</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>21.22</v>
+        <v>83.48999999999999</v>
       </c>
       <c r="C69" t="n">
-        <v>22</v>
+        <v>87.66</v>
       </c>
       <c r="D69" t="n">
-        <v>3.68</v>
+        <v>4.99</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>UNITEDTEA</t>
+          <t>OMAXAUTO</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>510.2</v>
+        <v>227.05</v>
       </c>
       <c r="C70" t="n">
-        <v>529</v>
+        <v>238.35</v>
       </c>
       <c r="D70" t="n">
-        <v>3.68</v>
+        <v>4.98</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>HAPPSTMNDS</t>
+          <t>GENXAI</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>345</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="C71" t="n">
-        <v>357.55</v>
+        <v>102.25</v>
       </c>
       <c r="D71" t="n">
-        <v>3.64</v>
+        <v>4.98</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>UNITEDPOLY</t>
+          <t>CPPLUS</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>33.29</v>
+        <v>3375.9</v>
       </c>
       <c r="C72" t="n">
-        <v>34.5</v>
+        <v>3544</v>
       </c>
       <c r="D72" t="n">
-        <v>3.63</v>
+        <v>4.98</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>IL&amp;FSENGG</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>74.3</v>
+        <v>28.92</v>
       </c>
       <c r="C73" t="n">
-        <v>76.98999999999999</v>
+        <v>30.36</v>
       </c>
       <c r="D73" t="n">
-        <v>3.62</v>
+        <v>4.98</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>NOIDATOLL</t>
+          <t>ORTEL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>4.98</v>
+        <v>1.61</v>
       </c>
       <c r="C74" t="n">
-        <v>5.16</v>
+        <v>1.69</v>
       </c>
       <c r="D74" t="n">
-        <v>3.61</v>
+        <v>4.97</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>ANIKINDS</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>13.51</v>
+        <v>42.98</v>
       </c>
       <c r="C75" t="n">
-        <v>13.99</v>
+        <v>45.11</v>
       </c>
       <c r="D75" t="n">
-        <v>3.55</v>
+        <v>4.96</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TARAPUR</t>
+          <t>GANESHIN</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>18.34</v>
+        <v>93.75</v>
       </c>
       <c r="C76" t="n">
-        <v>18.99</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="D76" t="n">
-        <v>3.54</v>
+        <v>4.96</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>HEXT</t>
+          <t>VEEDOL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>502.25</v>
+        <v>1418.8</v>
       </c>
       <c r="C77" t="n">
-        <v>520</v>
+        <v>1489</v>
       </c>
       <c r="D77" t="n">
-        <v>3.53</v>
+        <v>4.95</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>EXIMROUTES</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>100.45</v>
+        <v>45.45</v>
       </c>
       <c r="C78" t="n">
-        <v>104</v>
+        <v>47.7</v>
       </c>
       <c r="D78" t="n">
-        <v>3.53</v>
+        <v>4.95</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>OMINFRAL</t>
+          <t>SUBEXLTD</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>80.44</v>
+        <v>10.51</v>
       </c>
       <c r="C79" t="n">
-        <v>83.28</v>
+        <v>11.03</v>
       </c>
       <c r="D79" t="n">
-        <v>3.53</v>
+        <v>4.95</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CENTENKA</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>489.85</v>
+        <v>10.74</v>
       </c>
       <c r="C80" t="n">
-        <v>507.15</v>
+        <v>11.27</v>
       </c>
       <c r="D80" t="n">
-        <v>3.53</v>
+        <v>4.93</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BCG</t>
+          <t>SEMAC</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>10.23</v>
+        <v>324.95</v>
       </c>
       <c r="C81" t="n">
-        <v>10.59</v>
+        <v>340.95</v>
       </c>
       <c r="D81" t="n">
-        <v>3.52</v>
+        <v>4.92</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>KESORAMIND</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>23.57</v>
+        <v>10.98</v>
       </c>
       <c r="C82" t="n">
-        <v>24.4</v>
+        <v>11.52</v>
       </c>
       <c r="D82" t="n">
-        <v>3.52</v>
+        <v>4.92</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>BATLIBOI</t>
+          <t>GLFL</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>74.48</v>
+        <v>6.12</v>
       </c>
       <c r="C83" t="n">
-        <v>77.09999999999999</v>
+        <v>6.42</v>
       </c>
       <c r="D83" t="n">
-        <v>3.52</v>
+        <v>4.9</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>FIBERWEB</t>
+          <t>VALIANTORG</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>27.53</v>
+        <v>280.15</v>
       </c>
       <c r="C84" t="n">
-        <v>28.5</v>
+        <v>293.85</v>
       </c>
       <c r="D84" t="n">
-        <v>3.52</v>
+        <v>4.89</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>KRIDHANINF</t>
+          <t>WHITEFORCE</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>2.85</v>
+        <v>36.9</v>
       </c>
       <c r="C85" t="n">
-        <v>2.95</v>
+        <v>38.7</v>
       </c>
       <c r="D85" t="n">
-        <v>3.51</v>
+        <v>4.88</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>IRIS</t>
+          <t>QUICKTOUCH</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>223.65</v>
+        <v>26.65</v>
       </c>
       <c r="C86" t="n">
-        <v>231.5</v>
+        <v>27.95</v>
       </c>
       <c r="D86" t="n">
-        <v>3.51</v>
+        <v>4.88</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>NAMAN</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1323.8</v>
+        <v>47.15</v>
       </c>
       <c r="C87" t="n">
-        <v>1370.1</v>
+        <v>49.45</v>
       </c>
       <c r="D87" t="n">
-        <v>3.5</v>
+        <v>4.88</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>AVROIND</t>
+          <t>MKPL</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>10.58</v>
+        <v>4.73</v>
       </c>
       <c r="C88" t="n">
-        <v>10.95</v>
+        <v>4.96</v>
       </c>
       <c r="D88" t="n">
-        <v>3.5</v>
+        <v>4.86</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SILLYMONKS</t>
+          <t>HINDWAREAP</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>18.34</v>
+        <v>251.79</v>
       </c>
       <c r="C89" t="n">
-        <v>18.98</v>
+        <v>264</v>
       </c>
       <c r="D89" t="n">
-        <v>3.49</v>
+        <v>4.85</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SUDARCOLOR</t>
+          <t>ANLON</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>356.95</v>
+        <v>713.5</v>
       </c>
       <c r="C90" t="n">
-        <v>369.4</v>
+        <v>748</v>
       </c>
       <c r="D90" t="n">
-        <v>3.49</v>
+        <v>4.84</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>AARON</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>71.12</v>
+        <v>119.24</v>
       </c>
       <c r="C91" t="n">
-        <v>73.59999999999999</v>
+        <v>125</v>
       </c>
       <c r="D91" t="n">
-        <v>3.49</v>
+        <v>4.83</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SOUTHWEST</t>
+          <t>GREENLEAF</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>240.15</v>
+        <v>58</v>
       </c>
       <c r="C92" t="n">
-        <v>248.5</v>
+        <v>60.8</v>
       </c>
       <c r="D92" t="n">
-        <v>3.48</v>
+        <v>4.83</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>IGCL</t>
+          <t>ARTNIRMAN</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>55.85</v>
+        <v>40.07</v>
       </c>
       <c r="C93" t="n">
-        <v>57.79</v>
+        <v>42</v>
       </c>
       <c r="D93" t="n">
-        <v>3.47</v>
+        <v>4.82</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MVGJL</t>
+          <t>MOTISONS</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>143.91</v>
+        <v>14.79</v>
       </c>
       <c r="C94" t="n">
-        <v>148.9</v>
+        <v>15.5</v>
       </c>
       <c r="D94" t="n">
-        <v>3.47</v>
+        <v>4.8</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>SILLYMONKS</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>357.65</v>
+        <v>18.12</v>
       </c>
       <c r="C95" t="n">
-        <v>369.95</v>
+        <v>18.99</v>
       </c>
       <c r="D95" t="n">
-        <v>3.44</v>
+        <v>4.8</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>DIGIDRIVE</t>
+          <t>MANDEEP</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>17.89</v>
+        <v>18.8</v>
       </c>
       <c r="C96" t="n">
-        <v>18.5</v>
+        <v>19.7</v>
       </c>
       <c r="D96" t="n">
-        <v>3.41</v>
+        <v>4.79</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>VICTORYEV</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>34.33</v>
+        <v>17.75</v>
       </c>
       <c r="C97" t="n">
-        <v>35.5</v>
+        <v>18.6</v>
       </c>
       <c r="D97" t="n">
-        <v>3.41</v>
+        <v>4.79</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SHIVATEX</t>
+          <t>MANORG</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>147.86</v>
+        <v>470.5</v>
       </c>
       <c r="C98" t="n">
-        <v>152.9</v>
+        <v>492.85</v>
       </c>
       <c r="D98" t="n">
-        <v>3.41</v>
+        <v>4.75</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>IVC</t>
+          <t>ENSER</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>8.27</v>
+        <v>16</v>
       </c>
       <c r="C99" t="n">
-        <v>8.550000000000001</v>
+        <v>16.75</v>
       </c>
       <c r="D99" t="n">
-        <v>3.39</v>
+        <v>4.69</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CROWN</t>
+          <t>OSWALPUMPS</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>108.3</v>
+        <v>398.2</v>
       </c>
       <c r="C100" t="n">
-        <v>111.96</v>
+        <v>416.85</v>
       </c>
       <c r="D100" t="n">
-        <v>3.38</v>
+        <v>4.68</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FOODSIN</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>53.93</v>
+        <v>310.6</v>
       </c>
       <c r="C101" t="n">
-        <v>55.75</v>
+        <v>325</v>
       </c>
       <c r="D101" t="n">
-        <v>3.37</v>
+        <v>4.64</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>LOTUSDEV</t>
+          <t>CINEVISTA</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>129.27</v>
+        <v>15.1</v>
       </c>
       <c r="C102" t="n">
-        <v>133.62</v>
+        <v>15.8</v>
       </c>
       <c r="D102" t="n">
-        <v>3.37</v>
+        <v>4.64</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>KOTHARIPRO</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>68.5</v>
+        <v>10.82</v>
       </c>
       <c r="C103" t="n">
-        <v>70.8</v>
+        <v>11.32</v>
       </c>
       <c r="D103" t="n">
-        <v>3.36</v>
+        <v>4.62</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>47.02</v>
+        <v>1414.2</v>
       </c>
       <c r="C104" t="n">
-        <v>48.6</v>
+        <v>1479</v>
       </c>
       <c r="D104" t="n">
-        <v>3.36</v>
+        <v>4.58</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>HINDCOMPOS</t>
+          <t>HINDPETRO</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>402.5</v>
+        <v>388.9</v>
       </c>
       <c r="C105" t="n">
-        <v>416</v>
+        <v>406.7</v>
       </c>
       <c r="D105" t="n">
-        <v>3.35</v>
+        <v>4.58</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>6.87</v>
+        <v>94.2</v>
       </c>
       <c r="C106" t="n">
-        <v>7.1</v>
+        <v>98.5</v>
       </c>
       <c r="D106" t="n">
-        <v>3.35</v>
+        <v>4.56</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ASHOKLEY</t>
+          <t>UNIVCABLES</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>138.58</v>
+        <v>1176.6</v>
       </c>
       <c r="C107" t="n">
-        <v>143.22</v>
+        <v>1230.1</v>
       </c>
       <c r="D107" t="n">
-        <v>3.35</v>
+        <v>4.55</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>HISARMETAL</t>
+          <t>AURIONPRO</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>152.91</v>
+        <v>777.25</v>
       </c>
       <c r="C108" t="n">
-        <v>158</v>
+        <v>812.4</v>
       </c>
       <c r="D108" t="n">
-        <v>3.33</v>
+        <v>4.52</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>HCC</t>
+          <t>MBLINFRA</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>21.68</v>
+        <v>26.55</v>
       </c>
       <c r="C109" t="n">
-        <v>22.4</v>
+        <v>27.75</v>
       </c>
       <c r="D109" t="n">
-        <v>3.32</v>
+        <v>4.52</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BETA</t>
+          <t>CAPTRUST</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>1476</v>
+        <v>13.28</v>
       </c>
       <c r="C110" t="n">
-        <v>1525</v>
+        <v>13.88</v>
       </c>
       <c r="D110" t="n">
-        <v>3.32</v>
+        <v>4.52</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>KODYTECH</t>
+          <t>FAZE3Q</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>904.2</v>
+        <v>545.3</v>
       </c>
       <c r="C111" t="n">
-        <v>934</v>
+        <v>569.95</v>
       </c>
       <c r="D111" t="n">
-        <v>3.3</v>
+        <v>4.52</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>BAFNAPH</t>
+          <t>KDL</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>174.15</v>
+        <v>124.25</v>
       </c>
       <c r="C112" t="n">
-        <v>179.9</v>
+        <v>129.85</v>
       </c>
       <c r="D112" t="n">
-        <v>3.3</v>
+        <v>4.51</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>AEGISLOG</t>
+          <t>NGLFINE</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>925.9</v>
+        <v>3048.8</v>
       </c>
       <c r="C113" t="n">
-        <v>956.35</v>
+        <v>3186</v>
       </c>
       <c r="D113" t="n">
-        <v>3.29</v>
+        <v>4.5</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>COCKERILL</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>24.92</v>
+        <v>10011</v>
       </c>
       <c r="C114" t="n">
-        <v>25.74</v>
+        <v>10461</v>
       </c>
       <c r="D114" t="n">
-        <v>3.29</v>
+        <v>4.5</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>PRAJIND</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>18.01</v>
+        <v>332.1</v>
       </c>
       <c r="C115" t="n">
-        <v>18.6</v>
+        <v>347</v>
       </c>
       <c r="D115" t="n">
-        <v>3.28</v>
+        <v>4.49</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>HINDPETRO</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>365.7</v>
+        <v>7.17</v>
       </c>
       <c r="C116" t="n">
-        <v>377.7</v>
+        <v>7.49</v>
       </c>
       <c r="D116" t="n">
-        <v>3.28</v>
+        <v>4.46</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>PRAENG</t>
+          <t>LLOYDSENT</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>20.24</v>
+        <v>66.93000000000001</v>
       </c>
       <c r="C117" t="n">
-        <v>20.9</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D117" t="n">
-        <v>3.26</v>
+        <v>4.44</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ANURAS</t>
+          <t>SADHNANIQ</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>1258</v>
+        <v>2.27</v>
       </c>
       <c r="C118" t="n">
-        <v>1299</v>
+        <v>2.37</v>
       </c>
       <c r="D118" t="n">
-        <v>3.26</v>
+        <v>4.41</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CENTRUM</t>
+          <t>IRIS</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>21.5</v>
+        <v>238.5</v>
       </c>
       <c r="C119" t="n">
-        <v>22.2</v>
+        <v>249</v>
       </c>
       <c r="D119" t="n">
-        <v>3.26</v>
+        <v>4.4</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MOTISONS</t>
+          <t>POWERICA</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>13.22</v>
+        <v>458.75</v>
       </c>
       <c r="C120" t="n">
-        <v>13.65</v>
+        <v>478.95</v>
       </c>
       <c r="D120" t="n">
-        <v>3.25</v>
+        <v>4.4</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>FOODSIN</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>251.65</v>
+        <v>54.17</v>
       </c>
       <c r="C121" t="n">
-        <v>259.8</v>
+        <v>56.55</v>
       </c>
       <c r="D121" t="n">
-        <v>3.24</v>
+        <v>4.39</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>MMP</t>
+          <t>HMAAGRO</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>251.75</v>
+        <v>22.62</v>
       </c>
       <c r="C122" t="n">
-        <v>259.9</v>
+        <v>23.61</v>
       </c>
       <c r="D122" t="n">
-        <v>3.24</v>
+        <v>4.38</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>MAJESAUT</t>
+          <t>COMPINFO</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>334</v>
+        <v>1.38</v>
       </c>
       <c r="C123" t="n">
-        <v>344.8</v>
+        <v>1.44</v>
       </c>
       <c r="D123" t="n">
-        <v>3.23</v>
+        <v>4.35</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>EBGNG</t>
+          <t>BHANDARI</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>418.55</v>
+        <v>3</v>
       </c>
       <c r="C124" t="n">
-        <v>432</v>
+        <v>3.13</v>
       </c>
       <c r="D124" t="n">
-        <v>3.21</v>
+        <v>4.33</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>EVERESTIND</t>
+          <t>BAJAJST</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>331.4</v>
+        <v>367.05</v>
       </c>
       <c r="C125" t="n">
-        <v>342</v>
+        <v>382.9</v>
       </c>
       <c r="D125" t="n">
-        <v>3.2</v>
+        <v>4.32</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CYIENT</t>
+          <t>SAURASHCEM</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>846.65</v>
+        <v>59.43</v>
       </c>
       <c r="C126" t="n">
-        <v>873.7</v>
+        <v>61.99</v>
       </c>
       <c r="D126" t="n">
-        <v>3.19</v>
+        <v>4.31</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>KENNAMET</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>23.65</v>
+        <v>2780.3</v>
       </c>
       <c r="C127" t="n">
-        <v>24.4</v>
+        <v>2899.8</v>
       </c>
       <c r="D127" t="n">
-        <v>3.17</v>
+        <v>4.3</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>AARVI</t>
+          <t>IOC</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>142.31</v>
+        <v>140.94</v>
       </c>
       <c r="C128" t="n">
-        <v>146.8</v>
+        <v>147</v>
       </c>
       <c r="D128" t="n">
-        <v>3.16</v>
+        <v>4.3</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MANGALAM</t>
+          <t>ASHOKLEY</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>27.91</v>
+        <v>152.45</v>
       </c>
       <c r="C129" t="n">
-        <v>28.79</v>
+        <v>159</v>
       </c>
       <c r="D129" t="n">
-        <v>3.15</v>
+        <v>4.3</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>PRAVEG</t>
+          <t>TOLINS</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>212.35</v>
+        <v>102.3</v>
       </c>
       <c r="C130" t="n">
-        <v>219</v>
+        <v>106.69</v>
       </c>
       <c r="D130" t="n">
-        <v>3.13</v>
+        <v>4.29</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>BESTAGRO</t>
+          <t>FIVESTAR</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>15.33</v>
+        <v>439.15</v>
       </c>
       <c r="C131" t="n">
-        <v>15.81</v>
+        <v>458</v>
       </c>
       <c r="D131" t="n">
-        <v>3.13</v>
+        <v>4.29</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>PARACABLES</t>
+          <t>DEVX</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>60.85</v>
+        <v>36.64</v>
       </c>
       <c r="C132" t="n">
-        <v>62.75</v>
+        <v>38.2</v>
       </c>
       <c r="D132" t="n">
-        <v>3.12</v>
+        <v>4.26</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>TARMAT</t>
+          <t>FISCHER</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>51.84</v>
+        <v>36.15</v>
       </c>
       <c r="C133" t="n">
-        <v>53.45</v>
+        <v>37.68</v>
       </c>
       <c r="D133" t="n">
-        <v>3.11</v>
+        <v>4.23</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>FCL</t>
+          <t>AXISCADES</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>37.03</v>
+        <v>1947.6</v>
       </c>
       <c r="C134" t="n">
-        <v>38.18</v>
+        <v>2030</v>
       </c>
       <c r="D134" t="n">
-        <v>3.11</v>
+        <v>4.23</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>TIJARIA</t>
+          <t>SYRMA</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>4.52</v>
+        <v>1266.7</v>
       </c>
       <c r="C135" t="n">
-        <v>4.66</v>
+        <v>1320</v>
       </c>
       <c r="D135" t="n">
-        <v>3.1</v>
+        <v>4.21</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>VAKRANGEE</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>0.97</v>
+        <v>6.19</v>
       </c>
       <c r="C136" t="n">
-        <v>1</v>
+        <v>6.45</v>
       </c>
       <c r="D136" t="n">
-        <v>3.09</v>
+        <v>4.2</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>GABRIEL</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>1008.8</v>
+        <v>302.35</v>
       </c>
       <c r="C137" t="n">
-        <v>1040</v>
+        <v>315</v>
       </c>
       <c r="D137" t="n">
-        <v>3.09</v>
+        <v>4.18</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>COCKERILL</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>9605</v>
+        <v>0.48</v>
       </c>
       <c r="C138" t="n">
-        <v>9900</v>
+        <v>0.5</v>
       </c>
       <c r="D138" t="n">
-        <v>3.07</v>
+        <v>4.17</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>NETWEB</t>
+          <t>AMAGI</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>4191.4</v>
+        <v>425.95</v>
       </c>
       <c r="C139" t="n">
-        <v>4320</v>
+        <v>443.7</v>
       </c>
       <c r="D139" t="n">
-        <v>3.07</v>
+        <v>4.17</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>RAJTV</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>7.18</v>
+        <v>11.75</v>
       </c>
       <c r="C140" t="n">
-        <v>7.4</v>
+        <v>12.24</v>
       </c>
       <c r="D140" t="n">
-        <v>3.06</v>
+        <v>4.17</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>UCAL</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>482.25</v>
+        <v>100.05</v>
       </c>
       <c r="C141" t="n">
-        <v>497</v>
+        <v>104.2</v>
       </c>
       <c r="D141" t="n">
-        <v>3.06</v>
+        <v>4.15</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>IRISDOREME</t>
+          <t>MAXIND</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>35.89</v>
+        <v>158.44</v>
       </c>
       <c r="C142" t="n">
-        <v>36.99</v>
+        <v>165</v>
       </c>
       <c r="D142" t="n">
-        <v>3.06</v>
+        <v>4.14</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>IZMO</t>
+          <t>WEBELSOLAR</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>936.45</v>
+        <v>103.63</v>
       </c>
       <c r="C143" t="n">
-        <v>965</v>
+        <v>107.9</v>
       </c>
       <c r="D143" t="n">
-        <v>3.05</v>
+        <v>4.12</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>APTECHT</t>
+          <t>ASHIMASYN</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>106.74</v>
+        <v>16.04</v>
       </c>
       <c r="C144" t="n">
-        <v>110</v>
+        <v>16.7</v>
       </c>
       <c r="D144" t="n">
-        <v>3.05</v>
+        <v>4.11</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>MINDTECK</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>200.83</v>
+        <v>324.65</v>
       </c>
       <c r="C145" t="n">
-        <v>206.93</v>
+        <v>338</v>
       </c>
       <c r="D145" t="n">
-        <v>3.04</v>
+        <v>4.11</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>TCIEXP</t>
+          <t>KCPSUGIND</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>504.15</v>
+        <v>22.48</v>
       </c>
       <c r="C146" t="n">
-        <v>519.3</v>
+        <v>23.4</v>
       </c>
       <c r="D146" t="n">
-        <v>3.01</v>
+        <v>4.09</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>DAICHI</t>
+          <t>RATEGAIN</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>233</v>
+        <v>783.05</v>
       </c>
       <c r="C147" t="n">
-        <v>240</v>
+        <v>814.9</v>
       </c>
       <c r="D147" t="n">
-        <v>3</v>
+        <v>4.07</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>SHBAJRG</t>
+          <t>SEIL</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>200.97</v>
+        <v>197.03</v>
       </c>
       <c r="C148" t="n">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D148" t="n">
-        <v>3</v>
+        <v>4.05</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>JYOTISTRUC</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>304.9</v>
+        <v>12.14</v>
       </c>
       <c r="C149" t="n">
-        <v>314</v>
+        <v>12.63</v>
       </c>
       <c r="D149" t="n">
-        <v>2.98</v>
+        <v>4.04</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>PONNIERODE</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1.01</v>
+        <v>315.3</v>
       </c>
       <c r="C150" t="n">
-        <v>1.04</v>
+        <v>328</v>
       </c>
       <c r="D150" t="n">
-        <v>2.97</v>
+        <v>4.03</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>1351.1</v>
+        <v>21.86</v>
       </c>
       <c r="C151" t="n">
-        <v>1391</v>
+        <v>22.74</v>
       </c>
       <c r="D151" t="n">
-        <v>2.95</v>
+        <v>4.03</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>AEGISVOPAK</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>199.14</v>
+        <v>40.38</v>
       </c>
       <c r="C152" t="n">
-        <v>205</v>
+        <v>42</v>
       </c>
       <c r="D152" t="n">
-        <v>2.94</v>
+        <v>4.01</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>DOLPHIN</t>
+          <t>VPRPL</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>387.55</v>
+        <v>26.44</v>
       </c>
       <c r="C153" t="n">
-        <v>398.9</v>
+        <v>27.5</v>
       </c>
       <c r="D153" t="n">
-        <v>2.93</v>
+        <v>4.01</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>STEELCITY</t>
+          <t>SYSTMTXC</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>75.09</v>
+        <v>66.62</v>
       </c>
       <c r="C154" t="n">
-        <v>77.29000000000001</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="D154" t="n">
-        <v>2.93</v>
+        <v>4.01</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>HINDZINC</t>
+          <t>ASHOKA</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>545</v>
+        <v>123.06</v>
       </c>
       <c r="C155" t="n">
-        <v>560.95</v>
+        <v>128</v>
       </c>
       <c r="D155" t="n">
-        <v>2.93</v>
+        <v>4.01</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>STCINDIA</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>5.82</v>
+        <v>118.26</v>
       </c>
       <c r="C156" t="n">
-        <v>5.99</v>
+        <v>123</v>
       </c>
       <c r="D156" t="n">
-        <v>2.92</v>
+        <v>4.01</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>AEPL</t>
+          <t>HERANBA</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>15.88</v>
+        <v>188.88</v>
       </c>
       <c r="C157" t="n">
-        <v>16.34</v>
+        <v>196.44</v>
       </c>
       <c r="D157" t="n">
-        <v>2.9</v>
+        <v>4</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>SAGCEM</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>169.85</v>
+        <v>167.46</v>
       </c>
       <c r="C158" t="n">
-        <v>174.78</v>
+        <v>174.15</v>
       </c>
       <c r="D158" t="n">
-        <v>2.9</v>
+        <v>3.99</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>VASWANI</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>58.02</v>
+        <v>359.75</v>
       </c>
       <c r="C159" t="n">
-        <v>59.7</v>
+        <v>374.05</v>
       </c>
       <c r="D159" t="n">
-        <v>2.9</v>
+        <v>3.97</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>HARIOMPIPE</t>
+          <t>ATLANTAA</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>379.9</v>
+        <v>39.86</v>
       </c>
       <c r="C160" t="n">
-        <v>390.85</v>
+        <v>41.44</v>
       </c>
       <c r="D160" t="n">
-        <v>2.88</v>
+        <v>3.96</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>DHANBANK</t>
+          <t>GULFPETRO</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>31.24</v>
+        <v>39.92</v>
       </c>
       <c r="C161" t="n">
-        <v>32.14</v>
+        <v>41.5</v>
       </c>
       <c r="D161" t="n">
-        <v>2.88</v>
+        <v>3.96</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>JKIL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>0.35</v>
+        <v>458.9</v>
       </c>
       <c r="C162" t="n">
-        <v>0.36</v>
+        <v>476.95</v>
       </c>
       <c r="D162" t="n">
-        <v>2.86</v>
+        <v>3.93</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>MONOLITH</t>
+          <t>VIVIDHA</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>683.15</v>
+        <v>0.51</v>
       </c>
       <c r="C163" t="n">
-        <v>702.7</v>
+        <v>0.53</v>
       </c>
       <c r="D163" t="n">
-        <v>2.86</v>
+        <v>3.92</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>JAYNECOIND</t>
+          <t>EIHAHOTELS</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>87.31</v>
+        <v>302.85</v>
       </c>
       <c r="C164" t="n">
-        <v>89.8</v>
+        <v>314.7</v>
       </c>
       <c r="D164" t="n">
-        <v>2.85</v>
+        <v>3.91</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>YESBANK</t>
+          <t>MATRIMONY</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>22.22</v>
+        <v>390</v>
       </c>
       <c r="C165" t="n">
-        <v>22.85</v>
+        <v>405.2</v>
       </c>
       <c r="D165" t="n">
-        <v>2.84</v>
+        <v>3.9</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>RVNL</t>
+          <t>STARPAPER</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>222.19</v>
+        <v>135.55</v>
       </c>
       <c r="C166" t="n">
-        <v>228.5</v>
+        <v>140.8</v>
       </c>
       <c r="D166" t="n">
-        <v>2.84</v>
+        <v>3.87</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>TDPOWERSYS</t>
+          <t>KPEL</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>1126</v>
+        <v>344.2</v>
       </c>
       <c r="C167" t="n">
-        <v>1158</v>
+        <v>357.5</v>
       </c>
       <c r="D167" t="n">
-        <v>2.84</v>
+        <v>3.86</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>PNBGILTS</t>
+          <t>BCPL</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>85.47</v>
+        <v>77.03</v>
       </c>
       <c r="C168" t="n">
-        <v>87.88</v>
+        <v>80</v>
       </c>
       <c r="D168" t="n">
-        <v>2.82</v>
+        <v>3.86</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>VINDHYATEL</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>1979.6</v>
+        <v>381</v>
       </c>
       <c r="C169" t="n">
-        <v>2035.5</v>
+        <v>395.65</v>
       </c>
       <c r="D169" t="n">
-        <v>2.82</v>
+        <v>3.85</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>PARKHOSPS</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>273.25</v>
+        <v>570.35</v>
       </c>
       <c r="C170" t="n">
-        <v>280.95</v>
+        <v>592.25</v>
       </c>
       <c r="D170" t="n">
-        <v>2.82</v>
+        <v>3.84</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>REMSONSIND</t>
+          <t>DRONE</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>84.47</v>
+        <v>40.45</v>
       </c>
       <c r="C171" t="n">
-        <v>86.84</v>
+        <v>42</v>
       </c>
       <c r="D171" t="n">
-        <v>2.81</v>
+        <v>3.83</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>SENCO</t>
+          <t>REMUS</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>328.05</v>
+        <v>696.35</v>
       </c>
       <c r="C172" t="n">
-        <v>337.25</v>
+        <v>722.85</v>
       </c>
       <c r="D172" t="n">
-        <v>2.8</v>
+        <v>3.81</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>DYCL</t>
+          <t>GOKUL</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>303.3</v>
+        <v>40.66</v>
       </c>
       <c r="C173" t="n">
-        <v>311.8</v>
+        <v>42.2</v>
       </c>
       <c r="D173" t="n">
-        <v>2.8</v>
+        <v>3.79</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>UNIPARTS</t>
+          <t>APEX</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>637.15</v>
+        <v>419.15</v>
       </c>
       <c r="C174" t="n">
-        <v>655</v>
+        <v>435</v>
       </c>
       <c r="D174" t="n">
-        <v>2.8</v>
+        <v>3.78</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>SALASAR</t>
+          <t>ACSTECH</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>6.42</v>
+        <v>39.51</v>
       </c>
       <c r="C175" t="n">
-        <v>6.6</v>
+        <v>40.99</v>
       </c>
       <c r="D175" t="n">
-        <v>2.8</v>
+        <v>3.75</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>UFLEX</t>
+          <t>RVNL</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>406.15</v>
+        <v>233.26</v>
       </c>
       <c r="C176" t="n">
-        <v>417.5</v>
+        <v>242</v>
       </c>
       <c r="D176" t="n">
-        <v>2.79</v>
+        <v>3.75</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>MURUDCERA</t>
+          <t>OBSCP</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>30.45</v>
+        <v>539.75</v>
       </c>
       <c r="C177" t="n">
-        <v>31.3</v>
+        <v>560</v>
       </c>
       <c r="D177" t="n">
-        <v>2.79</v>
+        <v>3.75</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>ARTEMISMED</t>
+          <t>EMBDL</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>254.75</v>
+        <v>59.06</v>
       </c>
       <c r="C178" t="n">
-        <v>261.85</v>
+        <v>61.26</v>
       </c>
       <c r="D178" t="n">
-        <v>2.79</v>
+        <v>3.73</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>SENORES</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>1160.7</v>
+        <v>58.72</v>
       </c>
       <c r="C179" t="n">
-        <v>1193</v>
+        <v>60.9</v>
       </c>
       <c r="D179" t="n">
-        <v>2.78</v>
+        <v>3.71</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>MOTILALOFS</t>
+          <t>ENIL</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>831.6</v>
+        <v>109.92</v>
       </c>
       <c r="C180" t="n">
-        <v>854.7</v>
+        <v>114</v>
       </c>
       <c r="D180" t="n">
-        <v>2.78</v>
+        <v>3.71</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>CPPLUS</t>
+          <t>GTL</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>3343.5</v>
+        <v>8.41</v>
       </c>
       <c r="C181" t="n">
-        <v>3436.4</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="D181" t="n">
-        <v>2.78</v>
+        <v>3.69</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>NITIRAJ</t>
+          <t>SCPL</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>196.55</v>
+        <v>451.4</v>
       </c>
       <c r="C182" t="n">
-        <v>202</v>
+        <v>468</v>
       </c>
       <c r="D182" t="n">
-        <v>2.77</v>
+        <v>3.68</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>JKTYRE</t>
+          <t>NINSYS</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>352.45</v>
+        <v>689.55</v>
       </c>
       <c r="C183" t="n">
-        <v>362.2</v>
+        <v>714.95</v>
       </c>
       <c r="D183" t="n">
-        <v>2.77</v>
+        <v>3.68</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MAWANASUG</t>
+          <t>IFCI</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>101.1</v>
+        <v>84.56999999999999</v>
       </c>
       <c r="C184" t="n">
-        <v>103.9</v>
+        <v>87.67</v>
       </c>
       <c r="D184" t="n">
-        <v>2.77</v>
+        <v>3.67</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>A2ZINFRA</t>
+          <t>SSDL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>14.11</v>
+        <v>54.98</v>
       </c>
       <c r="C185" t="n">
-        <v>14.5</v>
+        <v>56.99</v>
       </c>
       <c r="D185" t="n">
-        <v>2.76</v>
+        <v>3.66</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>AVADHSUGAR</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>454.55</v>
+        <v>7.1</v>
       </c>
       <c r="C186" t="n">
-        <v>467.1</v>
+        <v>7.36</v>
       </c>
       <c r="D186" t="n">
-        <v>2.76</v>
+        <v>3.66</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>HINDCOPPER</t>
+          <t>GOODYEAR</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>499.25</v>
+        <v>733</v>
       </c>
       <c r="C187" t="n">
-        <v>512.95</v>
+        <v>759.8</v>
       </c>
       <c r="D187" t="n">
-        <v>2.74</v>
+        <v>3.66</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>GRMOVER</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>87.59999999999999</v>
+        <v>66.56</v>
       </c>
       <c r="C188" t="n">
-        <v>90</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="D188" t="n">
-        <v>2.74</v>
+        <v>3.65</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>DECNGOLD</t>
+          <t>HARIOMPIPE</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>153.09</v>
+        <v>408.2</v>
       </c>
       <c r="C189" t="n">
-        <v>157.29</v>
+        <v>423.1</v>
       </c>
       <c r="D189" t="n">
-        <v>2.74</v>
+        <v>3.65</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>SKIPPER</t>
+          <t>RAILTEL</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>520.8</v>
+        <v>308.75</v>
       </c>
       <c r="C190" t="n">
-        <v>535</v>
+        <v>320</v>
       </c>
       <c r="D190" t="n">
-        <v>2.73</v>
+        <v>3.64</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>BOSCH-HCIL</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>1201.2</v>
+        <v>1331.7</v>
       </c>
       <c r="C191" t="n">
-        <v>1234</v>
+        <v>1380</v>
       </c>
       <c r="D191" t="n">
-        <v>2.73</v>
+        <v>3.63</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>COMPUSOFT</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>13.58</v>
+        <v>14.38</v>
       </c>
       <c r="C192" t="n">
-        <v>13.95</v>
+        <v>14.9</v>
       </c>
       <c r="D192" t="n">
-        <v>2.72</v>
+        <v>3.62</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>ABCOTS</t>
+          <t>MERCANTILE</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>198.38</v>
+        <v>25.77</v>
       </c>
       <c r="C193" t="n">
-        <v>203.78</v>
+        <v>26.7</v>
       </c>
       <c r="D193" t="n">
-        <v>2.72</v>
+        <v>3.61</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>EMBDL</t>
+          <t>GOCOLORS</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>56.38</v>
+        <v>358.65</v>
       </c>
       <c r="C194" t="n">
-        <v>57.9</v>
+        <v>371.55</v>
       </c>
       <c r="D194" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>KRBL</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>373.95</v>
+        <v>366.8</v>
       </c>
       <c r="C195" t="n">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="D195" t="n">
-        <v>2.69</v>
+        <v>3.6</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>EPACKPEB</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>2.6</v>
+        <v>241.17</v>
       </c>
       <c r="C196" t="n">
-        <v>2.67</v>
+        <v>249.86</v>
       </c>
       <c r="D196" t="n">
-        <v>2.69</v>
+        <v>3.6</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>CARYSIL</t>
+          <t>CORALFINAC</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>1163.8</v>
+        <v>31.47</v>
       </c>
       <c r="C197" t="n">
-        <v>1195</v>
+        <v>32.6</v>
       </c>
       <c r="D197" t="n">
-        <v>2.68</v>
+        <v>3.59</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>JYOTISTRUC</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>11.63</v>
+        <v>40.64</v>
       </c>
       <c r="C198" t="n">
-        <v>11.94</v>
+        <v>42.1</v>
       </c>
       <c r="D198" t="n">
-        <v>2.67</v>
+        <v>3.59</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>50.27</v>
+        <v>3.9</v>
       </c>
       <c r="C199" t="n">
-        <v>51.6</v>
+        <v>4.04</v>
       </c>
       <c r="D199" t="n">
-        <v>2.65</v>
+        <v>3.59</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>175.31</v>
+        <v>3.9</v>
       </c>
       <c r="C200" t="n">
-        <v>179.94</v>
+        <v>4.04</v>
       </c>
       <c r="D200" t="n">
-        <v>2.64</v>
+        <v>3.59</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>TRUALT</t>
+          <t>BRNL</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>498.65</v>
+        <v>19.01</v>
       </c>
       <c r="C201" t="n">
-        <v>511.8</v>
+        <v>19.69</v>
       </c>
       <c r="D201" t="n">
-        <v>2.64</v>
+        <v>3.58</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-16 09:12 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="C2" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="D2" t="n">
-        <v>33.33</v>
+        <v>25</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SCANSTL</t>
+          <t>MCLOUD</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>37.51</v>
+        <v>26.66</v>
       </c>
       <c r="C3" t="n">
-        <v>43.5</v>
+        <v>28.97</v>
       </c>
       <c r="D3" t="n">
-        <v>15.97</v>
+        <v>8.66</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>K2INFRA</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50.25</v>
+        <v>36.21</v>
       </c>
       <c r="C4" t="n">
-        <v>57</v>
+        <v>38.99</v>
       </c>
       <c r="D4" t="n">
-        <v>13.43</v>
+        <v>7.68</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SEPC</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.91</v>
+        <v>5.61</v>
       </c>
       <c r="C5" t="n">
-        <v>7.64</v>
+        <v>6.04</v>
       </c>
       <c r="D5" t="n">
-        <v>10.56</v>
+        <v>7.66</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SELMC</t>
+          <t>INDPRUD</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>6271</v>
       </c>
       <c r="C6" t="n">
-        <v>32.98</v>
+        <v>6748</v>
       </c>
       <c r="D6" t="n">
-        <v>9.93</v>
+        <v>7.61</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>NIRAJISPAT</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3.25</v>
+        <v>194.83</v>
       </c>
       <c r="C7" t="n">
-        <v>3.57</v>
+        <v>207</v>
       </c>
       <c r="D7" t="n">
-        <v>9.85</v>
+        <v>6.25</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NFPSAMPOOR</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27.5</v>
+        <v>0.16</v>
       </c>
       <c r="C8" t="n">
-        <v>30.1</v>
+        <v>0.17</v>
       </c>
       <c r="D8" t="n">
-        <v>9.449999999999999</v>
+        <v>6.25</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PIONRINV</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>98.7</v>
+        <v>6.89</v>
       </c>
       <c r="C9" t="n">
-        <v>107.99</v>
+        <v>7.31</v>
       </c>
       <c r="D9" t="n">
-        <v>9.41</v>
+        <v>6.1</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VDEAL</t>
+          <t>NDGL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>161</v>
+        <v>2642</v>
       </c>
       <c r="C10" t="n">
-        <v>175.95</v>
+        <v>2779</v>
       </c>
       <c r="D10" t="n">
-        <v>9.289999999999999</v>
+        <v>5.19</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>86.68000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="C11" t="n">
-        <v>94</v>
+        <v>0.83</v>
       </c>
       <c r="D11" t="n">
-        <v>8.44</v>
+        <v>5.06</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BETA</t>
+          <t>MANORG</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1771.2</v>
+        <v>494</v>
       </c>
       <c r="C12" t="n">
-        <v>1920</v>
+        <v>518.7</v>
       </c>
       <c r="D12" t="n">
-        <v>8.4</v>
+        <v>5</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BHADORA</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>59.65</v>
+        <v>0.2</v>
       </c>
       <c r="C13" t="n">
-        <v>64.5</v>
+        <v>0.21</v>
       </c>
       <c r="D13" t="n">
-        <v>8.130000000000001</v>
+        <v>5</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>STEELXIND</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11.49</v>
+        <v>296.2</v>
       </c>
       <c r="C14" t="n">
-        <v>12.4</v>
+        <v>311</v>
       </c>
       <c r="D14" t="n">
-        <v>7.92</v>
+        <v>5</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>URAVIDEF</t>
+          <t>DEEDEV</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>113.74</v>
+        <v>689.5</v>
       </c>
       <c r="C15" t="n">
-        <v>122.7</v>
+        <v>723.95</v>
       </c>
       <c r="D15" t="n">
-        <v>7.88</v>
+        <v>5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>TECHERA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>32.93</v>
+        <v>154.1</v>
       </c>
       <c r="C16" t="n">
-        <v>35.5</v>
+        <v>161.8</v>
       </c>
       <c r="D16" t="n">
-        <v>7.8</v>
+        <v>5</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NIDAN</t>
+          <t>VISL</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13.9</v>
+        <v>21.06</v>
       </c>
       <c r="C17" t="n">
-        <v>14.95</v>
+        <v>22.11</v>
       </c>
       <c r="D17" t="n">
-        <v>7.55</v>
+        <v>4.99</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RSDFIN</t>
+          <t>SUBEXLTD</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>80</v>
+        <v>11.03</v>
       </c>
       <c r="C18" t="n">
-        <v>85.98999999999999</v>
+        <v>11.58</v>
       </c>
       <c r="D18" t="n">
-        <v>7.49</v>
+        <v>4.99</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ORCHASP</t>
+          <t>ACCORD</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1.84</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="C19" t="n">
-        <v>1.97</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>7.07</v>
+        <v>4.98</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MUKKA</t>
+          <t>SHYAMTEL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>22.81</v>
+        <v>15.65</v>
       </c>
       <c r="C20" t="n">
-        <v>24.4</v>
+        <v>16.43</v>
       </c>
       <c r="D20" t="n">
-        <v>6.97</v>
+        <v>4.98</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BANSALWIRE</t>
+          <t>GANESHIN</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>303.85</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="C21" t="n">
-        <v>325</v>
+        <v>103.3</v>
       </c>
       <c r="D21" t="n">
-        <v>6.96</v>
+        <v>4.98</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TREJHARA</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>140.55</v>
+        <v>22.95</v>
       </c>
       <c r="C22" t="n">
-        <v>149.99</v>
+        <v>24.09</v>
       </c>
       <c r="D22" t="n">
-        <v>6.72</v>
+        <v>4.97</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>VPRPL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.15</v>
+        <v>27.76</v>
       </c>
       <c r="C23" t="n">
-        <v>0.16</v>
+        <v>29.14</v>
       </c>
       <c r="D23" t="n">
-        <v>6.67</v>
+        <v>4.97</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HALEOSLABS</t>
+          <t>SMARTLINK</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1406.2</v>
+        <v>164.4</v>
       </c>
       <c r="C24" t="n">
-        <v>1499.9</v>
+        <v>172.55</v>
       </c>
       <c r="D24" t="n">
-        <v>6.66</v>
+        <v>4.96</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AKASH</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>26.02</v>
+        <v>108.85</v>
       </c>
       <c r="C25" t="n">
-        <v>27.74</v>
+        <v>114.25</v>
       </c>
       <c r="D25" t="n">
-        <v>6.61</v>
+        <v>4.96</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.46</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="C26" t="n">
-        <v>0.49</v>
+        <v>103.8</v>
       </c>
       <c r="D26" t="n">
-        <v>6.52</v>
+        <v>4.95</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>EMKAYTOOLS</t>
+          <t>SICALLOG</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>96</v>
+        <v>87.66</v>
       </c>
       <c r="C27" t="n">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="D27" t="n">
-        <v>6.25</v>
+        <v>4.95</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GICL</t>
+          <t>KESORAMIND</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>22.22</v>
+        <v>11.52</v>
       </c>
       <c r="C28" t="n">
-        <v>23.6</v>
+        <v>12.09</v>
       </c>
       <c r="D28" t="n">
-        <v>6.21</v>
+        <v>4.95</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MASON</t>
+          <t>BLUEWATER</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>138.1</v>
+        <v>328.8</v>
       </c>
       <c r="C29" t="n">
-        <v>146.6</v>
+        <v>345</v>
       </c>
       <c r="D29" t="n">
-        <v>6.15</v>
+        <v>4.93</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BIGBLOC</t>
+          <t>LAXMICOT</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>49.22</v>
+        <v>14.2</v>
       </c>
       <c r="C30" t="n">
-        <v>52.22</v>
+        <v>14.9</v>
       </c>
       <c r="D30" t="n">
-        <v>6.1</v>
+        <v>4.93</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DGCONTENT</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>25.78</v>
+        <v>2.44</v>
       </c>
       <c r="C31" t="n">
-        <v>27.3</v>
+        <v>2.56</v>
       </c>
       <c r="D31" t="n">
-        <v>5.9</v>
+        <v>4.92</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CEINSYS</t>
+          <t>CRAYONS</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>920.6</v>
+        <v>30.5</v>
       </c>
       <c r="C32" t="n">
-        <v>974</v>
+        <v>32</v>
       </c>
       <c r="D32" t="n">
-        <v>5.8</v>
+        <v>4.92</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>THEINVEST</t>
+          <t>CEREBRAINT</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>98.14</v>
+        <v>3.86</v>
       </c>
       <c r="C33" t="n">
-        <v>103.8</v>
+        <v>4.05</v>
       </c>
       <c r="D33" t="n">
-        <v>5.77</v>
+        <v>4.92</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>NURECA</t>
+          <t>VISHWAS</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>232.1</v>
+        <v>46.9</v>
       </c>
       <c r="C34" t="n">
-        <v>245.45</v>
+        <v>49.2</v>
       </c>
       <c r="D34" t="n">
-        <v>5.75</v>
+        <v>4.9</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AIROLAM</t>
+          <t>SAMAY</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>85.97</v>
+        <v>40.85</v>
       </c>
       <c r="C35" t="n">
-        <v>90.90000000000001</v>
+        <v>42.85</v>
       </c>
       <c r="D35" t="n">
-        <v>5.73</v>
+        <v>4.9</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MCLOUD</t>
+          <t>SRIVASAVI</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>22.22</v>
+        <v>55.3</v>
       </c>
       <c r="C36" t="n">
-        <v>23.49</v>
+        <v>58</v>
       </c>
       <c r="D36" t="n">
-        <v>5.72</v>
+        <v>4.88</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ORIENTALTL</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>6.29</v>
+        <v>47.7</v>
       </c>
       <c r="C37" t="n">
-        <v>6.65</v>
+        <v>50</v>
       </c>
       <c r="D37" t="n">
-        <v>5.72</v>
+        <v>4.82</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MUKTAARTS</t>
+          <t>FABTECH</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>60.55</v>
+        <v>145.96</v>
       </c>
       <c r="C38" t="n">
-        <v>64</v>
+        <v>153</v>
       </c>
       <c r="D38" t="n">
-        <v>5.7</v>
+        <v>4.82</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FINBUD</t>
+          <t>CALSOFT</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>124</v>
+        <v>20.94</v>
       </c>
       <c r="C39" t="n">
-        <v>131</v>
+        <v>21.95</v>
       </c>
       <c r="D39" t="n">
-        <v>5.65</v>
+        <v>4.82</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GODAVARIB</t>
+          <t>DIVINEHIRA</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>278.05</v>
+        <v>314.95</v>
       </c>
       <c r="C40" t="n">
-        <v>293.7</v>
+        <v>330</v>
       </c>
       <c r="D40" t="n">
-        <v>5.63</v>
+        <v>4.78</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>6.8</v>
+        <v>72.54000000000001</v>
       </c>
       <c r="C41" t="n">
-        <v>7.18</v>
+        <v>76</v>
       </c>
       <c r="D41" t="n">
-        <v>5.59</v>
+        <v>4.77</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SPUNWEB</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>109.9</v>
+        <v>3.79</v>
       </c>
       <c r="C42" t="n">
-        <v>116</v>
+        <v>3.97</v>
       </c>
       <c r="D42" t="n">
-        <v>5.55</v>
+        <v>4.75</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CHAMUNDA</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>39.7</v>
+        <v>155.57</v>
       </c>
       <c r="C43" t="n">
-        <v>41.9</v>
+        <v>162.95</v>
       </c>
       <c r="D43" t="n">
-        <v>5.54</v>
+        <v>4.74</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CURAA</t>
+          <t>ARVSMART</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>85.33</v>
+        <v>594.65</v>
       </c>
       <c r="C44" t="n">
-        <v>90.02</v>
+        <v>622.8</v>
       </c>
       <c r="D44" t="n">
-        <v>5.5</v>
+        <v>4.73</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AGARIND</t>
+          <t>TRIDHYA</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>483.55</v>
+        <v>10.6</v>
       </c>
       <c r="C45" t="n">
-        <v>510</v>
+        <v>11.1</v>
       </c>
       <c r="D45" t="n">
-        <v>5.47</v>
+        <v>4.72</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FINCABLES</t>
+          <t>SARVESHWAR</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1035.8</v>
+        <v>3.6</v>
       </c>
       <c r="C46" t="n">
-        <v>1092</v>
+        <v>3.77</v>
       </c>
       <c r="D46" t="n">
-        <v>5.43</v>
+        <v>4.72</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AMANTA</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>151.82</v>
+        <v>11.27</v>
       </c>
       <c r="C47" t="n">
-        <v>160</v>
+        <v>11.8</v>
       </c>
       <c r="D47" t="n">
-        <v>5.39</v>
+        <v>4.7</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CCCL</t>
+          <t>SEJALLTD</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>14.8</v>
+        <v>690.5</v>
       </c>
       <c r="C48" t="n">
-        <v>15.59</v>
+        <v>722.8</v>
       </c>
       <c r="D48" t="n">
-        <v>5.34</v>
+        <v>4.68</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>SADHNANIQ</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>23.97</v>
+        <v>2.38</v>
       </c>
       <c r="C49" t="n">
-        <v>25.25</v>
+        <v>2.49</v>
       </c>
       <c r="D49" t="n">
-        <v>5.34</v>
+        <v>4.62</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SOMATEX</t>
+          <t>UMAEXPORTS</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>94.95999999999999</v>
+        <v>23.9</v>
       </c>
       <c r="C50" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D50" t="n">
-        <v>5.31</v>
+        <v>4.6</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TMCV</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>390.3</v>
+        <v>2.84</v>
       </c>
       <c r="C51" t="n">
-        <v>411</v>
+        <v>2.97</v>
       </c>
       <c r="D51" t="n">
-        <v>5.3</v>
+        <v>4.58</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="C52" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="D52" t="n">
-        <v>5.26</v>
+        <v>4.55</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>RVTH</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>954.95</v>
+        <v>688.95</v>
       </c>
       <c r="C53" t="n">
-        <v>1005</v>
+        <v>720</v>
       </c>
       <c r="D53" t="n">
-        <v>5.24</v>
+        <v>4.51</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GGBL</t>
+          <t>MANGALAM</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>308.35</v>
+        <v>29.58</v>
       </c>
       <c r="C54" t="n">
-        <v>324</v>
+        <v>30.89</v>
       </c>
       <c r="D54" t="n">
-        <v>5.08</v>
+        <v>4.43</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>13.11</v>
+        <v>3.24</v>
       </c>
       <c r="C55" t="n">
-        <v>13.77</v>
+        <v>3.38</v>
       </c>
       <c r="D55" t="n">
-        <v>5.03</v>
+        <v>4.32</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SPCL</t>
+          <t>MUKTAARTS</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>70.90000000000001</v>
+        <v>63.1</v>
       </c>
       <c r="C56" t="n">
-        <v>74.45</v>
+        <v>65.8</v>
       </c>
       <c r="D56" t="n">
-        <v>5.01</v>
+        <v>4.28</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>VISHWARAJ</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5.8</v>
+        <v>17.89</v>
       </c>
       <c r="C57" t="n">
-        <v>6.09</v>
+        <v>18.65</v>
       </c>
       <c r="D57" t="n">
-        <v>5</v>
+        <v>4.25</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BIRLACABLE</t>
+          <t>USK</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>194.13</v>
+        <v>24.72</v>
       </c>
       <c r="C58" t="n">
-        <v>203.83</v>
+        <v>25.74</v>
       </c>
       <c r="D58" t="n">
-        <v>5</v>
+        <v>4.13</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>DAICHI</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>171.86</v>
+        <v>265.15</v>
       </c>
       <c r="C59" t="n">
-        <v>180.45</v>
+        <v>276</v>
       </c>
       <c r="D59" t="n">
-        <v>5</v>
+        <v>4.09</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>VIDYAWIRES</t>
+          <t>SHETHJI</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>89.08</v>
+        <v>160.2</v>
       </c>
       <c r="C60" t="n">
-        <v>93.53</v>
+        <v>166.7</v>
       </c>
       <c r="D60" t="n">
-        <v>5</v>
+        <v>4.06</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>OCCLLTD</t>
+          <t>TAALTECH</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>129</v>
+        <v>3363.4</v>
       </c>
       <c r="C61" t="n">
-        <v>135.45</v>
+        <v>3500</v>
       </c>
       <c r="D61" t="n">
-        <v>5</v>
+        <v>4.06</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>ASPINWALL</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>26.07</v>
+        <v>259.29</v>
       </c>
       <c r="C62" t="n">
-        <v>27.37</v>
+        <v>269.7</v>
       </c>
       <c r="D62" t="n">
-        <v>4.99</v>
+        <v>4.01</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>VEEKAYEM</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>134.2</v>
+        <v>373</v>
       </c>
       <c r="C63" t="n">
-        <v>140.9</v>
+        <v>387.95</v>
       </c>
       <c r="D63" t="n">
-        <v>4.99</v>
+        <v>4.01</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SIDDHIKA</t>
+          <t>IRMENERGY</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>205.5</v>
+        <v>280.9</v>
       </c>
       <c r="C64" t="n">
-        <v>215.75</v>
+        <v>292</v>
       </c>
       <c r="D64" t="n">
-        <v>4.99</v>
+        <v>3.95</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>NIRAJ</t>
+          <t>PATELENG</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>28.88</v>
+        <v>27.65</v>
       </c>
       <c r="C65" t="n">
-        <v>30.32</v>
+        <v>28.74</v>
       </c>
       <c r="D65" t="n">
-        <v>4.99</v>
+        <v>3.94</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AHLWEST</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>560.7</v>
+        <v>7.17</v>
       </c>
       <c r="C66" t="n">
-        <v>588.7</v>
+        <v>7.45</v>
       </c>
       <c r="D66" t="n">
-        <v>4.99</v>
+        <v>3.91</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>DEEDEV</t>
+          <t>MITTAL</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>656.7</v>
+        <v>1.04</v>
       </c>
       <c r="C67" t="n">
-        <v>689.5</v>
+        <v>1.08</v>
       </c>
       <c r="D67" t="n">
-        <v>4.99</v>
+        <v>3.85</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>HEXAGON</t>
+          <t>LATTEYS</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>50.66</v>
+        <v>22.1</v>
       </c>
       <c r="C68" t="n">
-        <v>53.19</v>
+        <v>22.95</v>
       </c>
       <c r="D68" t="n">
-        <v>4.99</v>
+        <v>3.85</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SICALLOG</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>83.48999999999999</v>
+        <v>5.74</v>
       </c>
       <c r="C69" t="n">
-        <v>87.66</v>
+        <v>5.96</v>
       </c>
       <c r="D69" t="n">
-        <v>4.99</v>
+        <v>3.83</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>OMAXAUTO</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>227.05</v>
+        <v>82.69</v>
       </c>
       <c r="C70" t="n">
-        <v>238.35</v>
+        <v>85.7</v>
       </c>
       <c r="D70" t="n">
-        <v>4.98</v>
+        <v>3.64</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>GENXAI</t>
+          <t>TREEHOUSE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>97.40000000000001</v>
+        <v>7.05</v>
       </c>
       <c r="C71" t="n">
-        <v>102.25</v>
+        <v>7.3</v>
       </c>
       <c r="D71" t="n">
-        <v>4.98</v>
+        <v>3.55</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CPPLUS</t>
+          <t>MADHAVIPL</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>3375.9</v>
+        <v>9.35</v>
       </c>
       <c r="C72" t="n">
-        <v>3544</v>
+        <v>9.68</v>
       </c>
       <c r="D72" t="n">
-        <v>4.98</v>
+        <v>3.53</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>IL&amp;FSENGG</t>
+          <t>JAYBARMARU</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>28.92</v>
+        <v>159.12</v>
       </c>
       <c r="C73" t="n">
-        <v>30.36</v>
+        <v>164.69</v>
       </c>
       <c r="D73" t="n">
-        <v>4.98</v>
+        <v>3.5</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ORTEL</t>
+          <t>TRANSPEK</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1.61</v>
+        <v>981.1</v>
       </c>
       <c r="C74" t="n">
-        <v>1.69</v>
+        <v>1015.4</v>
       </c>
       <c r="D74" t="n">
-        <v>4.97</v>
+        <v>3.5</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ANIKINDS</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>42.98</v>
+        <v>19.56</v>
       </c>
       <c r="C75" t="n">
-        <v>45.11</v>
+        <v>20.24</v>
       </c>
       <c r="D75" t="n">
-        <v>4.96</v>
+        <v>3.48</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>GANESHIN</t>
+          <t>SINTERCOM</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>93.75</v>
+        <v>72.38</v>
       </c>
       <c r="C76" t="n">
-        <v>98.40000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D76" t="n">
-        <v>4.96</v>
+        <v>3.48</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>VEEDOL</t>
+          <t>REGENCERAM</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1418.8</v>
+        <v>40.79</v>
       </c>
       <c r="C77" t="n">
-        <v>1489</v>
+        <v>42.2</v>
       </c>
       <c r="D77" t="n">
-        <v>4.95</v>
+        <v>3.46</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>UNIENTER</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>45.45</v>
+        <v>108.64</v>
       </c>
       <c r="C78" t="n">
-        <v>47.7</v>
+        <v>112.4</v>
       </c>
       <c r="D78" t="n">
-        <v>4.95</v>
+        <v>3.46</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SUBEXLTD</t>
+          <t>HGM</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>10.51</v>
+        <v>53.75</v>
       </c>
       <c r="C79" t="n">
-        <v>11.03</v>
+        <v>55.6</v>
       </c>
       <c r="D79" t="n">
-        <v>4.95</v>
+        <v>3.44</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>DAMODARIND</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>10.74</v>
+        <v>30.75</v>
       </c>
       <c r="C80" t="n">
-        <v>11.27</v>
+        <v>31.8</v>
       </c>
       <c r="D80" t="n">
-        <v>4.93</v>
+        <v>3.41</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SEMAC</t>
+          <t>AAKASH</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>324.95</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="C81" t="n">
-        <v>340.95</v>
+        <v>10.05</v>
       </c>
       <c r="D81" t="n">
-        <v>4.92</v>
+        <v>3.4</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>KESORAMIND</t>
+          <t>AGARIND</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>10.98</v>
+        <v>580.25</v>
       </c>
       <c r="C82" t="n">
-        <v>11.52</v>
+        <v>600</v>
       </c>
       <c r="D82" t="n">
-        <v>4.92</v>
+        <v>3.4</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>GLFL</t>
+          <t>BI</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>6.12</v>
+        <v>58.87</v>
       </c>
       <c r="C83" t="n">
-        <v>6.42</v>
+        <v>60.87</v>
       </c>
       <c r="D83" t="n">
-        <v>4.9</v>
+        <v>3.4</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>VALIANTORG</t>
+          <t>SHREEOSFM</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>280.15</v>
+        <v>59</v>
       </c>
       <c r="C84" t="n">
-        <v>293.85</v>
+        <v>61</v>
       </c>
       <c r="D84" t="n">
-        <v>4.89</v>
+        <v>3.39</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>WHITEFORCE</t>
+          <t>OSELDEVICE</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>36.9</v>
+        <v>480</v>
       </c>
       <c r="C85" t="n">
-        <v>38.7</v>
+        <v>496</v>
       </c>
       <c r="D85" t="n">
-        <v>4.88</v>
+        <v>3.33</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>QUICKTOUCH</t>
+          <t>MGSL</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>26.65</v>
+        <v>60</v>
       </c>
       <c r="C86" t="n">
-        <v>27.95</v>
+        <v>62</v>
       </c>
       <c r="D86" t="n">
-        <v>4.88</v>
+        <v>3.33</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>NAMAN</t>
+          <t>LAXMIINDIA</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>47.15</v>
+        <v>109.88</v>
       </c>
       <c r="C87" t="n">
-        <v>49.45</v>
+        <v>113.5</v>
       </c>
       <c r="D87" t="n">
-        <v>4.88</v>
+        <v>3.29</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>MKPL</t>
+          <t>SARTELE</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>4.73</v>
+        <v>133.5</v>
       </c>
       <c r="C88" t="n">
-        <v>4.96</v>
+        <v>137.85</v>
       </c>
       <c r="D88" t="n">
-        <v>4.86</v>
+        <v>3.26</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HINDWAREAP</t>
+          <t>HARRMALAYA</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>251.79</v>
+        <v>207.26</v>
       </c>
       <c r="C89" t="n">
-        <v>264</v>
+        <v>213.99</v>
       </c>
       <c r="D89" t="n">
-        <v>4.85</v>
+        <v>3.25</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ANLON</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>713.5</v>
+        <v>24.63</v>
       </c>
       <c r="C90" t="n">
-        <v>748</v>
+        <v>25.43</v>
       </c>
       <c r="D90" t="n">
-        <v>4.84</v>
+        <v>3.25</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>AARON</t>
+          <t>RAJESHEXPO</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>119.24</v>
+        <v>80.23</v>
       </c>
       <c r="C91" t="n">
-        <v>125</v>
+        <v>82.8</v>
       </c>
       <c r="D91" t="n">
-        <v>4.83</v>
+        <v>3.2</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GREENLEAF</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>58</v>
+        <v>20.64</v>
       </c>
       <c r="C92" t="n">
-        <v>60.8</v>
+        <v>21.3</v>
       </c>
       <c r="D92" t="n">
-        <v>4.83</v>
+        <v>3.2</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ARTNIRMAN</t>
+          <t>EUROBOND</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>40.07</v>
+        <v>174.46</v>
       </c>
       <c r="C93" t="n">
-        <v>42</v>
+        <v>180</v>
       </c>
       <c r="D93" t="n">
-        <v>4.82</v>
+        <v>3.18</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MOTISONS</t>
+          <t>K2INFRA</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>14.79</v>
+        <v>60.3</v>
       </c>
       <c r="C94" t="n">
-        <v>15.5</v>
+        <v>62.2</v>
       </c>
       <c r="D94" t="n">
-        <v>4.8</v>
+        <v>3.15</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SILLYMONKS</t>
+          <t>BBTCL</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>18.12</v>
+        <v>219.3</v>
       </c>
       <c r="C95" t="n">
-        <v>18.99</v>
+        <v>226.2</v>
       </c>
       <c r="D95" t="n">
-        <v>4.8</v>
+        <v>3.15</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>MANDEEP</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>18.8</v>
+        <v>326.1</v>
       </c>
       <c r="C96" t="n">
-        <v>19.7</v>
+        <v>336.3</v>
       </c>
       <c r="D96" t="n">
-        <v>4.79</v>
+        <v>3.13</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>VICTORYEV</t>
+          <t>TNTELE</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>17.75</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C97" t="n">
-        <v>18.6</v>
+        <v>9.59</v>
       </c>
       <c r="D97" t="n">
-        <v>4.79</v>
+        <v>3.12</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MANORG</t>
+          <t>GANGAFORGE</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>470.5</v>
+        <v>2.57</v>
       </c>
       <c r="C98" t="n">
-        <v>492.85</v>
+        <v>2.65</v>
       </c>
       <c r="D98" t="n">
-        <v>4.75</v>
+        <v>3.11</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ENSER</t>
+          <t>ARIHANT</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>16</v>
+        <v>873.55</v>
       </c>
       <c r="C99" t="n">
-        <v>16.75</v>
+        <v>900</v>
       </c>
       <c r="D99" t="n">
-        <v>4.69</v>
+        <v>3.03</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>OSWALPUMPS</t>
+          <t>DMCC</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>398.2</v>
+        <v>256.25</v>
       </c>
       <c r="C100" t="n">
-        <v>416.85</v>
+        <v>264</v>
       </c>
       <c r="D100" t="n">
-        <v>4.68</v>
+        <v>3.02</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>310.6</v>
+        <v>7.48</v>
       </c>
       <c r="C101" t="n">
-        <v>325</v>
+        <v>7.7</v>
       </c>
       <c r="D101" t="n">
-        <v>4.64</v>
+        <v>2.94</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CINEVISTA</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>15.1</v>
+        <v>422.6</v>
       </c>
       <c r="C102" t="n">
-        <v>15.8</v>
+        <v>435</v>
       </c>
       <c r="D102" t="n">
-        <v>4.64</v>
+        <v>2.93</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ABINFRA</t>
+          <t>SELMC</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>10.82</v>
+        <v>30.12</v>
       </c>
       <c r="C103" t="n">
-        <v>11.32</v>
+        <v>31</v>
       </c>
       <c r="D103" t="n">
-        <v>4.62</v>
+        <v>2.92</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>NITTAGELA</t>
+          <t>NAVKARURB</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>1414.2</v>
+        <v>1.03</v>
       </c>
       <c r="C104" t="n">
-        <v>1479</v>
+        <v>1.06</v>
       </c>
       <c r="D104" t="n">
-        <v>4.58</v>
+        <v>2.91</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>HINDPETRO</t>
+          <t>ASHOKAMET</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>388.9</v>
+        <v>15.2</v>
       </c>
       <c r="C105" t="n">
-        <v>406.7</v>
+        <v>15.64</v>
       </c>
       <c r="D105" t="n">
-        <v>4.58</v>
+        <v>2.89</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>OWAIS</t>
+          <t>MEGASTAR</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>94.2</v>
+        <v>325.6</v>
       </c>
       <c r="C106" t="n">
-        <v>98.5</v>
+        <v>335</v>
       </c>
       <c r="D106" t="n">
-        <v>4.56</v>
+        <v>2.89</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>UNIVCABLES</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>1176.6</v>
+        <v>976</v>
       </c>
       <c r="C107" t="n">
-        <v>1230.1</v>
+        <v>1004</v>
       </c>
       <c r="D107" t="n">
-        <v>4.55</v>
+        <v>2.87</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>AURIONPRO</t>
+          <t>VINYAS</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>777.25</v>
+        <v>1404.95</v>
       </c>
       <c r="C108" t="n">
-        <v>812.4</v>
+        <v>1445</v>
       </c>
       <c r="D108" t="n">
-        <v>4.52</v>
+        <v>2.85</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MBLINFRA</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>26.55</v>
+        <v>3.9</v>
       </c>
       <c r="C109" t="n">
-        <v>27.75</v>
+        <v>4.01</v>
       </c>
       <c r="D109" t="n">
-        <v>4.52</v>
+        <v>2.82</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>CAPTRUST</t>
+          <t>SITINET</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>13.28</v>
+        <v>0.36</v>
       </c>
       <c r="C110" t="n">
-        <v>13.88</v>
+        <v>0.37</v>
       </c>
       <c r="D110" t="n">
-        <v>4.52</v>
+        <v>2.78</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FAZE3Q</t>
+          <t>NOIDATOLL</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>545.3</v>
+        <v>5.05</v>
       </c>
       <c r="C111" t="n">
-        <v>569.95</v>
+        <v>5.19</v>
       </c>
       <c r="D111" t="n">
-        <v>4.52</v>
+        <v>2.77</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>KDL</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>124.25</v>
+        <v>1.1</v>
       </c>
       <c r="C112" t="n">
-        <v>129.85</v>
+        <v>1.13</v>
       </c>
       <c r="D112" t="n">
-        <v>4.51</v>
+        <v>2.73</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>NGLFINE</t>
+          <t>SEPC</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>3048.8</v>
+        <v>7.34</v>
       </c>
       <c r="C113" t="n">
-        <v>3186</v>
+        <v>7.54</v>
       </c>
       <c r="D113" t="n">
-        <v>4.5</v>
+        <v>2.72</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>COCKERILL</t>
+          <t>SAGARDEEP</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>10011</v>
+        <v>25.22</v>
       </c>
       <c r="C114" t="n">
-        <v>10461</v>
+        <v>25.9</v>
       </c>
       <c r="D114" t="n">
-        <v>4.5</v>
+        <v>2.7</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>PRAJIND</t>
+          <t>SUKHJITS</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>332.1</v>
+        <v>170.2</v>
       </c>
       <c r="C115" t="n">
-        <v>347</v>
+        <v>174.8</v>
       </c>
       <c r="D115" t="n">
-        <v>4.49</v>
+        <v>2.7</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>SAHANA</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>7.17</v>
+        <v>802.55</v>
       </c>
       <c r="C116" t="n">
-        <v>7.49</v>
+        <v>824</v>
       </c>
       <c r="D116" t="n">
-        <v>4.46</v>
+        <v>2.67</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>LLOYDSENT</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>66.93000000000001</v>
+        <v>45.29</v>
       </c>
       <c r="C117" t="n">
-        <v>69.90000000000001</v>
+        <v>46.49</v>
       </c>
       <c r="D117" t="n">
-        <v>4.44</v>
+        <v>2.65</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SADHNANIQ</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>2.27</v>
+        <v>4.93</v>
       </c>
       <c r="C118" t="n">
-        <v>2.37</v>
+        <v>5.06</v>
       </c>
       <c r="D118" t="n">
-        <v>4.41</v>
+        <v>2.64</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>IRIS</t>
+          <t>UNIHEALTH</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>238.5</v>
+        <v>496.95</v>
       </c>
       <c r="C119" t="n">
-        <v>249</v>
+        <v>510</v>
       </c>
       <c r="D119" t="n">
-        <v>4.4</v>
+        <v>2.63</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>POWERICA</t>
+          <t>AFFLE</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>458.75</v>
+        <v>1486.4</v>
       </c>
       <c r="C120" t="n">
-        <v>478.95</v>
+        <v>1525</v>
       </c>
       <c r="D120" t="n">
-        <v>4.4</v>
+        <v>2.6</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>FOODSIN</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>54.17</v>
+        <v>11.2</v>
       </c>
       <c r="C121" t="n">
-        <v>56.55</v>
+        <v>11.49</v>
       </c>
       <c r="D121" t="n">
-        <v>4.39</v>
+        <v>2.59</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>HMAAGRO</t>
+          <t>RELIABLE</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>22.62</v>
+        <v>154.91</v>
       </c>
       <c r="C122" t="n">
-        <v>23.61</v>
+        <v>158.9</v>
       </c>
       <c r="D122" t="n">
-        <v>4.38</v>
+        <v>2.58</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>COMPINFO</t>
+          <t>IGARASHI</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1.38</v>
+        <v>378.25</v>
       </c>
       <c r="C123" t="n">
-        <v>1.44</v>
+        <v>388</v>
       </c>
       <c r="D123" t="n">
-        <v>4.35</v>
+        <v>2.58</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>BHANDARI</t>
+          <t>STERTOOLS</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>3</v>
+        <v>239.54</v>
       </c>
       <c r="C124" t="n">
-        <v>3.13</v>
+        <v>245.69</v>
       </c>
       <c r="D124" t="n">
-        <v>4.33</v>
+        <v>2.57</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>BAJAJST</t>
+          <t>DREAMFOLKS</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>367.05</v>
+        <v>72.94</v>
       </c>
       <c r="C125" t="n">
-        <v>382.9</v>
+        <v>74.8</v>
       </c>
       <c r="D125" t="n">
-        <v>4.32</v>
+        <v>2.55</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SAURASHCEM</t>
+          <t>AGROPHOS</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>59.43</v>
+        <v>30.81</v>
       </c>
       <c r="C126" t="n">
-        <v>61.99</v>
+        <v>31.59</v>
       </c>
       <c r="D126" t="n">
-        <v>4.31</v>
+        <v>2.53</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>KENNAMET</t>
+          <t>GALAPREC</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>2780.3</v>
+        <v>1034.05</v>
       </c>
       <c r="C127" t="n">
-        <v>2899.8</v>
+        <v>1060</v>
       </c>
       <c r="D127" t="n">
-        <v>4.3</v>
+        <v>2.51</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>140.94</v>
+        <v>26.93</v>
       </c>
       <c r="C128" t="n">
-        <v>147</v>
+        <v>27.6</v>
       </c>
       <c r="D128" t="n">
-        <v>4.3</v>
+        <v>2.49</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ASHOKLEY</t>
+          <t>ALPA</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>152.45</v>
+        <v>70.26000000000001</v>
       </c>
       <c r="C129" t="n">
-        <v>159</v>
+        <v>72</v>
       </c>
       <c r="D129" t="n">
-        <v>4.3</v>
+        <v>2.48</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>TOLINS</t>
+          <t>SCHNEIDER</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>102.3</v>
+        <v>1216.2</v>
       </c>
       <c r="C130" t="n">
-        <v>106.69</v>
+        <v>1246.2</v>
       </c>
       <c r="D130" t="n">
-        <v>4.29</v>
+        <v>2.47</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>FIVESTAR</t>
+          <t>RPTECH</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>439.15</v>
+        <v>561.25</v>
       </c>
       <c r="C131" t="n">
-        <v>458</v>
+        <v>575</v>
       </c>
       <c r="D131" t="n">
-        <v>4.29</v>
+        <v>2.45</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>DEVX</t>
+          <t>SAPPHIRE</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>36.64</v>
+        <v>173.45</v>
       </c>
       <c r="C132" t="n">
-        <v>38.2</v>
+        <v>177.7</v>
       </c>
       <c r="D132" t="n">
-        <v>4.26</v>
+        <v>2.45</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>FISCHER</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>36.15</v>
+        <v>4.92</v>
       </c>
       <c r="C133" t="n">
-        <v>37.68</v>
+        <v>5.04</v>
       </c>
       <c r="D133" t="n">
-        <v>4.23</v>
+        <v>2.44</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>AXISCADES</t>
+          <t>KIRLFER</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>1947.6</v>
+        <v>434.45</v>
       </c>
       <c r="C134" t="n">
-        <v>2030</v>
+        <v>445</v>
       </c>
       <c r="D134" t="n">
-        <v>4.23</v>
+        <v>2.43</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SYRMA</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>1266.7</v>
+        <v>7.01</v>
       </c>
       <c r="C135" t="n">
-        <v>1320</v>
+        <v>7.18</v>
       </c>
       <c r="D135" t="n">
-        <v>4.21</v>
+        <v>2.43</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>VAKRANGEE</t>
+          <t>RPPINFRA</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>6.19</v>
+        <v>63.35</v>
       </c>
       <c r="C136" t="n">
-        <v>6.45</v>
+        <v>64.89</v>
       </c>
       <c r="D136" t="n">
-        <v>4.2</v>
+        <v>2.43</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>ELITECON</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>302.35</v>
+        <v>30.01</v>
       </c>
       <c r="C137" t="n">
-        <v>315</v>
+        <v>30.74</v>
       </c>
       <c r="D137" t="n">
-        <v>4.18</v>
+        <v>2.43</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>0.48</v>
+        <v>25.47</v>
       </c>
       <c r="C138" t="n">
-        <v>0.5</v>
+        <v>26.09</v>
       </c>
       <c r="D138" t="n">
-        <v>4.17</v>
+        <v>2.43</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>AMAGI</t>
+          <t>VGL</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>425.95</v>
+        <v>75.03</v>
       </c>
       <c r="C139" t="n">
-        <v>443.7</v>
+        <v>76.83</v>
       </c>
       <c r="D139" t="n">
-        <v>4.17</v>
+        <v>2.4</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>RAJTV</t>
+          <t>CURAA</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>11.75</v>
+        <v>91.76000000000001</v>
       </c>
       <c r="C140" t="n">
-        <v>12.24</v>
+        <v>93.95</v>
       </c>
       <c r="D140" t="n">
-        <v>4.17</v>
+        <v>2.39</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>UCAL</t>
+          <t>ELECTHERM</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>100.05</v>
+        <v>1122.25</v>
       </c>
       <c r="C141" t="n">
-        <v>104.2</v>
+        <v>1149</v>
       </c>
       <c r="D141" t="n">
-        <v>4.15</v>
+        <v>2.38</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>MAXIND</t>
+          <t>STEELCITY</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>158.44</v>
+        <v>77.53</v>
       </c>
       <c r="C142" t="n">
-        <v>165</v>
+        <v>79.37</v>
       </c>
       <c r="D142" t="n">
-        <v>4.14</v>
+        <v>2.37</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>WEBELSOLAR</t>
+          <t>BASML</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>103.63</v>
+        <v>24.52</v>
       </c>
       <c r="C143" t="n">
-        <v>107.9</v>
+        <v>25.1</v>
       </c>
       <c r="D143" t="n">
-        <v>4.12</v>
+        <v>2.37</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ASHIMASYN</t>
+          <t>SGL</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>16.04</v>
+        <v>10.69</v>
       </c>
       <c r="C144" t="n">
-        <v>16.7</v>
+        <v>10.94</v>
       </c>
       <c r="D144" t="n">
-        <v>4.11</v>
+        <v>2.34</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>DECCANCE</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>324.65</v>
+        <v>579.5</v>
       </c>
       <c r="C145" t="n">
-        <v>338</v>
+        <v>593</v>
       </c>
       <c r="D145" t="n">
-        <v>4.11</v>
+        <v>2.33</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>KCPSUGIND</t>
+          <t>HAVISHA</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>22.48</v>
+        <v>1.29</v>
       </c>
       <c r="C146" t="n">
-        <v>23.4</v>
+        <v>1.32</v>
       </c>
       <c r="D146" t="n">
-        <v>4.09</v>
+        <v>2.33</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>RATEGAIN</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>783.05</v>
+        <v>9</v>
       </c>
       <c r="C147" t="n">
-        <v>814.9</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="D147" t="n">
-        <v>4.07</v>
+        <v>2.33</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>SEIL</t>
+          <t>HCL-INSYS</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>197.03</v>
+        <v>12.51</v>
       </c>
       <c r="C148" t="n">
-        <v>205</v>
+        <v>12.8</v>
       </c>
       <c r="D148" t="n">
-        <v>4.05</v>
+        <v>2.32</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>JYOTISTRUC</t>
+          <t>DEVYANI</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>12.14</v>
+        <v>111.4</v>
       </c>
       <c r="C149" t="n">
-        <v>12.63</v>
+        <v>113.99</v>
       </c>
       <c r="D149" t="n">
-        <v>4.04</v>
+        <v>2.32</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PONNIERODE</t>
+          <t>KAPSTON</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>315.3</v>
+        <v>344.5</v>
       </c>
       <c r="C150" t="n">
-        <v>328</v>
+        <v>352.5</v>
       </c>
       <c r="D150" t="n">
-        <v>4.03</v>
+        <v>2.32</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>MAJESAUT</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>21.86</v>
+        <v>335.55</v>
       </c>
       <c r="C151" t="n">
-        <v>22.74</v>
+        <v>343.3</v>
       </c>
       <c r="D151" t="n">
-        <v>4.03</v>
+        <v>2.31</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>MAZDA</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>40.38</v>
+        <v>229.69</v>
       </c>
       <c r="C152" t="n">
-        <v>42</v>
+        <v>234.99</v>
       </c>
       <c r="D152" t="n">
-        <v>4.01</v>
+        <v>2.31</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>VPRPL</t>
+          <t>ECOSMOBLTY</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>26.44</v>
+        <v>131.47</v>
       </c>
       <c r="C153" t="n">
-        <v>27.5</v>
+        <v>134.49</v>
       </c>
       <c r="D153" t="n">
-        <v>4.01</v>
+        <v>2.3</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SYSTMTXC</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>66.62</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="C154" t="n">
-        <v>69.29000000000001</v>
+        <v>95.55</v>
       </c>
       <c r="D154" t="n">
-        <v>4.01</v>
+        <v>2.3</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>ASHOKA</t>
+          <t>VCL</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>123.06</v>
+        <v>1.31</v>
       </c>
       <c r="C155" t="n">
-        <v>128</v>
+        <v>1.34</v>
       </c>
       <c r="D155" t="n">
-        <v>4.01</v>
+        <v>2.29</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>STCINDIA</t>
+          <t>RUBFILA</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>118.26</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="C156" t="n">
-        <v>123</v>
+        <v>73.8</v>
       </c>
       <c r="D156" t="n">
-        <v>4.01</v>
+        <v>2.29</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>HERANBA</t>
+          <t>TAKE</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>188.88</v>
+        <v>29.53</v>
       </c>
       <c r="C157" t="n">
-        <v>196.44</v>
+        <v>30.2</v>
       </c>
       <c r="D157" t="n">
-        <v>4</v>
+        <v>2.27</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>SAGCEM</t>
+          <t>5PAISA</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>167.46</v>
+        <v>316.8</v>
       </c>
       <c r="C158" t="n">
-        <v>174.15</v>
+        <v>323.9</v>
       </c>
       <c r="D158" t="n">
-        <v>3.99</v>
+        <v>2.24</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>VASWANI</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>359.75</v>
+        <v>59.37</v>
       </c>
       <c r="C159" t="n">
-        <v>374.05</v>
+        <v>60.7</v>
       </c>
       <c r="D159" t="n">
-        <v>3.97</v>
+        <v>2.24</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ATLANTAA</t>
+          <t>GICL</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>39.86</v>
+        <v>23.28</v>
       </c>
       <c r="C160" t="n">
-        <v>41.44</v>
+        <v>23.8</v>
       </c>
       <c r="D160" t="n">
-        <v>3.96</v>
+        <v>2.23</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>GULFPETRO</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>39.92</v>
+        <v>168.25</v>
       </c>
       <c r="C161" t="n">
-        <v>41.5</v>
+        <v>171.98</v>
       </c>
       <c r="D161" t="n">
-        <v>3.96</v>
+        <v>2.22</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>JKIL</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>458.9</v>
+        <v>0.45</v>
       </c>
       <c r="C162" t="n">
-        <v>476.95</v>
+        <v>0.46</v>
       </c>
       <c r="D162" t="n">
-        <v>3.93</v>
+        <v>2.22</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>SHEEL</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>0.51</v>
+        <v>63</v>
       </c>
       <c r="C163" t="n">
-        <v>0.53</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="D163" t="n">
-        <v>3.92</v>
+        <v>2.22</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>EIHAHOTELS</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>302.85</v>
+        <v>48.81</v>
       </c>
       <c r="C164" t="n">
-        <v>314.7</v>
+        <v>49.89</v>
       </c>
       <c r="D164" t="n">
-        <v>3.91</v>
+        <v>2.21</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>MATRIMONY</t>
+          <t>CEMPRO</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>390</v>
+        <v>1178.5</v>
       </c>
       <c r="C165" t="n">
-        <v>405.2</v>
+        <v>1204.6</v>
       </c>
       <c r="D165" t="n">
-        <v>3.9</v>
+        <v>2.21</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>STARPAPER</t>
+          <t>ANNAPURNA</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>135.55</v>
+        <v>134.1</v>
       </c>
       <c r="C166" t="n">
-        <v>140.8</v>
+        <v>137.05</v>
       </c>
       <c r="D166" t="n">
-        <v>3.87</v>
+        <v>2.2</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>KPEL</t>
+          <t>SUTLEJTEX</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>344.2</v>
+        <v>37.59</v>
       </c>
       <c r="C167" t="n">
-        <v>357.5</v>
+        <v>38.41</v>
       </c>
       <c r="D167" t="n">
-        <v>3.86</v>
+        <v>2.18</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>BCPL</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>77.03</v>
+        <v>44.92</v>
       </c>
       <c r="C168" t="n">
-        <v>80</v>
+        <v>45.9</v>
       </c>
       <c r="D168" t="n">
-        <v>3.86</v>
+        <v>2.18</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>381</v>
+        <v>616.6</v>
       </c>
       <c r="C169" t="n">
-        <v>395.65</v>
+        <v>630</v>
       </c>
       <c r="D169" t="n">
-        <v>3.85</v>
+        <v>2.17</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>VIDYAWIRES</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>570.35</v>
+        <v>93.53</v>
       </c>
       <c r="C170" t="n">
-        <v>592.25</v>
+        <v>95.55</v>
       </c>
       <c r="D170" t="n">
-        <v>3.84</v>
+        <v>2.16</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>DRONE</t>
+          <t>BANG</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>40.45</v>
+        <v>30.69</v>
       </c>
       <c r="C171" t="n">
-        <v>42</v>
+        <v>31.35</v>
       </c>
       <c r="D171" t="n">
-        <v>3.83</v>
+        <v>2.15</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>REMUS</t>
+          <t>TTKHLTCARE</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>696.35</v>
+        <v>878.15</v>
       </c>
       <c r="C172" t="n">
-        <v>722.85</v>
+        <v>897</v>
       </c>
       <c r="D172" t="n">
-        <v>3.81</v>
+        <v>2.15</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>GOKUL</t>
+          <t>NINSYS</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>40.66</v>
+        <v>704.25</v>
       </c>
       <c r="C173" t="n">
-        <v>42.2</v>
+        <v>719.3</v>
       </c>
       <c r="D173" t="n">
-        <v>3.79</v>
+        <v>2.14</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>APEX</t>
+          <t>LIKHITHA</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>419.15</v>
+        <v>232.09</v>
       </c>
       <c r="C174" t="n">
-        <v>435</v>
+        <v>237</v>
       </c>
       <c r="D174" t="n">
-        <v>3.78</v>
+        <v>2.12</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ACSTECH</t>
+          <t>TERASOFT</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>39.51</v>
+        <v>437.65</v>
       </c>
       <c r="C175" t="n">
-        <v>40.99</v>
+        <v>446.9</v>
       </c>
       <c r="D175" t="n">
-        <v>3.75</v>
+        <v>2.11</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>RVNL</t>
+          <t>AMIRCHAND</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>233.26</v>
+        <v>129.12</v>
       </c>
       <c r="C176" t="n">
-        <v>242</v>
+        <v>131.85</v>
       </c>
       <c r="D176" t="n">
-        <v>3.75</v>
+        <v>2.11</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>OBSCP</t>
+          <t>INSPIRISYS</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>539.75</v>
+        <v>112.62</v>
       </c>
       <c r="C177" t="n">
-        <v>560</v>
+        <v>115</v>
       </c>
       <c r="D177" t="n">
-        <v>3.75</v>
+        <v>2.11</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>EMBDL</t>
+          <t>KRITINUT</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>59.06</v>
+        <v>82.48</v>
       </c>
       <c r="C178" t="n">
-        <v>61.26</v>
+        <v>84.20999999999999</v>
       </c>
       <c r="D178" t="n">
-        <v>3.73</v>
+        <v>2.1</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>58.72</v>
+        <v>41.58</v>
       </c>
       <c r="C179" t="n">
-        <v>60.9</v>
+        <v>42.45</v>
       </c>
       <c r="D179" t="n">
-        <v>3.71</v>
+        <v>2.09</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ENIL</t>
+          <t>RCOM</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>109.92</v>
+        <v>0.96</v>
       </c>
       <c r="C180" t="n">
-        <v>114</v>
+        <v>0.98</v>
       </c>
       <c r="D180" t="n">
-        <v>3.71</v>
+        <v>2.08</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>GTL</t>
+          <t>SAKUMA</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>8.41</v>
+        <v>1.93</v>
       </c>
       <c r="C181" t="n">
-        <v>8.720000000000001</v>
+        <v>1.97</v>
       </c>
       <c r="D181" t="n">
-        <v>3.69</v>
+        <v>2.07</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>SCPL</t>
+          <t>WAAREEINDO</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>451.4</v>
+        <v>389.95</v>
       </c>
       <c r="C182" t="n">
-        <v>468</v>
+        <v>398</v>
       </c>
       <c r="D182" t="n">
-        <v>3.68</v>
+        <v>2.06</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>NINSYS</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>689.55</v>
+        <v>197.73</v>
       </c>
       <c r="C183" t="n">
-        <v>714.95</v>
+        <v>201.8</v>
       </c>
       <c r="D183" t="n">
-        <v>3.68</v>
+        <v>2.06</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>IFCI</t>
+          <t>MAHESHWARI</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>84.56999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="C184" t="n">
-        <v>87.67</v>
+        <v>72.95999999999999</v>
       </c>
       <c r="D184" t="n">
-        <v>3.67</v>
+        <v>2.04</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SSDL</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>54.98</v>
+        <v>28.91</v>
       </c>
       <c r="C185" t="n">
-        <v>56.99</v>
+        <v>29.5</v>
       </c>
       <c r="D185" t="n">
-        <v>3.66</v>
+        <v>2.04</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>SWANDEF</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>7.1</v>
+        <v>1998.2</v>
       </c>
       <c r="C186" t="n">
-        <v>7.36</v>
+        <v>2039</v>
       </c>
       <c r="D186" t="n">
-        <v>3.66</v>
+        <v>2.04</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>GOODYEAR</t>
+          <t>SNOWMAN</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>733</v>
+        <v>38.51</v>
       </c>
       <c r="C187" t="n">
-        <v>759.8</v>
+        <v>39.29</v>
       </c>
       <c r="D187" t="n">
-        <v>3.66</v>
+        <v>2.03</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>AEROFLEX</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>66.56</v>
+        <v>478</v>
       </c>
       <c r="C188" t="n">
-        <v>68.98999999999999</v>
+        <v>487.65</v>
       </c>
       <c r="D188" t="n">
-        <v>3.65</v>
+        <v>2.02</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>HARIOMPIPE</t>
+          <t>JAYSREETEA</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>408.2</v>
+        <v>88.13</v>
       </c>
       <c r="C189" t="n">
-        <v>423.1</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="D189" t="n">
-        <v>3.65</v>
+        <v>2.01</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>RAILTEL</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>308.75</v>
+        <v>7.45</v>
       </c>
       <c r="C190" t="n">
-        <v>320</v>
+        <v>7.6</v>
       </c>
       <c r="D190" t="n">
-        <v>3.64</v>
+        <v>2.01</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>BOSCH-HCIL</t>
+          <t>GLOSTERLTD</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>1331.7</v>
+        <v>680.85</v>
       </c>
       <c r="C191" t="n">
-        <v>1380</v>
+        <v>694.5</v>
       </c>
       <c r="D191" t="n">
-        <v>3.63</v>
+        <v>2</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>PONNIERODE</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>14.38</v>
+        <v>320.1</v>
       </c>
       <c r="C192" t="n">
-        <v>14.9</v>
+        <v>326.5</v>
       </c>
       <c r="D192" t="n">
-        <v>3.62</v>
+        <v>2</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>MERCANTILE</t>
+          <t>BROOKS</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>25.77</v>
+        <v>67.55</v>
       </c>
       <c r="C193" t="n">
-        <v>26.7</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D193" t="n">
-        <v>3.61</v>
+        <v>2</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>GOCOLORS</t>
+          <t>ALPEXSOLAR</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>358.65</v>
+        <v>990.1</v>
       </c>
       <c r="C194" t="n">
-        <v>371.55</v>
+        <v>1009.9</v>
       </c>
       <c r="D194" t="n">
-        <v>3.6</v>
+        <v>2</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>KRBL</t>
+          <t>IWP</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>366.8</v>
+        <v>33.6</v>
       </c>
       <c r="C195" t="n">
-        <v>380</v>
+        <v>34.27</v>
       </c>
       <c r="D195" t="n">
-        <v>3.6</v>
+        <v>1.99</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>EPACKPEB</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>241.17</v>
+        <v>51.16</v>
       </c>
       <c r="C196" t="n">
-        <v>249.86</v>
+        <v>52.18</v>
       </c>
       <c r="D196" t="n">
-        <v>3.6</v>
+        <v>1.99</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>CORALFINAC</t>
+          <t>TRIGYN</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>31.47</v>
+        <v>55.7</v>
       </c>
       <c r="C197" t="n">
-        <v>32.6</v>
+        <v>56.8</v>
       </c>
       <c r="D197" t="n">
-        <v>3.59</v>
+        <v>1.97</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>NIPPOBATRY</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>40.64</v>
+        <v>356</v>
       </c>
       <c r="C198" t="n">
-        <v>42.1</v>
+        <v>363</v>
       </c>
       <c r="D198" t="n">
-        <v>3.59</v>
+        <v>1.97</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>3.9</v>
+        <v>180.45</v>
       </c>
       <c r="C199" t="n">
-        <v>4.04</v>
+        <v>184</v>
       </c>
       <c r="D199" t="n">
-        <v>3.59</v>
+        <v>1.97</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>ASTRON</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>3.9</v>
+        <v>0.51</v>
       </c>
       <c r="C200" t="n">
-        <v>4.04</v>
+        <v>0.52</v>
       </c>
       <c r="D200" t="n">
-        <v>3.59</v>
+        <v>1.96</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>BRNL</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>19.01</v>
+        <v>1119.3</v>
       </c>
       <c r="C201" t="n">
-        <v>19.69</v>
+        <v>1141</v>
       </c>
       <c r="D201" t="n">
-        <v>3.58</v>
+        <v>1.94</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-17 08:51 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -465,13 +465,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MCLOUD</t>
+          <t>COMFINTE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>26.66</v>
+        <v>5.87</v>
       </c>
       <c r="C3" t="n">
-        <v>28.97</v>
+        <v>7.04</v>
       </c>
       <c r="D3" t="n">
-        <v>8.66</v>
+        <v>19.93</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>36.21</v>
+        <v>39.83</v>
       </c>
       <c r="C4" t="n">
-        <v>38.99</v>
+        <v>43.78</v>
       </c>
       <c r="D4" t="n">
-        <v>7.68</v>
+        <v>9.92</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.61</v>
+        <v>6.03</v>
       </c>
       <c r="C5" t="n">
-        <v>6.04</v>
+        <v>6.59</v>
       </c>
       <c r="D5" t="n">
-        <v>7.66</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>INDPRUD</t>
+          <t>SARTELE</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6271</v>
+        <v>160.2</v>
       </c>
       <c r="C6" t="n">
-        <v>6748</v>
+        <v>174.9</v>
       </c>
       <c r="D6" t="n">
-        <v>7.61</v>
+        <v>9.18</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NIRAJISPAT</t>
+          <t>K2INFRA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>194.83</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>207</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>6.25</v>
+        <v>7.33</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>ONMOBILE</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.16</v>
+        <v>51.3</v>
       </c>
       <c r="C8" t="n">
-        <v>0.17</v>
+        <v>54.76</v>
       </c>
       <c r="D8" t="n">
-        <v>6.25</v>
+        <v>6.74</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>BABAFP</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6.89</v>
+        <v>23.75</v>
       </c>
       <c r="C9" t="n">
-        <v>7.31</v>
+        <v>25.25</v>
       </c>
       <c r="D9" t="n">
-        <v>6.1</v>
+        <v>6.32</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NDGL</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2642</v>
+        <v>0.16</v>
       </c>
       <c r="C10" t="n">
-        <v>2779</v>
+        <v>0.17</v>
       </c>
       <c r="D10" t="n">
-        <v>5.19</v>
+        <v>6.25</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>QMSMEDI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.79</v>
+        <v>97</v>
       </c>
       <c r="C11" t="n">
-        <v>0.83</v>
+        <v>102.9</v>
       </c>
       <c r="D11" t="n">
-        <v>5.06</v>
+        <v>6.08</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MANORG</t>
+          <t>RSDFIN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>494</v>
+        <v>82</v>
       </c>
       <c r="C12" t="n">
-        <v>518.7</v>
+        <v>86.98</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>6.07</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>SINCLAIR</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.2</v>
+        <v>76.22</v>
       </c>
       <c r="C13" t="n">
-        <v>0.21</v>
+        <v>80.68000000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>5.85</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>WTICAB</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>296.2</v>
+        <v>98.5</v>
       </c>
       <c r="C14" t="n">
-        <v>311</v>
+        <v>104</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>5.58</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DEEDEV</t>
+          <t>AAATECH</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>689.5</v>
+        <v>96.68000000000001</v>
       </c>
       <c r="C15" t="n">
-        <v>723.95</v>
+        <v>102</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TECHERA</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>154.1</v>
+        <v>8</v>
       </c>
       <c r="C16" t="n">
-        <v>161.8</v>
+        <v>8.44</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>VISL</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>21.06</v>
+        <v>25.61</v>
       </c>
       <c r="C17" t="n">
-        <v>22.11</v>
+        <v>26.97</v>
       </c>
       <c r="D17" t="n">
-        <v>4.99</v>
+        <v>5.31</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SUBEXLTD</t>
+          <t>SOMATEX</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11.03</v>
+        <v>97.68000000000001</v>
       </c>
       <c r="C18" t="n">
-        <v>11.58</v>
+        <v>102.7</v>
       </c>
       <c r="D18" t="n">
-        <v>4.99</v>
+        <v>5.14</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,17 +835,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ACCORD</t>
+          <t>RAJESHEXPO</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>90.40000000000001</v>
+        <v>84.23999999999999</v>
       </c>
       <c r="C19" t="n">
-        <v>94.90000000000001</v>
+        <v>88.45</v>
       </c>
       <c r="D19" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -857,17 +857,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SHYAMTEL</t>
+          <t>SICALLOG</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>15.65</v>
+        <v>92.04000000000001</v>
       </c>
       <c r="C20" t="n">
-        <v>16.43</v>
+        <v>96.64</v>
       </c>
       <c r="D20" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -879,17 +879,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GANESHIN</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>98.40000000000001</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>103.3</v>
+        <v>2.1</v>
       </c>
       <c r="D21" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>PFOCUS</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>22.95</v>
+        <v>234.15</v>
       </c>
       <c r="C22" t="n">
-        <v>24.09</v>
+        <v>245.85</v>
       </c>
       <c r="D22" t="n">
-        <v>4.97</v>
+        <v>5</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>VPRPL</t>
+          <t>SEJALLTD</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>27.76</v>
+        <v>725</v>
       </c>
       <c r="C23" t="n">
-        <v>29.14</v>
+        <v>761.25</v>
       </c>
       <c r="D23" t="n">
-        <v>4.97</v>
+        <v>5</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,17 +945,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SMARTLINK</t>
+          <t>PALREDTEC</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>164.4</v>
+        <v>48.31</v>
       </c>
       <c r="C24" t="n">
-        <v>172.55</v>
+        <v>50.72</v>
       </c>
       <c r="D24" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -967,17 +967,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>UHTL</t>
+          <t>GANESHIN</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>108.85</v>
+        <v>103.3</v>
       </c>
       <c r="C25" t="n">
-        <v>114.25</v>
+        <v>108.45</v>
       </c>
       <c r="D25" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -989,17 +989,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>OWAIS</t>
+          <t>MASKINVEST</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>98.90000000000001</v>
+        <v>155.39</v>
       </c>
       <c r="C26" t="n">
-        <v>103.8</v>
+        <v>163.15</v>
       </c>
       <c r="D26" t="n">
-        <v>4.95</v>
+        <v>4.99</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SICALLOG</t>
+          <t>UNIHEALTH</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>87.66</v>
+        <v>521.75</v>
       </c>
       <c r="C27" t="n">
-        <v>92</v>
+        <v>547.8</v>
       </c>
       <c r="D27" t="n">
-        <v>4.95</v>
+        <v>4.99</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>KESORAMIND</t>
+          <t>MANORG</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>11.52</v>
+        <v>518.7</v>
       </c>
       <c r="C28" t="n">
-        <v>12.09</v>
+        <v>544.6</v>
       </c>
       <c r="D28" t="n">
-        <v>4.95</v>
+        <v>4.99</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BLUEWATER</t>
+          <t>SIGNORIA</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>328.8</v>
+        <v>76.2</v>
       </c>
       <c r="C29" t="n">
-        <v>345</v>
+        <v>80</v>
       </c>
       <c r="D29" t="n">
-        <v>4.93</v>
+        <v>4.99</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LAXMICOT</t>
+          <t>VPRPL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>14.2</v>
+        <v>29.14</v>
       </c>
       <c r="C30" t="n">
-        <v>14.9</v>
+        <v>30.59</v>
       </c>
       <c r="D30" t="n">
-        <v>4.93</v>
+        <v>4.98</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IL&amp;FSTRANS</t>
+          <t>NIRAJ</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2.44</v>
+        <v>29.53</v>
       </c>
       <c r="C31" t="n">
-        <v>2.56</v>
+        <v>31</v>
       </c>
       <c r="D31" t="n">
-        <v>4.92</v>
+        <v>4.98</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CRAYONS</t>
+          <t>GAYAPROJ</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>30.5</v>
+        <v>24.09</v>
       </c>
       <c r="C32" t="n">
-        <v>32</v>
+        <v>25.29</v>
       </c>
       <c r="D32" t="n">
-        <v>4.92</v>
+        <v>4.98</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CEREBRAINT</t>
+          <t>TECHERA</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3.86</v>
+        <v>161.8</v>
       </c>
       <c r="C33" t="n">
-        <v>4.05</v>
+        <v>169.85</v>
       </c>
       <c r="D33" t="n">
-        <v>4.92</v>
+        <v>4.98</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>VISHWAS</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>46.9</v>
+        <v>20.53</v>
       </c>
       <c r="C34" t="n">
-        <v>49.2</v>
+        <v>21.55</v>
       </c>
       <c r="D34" t="n">
-        <v>4.9</v>
+        <v>4.97</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SAMAY</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>40.85</v>
+        <v>103.8</v>
       </c>
       <c r="C35" t="n">
-        <v>42.85</v>
+        <v>108.95</v>
       </c>
       <c r="D35" t="n">
-        <v>4.9</v>
+        <v>4.96</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SRIVASAVI</t>
+          <t>ORTEL</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>55.3</v>
+        <v>1.62</v>
       </c>
       <c r="C36" t="n">
-        <v>58</v>
+        <v>1.7</v>
       </c>
       <c r="D36" t="n">
-        <v>4.88</v>
+        <v>4.94</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>PROLIFE</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>47.7</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="C37" t="n">
-        <v>50</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="D37" t="n">
-        <v>4.82</v>
+        <v>4.93</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FABTECH</t>
+          <t>INNOMET</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>145.96</v>
+        <v>106.6</v>
       </c>
       <c r="C38" t="n">
-        <v>153</v>
+        <v>111.85</v>
       </c>
       <c r="D38" t="n">
-        <v>4.82</v>
+        <v>4.92</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CALSOFT</t>
+          <t>SUBEXLTD</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>20.94</v>
+        <v>11.58</v>
       </c>
       <c r="C39" t="n">
-        <v>21.95</v>
+        <v>12.15</v>
       </c>
       <c r="D39" t="n">
-        <v>4.82</v>
+        <v>4.92</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DIVINEHIRA</t>
+          <t>IEML</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>314.95</v>
+        <v>50.05</v>
       </c>
       <c r="C40" t="n">
-        <v>330</v>
+        <v>52.5</v>
       </c>
       <c r="D40" t="n">
-        <v>4.78</v>
+        <v>4.9</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>AILIMITED</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>72.54000000000001</v>
+        <v>37.9</v>
       </c>
       <c r="C41" t="n">
-        <v>76</v>
+        <v>39.75</v>
       </c>
       <c r="D41" t="n">
-        <v>4.77</v>
+        <v>4.88</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>SADHNANIQ</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>3.79</v>
+        <v>2.49</v>
       </c>
       <c r="C42" t="n">
-        <v>3.97</v>
+        <v>2.61</v>
       </c>
       <c r="D42" t="n">
-        <v>4.75</v>
+        <v>4.82</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>GOLDENTOBC</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>155.57</v>
+        <v>25.09</v>
       </c>
       <c r="C43" t="n">
-        <v>162.95</v>
+        <v>26.29</v>
       </c>
       <c r="D43" t="n">
-        <v>4.74</v>
+        <v>4.78</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ARVSMART</t>
+          <t>SARVESHWAR</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>594.65</v>
+        <v>3.78</v>
       </c>
       <c r="C44" t="n">
-        <v>622.8</v>
+        <v>3.96</v>
       </c>
       <c r="D44" t="n">
-        <v>4.73</v>
+        <v>4.76</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TRIDHYA</t>
+          <t>MAL</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>10.6</v>
+        <v>32</v>
       </c>
       <c r="C45" t="n">
-        <v>11.1</v>
+        <v>33.5</v>
       </c>
       <c r="D45" t="n">
-        <v>4.72</v>
+        <v>4.69</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SARVESHWAR</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3.6</v>
+        <v>180.11</v>
       </c>
       <c r="C46" t="n">
-        <v>3.77</v>
+        <v>188.5</v>
       </c>
       <c r="D46" t="n">
-        <v>4.72</v>
+        <v>4.66</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>ARVINDPORT</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>11.27</v>
+        <v>28.2</v>
       </c>
       <c r="C47" t="n">
-        <v>11.8</v>
+        <v>29.5</v>
       </c>
       <c r="D47" t="n">
-        <v>4.7</v>
+        <v>4.61</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SEJALLTD</t>
+          <t>HMT</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>690.5</v>
+        <v>55.94</v>
       </c>
       <c r="C48" t="n">
-        <v>722.8</v>
+        <v>58.5</v>
       </c>
       <c r="D48" t="n">
-        <v>4.68</v>
+        <v>4.58</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SADHNANIQ</t>
+          <t>TBI</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2.38</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C49" t="n">
-        <v>2.49</v>
+        <v>68</v>
       </c>
       <c r="D49" t="n">
-        <v>4.62</v>
+        <v>4.37</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>UMAEXPORTS</t>
+          <t>RRIL</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>23.9</v>
+        <v>19.84</v>
       </c>
       <c r="C50" t="n">
-        <v>25</v>
+        <v>20.7</v>
       </c>
       <c r="D50" t="n">
-        <v>4.6</v>
+        <v>4.33</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>KESORAMIND</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2.84</v>
+        <v>12.09</v>
       </c>
       <c r="C51" t="n">
-        <v>2.97</v>
+        <v>12.59</v>
       </c>
       <c r="D51" t="n">
-        <v>4.58</v>
+        <v>4.14</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SANWARIA</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.22</v>
+        <v>162.88</v>
       </c>
       <c r="C52" t="n">
-        <v>0.23</v>
+        <v>169.44</v>
       </c>
       <c r="D52" t="n">
-        <v>4.55</v>
+        <v>4.03</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>RVTH</t>
+          <t>MITCON</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>688.95</v>
+        <v>79.51000000000001</v>
       </c>
       <c r="C53" t="n">
-        <v>720</v>
+        <v>82.68000000000001</v>
       </c>
       <c r="D53" t="n">
-        <v>4.51</v>
+        <v>3.99</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MANGALAM</t>
+          <t>LEXUS</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>29.58</v>
+        <v>15.86</v>
       </c>
       <c r="C54" t="n">
-        <v>30.89</v>
+        <v>16.49</v>
       </c>
       <c r="D54" t="n">
-        <v>4.43</v>
+        <v>3.97</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>3.24</v>
+        <v>21.18</v>
       </c>
       <c r="C55" t="n">
-        <v>3.38</v>
+        <v>22</v>
       </c>
       <c r="D55" t="n">
-        <v>4.32</v>
+        <v>3.87</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MUKTAARTS</t>
+          <t>JETFREIGHT</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>63.1</v>
+        <v>21.63</v>
       </c>
       <c r="C56" t="n">
-        <v>65.8</v>
+        <v>22.45</v>
       </c>
       <c r="D56" t="n">
-        <v>4.28</v>
+        <v>3.79</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>RUSHIL</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>17.89</v>
+        <v>73.2</v>
       </c>
       <c r="C57" t="n">
-        <v>18.65</v>
+        <v>75.94</v>
       </c>
       <c r="D57" t="n">
-        <v>4.25</v>
+        <v>3.74</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>USK</t>
+          <t>IDEAFORGE</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>24.72</v>
+        <v>908.05</v>
       </c>
       <c r="C58" t="n">
-        <v>25.74</v>
+        <v>942</v>
       </c>
       <c r="D58" t="n">
-        <v>4.13</v>
+        <v>3.74</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DAICHI</t>
+          <t>SBGLP</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>265.15</v>
+        <v>26.01</v>
       </c>
       <c r="C59" t="n">
-        <v>276</v>
+        <v>26.98</v>
       </c>
       <c r="D59" t="n">
-        <v>4.09</v>
+        <v>3.73</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SHETHJI</t>
+          <t>HIGREEN</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>160.2</v>
+        <v>137.85</v>
       </c>
       <c r="C60" t="n">
-        <v>166.7</v>
+        <v>142.95</v>
       </c>
       <c r="D60" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TAALTECH</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>3363.4</v>
+        <v>9.35</v>
       </c>
       <c r="C61" t="n">
-        <v>3500</v>
+        <v>9.69</v>
       </c>
       <c r="D61" t="n">
-        <v>4.06</v>
+        <v>3.64</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASPINWALL</t>
+          <t>INCREDIBLE</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>259.29</v>
+        <v>34.84</v>
       </c>
       <c r="C62" t="n">
-        <v>269.7</v>
+        <v>36.1</v>
       </c>
       <c r="D62" t="n">
-        <v>4.01</v>
+        <v>3.62</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>SIGMA</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>373</v>
+        <v>39.1</v>
       </c>
       <c r="C63" t="n">
-        <v>387.95</v>
+        <v>40.51</v>
       </c>
       <c r="D63" t="n">
-        <v>4.01</v>
+        <v>3.61</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>IRMENERGY</t>
+          <t>BCONCEPTS</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>280.9</v>
+        <v>175.1</v>
       </c>
       <c r="C64" t="n">
-        <v>292</v>
+        <v>181.2</v>
       </c>
       <c r="D64" t="n">
-        <v>3.95</v>
+        <v>3.48</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PATELENG</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>27.65</v>
+        <v>7.2</v>
       </c>
       <c r="C65" t="n">
-        <v>28.74</v>
+        <v>7.45</v>
       </c>
       <c r="D65" t="n">
-        <v>3.94</v>
+        <v>3.47</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>AARTECH</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>7.17</v>
+        <v>49.05</v>
       </c>
       <c r="C66" t="n">
-        <v>7.45</v>
+        <v>50.75</v>
       </c>
       <c r="D66" t="n">
-        <v>3.91</v>
+        <v>3.47</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>MITTAL</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1.04</v>
+        <v>5.79</v>
       </c>
       <c r="C67" t="n">
-        <v>1.08</v>
+        <v>5.99</v>
       </c>
       <c r="D67" t="n">
-        <v>3.85</v>
+        <v>3.45</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>LATTEYS</t>
+          <t>NAGREEKCAP</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>22.1</v>
+        <v>29</v>
       </c>
       <c r="C68" t="n">
-        <v>22.95</v>
+        <v>30</v>
       </c>
       <c r="D68" t="n">
-        <v>3.85</v>
+        <v>3.45</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>5.74</v>
+        <v>572.4</v>
       </c>
       <c r="C69" t="n">
-        <v>5.96</v>
+        <v>592</v>
       </c>
       <c r="D69" t="n">
-        <v>3.83</v>
+        <v>3.42</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>LAGNAM</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>82.69</v>
+        <v>80.84</v>
       </c>
       <c r="C70" t="n">
-        <v>85.7</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="D70" t="n">
-        <v>3.64</v>
+        <v>3.41</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TREEHOUSE</t>
+          <t>AMDIND</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>7.05</v>
+        <v>47.29</v>
       </c>
       <c r="C71" t="n">
-        <v>7.3</v>
+        <v>48.9</v>
       </c>
       <c r="D71" t="n">
-        <v>3.55</v>
+        <v>3.4</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>MADHAVIPL</t>
+          <t>RVTH</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>9.35</v>
+        <v>705.15</v>
       </c>
       <c r="C72" t="n">
-        <v>9.68</v>
+        <v>728.95</v>
       </c>
       <c r="D72" t="n">
-        <v>3.53</v>
+        <v>3.38</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>JAYBARMARU</t>
+          <t>FLYSBS</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>159.12</v>
+        <v>456.6</v>
       </c>
       <c r="C73" t="n">
-        <v>164.69</v>
+        <v>472</v>
       </c>
       <c r="D73" t="n">
-        <v>3.5</v>
+        <v>3.37</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>TRANSPEK</t>
+          <t>CHAMUNDA</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>981.1</v>
+        <v>39.2</v>
       </c>
       <c r="C74" t="n">
-        <v>1015.4</v>
+        <v>40.5</v>
       </c>
       <c r="D74" t="n">
-        <v>3.5</v>
+        <v>3.32</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>19.56</v>
+        <v>1227.6</v>
       </c>
       <c r="C75" t="n">
-        <v>20.24</v>
+        <v>1268</v>
       </c>
       <c r="D75" t="n">
-        <v>3.48</v>
+        <v>3.29</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SINTERCOM</t>
+          <t>EXXARO</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>72.38</v>
+        <v>6.78</v>
       </c>
       <c r="C76" t="n">
-        <v>74.90000000000001</v>
+        <v>7</v>
       </c>
       <c r="D76" t="n">
-        <v>3.48</v>
+        <v>3.24</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>REGENCERAM</t>
+          <t>LIBAS</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>40.79</v>
+        <v>11.91</v>
       </c>
       <c r="C77" t="n">
-        <v>42.2</v>
+        <v>12.29</v>
       </c>
       <c r="D77" t="n">
-        <v>3.46</v>
+        <v>3.19</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>UNIENTER</t>
+          <t>EMAMIREAL</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>108.64</v>
+        <v>92.05</v>
       </c>
       <c r="C78" t="n">
-        <v>112.4</v>
+        <v>94.98</v>
       </c>
       <c r="D78" t="n">
-        <v>3.46</v>
+        <v>3.18</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>HGM</t>
+          <t>ARCHIDPLY</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>53.75</v>
+        <v>81.34</v>
       </c>
       <c r="C79" t="n">
-        <v>55.6</v>
+        <v>83.92</v>
       </c>
       <c r="D79" t="n">
-        <v>3.44</v>
+        <v>3.17</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>DAMODARIND</t>
+          <t>GFLLIMITED</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>30.75</v>
+        <v>47.11</v>
       </c>
       <c r="C80" t="n">
-        <v>31.8</v>
+        <v>48.6</v>
       </c>
       <c r="D80" t="n">
-        <v>3.41</v>
+        <v>3.16</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>AAKASH</t>
+          <t>CYBERTECH</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>9.720000000000001</v>
+        <v>143.53</v>
       </c>
       <c r="C81" t="n">
-        <v>10.05</v>
+        <v>147.99</v>
       </c>
       <c r="D81" t="n">
-        <v>3.4</v>
+        <v>3.11</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>AGARIND</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>580.25</v>
+        <v>17.66</v>
       </c>
       <c r="C82" t="n">
-        <v>600</v>
+        <v>18.2</v>
       </c>
       <c r="D82" t="n">
-        <v>3.4</v>
+        <v>3.06</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>BI</t>
+          <t>JKIPL</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>58.87</v>
+        <v>113.05</v>
       </c>
       <c r="C83" t="n">
-        <v>60.87</v>
+        <v>116.5</v>
       </c>
       <c r="D83" t="n">
-        <v>3.4</v>
+        <v>3.05</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SHREEOSFM</t>
+          <t>LEMERITE</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>59</v>
+        <v>28.51</v>
       </c>
       <c r="C84" t="n">
-        <v>61</v>
+        <v>29.38</v>
       </c>
       <c r="D84" t="n">
-        <v>3.39</v>
+        <v>3.05</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>OSELDEVICE</t>
+          <t>TARSONS</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>480</v>
+        <v>238.73</v>
       </c>
       <c r="C85" t="n">
-        <v>496</v>
+        <v>246</v>
       </c>
       <c r="D85" t="n">
-        <v>3.33</v>
+        <v>3.05</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>MGSL</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>60</v>
+        <v>3.97</v>
       </c>
       <c r="C86" t="n">
-        <v>62</v>
+        <v>4.09</v>
       </c>
       <c r="D86" t="n">
-        <v>3.33</v>
+        <v>3.02</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>LAXMIINDIA</t>
+          <t>TRIGYN</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>109.88</v>
+        <v>55.34</v>
       </c>
       <c r="C87" t="n">
-        <v>113.5</v>
+        <v>57</v>
       </c>
       <c r="D87" t="n">
-        <v>3.29</v>
+        <v>3</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SARTELE</t>
+          <t>ORBTEXP</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>133.5</v>
+        <v>229.16</v>
       </c>
       <c r="C88" t="n">
-        <v>137.85</v>
+        <v>235.99</v>
       </c>
       <c r="D88" t="n">
-        <v>3.26</v>
+        <v>2.98</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HARRMALAYA</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>207.26</v>
+        <v>2.03</v>
       </c>
       <c r="C89" t="n">
-        <v>213.99</v>
+        <v>2.09</v>
       </c>
       <c r="D89" t="n">
-        <v>3.25</v>
+        <v>2.96</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>24.63</v>
+        <v>45.17</v>
       </c>
       <c r="C90" t="n">
-        <v>25.43</v>
+        <v>46.5</v>
       </c>
       <c r="D90" t="n">
-        <v>3.25</v>
+        <v>2.94</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>RAJESHEXPO</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>80.23</v>
+        <v>311</v>
       </c>
       <c r="C91" t="n">
-        <v>82.8</v>
+        <v>320</v>
       </c>
       <c r="D91" t="n">
-        <v>3.2</v>
+        <v>2.89</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>VARDMNPOLY</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>20.64</v>
+        <v>7</v>
       </c>
       <c r="C92" t="n">
-        <v>21.3</v>
+        <v>7.2</v>
       </c>
       <c r="D92" t="n">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>EUROBOND</t>
+          <t>ORIENTLTD</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>174.46</v>
+        <v>63.1</v>
       </c>
       <c r="C93" t="n">
-        <v>180</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="D93" t="n">
-        <v>3.18</v>
+        <v>2.85</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>K2INFRA</t>
+          <t>ELGIRUBCO</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>60.3</v>
+        <v>49.55</v>
       </c>
       <c r="C94" t="n">
-        <v>62.2</v>
+        <v>50.95</v>
       </c>
       <c r="D94" t="n">
-        <v>3.15</v>
+        <v>2.83</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>BBTCL</t>
+          <t>CORONA</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>219.3</v>
+        <v>1750.6</v>
       </c>
       <c r="C95" t="n">
-        <v>226.2</v>
+        <v>1800</v>
       </c>
       <c r="D95" t="n">
-        <v>3.15</v>
+        <v>2.82</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>BODALCHEM</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>326.1</v>
+        <v>65.38</v>
       </c>
       <c r="C96" t="n">
-        <v>336.3</v>
+        <v>67.2</v>
       </c>
       <c r="D96" t="n">
-        <v>3.13</v>
+        <v>2.78</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>TNTELE</t>
+          <t>DBEIL</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>9.300000000000001</v>
+        <v>86.81</v>
       </c>
       <c r="C97" t="n">
-        <v>9.59</v>
+        <v>89.2</v>
       </c>
       <c r="D97" t="n">
-        <v>3.12</v>
+        <v>2.75</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>GANGAFORGE</t>
+          <t>BESTAGRO</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>2.57</v>
+        <v>15.96</v>
       </c>
       <c r="C98" t="n">
-        <v>2.65</v>
+        <v>16.39</v>
       </c>
       <c r="D98" t="n">
-        <v>3.11</v>
+        <v>2.69</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ARIHANT</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>873.55</v>
+        <v>51.37</v>
       </c>
       <c r="C99" t="n">
-        <v>900</v>
+        <v>52.74</v>
       </c>
       <c r="D99" t="n">
-        <v>3.03</v>
+        <v>2.67</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>DMCC</t>
+          <t>BIRLAPREC</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>256.25</v>
+        <v>37.78</v>
       </c>
       <c r="C100" t="n">
-        <v>264</v>
+        <v>38.79</v>
       </c>
       <c r="D100" t="n">
-        <v>3.02</v>
+        <v>2.67</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>XPROINDIA</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>7.48</v>
+        <v>1393.8</v>
       </c>
       <c r="C101" t="n">
-        <v>7.7</v>
+        <v>1431</v>
       </c>
       <c r="D101" t="n">
-        <v>2.94</v>
+        <v>2.67</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>C2C</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>422.6</v>
+        <v>19</v>
       </c>
       <c r="C102" t="n">
-        <v>435</v>
+        <v>19.5</v>
       </c>
       <c r="D102" t="n">
-        <v>2.93</v>
+        <v>2.63</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SELMC</t>
+          <t>ALPA</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>30.12</v>
+        <v>70.55</v>
       </c>
       <c r="C103" t="n">
-        <v>31</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D103" t="n">
-        <v>2.92</v>
+        <v>2.62</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>NAVKARURB</t>
+          <t>VARDHACRLC</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>1.03</v>
+        <v>44.71</v>
       </c>
       <c r="C104" t="n">
-        <v>1.06</v>
+        <v>45.88</v>
       </c>
       <c r="D104" t="n">
-        <v>2.91</v>
+        <v>2.62</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ASHOKAMET</t>
+          <t>AARON</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>15.2</v>
+        <v>124.45</v>
       </c>
       <c r="C105" t="n">
-        <v>15.64</v>
+        <v>127.7</v>
       </c>
       <c r="D105" t="n">
-        <v>2.89</v>
+        <v>2.61</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MEGASTAR</t>
+          <t>SAKUMA</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>325.6</v>
+        <v>1.93</v>
       </c>
       <c r="C106" t="n">
-        <v>335</v>
+        <v>1.98</v>
       </c>
       <c r="D106" t="n">
-        <v>2.89</v>
+        <v>2.59</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>SUVIDHAA</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>976</v>
+        <v>2.71</v>
       </c>
       <c r="C107" t="n">
-        <v>1004</v>
+        <v>2.78</v>
       </c>
       <c r="D107" t="n">
-        <v>2.87</v>
+        <v>2.58</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>VINYAS</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>1404.95</v>
+        <v>11.25</v>
       </c>
       <c r="C108" t="n">
-        <v>1445</v>
+        <v>11.54</v>
       </c>
       <c r="D108" t="n">
-        <v>2.85</v>
+        <v>2.58</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>SURAKSHA</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>3.9</v>
+        <v>270.05</v>
       </c>
       <c r="C109" t="n">
-        <v>4.01</v>
+        <v>277</v>
       </c>
       <c r="D109" t="n">
-        <v>2.82</v>
+        <v>2.57</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SITINET</t>
+          <t>AMBALALSA</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.36</v>
+        <v>32.18</v>
       </c>
       <c r="C110" t="n">
-        <v>0.37</v>
+        <v>33</v>
       </c>
       <c r="D110" t="n">
-        <v>2.78</v>
+        <v>2.55</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>NOIDATOLL</t>
+          <t>DAICHI</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>5.05</v>
+        <v>284.55</v>
       </c>
       <c r="C111" t="n">
-        <v>5.19</v>
+        <v>291.79</v>
       </c>
       <c r="D111" t="n">
-        <v>2.77</v>
+        <v>2.54</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>1.1</v>
+        <v>3.15</v>
       </c>
       <c r="C112" t="n">
-        <v>1.13</v>
+        <v>3.23</v>
       </c>
       <c r="D112" t="n">
-        <v>2.73</v>
+        <v>2.54</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SEPC</t>
+          <t>VASWANI</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>7.34</v>
+        <v>58.52</v>
       </c>
       <c r="C113" t="n">
-        <v>7.54</v>
+        <v>60</v>
       </c>
       <c r="D113" t="n">
-        <v>2.72</v>
+        <v>2.53</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SAGARDEEP</t>
+          <t>CORALFINAC</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>25.22</v>
+        <v>32.18</v>
       </c>
       <c r="C114" t="n">
-        <v>25.9</v>
+        <v>32.99</v>
       </c>
       <c r="D114" t="n">
-        <v>2.7</v>
+        <v>2.52</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SUKHJITS</t>
+          <t>ALANKIT</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>170.2</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="C115" t="n">
-        <v>174.8</v>
+        <v>8.57</v>
       </c>
       <c r="D115" t="n">
-        <v>2.7</v>
+        <v>2.51</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SAHANA</t>
+          <t>NILAINFRA</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>802.55</v>
+        <v>7.99</v>
       </c>
       <c r="C116" t="n">
-        <v>824</v>
+        <v>8.19</v>
       </c>
       <c r="D116" t="n">
-        <v>2.67</v>
+        <v>2.5</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>WEWIN</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>45.29</v>
+        <v>50.48</v>
       </c>
       <c r="C117" t="n">
-        <v>46.49</v>
+        <v>51.74</v>
       </c>
       <c r="D117" t="n">
-        <v>2.65</v>
+        <v>2.5</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SHAH</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>4.93</v>
+        <v>6.41</v>
       </c>
       <c r="C118" t="n">
-        <v>5.06</v>
+        <v>6.57</v>
       </c>
       <c r="D118" t="n">
-        <v>2.64</v>
+        <v>2.5</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>UNIHEALTH</t>
+          <t>ONELIFECAP</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>496.95</v>
+        <v>28.08</v>
       </c>
       <c r="C119" t="n">
-        <v>510</v>
+        <v>28.78</v>
       </c>
       <c r="D119" t="n">
-        <v>2.63</v>
+        <v>2.49</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>AFFLE</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>1486.4</v>
+        <v>7.67</v>
       </c>
       <c r="C120" t="n">
-        <v>1525</v>
+        <v>7.86</v>
       </c>
       <c r="D120" t="n">
-        <v>2.6</v>
+        <v>2.48</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>ANTGRAPHIC</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>11.2</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C121" t="n">
-        <v>11.49</v>
+        <v>0.83</v>
       </c>
       <c r="D121" t="n">
-        <v>2.59</v>
+        <v>2.47</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>RELIABLE</t>
+          <t>AVG</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>154.91</v>
+        <v>169.83</v>
       </c>
       <c r="C122" t="n">
-        <v>158.9</v>
+        <v>174</v>
       </c>
       <c r="D122" t="n">
-        <v>2.58</v>
+        <v>2.46</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IGARASHI</t>
+          <t>FINKURVE</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>378.25</v>
+        <v>71.27</v>
       </c>
       <c r="C123" t="n">
-        <v>388</v>
+        <v>73.02</v>
       </c>
       <c r="D123" t="n">
-        <v>2.58</v>
+        <v>2.46</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>STERTOOLS</t>
+          <t>SJLOGISTIC</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>239.54</v>
+        <v>344.6</v>
       </c>
       <c r="C124" t="n">
-        <v>245.69</v>
+        <v>352.95</v>
       </c>
       <c r="D124" t="n">
-        <v>2.57</v>
+        <v>2.42</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>DREAMFOLKS</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>72.94</v>
+        <v>3.35</v>
       </c>
       <c r="C125" t="n">
-        <v>74.8</v>
+        <v>3.43</v>
       </c>
       <c r="D125" t="n">
-        <v>2.55</v>
+        <v>2.39</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>AGROPHOS</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>30.81</v>
+        <v>5.86</v>
       </c>
       <c r="C126" t="n">
-        <v>31.59</v>
+        <v>6</v>
       </c>
       <c r="D126" t="n">
-        <v>2.53</v>
+        <v>2.39</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>GALAPREC</t>
+          <t>UNIMECH</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>1034.05</v>
+        <v>1137.9</v>
       </c>
       <c r="C127" t="n">
-        <v>1060</v>
+        <v>1164.95</v>
       </c>
       <c r="D127" t="n">
-        <v>2.51</v>
+        <v>2.38</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>GANGAFORGE</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>26.93</v>
+        <v>2.53</v>
       </c>
       <c r="C128" t="n">
-        <v>27.6</v>
+        <v>2.59</v>
       </c>
       <c r="D128" t="n">
-        <v>2.49</v>
+        <v>2.37</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ALPA</t>
+          <t>GVPIL</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>70.26000000000001</v>
+        <v>1024.8</v>
       </c>
       <c r="C129" t="n">
-        <v>72</v>
+        <v>1048.95</v>
       </c>
       <c r="D129" t="n">
-        <v>2.48</v>
+        <v>2.36</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>SCHNEIDER</t>
+          <t>VLEGOV</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>1216.2</v>
+        <v>13.97</v>
       </c>
       <c r="C130" t="n">
-        <v>1246.2</v>
+        <v>14.3</v>
       </c>
       <c r="D130" t="n">
-        <v>2.47</v>
+        <v>2.36</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>RPTECH</t>
+          <t>AMANTA</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>561.25</v>
+        <v>150.27</v>
       </c>
       <c r="C131" t="n">
-        <v>575</v>
+        <v>153.8</v>
       </c>
       <c r="D131" t="n">
-        <v>2.45</v>
+        <v>2.35</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SAPPHIRE</t>
+          <t>3BBLACKBIO</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>173.45</v>
+        <v>1258.7</v>
       </c>
       <c r="C132" t="n">
-        <v>177.7</v>
+        <v>1288</v>
       </c>
       <c r="D132" t="n">
-        <v>2.45</v>
+        <v>2.33</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>AKI</t>
+          <t>ODIGMA</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>4.92</v>
+        <v>23.15</v>
       </c>
       <c r="C133" t="n">
-        <v>5.04</v>
+        <v>23.69</v>
       </c>
       <c r="D133" t="n">
-        <v>2.44</v>
+        <v>2.33</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>KIRLFER</t>
+          <t>360ONE</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>434.45</v>
+        <v>1133.6</v>
       </c>
       <c r="C134" t="n">
-        <v>445</v>
+        <v>1160</v>
       </c>
       <c r="D134" t="n">
-        <v>2.43</v>
+        <v>2.33</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>LPDC</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>7.01</v>
+        <v>2.17</v>
       </c>
       <c r="C135" t="n">
-        <v>7.18</v>
+        <v>2.22</v>
       </c>
       <c r="D135" t="n">
-        <v>2.43</v>
+        <v>2.3</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>RPPINFRA</t>
+          <t>BGRENERGY</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>63.35</v>
+        <v>330.25</v>
       </c>
       <c r="C136" t="n">
-        <v>64.89</v>
+        <v>337.8</v>
       </c>
       <c r="D136" t="n">
-        <v>2.43</v>
+        <v>2.29</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ELITECON</t>
+          <t>GLOBECIVIL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>30.01</v>
+        <v>43.65</v>
       </c>
       <c r="C137" t="n">
-        <v>30.74</v>
+        <v>44.65</v>
       </c>
       <c r="D137" t="n">
-        <v>2.43</v>
+        <v>2.29</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>JISLDVREQS</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>25.47</v>
+        <v>23.76</v>
       </c>
       <c r="C138" t="n">
-        <v>26.09</v>
+        <v>24.3</v>
       </c>
       <c r="D138" t="n">
-        <v>2.43</v>
+        <v>2.27</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>VGL</t>
+          <t>GAYAHWS</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>75.03</v>
+        <v>2.21</v>
       </c>
       <c r="C139" t="n">
-        <v>76.83</v>
+        <v>2.26</v>
       </c>
       <c r="D139" t="n">
-        <v>2.4</v>
+        <v>2.26</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CURAA</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>91.76000000000001</v>
+        <v>3.61</v>
       </c>
       <c r="C140" t="n">
-        <v>93.95</v>
+        <v>3.69</v>
       </c>
       <c r="D140" t="n">
-        <v>2.39</v>
+        <v>2.22</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ELECTHERM</t>
+          <t>AKSHAR</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>1122.25</v>
+        <v>0.45</v>
       </c>
       <c r="C141" t="n">
-        <v>1149</v>
+        <v>0.46</v>
       </c>
       <c r="D141" t="n">
-        <v>2.38</v>
+        <v>2.22</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>STEELCITY</t>
+          <t>DRCSYSTEMS</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>77.53</v>
+        <v>14.42</v>
       </c>
       <c r="C142" t="n">
-        <v>79.37</v>
+        <v>14.74</v>
       </c>
       <c r="D142" t="n">
-        <v>2.37</v>
+        <v>2.22</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>BASML</t>
+          <t>BANKA</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>24.52</v>
+        <v>87.09</v>
       </c>
       <c r="C143" t="n">
-        <v>25.1</v>
+        <v>89</v>
       </c>
       <c r="D143" t="n">
-        <v>2.37</v>
+        <v>2.19</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SGL</t>
+          <t>XTGLOBAL</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>10.69</v>
+        <v>29.26</v>
       </c>
       <c r="C144" t="n">
-        <v>10.94</v>
+        <v>29.9</v>
       </c>
       <c r="D144" t="n">
-        <v>2.34</v>
+        <v>2.19</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>DECCANCE</t>
+          <t>SHREDIGCEM</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>579.5</v>
+        <v>73.38</v>
       </c>
       <c r="C145" t="n">
-        <v>593</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="D145" t="n">
-        <v>2.33</v>
+        <v>2.19</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>1.29</v>
+        <v>11.12</v>
       </c>
       <c r="C146" t="n">
-        <v>1.32</v>
+        <v>11.36</v>
       </c>
       <c r="D146" t="n">
-        <v>2.33</v>
+        <v>2.16</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>NDRAUTO</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>9</v>
+        <v>843.85</v>
       </c>
       <c r="C147" t="n">
-        <v>9.210000000000001</v>
+        <v>862</v>
       </c>
       <c r="D147" t="n">
-        <v>2.33</v>
+        <v>2.15</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>HCL-INSYS</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>12.51</v>
+        <v>0.47</v>
       </c>
       <c r="C148" t="n">
-        <v>12.8</v>
+        <v>0.48</v>
       </c>
       <c r="D148" t="n">
-        <v>2.32</v>
+        <v>2.13</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>DEVYANI</t>
+          <t>DPWIRES</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>111.4</v>
+        <v>176.25</v>
       </c>
       <c r="C149" t="n">
-        <v>113.99</v>
+        <v>179.99</v>
       </c>
       <c r="D149" t="n">
-        <v>2.32</v>
+        <v>2.12</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>KAPSTON</t>
+          <t>KFINTECH</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>344.5</v>
+        <v>861.75</v>
       </c>
       <c r="C150" t="n">
-        <v>352.5</v>
+        <v>880</v>
       </c>
       <c r="D150" t="n">
-        <v>2.32</v>
+        <v>2.12</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MAJESAUT</t>
+          <t>MDL</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>335.55</v>
+        <v>73.45</v>
       </c>
       <c r="C151" t="n">
-        <v>343.3</v>
+        <v>75</v>
       </c>
       <c r="D151" t="n">
-        <v>2.31</v>
+        <v>2.11</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MAZDA</t>
+          <t>CKKRETAIL</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>229.69</v>
+        <v>145</v>
       </c>
       <c r="C152" t="n">
-        <v>234.99</v>
+        <v>148.05</v>
       </c>
       <c r="D152" t="n">
-        <v>2.31</v>
+        <v>2.1</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ECOSMOBLTY</t>
+          <t>BORANA</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>131.47</v>
+        <v>317.25</v>
       </c>
       <c r="C153" t="n">
-        <v>134.49</v>
+        <v>323.9</v>
       </c>
       <c r="D153" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>93.40000000000001</v>
+        <v>44.56</v>
       </c>
       <c r="C154" t="n">
-        <v>95.55</v>
+        <v>45.49</v>
       </c>
       <c r="D154" t="n">
-        <v>2.3</v>
+        <v>2.09</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>SPCENET</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>1.31</v>
+        <v>3.36</v>
       </c>
       <c r="C155" t="n">
-        <v>1.34</v>
+        <v>3.43</v>
       </c>
       <c r="D155" t="n">
-        <v>2.29</v>
+        <v>2.08</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>RUBFILA</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>72.15000000000001</v>
+        <v>391.65</v>
       </c>
       <c r="C156" t="n">
-        <v>73.8</v>
+        <v>399.8</v>
       </c>
       <c r="D156" t="n">
-        <v>2.29</v>
+        <v>2.08</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>TAKE</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>29.53</v>
+        <v>401.65</v>
       </c>
       <c r="C157" t="n">
-        <v>30.2</v>
+        <v>409.95</v>
       </c>
       <c r="D157" t="n">
-        <v>2.27</v>
+        <v>2.07</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>5PAISA</t>
+          <t>COFORGE</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>316.8</v>
+        <v>1464.8</v>
       </c>
       <c r="C158" t="n">
-        <v>323.9</v>
+        <v>1494.5</v>
       </c>
       <c r="D158" t="n">
-        <v>2.24</v>
+        <v>2.03</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>VASWANI</t>
+          <t>FIBERWEB</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>59.37</v>
+        <v>29</v>
       </c>
       <c r="C159" t="n">
-        <v>60.7</v>
+        <v>29.59</v>
       </c>
       <c r="D159" t="n">
-        <v>2.24</v>
+        <v>2.03</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>GICL</t>
+          <t>LASA</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>23.28</v>
+        <v>7.44</v>
       </c>
       <c r="C160" t="n">
-        <v>23.8</v>
+        <v>7.59</v>
       </c>
       <c r="D160" t="n">
-        <v>2.23</v>
+        <v>2.02</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>168.25</v>
+        <v>20.34</v>
       </c>
       <c r="C161" t="n">
-        <v>171.98</v>
+        <v>20.75</v>
       </c>
       <c r="D161" t="n">
-        <v>2.22</v>
+        <v>2.02</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>KPL</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>0.45</v>
+        <v>2413.6</v>
       </c>
       <c r="C162" t="n">
-        <v>0.46</v>
+        <v>2462</v>
       </c>
       <c r="D162" t="n">
-        <v>2.22</v>
+        <v>2.01</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SHEEL</t>
+          <t>LATTEYS</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>63</v>
+        <v>22.4</v>
       </c>
       <c r="C163" t="n">
-        <v>64.40000000000001</v>
+        <v>22.85</v>
       </c>
       <c r="D163" t="n">
-        <v>2.22</v>
+        <v>2.01</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>UMAEXPORTS</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>48.81</v>
+        <v>25</v>
       </c>
       <c r="C164" t="n">
-        <v>49.89</v>
+        <v>25.5</v>
       </c>
       <c r="D164" t="n">
-        <v>2.21</v>
+        <v>2</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>CEMPRO</t>
+          <t>MAJESAUT</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>1178.5</v>
+        <v>338.15</v>
       </c>
       <c r="C165" t="n">
-        <v>1204.6</v>
+        <v>344.9</v>
       </c>
       <c r="D165" t="n">
-        <v>2.21</v>
+        <v>2</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>ANNAPURNA</t>
+          <t>MHLXMIRU</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>134.1</v>
+        <v>170.59</v>
       </c>
       <c r="C166" t="n">
-        <v>137.05</v>
+        <v>174</v>
       </c>
       <c r="D166" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>PLASTIBLEN</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>37.59</v>
+        <v>173</v>
       </c>
       <c r="C167" t="n">
-        <v>38.41</v>
+        <v>176.45</v>
       </c>
       <c r="D167" t="n">
-        <v>2.18</v>
+        <v>1.99</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>ESTER</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>44.92</v>
+        <v>91.18000000000001</v>
       </c>
       <c r="C168" t="n">
-        <v>45.9</v>
+        <v>92.98999999999999</v>
       </c>
       <c r="D168" t="n">
-        <v>2.18</v>
+        <v>1.99</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>SUTLEJTEX</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>616.6</v>
+        <v>38.24</v>
       </c>
       <c r="C169" t="n">
-        <v>630</v>
+        <v>39</v>
       </c>
       <c r="D169" t="n">
-        <v>2.17</v>
+        <v>1.99</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>VIDYAWIRES</t>
+          <t>BIGBLOC</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>93.53</v>
+        <v>50.46</v>
       </c>
       <c r="C170" t="n">
-        <v>95.55</v>
+        <v>51.46</v>
       </c>
       <c r="D170" t="n">
-        <v>2.16</v>
+        <v>1.98</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>BANG</t>
+          <t>TPLPLASTEH</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>30.69</v>
+        <v>67.06999999999999</v>
       </c>
       <c r="C171" t="n">
-        <v>31.35</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="D171" t="n">
-        <v>2.15</v>
+        <v>1.98</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>TTKHLTCARE</t>
+          <t>MURUDCERA</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>878.15</v>
+        <v>31.5</v>
       </c>
       <c r="C172" t="n">
-        <v>897</v>
+        <v>32.12</v>
       </c>
       <c r="D172" t="n">
-        <v>2.15</v>
+        <v>1.97</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>NINSYS</t>
+          <t>PRAENG</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>704.25</v>
+        <v>21.35</v>
       </c>
       <c r="C173" t="n">
-        <v>719.3</v>
+        <v>21.77</v>
       </c>
       <c r="D173" t="n">
-        <v>2.14</v>
+        <v>1.97</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>LIKHITHA</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>232.09</v>
+        <v>7.16</v>
       </c>
       <c r="C174" t="n">
-        <v>237</v>
+        <v>7.3</v>
       </c>
       <c r="D174" t="n">
-        <v>2.12</v>
+        <v>1.96</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>TERASOFT</t>
+          <t>ROML</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>437.65</v>
+        <v>45.51</v>
       </c>
       <c r="C175" t="n">
-        <v>446.9</v>
+        <v>46.4</v>
       </c>
       <c r="D175" t="n">
-        <v>2.11</v>
+        <v>1.96</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>AMIRCHAND</t>
+          <t>MANBA</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>129.12</v>
+        <v>127.52</v>
       </c>
       <c r="C176" t="n">
-        <v>131.85</v>
+        <v>130</v>
       </c>
       <c r="D176" t="n">
-        <v>2.11</v>
+        <v>1.94</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>INSPIRISYS</t>
+          <t>NIPPOBATRY</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>112.62</v>
+        <v>358.95</v>
       </c>
       <c r="C177" t="n">
-        <v>115</v>
+        <v>365.9</v>
       </c>
       <c r="D177" t="n">
-        <v>2.11</v>
+        <v>1.94</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>KRITINUT</t>
+          <t>GOKUL</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>82.48</v>
+        <v>40.71</v>
       </c>
       <c r="C178" t="n">
-        <v>84.20999999999999</v>
+        <v>41.5</v>
       </c>
       <c r="D178" t="n">
-        <v>2.1</v>
+        <v>1.94</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>21STCENMGM</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>41.58</v>
+        <v>32.13</v>
       </c>
       <c r="C179" t="n">
-        <v>42.45</v>
+        <v>32.75</v>
       </c>
       <c r="D179" t="n">
-        <v>2.09</v>
+        <v>1.93</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>RCOM</t>
+          <t>SURANAT&amp;P</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>0.96</v>
+        <v>19.14</v>
       </c>
       <c r="C180" t="n">
-        <v>0.98</v>
+        <v>19.51</v>
       </c>
       <c r="D180" t="n">
-        <v>2.08</v>
+        <v>1.93</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>SAKUMA</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>1.93</v>
+        <v>0.52</v>
       </c>
       <c r="C181" t="n">
-        <v>1.97</v>
+        <v>0.53</v>
       </c>
       <c r="D181" t="n">
-        <v>2.07</v>
+        <v>1.92</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>WAAREEINDO</t>
+          <t>PINELABS</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>389.95</v>
+        <v>150.09</v>
       </c>
       <c r="C182" t="n">
-        <v>398</v>
+        <v>152.94</v>
       </c>
       <c r="D182" t="n">
-        <v>2.06</v>
+        <v>1.9</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>SREEL</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>197.73</v>
+        <v>53.91</v>
       </c>
       <c r="C183" t="n">
-        <v>201.8</v>
+        <v>54.93</v>
       </c>
       <c r="D183" t="n">
-        <v>2.06</v>
+        <v>1.89</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MAHESHWARI</t>
+          <t>NECLIFE</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>71.5</v>
+        <v>11.78</v>
       </c>
       <c r="C184" t="n">
-        <v>72.95999999999999</v>
+        <v>12</v>
       </c>
       <c r="D184" t="n">
-        <v>2.04</v>
+        <v>1.87</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>28.91</v>
+        <v>54.47</v>
       </c>
       <c r="C185" t="n">
-        <v>29.5</v>
+        <v>55.49</v>
       </c>
       <c r="D185" t="n">
-        <v>2.04</v>
+        <v>1.87</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>SWANDEF</t>
+          <t>PAVNAIND</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>1998.2</v>
+        <v>17.08</v>
       </c>
       <c r="C186" t="n">
-        <v>2039</v>
+        <v>17.4</v>
       </c>
       <c r="D186" t="n">
-        <v>2.04</v>
+        <v>1.87</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SNOWMAN</t>
+          <t>EMAMIPAP</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>38.51</v>
+        <v>84.23999999999999</v>
       </c>
       <c r="C187" t="n">
-        <v>39.29</v>
+        <v>85.8</v>
       </c>
       <c r="D187" t="n">
-        <v>2.03</v>
+        <v>1.85</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>AEROFLEX</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>478</v>
+        <v>348.6</v>
       </c>
       <c r="C188" t="n">
-        <v>487.65</v>
+        <v>355</v>
       </c>
       <c r="D188" t="n">
-        <v>2.02</v>
+        <v>1.84</v>
       </c>
       <c r="E188" t="b">
         <v>0</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>JAYSREETEA</t>
+          <t>NAUKRI</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>88.13</v>
+        <v>997.65</v>
       </c>
       <c r="C189" t="n">
-        <v>89.90000000000001</v>
+        <v>1016</v>
       </c>
       <c r="D189" t="n">
-        <v>2.01</v>
+        <v>1.84</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>HINDCOMPOS</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>7.45</v>
+        <v>419.4</v>
       </c>
       <c r="C190" t="n">
-        <v>7.6</v>
+        <v>427</v>
       </c>
       <c r="D190" t="n">
-        <v>2.01</v>
+        <v>1.81</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>GLOSTERLTD</t>
+          <t>MKPL</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>680.85</v>
+        <v>4.97</v>
       </c>
       <c r="C191" t="n">
-        <v>694.5</v>
+        <v>5.06</v>
       </c>
       <c r="D191" t="n">
-        <v>2</v>
+        <v>1.81</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>PONNIERODE</t>
+          <t>APOLLOTYRE</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>320.1</v>
+        <v>416.45</v>
       </c>
       <c r="C192" t="n">
-        <v>326.5</v>
+        <v>424</v>
       </c>
       <c r="D192" t="n">
-        <v>2</v>
+        <v>1.81</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>BROOKS</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>67.55</v>
+        <v>24.4</v>
       </c>
       <c r="C193" t="n">
-        <v>68.90000000000001</v>
+        <v>24.84</v>
       </c>
       <c r="D193" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>ALPEXSOLAR</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>990.1</v>
+        <v>3.91</v>
       </c>
       <c r="C194" t="n">
-        <v>1009.9</v>
+        <v>3.98</v>
       </c>
       <c r="D194" t="n">
-        <v>2</v>
+        <v>1.79</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>IWP</t>
+          <t>DMCC</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>33.6</v>
+        <v>258.4</v>
       </c>
       <c r="C195" t="n">
-        <v>34.27</v>
+        <v>263</v>
       </c>
       <c r="D195" t="n">
-        <v>1.99</v>
+        <v>1.78</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>CIFL</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>51.16</v>
+        <v>24.9</v>
       </c>
       <c r="C196" t="n">
-        <v>52.18</v>
+        <v>25.34</v>
       </c>
       <c r="D196" t="n">
-        <v>1.99</v>
+        <v>1.77</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>TRIGYN</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>55.7</v>
+        <v>13.76</v>
       </c>
       <c r="C197" t="n">
-        <v>56.8</v>
+        <v>14</v>
       </c>
       <c r="D197" t="n">
-        <v>1.97</v>
+        <v>1.74</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>NIPPOBATRY</t>
+          <t>GLOBE</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>356</v>
+        <v>2.31</v>
       </c>
       <c r="C198" t="n">
-        <v>363</v>
+        <v>2.35</v>
       </c>
       <c r="D198" t="n">
-        <v>1.97</v>
+        <v>1.73</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,17 +4795,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>180.45</v>
+        <v>49.15</v>
       </c>
       <c r="C199" t="n">
-        <v>184</v>
+        <v>50</v>
       </c>
       <c r="D199" t="n">
-        <v>1.97</v>
+        <v>1.73</v>
       </c>
       <c r="E199" t="b">
         <v>0</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>0.51</v>
+        <v>28.95</v>
       </c>
       <c r="C200" t="n">
-        <v>0.52</v>
+        <v>29.45</v>
       </c>
       <c r="D200" t="n">
-        <v>1.96</v>
+        <v>1.73</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>BALAJEE</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>1119.3</v>
+        <v>29.3</v>
       </c>
       <c r="C201" t="n">
-        <v>1141</v>
+        <v>29.8</v>
       </c>
       <c r="D201" t="n">
-        <v>1.94</v>
+        <v>1.71</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-18 08:27 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SHAH-RE1</t>
+          <t>EIFFL</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.05</v>
+        <v>298.57</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06</v>
+        <v>355</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>18.9</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -483,17 +483,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>COMFINTE</t>
+          <t>SHAH-RE1</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5.87</v>
+        <v>0.06</v>
       </c>
       <c r="C3" t="n">
-        <v>7.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>19.93</v>
+        <v>16.67</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>DHARIWAL</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39.83</v>
+        <v>28.7</v>
       </c>
       <c r="C4" t="n">
-        <v>43.78</v>
+        <v>32.5</v>
       </c>
       <c r="D4" t="n">
-        <v>9.92</v>
+        <v>13.24</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MADHUCON</t>
+          <t>LPDC</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.03</v>
+        <v>6.76</v>
       </c>
       <c r="C5" t="n">
-        <v>6.59</v>
+        <v>7.3</v>
       </c>
       <c r="D5" t="n">
-        <v>9.289999999999999</v>
+        <v>7.99</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SARTELE</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>160.2</v>
+        <v>0.16</v>
       </c>
       <c r="C6" t="n">
-        <v>174.9</v>
+        <v>0.17</v>
       </c>
       <c r="D6" t="n">
-        <v>9.18</v>
+        <v>6.25</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>K2INFRA</t>
+          <t>ACEINTEG</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>68.84999999999999</v>
+        <v>20.7</v>
       </c>
       <c r="C7" t="n">
-        <v>73.90000000000001</v>
+        <v>21.99</v>
       </c>
       <c r="D7" t="n">
-        <v>7.33</v>
+        <v>6.23</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ONMOBILE</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>51.3</v>
+        <v>43.81</v>
       </c>
       <c r="C8" t="n">
-        <v>54.76</v>
+        <v>46.49</v>
       </c>
       <c r="D8" t="n">
-        <v>6.74</v>
+        <v>6.12</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BABAFP</t>
+          <t>POWERICA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23.75</v>
+        <v>529.8</v>
       </c>
       <c r="C9" t="n">
-        <v>25.25</v>
+        <v>560.95</v>
       </c>
       <c r="D9" t="n">
-        <v>6.32</v>
+        <v>5.88</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>ZENITHSTL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.16</v>
+        <v>5.93</v>
       </c>
       <c r="C10" t="n">
-        <v>0.17</v>
+        <v>6.27</v>
       </c>
       <c r="D10" t="n">
-        <v>6.25</v>
+        <v>5.73</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>QMSMEDI</t>
+          <t>ABMINTLLTD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>97</v>
+        <v>40.79</v>
       </c>
       <c r="C11" t="n">
-        <v>102.9</v>
+        <v>42.94</v>
       </c>
       <c r="D11" t="n">
-        <v>6.08</v>
+        <v>5.27</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RSDFIN</t>
+          <t>KIRLFER</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>82</v>
+        <v>444.3</v>
       </c>
       <c r="C12" t="n">
-        <v>86.98</v>
+        <v>467</v>
       </c>
       <c r="D12" t="n">
-        <v>6.07</v>
+        <v>5.11</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SINCLAIR</t>
+          <t>SIGNORIA</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>76.22</v>
+        <v>80</v>
       </c>
       <c r="C13" t="n">
-        <v>80.68000000000001</v>
+        <v>84</v>
       </c>
       <c r="D13" t="n">
-        <v>5.85</v>
+        <v>5</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WTICAB</t>
+          <t>RAJESHEXPO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>98.5</v>
+        <v>88.45</v>
       </c>
       <c r="C14" t="n">
-        <v>104</v>
+        <v>92.87</v>
       </c>
       <c r="D14" t="n">
-        <v>5.58</v>
+        <v>5</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AAATECH</t>
+          <t>NIRAJ</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>96.68000000000001</v>
+        <v>31</v>
       </c>
       <c r="C15" t="n">
-        <v>102</v>
+        <v>32.55</v>
       </c>
       <c r="D15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>MARC</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>8.44</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="D16" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>SICALLOG</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>25.61</v>
+        <v>96.64</v>
       </c>
       <c r="C17" t="n">
-        <v>26.97</v>
+        <v>101.47</v>
       </c>
       <c r="D17" t="n">
-        <v>5.31</v>
+        <v>5</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,17 +813,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOMATEX</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>97.68000000000001</v>
+        <v>8</v>
       </c>
       <c r="C18" t="n">
-        <v>102.7</v>
+        <v>8.4</v>
       </c>
       <c r="D18" t="n">
-        <v>5.14</v>
+        <v>5</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -835,14 +835,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RAJESHEXPO</t>
+          <t>APEXECO</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>84.23999999999999</v>
+        <v>213.15</v>
       </c>
       <c r="C19" t="n">
-        <v>88.45</v>
+        <v>223.8</v>
       </c>
       <c r="D19" t="n">
         <v>5</v>
@@ -857,14 +857,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SICALLOG</t>
+          <t>SEJALLTD</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>92.04000000000001</v>
+        <v>761.25</v>
       </c>
       <c r="C20" t="n">
-        <v>96.64</v>
+        <v>799.3</v>
       </c>
       <c r="D20" t="n">
         <v>5</v>
@@ -879,14 +879,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MTEDUCARE</t>
+          <t>VISL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>23.21</v>
       </c>
       <c r="C21" t="n">
-        <v>2.1</v>
+        <v>24.37</v>
       </c>
       <c r="D21" t="n">
         <v>5</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PFOCUS</t>
+          <t>HMT</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>234.15</v>
+        <v>58.73</v>
       </c>
       <c r="C22" t="n">
-        <v>245.85</v>
+        <v>61.66</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SEJALLTD</t>
+          <t>SHYAMTEL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>725</v>
+        <v>17.25</v>
       </c>
       <c r="C23" t="n">
-        <v>761.25</v>
+        <v>18.11</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,14 +945,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PALREDTEC</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>48.31</v>
+        <v>359.5</v>
       </c>
       <c r="C24" t="n">
-        <v>50.72</v>
+        <v>377.45</v>
       </c>
       <c r="D24" t="n">
         <v>4.99</v>
@@ -967,14 +967,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GANESHIN</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>103.3</v>
+        <v>326.55</v>
       </c>
       <c r="C25" t="n">
-        <v>108.45</v>
+        <v>342.85</v>
       </c>
       <c r="D25" t="n">
         <v>4.99</v>
@@ -989,14 +989,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MASKINVEST</t>
+          <t>VIDYAWIRES</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>155.39</v>
+        <v>103.11</v>
       </c>
       <c r="C26" t="n">
-        <v>163.15</v>
+        <v>108.26</v>
       </c>
       <c r="D26" t="n">
         <v>4.99</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>UNIHEALTH</t>
+          <t>CALSOFT</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>521.75</v>
+        <v>23.07</v>
       </c>
       <c r="C27" t="n">
-        <v>547.8</v>
+        <v>24.22</v>
       </c>
       <c r="D27" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MANORG</t>
+          <t>GANESHIN</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>518.7</v>
+        <v>108.45</v>
       </c>
       <c r="C28" t="n">
-        <v>544.6</v>
+        <v>113.85</v>
       </c>
       <c r="D28" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,17 +1055,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SIGNORIA</t>
+          <t>SMARTEN</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>76.2</v>
+        <v>59.2</v>
       </c>
       <c r="C29" t="n">
-        <v>80</v>
+        <v>62.15</v>
       </c>
       <c r="D29" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>VPRPL</t>
+          <t>ACCORD</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>29.14</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="C30" t="n">
-        <v>30.59</v>
+        <v>104.55</v>
       </c>
       <c r="D30" t="n">
-        <v>4.98</v>
+        <v>4.97</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NIRAJ</t>
+          <t>TECHERA</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>29.53</v>
+        <v>169.85</v>
       </c>
       <c r="C31" t="n">
-        <v>31</v>
+        <v>178.3</v>
       </c>
       <c r="D31" t="n">
-        <v>4.98</v>
+        <v>4.97</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GAYAPROJ</t>
+          <t>INNOMET</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>24.09</v>
+        <v>111.9</v>
       </c>
       <c r="C32" t="n">
-        <v>25.29</v>
+        <v>117.45</v>
       </c>
       <c r="D32" t="n">
-        <v>4.98</v>
+        <v>4.96</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TECHERA</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>161.8</v>
+        <v>108.95</v>
       </c>
       <c r="C33" t="n">
-        <v>169.85</v>
+        <v>114.35</v>
       </c>
       <c r="D33" t="n">
-        <v>4.98</v>
+        <v>4.96</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>HILTON</t>
+          <t>PALREDTEC</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>20.53</v>
+        <v>50.72</v>
       </c>
       <c r="C34" t="n">
-        <v>21.55</v>
+        <v>53.2</v>
       </c>
       <c r="D34" t="n">
-        <v>4.97</v>
+        <v>4.89</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OWAIS</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>103.8</v>
+        <v>4.1</v>
       </c>
       <c r="C35" t="n">
-        <v>108.95</v>
+        <v>4.3</v>
       </c>
       <c r="D35" t="n">
-        <v>4.96</v>
+        <v>4.88</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ORTEL</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1.62</v>
+        <v>3.09</v>
       </c>
       <c r="C36" t="n">
-        <v>1.7</v>
+        <v>3.24</v>
       </c>
       <c r="D36" t="n">
-        <v>4.94</v>
+        <v>4.85</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PROLIFE</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>65.90000000000001</v>
+        <v>3.51</v>
       </c>
       <c r="C37" t="n">
-        <v>69.15000000000001</v>
+        <v>3.68</v>
       </c>
       <c r="D37" t="n">
-        <v>4.93</v>
+        <v>4.84</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>INNOMET</t>
+          <t>UTSSAV</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>106.6</v>
+        <v>346.25</v>
       </c>
       <c r="C38" t="n">
-        <v>111.85</v>
+        <v>363</v>
       </c>
       <c r="D38" t="n">
-        <v>4.92</v>
+        <v>4.84</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SUBEXLTD</t>
+          <t>BILVYAPAR</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>11.58</v>
+        <v>4.13</v>
       </c>
       <c r="C39" t="n">
-        <v>12.15</v>
+        <v>4.33</v>
       </c>
       <c r="D39" t="n">
-        <v>4.92</v>
+        <v>4.84</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IEML</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>50.05</v>
+        <v>0.21</v>
       </c>
       <c r="C40" t="n">
-        <v>52.5</v>
+        <v>0.22</v>
       </c>
       <c r="D40" t="n">
-        <v>4.9</v>
+        <v>4.76</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AILIMITED</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>37.9</v>
+        <v>137.31</v>
       </c>
       <c r="C41" t="n">
-        <v>39.75</v>
+        <v>143.85</v>
       </c>
       <c r="D41" t="n">
-        <v>4.88</v>
+        <v>4.76</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,17 +1341,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SADHNANIQ</t>
+          <t>SETUINFRA</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2.49</v>
+        <v>0.42</v>
       </c>
       <c r="C42" t="n">
-        <v>2.61</v>
+        <v>0.44</v>
       </c>
       <c r="D42" t="n">
-        <v>4.82</v>
+        <v>4.76</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GOLDENTOBC</t>
+          <t>MANINDS</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>25.09</v>
+        <v>592.6</v>
       </c>
       <c r="C43" t="n">
-        <v>26.29</v>
+        <v>620</v>
       </c>
       <c r="D43" t="n">
-        <v>4.78</v>
+        <v>4.62</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SARVESHWAR</t>
+          <t>VPRPL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3.78</v>
+        <v>30.59</v>
       </c>
       <c r="C44" t="n">
-        <v>3.96</v>
+        <v>32</v>
       </c>
       <c r="D44" t="n">
-        <v>4.76</v>
+        <v>4.61</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MAL</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>32</v>
+        <v>1.53</v>
       </c>
       <c r="C45" t="n">
-        <v>33.5</v>
+        <v>1.6</v>
       </c>
       <c r="D45" t="n">
-        <v>4.69</v>
+        <v>4.58</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>SECURKLOUD</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>180.11</v>
+        <v>18.94</v>
       </c>
       <c r="C46" t="n">
-        <v>188.5</v>
+        <v>19.78</v>
       </c>
       <c r="D46" t="n">
-        <v>4.66</v>
+        <v>4.44</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ARVINDPORT</t>
+          <t>SHIVAMILLS</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>28.2</v>
+        <v>62.05</v>
       </c>
       <c r="C47" t="n">
-        <v>29.5</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="D47" t="n">
-        <v>4.61</v>
+        <v>4.42</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>HMT</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>55.94</v>
+        <v>8.24</v>
       </c>
       <c r="C48" t="n">
-        <v>58.5</v>
+        <v>8.6</v>
       </c>
       <c r="D48" t="n">
-        <v>4.58</v>
+        <v>4.37</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TBI</t>
+          <t>SEMAC</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>65.15000000000001</v>
+        <v>324.85</v>
       </c>
       <c r="C49" t="n">
-        <v>68</v>
+        <v>339</v>
       </c>
       <c r="D49" t="n">
-        <v>4.37</v>
+        <v>4.36</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>RRIL</t>
+          <t>PRITI</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>19.84</v>
+        <v>42.5</v>
       </c>
       <c r="C50" t="n">
-        <v>20.7</v>
+        <v>44.31</v>
       </c>
       <c r="D50" t="n">
-        <v>4.33</v>
+        <v>4.26</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>KESORAMIND</t>
+          <t>EFFWA</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>12.09</v>
+        <v>345.3</v>
       </c>
       <c r="C51" t="n">
-        <v>12.59</v>
+        <v>359.9</v>
       </c>
       <c r="D51" t="n">
-        <v>4.14</v>
+        <v>4.23</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>162.88</v>
+        <v>6.24</v>
       </c>
       <c r="C52" t="n">
-        <v>169.44</v>
+        <v>6.5</v>
       </c>
       <c r="D52" t="n">
-        <v>4.03</v>
+        <v>4.17</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MITCON</t>
+          <t>KONSTELEC</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>79.51000000000001</v>
+        <v>48.7</v>
       </c>
       <c r="C53" t="n">
-        <v>82.68000000000001</v>
+        <v>50.7</v>
       </c>
       <c r="D53" t="n">
-        <v>3.99</v>
+        <v>4.11</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LEXUS</t>
+          <t>KANORICHEM</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>15.86</v>
+        <v>109.51</v>
       </c>
       <c r="C54" t="n">
-        <v>16.49</v>
+        <v>113.99</v>
       </c>
       <c r="D54" t="n">
-        <v>3.97</v>
+        <v>4.09</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>NITCO</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>21.18</v>
+        <v>95.91</v>
       </c>
       <c r="C55" t="n">
-        <v>22</v>
+        <v>99.8</v>
       </c>
       <c r="D55" t="n">
-        <v>3.87</v>
+        <v>4.06</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>JETFREIGHT</t>
+          <t>SILINV</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>21.63</v>
+        <v>429.2</v>
       </c>
       <c r="C56" t="n">
-        <v>22.45</v>
+        <v>446.5</v>
       </c>
       <c r="D56" t="n">
-        <v>3.79</v>
+        <v>4.03</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>REPL</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>73.2</v>
+        <v>168.35</v>
       </c>
       <c r="C57" t="n">
-        <v>75.94</v>
+        <v>174.99</v>
       </c>
       <c r="D57" t="n">
-        <v>3.74</v>
+        <v>3.94</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>IDEAFORGE</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>908.05</v>
+        <v>24.28</v>
       </c>
       <c r="C58" t="n">
-        <v>942</v>
+        <v>25.22</v>
       </c>
       <c r="D58" t="n">
-        <v>3.74</v>
+        <v>3.87</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SBGLP</t>
+          <t>DSFCL</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>26.01</v>
+        <v>23.4</v>
       </c>
       <c r="C59" t="n">
-        <v>26.98</v>
+        <v>24.3</v>
       </c>
       <c r="D59" t="n">
-        <v>3.73</v>
+        <v>3.85</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>HIGREEN</t>
+          <t>AHLWEST</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>137.85</v>
+        <v>544.1</v>
       </c>
       <c r="C60" t="n">
-        <v>142.95</v>
+        <v>565</v>
       </c>
       <c r="D60" t="n">
-        <v>3.7</v>
+        <v>3.84</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>AEROENTER</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>9.35</v>
+        <v>115.65</v>
       </c>
       <c r="C61" t="n">
-        <v>9.69</v>
+        <v>120</v>
       </c>
       <c r="D61" t="n">
-        <v>3.64</v>
+        <v>3.76</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>INCREDIBLE</t>
+          <t>UNITECH</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>34.84</v>
+        <v>5.09</v>
       </c>
       <c r="C62" t="n">
-        <v>36.1</v>
+        <v>5.28</v>
       </c>
       <c r="D62" t="n">
-        <v>3.62</v>
+        <v>3.73</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SIGMA</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>39.1</v>
+        <v>190.13</v>
       </c>
       <c r="C63" t="n">
-        <v>40.51</v>
+        <v>197.13</v>
       </c>
       <c r="D63" t="n">
-        <v>3.61</v>
+        <v>3.68</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BCONCEPTS</t>
+          <t>NAGREEKEXP</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>175.1</v>
+        <v>27.71</v>
       </c>
       <c r="C64" t="n">
-        <v>181.2</v>
+        <v>28.7</v>
       </c>
       <c r="D64" t="n">
-        <v>3.48</v>
+        <v>3.57</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>3PLAND</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>7.2</v>
+        <v>31.19</v>
       </c>
       <c r="C65" t="n">
-        <v>7.45</v>
+        <v>32.3</v>
       </c>
       <c r="D65" t="n">
-        <v>3.47</v>
+        <v>3.56</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AARTECH</t>
+          <t>DPWIRES</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>49.05</v>
+        <v>178.42</v>
       </c>
       <c r="C66" t="n">
-        <v>50.75</v>
+        <v>184.7</v>
       </c>
       <c r="D66" t="n">
-        <v>3.47</v>
+        <v>3.52</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>KEEPLEARN</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>5.79</v>
+        <v>2</v>
       </c>
       <c r="C67" t="n">
-        <v>5.99</v>
+        <v>2.07</v>
       </c>
       <c r="D67" t="n">
-        <v>3.45</v>
+        <v>3.5</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>NAGREEKCAP</t>
+          <t>METROGLOBL</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>29</v>
+        <v>128.02</v>
       </c>
       <c r="C68" t="n">
-        <v>30</v>
+        <v>132.5</v>
       </c>
       <c r="D68" t="n">
-        <v>3.45</v>
+        <v>3.5</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>TOUCHWOOD</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>572.4</v>
+        <v>75.06999999999999</v>
       </c>
       <c r="C69" t="n">
-        <v>592</v>
+        <v>77.69</v>
       </c>
       <c r="D69" t="n">
-        <v>3.42</v>
+        <v>3.49</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LAGNAM</t>
+          <t>ADROITINFO</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>80.84</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="C70" t="n">
-        <v>83.59999999999999</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="D70" t="n">
-        <v>3.41</v>
+        <v>3.49</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>AMDIND</t>
+          <t>RVTH</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>47.29</v>
+        <v>716.75</v>
       </c>
       <c r="C71" t="n">
-        <v>48.9</v>
+        <v>741.7</v>
       </c>
       <c r="D71" t="n">
-        <v>3.4</v>
+        <v>3.48</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,17 +2001,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>RVTH</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>705.15</v>
+        <v>44.46</v>
       </c>
       <c r="C72" t="n">
-        <v>728.95</v>
+        <v>46</v>
       </c>
       <c r="D72" t="n">
-        <v>3.38</v>
+        <v>3.46</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>FLYSBS</t>
+          <t>BASML</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>456.6</v>
+        <v>24.89</v>
       </c>
       <c r="C73" t="n">
-        <v>472</v>
+        <v>25.75</v>
       </c>
       <c r="D73" t="n">
-        <v>3.37</v>
+        <v>3.46</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,17 +2045,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CHAMUNDA</t>
+          <t>PML</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>39.2</v>
+        <v>501</v>
       </c>
       <c r="C74" t="n">
-        <v>40.5</v>
+        <v>518</v>
       </c>
       <c r="D74" t="n">
-        <v>3.32</v>
+        <v>3.39</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>SUTLEJTEX</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1227.6</v>
+        <v>37.34</v>
       </c>
       <c r="C75" t="n">
-        <v>1268</v>
+        <v>38.6</v>
       </c>
       <c r="D75" t="n">
-        <v>3.29</v>
+        <v>3.37</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>EXXARO</t>
+          <t>AMBICAAGAR</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>6.78</v>
+        <v>24.58</v>
       </c>
       <c r="C76" t="n">
-        <v>7</v>
+        <v>25.39</v>
       </c>
       <c r="D76" t="n">
-        <v>3.24</v>
+        <v>3.3</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>LIBAS</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>11.91</v>
+        <v>59.91</v>
       </c>
       <c r="C77" t="n">
-        <v>12.29</v>
+        <v>61.88</v>
       </c>
       <c r="D77" t="n">
-        <v>3.19</v>
+        <v>3.29</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>EMAMIREAL</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>92.05</v>
+        <v>6.39</v>
       </c>
       <c r="C78" t="n">
-        <v>94.98</v>
+        <v>6.6</v>
       </c>
       <c r="D78" t="n">
-        <v>3.18</v>
+        <v>3.29</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ARCHIDPLY</t>
+          <t>HEADSUP</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>81.34</v>
+        <v>7.65</v>
       </c>
       <c r="C79" t="n">
-        <v>83.92</v>
+        <v>7.9</v>
       </c>
       <c r="D79" t="n">
-        <v>3.17</v>
+        <v>3.27</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>GFLLIMITED</t>
+          <t>TFL</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>47.11</v>
+        <v>12.88</v>
       </c>
       <c r="C80" t="n">
-        <v>48.6</v>
+        <v>13.3</v>
       </c>
       <c r="D80" t="n">
-        <v>3.16</v>
+        <v>3.26</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CYBERTECH</t>
+          <t>LAGNAM</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>143.53</v>
+        <v>80.2</v>
       </c>
       <c r="C81" t="n">
-        <v>147.99</v>
+        <v>82.8</v>
       </c>
       <c r="D81" t="n">
-        <v>3.11</v>
+        <v>3.24</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>RUSHIL</t>
+          <t>CELEBRITY</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>17.66</v>
+        <v>7.31</v>
       </c>
       <c r="C82" t="n">
-        <v>18.2</v>
+        <v>7.54</v>
       </c>
       <c r="D82" t="n">
-        <v>3.06</v>
+        <v>3.15</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>JKIPL</t>
+          <t>LAMOSAIC</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>113.05</v>
+        <v>33.5</v>
       </c>
       <c r="C83" t="n">
-        <v>116.5</v>
+        <v>34.55</v>
       </c>
       <c r="D83" t="n">
-        <v>3.05</v>
+        <v>3.13</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>LEMERITE</t>
+          <t>HYBRIDFIN</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>28.51</v>
+        <v>18.91</v>
       </c>
       <c r="C84" t="n">
-        <v>29.38</v>
+        <v>19.5</v>
       </c>
       <c r="D84" t="n">
-        <v>3.05</v>
+        <v>3.12</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>TARSONS</t>
+          <t>HARRMALAYA</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>238.73</v>
+        <v>205.57</v>
       </c>
       <c r="C85" t="n">
-        <v>246</v>
+        <v>211.9</v>
       </c>
       <c r="D85" t="n">
-        <v>3.05</v>
+        <v>3.08</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ASTRON</t>
+          <t>BALKRISHNA</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>3.97</v>
+        <v>17.95</v>
       </c>
       <c r="C86" t="n">
-        <v>4.09</v>
+        <v>18.5</v>
       </c>
       <c r="D86" t="n">
-        <v>3.02</v>
+        <v>3.06</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>TRIGYN</t>
+          <t>LAXMICOT</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>55.34</v>
+        <v>15.04</v>
       </c>
       <c r="C87" t="n">
-        <v>57</v>
+        <v>15.5</v>
       </c>
       <c r="D87" t="n">
-        <v>3</v>
+        <v>3.06</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ORBTEXP</t>
+          <t>SUYOG</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>229.16</v>
+        <v>792.2</v>
       </c>
       <c r="C88" t="n">
-        <v>235.99</v>
+        <v>816</v>
       </c>
       <c r="D88" t="n">
-        <v>2.98</v>
+        <v>3</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>ICIL</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>2.03</v>
+        <v>342.1</v>
       </c>
       <c r="C89" t="n">
-        <v>2.09</v>
+        <v>352.35</v>
       </c>
       <c r="D89" t="n">
-        <v>2.96</v>
+        <v>3</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>VERTOZ</t>
+          <t>BORANA</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>45.17</v>
+        <v>318.5</v>
       </c>
       <c r="C90" t="n">
-        <v>46.5</v>
+        <v>328</v>
       </c>
       <c r="D90" t="n">
-        <v>2.94</v>
+        <v>2.98</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>PANACHE</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>311</v>
+        <v>411.2</v>
       </c>
       <c r="C91" t="n">
-        <v>320</v>
+        <v>423.35</v>
       </c>
       <c r="D91" t="n">
-        <v>2.89</v>
+        <v>2.95</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>VARDMNPOLY</t>
+          <t>AURIGROW</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>7</v>
+        <v>0.34</v>
       </c>
       <c r="C92" t="n">
-        <v>7.2</v>
+        <v>0.35</v>
       </c>
       <c r="D92" t="n">
-        <v>2.86</v>
+        <v>2.94</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ORIENTLTD</t>
+          <t>KDL</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>63.1</v>
+        <v>123.1</v>
       </c>
       <c r="C93" t="n">
-        <v>64.90000000000001</v>
+        <v>126.7</v>
       </c>
       <c r="D93" t="n">
-        <v>2.85</v>
+        <v>2.92</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ELGIRUBCO</t>
+          <t>XTGLOBAL</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>49.55</v>
+        <v>29.04</v>
       </c>
       <c r="C94" t="n">
-        <v>50.95</v>
+        <v>29.88</v>
       </c>
       <c r="D94" t="n">
-        <v>2.83</v>
+        <v>2.89</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CORONA</t>
+          <t>DEEDEV</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1750.6</v>
+        <v>738.75</v>
       </c>
       <c r="C95" t="n">
-        <v>1800</v>
+        <v>760</v>
       </c>
       <c r="D95" t="n">
-        <v>2.82</v>
+        <v>2.88</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BODALCHEM</t>
+          <t>BUTTERFLY</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>65.38</v>
+        <v>664.1</v>
       </c>
       <c r="C96" t="n">
-        <v>67.2</v>
+        <v>683</v>
       </c>
       <c r="D96" t="n">
-        <v>2.78</v>
+        <v>2.85</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>DBEIL</t>
+          <t>ESSENTIA</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>86.81</v>
+        <v>1.41</v>
       </c>
       <c r="C97" t="n">
-        <v>89.2</v>
+        <v>1.45</v>
       </c>
       <c r="D97" t="n">
-        <v>2.75</v>
+        <v>2.84</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>BESTAGRO</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>15.96</v>
+        <v>411.2</v>
       </c>
       <c r="C98" t="n">
-        <v>16.39</v>
+        <v>422.8</v>
       </c>
       <c r="D98" t="n">
-        <v>2.69</v>
+        <v>2.82</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>NDLVENTURE</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>51.37</v>
+        <v>128.33</v>
       </c>
       <c r="C99" t="n">
-        <v>52.74</v>
+        <v>131.95</v>
       </c>
       <c r="D99" t="n">
-        <v>2.67</v>
+        <v>2.82</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>BIRLAPREC</t>
+          <t>DSSL</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>37.78</v>
+        <v>1352.6</v>
       </c>
       <c r="C100" t="n">
-        <v>38.79</v>
+        <v>1390</v>
       </c>
       <c r="D100" t="n">
-        <v>2.67</v>
+        <v>2.77</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>GOKEX</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1393.8</v>
+        <v>729.85</v>
       </c>
       <c r="C101" t="n">
-        <v>1431</v>
+        <v>750</v>
       </c>
       <c r="D101" t="n">
-        <v>2.67</v>
+        <v>2.76</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>RHL</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>19</v>
+        <v>186.64</v>
       </c>
       <c r="C102" t="n">
-        <v>19.5</v>
+        <v>191.8</v>
       </c>
       <c r="D102" t="n">
-        <v>2.63</v>
+        <v>2.76</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ALPA</t>
+          <t>TICL</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>70.55</v>
+        <v>20.35</v>
       </c>
       <c r="C103" t="n">
-        <v>72.40000000000001</v>
+        <v>20.89</v>
       </c>
       <c r="D103" t="n">
-        <v>2.62</v>
+        <v>2.65</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,14 +2705,14 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>VARDHACRLC</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>44.71</v>
+        <v>4.96</v>
       </c>
       <c r="C104" t="n">
-        <v>45.88</v>
+        <v>5.09</v>
       </c>
       <c r="D104" t="n">
         <v>2.62</v>
@@ -2727,14 +2727,14 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>AARON</t>
+          <t>TECILCHEM</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>124.45</v>
+        <v>11.1</v>
       </c>
       <c r="C105" t="n">
-        <v>127.7</v>
+        <v>11.39</v>
       </c>
       <c r="D105" t="n">
         <v>2.61</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>SAKUMA</t>
+          <t>PEARLPOLY</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>1.93</v>
+        <v>18.99</v>
       </c>
       <c r="C106" t="n">
-        <v>1.98</v>
+        <v>19.48</v>
       </c>
       <c r="D106" t="n">
-        <v>2.59</v>
+        <v>2.58</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SUVIDHAA</t>
+          <t>KRISHNADEF</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>2.71</v>
+        <v>1306</v>
       </c>
       <c r="C107" t="n">
-        <v>2.78</v>
+        <v>1339</v>
       </c>
       <c r="D107" t="n">
-        <v>2.58</v>
+        <v>2.53</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>EUROBOND</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>11.25</v>
+        <v>179.46</v>
       </c>
       <c r="C108" t="n">
-        <v>11.54</v>
+        <v>184</v>
       </c>
       <c r="D108" t="n">
-        <v>2.58</v>
+        <v>2.53</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SURAKSHA</t>
+          <t>DELTAMAGNT</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>270.05</v>
+        <v>61.45</v>
       </c>
       <c r="C109" t="n">
-        <v>277</v>
+        <v>63</v>
       </c>
       <c r="D109" t="n">
-        <v>2.57</v>
+        <v>2.52</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>AMBALALSA</t>
+          <t>IVP</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>32.18</v>
+        <v>158.01</v>
       </c>
       <c r="C110" t="n">
-        <v>33</v>
+        <v>161.99</v>
       </c>
       <c r="D110" t="n">
-        <v>2.55</v>
+        <v>2.52</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>DAICHI</t>
+          <t>VIGOR</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>284.55</v>
+        <v>89.65000000000001</v>
       </c>
       <c r="C111" t="n">
-        <v>291.79</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="D111" t="n">
-        <v>2.54</v>
+        <v>2.51</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>HLVLTD</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>3.15</v>
+        <v>7.98</v>
       </c>
       <c r="C112" t="n">
-        <v>3.23</v>
+        <v>8.18</v>
       </c>
       <c r="D112" t="n">
-        <v>2.54</v>
+        <v>2.51</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>VASWANI</t>
+          <t>SARTELE</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>58.52</v>
+        <v>160.65</v>
       </c>
       <c r="C113" t="n">
-        <v>60</v>
+        <v>164.65</v>
       </c>
       <c r="D113" t="n">
-        <v>2.53</v>
+        <v>2.49</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CORALFINAC</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>32.18</v>
+        <v>5289</v>
       </c>
       <c r="C114" t="n">
-        <v>32.99</v>
+        <v>5420</v>
       </c>
       <c r="D114" t="n">
-        <v>2.52</v>
+        <v>2.48</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ALANKIT</t>
+          <t>RAYMONDREL</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>8.359999999999999</v>
+        <v>595.3</v>
       </c>
       <c r="C115" t="n">
-        <v>8.57</v>
+        <v>609.95</v>
       </c>
       <c r="D115" t="n">
-        <v>2.51</v>
+        <v>2.46</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>NILAINFRA</t>
+          <t>NIBE</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>7.99</v>
+        <v>1625.3</v>
       </c>
       <c r="C116" t="n">
-        <v>8.19</v>
+        <v>1665</v>
       </c>
       <c r="D116" t="n">
-        <v>2.5</v>
+        <v>2.44</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>WEWIN</t>
+          <t>RVNL</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>50.48</v>
+        <v>245.14</v>
       </c>
       <c r="C117" t="n">
-        <v>51.74</v>
+        <v>251.02</v>
       </c>
       <c r="D117" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>GVPTECH</t>
+          <t>PRITIKAUTO</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>6.41</v>
+        <v>16.66</v>
       </c>
       <c r="C118" t="n">
-        <v>6.57</v>
+        <v>17.06</v>
       </c>
       <c r="D118" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ONELIFECAP</t>
+          <t>CLSEL</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>28.08</v>
+        <v>296.35</v>
       </c>
       <c r="C119" t="n">
-        <v>28.78</v>
+        <v>303.45</v>
       </c>
       <c r="D119" t="n">
-        <v>2.49</v>
+        <v>2.4</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>7.67</v>
+        <v>33.21</v>
       </c>
       <c r="C120" t="n">
-        <v>7.86</v>
+        <v>34</v>
       </c>
       <c r="D120" t="n">
-        <v>2.48</v>
+        <v>2.38</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ANTGRAPHIC</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.42</v>
       </c>
       <c r="C121" t="n">
-        <v>0.83</v>
+        <v>0.43</v>
       </c>
       <c r="D121" t="n">
-        <v>2.47</v>
+        <v>2.38</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>AVG</t>
+          <t>WEALTH</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>169.83</v>
+        <v>952.5</v>
       </c>
       <c r="C122" t="n">
-        <v>174</v>
+        <v>975</v>
       </c>
       <c r="D122" t="n">
-        <v>2.46</v>
+        <v>2.36</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>FINKURVE</t>
+          <t>PANSARI</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>71.27</v>
+        <v>309.7</v>
       </c>
       <c r="C123" t="n">
-        <v>73.02</v>
+        <v>316.95</v>
       </c>
       <c r="D123" t="n">
-        <v>2.46</v>
+        <v>2.34</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SJLOGISTIC</t>
+          <t>AARON</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>344.6</v>
+        <v>124.58</v>
       </c>
       <c r="C124" t="n">
-        <v>352.95</v>
+        <v>127.5</v>
       </c>
       <c r="D124" t="n">
-        <v>2.42</v>
+        <v>2.34</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>BLUSPRING</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>3.35</v>
+        <v>109.35</v>
       </c>
       <c r="C125" t="n">
-        <v>3.43</v>
+        <v>111.89</v>
       </c>
       <c r="D125" t="n">
-        <v>2.39</v>
+        <v>2.32</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>GSLSU</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>5.86</v>
+        <v>51.8</v>
       </c>
       <c r="C126" t="n">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="D126" t="n">
-        <v>2.39</v>
+        <v>2.32</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>UNIMECH</t>
+          <t>PENINLAND</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>1137.9</v>
+        <v>16.03</v>
       </c>
       <c r="C127" t="n">
-        <v>1164.95</v>
+        <v>16.4</v>
       </c>
       <c r="D127" t="n">
-        <v>2.38</v>
+        <v>2.31</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>GANGAFORGE</t>
+          <t>HPAL</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>2.53</v>
+        <v>36.12</v>
       </c>
       <c r="C128" t="n">
-        <v>2.59</v>
+        <v>36.95</v>
       </c>
       <c r="D128" t="n">
-        <v>2.37</v>
+        <v>2.3</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>GVPIL</t>
+          <t>AGRITECH</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>1024.8</v>
+        <v>116.81</v>
       </c>
       <c r="C129" t="n">
-        <v>1048.95</v>
+        <v>119.5</v>
       </c>
       <c r="D129" t="n">
-        <v>2.36</v>
+        <v>2.3</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>VLEGOV</t>
+          <t>EVERESTIND</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>13.97</v>
+        <v>371.3</v>
       </c>
       <c r="C130" t="n">
-        <v>14.3</v>
+        <v>379.8</v>
       </c>
       <c r="D130" t="n">
-        <v>2.36</v>
+        <v>2.29</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>AMANTA</t>
+          <t>SPAL</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>150.27</v>
+        <v>830.95</v>
       </c>
       <c r="C131" t="n">
-        <v>153.8</v>
+        <v>850</v>
       </c>
       <c r="D131" t="n">
-        <v>2.35</v>
+        <v>2.29</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>3BBLACKBIO</t>
+          <t>SANGHVIMOV</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>1258.7</v>
+        <v>416.5</v>
       </c>
       <c r="C132" t="n">
-        <v>1288</v>
+        <v>425.95</v>
       </c>
       <c r="D132" t="n">
-        <v>2.33</v>
+        <v>2.27</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ODIGMA</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>23.15</v>
+        <v>767.5</v>
       </c>
       <c r="C133" t="n">
-        <v>23.69</v>
+        <v>784.95</v>
       </c>
       <c r="D133" t="n">
-        <v>2.33</v>
+        <v>2.27</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>360ONE</t>
+          <t>ALMONDZ</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>1133.6</v>
+        <v>13.45</v>
       </c>
       <c r="C134" t="n">
-        <v>1160</v>
+        <v>13.75</v>
       </c>
       <c r="D134" t="n">
-        <v>2.33</v>
+        <v>2.23</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>GRADIENTE</t>
+          <t>METROBRAND</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>2.17</v>
+        <v>1022.2</v>
       </c>
       <c r="C135" t="n">
-        <v>2.22</v>
+        <v>1045</v>
       </c>
       <c r="D135" t="n">
-        <v>2.3</v>
+        <v>2.23</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>BGRENERGY</t>
+          <t>HDIL</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>330.25</v>
+        <v>1.8</v>
       </c>
       <c r="C136" t="n">
-        <v>337.8</v>
+        <v>1.84</v>
       </c>
       <c r="D136" t="n">
-        <v>2.29</v>
+        <v>2.22</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>GLOBECIVIL</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>43.65</v>
+        <v>6.31</v>
       </c>
       <c r="C137" t="n">
-        <v>44.65</v>
+        <v>6.45</v>
       </c>
       <c r="D137" t="n">
-        <v>2.29</v>
+        <v>2.22</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>JISLDVREQS</t>
+          <t>BBTCL</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>23.76</v>
+        <v>218.16</v>
       </c>
       <c r="C138" t="n">
-        <v>24.3</v>
+        <v>223</v>
       </c>
       <c r="D138" t="n">
-        <v>2.27</v>
+        <v>2.22</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>GAYAHWS</t>
+          <t>JHS</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>2.21</v>
+        <v>8.1</v>
       </c>
       <c r="C139" t="n">
-        <v>2.26</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="D139" t="n">
-        <v>2.26</v>
+        <v>2.22</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>DUCON</t>
+          <t>INDOUS</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>3.61</v>
+        <v>90.47</v>
       </c>
       <c r="C140" t="n">
-        <v>3.69</v>
+        <v>92.45</v>
       </c>
       <c r="D140" t="n">
-        <v>2.22</v>
+        <v>2.19</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>AKSHAR</t>
+          <t>UNIHEALTH</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>0.45</v>
+        <v>547.8</v>
       </c>
       <c r="C141" t="n">
-        <v>0.46</v>
+        <v>559.8</v>
       </c>
       <c r="D141" t="n">
-        <v>2.22</v>
+        <v>2.19</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>DRCSYSTEMS</t>
+          <t>K2INFRA</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>14.42</v>
+        <v>78.3</v>
       </c>
       <c r="C142" t="n">
-        <v>14.74</v>
+        <v>80</v>
       </c>
       <c r="D142" t="n">
-        <v>2.22</v>
+        <v>2.17</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>BANKA</t>
+          <t>NILASPACES</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>87.09</v>
+        <v>13.02</v>
       </c>
       <c r="C143" t="n">
-        <v>89</v>
+        <v>13.3</v>
       </c>
       <c r="D143" t="n">
-        <v>2.19</v>
+        <v>2.15</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>RUSHIL</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>29.26</v>
+        <v>17.81</v>
       </c>
       <c r="C144" t="n">
-        <v>29.9</v>
+        <v>18.19</v>
       </c>
       <c r="D144" t="n">
-        <v>2.19</v>
+        <v>2.13</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>SHREDIGCEM</t>
+          <t>GATECHDVR</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>73.38</v>
+        <v>0.47</v>
       </c>
       <c r="C145" t="n">
-        <v>74.98999999999999</v>
+        <v>0.48</v>
       </c>
       <c r="D145" t="n">
-        <v>2.19</v>
+        <v>2.13</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>ENERGYDEV</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>11.12</v>
+        <v>16.98</v>
       </c>
       <c r="C146" t="n">
-        <v>11.36</v>
+        <v>17.34</v>
       </c>
       <c r="D146" t="n">
-        <v>2.16</v>
+        <v>2.12</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>NDRAUTO</t>
+          <t>THYROCARE</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>843.85</v>
+        <v>533.5</v>
       </c>
       <c r="C147" t="n">
-        <v>862</v>
+        <v>544.8</v>
       </c>
       <c r="D147" t="n">
-        <v>2.15</v>
+        <v>2.12</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>COASTCORP</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.47</v>
+        <v>51.16</v>
       </c>
       <c r="C148" t="n">
-        <v>0.48</v>
+        <v>52.24</v>
       </c>
       <c r="D148" t="n">
-        <v>2.13</v>
+        <v>2.11</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>DPWIRES</t>
+          <t>VIPCLOTHNG</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>176.25</v>
+        <v>25.15</v>
       </c>
       <c r="C149" t="n">
-        <v>179.99</v>
+        <v>25.68</v>
       </c>
       <c r="D149" t="n">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>KFINTECH</t>
+          <t>MALLCOM</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>861.75</v>
+        <v>1097</v>
       </c>
       <c r="C150" t="n">
-        <v>880</v>
+        <v>1120</v>
       </c>
       <c r="D150" t="n">
-        <v>2.12</v>
+        <v>2.1</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MDL</t>
+          <t>DMCC</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>73.45</v>
+        <v>252.65</v>
       </c>
       <c r="C151" t="n">
-        <v>75</v>
+        <v>257.9</v>
       </c>
       <c r="D151" t="n">
-        <v>2.11</v>
+        <v>2.08</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CKKRETAIL</t>
+          <t>GEEKAYWIRE</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>145</v>
+        <v>25.42</v>
       </c>
       <c r="C152" t="n">
-        <v>148.05</v>
+        <v>25.95</v>
       </c>
       <c r="D152" t="n">
-        <v>2.1</v>
+        <v>2.08</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>BORANA</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>317.25</v>
+        <v>4.38</v>
       </c>
       <c r="C153" t="n">
-        <v>323.9</v>
+        <v>4.47</v>
       </c>
       <c r="D153" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>ROSSELLIND</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>44.56</v>
+        <v>55.91</v>
       </c>
       <c r="C154" t="n">
-        <v>45.49</v>
+        <v>57.05</v>
       </c>
       <c r="D154" t="n">
-        <v>2.09</v>
+        <v>2.04</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>SPCENET</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>3.36</v>
+        <v>0.49</v>
       </c>
       <c r="C155" t="n">
-        <v>3.43</v>
+        <v>0.5</v>
       </c>
       <c r="D155" t="n">
-        <v>2.08</v>
+        <v>2.04</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>BIKEWO</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>391.65</v>
+        <v>29.6</v>
       </c>
       <c r="C156" t="n">
-        <v>399.8</v>
+        <v>30.2</v>
       </c>
       <c r="D156" t="n">
-        <v>2.08</v>
+        <v>2.03</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>C2C</t>
+          <t>AKSHOPTFBR</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>401.65</v>
+        <v>6.9</v>
       </c>
       <c r="C157" t="n">
-        <v>409.95</v>
+        <v>7.04</v>
       </c>
       <c r="D157" t="n">
-        <v>2.07</v>
+        <v>2.03</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>COFORGE</t>
+          <t>HAPPYFORGE</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>1464.8</v>
+        <v>1431.2</v>
       </c>
       <c r="C158" t="n">
-        <v>1494.5</v>
+        <v>1460</v>
       </c>
       <c r="D158" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>FIBERWEB</t>
+          <t>VAISHALI</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>29</v>
+        <v>7.45</v>
       </c>
       <c r="C159" t="n">
-        <v>29.59</v>
+        <v>7.6</v>
       </c>
       <c r="D159" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>LASA</t>
+          <t>JKIPL</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>7.44</v>
+        <v>117.34</v>
       </c>
       <c r="C160" t="n">
-        <v>7.59</v>
+        <v>119.7</v>
       </c>
       <c r="D160" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>BRANDMAN</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>20.34</v>
+        <v>182</v>
       </c>
       <c r="C161" t="n">
-        <v>20.75</v>
+        <v>185.65</v>
       </c>
       <c r="D161" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>KPL</t>
+          <t>MOKSH</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>2413.6</v>
+        <v>11.99</v>
       </c>
       <c r="C162" t="n">
-        <v>2462</v>
+        <v>12.23</v>
       </c>
       <c r="D162" t="n">
-        <v>2.01</v>
+        <v>2</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>LATTEYS</t>
+          <t>SILLYMONKS</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>22.4</v>
+        <v>17.02</v>
       </c>
       <c r="C163" t="n">
-        <v>22.85</v>
+        <v>17.36</v>
       </c>
       <c r="D163" t="n">
-        <v>2.01</v>
+        <v>2</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>UMAEXPORTS</t>
+          <t>MAHESHWARI</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>25</v>
+        <v>71.33</v>
       </c>
       <c r="C164" t="n">
-        <v>25.5</v>
+        <v>72.75</v>
       </c>
       <c r="D164" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>MAJESAUT</t>
+          <t>TRANSPEK</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>338.15</v>
+        <v>998.5</v>
       </c>
       <c r="C165" t="n">
-        <v>344.9</v>
+        <v>1018.4</v>
       </c>
       <c r="D165" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>MHLXMIRU</t>
+          <t>SHEMAROO</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>170.59</v>
+        <v>129.53</v>
       </c>
       <c r="C166" t="n">
-        <v>174</v>
+        <v>132.1</v>
       </c>
       <c r="D166" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>PLASTIBLEN</t>
+          <t>SIL</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>173</v>
+        <v>15.68</v>
       </c>
       <c r="C167" t="n">
-        <v>176.45</v>
+        <v>15.99</v>
       </c>
       <c r="D167" t="n">
-        <v>1.99</v>
+        <v>1.98</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>ESTER</t>
+          <t>BHARATSE</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>91.18000000000001</v>
+        <v>184.37</v>
       </c>
       <c r="C168" t="n">
-        <v>92.98999999999999</v>
+        <v>188</v>
       </c>
       <c r="D168" t="n">
-        <v>1.99</v>
+        <v>1.97</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>BHANDARI</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>38.24</v>
+        <v>3.06</v>
       </c>
       <c r="C169" t="n">
-        <v>39</v>
+        <v>3.12</v>
       </c>
       <c r="D169" t="n">
-        <v>1.99</v>
+        <v>1.96</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>BIGBLOC</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>50.46</v>
+        <v>8.66</v>
       </c>
       <c r="C170" t="n">
-        <v>51.46</v>
+        <v>8.83</v>
       </c>
       <c r="D170" t="n">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>TPLPLASTEH</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>67.06999999999999</v>
+        <v>196.16</v>
       </c>
       <c r="C171" t="n">
-        <v>68.40000000000001</v>
+        <v>200</v>
       </c>
       <c r="D171" t="n">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>MURUDCERA</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>31.5</v>
+        <v>0.51</v>
       </c>
       <c r="C172" t="n">
-        <v>32.12</v>
+        <v>0.52</v>
       </c>
       <c r="D172" t="n">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>PRAENG</t>
+          <t>IGCL</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>21.35</v>
+        <v>63.71</v>
       </c>
       <c r="C173" t="n">
-        <v>21.77</v>
+        <v>64.95999999999999</v>
       </c>
       <c r="D173" t="n">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>7.16</v>
+        <v>955.55</v>
       </c>
       <c r="C174" t="n">
-        <v>7.3</v>
+        <v>974.15</v>
       </c>
       <c r="D174" t="n">
-        <v>1.96</v>
+        <v>1.95</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ROML</t>
+          <t>SAHANA</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>45.51</v>
+        <v>936.8</v>
       </c>
       <c r="C175" t="n">
-        <v>46.4</v>
+        <v>954.95</v>
       </c>
       <c r="D175" t="n">
-        <v>1.96</v>
+        <v>1.94</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MANBA</t>
+          <t>RPTECH</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>127.52</v>
+        <v>685.8</v>
       </c>
       <c r="C176" t="n">
-        <v>130</v>
+        <v>699.05</v>
       </c>
       <c r="D176" t="n">
-        <v>1.94</v>
+        <v>1.93</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>NIPPOBATRY</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>358.95</v>
+        <v>20.74</v>
       </c>
       <c r="C177" t="n">
-        <v>365.9</v>
+        <v>21.14</v>
       </c>
       <c r="D177" t="n">
-        <v>1.94</v>
+        <v>1.93</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>GOKUL</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>40.71</v>
+        <v>10.94</v>
       </c>
       <c r="C178" t="n">
-        <v>41.5</v>
+        <v>11.15</v>
       </c>
       <c r="D178" t="n">
-        <v>1.94</v>
+        <v>1.92</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>21STCENMGM</t>
+          <t>SACHEEROME</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>32.13</v>
+        <v>322.8</v>
       </c>
       <c r="C179" t="n">
-        <v>32.75</v>
+        <v>329</v>
       </c>
       <c r="D179" t="n">
-        <v>1.93</v>
+        <v>1.92</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>SURANAT&amp;P</t>
+          <t>VIVIDHA</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>19.14</v>
+        <v>0.52</v>
       </c>
       <c r="C180" t="n">
-        <v>19.51</v>
+        <v>0.53</v>
       </c>
       <c r="D180" t="n">
-        <v>1.93</v>
+        <v>1.92</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>HIMATSEIDE</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>0.52</v>
+        <v>78.55</v>
       </c>
       <c r="C181" t="n">
-        <v>0.53</v>
+        <v>80.05</v>
       </c>
       <c r="D181" t="n">
-        <v>1.92</v>
+        <v>1.91</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,14 +4421,14 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>PINELABS</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>150.09</v>
+        <v>3.16</v>
       </c>
       <c r="C182" t="n">
-        <v>152.94</v>
+        <v>3.22</v>
       </c>
       <c r="D182" t="n">
         <v>1.9</v>
@@ -4443,14 +4443,14 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>ARSHIYA</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>53.91</v>
+        <v>1.06</v>
       </c>
       <c r="C183" t="n">
-        <v>54.93</v>
+        <v>1.08</v>
       </c>
       <c r="D183" t="n">
         <v>1.89</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>NECLIFE</t>
+          <t>MAHEPC</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>11.78</v>
+        <v>116.71</v>
       </c>
       <c r="C184" t="n">
-        <v>12</v>
+        <v>118.9</v>
       </c>
       <c r="D184" t="n">
-        <v>1.87</v>
+        <v>1.88</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>KALYANIFRG</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>54.47</v>
+        <v>593</v>
       </c>
       <c r="C185" t="n">
-        <v>55.49</v>
+        <v>604</v>
       </c>
       <c r="D185" t="n">
-        <v>1.87</v>
+        <v>1.85</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>PAVNAIND</t>
+          <t>GRPLTD</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>17.08</v>
+        <v>1811.4</v>
       </c>
       <c r="C186" t="n">
-        <v>17.4</v>
+        <v>1845</v>
       </c>
       <c r="D186" t="n">
-        <v>1.87</v>
+        <v>1.85</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>EMAMIPAP</t>
+          <t>AMIRCHAND</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>84.23999999999999</v>
+        <v>129.52</v>
       </c>
       <c r="C187" t="n">
-        <v>85.8</v>
+        <v>131.9</v>
       </c>
       <c r="D187" t="n">
-        <v>1.85</v>
+        <v>1.84</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,14 +4553,14 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>SIGNATURE</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>348.6</v>
+        <v>792.35</v>
       </c>
       <c r="C188" t="n">
-        <v>355</v>
+        <v>806.95</v>
       </c>
       <c r="D188" t="n">
         <v>1.84</v>
@@ -4575,17 +4575,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>NAUKRI</t>
+          <t>PIGL</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>997.65</v>
+        <v>107.04</v>
       </c>
       <c r="C189" t="n">
-        <v>1016</v>
+        <v>109</v>
       </c>
       <c r="D189" t="n">
-        <v>1.84</v>
+        <v>1.83</v>
       </c>
       <c r="E189" t="b">
         <v>0</v>
@@ -4597,17 +4597,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>HINDCOMPOS</t>
+          <t>FAZE3Q</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>419.4</v>
+        <v>565.65</v>
       </c>
       <c r="C190" t="n">
-        <v>427</v>
+        <v>576</v>
       </c>
       <c r="D190" t="n">
-        <v>1.81</v>
+        <v>1.83</v>
       </c>
       <c r="E190" t="b">
         <v>0</v>
@@ -4619,17 +4619,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>MKPL</t>
+          <t>PONNIERODE</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>4.97</v>
+        <v>317.3</v>
       </c>
       <c r="C191" t="n">
-        <v>5.06</v>
+        <v>323</v>
       </c>
       <c r="D191" t="n">
-        <v>1.81</v>
+        <v>1.8</v>
       </c>
       <c r="E191" t="b">
         <v>0</v>
@@ -4641,17 +4641,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>APOLLOTYRE</t>
+          <t>EMCURE</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>416.45</v>
+        <v>1725.7</v>
       </c>
       <c r="C192" t="n">
-        <v>424</v>
+        <v>1756.8</v>
       </c>
       <c r="D192" t="n">
-        <v>1.81</v>
+        <v>1.8</v>
       </c>
       <c r="E192" t="b">
         <v>0</v>
@@ -4663,17 +4663,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>SASKEN</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>24.4</v>
+        <v>2407.2</v>
       </c>
       <c r="C193" t="n">
-        <v>24.84</v>
+        <v>2450</v>
       </c>
       <c r="D193" t="n">
-        <v>1.8</v>
+        <v>1.78</v>
       </c>
       <c r="E193" t="b">
         <v>0</v>
@@ -4685,17 +4685,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>MAFATIND</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>3.91</v>
+        <v>128.72</v>
       </c>
       <c r="C194" t="n">
-        <v>3.98</v>
+        <v>131</v>
       </c>
       <c r="D194" t="n">
-        <v>1.79</v>
+        <v>1.77</v>
       </c>
       <c r="E194" t="b">
         <v>0</v>
@@ -4707,17 +4707,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>DMCC</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>258.4</v>
+        <v>14.14</v>
       </c>
       <c r="C195" t="n">
-        <v>263</v>
+        <v>14.39</v>
       </c>
       <c r="D195" t="n">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
       <c r="E195" t="b">
         <v>0</v>
@@ -4729,17 +4729,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>CIFL</t>
+          <t>BLUECOAST</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>24.9</v>
+        <v>28.5</v>
       </c>
       <c r="C196" t="n">
-        <v>25.34</v>
+        <v>29</v>
       </c>
       <c r="D196" t="n">
-        <v>1.77</v>
+        <v>1.75</v>
       </c>
       <c r="E196" t="b">
         <v>0</v>
@@ -4751,17 +4751,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>PATINTLOG</t>
+          <t>PANACEABIO</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>13.76</v>
+        <v>532.2</v>
       </c>
       <c r="C197" t="n">
-        <v>14</v>
+        <v>541.5</v>
       </c>
       <c r="D197" t="n">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
       <c r="E197" t="b">
         <v>0</v>
@@ -4773,17 +4773,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>REDINGTON</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>2.31</v>
+        <v>248.92</v>
       </c>
       <c r="C198" t="n">
-        <v>2.35</v>
+        <v>253.24</v>
       </c>
       <c r="D198" t="n">
-        <v>1.73</v>
+        <v>1.74</v>
       </c>
       <c r="E198" t="b">
         <v>0</v>
@@ -4795,14 +4795,14 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>KPRMILL</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>49.15</v>
+        <v>1043.25</v>
       </c>
       <c r="C199" t="n">
-        <v>50</v>
+        <v>1061.35</v>
       </c>
       <c r="D199" t="n">
         <v>1.73</v>
@@ -4817,17 +4817,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>FEDFINA</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>28.95</v>
+        <v>159.64</v>
       </c>
       <c r="C200" t="n">
-        <v>29.45</v>
+        <v>162.39</v>
       </c>
       <c r="D200" t="n">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
       <c r="E200" t="b">
         <v>0</v>
@@ -4839,17 +4839,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>BALAJEE</t>
+          <t>KRMAYURVED</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>29.3</v>
+        <v>250</v>
       </c>
       <c r="C201" t="n">
-        <v>29.8</v>
+        <v>254.25</v>
       </c>
       <c r="D201" t="n">
-        <v>1.71</v>
+        <v>1.7</v>
       </c>
       <c r="E201" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Auto: update momentum data - 2026-06-19 08:55 UTC
</commit_message>
<xml_diff>
--- a/data/trending_momentum_stocks.xlsx
+++ b/data/trending_momentum_stocks.xlsx
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EIFFL</t>
+          <t>RELTD-RE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>298.57</v>
+        <v>25.98</v>
       </c>
       <c r="C2" t="n">
-        <v>355</v>
+        <v>36.37</v>
       </c>
       <c r="D2" t="n">
-        <v>18.9</v>
+        <v>39.99</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="D3" t="n">
-        <v>16.67</v>
+        <v>14.29</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -505,17 +505,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DHARIWAL</t>
+          <t>REGENCERAM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28.7</v>
+        <v>40.51</v>
       </c>
       <c r="C4" t="n">
-        <v>32.5</v>
+        <v>44.75</v>
       </c>
       <c r="D4" t="n">
-        <v>13.24</v>
+        <v>10.47</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LPDC</t>
+          <t>VIPULLTD</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.76</v>
+        <v>10.13</v>
       </c>
       <c r="C5" t="n">
-        <v>7.3</v>
+        <v>11.14</v>
       </c>
       <c r="D5" t="n">
-        <v>7.99</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -549,17 +549,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DHARAN</t>
+          <t>DELPHIFX</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.16</v>
+        <v>8.4</v>
       </c>
       <c r="C6" t="n">
-        <v>0.17</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>6.25</v>
+        <v>9.52</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -571,17 +571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ACEINTEG</t>
+          <t>HYBRIDFIN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20.7</v>
+        <v>22.69</v>
       </c>
       <c r="C7" t="n">
-        <v>21.99</v>
+        <v>24.5</v>
       </c>
       <c r="D7" t="n">
-        <v>6.23</v>
+        <v>7.98</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -593,17 +593,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GRANDOAK</t>
+          <t>RKEC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>43.81</v>
+        <v>26.7</v>
       </c>
       <c r="C8" t="n">
-        <v>46.49</v>
+        <v>28.8</v>
       </c>
       <c r="D8" t="n">
-        <v>6.12</v>
+        <v>7.87</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>POWERICA</t>
+          <t>SELMC</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>529.8</v>
+        <v>29.68</v>
       </c>
       <c r="C9" t="n">
-        <v>560.95</v>
+        <v>31.8</v>
       </c>
       <c r="D9" t="n">
-        <v>5.88</v>
+        <v>7.14</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -637,17 +637,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ZENITHSTL</t>
+          <t>SHRIKRISH</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5.93</v>
+        <v>42.94</v>
       </c>
       <c r="C10" t="n">
-        <v>6.27</v>
+        <v>45.85</v>
       </c>
       <c r="D10" t="n">
-        <v>5.73</v>
+        <v>6.78</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABMINTLLTD</t>
+          <t>DHARAN</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>40.79</v>
+        <v>0.16</v>
       </c>
       <c r="C11" t="n">
-        <v>42.94</v>
+        <v>0.17</v>
       </c>
       <c r="D11" t="n">
-        <v>5.27</v>
+        <v>6.25</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>KIRLFER</t>
+          <t>SURYALA</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>444.3</v>
+        <v>452.35</v>
       </c>
       <c r="C12" t="n">
-        <v>467</v>
+        <v>479.95</v>
       </c>
       <c r="D12" t="n">
-        <v>5.11</v>
+        <v>6.1</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -703,17 +703,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SIGNORIA</t>
+          <t>NIBL</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>80</v>
+        <v>30.94</v>
       </c>
       <c r="C13" t="n">
-        <v>84</v>
+        <v>32.78</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>5.95</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -725,17 +725,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RAJESHEXPO</t>
+          <t>ORCHASP</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>88.45</v>
+        <v>1.86</v>
       </c>
       <c r="C14" t="n">
-        <v>92.87</v>
+        <v>1.97</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>5.91</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -747,17 +747,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NIRAJ</t>
+          <t>AIRAN</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>31</v>
+        <v>16.27</v>
       </c>
       <c r="C15" t="n">
-        <v>32.55</v>
+        <v>17.15</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>5.41</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -769,17 +769,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MARC</t>
+          <t>SHANTI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>6.55</v>
       </c>
       <c r="C16" t="n">
-        <v>76.65000000000001</v>
+        <v>6.9</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>5.34</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -791,17 +791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SICALLOG</t>
+          <t>PATINTLOG</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>96.64</v>
+        <v>14.28</v>
       </c>
       <c r="C17" t="n">
-        <v>101.47</v>
+        <v>15</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>5.04</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -813,14 +813,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ZEELEARN</t>
+          <t>DIVYADHAN</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="C18" t="n">
-        <v>8.4</v>
+        <v>39.9</v>
       </c>
       <c r="D18" t="n">
         <v>5</v>
@@ -835,14 +835,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>APEXECO</t>
+          <t>RAJESHEXPO</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>213.15</v>
+        <v>92.87</v>
       </c>
       <c r="C19" t="n">
-        <v>223.8</v>
+        <v>97.51000000000001</v>
       </c>
       <c r="D19" t="n">
         <v>5</v>
@@ -857,14 +857,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SEJALLTD</t>
+          <t>AHLWEST</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>761.25</v>
+        <v>571.3</v>
       </c>
       <c r="C20" t="n">
-        <v>799.3</v>
+        <v>599.85</v>
       </c>
       <c r="D20" t="n">
         <v>5</v>
@@ -879,14 +879,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>VISL</t>
+          <t>ZEELEARN</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>23.21</v>
+        <v>8.4</v>
       </c>
       <c r="C21" t="n">
-        <v>24.37</v>
+        <v>8.82</v>
       </c>
       <c r="D21" t="n">
         <v>5</v>
@@ -901,17 +901,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HMT</t>
+          <t>SEJALLTD</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>58.73</v>
+        <v>799.3</v>
       </c>
       <c r="C22" t="n">
-        <v>61.66</v>
+        <v>839.25</v>
       </c>
       <c r="D22" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -923,17 +923,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SHYAMTEL</t>
+          <t>HMT</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>17.25</v>
+        <v>61.66</v>
       </c>
       <c r="C23" t="n">
-        <v>18.11</v>
+        <v>64.73999999999999</v>
       </c>
       <c r="D23" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -945,14 +945,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BHAGYANGR</t>
+          <t>UTSSAV</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>359.5</v>
+        <v>363.55</v>
       </c>
       <c r="C24" t="n">
-        <v>377.45</v>
+        <v>381.7</v>
       </c>
       <c r="D24" t="n">
         <v>4.99</v>
@@ -967,14 +967,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SAHASRA</t>
+          <t>RSSOFTWARE</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>326.55</v>
+        <v>34.87</v>
       </c>
       <c r="C25" t="n">
-        <v>342.85</v>
+        <v>36.61</v>
       </c>
       <c r="D25" t="n">
         <v>4.99</v>
@@ -989,14 +989,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VIDYAWIRES</t>
+          <t>KANORICHEM</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>103.11</v>
+        <v>114.98</v>
       </c>
       <c r="C26" t="n">
-        <v>108.26</v>
+        <v>120.72</v>
       </c>
       <c r="D26" t="n">
         <v>4.99</v>
@@ -1011,17 +1011,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CALSOFT</t>
+          <t>TROM</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>23.07</v>
+        <v>57.1</v>
       </c>
       <c r="C27" t="n">
-        <v>24.22</v>
+        <v>59.95</v>
       </c>
       <c r="D27" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1033,17 +1033,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GANESHIN</t>
+          <t>IBULLSLTD</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>108.45</v>
+        <v>25.25</v>
       </c>
       <c r="C28" t="n">
-        <v>113.85</v>
+        <v>26.51</v>
       </c>
       <c r="D28" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1055,14 +1055,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SMARTEN</t>
+          <t>MRIL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>59.2</v>
+        <v>56.2</v>
       </c>
       <c r="C29" t="n">
-        <v>62.15</v>
+        <v>59</v>
       </c>
       <c r="D29" t="n">
         <v>4.98</v>
@@ -1077,17 +1077,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ACCORD</t>
+          <t>APEXECO</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>99.59999999999999</v>
+        <v>223.8</v>
       </c>
       <c r="C30" t="n">
-        <v>104.55</v>
+        <v>234.95</v>
       </c>
       <c r="D30" t="n">
-        <v>4.97</v>
+        <v>4.98</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1099,17 +1099,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TECHERA</t>
+          <t>OWAIS</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>169.85</v>
+        <v>114.35</v>
       </c>
       <c r="C31" t="n">
-        <v>178.3</v>
+        <v>120.05</v>
       </c>
       <c r="D31" t="n">
-        <v>4.97</v>
+        <v>4.98</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1121,17 +1121,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>INNOMET</t>
+          <t>PALREDTEC</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>111.9</v>
+        <v>53.25</v>
       </c>
       <c r="C32" t="n">
-        <v>117.45</v>
+        <v>55.9</v>
       </c>
       <c r="D32" t="n">
-        <v>4.96</v>
+        <v>4.98</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1143,17 +1143,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OWAIS</t>
+          <t>NIRAJ</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>108.95</v>
+        <v>32.55</v>
       </c>
       <c r="C33" t="n">
-        <v>114.35</v>
+        <v>34.17</v>
       </c>
       <c r="D33" t="n">
-        <v>4.96</v>
+        <v>4.98</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1165,17 +1165,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PALREDTEC</t>
+          <t>AKSHOPTFBR</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>50.72</v>
+        <v>7.24</v>
       </c>
       <c r="C34" t="n">
-        <v>53.2</v>
+        <v>7.6</v>
       </c>
       <c r="D34" t="n">
-        <v>4.89</v>
+        <v>4.97</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1187,17 +1187,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>VIJIFIN</t>
+          <t>BHAGYANGR</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4.1</v>
+        <v>377.45</v>
       </c>
       <c r="C35" t="n">
-        <v>4.3</v>
+        <v>396.2</v>
       </c>
       <c r="D35" t="n">
-        <v>4.88</v>
+        <v>4.97</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1209,17 +1209,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ROLLT</t>
+          <t>NEAGI</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3.09</v>
+        <v>3248.8</v>
       </c>
       <c r="C36" t="n">
-        <v>3.24</v>
+        <v>3410</v>
       </c>
       <c r="D36" t="n">
-        <v>4.85</v>
+        <v>4.96</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1231,17 +1231,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OSIAHYPER</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3.51</v>
+        <v>3.24</v>
       </c>
       <c r="C37" t="n">
-        <v>3.68</v>
+        <v>3.4</v>
       </c>
       <c r="D37" t="n">
-        <v>4.84</v>
+        <v>4.94</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1253,17 +1253,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>UTSSAV</t>
+          <t>SVPGLOB</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>346.25</v>
+        <v>4.07</v>
       </c>
       <c r="C38" t="n">
-        <v>363</v>
+        <v>4.27</v>
       </c>
       <c r="D38" t="n">
-        <v>4.84</v>
+        <v>4.91</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1275,17 +1275,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BILVYAPAR</t>
+          <t>OSIAHYPER</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>4.13</v>
+        <v>3.68</v>
       </c>
       <c r="C39" t="n">
-        <v>4.33</v>
+        <v>3.86</v>
       </c>
       <c r="D39" t="n">
-        <v>4.84</v>
+        <v>4.89</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1297,17 +1297,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>VIJIFIN</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.21</v>
+        <v>4.3</v>
       </c>
       <c r="C40" t="n">
-        <v>0.22</v>
+        <v>4.51</v>
       </c>
       <c r="D40" t="n">
-        <v>4.76</v>
+        <v>4.88</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1319,17 +1319,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>VHLTD</t>
+          <t>LCCINFOTEC</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>137.31</v>
+        <v>4.59</v>
       </c>
       <c r="C41" t="n">
-        <v>143.85</v>
+        <v>4.81</v>
       </c>
       <c r="D41" t="n">
-        <v>4.76</v>
+        <v>4.79</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1341,14 +1341,14 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SETUINFRA</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.42</v>
+        <v>0.21</v>
       </c>
       <c r="C42" t="n">
-        <v>0.44</v>
+        <v>0.22</v>
       </c>
       <c r="D42" t="n">
         <v>4.76</v>
@@ -1363,17 +1363,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MANINDS</t>
+          <t>GLFL</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>592.6</v>
+        <v>7.14</v>
       </c>
       <c r="C43" t="n">
-        <v>620</v>
+        <v>7.48</v>
       </c>
       <c r="D43" t="n">
-        <v>4.62</v>
+        <v>4.76</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1385,17 +1385,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>VPRPL</t>
+          <t>FELDVR</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>30.59</v>
+        <v>2.52</v>
       </c>
       <c r="C44" t="n">
-        <v>32</v>
+        <v>2.64</v>
       </c>
       <c r="D44" t="n">
-        <v>4.61</v>
+        <v>4.76</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1407,17 +1407,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ANKITMETAL</t>
+          <t>CEREBRAINT</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1.53</v>
+        <v>4.01</v>
       </c>
       <c r="C45" t="n">
-        <v>1.6</v>
+        <v>4.2</v>
       </c>
       <c r="D45" t="n">
-        <v>4.58</v>
+        <v>4.74</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1429,17 +1429,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SECURKLOUD</t>
+          <t>COOLCAPS</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>18.94</v>
+        <v>27.6</v>
       </c>
       <c r="C46" t="n">
-        <v>19.78</v>
+        <v>28.9</v>
       </c>
       <c r="D46" t="n">
-        <v>4.44</v>
+        <v>4.71</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1451,17 +1451,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SHIVAMILLS</t>
+          <t>VIVIDEL</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>62.05</v>
+        <v>1212.95</v>
       </c>
       <c r="C47" t="n">
-        <v>64.79000000000001</v>
+        <v>1270</v>
       </c>
       <c r="D47" t="n">
-        <v>4.42</v>
+        <v>4.7</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1473,17 +1473,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PRAXIS</t>
+          <t>S&amp;SPOWER</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>8.24</v>
+        <v>380.95</v>
       </c>
       <c r="C48" t="n">
-        <v>8.6</v>
+        <v>398.8</v>
       </c>
       <c r="D48" t="n">
-        <v>4.37</v>
+        <v>4.69</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1495,17 +1495,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SEMAC</t>
+          <t>DBSTOCKBRO</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>324.85</v>
+        <v>29.45</v>
       </c>
       <c r="C49" t="n">
-        <v>339</v>
+        <v>30.8</v>
       </c>
       <c r="D49" t="n">
-        <v>4.36</v>
+        <v>4.58</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1517,17 +1517,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PRITI</t>
+          <t>SANWARIA</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>42.5</v>
+        <v>0.22</v>
       </c>
       <c r="C50" t="n">
-        <v>44.31</v>
+        <v>0.23</v>
       </c>
       <c r="D50" t="n">
-        <v>4.26</v>
+        <v>4.55</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1539,17 +1539,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>EFFWA</t>
+          <t>PRECOT</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>345.3</v>
+        <v>727.4</v>
       </c>
       <c r="C51" t="n">
-        <v>359.9</v>
+        <v>760</v>
       </c>
       <c r="D51" t="n">
-        <v>4.23</v>
+        <v>4.48</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1561,17 +1561,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>RADIOCITY</t>
+          <t>ORIENTLTD</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>6.24</v>
+        <v>70.56999999999999</v>
       </c>
       <c r="C52" t="n">
-        <v>6.5</v>
+        <v>73.7</v>
       </c>
       <c r="D52" t="n">
-        <v>4.17</v>
+        <v>4.44</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1583,17 +1583,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>KONSTELEC</t>
+          <t>UHTL</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>48.7</v>
+        <v>113.95</v>
       </c>
       <c r="C53" t="n">
-        <v>50.7</v>
+        <v>119</v>
       </c>
       <c r="D53" t="n">
-        <v>4.11</v>
+        <v>4.43</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1605,17 +1605,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>KANORICHEM</t>
+          <t>ISHANCH</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>109.51</v>
+        <v>58.32</v>
       </c>
       <c r="C54" t="n">
-        <v>113.99</v>
+        <v>60.9</v>
       </c>
       <c r="D54" t="n">
-        <v>4.09</v>
+        <v>4.42</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1627,17 +1627,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>NITCO</t>
+          <t>SAHASRA</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>95.91</v>
+        <v>342.85</v>
       </c>
       <c r="C55" t="n">
-        <v>99.8</v>
+        <v>358</v>
       </c>
       <c r="D55" t="n">
-        <v>4.06</v>
+        <v>4.42</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1649,17 +1649,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SILINV</t>
+          <t>GRANDOAK</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>429.2</v>
+        <v>48.19</v>
       </c>
       <c r="C56" t="n">
-        <v>446.5</v>
+        <v>50.3</v>
       </c>
       <c r="D56" t="n">
-        <v>4.03</v>
+        <v>4.38</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1671,17 +1671,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>RPPL</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>168.35</v>
+        <v>18.49</v>
       </c>
       <c r="C57" t="n">
-        <v>174.99</v>
+        <v>19.29</v>
       </c>
       <c r="D57" t="n">
-        <v>3.94</v>
+        <v>4.33</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1693,17 +1693,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>RKEC</t>
+          <t>GRADIENTE</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>24.28</v>
+        <v>2.35</v>
       </c>
       <c r="C58" t="n">
-        <v>25.22</v>
+        <v>2.45</v>
       </c>
       <c r="D58" t="n">
-        <v>3.87</v>
+        <v>4.26</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1715,17 +1715,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DSFCL</t>
+          <t>IL&amp;FSTRANS</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>23.4</v>
+        <v>2.58</v>
       </c>
       <c r="C59" t="n">
-        <v>24.3</v>
+        <v>2.69</v>
       </c>
       <c r="D59" t="n">
-        <v>3.85</v>
+        <v>4.26</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1737,17 +1737,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AHLWEST</t>
+          <t>RELTD</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>544.1</v>
+        <v>143.96</v>
       </c>
       <c r="C60" t="n">
-        <v>565</v>
+        <v>150</v>
       </c>
       <c r="D60" t="n">
-        <v>3.84</v>
+        <v>4.2</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1759,17 +1759,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>AEROENTER</t>
+          <t>GOLDENTOBC</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>115.65</v>
+        <v>25.17</v>
       </c>
       <c r="C61" t="n">
-        <v>120</v>
+        <v>26.2</v>
       </c>
       <c r="D61" t="n">
-        <v>3.76</v>
+        <v>4.09</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1781,17 +1781,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>UNITECH</t>
+          <t>VERTOZ</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>5.09</v>
+        <v>44.11</v>
       </c>
       <c r="C62" t="n">
-        <v>5.28</v>
+        <v>45.9</v>
       </c>
       <c r="D62" t="n">
-        <v>3.73</v>
+        <v>4.06</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1803,17 +1803,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>BANARBEADS</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>190.13</v>
+        <v>99.53</v>
       </c>
       <c r="C63" t="n">
-        <v>197.13</v>
+        <v>103.49</v>
       </c>
       <c r="D63" t="n">
-        <v>3.68</v>
+        <v>3.98</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1825,17 +1825,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>NAGREEKEXP</t>
+          <t>EUROBOND</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>27.71</v>
+        <v>178.91</v>
       </c>
       <c r="C64" t="n">
-        <v>28.7</v>
+        <v>185.99</v>
       </c>
       <c r="D64" t="n">
-        <v>3.57</v>
+        <v>3.96</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1847,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>3PLAND</t>
+          <t>HILTON</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>31.19</v>
+        <v>22.62</v>
       </c>
       <c r="C65" t="n">
-        <v>32.3</v>
+        <v>23.5</v>
       </c>
       <c r="D65" t="n">
-        <v>3.56</v>
+        <v>3.89</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1869,17 +1869,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>DPWIRES</t>
+          <t>ANKITMETAL</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>178.42</v>
+        <v>1.55</v>
       </c>
       <c r="C66" t="n">
-        <v>184.7</v>
+        <v>1.61</v>
       </c>
       <c r="D66" t="n">
-        <v>3.52</v>
+        <v>3.87</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1891,17 +1891,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>KEEPLEARN</t>
+          <t>RADIOCITY</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>2</v>
+        <v>6.24</v>
       </c>
       <c r="C67" t="n">
-        <v>2.07</v>
+        <v>6.48</v>
       </c>
       <c r="D67" t="n">
-        <v>3.5</v>
+        <v>3.85</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1913,17 +1913,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>METROGLOBL</t>
+          <t>APCL</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>128.02</v>
+        <v>114.32</v>
       </c>
       <c r="C68" t="n">
-        <v>132.5</v>
+        <v>118.66</v>
       </c>
       <c r="D68" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1935,17 +1935,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TOUCHWOOD</t>
+          <t>INFOMEDIA</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>75.06999999999999</v>
+        <v>5.86</v>
       </c>
       <c r="C69" t="n">
-        <v>77.69</v>
+        <v>6.08</v>
       </c>
       <c r="D69" t="n">
-        <v>3.49</v>
+        <v>3.75</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1957,17 +1957,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ADROITINFO</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>9.460000000000001</v>
+        <v>199.63</v>
       </c>
       <c r="C70" t="n">
-        <v>9.789999999999999</v>
+        <v>206.99</v>
       </c>
       <c r="D70" t="n">
-        <v>3.49</v>
+        <v>3.69</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1979,17 +1979,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>RVTH</t>
+          <t>ANIKINDS</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>716.75</v>
+        <v>46.79</v>
       </c>
       <c r="C71" t="n">
-        <v>741.7</v>
+        <v>48.5</v>
       </c>
       <c r="D71" t="n">
-        <v>3.48</v>
+        <v>3.65</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -2001,14 +2001,14 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>RVHL</t>
+          <t>SUPERSPIN</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>44.46</v>
+        <v>4.92</v>
       </c>
       <c r="C72" t="n">
-        <v>46</v>
+        <v>5.09</v>
       </c>
       <c r="D72" t="n">
         <v>3.46</v>
@@ -2023,17 +2023,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BASML</t>
+          <t>STLTECH</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>24.89</v>
+        <v>647.2</v>
       </c>
       <c r="C73" t="n">
-        <v>25.75</v>
+        <v>669.5</v>
       </c>
       <c r="D73" t="n">
-        <v>3.46</v>
+        <v>3.45</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -2045,14 +2045,14 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>PML</t>
+          <t>PIGL</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>501</v>
+        <v>105.43</v>
       </c>
       <c r="C74" t="n">
-        <v>518</v>
+        <v>109</v>
       </c>
       <c r="D74" t="n">
         <v>3.39</v>
@@ -2067,17 +2067,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SUTLEJTEX</t>
+          <t>CCCL</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>37.34</v>
+        <v>14.78</v>
       </c>
       <c r="C75" t="n">
-        <v>38.6</v>
+        <v>15.28</v>
       </c>
       <c r="D75" t="n">
-        <v>3.37</v>
+        <v>3.38</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2089,17 +2089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>AMBICAAGAR</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>24.58</v>
+        <v>405.7</v>
       </c>
       <c r="C76" t="n">
-        <v>25.39</v>
+        <v>419</v>
       </c>
       <c r="D76" t="n">
-        <v>3.3</v>
+        <v>3.28</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2111,17 +2111,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>AKG</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>59.91</v>
+        <v>11.12</v>
       </c>
       <c r="C77" t="n">
-        <v>61.88</v>
+        <v>11.48</v>
       </c>
       <c r="D77" t="n">
-        <v>3.29</v>
+        <v>3.24</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2133,17 +2133,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SHANTI</t>
+          <t>CALSOFT</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>6.39</v>
+        <v>24.22</v>
       </c>
       <c r="C78" t="n">
-        <v>6.6</v>
+        <v>25</v>
       </c>
       <c r="D78" t="n">
-        <v>3.29</v>
+        <v>3.22</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2155,17 +2155,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>HEADSUP</t>
+          <t>NAHARPOLY</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>7.65</v>
+        <v>253.95</v>
       </c>
       <c r="C79" t="n">
-        <v>7.9</v>
+        <v>262</v>
       </c>
       <c r="D79" t="n">
-        <v>3.27</v>
+        <v>3.17</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2177,17 +2177,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>TFL</t>
+          <t>AMBER</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>12.88</v>
+        <v>7965.5</v>
       </c>
       <c r="C80" t="n">
-        <v>13.3</v>
+        <v>8218</v>
       </c>
       <c r="D80" t="n">
-        <v>3.26</v>
+        <v>3.17</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2199,17 +2199,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>LAGNAM</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>80.2</v>
+        <v>178.38</v>
       </c>
       <c r="C81" t="n">
-        <v>82.8</v>
+        <v>184</v>
       </c>
       <c r="D81" t="n">
-        <v>3.24</v>
+        <v>3.15</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2221,17 +2221,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CELEBRITY</t>
+          <t>PRAENG</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>7.31</v>
+        <v>21.47</v>
       </c>
       <c r="C82" t="n">
-        <v>7.54</v>
+        <v>22.14</v>
       </c>
       <c r="D82" t="n">
-        <v>3.15</v>
+        <v>3.12</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2243,17 +2243,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>LAMOSAIC</t>
+          <t>DREAMFOLKS</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>33.5</v>
+        <v>71.81999999999999</v>
       </c>
       <c r="C83" t="n">
-        <v>34.55</v>
+        <v>73.98</v>
       </c>
       <c r="D83" t="n">
-        <v>3.13</v>
+        <v>3.01</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>HYBRIDFIN</t>
+          <t>EBGNG</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>18.91</v>
+        <v>456.35</v>
       </c>
       <c r="C84" t="n">
-        <v>19.5</v>
+        <v>469.95</v>
       </c>
       <c r="D84" t="n">
-        <v>3.12</v>
+        <v>2.98</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2287,17 +2287,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>HARRMALAYA</t>
+          <t>SPAL</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>205.57</v>
+        <v>920.95</v>
       </c>
       <c r="C85" t="n">
-        <v>211.9</v>
+        <v>948</v>
       </c>
       <c r="D85" t="n">
-        <v>3.08</v>
+        <v>2.94</v>
       </c>
       <c r="E85" t="b">
         <v>0</v>
@@ -2309,17 +2309,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>BALKRISHNA</t>
+          <t>DHARIWAL</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>17.95</v>
+        <v>33.05</v>
       </c>
       <c r="C86" t="n">
-        <v>18.5</v>
+        <v>34</v>
       </c>
       <c r="D86" t="n">
-        <v>3.06</v>
+        <v>2.87</v>
       </c>
       <c r="E86" t="b">
         <v>0</v>
@@ -2331,17 +2331,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>LAXMICOT</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>15.04</v>
+        <v>13.03</v>
       </c>
       <c r="C87" t="n">
-        <v>15.5</v>
+        <v>13.4</v>
       </c>
       <c r="D87" t="n">
-        <v>3.06</v>
+        <v>2.84</v>
       </c>
       <c r="E87" t="b">
         <v>0</v>
@@ -2353,17 +2353,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SUYOG</t>
+          <t>SHRENIK</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>792.2</v>
+        <v>0.36</v>
       </c>
       <c r="C88" t="n">
-        <v>816</v>
+        <v>0.37</v>
       </c>
       <c r="D88" t="n">
-        <v>3</v>
+        <v>2.78</v>
       </c>
       <c r="E88" t="b">
         <v>0</v>
@@ -2375,17 +2375,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ICIL</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>342.1</v>
+        <v>61.12</v>
       </c>
       <c r="C89" t="n">
-        <v>352.35</v>
+        <v>62.8</v>
       </c>
       <c r="D89" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="E89" t="b">
         <v>0</v>
@@ -2397,17 +2397,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BORANA</t>
+          <t>OILCOUNTUB</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>318.5</v>
+        <v>56.54</v>
       </c>
       <c r="C90" t="n">
-        <v>328</v>
+        <v>58.09</v>
       </c>
       <c r="D90" t="n">
-        <v>2.98</v>
+        <v>2.74</v>
       </c>
       <c r="E90" t="b">
         <v>0</v>
@@ -2419,17 +2419,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>PANACHE</t>
+          <t>ARVINDPORT</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>411.2</v>
+        <v>31.05</v>
       </c>
       <c r="C91" t="n">
-        <v>423.35</v>
+        <v>31.9</v>
       </c>
       <c r="D91" t="n">
-        <v>2.95</v>
+        <v>2.74</v>
       </c>
       <c r="E91" t="b">
         <v>0</v>
@@ -2441,17 +2441,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>AURIGROW</t>
+          <t>ALPA</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.34</v>
+        <v>67.86</v>
       </c>
       <c r="C92" t="n">
-        <v>0.35</v>
+        <v>69.7</v>
       </c>
       <c r="D92" t="n">
-        <v>2.94</v>
+        <v>2.71</v>
       </c>
       <c r="E92" t="b">
         <v>0</v>
@@ -2463,17 +2463,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>KDL</t>
+          <t>BIGBLOC</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>123.1</v>
+        <v>48.99</v>
       </c>
       <c r="C93" t="n">
-        <v>126.7</v>
+        <v>50.3</v>
       </c>
       <c r="D93" t="n">
-        <v>2.92</v>
+        <v>2.67</v>
       </c>
       <c r="E93" t="b">
         <v>0</v>
@@ -2485,17 +2485,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>XTGLOBAL</t>
+          <t>DMCC</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>29.04</v>
+        <v>249.4</v>
       </c>
       <c r="C94" t="n">
-        <v>29.88</v>
+        <v>256</v>
       </c>
       <c r="D94" t="n">
-        <v>2.89</v>
+        <v>2.65</v>
       </c>
       <c r="E94" t="b">
         <v>0</v>
@@ -2507,17 +2507,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>DEEDEV</t>
+          <t>MTARTECH</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>738.75</v>
+        <v>8305.5</v>
       </c>
       <c r="C95" t="n">
-        <v>760</v>
+        <v>8525</v>
       </c>
       <c r="D95" t="n">
-        <v>2.88</v>
+        <v>2.64</v>
       </c>
       <c r="E95" t="b">
         <v>0</v>
@@ -2529,17 +2529,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BUTTERFLY</t>
+          <t>LAL</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>664.1</v>
+        <v>7.6</v>
       </c>
       <c r="C96" t="n">
-        <v>683</v>
+        <v>7.8</v>
       </c>
       <c r="D96" t="n">
-        <v>2.85</v>
+        <v>2.63</v>
       </c>
       <c r="E96" t="b">
         <v>0</v>
@@ -2551,17 +2551,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ESSENTIA</t>
+          <t>RILINFRA</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1.41</v>
+        <v>38.5</v>
       </c>
       <c r="C97" t="n">
-        <v>1.45</v>
+        <v>39.5</v>
       </c>
       <c r="D97" t="n">
-        <v>2.84</v>
+        <v>2.6</v>
       </c>
       <c r="E97" t="b">
         <v>0</v>
@@ -2573,17 +2573,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>SIGMAADV</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>411.2</v>
+        <v>500.05</v>
       </c>
       <c r="C98" t="n">
-        <v>422.8</v>
+        <v>513</v>
       </c>
       <c r="D98" t="n">
-        <v>2.82</v>
+        <v>2.59</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -2595,17 +2595,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>NDLVENTURE</t>
+          <t>ATAM</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>128.33</v>
+        <v>71.98</v>
       </c>
       <c r="C99" t="n">
-        <v>131.95</v>
+        <v>73.8</v>
       </c>
       <c r="D99" t="n">
-        <v>2.82</v>
+        <v>2.53</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -2617,17 +2617,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>DSSL</t>
+          <t>UFLEX</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1352.6</v>
+        <v>424.3</v>
       </c>
       <c r="C100" t="n">
-        <v>1390</v>
+        <v>435</v>
       </c>
       <c r="D100" t="n">
-        <v>2.77</v>
+        <v>2.52</v>
       </c>
       <c r="E100" t="b">
         <v>0</v>
@@ -2639,17 +2639,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>GOKEX</t>
+          <t>SSDL</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>729.85</v>
+        <v>57.18</v>
       </c>
       <c r="C101" t="n">
-        <v>750</v>
+        <v>58.59</v>
       </c>
       <c r="D101" t="n">
-        <v>2.76</v>
+        <v>2.47</v>
       </c>
       <c r="E101" t="b">
         <v>0</v>
@@ -2661,17 +2661,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>RHL</t>
+          <t>SUDARCOLOR</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>186.64</v>
+        <v>369.85</v>
       </c>
       <c r="C102" t="n">
-        <v>191.8</v>
+        <v>378.95</v>
       </c>
       <c r="D102" t="n">
-        <v>2.76</v>
+        <v>2.46</v>
       </c>
       <c r="E102" t="b">
         <v>0</v>
@@ -2683,17 +2683,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>TICL</t>
+          <t>FEL</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>20.35</v>
+        <v>0.41</v>
       </c>
       <c r="C103" t="n">
-        <v>20.89</v>
+        <v>0.42</v>
       </c>
       <c r="D103" t="n">
-        <v>2.65</v>
+        <v>2.44</v>
       </c>
       <c r="E103" t="b">
         <v>0</v>
@@ -2705,17 +2705,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>BLBLIMITED</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>4.96</v>
+        <v>16.1</v>
       </c>
       <c r="C104" t="n">
-        <v>5.09</v>
+        <v>16.49</v>
       </c>
       <c r="D104" t="n">
-        <v>2.62</v>
+        <v>2.42</v>
       </c>
       <c r="E104" t="b">
         <v>0</v>
@@ -2727,17 +2727,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>TECILCHEM</t>
+          <t>SHEKHAWATI</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>11.1</v>
+        <v>14.94</v>
       </c>
       <c r="C105" t="n">
-        <v>11.39</v>
+        <v>15.3</v>
       </c>
       <c r="D105" t="n">
-        <v>2.61</v>
+        <v>2.41</v>
       </c>
       <c r="E105" t="b">
         <v>0</v>
@@ -2749,17 +2749,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PEARLPOLY</t>
+          <t>MCLOUD</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>18.99</v>
+        <v>31.53</v>
       </c>
       <c r="C106" t="n">
-        <v>19.48</v>
+        <v>32.29</v>
       </c>
       <c r="D106" t="n">
-        <v>2.58</v>
+        <v>2.41</v>
       </c>
       <c r="E106" t="b">
         <v>0</v>
@@ -2771,17 +2771,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>KRISHNADEF</t>
+          <t>SUPREME</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>1306</v>
+        <v>45.89</v>
       </c>
       <c r="C107" t="n">
-        <v>1339</v>
+        <v>46.99</v>
       </c>
       <c r="D107" t="n">
-        <v>2.53</v>
+        <v>2.4</v>
       </c>
       <c r="E107" t="b">
         <v>0</v>
@@ -2793,17 +2793,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>EUROBOND</t>
+          <t>ADL</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>179.46</v>
+        <v>69.34</v>
       </c>
       <c r="C108" t="n">
-        <v>184</v>
+        <v>71</v>
       </c>
       <c r="D108" t="n">
-        <v>2.53</v>
+        <v>2.39</v>
       </c>
       <c r="E108" t="b">
         <v>0</v>
@@ -2815,17 +2815,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>DELTAMAGNT</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>61.45</v>
+        <v>25.87</v>
       </c>
       <c r="C109" t="n">
-        <v>63</v>
+        <v>26.48</v>
       </c>
       <c r="D109" t="n">
-        <v>2.52</v>
+        <v>2.36</v>
       </c>
       <c r="E109" t="b">
         <v>0</v>
@@ -2837,17 +2837,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>IVP</t>
+          <t>RELCHEMQ</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>158.01</v>
+        <v>137.76</v>
       </c>
       <c r="C110" t="n">
-        <v>161.99</v>
+        <v>141</v>
       </c>
       <c r="D110" t="n">
-        <v>2.52</v>
+        <v>2.35</v>
       </c>
       <c r="E110" t="b">
         <v>0</v>
@@ -2859,17 +2859,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>VIGOR</t>
+          <t>DCMSRIND</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>89.65000000000001</v>
+        <v>38.5</v>
       </c>
       <c r="C111" t="n">
-        <v>91.90000000000001</v>
+        <v>39.4</v>
       </c>
       <c r="D111" t="n">
-        <v>2.51</v>
+        <v>2.34</v>
       </c>
       <c r="E111" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>HLVLTD</t>
+          <t>ANMOL</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>7.98</v>
+        <v>12</v>
       </c>
       <c r="C112" t="n">
-        <v>8.18</v>
+        <v>12.28</v>
       </c>
       <c r="D112" t="n">
-        <v>2.51</v>
+        <v>2.33</v>
       </c>
       <c r="E112" t="b">
         <v>0</v>
@@ -2903,17 +2903,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SARTELE</t>
+          <t>HATHWAY</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>160.65</v>
+        <v>11.6</v>
       </c>
       <c r="C113" t="n">
-        <v>164.65</v>
+        <v>11.87</v>
       </c>
       <c r="D113" t="n">
-        <v>2.49</v>
+        <v>2.33</v>
       </c>
       <c r="E113" t="b">
         <v>0</v>
@@ -2925,17 +2925,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>FOSECOIND</t>
+          <t>AKSHARCHEM</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>5289</v>
+        <v>219.95</v>
       </c>
       <c r="C114" t="n">
-        <v>5420</v>
+        <v>225</v>
       </c>
       <c r="D114" t="n">
-        <v>2.48</v>
+        <v>2.3</v>
       </c>
       <c r="E114" t="b">
         <v>0</v>
@@ -2947,17 +2947,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>RAYMONDREL</t>
+          <t>POWERICA</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>595.3</v>
+        <v>551.6</v>
       </c>
       <c r="C115" t="n">
-        <v>609.95</v>
+        <v>564</v>
       </c>
       <c r="D115" t="n">
-        <v>2.46</v>
+        <v>2.25</v>
       </c>
       <c r="E115" t="b">
         <v>0</v>
@@ -2969,17 +2969,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>NIBE</t>
+          <t>DIGIDRIVE</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>1625.3</v>
+        <v>18.86</v>
       </c>
       <c r="C116" t="n">
-        <v>1665</v>
+        <v>19.28</v>
       </c>
       <c r="D116" t="n">
-        <v>2.44</v>
+        <v>2.23</v>
       </c>
       <c r="E116" t="b">
         <v>0</v>
@@ -2991,17 +2991,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>RVNL</t>
+          <t>DEVIT</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>245.14</v>
+        <v>28.27</v>
       </c>
       <c r="C117" t="n">
-        <v>251.02</v>
+        <v>28.9</v>
       </c>
       <c r="D117" t="n">
-        <v>2.4</v>
+        <v>2.23</v>
       </c>
       <c r="E117" t="b">
         <v>0</v>
@@ -3013,17 +3013,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>PRITIKAUTO</t>
+          <t>ANONDITA</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>16.66</v>
+        <v>1172.3</v>
       </c>
       <c r="C118" t="n">
-        <v>17.06</v>
+        <v>1198</v>
       </c>
       <c r="D118" t="n">
-        <v>2.4</v>
+        <v>2.19</v>
       </c>
       <c r="E118" t="b">
         <v>0</v>
@@ -3035,17 +3035,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CLSEL</t>
+          <t>KAVDEFENCE</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>296.35</v>
+        <v>66.03</v>
       </c>
       <c r="C119" t="n">
-        <v>303.45</v>
+        <v>67.41</v>
       </c>
       <c r="D119" t="n">
-        <v>2.4</v>
+        <v>2.09</v>
       </c>
       <c r="E119" t="b">
         <v>0</v>
@@ -3057,17 +3057,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>RSSOFTWARE</t>
+          <t>AERONEU</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>33.21</v>
+        <v>93.95</v>
       </c>
       <c r="C120" t="n">
-        <v>34</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="D120" t="n">
-        <v>2.38</v>
+        <v>2.08</v>
       </c>
       <c r="E120" t="b">
         <v>0</v>
@@ -3079,17 +3079,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>FEL</t>
+          <t>HITECHGEAR</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.42</v>
+        <v>576.1</v>
       </c>
       <c r="C121" t="n">
-        <v>0.43</v>
+        <v>588</v>
       </c>
       <c r="D121" t="n">
-        <v>2.38</v>
+        <v>2.07</v>
       </c>
       <c r="E121" t="b">
         <v>0</v>
@@ -3101,17 +3101,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>WEALTH</t>
+          <t>ZSARACOM</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>952.5</v>
+        <v>9706.5</v>
       </c>
       <c r="C122" t="n">
-        <v>975</v>
+        <v>9905</v>
       </c>
       <c r="D122" t="n">
-        <v>2.36</v>
+        <v>2.05</v>
       </c>
       <c r="E122" t="b">
         <v>0</v>
@@ -3123,17 +3123,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>PANSARI</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>309.7</v>
+        <v>3.95</v>
       </c>
       <c r="C123" t="n">
-        <v>316.95</v>
+        <v>4.03</v>
       </c>
       <c r="D123" t="n">
-        <v>2.34</v>
+        <v>2.03</v>
       </c>
       <c r="E123" t="b">
         <v>0</v>
@@ -3145,17 +3145,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>AARON</t>
+          <t>TRUALT</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>124.58</v>
+        <v>489</v>
       </c>
       <c r="C124" t="n">
-        <v>127.5</v>
+        <v>498.85</v>
       </c>
       <c r="D124" t="n">
-        <v>2.34</v>
+        <v>2.01</v>
       </c>
       <c r="E124" t="b">
         <v>0</v>
@@ -3167,17 +3167,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>BLUSPRING</t>
+          <t>GTPL</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>109.35</v>
+        <v>63.61</v>
       </c>
       <c r="C125" t="n">
-        <v>111.89</v>
+        <v>64.88</v>
       </c>
       <c r="D125" t="n">
-        <v>2.32</v>
+        <v>2</v>
       </c>
       <c r="E125" t="b">
         <v>0</v>
@@ -3189,17 +3189,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>GSLSU</t>
+          <t>INVPRECQ</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>51.8</v>
+        <v>646.85</v>
       </c>
       <c r="C126" t="n">
-        <v>53</v>
+        <v>659.7</v>
       </c>
       <c r="D126" t="n">
-        <v>2.32</v>
+        <v>1.99</v>
       </c>
       <c r="E126" t="b">
         <v>0</v>
@@ -3211,17 +3211,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>PENINLAND</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>16.03</v>
+        <v>7.6</v>
       </c>
       <c r="C127" t="n">
-        <v>16.4</v>
+        <v>7.75</v>
       </c>
       <c r="D127" t="n">
-        <v>2.31</v>
+        <v>1.97</v>
       </c>
       <c r="E127" t="b">
         <v>0</v>
@@ -3233,17 +3233,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>HPAL</t>
+          <t>DUCON</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>36.12</v>
+        <v>3.56</v>
       </c>
       <c r="C128" t="n">
-        <v>36.95</v>
+        <v>3.63</v>
       </c>
       <c r="D128" t="n">
-        <v>2.3</v>
+        <v>1.97</v>
       </c>
       <c r="E128" t="b">
         <v>0</v>
@@ -3255,17 +3255,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>AGRITECH</t>
+          <t>INDSWFTLAB</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>116.81</v>
+        <v>168.68</v>
       </c>
       <c r="C129" t="n">
-        <v>119.5</v>
+        <v>172</v>
       </c>
       <c r="D129" t="n">
-        <v>2.3</v>
+        <v>1.97</v>
       </c>
       <c r="E129" t="b">
         <v>0</v>
@@ -3277,17 +3277,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>EVERESTIND</t>
+          <t>GVPTECH</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>371.3</v>
+        <v>6.61</v>
       </c>
       <c r="C130" t="n">
-        <v>379.8</v>
+        <v>6.74</v>
       </c>
       <c r="D130" t="n">
-        <v>2.29</v>
+        <v>1.97</v>
       </c>
       <c r="E130" t="b">
         <v>0</v>
@@ -3299,17 +3299,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SPAL</t>
+          <t>GATECH</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>830.95</v>
+        <v>0.51</v>
       </c>
       <c r="C131" t="n">
-        <v>850</v>
+        <v>0.52</v>
       </c>
       <c r="D131" t="n">
-        <v>2.29</v>
+        <v>1.96</v>
       </c>
       <c r="E131" t="b">
         <v>0</v>
@@ -3321,17 +3321,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SANGHVIMOV</t>
+          <t>PENINLAND</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>416.5</v>
+        <v>16.36</v>
       </c>
       <c r="C132" t="n">
-        <v>425.95</v>
+        <v>16.68</v>
       </c>
       <c r="D132" t="n">
-        <v>2.27</v>
+        <v>1.96</v>
       </c>
       <c r="E132" t="b">
         <v>0</v>
@@ -3343,17 +3343,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>SASKEN</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>767.5</v>
+        <v>2647.9</v>
       </c>
       <c r="C133" t="n">
-        <v>784.95</v>
+        <v>2699.6</v>
       </c>
       <c r="D133" t="n">
-        <v>2.27</v>
+        <v>1.95</v>
       </c>
       <c r="E133" t="b">
         <v>0</v>
@@ -3365,17 +3365,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ALMONDZ</t>
+          <t>PML</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>13.45</v>
+        <v>499.3</v>
       </c>
       <c r="C134" t="n">
-        <v>13.75</v>
+        <v>509</v>
       </c>
       <c r="D134" t="n">
-        <v>2.23</v>
+        <v>1.94</v>
       </c>
       <c r="E134" t="b">
         <v>0</v>
@@ -3387,17 +3387,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>METROBRAND</t>
+          <t>KOTYARK</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>1022.2</v>
+        <v>400</v>
       </c>
       <c r="C135" t="n">
-        <v>1045</v>
+        <v>407.7</v>
       </c>
       <c r="D135" t="n">
-        <v>2.23</v>
+        <v>1.92</v>
       </c>
       <c r="E135" t="b">
         <v>0</v>
@@ -3409,17 +3409,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>HDIL</t>
+          <t>RUCHINFRA</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>1.8</v>
+        <v>6.34</v>
       </c>
       <c r="C136" t="n">
-        <v>1.84</v>
+        <v>6.46</v>
       </c>
       <c r="D136" t="n">
-        <v>2.22</v>
+        <v>1.89</v>
       </c>
       <c r="E136" t="b">
         <v>0</v>
@@ -3431,17 +3431,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>RUCHINFRA</t>
+          <t>SHYAMTEL</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>6.31</v>
+        <v>18.11</v>
       </c>
       <c r="C137" t="n">
-        <v>6.45</v>
+        <v>18.45</v>
       </c>
       <c r="D137" t="n">
-        <v>2.22</v>
+        <v>1.88</v>
       </c>
       <c r="E137" t="b">
         <v>0</v>
@@ -3453,17 +3453,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>BBTCL</t>
+          <t>CUBEXTUB</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>218.16</v>
+        <v>86.19</v>
       </c>
       <c r="C138" t="n">
-        <v>223</v>
+        <v>87.8</v>
       </c>
       <c r="D138" t="n">
-        <v>2.22</v>
+        <v>1.87</v>
       </c>
       <c r="E138" t="b">
         <v>0</v>
@@ -3475,17 +3475,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>JHS</t>
+          <t>HMAAGRO</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>8.1</v>
+        <v>22.46</v>
       </c>
       <c r="C139" t="n">
-        <v>8.279999999999999</v>
+        <v>22.88</v>
       </c>
       <c r="D139" t="n">
-        <v>2.22</v>
+        <v>1.87</v>
       </c>
       <c r="E139" t="b">
         <v>0</v>
@@ -3497,17 +3497,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>INDOUS</t>
+          <t>MALLCOM</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>90.47</v>
+        <v>1080.8</v>
       </c>
       <c r="C140" t="n">
-        <v>92.45</v>
+        <v>1101</v>
       </c>
       <c r="D140" t="n">
-        <v>2.19</v>
+        <v>1.87</v>
       </c>
       <c r="E140" t="b">
         <v>0</v>
@@ -3519,17 +3519,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>UNIHEALTH</t>
+          <t>GROBTEA</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>547.8</v>
+        <v>942.6</v>
       </c>
       <c r="C141" t="n">
-        <v>559.8</v>
+        <v>960</v>
       </c>
       <c r="D141" t="n">
-        <v>2.19</v>
+        <v>1.85</v>
       </c>
       <c r="E141" t="b">
         <v>0</v>
@@ -3541,17 +3541,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>K2INFRA</t>
+          <t>VIGOR</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>78.3</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="C142" t="n">
-        <v>80</v>
+        <v>95.8</v>
       </c>
       <c r="D142" t="n">
-        <v>2.17</v>
+        <v>1.81</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
@@ -3563,17 +3563,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>NILASPACES</t>
+          <t>KNAGRI</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>13.02</v>
+        <v>204.28</v>
       </c>
       <c r="C143" t="n">
-        <v>13.3</v>
+        <v>207.95</v>
       </c>
       <c r="D143" t="n">
-        <v>2.15</v>
+        <v>1.8</v>
       </c>
       <c r="E143" t="b">
         <v>0</v>
@@ -3585,17 +3585,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>RUSHIL</t>
+          <t>BRNL</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>17.81</v>
+        <v>18.85</v>
       </c>
       <c r="C144" t="n">
-        <v>18.19</v>
+        <v>19.19</v>
       </c>
       <c r="D144" t="n">
-        <v>2.13</v>
+        <v>1.8</v>
       </c>
       <c r="E144" t="b">
         <v>0</v>
@@ -3607,17 +3607,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>GATECHDVR</t>
+          <t>UGARSUGAR</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>0.47</v>
+        <v>39.59</v>
       </c>
       <c r="C145" t="n">
-        <v>0.48</v>
+        <v>40.3</v>
       </c>
       <c r="D145" t="n">
-        <v>2.13</v>
+        <v>1.79</v>
       </c>
       <c r="E145" t="b">
         <v>0</v>
@@ -3629,17 +3629,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ENERGYDEV</t>
+          <t>GICL</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>16.98</v>
+        <v>22.94</v>
       </c>
       <c r="C146" t="n">
-        <v>17.34</v>
+        <v>23.35</v>
       </c>
       <c r="D146" t="n">
-        <v>2.12</v>
+        <v>1.79</v>
       </c>
       <c r="E146" t="b">
         <v>0</v>
@@ -3651,17 +3651,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>THYROCARE</t>
+          <t>VHLTD</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>533.5</v>
+        <v>137.49</v>
       </c>
       <c r="C147" t="n">
-        <v>544.8</v>
+        <v>139.94</v>
       </c>
       <c r="D147" t="n">
-        <v>2.12</v>
+        <v>1.78</v>
       </c>
       <c r="E147" t="b">
         <v>0</v>
@@ -3673,17 +3673,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>COASTCORP</t>
+          <t>SAKHTISUG</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>51.16</v>
+        <v>18.13</v>
       </c>
       <c r="C148" t="n">
-        <v>52.24</v>
+        <v>18.45</v>
       </c>
       <c r="D148" t="n">
-        <v>2.11</v>
+        <v>1.77</v>
       </c>
       <c r="E148" t="b">
         <v>0</v>
@@ -3695,17 +3695,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>VIPCLOTHNG</t>
+          <t>MVGJL</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>25.15</v>
+        <v>148.38</v>
       </c>
       <c r="C149" t="n">
-        <v>25.68</v>
+        <v>151</v>
       </c>
       <c r="D149" t="n">
-        <v>2.11</v>
+        <v>1.77</v>
       </c>
       <c r="E149" t="b">
         <v>0</v>
@@ -3717,17 +3717,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MALLCOM</t>
+          <t>RVHL</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1097</v>
+        <v>45.2</v>
       </c>
       <c r="C150" t="n">
-        <v>1120</v>
+        <v>45.99</v>
       </c>
       <c r="D150" t="n">
-        <v>2.1</v>
+        <v>1.75</v>
       </c>
       <c r="E150" t="b">
         <v>0</v>
@@ -3739,17 +3739,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>DMCC</t>
+          <t>AQYLON</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>252.65</v>
+        <v>48.04</v>
       </c>
       <c r="C151" t="n">
-        <v>257.9</v>
+        <v>48.87</v>
       </c>
       <c r="D151" t="n">
-        <v>2.08</v>
+        <v>1.73</v>
       </c>
       <c r="E151" t="b">
         <v>0</v>
@@ -3761,17 +3761,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>GEEKAYWIRE</t>
+          <t>GEECEE</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>25.42</v>
+        <v>350.35</v>
       </c>
       <c r="C152" t="n">
-        <v>25.95</v>
+        <v>356.4</v>
       </c>
       <c r="D152" t="n">
-        <v>2.08</v>
+        <v>1.73</v>
       </c>
       <c r="E152" t="b">
         <v>0</v>
@@ -3783,17 +3783,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>LCCINFOTEC</t>
+          <t>ESTER</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>4.38</v>
+        <v>90.95</v>
       </c>
       <c r="C153" t="n">
-        <v>4.47</v>
+        <v>92.48999999999999</v>
       </c>
       <c r="D153" t="n">
-        <v>2.05</v>
+        <v>1.69</v>
       </c>
       <c r="E153" t="b">
         <v>0</v>
@@ -3805,17 +3805,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ROSSELLIND</t>
+          <t>BCPL</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>55.91</v>
+        <v>76.41</v>
       </c>
       <c r="C154" t="n">
-        <v>57.05</v>
+        <v>77.7</v>
       </c>
       <c r="D154" t="n">
-        <v>2.04</v>
+        <v>1.69</v>
       </c>
       <c r="E154" t="b">
         <v>0</v>
@@ -3827,17 +3827,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>AMBALALSA</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>0.49</v>
+        <v>32.15</v>
       </c>
       <c r="C155" t="n">
-        <v>0.5</v>
+        <v>32.69</v>
       </c>
       <c r="D155" t="n">
-        <v>2.04</v>
+        <v>1.68</v>
       </c>
       <c r="E155" t="b">
         <v>0</v>
@@ -3849,17 +3849,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>BIKEWO</t>
+          <t>VINNY</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>29.6</v>
+        <v>1.2</v>
       </c>
       <c r="C156" t="n">
-        <v>30.2</v>
+        <v>1.22</v>
       </c>
       <c r="D156" t="n">
-        <v>2.03</v>
+        <v>1.67</v>
       </c>
       <c r="E156" t="b">
         <v>0</v>
@@ -3871,17 +3871,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>AKSHOPTFBR</t>
+          <t>COUNCODOS</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>6.9</v>
+        <v>4.81</v>
       </c>
       <c r="C157" t="n">
-        <v>7.04</v>
+        <v>4.89</v>
       </c>
       <c r="D157" t="n">
-        <v>2.03</v>
+        <v>1.66</v>
       </c>
       <c r="E157" t="b">
         <v>0</v>
@@ -3893,17 +3893,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>HAPPYFORGE</t>
+          <t>RAJRILTD</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>1431.2</v>
+        <v>21.15</v>
       </c>
       <c r="C158" t="n">
-        <v>1460</v>
+        <v>21.5</v>
       </c>
       <c r="D158" t="n">
-        <v>2.01</v>
+        <v>1.65</v>
       </c>
       <c r="E158" t="b">
         <v>0</v>
@@ -3915,17 +3915,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>VAISHALI</t>
+          <t>WABAG</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>7.45</v>
+        <v>1821.8</v>
       </c>
       <c r="C159" t="n">
-        <v>7.6</v>
+        <v>1851.8</v>
       </c>
       <c r="D159" t="n">
-        <v>2.01</v>
+        <v>1.65</v>
       </c>
       <c r="E159" t="b">
         <v>0</v>
@@ -3937,17 +3937,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>JKIPL</t>
+          <t>LGHL</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>117.34</v>
+        <v>229.73</v>
       </c>
       <c r="C160" t="n">
-        <v>119.7</v>
+        <v>233.5</v>
       </c>
       <c r="D160" t="n">
-        <v>2.01</v>
+        <v>1.64</v>
       </c>
       <c r="E160" t="b">
         <v>0</v>
@@ -3959,17 +3959,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>BRANDMAN</t>
+          <t>SRTL</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>182</v>
+        <v>39.85</v>
       </c>
       <c r="C161" t="n">
-        <v>185.65</v>
+        <v>40.5</v>
       </c>
       <c r="D161" t="n">
-        <v>2.01</v>
+        <v>1.63</v>
       </c>
       <c r="E161" t="b">
         <v>0</v>
@@ -3981,17 +3981,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>MOKSH</t>
+          <t>MUKKA</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>11.99</v>
+        <v>24.55</v>
       </c>
       <c r="C162" t="n">
-        <v>12.23</v>
+        <v>24.95</v>
       </c>
       <c r="D162" t="n">
-        <v>2</v>
+        <v>1.63</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
@@ -4003,17 +4003,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SILLYMONKS</t>
+          <t>ROHLTD</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>17.02</v>
+        <v>331.6</v>
       </c>
       <c r="C163" t="n">
-        <v>17.36</v>
+        <v>337</v>
       </c>
       <c r="D163" t="n">
-        <v>2</v>
+        <v>1.63</v>
       </c>
       <c r="E163" t="b">
         <v>0</v>
@@ -4025,17 +4025,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>MAHESHWARI</t>
+          <t>NELCO</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>71.33</v>
+        <v>871.9</v>
       </c>
       <c r="C164" t="n">
-        <v>72.75</v>
+        <v>886</v>
       </c>
       <c r="D164" t="n">
-        <v>1.99</v>
+        <v>1.62</v>
       </c>
       <c r="E164" t="b">
         <v>0</v>
@@ -4047,17 +4047,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>TRANSPEK</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>998.5</v>
+        <v>226.35</v>
       </c>
       <c r="C165" t="n">
-        <v>1018.4</v>
+        <v>229.99</v>
       </c>
       <c r="D165" t="n">
-        <v>1.99</v>
+        <v>1.61</v>
       </c>
       <c r="E165" t="b">
         <v>0</v>
@@ -4069,17 +4069,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>SHEMAROO</t>
+          <t>BAHETI</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>129.53</v>
+        <v>679.05</v>
       </c>
       <c r="C166" t="n">
-        <v>132.1</v>
+        <v>690</v>
       </c>
       <c r="D166" t="n">
-        <v>1.98</v>
+        <v>1.61</v>
       </c>
       <c r="E166" t="b">
         <v>0</v>
@@ -4091,17 +4091,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>SIL</t>
+          <t>ELANTAS</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>15.68</v>
+        <v>10505.5</v>
       </c>
       <c r="C167" t="n">
-        <v>15.99</v>
+        <v>10675</v>
       </c>
       <c r="D167" t="n">
-        <v>1.98</v>
+        <v>1.61</v>
       </c>
       <c r="E167" t="b">
         <v>0</v>
@@ -4113,17 +4113,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>ASAL</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>184.37</v>
+        <v>507.85</v>
       </c>
       <c r="C168" t="n">
-        <v>188</v>
+        <v>516</v>
       </c>
       <c r="D168" t="n">
-        <v>1.97</v>
+        <v>1.6</v>
       </c>
       <c r="E168" t="b">
         <v>0</v>
@@ -4135,17 +4135,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>BHANDARI</t>
+          <t>CENTRUM</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>3.06</v>
+        <v>21.95</v>
       </c>
       <c r="C169" t="n">
-        <v>3.12</v>
+        <v>22.3</v>
       </c>
       <c r="D169" t="n">
-        <v>1.96</v>
+        <v>1.59</v>
       </c>
       <c r="E169" t="b">
         <v>0</v>
@@ -4157,17 +4157,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>DELPHIFX</t>
+          <t>ABINFRA</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>8.66</v>
+        <v>10.24</v>
       </c>
       <c r="C170" t="n">
-        <v>8.83</v>
+        <v>10.4</v>
       </c>
       <c r="D170" t="n">
-        <v>1.96</v>
+        <v>1.56</v>
       </c>
       <c r="E170" t="b">
         <v>0</v>
@@ -4179,17 +4179,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>V2RETAIL</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>196.16</v>
+        <v>230.44</v>
       </c>
       <c r="C171" t="n">
-        <v>200</v>
+        <v>234</v>
       </c>
       <c r="D171" t="n">
-        <v>1.96</v>
+        <v>1.54</v>
       </c>
       <c r="E171" t="b">
         <v>0</v>
@@ -4201,17 +4201,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>GATECH</t>
+          <t>MTEDUCARE</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.51</v>
+        <v>1.96</v>
       </c>
       <c r="C172" t="n">
-        <v>0.52</v>
+        <v>1.99</v>
       </c>
       <c r="D172" t="n">
-        <v>1.96</v>
+        <v>1.53</v>
       </c>
       <c r="E172" t="b">
         <v>0</v>
@@ -4223,17 +4223,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>IGCL</t>
+          <t>IZMO</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>63.71</v>
+        <v>1024.35</v>
       </c>
       <c r="C173" t="n">
-        <v>64.95999999999999</v>
+        <v>1040</v>
       </c>
       <c r="D173" t="n">
-        <v>1.96</v>
+        <v>1.53</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -4245,17 +4245,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ZODIACLOTH</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>955.55</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="C174" t="n">
-        <v>974.15</v>
+        <v>84.37</v>
       </c>
       <c r="D174" t="n">
-        <v>1.95</v>
+        <v>1.53</v>
       </c>
       <c r="E174" t="b">
         <v>0</v>
@@ -4267,17 +4267,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>SAHANA</t>
+          <t>LINCOLN</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>936.8</v>
+        <v>608.75</v>
       </c>
       <c r="C175" t="n">
-        <v>954.95</v>
+        <v>618</v>
       </c>
       <c r="D175" t="n">
-        <v>1.94</v>
+        <v>1.52</v>
       </c>
       <c r="E175" t="b">
         <v>0</v>
@@ -4289,17 +4289,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>RPTECH</t>
+          <t>KAMOPAINTS</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>685.8</v>
+        <v>5.28</v>
       </c>
       <c r="C176" t="n">
-        <v>699.05</v>
+        <v>5.36</v>
       </c>
       <c r="D176" t="n">
-        <v>1.93</v>
+        <v>1.52</v>
       </c>
       <c r="E176" t="b">
         <v>0</v>
@@ -4311,17 +4311,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>RAJRILTD</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>20.74</v>
+        <v>125.41</v>
       </c>
       <c r="C177" t="n">
-        <v>21.14</v>
+        <v>127.3</v>
       </c>
       <c r="D177" t="n">
-        <v>1.93</v>
+        <v>1.51</v>
       </c>
       <c r="E177" t="b">
         <v>0</v>
@@ -4333,17 +4333,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>RNBDENIMS</t>
+          <t>ESAFSFB</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>10.94</v>
+        <v>32.02</v>
       </c>
       <c r="C178" t="n">
-        <v>11.15</v>
+        <v>32.5</v>
       </c>
       <c r="D178" t="n">
-        <v>1.92</v>
+        <v>1.5</v>
       </c>
       <c r="E178" t="b">
         <v>0</v>
@@ -4355,17 +4355,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>SACHEEROME</t>
+          <t>CONFIPET</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>322.8</v>
+        <v>67.89</v>
       </c>
       <c r="C179" t="n">
-        <v>329</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D179" t="n">
-        <v>1.92</v>
+        <v>1.49</v>
       </c>
       <c r="E179" t="b">
         <v>0</v>
@@ -4377,17 +4377,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>VIVIDHA</t>
+          <t>ATGL</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>0.52</v>
+        <v>724.35</v>
       </c>
       <c r="C180" t="n">
-        <v>0.53</v>
+        <v>735</v>
       </c>
       <c r="D180" t="n">
-        <v>1.92</v>
+        <v>1.47</v>
       </c>
       <c r="E180" t="b">
         <v>0</v>
@@ -4399,17 +4399,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>HIMATSEIDE</t>
+          <t>PRAXIS</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>78.55</v>
+        <v>8.18</v>
       </c>
       <c r="C181" t="n">
-        <v>80.05</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D181" t="n">
-        <v>1.91</v>
+        <v>1.47</v>
       </c>
       <c r="E181" t="b">
         <v>0</v>
@@ -4421,17 +4421,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>INDBANK</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>3.16</v>
+        <v>34.26</v>
       </c>
       <c r="C182" t="n">
-        <v>3.22</v>
+        <v>34.75</v>
       </c>
       <c r="D182" t="n">
-        <v>1.9</v>
+        <v>1.43</v>
       </c>
       <c r="E182" t="b">
         <v>0</v>
@@ -4443,17 +4443,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>ARSHIYA</t>
+          <t>NAHARSPING</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>1.06</v>
+        <v>256.35</v>
       </c>
       <c r="C183" t="n">
-        <v>1.08</v>
+        <v>260</v>
       </c>
       <c r="D183" t="n">
-        <v>1.89</v>
+        <v>1.42</v>
       </c>
       <c r="E183" t="b">
         <v>0</v>
@@ -4465,17 +4465,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MAHEPC</t>
+          <t>LOVABLE</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>116.71</v>
+        <v>73.66</v>
       </c>
       <c r="C184" t="n">
-        <v>118.9</v>
+        <v>74.7</v>
       </c>
       <c r="D184" t="n">
-        <v>1.88</v>
+        <v>1.41</v>
       </c>
       <c r="E184" t="b">
         <v>0</v>
@@ -4487,17 +4487,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>KALYANIFRG</t>
+          <t>NOIDATOLL</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>593</v>
+        <v>4.96</v>
       </c>
       <c r="C185" t="n">
-        <v>604</v>
+        <v>5.03</v>
       </c>
       <c r="D185" t="n">
-        <v>1.85</v>
+        <v>1.41</v>
       </c>
       <c r="E185" t="b">
         <v>0</v>
@@ -4509,17 +4509,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>GRPLTD</t>
+          <t>DIGISPICE</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>1811.4</v>
+        <v>20.01</v>
       </c>
       <c r="C186" t="n">
-        <v>1845</v>
+        <v>20.29</v>
       </c>
       <c r="D186" t="n">
-        <v>1.85</v>
+        <v>1.4</v>
       </c>
       <c r="E186" t="b">
         <v>0</v>
@@ -4531,17 +4531,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>AMIRCHAND</t>
+          <t>NITTAGELA</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>129.52</v>
+        <v>1602.7</v>
       </c>
       <c r="C187" t="n">
-        <v>131.9</v>
+        <v>1625</v>
       </c>
       <c r="D187" t="n">
-        <v>1.84</v>
+        <v>1.39</v>
       </c>
       <c r="E187" t="b">
         <v>0</v>
@@ -4553,17 +4553,17 @@
     <row r="188">
       <c r="A188